<commit_message>
Benchmark_Anamnesis: iteración 2 (+Clinia, MiRedSalud, Mediko)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Fqg9EeHAPQipmpACMWyqBb
</commit_message>
<xml_diff>
--- a/Outputs/Benchmark_Anamnesis.xlsx
+++ b/Outputs/Benchmark_Anamnesis.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -488,7 +488,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>[DIRECTO · Chile · etapas A+B] Lanzada 25-sep-2024 en App Store (Android previsto la misma semana). &gt;1.500 usuarios en los primeros días; meta 32.000 (cofundador Francisco González). Funciones: gestión de documentos, importar solicitudes, SOS con alergias/medicación, calendario de citas, recordatorios, compartir con profesionales elegidos. Sin blockchain. Precio y estado actual NO verificados; única fuente es una nota de prensa. Sitio oficial por confirmar.</t>
+          <t>[DIRECTO · Chile · etapas A+B] Lanzada 25-sep-2024 en App Store (Android previsto la misma semana). &gt;1.500 usuarios en los primeros días; meta 32.000 (cofundador Francisco González). Funciones: gestión de documentos, importar solicitudes, SOS con alergias/medicación, calendario de citas, recordatorios, compartir con profesionales elegidos. Sin blockchain. Precio y estado actual NO verificados; única fuente es una nota de prensa. Sitio oficial por confirmar. [Iter. 2] Hay cobertura adicional en Portal Innova (portalinnova.cl); sitio bloqueado en este entorno, estado actual sigue sin verificar.</t>
         </is>
       </c>
     </row>
@@ -786,6 +786,87 @@
       <c r="E13" s="2" t="inlineStr">
         <is>
           <t>[SUSTITUTO PARCIAL · Chile] Reservar hora, ver historial de esa institución, vincular familiar. Gratis; no consolida datos de otras instituciones.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Clinia (Reservo)</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Otro: Salud (PHR paciente)</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>https://www.zoomtecnologico.com/2026/09/16/clinia-historia-medico/</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>[DIRECTO · Chile · etapa A] App móvil anunciada en sep-2026 para centralizar recetas, diagnósticos y laboratorios en un solo lugar; respaldada por Reservo (tecnológica chilena desde 2015, software para profesionales y centros de salud). AMENAZA ALTA: Reservo ya tiene red de profesionales/centros que podrían alimentar el historial. Fuente: solo snippet de búsqueda (sitio bloqueado en este entorno); precio, funciones de compartir y sitio oficial por verificar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>MiRedSalud (RedSalud)</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Otro: Salud (portal de red de clínicas)</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>https://www.redsalud.cl/noticias/miredsalud-lanza-su-nueva-app-movil-tu-salud-ahora-mas-cerca-que-nunca</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>[SUSTITUTO PARCIAL · Chile] Nueva app móvil de la red RedSalud anunciada dic-2025: acceso a información clínica y servicios, guardar y administrar historial propio y familiar. Limitación: solo datos de la propia red; no consolida otras instituciones. Precio por verificar (probablemente gratis).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Mediko</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Otro: Salud (asistente IA / orientación médica)</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>https://mediko.cl</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>[ADYACENTE · Chile] Fundada 2022. Orientación médica inmediata, interpretación de exámenes y órdenes médicas digitales con IA; modelo freemium, suscripción y pago por servicio; menciona centralizar registros y monitoreo. Foco asistencial, no archivo personal; vigilar si añade historial. Grants por ~$40M según Descubre.vc.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Benchmark_Anamnesis: iteración 3 (+Mi Bupa, datos de Reservo/Clinia)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Fqg9EeHAPQipmpACMWyqBb
</commit_message>
<xml_diff>
--- a/Outputs/Benchmark_Anamnesis.xlsx
+++ b/Outputs/Benchmark_Anamnesis.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -812,7 +812,7 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>[DIRECTO · Chile · etapa A] App móvil anunciada en sep-2026 para centralizar recetas, diagnósticos y laboratorios en un solo lugar; respaldada por Reservo (tecnológica chilena desde 2015, software para profesionales y centros de salud). AMENAZA ALTA: Reservo ya tiene red de profesionales/centros que podrían alimentar el historial. Fuente: solo snippet de búsqueda (sitio bloqueado en este entorno); precio, funciones de compartir y sitio oficial por verificar.</t>
+          <t>[DIRECTO · Chile · etapa A] App móvil anunciada en sep-2026 para centralizar recetas, diagnósticos y laboratorios en un solo lugar; respaldada por Reservo (tecnológica chilena desde 2015, software para profesionales y centros de salud). AMENAZA ALTA: Reservo ya tiene red de profesionales/centros que podrían alimentar el historial. Fuente: solo snippet de búsqueda (sitio bloqueado en este entorno); precio, funciones de compartir y sitio oficial por verificar. [Iter. 3] Reservo (fundada 2015; opera en Chile, México y Argentina) reporta &gt;36.500 profesionales y centros y ~14 millones de reservas al año (chocale.cl, sep-2026): base de distribución potencial enorme. No se pudo confirmar Clinia en una segunda búsqueda; sigue pendiente su sitio oficial.</t>
         </is>
       </c>
     </row>
@@ -867,6 +867,33 @@
       <c r="E16" s="2" t="inlineStr">
         <is>
           <t>[ADYACENTE · Chile] Fundada 2022. Orientación médica inmediata, interpretación de exámenes y órdenes médicas digitales con IA; modelo freemium, suscripción y pago por servicio; menciona centralizar registros y monitoreo. Foco asistencial, no archivo personal; vigilar si añade historial. Grants por ~$40M según Descubre.vc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Mi Bupa (Bupa / Integramédica / Cruz Blanca)</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Otro: Salud (portal de red de clínicas y aseguradora)</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>https://chocale.cl/2020/10/app-mi-bupa-integramedica-cruz-blanca/</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>[SUSTITUTO PARCIAL · Chile] App lanzada oct-2020 para pacientes de Integramédica y Clínica Bupa y afiliados de Isapre Cruz Blanca. Incluye 'Carpeta Personal de Salud' que consolida exámenes (Integramédica), cirugías (Clínica Bupa) y licencias (Cruz Blanca). Limitación: solo datos del grupo Bupa; no es portable ni consolida otras instituciones. Relevante porque une prestador + aseguradora, el caso que Anamnesis quiere evitar o controlar (etapa B con aseguradoras).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Benchmark: vuelta 2, iteración 1 (Meedika, Infomed, MediPlanner, Clingot)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MVcXu8vTBu7EKfj3YdEvae
</commit_message>
<xml_diff>
--- a/Outputs/Benchmark_Anamnesis.xlsx
+++ b/Outputs/Benchmark_Anamnesis.xlsx
@@ -518,7 +518,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G2" t="n">
@@ -558,7 +558,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G3" t="n">
@@ -598,7 +598,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G4" t="n">
@@ -638,7 +638,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G5" t="n">
@@ -1102,7 +1102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F68"/>
+  <dimension ref="A1:F81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3286,6 +3286,422 @@
       <c r="F68" t="inlineStr">
         <is>
           <t>Búsqueda web (Descubre.vc, Salud Digital); sitio bloqueado</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Infomed</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Seguridad, privacidad y blockchain</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Seguridad y confianza tipo banca</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Almacenamiento seguro del historial con criterios de seguridad estrictos, comparable a apps bancarias.</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>DF (2021); estado actual no verificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Infomed</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Compartición y consentimiento</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Revisión del historial por el médico</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>El médico puede revisar el historial e ingresar datos automáticamente.</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>DF (2021)</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Infomed</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Seguimiento y bienestar</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Educación del paciente sobre su enfermedad</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Busca que el paciente aprenda sobre sus enfermedades y sea más autónomo.</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>DF (2021)</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>MediPlanner</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Medicación y recordatorios</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Bitácora de medicamentos y adherencia</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Registro de cada toma y control de adherencia; gestiona medicamentos propios y de familiares.</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Latam</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>Búsqueda web (ficha App Store MX)</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>MediPlanner</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Citas y agenda</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Búsqueda y agenda de médicos</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Busca profesionales y agenda citas desde la app.</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Latam</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>Búsqueda web (ficha App Store MX)</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>MediPlanner</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Gestión documental</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Documentos con buscador y filtros</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Guarda resultados de laboratorio, imágenes y PDFs; búsqueda y filtros.</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Latam</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>Búsqueda web (ficha App Store MX)</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>MediPlanner</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Compartición y consentimiento</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Compartir con cuidadores, maestros y profesionales</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Comparte información con cuidadores, maestros o profesionales de confianza.</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Latam</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>Búsqueda web (ficha App Store MX)</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Clingot</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Gestión documental</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Carga de estudios, imágenes, indicaciones y notas</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Sube estudios, imágenes, indicaciones médicas y notas personales; accesible en consulta o por terceros en emergencias.</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Latam</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>Búsqueda web (La Nación, grupoanimal.mx); confianza media</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Clingot</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Citas y agenda</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Directorio médico filtrable</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Directorio filtrable por obra social, especialidad, subespecialidad y cercanía.</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Latam</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>Búsqueda web (La Nación)</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Clingot</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Citas y agenda</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Ubicación de centros médicos y farmacias</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Localiza centros médicos y farmacias.</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>Latam</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>Búsqueda web (La Nación)</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Clingot</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Familia y dependientes</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Seguimiento de salud de hijos</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Los padres pueden monitorear la salud de hijos pequeños.</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Latam</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>Búsqueda web (La Nación)</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Clingot</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Seguimiento y bienestar</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Valoración de profesionales</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Calificación de la atención de profesionales con autorización previa, compartible con otros usuarios.</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Latam</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>Búsqueda web (La Nación)</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Clingot</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Interoperabilidad y fuentes de datos</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Acceso móvil y de escritorio; funciones para médicos</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Android, iOS y escritorio; médicos acceden a historias digitalizadas, envían estudios e indicaciones y organizan agenda.</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Latam</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>Búsqueda web (La Nación)</t>
         </is>
       </c>
     </row>
@@ -5288,24 +5704,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
       <c r="R2">
         <f>COUNTIF(C2:Q2,"✓")</f>
         <v/>
@@ -5322,25 +5725,11 @@
           <t>Reserva de citas médicas</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
       <c r="R3">
         <f>COUNTIF(C3:Q3,"✓")</f>
         <v/>
@@ -5362,19 +5751,16 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr">
         <is>
           <t>✓</t>
@@ -5390,12 +5776,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
       <c r="R4">
         <f>COUNTIF(C4:Q4,"✓")</f>
         <v/>
@@ -5412,25 +5792,11 @@
           <t>Gestión de consentimiento sobre uso de datos</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr"/>
       <c r="R5">
         <f>COUNTIF(C5:Q5,"✓")</f>
         <v/>
@@ -5447,25 +5813,11 @@
           <t>Ingreso de datos por profesional con consentimiento</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="inlineStr"/>
       <c r="R6">
         <f>COUNTIF(C6:Q6,"✓")</f>
         <v/>
@@ -5492,23 +5844,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr"/>
-      <c r="Q7" t="inlineStr"/>
       <c r="R7">
         <f>COUNTIF(C7:Q7,"✓")</f>
         <v/>
@@ -5525,33 +5865,21 @@
           <t>Perfiles familiares / dependientes</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
       <c r="N8" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="Q8" t="inlineStr"/>
       <c r="R8">
         <f>COUNTIF(C8:Q8,"✓")</f>
         <v/>
@@ -5573,28 +5901,16 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
       <c r="O9" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="P9" t="inlineStr"/>
-      <c r="Q9" t="inlineStr"/>
       <c r="R9">
         <f>COUNTIF(C9:Q9,"✓")</f>
         <v/>
@@ -5611,25 +5927,11 @@
           <t>Almacenamiento de recetas</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
-      <c r="O10" t="inlineStr"/>
-      <c r="P10" t="inlineStr"/>
-      <c r="Q10" t="inlineStr"/>
       <c r="R10">
         <f>COUNTIF(C10:Q10,"✓")</f>
         <v/>
@@ -5651,19 +5953,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr"/>
-      <c r="P11" t="inlineStr"/>
       <c r="Q11" t="inlineStr">
         <is>
           <t>✓</t>
@@ -5685,29 +5974,16 @@
           <t>Historial institucional (solo datos de la propia red)</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
       <c r="N12" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="Q12" t="inlineStr"/>
       <c r="R12">
         <f>COUNTIF(C12:Q12,"✓")</f>
         <v/>
@@ -5724,36 +6000,26 @@
           <t>Historial médico centralizado</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr"/>
-      <c r="O13" t="inlineStr"/>
-      <c r="P13" t="inlineStr"/>
       <c r="Q13" t="inlineStr">
         <is>
           <t>✓</t>
@@ -5775,25 +6041,11 @@
           <t>Línea de tiempo de salud</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
-      <c r="M14" t="inlineStr"/>
-      <c r="N14" t="inlineStr"/>
-      <c r="O14" t="inlineStr"/>
-      <c r="P14" t="inlineStr"/>
-      <c r="Q14" t="inlineStr"/>
       <c r="R14">
         <f>COUNTIF(C14:Q14,"✓")</f>
         <v/>
@@ -5810,25 +6062,11 @@
           <t>Registro de alergias y vacunas</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr"/>
-      <c r="N15" t="inlineStr"/>
-      <c r="O15" t="inlineStr"/>
-      <c r="P15" t="inlineStr"/>
-      <c r="Q15" t="inlineStr"/>
       <c r="R15">
         <f>COUNTIF(C15:Q15,"✓")</f>
         <v/>
@@ -5845,25 +6083,11 @@
           <t>Recompensas / monetización de datos del usuario</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
-      <c r="M16" t="inlineStr"/>
-      <c r="N16" t="inlineStr"/>
-      <c r="O16" t="inlineStr"/>
-      <c r="P16" t="inlineStr"/>
-      <c r="Q16" t="inlineStr"/>
       <c r="R16">
         <f>COUNTIF(C16:Q16,"✓")</f>
         <v/>
@@ -5880,25 +6104,11 @@
           <t>Coaching de salud con IA</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr"/>
-      <c r="N17" t="inlineStr"/>
-      <c r="O17" t="inlineStr"/>
-      <c r="P17" t="inlineStr"/>
-      <c r="Q17" t="inlineStr"/>
       <c r="R17">
         <f>COUNTIF(C17:Q17,"✓")</f>
         <v/>
@@ -5915,25 +6125,11 @@
           <t>Detección de patrones en métricas de salud con IA</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr"/>
       <c r="M18" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="N18" t="inlineStr"/>
-      <c r="O18" t="inlineStr"/>
-      <c r="P18" t="inlineStr"/>
-      <c r="Q18" t="inlineStr"/>
       <c r="R18">
         <f>COUNTIF(C18:Q18,"✓")</f>
         <v/>
@@ -5950,15 +6146,6 @@
           <t>Interpretación de exámenes con IA</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr">
         <is>
           <t>✓</t>
@@ -5969,9 +6156,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="N19" t="inlineStr"/>
-      <c r="O19" t="inlineStr"/>
-      <c r="P19" t="inlineStr"/>
       <c r="Q19" t="inlineStr">
         <is>
           <t>✓</t>
@@ -5993,20 +6177,6 @@
           <t>Orientación médica con IA</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr"/>
-      <c r="M20" t="inlineStr"/>
-      <c r="N20" t="inlineStr"/>
-      <c r="O20" t="inlineStr"/>
-      <c r="P20" t="inlineStr"/>
       <c r="Q20" t="inlineStr">
         <is>
           <t>✓</t>
@@ -6028,15 +6198,6 @@
           <t>Preparación de consultas médicas con IA</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr">
         <is>
           <t>✓</t>
@@ -6047,10 +6208,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="N21" t="inlineStr"/>
-      <c r="O21" t="inlineStr"/>
-      <c r="P21" t="inlineStr"/>
-      <c r="Q21" t="inlineStr"/>
       <c r="R21">
         <f>COUNTIF(C21:Q21,"✓")</f>
         <v/>
@@ -6067,15 +6224,6 @@
           <t>Resumen de historial con IA</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr">
         <is>
           <t>✓</t>
@@ -6086,10 +6234,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="N22" t="inlineStr"/>
-      <c r="O22" t="inlineStr"/>
-      <c r="P22" t="inlineStr"/>
-      <c r="Q22" t="inlineStr"/>
       <c r="R22">
         <f>COUNTIF(C22:Q22,"✓")</f>
         <v/>
@@ -6106,18 +6250,11 @@
           <t>Agregación de registros de múltiples instituciones</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr">
         <is>
           <t>✓</t>
@@ -6133,14 +6270,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="N23" t="inlineStr"/>
       <c r="O23" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="P23" t="inlineStr"/>
-      <c r="Q23" t="inlineStr"/>
       <c r="R23">
         <f>COUNTIF(C23:Q23,"✓")</f>
         <v/>
@@ -6157,25 +6291,11 @@
           <t>Analítica poblacional B2B</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
-      <c r="L24" t="inlineStr"/>
-      <c r="M24" t="inlineStr"/>
-      <c r="N24" t="inlineStr"/>
-      <c r="O24" t="inlineStr"/>
-      <c r="P24" t="inlineStr"/>
-      <c r="Q24" t="inlineStr"/>
       <c r="R24">
         <f>COUNTIF(C24:Q24,"✓")</f>
         <v/>
@@ -6192,25 +6312,11 @@
           <t>Disponibilidad multiplataforma (web/iOS/Android)</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr"/>
-      <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr"/>
-      <c r="L25" t="inlineStr"/>
-      <c r="M25" t="inlineStr"/>
-      <c r="N25" t="inlineStr"/>
-      <c r="O25" t="inlineStr"/>
-      <c r="P25" t="inlineStr"/>
-      <c r="Q25" t="inlineStr"/>
       <c r="R25">
         <f>COUNTIF(C25:Q25,"✓")</f>
         <v/>
@@ -6227,25 +6333,11 @@
           <t>Historial médico centralizado</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr"/>
-      <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr"/>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="K26" t="inlineStr"/>
-      <c r="L26" t="inlineStr"/>
-      <c r="M26" t="inlineStr"/>
-      <c r="N26" t="inlineStr"/>
-      <c r="O26" t="inlineStr"/>
-      <c r="P26" t="inlineStr"/>
-      <c r="Q26" t="inlineStr"/>
       <c r="R26">
         <f>COUNTIF(C26:Q26,"✓")</f>
         <v/>
@@ -6262,29 +6354,16 @@
           <t>Integración con wearables y apps de salud</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr"/>
-      <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
-      <c r="L27" t="inlineStr"/>
       <c r="M27" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="N27" t="inlineStr"/>
-      <c r="O27" t="inlineStr"/>
-      <c r="P27" t="inlineStr"/>
-      <c r="Q27" t="inlineStr"/>
       <c r="R27">
         <f>COUNTIF(C27:Q27,"✓")</f>
         <v/>
@@ -6306,24 +6385,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
       <c r="K28" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="L28" t="inlineStr"/>
-      <c r="M28" t="inlineStr"/>
-      <c r="N28" t="inlineStr"/>
-      <c r="O28" t="inlineStr"/>
-      <c r="P28" t="inlineStr"/>
-      <c r="Q28" t="inlineStr"/>
       <c r="R28">
         <f>COUNTIF(C28:Q28,"✓")</f>
         <v/>
@@ -6340,25 +6406,11 @@
           <t>Gráficas de evolución de indicadores</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr"/>
-      <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr"/>
-      <c r="H29" t="inlineStr"/>
-      <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr"/>
-      <c r="L29" t="inlineStr"/>
-      <c r="M29" t="inlineStr"/>
-      <c r="N29" t="inlineStr"/>
-      <c r="O29" t="inlineStr"/>
-      <c r="P29" t="inlineStr"/>
-      <c r="Q29" t="inlineStr"/>
       <c r="R29">
         <f>COUNTIF(C29:Q29,"✓")</f>
         <v/>
@@ -6375,25 +6427,11 @@
           <t>Integración con wearables y apps de salud</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr"/>
-      <c r="E30" t="inlineStr"/>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr"/>
-      <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
       <c r="K30" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="L30" t="inlineStr"/>
-      <c r="M30" t="inlineStr"/>
-      <c r="N30" t="inlineStr"/>
-      <c r="O30" t="inlineStr"/>
-      <c r="P30" t="inlineStr"/>
-      <c r="Q30" t="inlineStr"/>
       <c r="R30">
         <f>COUNTIF(C30:Q30,"✓")</f>
         <v/>
@@ -6410,25 +6448,11 @@
           <t>Panel de seguimiento de salud y bienestar</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr"/>
-      <c r="D31" t="inlineStr"/>
-      <c r="E31" t="inlineStr"/>
-      <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr"/>
-      <c r="L31" t="inlineStr"/>
-      <c r="M31" t="inlineStr"/>
-      <c r="N31" t="inlineStr"/>
-      <c r="O31" t="inlineStr"/>
-      <c r="P31" t="inlineStr"/>
-      <c r="Q31" t="inlineStr"/>
       <c r="R31">
         <f>COUNTIF(C31:Q31,"✓")</f>
         <v/>
@@ -6445,11 +6469,6 @@
           <t>Blockchain para integridad y trazabilidad de datos</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr"/>
-      <c r="D32" t="inlineStr"/>
-      <c r="E32" t="inlineStr"/>
-      <c r="F32" t="inlineStr"/>
-      <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr">
         <is>
           <t>✓</t>
@@ -6465,13 +6484,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="K32" t="inlineStr"/>
-      <c r="L32" t="inlineStr"/>
-      <c r="M32" t="inlineStr"/>
-      <c r="N32" t="inlineStr"/>
-      <c r="O32" t="inlineStr"/>
-      <c r="P32" t="inlineStr"/>
-      <c r="Q32" t="inlineStr"/>
       <c r="R32">
         <f>COUNTIF(C32:Q32,"✓")</f>
         <v/>
@@ -6488,25 +6500,11 @@
           <t>Cifrado y control de acceso biométrico</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr"/>
-      <c r="D33" t="inlineStr"/>
-      <c r="E33" t="inlineStr"/>
-      <c r="F33" t="inlineStr"/>
-      <c r="G33" t="inlineStr"/>
-      <c r="H33" t="inlineStr"/>
-      <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr"/>
       <c r="K33" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="L33" t="inlineStr"/>
-      <c r="M33" t="inlineStr"/>
-      <c r="N33" t="inlineStr"/>
-      <c r="O33" t="inlineStr"/>
-      <c r="P33" t="inlineStr"/>
-      <c r="Q33" t="inlineStr"/>
       <c r="R33">
         <f>COUNTIF(C33:Q33,"✓")</f>
         <v/>
@@ -6523,25 +6521,11 @@
           <t>Privacidad reforzada para datos de salud</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr"/>
-      <c r="D34" t="inlineStr"/>
-      <c r="E34" t="inlineStr"/>
-      <c r="F34" t="inlineStr"/>
-      <c r="G34" t="inlineStr"/>
-      <c r="H34" t="inlineStr"/>
-      <c r="I34" t="inlineStr"/>
-      <c r="J34" t="inlineStr"/>
-      <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="M34" t="inlineStr"/>
-      <c r="N34" t="inlineStr"/>
-      <c r="O34" t="inlineStr"/>
-      <c r="P34" t="inlineStr"/>
-      <c r="Q34" t="inlineStr"/>
       <c r="R34">
         <f>COUNTIF(C34:Q34,"✓")</f>
         <v/>
@@ -6558,20 +6542,6 @@
           <t>Modelo freemium y suscripción</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr"/>
-      <c r="D35" t="inlineStr"/>
-      <c r="E35" t="inlineStr"/>
-      <c r="F35" t="inlineStr"/>
-      <c r="G35" t="inlineStr"/>
-      <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr"/>
-      <c r="K35" t="inlineStr"/>
-      <c r="L35" t="inlineStr"/>
-      <c r="M35" t="inlineStr"/>
-      <c r="N35" t="inlineStr"/>
-      <c r="O35" t="inlineStr"/>
-      <c r="P35" t="inlineStr"/>
       <c r="Q35" t="inlineStr">
         <is>
           <t>✓</t>
@@ -6593,25 +6563,11 @@
           <t>Pagos con criptomoneda</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr"/>
-      <c r="D36" t="inlineStr"/>
-      <c r="E36" t="inlineStr"/>
-      <c r="F36" t="inlineStr"/>
-      <c r="G36" t="inlineStr"/>
-      <c r="H36" t="inlineStr"/>
-      <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="K36" t="inlineStr"/>
-      <c r="L36" t="inlineStr"/>
-      <c r="M36" t="inlineStr"/>
-      <c r="N36" t="inlineStr"/>
-      <c r="O36" t="inlineStr"/>
-      <c r="P36" t="inlineStr"/>
-      <c r="Q36" t="inlineStr"/>
       <c r="R36">
         <f>COUNTIF(C36:Q36,"✓")</f>
         <v/>
@@ -6628,25 +6584,11 @@
           <t>Reclamos y trámites con seguros</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr"/>
-      <c r="D37" t="inlineStr"/>
-      <c r="E37" t="inlineStr"/>
-      <c r="F37" t="inlineStr"/>
-      <c r="G37" t="inlineStr"/>
-      <c r="H37" t="inlineStr"/>
       <c r="I37" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="J37" t="inlineStr"/>
-      <c r="K37" t="inlineStr"/>
-      <c r="L37" t="inlineStr"/>
-      <c r="M37" t="inlineStr"/>
-      <c r="N37" t="inlineStr"/>
-      <c r="O37" t="inlineStr"/>
-      <c r="P37" t="inlineStr"/>
-      <c r="Q37" t="inlineStr"/>
       <c r="R37">
         <f>COUNTIF(C37:Q37,"✓")</f>
         <v/>
@@ -6663,25 +6605,11 @@
           <t>Teleconsulta con profesionales</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr"/>
-      <c r="D38" t="inlineStr"/>
-      <c r="E38" t="inlineStr"/>
-      <c r="F38" t="inlineStr"/>
-      <c r="G38" t="inlineStr"/>
-      <c r="H38" t="inlineStr"/>
-      <c r="I38" t="inlineStr"/>
       <c r="J38" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="K38" t="inlineStr"/>
-      <c r="L38" t="inlineStr"/>
-      <c r="M38" t="inlineStr"/>
-      <c r="N38" t="inlineStr"/>
-      <c r="O38" t="inlineStr"/>
-      <c r="P38" t="inlineStr"/>
-      <c r="Q38" t="inlineStr"/>
       <c r="R38">
         <f>COUNTIF(C38:Q38,"✓")</f>
         <v/>
@@ -6698,7 +6626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -6767,6 +6695,13 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Vuelta 2 (iter. 1): Meedika (sin cambios; sitio oficial y precio siguen sin verificar), Infomed, MediPlanner, Clingot revisados. Pendientes: Healfies, Patientory, MediBloc, Medicalchain, etc.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Benchmark: vuelta 2, iteración 2 (Healfies, Patientory, MediBloc, Medicalchain)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MVcXu8vTBu7EKfj3YdEvae
</commit_message>
<xml_diff>
--- a/Outputs/Benchmark_Anamnesis.xlsx
+++ b/Outputs/Benchmark_Anamnesis.xlsx
@@ -673,12 +673,12 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>[REGIONAL · Brasil] Fundada ene-2015 en Florianópolis por Helyson Lewis Velasco. Centraliza registros de salud personales: carpetas, etiquetas, línea de tiempo (medicación, exámenes, citas, dieta), compartir con familia o profesionales. Gratis; web, iOS y Android. Estado actual NO verificado (fuentes de 2015-2016). Referencia funcional cercana a etapas A+B.</t>
+          <t>[REGIONAL · Brasil] Fundada ene-2015 en Florianópolis por Helyson Lewis Velasco. Centraliza registros de salud personales: carpetas, etiquetas, línea de tiempo (medicación, exámenes, citas, dieta), compartir con familia o profesionales. Gratis; web, iOS y Android. Estado actual NO verificado (fuentes de 2015-2016). Referencia funcional cercana a etapas A+B. [Vuelta 2] Lanzada simultáneamente en Brasil, Argentina y EE.UU.; permite compartir con no registrados vía clave por email. Sin novedades posteriores a 2016.</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G6" t="n">
@@ -713,12 +713,12 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>[BLOCKCHAIN · EE.UU.] Atlanta, fundada 2015, ~9 empleados. Levantó US$7,2M vía financiamiento cripto. App con registros de hospitales y wearables, coaching de salud con IA y recompensas en cripto; también dashboard empresarial Neith. PitchBook indica actividad y financiamiento hasta abr-2026: sigue operando. Sin presencia conocida en Chile. Referencia directa para la hipótesis blockchain.</t>
+          <t>[BLOCKCHAIN · EE.UU.] Atlanta, fundada 2015, ~9 empleados. Levantó US$7,2M vía financiamiento cripto. App con registros de hospitales y wearables, coaching de salud con IA y recompensas en cripto; también dashboard empresarial Neith. PitchBook indica actividad y financiamiento hasta abr-2026: sigue operando. Sin presencia conocida en Chile. Referencia directa para la hipótesis blockchain. [Vuelta 2] Sin noticias 2026 encontradas en búsqueda; sitio oficial bloqueado.</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G7" t="n">
@@ -753,12 +753,12 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>[BLOCKCHAIN · Corea del Sur] Fundada 2017, Seúl. Blockchain propia Panacea (Cosmos SDK, mainnet 2019) para que el paciente gestione y transfiera sus registros; app Medipass para seguros. Serie A de ₩4.000 millones (Naver); alianzas con hospitales (Seoul National, Severance). Estado 2025-26 NO verificado. Referencia sobre seguros + blockchain.</t>
+          <t>[BLOCKCHAIN · Corea del Sur] Fundada 2017, Seúl. Blockchain propia Panacea (Cosmos SDK, mainnet 2019) para que el paciente gestione y transfiera sus registros; app Medipass para seguros. Serie A de ₩4.000 millones (Naver); alianzas con hospitales (Seoul National, Severance). Estado 2025-26 NO verificado. Referencia sobre seguros + blockchain. [Vuelta 2] Panacea incluye DID, Append Only Log, IBC y PNFT; sin anuncios 2026 localizados.</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G8" t="n">
@@ -793,12 +793,12 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>[BLOCKCHAIN · Reino Unido · INACTIVO] Londres, 2017, Ethereum, con telemedicina. Piloto según registro de la UE (2020). Tracxn/PitchBook lo marcan fuera de operación (ago-2025). Solo caso de aprendizaje: no cuenta como competidor activo.</t>
+          <t>[BLOCKCHAIN · Reino Unido · INACTIVO] Londres, 2017, Ethereum, con telemedicina. Piloto según registro de la UE (2020). Tracxn/PitchBook lo marcan fuera de operación (ago-2025). Solo caso de aprendizaje: no cuenta como competidor activo. [Vuelta 2] Token MTN deslistado de Bitfinex el 26-mar-2021; sin hallazgos de actividad posterior.</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G9" t="n">
@@ -1102,7 +1102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F81"/>
+  <dimension ref="A1:F88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3702,6 +3702,230 @@
       <c r="F81" t="inlineStr">
         <is>
           <t>Búsqueda web (La Nación)</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Healfies</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Historial y perfil clínico</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Línea de tiempo ampliada: recetas, actividad física y dieta</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Registra notas de medicación, exámenes (laboratorio e imagen), actividad física, recetas, dieta y citas.</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Latam</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>Búsqueda web (Baguete); lanzada en Brasil, Argentina y EE.UU. (2015); estado actual no verificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Healfies</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Compartición y consentimiento</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Red social con profesionales y familiares</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Interacción con médicos, dentistas, kinesiólogos, entrenadores y familiares dentro de la red.</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Latam</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>Búsqueda web (Baguete)</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Healfies</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Compartición y consentimiento</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Compartir con no registrados por clave segura</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Datos compartibles con personas sin cuenta mediante clave de acceso segura enviada por email.</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Latam</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>Búsqueda web (Baguete)</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Patientory</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Compartición y consentimiento</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Autorización de acceso a proveedores con consentimiento</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>El usuario autoriza a proveedores a acceder y usar sus datos de salud.</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>Búsqueda web (Cryptopolitan); sitio bloqueado</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Patientory</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Gestión documental</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Gestión de citas, recetas y archivos</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Administra fechas, prescripciones, archivos y citas desde la app.</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>Búsqueda web (Newswire 2016)</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>MediBloc</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Seguridad, privacidad y blockchain</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Identidad descentralizada (DID)</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Gestión de identificadores descentralizados en Panacea.</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>Búsqueda web (pkg.go.dev panacea-core)</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>MediBloc</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Seguridad, privacidad y blockchain</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Registro de huellas de datos (Append Only Log)</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Almacena huellas de datos médicos en un registro de solo escritura, sin guardar datos clínicos en cadena.</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>Búsqueda web (pkg.go.dev panacea-core)</t>
         </is>
       </c>
     </row>
@@ -6626,7 +6850,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:A11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -6702,6 +6926,13 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Vuelta 2 (iter. 2, 2026-10-07 16:08 UTC): Healfies, Patientory, MediBloc, Medicalchain revisados (+7 filas). Pendientes: Apple Health, ChatGPT Health, Claude for Healthcare, Apps de clínicas, Clinia, MiRedSalud, Mediko.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Benchmark: vuelta 2, iteración 3 (Apple Health, ChatGPT Health, Claude for Healthcare, Apps de clínicas)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MVcXu8vTBu7EKfj3YdEvae
</commit_message>
<xml_diff>
--- a/Outputs/Benchmark_Anamnesis.xlsx
+++ b/Outputs/Benchmark_Anamnesis.xlsx
@@ -833,12 +833,12 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>[ADYACENTE · global] Agrega registros clínicos vía FHIR; &gt;500 instituciones conectadas en EE.UU. (2018). Sin evidencia de disponibilidad en Chile. Incluida en el dispositivo. Amenaza si FHIR/IPS-CL se adopta en Chile.</t>
+          <t>[ADYACENTE · global] Agrega registros clínicos vía FHIR; &gt;500 instituciones conectadas en EE.UU. (2018). Sin evidencia de disponibilidad en Chile. Incluida en el dispositivo. Amenaza si FHIR/IPS-CL se adopta en Chile. [Vuelta 2] Sin disponibilidad de registros clínicos en Chile (solo EE.UU., Reino Unido, Canadá).</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G10" t="n">
@@ -873,12 +873,12 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>[ADYACENTE · global] Lanzado 7-ene-2026. Conecta registros médicos; conectores solo en EE.UU. Dentro de suscripción del asistente. Fija la expectativa de consultar y resumir el historial.</t>
+          <t>[ADYACENTE · global] Lanzado 7-ene-2026. Conecta registros médicos; conectores solo en EE.UU. Dentro de suscripción del asistente. Fija la expectativa de consultar y resumir el historial. [Vuelta 2] Confirmado: registros solo EE.UU.; sin anuncios para Latinoamérica. Hay inconsistencia de fechas entre fuentes (7-ene-2026 lanzamiento vs. jul-2026 despliegue de registros).</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G11" t="n">
@@ -913,12 +913,12 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>[ADYACENTE · global] Lanzado 11-ene-2026. Conectores solo en EE.UU., planes Pro/Max. Nota: producto de Anthropic, conflicto de interés al evaluarlo.</t>
+          <t>[ADYACENTE · global] Lanzado 11-ene-2026. Conectores solo en EE.UU., planes Pro/Max. Nota: producto de Anthropic, conflicto de interés al evaluarlo. [Vuelta 2] Sin cambios fuera de EE.UU. (HealthEx y Function para Pro/Max).</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G12" t="n">
@@ -953,12 +953,12 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>[SUSTITUTO PARCIAL · Chile] Reservar hora, ver historial de esa institución, vincular familiar. Gratis; no consolida datos de otras instituciones.</t>
+          <t>[SUSTITUTO PARCIAL · Chile] Reservar hora, ver historial de esa institución, vincular familiar. Gratis; no consolida datos de otras instituciones. [Vuelta 2] App concreta: Mi Alemana Go (Clínica Alemana, Chile), con historial desde 2018, recetas, órdenes, familiar vinculado y resultados.</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G13" t="n">
@@ -1102,7 +1102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F88"/>
+  <dimension ref="A1:F96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3926,6 +3926,262 @@
       <c r="F88" t="inlineStr">
         <is>
           <t>Búsqueda web (pkg.go.dev panacea-core)</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Apple Health (Health Records)</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Compartición y consentimiento</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Compartir datos con pareja o cuidador (pestaña Sharing)</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Comparte de forma privada datos de salud (actividad, corazón, movilidad) con una persona de confianza, eligiendo qué y con quién.</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>Búsqueda web (HIT/Healthcare IT News); registros clínicos solo EE.UU., Reino Unido y Canadá</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Apple Health (Health Records)</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Medicación y recordatorios</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Medicamentos: listas, horarios y escaneo de etiquetas</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Listas de medicamentos, vitaminas y suplementos con horarios; escaneo de etiqueta del frasco solo en EE.UU.</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>Búsqueda web (MobiHealthNews)</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>ChatGPT Health (OpenAI)</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Interoperabilidad y fuentes de datos</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Conexión de registros con b.well (&gt;2,2 millones de proveedores)</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Acceso a historiales electrónicos de proveedores de EE.UU. vía b.well; solo EE.UU., sin plazo anunciado para Latinoamérica.</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>Búsqueda web (Analytics Insight, HT World)</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Claude for Healthcare (Anthropic)</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Interoperabilidad y fuentes de datos</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Integración con Android Health Connect</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Integración beta con Health Connect en la app móvil; conectores de registros (HealthEx, Function) solo para Pro/Max en EE.UU.</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>Búsqueda web (Fortune, Help Net Security)</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Apps de clínicas (ej. Clínica Alemana de Valdivia)</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Gestión documental</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Notificación de resultados y compartir por email/WhatsApp (Mi Alemana Go)</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Avisa cuando hay exámenes/documentos disponibles; resultados de laboratorio y anatomía patológica compartibles por email o WhatsApp.</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>Ficha App Store Chile (Mi Alemana Go)</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Apps de clínicas (ej. Clínica Alemana de Valdivia)</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Historial y perfil clínico</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Historial de consultas, urgencias y hospitalizaciones desde 2018</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Historial institucional de consultas, urgencias y hospitalizaciones (solo datos de esa clínica).</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>Ficha App Store Chile (Mi Alemana Go)</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Apps de clínicas (ej. Clínica Alemana de Valdivia)</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Gestión documental</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Descarga de recetas, órdenes de examen y derivaciones</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Ver y descargar recetas, órdenes de examen y derivaciones.</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>Ficha App Store Chile (Mi Alemana Go)</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Apps de clínicas (ej. Clínica Alemana de Valdivia)</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Citas y agenda</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Reservar, cancelar y reprogramar horas, exámenes y procedimientos</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Gestión completa de agenda dentro de la institución.</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>Ficha App Store Chile (Mi Alemana Go)</t>
         </is>
       </c>
     </row>
@@ -6850,7 +7106,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:A12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -6933,6 +7189,13 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Vuelta 2 (iter. 3, 2026-10-07 18:08 UTC): Apple Health, ChatGPT Health, Claude for Healthcare, Apps de clínicas revisados (+8 filas). Pendientes: Clinia, MiRedSalud, Mediko.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Benchmark: vuelta 3, iteración 1 (Meedika, Infomed, MediPlanner, Clingot)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MVcXu8vTBu7EKfj3YdEvae
</commit_message>
<xml_diff>
--- a/Outputs/Benchmark_Anamnesis.xlsx
+++ b/Outputs/Benchmark_Anamnesis.xlsx
@@ -513,12 +513,12 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>[DIRECTO · Chile · etapas A+B] Lanzada 25-sep-2024 en App Store (Android previsto la misma semana). &gt;1.500 usuarios en los primeros días; meta 32.000 (cofundador Francisco González). Funciones: gestión de documentos, importar solicitudes, SOS con alergias/medicación, calendario de citas, recordatorios, compartir con profesionales elegidos. Sin blockchain. Precio y estado actual NO verificados; única fuente es una nota de prensa. Sitio oficial por confirmar. [Iter. 2] Hay cobertura adicional en Portal Innova (portalinnova.cl); sitio bloqueado en este entorno, estado actual sigue sin verificar.</t>
+          <t>[DIRECTO · Chile · etapas A+B] Lanzada 25-sep-2024 en App Store (Android previsto la misma semana). &gt;1.500 usuarios en los primeros días; meta 32.000 (cofundador Francisco González). Funciones: gestión de documentos, importar solicitudes, SOS con alergias/medicación, calendario de citas, recordatorios, compartir con profesionales elegidos. Sin blockchain. Precio y estado actual NO verificados; única fuente es una nota de prensa. Sitio oficial por confirmar. [Iter. 2] Hay cobertura adicional en Portal Innova (portalinnova.cl); sitio bloqueado en este entorno, estado actual sigue sin verificar. [Vuelta 3] Sin novedades 2026 ni confirmación de la app Android en Google Play; usuarios actuales desconocidos. Nota de prensa no indica año de lanzamiento explícito.</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G2" t="n">
@@ -553,12 +553,12 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>[DIRECTO · Chile · etapa A] Fundada 2019 por Diego Ibarra, Andrés Fantuzzi y Gabriel Zamora. Lanzada mar-2021 en App Store y Play Store con 1.200 usuarios; planeaba nueva versión jul-2021 y ronda de US$500 mil. Objetivo: llevar el historial en el celular, acceso en emergencias, médico puede ingresar datos con consentimiento. Estado actual NO verificado (posible app inactiva). URL es la nota de prensa; sitio oficial por confirmar.</t>
+          <t>[DIRECTO · Chile · etapa A] Fundada 2019 por Diego Ibarra, Andrés Fantuzzi y Gabriel Zamora. Lanzada mar-2021 en App Store y Play Store con 1.200 usuarios; planeaba nueva versión jul-2021 y ronda de US$500 mil. Objetivo: llevar el historial en el celular, acceso en emergencias, médico puede ingresar datos con consentimiento. Estado actual NO verificado (posible app inactiva). URL es la nota de prensa; sitio oficial por confirmar. [Vuelta 3] Sin evidencia posterior a 2021; relanzamiento previsto jul-2021 no confirmado. Probable app inactiva.</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G3" t="n">
@@ -593,12 +593,12 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>[REGIONAL · México] Historial por perfil familiar, alergias, vacunas, recetas digitales, gráficas de evolución, agendamiento, compartir con profesionales. Gratis en App Store MX. Sin evidencia de uso en Chile. Cubre parte de la etapa C (familia).</t>
+          <t>[REGIONAL · México] Historial por perfil familiar, alergias, vacunas, recetas digitales, gráficas de evolución, agendamiento, compartir con profesionales. Gratis en App Store MX. Sin evidencia de uso en Chile. Cubre parte de la etapa C (familia). [Vuelta 3] Existen dos apps distintas: MediPlanner (gratis, Rym Solutions, MX, 3,7/5 con 3 calificaciones) y MediPlanner Pro (otro desarrollador, $39 MXN). Sin presencia verificada en Chile.</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G4" t="n">
@@ -633,12 +633,12 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>[REGIONAL · Argentina · débil] App para cargar antecedentes médicos propios. Única referencia: nota de opinión en grupoanimal.mx sin fecha verificada. Estado y sitio por confirmar.</t>
+          <t>[REGIONAL · Argentina · débil] App para cargar antecedentes médicos propios. Única referencia: nota de opinión en grupoanimal.mx sin fecha verificada. Estado y sitio por confirmar. [Vuelta 3] Referencias de 2017 (apps4citizens, La Nación); sitio y precio no verificados; puede estar inactiva.</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G5" t="n">
@@ -1102,7 +1102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F99"/>
+  <dimension ref="A1:F102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4278,6 +4278,102 @@
       <c r="F99" t="inlineStr">
         <is>
           <t>Búsqueda web (Chocale, sep-2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Meedika</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Interoperabilidad y fuentes de datos</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Sincronización de resultados desde centros de salud</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Sincroniza resultados desde centros de salud y permite subir fotos o documentos de las solicitudes médicas.</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>Búsqueda web (Diario Estrategia / Europa Press); vuelta 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>MediPlanner</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Interoperabilidad y fuentes de datos</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Importar y exportar información (versión Pro)</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Importar/exportar datos para compartir de forma segura con familias o cuidadores. Es MediPlanner Pro, de otro desarrollador (App Store MX, $39 MXN).</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>Latam</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>Búsqueda web (ficha App Store MX); vuelta 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>MediPlanner</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Citas y agenda</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Integración con el calendario del dispositivo</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Permite añadir las citas a la app Calendario del teléfono (versión Pro).</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>Latam</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>Búsqueda web (ficha App Store MX); vuelta 3</t>
         </is>
       </c>
     </row>
@@ -7112,8 +7208,6 @@
           <t>Búsqueda de profesionales de salud</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
           <t>✓</t>
@@ -7124,17 +7218,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
       <c r="R2">
         <f>COUNTIF(C2:Q2,"✓")</f>
         <v/>
@@ -7156,24 +7239,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
       <c r="R3">
         <f>COUNTIF(C3:Q3,"✓")</f>
         <v/>
@@ -7190,25 +7260,11 @@
           <t>Localización de centros médicos y farmacias</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
       <c r="R4">
         <f>COUNTIF(C4:Q4,"✓")</f>
         <v/>
@@ -7225,25 +7281,11 @@
           <t>Reserva de citas médicas</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr"/>
       <c r="R5">
         <f>COUNTIF(C5:Q5,"✓")</f>
         <v/>
@@ -7260,25 +7302,11 @@
           <t>Acceso del profesional al historial del paciente</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="inlineStr"/>
       <c r="R6">
         <f>COUNTIF(C6:Q6,"✓")</f>
         <v/>
@@ -7295,25 +7323,11 @@
           <t>Compartir con personas sin cuenta mediante clave segura</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr"/>
-      <c r="Q7" t="inlineStr"/>
       <c r="R7">
         <f>COUNTIF(C7:Q7,"✓")</f>
         <v/>
@@ -7330,25 +7344,11 @@
           <t>Compartir datos con cuidador o persona de confianza</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
-      <c r="P8" t="inlineStr"/>
-      <c r="Q8" t="inlineStr"/>
       <c r="R8">
         <f>COUNTIF(C8:Q8,"✓")</f>
         <v/>
@@ -7370,13 +7370,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
           <t>✓</t>
@@ -7402,16 +7400,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
       <c r="O9" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="P9" t="inlineStr"/>
-      <c r="Q9" t="inlineStr"/>
       <c r="R9">
         <f>COUNTIF(C9:Q9,"✓")</f>
         <v/>
@@ -7428,25 +7421,11 @@
           <t>Gestión de consentimiento sobre uso de datos</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
-      <c r="O10" t="inlineStr"/>
-      <c r="P10" t="inlineStr"/>
-      <c r="Q10" t="inlineStr"/>
       <c r="R10">
         <f>COUNTIF(C10:Q10,"✓")</f>
         <v/>
@@ -7463,25 +7442,11 @@
           <t>Ingreso de datos por profesional con consentimiento</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr"/>
-      <c r="P11" t="inlineStr"/>
-      <c r="Q11" t="inlineStr"/>
       <c r="R11">
         <f>COUNTIF(C11:Q11,"✓")</f>
         <v/>
@@ -7498,25 +7463,11 @@
           <t>Red social con profesionales y familiares</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
-      <c r="O12" t="inlineStr"/>
-      <c r="P12" t="inlineStr"/>
-      <c r="Q12" t="inlineStr"/>
       <c r="R12">
         <f>COUNTIF(C12:Q12,"✓")</f>
         <v/>
@@ -7543,23 +7494,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr"/>
-      <c r="O13" t="inlineStr"/>
-      <c r="P13" t="inlineStr"/>
-      <c r="Q13" t="inlineStr"/>
       <c r="R13">
         <f>COUNTIF(C13:Q13,"✓")</f>
         <v/>
@@ -7576,8 +7515,6 @@
           <t>Perfiles familiares / dependientes</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
           <t>✓</t>
@@ -7588,25 +7525,16 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
-      <c r="M14" t="inlineStr"/>
       <c r="N14" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="Q14" t="inlineStr"/>
       <c r="R14">
         <f>COUNTIF(C14:Q14,"✓")</f>
         <v/>
@@ -7628,8 +7556,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
           <t>✓</t>
@@ -7645,19 +7571,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr"/>
-      <c r="N15" t="inlineStr"/>
       <c r="O15" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="P15" t="inlineStr"/>
-      <c r="Q15" t="inlineStr"/>
       <c r="R15">
         <f>COUNTIF(C15:Q15,"✓")</f>
         <v/>
@@ -7674,29 +7592,16 @@
           <t>Almacenamiento de recetas</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
-      <c r="M16" t="inlineStr"/>
       <c r="N16" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="O16" t="inlineStr"/>
-      <c r="P16" t="inlineStr"/>
-      <c r="Q16" t="inlineStr"/>
       <c r="R16">
         <f>COUNTIF(C16:Q16,"✓")</f>
         <v/>
@@ -7713,25 +7618,11 @@
           <t>Búsqueda y filtros de documentos</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr"/>
-      <c r="N17" t="inlineStr"/>
-      <c r="O17" t="inlineStr"/>
-      <c r="P17" t="inlineStr"/>
-      <c r="Q17" t="inlineStr"/>
       <c r="R17">
         <f>COUNTIF(C17:Q17,"✓")</f>
         <v/>
@@ -7753,19 +7644,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr"/>
-      <c r="M18" t="inlineStr"/>
-      <c r="N18" t="inlineStr"/>
-      <c r="O18" t="inlineStr"/>
-      <c r="P18" t="inlineStr"/>
       <c r="Q18" t="inlineStr">
         <is>
           <t>✓</t>
@@ -7787,25 +7665,11 @@
           <t>Notificación y envío de resultados</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr"/>
-      <c r="M19" t="inlineStr"/>
       <c r="N19" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="O19" t="inlineStr"/>
-      <c r="P19" t="inlineStr"/>
-      <c r="Q19" t="inlineStr"/>
       <c r="R19">
         <f>COUNTIF(C19:Q19,"✓")</f>
         <v/>
@@ -7822,29 +7686,16 @@
           <t>Historial institucional (solo datos de la propia red)</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr"/>
-      <c r="M20" t="inlineStr"/>
       <c r="N20" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="O20" t="inlineStr"/>
       <c r="P20" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="Q20" t="inlineStr"/>
       <c r="R20">
         <f>COUNTIF(C20:Q20,"✓")</f>
         <v/>
@@ -7861,36 +7712,26 @@
           <t>Historial médico centralizado</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="L21" t="inlineStr"/>
-      <c r="M21" t="inlineStr"/>
-      <c r="N21" t="inlineStr"/>
-      <c r="O21" t="inlineStr"/>
-      <c r="P21" t="inlineStr"/>
       <c r="Q21" t="inlineStr">
         <is>
           <t>✓</t>
@@ -7912,25 +7753,11 @@
           <t>Línea de tiempo de salud</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
-      <c r="L22" t="inlineStr"/>
-      <c r="M22" t="inlineStr"/>
-      <c r="N22" t="inlineStr"/>
-      <c r="O22" t="inlineStr"/>
-      <c r="P22" t="inlineStr"/>
-      <c r="Q22" t="inlineStr"/>
       <c r="R22">
         <f>COUNTIF(C22:Q22,"✓")</f>
         <v/>
@@ -7947,25 +7774,11 @@
           <t>Registro de alergias y vacunas</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
-      <c r="L23" t="inlineStr"/>
-      <c r="M23" t="inlineStr"/>
-      <c r="N23" t="inlineStr"/>
-      <c r="O23" t="inlineStr"/>
-      <c r="P23" t="inlineStr"/>
-      <c r="Q23" t="inlineStr"/>
       <c r="R23">
         <f>COUNTIF(C23:Q23,"✓")</f>
         <v/>
@@ -7982,25 +7795,11 @@
           <t>Recompensas / monetización de datos del usuario</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
-      <c r="L24" t="inlineStr"/>
-      <c r="M24" t="inlineStr"/>
-      <c r="N24" t="inlineStr"/>
-      <c r="O24" t="inlineStr"/>
-      <c r="P24" t="inlineStr"/>
-      <c r="Q24" t="inlineStr"/>
       <c r="R24">
         <f>COUNTIF(C24:Q24,"✓")</f>
         <v/>
@@ -8017,25 +7816,11 @@
           <t>Coaching de salud con IA</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr"/>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr"/>
-      <c r="L25" t="inlineStr"/>
-      <c r="M25" t="inlineStr"/>
-      <c r="N25" t="inlineStr"/>
-      <c r="O25" t="inlineStr"/>
-      <c r="P25" t="inlineStr"/>
-      <c r="Q25" t="inlineStr"/>
       <c r="R25">
         <f>COUNTIF(C25:Q25,"✓")</f>
         <v/>
@@ -8052,25 +7837,11 @@
           <t>Detección de patrones en métricas de salud con IA</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr"/>
-      <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr"/>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
-      <c r="L26" t="inlineStr"/>
       <c r="M26" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="N26" t="inlineStr"/>
-      <c r="O26" t="inlineStr"/>
-      <c r="P26" t="inlineStr"/>
-      <c r="Q26" t="inlineStr"/>
       <c r="R26">
         <f>COUNTIF(C26:Q26,"✓")</f>
         <v/>
@@ -8087,15 +7858,6 @@
           <t>Interpretación de exámenes con IA</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr"/>
-      <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr"/>
-      <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr">
         <is>
           <t>✓</t>
@@ -8106,9 +7868,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="N27" t="inlineStr"/>
-      <c r="O27" t="inlineStr"/>
-      <c r="P27" t="inlineStr"/>
       <c r="Q27" t="inlineStr">
         <is>
           <t>✓</t>
@@ -8130,20 +7889,6 @@
           <t>Orientación médica con IA</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr"/>
-      <c r="M28" t="inlineStr"/>
-      <c r="N28" t="inlineStr"/>
-      <c r="O28" t="inlineStr"/>
-      <c r="P28" t="inlineStr"/>
       <c r="Q28" t="inlineStr">
         <is>
           <t>✓</t>
@@ -8165,15 +7910,6 @@
           <t>Preparación de consultas médicas con IA</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr"/>
-      <c r="D29" t="inlineStr"/>
-      <c r="E29" t="inlineStr"/>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr"/>
-      <c r="H29" t="inlineStr"/>
-      <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr">
         <is>
           <t>✓</t>
@@ -8184,10 +7920,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="N29" t="inlineStr"/>
-      <c r="O29" t="inlineStr"/>
-      <c r="P29" t="inlineStr"/>
-      <c r="Q29" t="inlineStr"/>
       <c r="R29">
         <f>COUNTIF(C29:Q29,"✓")</f>
         <v/>
@@ -8204,15 +7936,6 @@
           <t>Resumen de historial con IA</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr"/>
-      <c r="E30" t="inlineStr"/>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr"/>
-      <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr">
         <is>
           <t>✓</t>
@@ -8223,10 +7946,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="N30" t="inlineStr"/>
-      <c r="O30" t="inlineStr"/>
-      <c r="P30" t="inlineStr"/>
-      <c r="Q30" t="inlineStr"/>
       <c r="R30">
         <f>COUNTIF(C30:Q30,"✓")</f>
         <v/>
@@ -8243,18 +7962,11 @@
           <t>Agregación de registros de múltiples instituciones</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr"/>
-      <c r="D31" t="inlineStr"/>
-      <c r="E31" t="inlineStr"/>
-      <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr"/>
       <c r="K31" t="inlineStr">
         <is>
           <t>✓</t>
@@ -8270,14 +7982,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="N31" t="inlineStr"/>
       <c r="O31" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="P31" t="inlineStr"/>
-      <c r="Q31" t="inlineStr"/>
       <c r="R31">
         <f>COUNTIF(C31:Q31,"✓")</f>
         <v/>
@@ -8294,25 +8003,11 @@
           <t>Analítica poblacional B2B</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr"/>
-      <c r="D32" t="inlineStr"/>
-      <c r="E32" t="inlineStr"/>
-      <c r="F32" t="inlineStr"/>
-      <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr"/>
-      <c r="K32" t="inlineStr"/>
-      <c r="L32" t="inlineStr"/>
-      <c r="M32" t="inlineStr"/>
-      <c r="N32" t="inlineStr"/>
-      <c r="O32" t="inlineStr"/>
-      <c r="P32" t="inlineStr"/>
-      <c r="Q32" t="inlineStr"/>
       <c r="R32">
         <f>COUNTIF(C32:Q32,"✓")</f>
         <v/>
@@ -8329,9 +8024,6 @@
           <t>Disponibilidad multiplataforma (web/iOS/Android)</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr"/>
-      <c r="D33" t="inlineStr"/>
-      <c r="E33" t="inlineStr"/>
       <c r="F33" t="inlineStr">
         <is>
           <t>✓</t>
@@ -8342,20 +8034,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr"/>
-      <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr"/>
-      <c r="K33" t="inlineStr"/>
-      <c r="L33" t="inlineStr"/>
-      <c r="M33" t="inlineStr"/>
-      <c r="N33" t="inlineStr"/>
       <c r="O33" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="P33" t="inlineStr"/>
-      <c r="Q33" t="inlineStr"/>
       <c r="R33">
         <f>COUNTIF(C33:Q33,"✓")</f>
         <v/>
@@ -8372,25 +8055,11 @@
           <t>Historial médico centralizado</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr"/>
-      <c r="D34" t="inlineStr"/>
-      <c r="E34" t="inlineStr"/>
-      <c r="F34" t="inlineStr"/>
-      <c r="G34" t="inlineStr"/>
-      <c r="H34" t="inlineStr"/>
-      <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="K34" t="inlineStr"/>
-      <c r="L34" t="inlineStr"/>
-      <c r="M34" t="inlineStr"/>
-      <c r="N34" t="inlineStr"/>
-      <c r="O34" t="inlineStr"/>
-      <c r="P34" t="inlineStr"/>
-      <c r="Q34" t="inlineStr"/>
       <c r="R34">
         <f>COUNTIF(C34:Q34,"✓")</f>
         <v/>
@@ -8407,29 +8076,16 @@
           <t>Integración con wearables y apps de salud</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr"/>
-      <c r="D35" t="inlineStr"/>
-      <c r="E35" t="inlineStr"/>
-      <c r="F35" t="inlineStr"/>
-      <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr"/>
-      <c r="K35" t="inlineStr"/>
-      <c r="L35" t="inlineStr"/>
       <c r="M35" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="N35" t="inlineStr"/>
-      <c r="O35" t="inlineStr"/>
-      <c r="P35" t="inlineStr"/>
-      <c r="Q35" t="inlineStr"/>
       <c r="R35">
         <f>COUNTIF(C35:Q35,"✓")</f>
         <v/>
@@ -8446,25 +8102,11 @@
           <t>Gestión de lista de medicamentos</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr"/>
-      <c r="D36" t="inlineStr"/>
-      <c r="E36" t="inlineStr"/>
-      <c r="F36" t="inlineStr"/>
-      <c r="G36" t="inlineStr"/>
-      <c r="H36" t="inlineStr"/>
-      <c r="I36" t="inlineStr"/>
-      <c r="J36" t="inlineStr"/>
       <c r="K36" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="L36" t="inlineStr"/>
-      <c r="M36" t="inlineStr"/>
-      <c r="N36" t="inlineStr"/>
-      <c r="O36" t="inlineStr"/>
-      <c r="P36" t="inlineStr"/>
-      <c r="Q36" t="inlineStr"/>
       <c r="R36">
         <f>COUNTIF(C36:Q36,"✓")</f>
         <v/>
@@ -8486,24 +8128,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr"/>
-      <c r="E37" t="inlineStr"/>
-      <c r="F37" t="inlineStr"/>
-      <c r="G37" t="inlineStr"/>
-      <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr"/>
-      <c r="J37" t="inlineStr"/>
       <c r="K37" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="L37" t="inlineStr"/>
-      <c r="M37" t="inlineStr"/>
-      <c r="N37" t="inlineStr"/>
-      <c r="O37" t="inlineStr"/>
-      <c r="P37" t="inlineStr"/>
-      <c r="Q37" t="inlineStr"/>
       <c r="R37">
         <f>COUNTIF(C37:Q37,"✓")</f>
         <v/>
@@ -8520,25 +8149,11 @@
           <t>Registro de tomas y adherencia al tratamiento</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr"/>
-      <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr"/>
-      <c r="G38" t="inlineStr"/>
-      <c r="H38" t="inlineStr"/>
-      <c r="I38" t="inlineStr"/>
-      <c r="J38" t="inlineStr"/>
-      <c r="K38" t="inlineStr"/>
-      <c r="L38" t="inlineStr"/>
-      <c r="M38" t="inlineStr"/>
-      <c r="N38" t="inlineStr"/>
-      <c r="O38" t="inlineStr"/>
-      <c r="P38" t="inlineStr"/>
-      <c r="Q38" t="inlineStr"/>
       <c r="R38">
         <f>COUNTIF(C38:Q38,"✓")</f>
         <v/>
@@ -8555,25 +8170,11 @@
           <t>Contenido educativo sobre salud</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr"/>
-      <c r="F39" t="inlineStr"/>
-      <c r="G39" t="inlineStr"/>
-      <c r="H39" t="inlineStr"/>
-      <c r="I39" t="inlineStr"/>
-      <c r="J39" t="inlineStr"/>
-      <c r="K39" t="inlineStr"/>
-      <c r="L39" t="inlineStr"/>
-      <c r="M39" t="inlineStr"/>
-      <c r="N39" t="inlineStr"/>
-      <c r="O39" t="inlineStr"/>
-      <c r="P39" t="inlineStr"/>
-      <c r="Q39" t="inlineStr"/>
       <c r="R39">
         <f>COUNTIF(C39:Q39,"✓")</f>
         <v/>
@@ -8590,25 +8191,11 @@
           <t>Gráficas de evolución de indicadores</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr"/>
-      <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr"/>
-      <c r="G40" t="inlineStr"/>
-      <c r="H40" t="inlineStr"/>
-      <c r="I40" t="inlineStr"/>
-      <c r="J40" t="inlineStr"/>
-      <c r="K40" t="inlineStr"/>
-      <c r="L40" t="inlineStr"/>
-      <c r="M40" t="inlineStr"/>
-      <c r="N40" t="inlineStr"/>
-      <c r="O40" t="inlineStr"/>
-      <c r="P40" t="inlineStr"/>
-      <c r="Q40" t="inlineStr"/>
       <c r="R40">
         <f>COUNTIF(C40:Q40,"✓")</f>
         <v/>
@@ -8625,25 +8212,11 @@
           <t>Integración con wearables y apps de salud</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr"/>
-      <c r="D41" t="inlineStr"/>
-      <c r="E41" t="inlineStr"/>
-      <c r="F41" t="inlineStr"/>
-      <c r="G41" t="inlineStr"/>
-      <c r="H41" t="inlineStr"/>
-      <c r="I41" t="inlineStr"/>
-      <c r="J41" t="inlineStr"/>
       <c r="K41" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="L41" t="inlineStr"/>
-      <c r="M41" t="inlineStr"/>
-      <c r="N41" t="inlineStr"/>
-      <c r="O41" t="inlineStr"/>
-      <c r="P41" t="inlineStr"/>
-      <c r="Q41" t="inlineStr"/>
       <c r="R41">
         <f>COUNTIF(C41:Q41,"✓")</f>
         <v/>
@@ -8660,25 +8233,11 @@
           <t>Panel de seguimiento de salud y bienestar</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr"/>
-      <c r="D42" t="inlineStr"/>
-      <c r="E42" t="inlineStr"/>
-      <c r="F42" t="inlineStr"/>
-      <c r="G42" t="inlineStr"/>
       <c r="H42" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="I42" t="inlineStr"/>
-      <c r="J42" t="inlineStr"/>
-      <c r="K42" t="inlineStr"/>
-      <c r="L42" t="inlineStr"/>
-      <c r="M42" t="inlineStr"/>
-      <c r="N42" t="inlineStr"/>
-      <c r="O42" t="inlineStr"/>
-      <c r="P42" t="inlineStr"/>
-      <c r="Q42" t="inlineStr"/>
       <c r="R42">
         <f>COUNTIF(C42:Q42,"✓")</f>
         <v/>
@@ -8695,25 +8254,11 @@
           <t>Valoración de profesionales</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr"/>
-      <c r="D43" t="inlineStr"/>
-      <c r="E43" t="inlineStr"/>
       <c r="F43" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="G43" t="inlineStr"/>
-      <c r="H43" t="inlineStr"/>
-      <c r="I43" t="inlineStr"/>
-      <c r="J43" t="inlineStr"/>
-      <c r="K43" t="inlineStr"/>
-      <c r="L43" t="inlineStr"/>
-      <c r="M43" t="inlineStr"/>
-      <c r="N43" t="inlineStr"/>
-      <c r="O43" t="inlineStr"/>
-      <c r="P43" t="inlineStr"/>
-      <c r="Q43" t="inlineStr"/>
       <c r="R43">
         <f>COUNTIF(C43:Q43,"✓")</f>
         <v/>
@@ -8730,11 +8275,6 @@
           <t>Blockchain para integridad y trazabilidad de datos</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr"/>
-      <c r="D44" t="inlineStr"/>
-      <c r="E44" t="inlineStr"/>
-      <c r="F44" t="inlineStr"/>
-      <c r="G44" t="inlineStr"/>
       <c r="H44" t="inlineStr">
         <is>
           <t>✓</t>
@@ -8750,13 +8290,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="K44" t="inlineStr"/>
-      <c r="L44" t="inlineStr"/>
-      <c r="M44" t="inlineStr"/>
-      <c r="N44" t="inlineStr"/>
-      <c r="O44" t="inlineStr"/>
-      <c r="P44" t="inlineStr"/>
-      <c r="Q44" t="inlineStr"/>
       <c r="R44">
         <f>COUNTIF(C44:Q44,"✓")</f>
         <v/>
@@ -8773,29 +8306,16 @@
           <t>Cifrado y control de acceso</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr"/>
       <c r="D45" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr"/>
-      <c r="F45" t="inlineStr"/>
-      <c r="G45" t="inlineStr"/>
-      <c r="H45" t="inlineStr"/>
-      <c r="I45" t="inlineStr"/>
-      <c r="J45" t="inlineStr"/>
       <c r="K45" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="L45" t="inlineStr"/>
-      <c r="M45" t="inlineStr"/>
-      <c r="N45" t="inlineStr"/>
-      <c r="O45" t="inlineStr"/>
-      <c r="P45" t="inlineStr"/>
-      <c r="Q45" t="inlineStr"/>
       <c r="R45">
         <f>COUNTIF(C45:Q45,"✓")</f>
         <v/>
@@ -8812,25 +8332,11 @@
           <t>Identidad descentralizada (DID)</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr"/>
-      <c r="D46" t="inlineStr"/>
-      <c r="E46" t="inlineStr"/>
-      <c r="F46" t="inlineStr"/>
-      <c r="G46" t="inlineStr"/>
-      <c r="H46" t="inlineStr"/>
       <c r="I46" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="J46" t="inlineStr"/>
-      <c r="K46" t="inlineStr"/>
-      <c r="L46" t="inlineStr"/>
-      <c r="M46" t="inlineStr"/>
-      <c r="N46" t="inlineStr"/>
-      <c r="O46" t="inlineStr"/>
-      <c r="P46" t="inlineStr"/>
-      <c r="Q46" t="inlineStr"/>
       <c r="R46">
         <f>COUNTIF(C46:Q46,"✓")</f>
         <v/>
@@ -8847,25 +8353,11 @@
           <t>Privacidad reforzada para datos de salud</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr"/>
-      <c r="D47" t="inlineStr"/>
-      <c r="E47" t="inlineStr"/>
-      <c r="F47" t="inlineStr"/>
-      <c r="G47" t="inlineStr"/>
-      <c r="H47" t="inlineStr"/>
-      <c r="I47" t="inlineStr"/>
-      <c r="J47" t="inlineStr"/>
-      <c r="K47" t="inlineStr"/>
       <c r="L47" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="M47" t="inlineStr"/>
-      <c r="N47" t="inlineStr"/>
-      <c r="O47" t="inlineStr"/>
-      <c r="P47" t="inlineStr"/>
-      <c r="Q47" t="inlineStr"/>
       <c r="R47">
         <f>COUNTIF(C47:Q47,"✓")</f>
         <v/>
@@ -8882,20 +8374,6 @@
           <t>Modelo freemium y suscripción</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr"/>
-      <c r="D48" t="inlineStr"/>
-      <c r="E48" t="inlineStr"/>
-      <c r="F48" t="inlineStr"/>
-      <c r="G48" t="inlineStr"/>
-      <c r="H48" t="inlineStr"/>
-      <c r="I48" t="inlineStr"/>
-      <c r="J48" t="inlineStr"/>
-      <c r="K48" t="inlineStr"/>
-      <c r="L48" t="inlineStr"/>
-      <c r="M48" t="inlineStr"/>
-      <c r="N48" t="inlineStr"/>
-      <c r="O48" t="inlineStr"/>
-      <c r="P48" t="inlineStr"/>
       <c r="Q48" t="inlineStr">
         <is>
           <t>✓</t>
@@ -8917,25 +8395,11 @@
           <t>Pagos con criptomoneda</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr"/>
-      <c r="D49" t="inlineStr"/>
-      <c r="E49" t="inlineStr"/>
-      <c r="F49" t="inlineStr"/>
-      <c r="G49" t="inlineStr"/>
-      <c r="H49" t="inlineStr"/>
-      <c r="I49" t="inlineStr"/>
       <c r="J49" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="K49" t="inlineStr"/>
-      <c r="L49" t="inlineStr"/>
-      <c r="M49" t="inlineStr"/>
-      <c r="N49" t="inlineStr"/>
-      <c r="O49" t="inlineStr"/>
-      <c r="P49" t="inlineStr"/>
-      <c r="Q49" t="inlineStr"/>
       <c r="R49">
         <f>COUNTIF(C49:Q49,"✓")</f>
         <v/>
@@ -8952,25 +8416,11 @@
           <t>Reclamos y trámites con seguros</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr"/>
-      <c r="D50" t="inlineStr"/>
-      <c r="E50" t="inlineStr"/>
-      <c r="F50" t="inlineStr"/>
-      <c r="G50" t="inlineStr"/>
-      <c r="H50" t="inlineStr"/>
       <c r="I50" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="J50" t="inlineStr"/>
-      <c r="K50" t="inlineStr"/>
-      <c r="L50" t="inlineStr"/>
-      <c r="M50" t="inlineStr"/>
-      <c r="N50" t="inlineStr"/>
-      <c r="O50" t="inlineStr"/>
-      <c r="P50" t="inlineStr"/>
-      <c r="Q50" t="inlineStr"/>
       <c r="R50">
         <f>COUNTIF(C50:Q50,"✓")</f>
         <v/>
@@ -8987,25 +8437,11 @@
           <t>Teleconsulta con profesionales</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr"/>
-      <c r="D51" t="inlineStr"/>
-      <c r="E51" t="inlineStr"/>
-      <c r="F51" t="inlineStr"/>
-      <c r="G51" t="inlineStr"/>
-      <c r="H51" t="inlineStr"/>
-      <c r="I51" t="inlineStr"/>
       <c r="J51" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="K51" t="inlineStr"/>
-      <c r="L51" t="inlineStr"/>
-      <c r="M51" t="inlineStr"/>
-      <c r="N51" t="inlineStr"/>
-      <c r="O51" t="inlineStr"/>
-      <c r="P51" t="inlineStr"/>
-      <c r="Q51" t="inlineStr"/>
       <c r="R51">
         <f>COUNTIF(C51:Q51,"✓")</f>
         <v/>
@@ -9022,7 +8458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -9119,6 +8555,13 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Vuelta 3 (iter. 1, 2026-10-07 22:08 UTC): Meedika, Infomed, MediPlanner, Clingot verificados (+3 filas). Pendientes: Healfies, Patientory, MediBloc, Medicalchain, etc. Las filas nuevas aún no están en func_norm/tabla_frecuencia (se regeneran al cerrar la vuelta).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Benchmark: vuelta 3, iteración 2 (Healfies, Patientory, MediBloc, Medicalchain)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MVcXu8vTBu7EKfj3YdEvae
</commit_message>
<xml_diff>
--- a/Outputs/Benchmark_Anamnesis.xlsx
+++ b/Outputs/Benchmark_Anamnesis.xlsx
@@ -673,12 +673,12 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>[REGIONAL · Brasil] Fundada ene-2015 en Florianópolis por Helyson Lewis Velasco. Centraliza registros de salud personales: carpetas, etiquetas, línea de tiempo (medicación, exámenes, citas, dieta), compartir con familia o profesionales. Gratis; web, iOS y Android. Estado actual NO verificado (fuentes de 2015-2016). Referencia funcional cercana a etapas A+B. [Vuelta 2] Lanzada simultáneamente en Brasil, Argentina y EE.UU.; permite compartir con no registrados vía clave por email. Sin novedades posteriores a 2016.</t>
+          <t>[REGIONAL · Brasil] Fundada ene-2015 en Florianópolis por Helyson Lewis Velasco. Centraliza registros de salud personales: carpetas, etiquetas, línea de tiempo (medicación, exámenes, citas, dieta), compartir con familia o profesionales. Gratis; web, iOS y Android. Estado actual NO verificado (fuentes de 2015-2016). Referencia funcional cercana a etapas A+B. [Vuelta 2] Lanzada simultáneamente en Brasil, Argentina y EE.UU.; permite compartir con no registrados vía clave por email. Sin novedades posteriores a 2016. [Vuelta 3] Sin evidencia de actividad reciente ni de cierre; Gust/Dealroom la listan en Florianópolis (10 empleados, healfies.com) sin fecha de actualización. Estado sin confirmar.</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G6" t="n">
@@ -686,7 +686,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -713,12 +713,12 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>[BLOCKCHAIN · EE.UU.] Atlanta, fundada 2015, ~9 empleados. Levantó US$7,2M vía financiamiento cripto. App con registros de hospitales y wearables, coaching de salud con IA y recompensas en cripto; también dashboard empresarial Neith. PitchBook indica actividad y financiamiento hasta abr-2026: sigue operando. Sin presencia conocida en Chile. Referencia directa para la hipótesis blockchain. [Vuelta 2] Sin noticias 2026 encontradas en búsqueda; sitio oficial bloqueado.</t>
+          <t>[BLOCKCHAIN · EE.UU.] Atlanta, fundada 2015, ~9 empleados. Levantó US$7,2M vía financiamiento cripto. App con registros de hospitales y wearables, coaching de salud con IA y recompensas en cripto; también dashboard empresarial Neith. PitchBook indica actividad y financiamiento hasta abr-2026: sigue operando. Sin presencia conocida en Chile. Referencia directa para la hipótesis blockchain. [Vuelta 2] Sin noticias 2026 encontradas en búsqueda; sitio oficial bloqueado. [Vuelta 3] Búsqueda adicional solo devuelve hitos de 2017 (token sale US$7,2M) y 2019 (Serie A de US$5,3M, cierre no confirmado); sin datos 2025-26 propios.</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G7" t="n">
@@ -726,7 +726,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -753,12 +753,12 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>[BLOCKCHAIN · Corea del Sur] Fundada 2017, Seúl. Blockchain propia Panacea (Cosmos SDK, mainnet 2019) para que el paciente gestione y transfiera sus registros; app Medipass para seguros. Serie A de ₩4.000 millones (Naver); alianzas con hospitales (Seoul National, Severance). Estado 2025-26 NO verificado. Referencia sobre seguros + blockchain. [Vuelta 2] Panacea incluye DID, Append Only Log, IBC y PNFT; sin anuncios 2026 localizados.</t>
+          <t>[BLOCKCHAIN · Corea del Sur] Fundada 2017, Seúl. Blockchain propia Panacea (Cosmos SDK, mainnet 2019) para que el paciente gestione y transfiera sus registros; app Medipass para seguros. Serie A de ₩4.000 millones (Naver); alianzas con hospitales (Seoul National, Severance). Estado 2025-26 NO verificado. Referencia sobre seguros + blockchain. [Vuelta 2] Panacea incluye DID, Append Only Log, IBC y PNFT; sin anuncios 2026 localizados. [Vuelta 3] Medipass: app en Corea con 20 hospitales/aseguradoras integrados (fecha de la lista desconocida) y plan 2022 de superapp con marketplace de datos; operación actual sin confirmar.</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G8" t="n">
@@ -766,7 +766,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -793,12 +793,12 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>[BLOCKCHAIN · Reino Unido · INACTIVO] Londres, 2017, Ethereum, con telemedicina. Piloto según registro de la UE (2020). Tracxn/PitchBook lo marcan fuera de operación (ago-2025). Solo caso de aprendizaje: no cuenta como competidor activo. [Vuelta 2] Token MTN deslistado de Bitfinex el 26-mar-2021; sin hallazgos de actividad posterior.</t>
+          <t>[BLOCKCHAIN · Reino Unido · INACTIVO] Londres, 2017, Ethereum, con telemedicina. Piloto según registro de la UE (2020). Tracxn/PitchBook lo marcan fuera de operación (ago-2025). Solo caso de aprendizaje: no cuenta como competidor activo. [Vuelta 2] Token MTN deslistado de Bitfinex el 26-mar-2021; sin hallazgos de actividad posterior. [Vuelta 3] Seedtable la marca activa sin fuente; no hallé registro en Companies House. Sigue tratándose como caso de aprendizaje.</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G9" t="n">
@@ -806,7 +806,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -1102,7 +1102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F102"/>
+  <dimension ref="A1:F106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4374,6 +4374,134 @@
       <c r="F102" t="inlineStr">
         <is>
           <t>Búsqueda web (ficha App Store MX); vuelta 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>MediBloc</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Interoperabilidad y fuentes de datos</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Consulta de historial de hospitales conectados (3 años)</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Tras autenticación simple, trae los últimos 3 años de historial de hospitales integrados (p. ej. Samsung Seoul, SNUH, Severance).</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>Búsqueda web (Dealsite, Blockmedia, ficha App Store Corea); app Medipass</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>MediBloc</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Seguros y pagos</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Reclamación de seguro desde el móvil en segundos</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Reclamo de seguro médico (indemnización) desde la app, con verificación de autenticidad de los registros vía blockchain por la aseguradora.</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>Búsqueda web (Blockmedia 2019)</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>MediBloc</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Gestión documental</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Emisión de certificados y consulta de chequeos</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>La ficha de la app incluye consulta de chequeos de salud y emisión de certificados médicos.</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>Búsqueda web (ficha App Store Corea)</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>MediBloc</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Incentivos y monetización de datos</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Marketplace de datos (planificado 2022)</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>Plan de convertir Medipass en superapp con gestión de salud diaria y mercado de datos, integrada con la EMR Dr.Palette.</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>Búsqueda web (Dealsite 2022); sin confirmación de ejecución</t>
         </is>
       </c>
     </row>
@@ -8458,7 +8586,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A14"/>
+  <dimension ref="A1:A15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -8562,6 +8690,13 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Vuelta 3 (iter. 2, 2026-10-08 00:08 UTC): Healfies, Patientory, MediBloc, Medicalchain verificados (+4 filas, todas de MediBloc). Pendientes: Apple Health, ChatGPT Health, Claude for Healthcare, Apps de clínicas, Clinia, MiRedSalud, Mediko.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Benchmark: vuelta 3, iteración 3 (Apple Health, ChatGPT Health, Claude for Healthcare, Apps de clínicas)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MVcXu8vTBu7EKfj3YdEvae
</commit_message>
<xml_diff>
--- a/Outputs/Benchmark_Anamnesis.xlsx
+++ b/Outputs/Benchmark_Anamnesis.xlsx
@@ -833,12 +833,12 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>[ADYACENTE · global] Agrega registros clínicos vía FHIR; &gt;500 instituciones conectadas en EE.UU. (2018). Sin evidencia de disponibilidad en Chile. Incluida en el dispositivo. Amenaza si FHIR/IPS-CL se adopta en Chile. [Vuelta 2] Sin disponibilidad de registros clínicos en Chile (solo EE.UU., Reino Unido, Canadá).</t>
+          <t>[ADYACENTE · global] Agrega registros clínicos vía FHIR; &gt;500 instituciones conectadas en EE.UU. (2018). Sin evidencia de disponibilidad en Chile. Incluida en el dispositivo. Amenaza si FHIR/IPS-CL se adopta en Chile. [Vuelta 2] Sin disponibilidad de registros clínicos en Chile (solo EE.UU., Reino Unido, Canadá). [Vuelta 3] iOS 27 (WWDC 8-jun-2026; publicado ~14-sep-2026): rediseño del app Health, menopausia, nutrición por cámara. El coach de salud con IA no se anunció. Sin ampliación de Health Records a Chile.</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G10" t="n">
@@ -846,7 +846,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -873,12 +873,12 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>[ADYACENTE · global] Lanzado 7-ene-2026. Conecta registros médicos; conectores solo en EE.UU. Dentro de suscripción del asistente. Fija la expectativa de consultar y resumir el historial. [Vuelta 2] Confirmado: registros solo EE.UU.; sin anuncios para Latinoamérica. Hay inconsistencia de fechas entre fuentes (7-ene-2026 lanzamiento vs. jul-2026 despliegue de registros).</t>
+          <t>[ADYACENTE · global] Lanzado 7-ene-2026. Conecta registros médicos; conectores solo en EE.UU. Dentro de suscripción del asistente. Fija la expectativa de consultar y resumir el historial. [Vuelta 2] Confirmado: registros solo EE.UU.; sin anuncios para Latinoamérica. Hay inconsistencia de fechas entre fuentes (7-ene-2026 lanzamiento vs. jul-2026 despliegue de registros). [Vuelta 3] Fechas aclaradas: presentación 7-ene-2026 (acceso limitado); despliegue de Health in ChatGPT con Apple Health y registros en EE.UU. el 23-jul-2026; mejora de salud jun-2026. Sin anuncios para Latinoamérica ni para sep-oct 2026.</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G11" t="n">
@@ -886,7 +886,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -913,12 +913,12 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>[ADYACENTE · global] Lanzado 11-ene-2026. Conectores solo en EE.UU., planes Pro/Max. Nota: producto de Anthropic, conflicto de interés al evaluarlo. [Vuelta 2] Sin cambios fuera de EE.UU. (HealthEx y Function para Pro/Max).</t>
+          <t>[ADYACENTE · global] Lanzado 11-ene-2026. Conectores solo en EE.UU., planes Pro/Max. Nota: producto de Anthropic, conflicto de interés al evaluarlo. [Vuelta 2] Sin cambios fuera de EE.UU. (HealthEx y Function para Pro/Max). [Vuelta 3] Sin anuncios posteriores a enero de 2026. Hoja de ruta de HealthEx (agendar, buscar prestadores, recetas) sin confirmar como lanzada.</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G12" t="n">
@@ -926,7 +926,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -953,12 +953,12 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>[SUSTITUTO PARCIAL · Chile] Reservar hora, ver historial de esa institución, vincular familiar. Gratis; no consolida datos de otras instituciones. [Vuelta 2] App concreta: Mi Alemana Go (Clínica Alemana, Chile), con historial desde 2018, recetas, órdenes, familiar vinculado y resultados.</t>
+          <t>[SUSTITUTO PARCIAL · Chile] Reservar hora, ver historial de esa institución, vincular familiar. Gratis; no consolida datos de otras instituciones. [Vuelta 2] App concreta: Mi Alemana Go (Clínica Alemana, Chile), con historial desde 2018, recetas, órdenes, familiar vinculado y resultados. [Vuelta 3] Búsqueda de otras clínicas (Las Condes, Santa María, UC Christus) sin ficha de app confirmada; solo canales digitales genéricos.</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G13" t="n">
@@ -966,7 +966,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -1102,7 +1102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F106"/>
+  <dimension ref="A1:F112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4502,6 +4502,198 @@
       <c r="F106" t="inlineStr">
         <is>
           <t>Búsqueda web (Dealsite 2022); sin confirmación de ejecución</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Apple Health (Health Records)</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Seguimiento y bienestar</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Seguimiento de perimenopausia y menopausia (iOS 27)</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Extiende el seguimiento de ciclo con perimenopausia y menopausia.</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>Búsqueda web (MacRumors, Sahha, Macwelt); iOS 27 publicado 14-sep-2026 según un reporte</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Apple Health (Health Records)</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Seguimiento y bienestar</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Registro de nutrición con cámara (iOS 27)</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Escaneo de etiquetas nutricionales con la cámara; según un análisis, no escribe en HealthKit.</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>Búsqueda web (MacRumors, Sahha)</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>ChatGPT Health (OpenAI)</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Interoperabilidad y fuentes de datos</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Conectores a One Medical y Function Health</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Además de b.well y Apple Health, vincula registros de One Medical y Function Health (solo EE.UU., Free/Go/Plus/Pro, web e iOS).</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>Búsqueda web (IT Brief, OpenAI); lanzamiento EE.UU. 23-jul-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>ChatGPT Health (OpenAI)</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Inteligencia artificial</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Detección de cambios en contexto de datos conectados</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Interpreta datos de Apple Health y registros en contexto y detecta cambios.</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>Búsqueda web (OpenAI, IT Brief)</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>ChatGPT Health (OpenAI)</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Inteligencia artificial</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Reconocimiento de urgencia y explicación de incertidumbre</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>Mejora de jun-2026 (GPT-5.5 Instant): detecta cuándo puede requerirse atención urgente, pide contexto y explica la incertidumbre.</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>Búsqueda web (OpenAI, jun-2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Claude for Healthcare (Anthropic)</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Seguridad, privacidad y blockchain</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Permisos opt-in y revocables; datos fuera de memoria y entrenamiento</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>El usuario activa y revoca permisos; los datos de salud compartidos se excluyen de la memoria de Claude y del entrenamiento.</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>Búsqueda web (Help Net Security, NBC News)</t>
         </is>
       </c>
     </row>
@@ -8586,7 +8778,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A15"/>
+  <dimension ref="A1:A16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -8697,6 +8889,13 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Vuelta 3 (iter. 3, 2026-10-08 02:08 UTC): Apple Health, ChatGPT Health, Claude for Healthcare, Apps de clínicas verificados (+6 filas). Aclarada discrepancia de fechas de ChatGPT Health. Pendientes: Clinia, MiRedSalud, Mediko (cierran la vuelta 3).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Benchmark: vuelta 4, iteración 1 (Meedika, Infomed, MediPlanner, Clingot)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MVcXu8vTBu7EKfj3YdEvae
</commit_message>
<xml_diff>
--- a/Outputs/Benchmark_Anamnesis.xlsx
+++ b/Outputs/Benchmark_Anamnesis.xlsx
@@ -513,12 +513,12 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>[DIRECTO · Chile · etapas A+B] Lanzada 25-sep-2024 en App Store (Android previsto la misma semana). &gt;1.500 usuarios en los primeros días; meta 32.000 (cofundador Francisco González). Funciones: gestión de documentos, importar solicitudes, SOS con alergias/medicación, calendario de citas, recordatorios, compartir con profesionales elegidos. Sin blockchain. Precio y estado actual NO verificados; única fuente es una nota de prensa. Sitio oficial por confirmar. [Iter. 2] Hay cobertura adicional en Portal Innova (portalinnova.cl); sitio bloqueado en este entorno, estado actual sigue sin verificar. [Vuelta 3] Sin novedades 2026 ni confirmación de la app Android en Google Play; usuarios actuales desconocidos. Nota de prensa no indica año de lanzamiento explícito.</t>
+          <t>[DIRECTO · Chile · etapas A+B] Lanzada 25-sep-2024 en App Store (Android previsto la misma semana). &gt;1.500 usuarios en los primeros días; meta 32.000 (cofundador Francisco González). Funciones: gestión de documentos, importar solicitudes, SOS con alergias/medicación, calendario de citas, recordatorios, compartir con profesionales elegidos. Sin blockchain. Precio y estado actual NO verificados; única fuente es una nota de prensa. Sitio oficial por confirmar. [Iter. 2] Hay cobertura adicional en Portal Innova (portalinnova.cl); sitio bloqueado en este entorno, estado actual sigue sin verificar. [Vuelta 3] Sin novedades 2026 ni confirmación de la app Android en Google Play; usuarios actuales desconocidos. Nota de prensa no indica año de lanzamiento explícito. [Vuelta 4] Sin fuentes nuevas; portalinnova.cl no aparece en búsquedas. Sigue dependiendo de una sola nota de prensa.</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G2" t="n">
@@ -553,12 +553,12 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>[DIRECTO · Chile · etapa A] Fundada 2019 por Diego Ibarra, Andrés Fantuzzi y Gabriel Zamora. Lanzada mar-2021 en App Store y Play Store con 1.200 usuarios; planeaba nueva versión jul-2021 y ronda de US$500 mil. Objetivo: llevar el historial en el celular, acceso en emergencias, médico puede ingresar datos con consentimiento. Estado actual NO verificado (posible app inactiva). URL es la nota de prensa; sitio oficial por confirmar. [Vuelta 3] Sin evidencia posterior a 2021; relanzamiento previsto jul-2021 no confirmado. Probable app inactiva.</t>
+          <t>[DIRECTO · Chile · etapa A] Fundada 2019 por Diego Ibarra, Andrés Fantuzzi y Gabriel Zamora. Lanzada mar-2021 en App Store y Play Store con 1.200 usuarios; planeaba nueva versión jul-2021 y ronda de US$500 mil. Objetivo: llevar el historial en el celular, acceso en emergencias, médico puede ingresar datos con consentimiento. Estado actual NO verificado (posible app inactiva). URL es la nota de prensa; sitio oficial por confirmar. [Vuelta 3] Sin evidencia posterior a 2021; relanzamiento previsto jul-2021 no confirmado. Probable app inactiva. [Vuelta 4] Sin cambios; sigue sin evidencia posterior a 2021.</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G3" t="n">
@@ -593,12 +593,12 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>[REGIONAL · México] Historial por perfil familiar, alergias, vacunas, recetas digitales, gráficas de evolución, agendamiento, compartir con profesionales. Gratis en App Store MX. Sin evidencia de uso en Chile. Cubre parte de la etapa C (familia). [Vuelta 3] Existen dos apps distintas: MediPlanner (gratis, Rym Solutions, MX, 3,7/5 con 3 calificaciones) y MediPlanner Pro (otro desarrollador, $39 MXN). Sin presencia verificada en Chile.</t>
+          <t>[REGIONAL · México] Historial por perfil familiar, alergias, vacunas, recetas digitales, gráficas de evolución, agendamiento, compartir con profesionales. Gratis en App Store MX. Sin evidencia de uso en Chile. Cubre parte de la etapa C (familia). [Vuelta 3] Existen dos apps distintas: MediPlanner (gratis, Rym Solutions, MX, 3,7/5 con 3 calificaciones) y MediPlanner Pro (otro desarrollador, $39 MXN). Sin presencia verificada en Chile. [Vuelta 4] No pude confirmar el desarrollador de la versión gratuita (Rym Solutions no se repite en esta búsqueda). MediPlanner Pro (fichas BR/OM) guardaría datos solo en el dispositivo, sin nube; no confundir con MedPlanner/AskHEMI (otra empresa).</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G4" t="n">
@@ -633,12 +633,12 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>[REGIONAL · Argentina · débil] App para cargar antecedentes médicos propios. Única referencia: nota de opinión en grupoanimal.mx sin fecha verificada. Estado y sitio por confirmar. [Vuelta 3] Referencias de 2017 (apps4citizens, La Nación); sitio y precio no verificados; puede estar inactiva.</t>
+          <t>[REGIONAL · Argentina · débil] App para cargar antecedentes médicos propios. Única referencia: nota de opinión en grupoanimal.mx sin fecha verificada. Estado y sitio por confirmar. [Vuelta 3] Referencias de 2017 (apps4citizens, La Nación); sitio y precio no verificados; puede estar inactiva. [Vuelta 4] Sin fuentes nuevas.</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G5" t="n">
@@ -1102,7 +1102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F114"/>
+  <dimension ref="A1:F115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4758,6 +4758,38 @@
       <c r="F114" t="inlineStr">
         <is>
           <t>Búsqueda web (Medesk, Comparasoftware); no es parte de la app Clinia</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>MediPlanner</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Medicación y recordatorios</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Tratamientos automáticos desde la receta digital del médico</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>Según la ficha de la App Store MX, los tratamientos llegan automáticamente desde la receta digital del médico (autodeclarado, sin verificar).</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>Latam</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>Búsqueda web (ficha App Store MX); vuelta 4</t>
         </is>
       </c>
     </row>
@@ -7997,8 +8029,6 @@
           <t>Búsqueda de profesionales de salud</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
           <t>✓</t>
@@ -8009,17 +8039,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
       <c r="R2">
         <f>COUNTIF(C2:Q2,"✓")</f>
         <v/>
@@ -8041,24 +8060,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
       <c r="R3">
         <f>COUNTIF(C3:Q3,"✓")</f>
         <v/>
@@ -8075,25 +8081,11 @@
           <t>Integración con calendario del dispositivo</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
       <c r="R4">
         <f>COUNTIF(C4:Q4,"✓")</f>
         <v/>
@@ -8110,25 +8102,11 @@
           <t>Localización de centros médicos y farmacias</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr"/>
       <c r="R5">
         <f>COUNTIF(C5:Q5,"✓")</f>
         <v/>
@@ -8145,17 +8123,6 @@
           <t>Reserva de citas médicas</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr">
         <is>
           <t>✓</t>
@@ -8166,8 +8133,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="inlineStr"/>
       <c r="R6">
         <f>COUNTIF(C6:Q6,"✓")</f>
         <v/>
@@ -8184,25 +8149,11 @@
           <t>Acceso del profesional al historial del paciente</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr"/>
-      <c r="Q7" t="inlineStr"/>
       <c r="R7">
         <f>COUNTIF(C7:Q7,"✓")</f>
         <v/>
@@ -8219,25 +8170,11 @@
           <t>Compartir con personas sin cuenta mediante clave segura</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
-      <c r="P8" t="inlineStr"/>
-      <c r="Q8" t="inlineStr"/>
       <c r="R8">
         <f>COUNTIF(C8:Q8,"✓")</f>
         <v/>
@@ -8254,25 +8191,11 @@
           <t>Compartir datos con cuidador o persona de confianza</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
-      <c r="P9" t="inlineStr"/>
-      <c r="Q9" t="inlineStr"/>
       <c r="R9">
         <f>COUNTIF(C9:Q9,"✓")</f>
         <v/>
@@ -8294,13 +8217,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
           <t>✓</t>
@@ -8326,16 +8247,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
       <c r="O10" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="P10" t="inlineStr"/>
-      <c r="Q10" t="inlineStr"/>
       <c r="R10">
         <f>COUNTIF(C10:Q10,"✓")</f>
         <v/>
@@ -8352,25 +8268,11 @@
           <t>Gestión de consentimiento sobre uso de datos</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr"/>
-      <c r="P11" t="inlineStr"/>
-      <c r="Q11" t="inlineStr"/>
       <c r="R11">
         <f>COUNTIF(C11:Q11,"✓")</f>
         <v/>
@@ -8387,25 +8289,11 @@
           <t>Ingreso de datos por profesional con consentimiento</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
-      <c r="O12" t="inlineStr"/>
-      <c r="P12" t="inlineStr"/>
-      <c r="Q12" t="inlineStr"/>
       <c r="R12">
         <f>COUNTIF(C12:Q12,"✓")</f>
         <v/>
@@ -8422,25 +8310,11 @@
           <t>Red social con profesionales y familiares</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr"/>
-      <c r="O13" t="inlineStr"/>
-      <c r="P13" t="inlineStr"/>
-      <c r="Q13" t="inlineStr"/>
       <c r="R13">
         <f>COUNTIF(C13:Q13,"✓")</f>
         <v/>
@@ -8467,23 +8341,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
-      <c r="M14" t="inlineStr"/>
-      <c r="N14" t="inlineStr"/>
-      <c r="O14" t="inlineStr"/>
-      <c r="P14" t="inlineStr"/>
-      <c r="Q14" t="inlineStr"/>
       <c r="R14">
         <f>COUNTIF(C14:Q14,"✓")</f>
         <v/>
@@ -8500,8 +8362,6 @@
           <t>Perfiles familiares / dependientes</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
           <t>✓</t>
@@ -8512,25 +8372,16 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr"/>
       <c r="N15" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="Q15" t="inlineStr"/>
       <c r="R15">
         <f>COUNTIF(C15:Q15,"✓")</f>
         <v/>
@@ -8552,8 +8403,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
           <t>✓</t>
@@ -8569,19 +8418,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
-      <c r="M16" t="inlineStr"/>
-      <c r="N16" t="inlineStr"/>
       <c r="O16" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="P16" t="inlineStr"/>
-      <c r="Q16" t="inlineStr"/>
       <c r="R16">
         <f>COUNTIF(C16:Q16,"✓")</f>
         <v/>
@@ -8598,29 +8439,16 @@
           <t>Almacenamiento de recetas</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr"/>
       <c r="N17" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="O17" t="inlineStr"/>
-      <c r="P17" t="inlineStr"/>
-      <c r="Q17" t="inlineStr"/>
       <c r="R17">
         <f>COUNTIF(C17:Q17,"✓")</f>
         <v/>
@@ -8637,25 +8465,11 @@
           <t>Búsqueda y filtros de documentos</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr"/>
-      <c r="M18" t="inlineStr"/>
-      <c r="N18" t="inlineStr"/>
-      <c r="O18" t="inlineStr"/>
-      <c r="P18" t="inlineStr"/>
-      <c r="Q18" t="inlineStr"/>
       <c r="R18">
         <f>COUNTIF(C18:Q18,"✓")</f>
         <v/>
@@ -8672,25 +8486,11 @@
           <t>Emisión de certificados médicos</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr"/>
-      <c r="M19" t="inlineStr"/>
-      <c r="N19" t="inlineStr"/>
-      <c r="O19" t="inlineStr"/>
-      <c r="P19" t="inlineStr"/>
-      <c r="Q19" t="inlineStr"/>
       <c r="R19">
         <f>COUNTIF(C19:Q19,"✓")</f>
         <v/>
@@ -8712,19 +8512,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr"/>
-      <c r="M20" t="inlineStr"/>
-      <c r="N20" t="inlineStr"/>
-      <c r="O20" t="inlineStr"/>
-      <c r="P20" t="inlineStr"/>
       <c r="Q20" t="inlineStr">
         <is>
           <t>✓</t>
@@ -8746,25 +8533,11 @@
           <t>Notificación y envío de resultados</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr"/>
-      <c r="M21" t="inlineStr"/>
       <c r="N21" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="O21" t="inlineStr"/>
-      <c r="P21" t="inlineStr"/>
-      <c r="Q21" t="inlineStr"/>
       <c r="R21">
         <f>COUNTIF(C21:Q21,"✓")</f>
         <v/>
@@ -8781,29 +8554,16 @@
           <t>Historial institucional (solo datos de la propia red)</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
-      <c r="L22" t="inlineStr"/>
-      <c r="M22" t="inlineStr"/>
       <c r="N22" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="O22" t="inlineStr"/>
       <c r="P22" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="Q22" t="inlineStr"/>
       <c r="R22">
         <f>COUNTIF(C22:Q22,"✓")</f>
         <v/>
@@ -8820,36 +8580,26 @@
           <t>Historial médico centralizado</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="L23" t="inlineStr"/>
-      <c r="M23" t="inlineStr"/>
-      <c r="N23" t="inlineStr"/>
-      <c r="O23" t="inlineStr"/>
-      <c r="P23" t="inlineStr"/>
       <c r="Q23" t="inlineStr">
         <is>
           <t>✓</t>
@@ -8871,25 +8621,11 @@
           <t>Línea de tiempo de salud</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
-      <c r="L24" t="inlineStr"/>
-      <c r="M24" t="inlineStr"/>
-      <c r="N24" t="inlineStr"/>
-      <c r="O24" t="inlineStr"/>
-      <c r="P24" t="inlineStr"/>
-      <c r="Q24" t="inlineStr"/>
       <c r="R24">
         <f>COUNTIF(C24:Q24,"✓")</f>
         <v/>
@@ -8906,25 +8642,11 @@
           <t>Registro de alergias y vacunas</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr"/>
-      <c r="L25" t="inlineStr"/>
-      <c r="M25" t="inlineStr"/>
-      <c r="N25" t="inlineStr"/>
-      <c r="O25" t="inlineStr"/>
-      <c r="P25" t="inlineStr"/>
-      <c r="Q25" t="inlineStr"/>
       <c r="R25">
         <f>COUNTIF(C25:Q25,"✓")</f>
         <v/>
@@ -8941,11 +8663,6 @@
           <t>Recompensas / monetización de datos del usuario</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr"/>
-      <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr"/>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr">
         <is>
           <t>✓</t>
@@ -8956,14 +8673,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
-      <c r="L26" t="inlineStr"/>
-      <c r="M26" t="inlineStr"/>
-      <c r="N26" t="inlineStr"/>
-      <c r="O26" t="inlineStr"/>
-      <c r="P26" t="inlineStr"/>
-      <c r="Q26" t="inlineStr"/>
       <c r="R26">
         <f>COUNTIF(C26:Q26,"✓")</f>
         <v/>
@@ -8980,25 +8689,11 @@
           <t>Coaching de salud con IA</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr"/>
-      <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
-      <c r="L27" t="inlineStr"/>
-      <c r="M27" t="inlineStr"/>
-      <c r="N27" t="inlineStr"/>
-      <c r="O27" t="inlineStr"/>
-      <c r="P27" t="inlineStr"/>
-      <c r="Q27" t="inlineStr"/>
       <c r="R27">
         <f>COUNTIF(C27:Q27,"✓")</f>
         <v/>
@@ -9015,15 +8710,6 @@
           <t>Detección de patrones en métricas de salud con IA</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9034,10 +8720,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="N28" t="inlineStr"/>
-      <c r="O28" t="inlineStr"/>
-      <c r="P28" t="inlineStr"/>
-      <c r="Q28" t="inlineStr"/>
       <c r="R28">
         <f>COUNTIF(C28:Q28,"✓")</f>
         <v/>
@@ -9054,15 +8736,6 @@
           <t>Interpretación de exámenes con IA</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr"/>
-      <c r="D29" t="inlineStr"/>
-      <c r="E29" t="inlineStr"/>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr"/>
-      <c r="H29" t="inlineStr"/>
-      <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9073,9 +8746,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="N29" t="inlineStr"/>
-      <c r="O29" t="inlineStr"/>
-      <c r="P29" t="inlineStr"/>
       <c r="Q29" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9097,24 +8767,11 @@
           <t>Orientación médica con IA</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr"/>
-      <c r="E30" t="inlineStr"/>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr"/>
-      <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="M30" t="inlineStr"/>
-      <c r="N30" t="inlineStr"/>
-      <c r="O30" t="inlineStr"/>
-      <c r="P30" t="inlineStr"/>
       <c r="Q30" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9136,15 +8793,6 @@
           <t>Preparación de consultas médicas con IA</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr"/>
-      <c r="D31" t="inlineStr"/>
-      <c r="E31" t="inlineStr"/>
-      <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr"/>
-      <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9155,10 +8803,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="N31" t="inlineStr"/>
-      <c r="O31" t="inlineStr"/>
-      <c r="P31" t="inlineStr"/>
-      <c r="Q31" t="inlineStr"/>
       <c r="R31">
         <f>COUNTIF(C31:Q31,"✓")</f>
         <v/>
@@ -9175,15 +8819,6 @@
           <t>Resumen de historial con IA</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr"/>
-      <c r="D32" t="inlineStr"/>
-      <c r="E32" t="inlineStr"/>
-      <c r="F32" t="inlineStr"/>
-      <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr"/>
-      <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr"/>
-      <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9194,10 +8829,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="N32" t="inlineStr"/>
-      <c r="O32" t="inlineStr"/>
-      <c r="P32" t="inlineStr"/>
-      <c r="Q32" t="inlineStr"/>
       <c r="R32">
         <f>COUNTIF(C32:Q32,"✓")</f>
         <v/>
@@ -9219,10 +8850,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr"/>
-      <c r="E33" t="inlineStr"/>
-      <c r="F33" t="inlineStr"/>
-      <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9233,7 +8860,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="J33" t="inlineStr"/>
       <c r="K33" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9249,14 +8875,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="N33" t="inlineStr"/>
       <c r="O33" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="P33" t="inlineStr"/>
-      <c r="Q33" t="inlineStr"/>
       <c r="R33">
         <f>COUNTIF(C33:Q33,"✓")</f>
         <v/>
@@ -9273,25 +8896,11 @@
           <t>Analítica poblacional B2B</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr"/>
-      <c r="D34" t="inlineStr"/>
-      <c r="E34" t="inlineStr"/>
-      <c r="F34" t="inlineStr"/>
-      <c r="G34" t="inlineStr"/>
       <c r="H34" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="I34" t="inlineStr"/>
-      <c r="J34" t="inlineStr"/>
-      <c r="K34" t="inlineStr"/>
-      <c r="L34" t="inlineStr"/>
-      <c r="M34" t="inlineStr"/>
-      <c r="N34" t="inlineStr"/>
-      <c r="O34" t="inlineStr"/>
-      <c r="P34" t="inlineStr"/>
-      <c r="Q34" t="inlineStr"/>
       <c r="R34">
         <f>COUNTIF(C34:Q34,"✓")</f>
         <v/>
@@ -9308,9 +8917,6 @@
           <t>Disponibilidad multiplataforma (web/iOS/Android)</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr"/>
-      <c r="D35" t="inlineStr"/>
-      <c r="E35" t="inlineStr"/>
       <c r="F35" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9321,20 +8927,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr"/>
-      <c r="K35" t="inlineStr"/>
-      <c r="L35" t="inlineStr"/>
-      <c r="M35" t="inlineStr"/>
-      <c r="N35" t="inlineStr"/>
       <c r="O35" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="P35" t="inlineStr"/>
-      <c r="Q35" t="inlineStr"/>
       <c r="R35">
         <f>COUNTIF(C35:Q35,"✓")</f>
         <v/>
@@ -9351,25 +8948,11 @@
           <t>Historial médico centralizado</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr"/>
-      <c r="D36" t="inlineStr"/>
-      <c r="E36" t="inlineStr"/>
-      <c r="F36" t="inlineStr"/>
-      <c r="G36" t="inlineStr"/>
-      <c r="H36" t="inlineStr"/>
-      <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="K36" t="inlineStr"/>
-      <c r="L36" t="inlineStr"/>
-      <c r="M36" t="inlineStr"/>
-      <c r="N36" t="inlineStr"/>
-      <c r="O36" t="inlineStr"/>
-      <c r="P36" t="inlineStr"/>
-      <c r="Q36" t="inlineStr"/>
       <c r="R36">
         <f>COUNTIF(C36:Q36,"✓")</f>
         <v/>
@@ -9386,25 +8969,11 @@
           <t>Importación y exportación de datos</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr"/>
-      <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr"/>
-      <c r="G37" t="inlineStr"/>
-      <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr"/>
-      <c r="J37" t="inlineStr"/>
-      <c r="K37" t="inlineStr"/>
-      <c r="L37" t="inlineStr"/>
-      <c r="M37" t="inlineStr"/>
-      <c r="N37" t="inlineStr"/>
-      <c r="O37" t="inlineStr"/>
-      <c r="P37" t="inlineStr"/>
-      <c r="Q37" t="inlineStr"/>
       <c r="R37">
         <f>COUNTIF(C37:Q37,"✓")</f>
         <v/>
@@ -9421,29 +8990,16 @@
           <t>Integración con wearables y apps de salud</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr"/>
-      <c r="D38" t="inlineStr"/>
-      <c r="E38" t="inlineStr"/>
-      <c r="F38" t="inlineStr"/>
-      <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="I38" t="inlineStr"/>
-      <c r="J38" t="inlineStr"/>
-      <c r="K38" t="inlineStr"/>
-      <c r="L38" t="inlineStr"/>
       <c r="M38" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="N38" t="inlineStr"/>
-      <c r="O38" t="inlineStr"/>
-      <c r="P38" t="inlineStr"/>
-      <c r="Q38" t="inlineStr"/>
       <c r="R38">
         <f>COUNTIF(C38:Q38,"✓")</f>
         <v/>
@@ -9460,25 +9016,11 @@
           <t>Gestión de lista de medicamentos</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr"/>
-      <c r="D39" t="inlineStr"/>
-      <c r="E39" t="inlineStr"/>
-      <c r="F39" t="inlineStr"/>
-      <c r="G39" t="inlineStr"/>
-      <c r="H39" t="inlineStr"/>
-      <c r="I39" t="inlineStr"/>
-      <c r="J39" t="inlineStr"/>
       <c r="K39" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="L39" t="inlineStr"/>
-      <c r="M39" t="inlineStr"/>
-      <c r="N39" t="inlineStr"/>
-      <c r="O39" t="inlineStr"/>
-      <c r="P39" t="inlineStr"/>
-      <c r="Q39" t="inlineStr"/>
       <c r="R39">
         <f>COUNTIF(C39:Q39,"✓")</f>
         <v/>
@@ -9500,24 +9042,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr"/>
-      <c r="E40" t="inlineStr"/>
-      <c r="F40" t="inlineStr"/>
-      <c r="G40" t="inlineStr"/>
-      <c r="H40" t="inlineStr"/>
-      <c r="I40" t="inlineStr"/>
-      <c r="J40" t="inlineStr"/>
       <c r="K40" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="L40" t="inlineStr"/>
-      <c r="M40" t="inlineStr"/>
-      <c r="N40" t="inlineStr"/>
-      <c r="O40" t="inlineStr"/>
-      <c r="P40" t="inlineStr"/>
-      <c r="Q40" t="inlineStr"/>
       <c r="R40">
         <f>COUNTIF(C40:Q40,"✓")</f>
         <v/>
@@ -9534,25 +9063,11 @@
           <t>Registro de tomas y adherencia al tratamiento</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr"/>
-      <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr"/>
-      <c r="G41" t="inlineStr"/>
-      <c r="H41" t="inlineStr"/>
-      <c r="I41" t="inlineStr"/>
-      <c r="J41" t="inlineStr"/>
-      <c r="K41" t="inlineStr"/>
-      <c r="L41" t="inlineStr"/>
-      <c r="M41" t="inlineStr"/>
-      <c r="N41" t="inlineStr"/>
-      <c r="O41" t="inlineStr"/>
-      <c r="P41" t="inlineStr"/>
-      <c r="Q41" t="inlineStr"/>
       <c r="R41">
         <f>COUNTIF(C41:Q41,"✓")</f>
         <v/>
@@ -9569,25 +9084,11 @@
           <t>Contenido educativo sobre salud</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr"/>
       <c r="D42" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr"/>
-      <c r="F42" t="inlineStr"/>
-      <c r="G42" t="inlineStr"/>
-      <c r="H42" t="inlineStr"/>
-      <c r="I42" t="inlineStr"/>
-      <c r="J42" t="inlineStr"/>
-      <c r="K42" t="inlineStr"/>
-      <c r="L42" t="inlineStr"/>
-      <c r="M42" t="inlineStr"/>
-      <c r="N42" t="inlineStr"/>
-      <c r="O42" t="inlineStr"/>
-      <c r="P42" t="inlineStr"/>
-      <c r="Q42" t="inlineStr"/>
       <c r="R42">
         <f>COUNTIF(C42:Q42,"✓")</f>
         <v/>
@@ -9604,25 +9105,11 @@
           <t>Gráficas de evolución de indicadores</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr"/>
-      <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr"/>
-      <c r="G43" t="inlineStr"/>
-      <c r="H43" t="inlineStr"/>
-      <c r="I43" t="inlineStr"/>
-      <c r="J43" t="inlineStr"/>
-      <c r="K43" t="inlineStr"/>
-      <c r="L43" t="inlineStr"/>
-      <c r="M43" t="inlineStr"/>
-      <c r="N43" t="inlineStr"/>
-      <c r="O43" t="inlineStr"/>
-      <c r="P43" t="inlineStr"/>
-      <c r="Q43" t="inlineStr"/>
       <c r="R43">
         <f>COUNTIF(C43:Q43,"✓")</f>
         <v/>
@@ -9639,25 +9126,11 @@
           <t>Integración con wearables y apps de salud</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr"/>
-      <c r="D44" t="inlineStr"/>
-      <c r="E44" t="inlineStr"/>
-      <c r="F44" t="inlineStr"/>
-      <c r="G44" t="inlineStr"/>
-      <c r="H44" t="inlineStr"/>
-      <c r="I44" t="inlineStr"/>
-      <c r="J44" t="inlineStr"/>
       <c r="K44" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="L44" t="inlineStr"/>
-      <c r="M44" t="inlineStr"/>
-      <c r="N44" t="inlineStr"/>
-      <c r="O44" t="inlineStr"/>
-      <c r="P44" t="inlineStr"/>
-      <c r="Q44" t="inlineStr"/>
       <c r="R44">
         <f>COUNTIF(C44:Q44,"✓")</f>
         <v/>
@@ -9674,25 +9147,11 @@
           <t>Panel de seguimiento de salud y bienestar</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr"/>
-      <c r="D45" t="inlineStr"/>
-      <c r="E45" t="inlineStr"/>
-      <c r="F45" t="inlineStr"/>
-      <c r="G45" t="inlineStr"/>
       <c r="H45" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="I45" t="inlineStr"/>
-      <c r="J45" t="inlineStr"/>
-      <c r="K45" t="inlineStr"/>
-      <c r="L45" t="inlineStr"/>
-      <c r="M45" t="inlineStr"/>
-      <c r="N45" t="inlineStr"/>
-      <c r="O45" t="inlineStr"/>
-      <c r="P45" t="inlineStr"/>
-      <c r="Q45" t="inlineStr"/>
       <c r="R45">
         <f>COUNTIF(C45:Q45,"✓")</f>
         <v/>
@@ -9709,25 +9168,11 @@
           <t>Registro de nutrición</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr"/>
-      <c r="D46" t="inlineStr"/>
-      <c r="E46" t="inlineStr"/>
-      <c r="F46" t="inlineStr"/>
-      <c r="G46" t="inlineStr"/>
-      <c r="H46" t="inlineStr"/>
-      <c r="I46" t="inlineStr"/>
-      <c r="J46" t="inlineStr"/>
       <c r="K46" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="L46" t="inlineStr"/>
-      <c r="M46" t="inlineStr"/>
-      <c r="N46" t="inlineStr"/>
-      <c r="O46" t="inlineStr"/>
-      <c r="P46" t="inlineStr"/>
-      <c r="Q46" t="inlineStr"/>
       <c r="R46">
         <f>COUNTIF(C46:Q46,"✓")</f>
         <v/>
@@ -9744,25 +9189,11 @@
           <t>Seguimiento de salud femenina</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr"/>
-      <c r="D47" t="inlineStr"/>
-      <c r="E47" t="inlineStr"/>
-      <c r="F47" t="inlineStr"/>
-      <c r="G47" t="inlineStr"/>
-      <c r="H47" t="inlineStr"/>
-      <c r="I47" t="inlineStr"/>
-      <c r="J47" t="inlineStr"/>
       <c r="K47" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="L47" t="inlineStr"/>
-      <c r="M47" t="inlineStr"/>
-      <c r="N47" t="inlineStr"/>
-      <c r="O47" t="inlineStr"/>
-      <c r="P47" t="inlineStr"/>
-      <c r="Q47" t="inlineStr"/>
       <c r="R47">
         <f>COUNTIF(C47:Q47,"✓")</f>
         <v/>
@@ -9779,25 +9210,11 @@
           <t>Valoración de profesionales</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr"/>
-      <c r="D48" t="inlineStr"/>
-      <c r="E48" t="inlineStr"/>
       <c r="F48" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="G48" t="inlineStr"/>
-      <c r="H48" t="inlineStr"/>
-      <c r="I48" t="inlineStr"/>
-      <c r="J48" t="inlineStr"/>
-      <c r="K48" t="inlineStr"/>
-      <c r="L48" t="inlineStr"/>
-      <c r="M48" t="inlineStr"/>
-      <c r="N48" t="inlineStr"/>
-      <c r="O48" t="inlineStr"/>
-      <c r="P48" t="inlineStr"/>
-      <c r="Q48" t="inlineStr"/>
       <c r="R48">
         <f>COUNTIF(C48:Q48,"✓")</f>
         <v/>
@@ -9814,11 +9231,6 @@
           <t>Blockchain para integridad y trazabilidad de datos</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr"/>
-      <c r="D49" t="inlineStr"/>
-      <c r="E49" t="inlineStr"/>
-      <c r="F49" t="inlineStr"/>
-      <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9834,13 +9246,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="K49" t="inlineStr"/>
-      <c r="L49" t="inlineStr"/>
-      <c r="M49" t="inlineStr"/>
-      <c r="N49" t="inlineStr"/>
-      <c r="O49" t="inlineStr"/>
-      <c r="P49" t="inlineStr"/>
-      <c r="Q49" t="inlineStr"/>
       <c r="R49">
         <f>COUNTIF(C49:Q49,"✓")</f>
         <v/>
@@ -9857,29 +9262,16 @@
           <t>Cifrado y control de acceso</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr"/>
       <c r="D50" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr"/>
-      <c r="F50" t="inlineStr"/>
-      <c r="G50" t="inlineStr"/>
-      <c r="H50" t="inlineStr"/>
-      <c r="I50" t="inlineStr"/>
-      <c r="J50" t="inlineStr"/>
       <c r="K50" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="L50" t="inlineStr"/>
-      <c r="M50" t="inlineStr"/>
-      <c r="N50" t="inlineStr"/>
-      <c r="O50" t="inlineStr"/>
-      <c r="P50" t="inlineStr"/>
-      <c r="Q50" t="inlineStr"/>
       <c r="R50">
         <f>COUNTIF(C50:Q50,"✓")</f>
         <v/>
@@ -9896,25 +9288,11 @@
           <t>Cumplimiento regulatorio de salud y datos</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr"/>
-      <c r="D51" t="inlineStr"/>
-      <c r="E51" t="inlineStr"/>
-      <c r="F51" t="inlineStr"/>
-      <c r="G51" t="inlineStr"/>
-      <c r="H51" t="inlineStr"/>
-      <c r="I51" t="inlineStr"/>
-      <c r="J51" t="inlineStr"/>
-      <c r="K51" t="inlineStr"/>
-      <c r="L51" t="inlineStr"/>
-      <c r="M51" t="inlineStr"/>
-      <c r="N51" t="inlineStr"/>
       <c r="O51" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="P51" t="inlineStr"/>
-      <c r="Q51" t="inlineStr"/>
       <c r="R51">
         <f>COUNTIF(C51:Q51,"✓")</f>
         <v/>
@@ -9931,25 +9309,11 @@
           <t>Identidad descentralizada (DID)</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr"/>
-      <c r="D52" t="inlineStr"/>
-      <c r="E52" t="inlineStr"/>
-      <c r="F52" t="inlineStr"/>
-      <c r="G52" t="inlineStr"/>
-      <c r="H52" t="inlineStr"/>
       <c r="I52" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="J52" t="inlineStr"/>
-      <c r="K52" t="inlineStr"/>
-      <c r="L52" t="inlineStr"/>
-      <c r="M52" t="inlineStr"/>
-      <c r="N52" t="inlineStr"/>
-      <c r="O52" t="inlineStr"/>
-      <c r="P52" t="inlineStr"/>
-      <c r="Q52" t="inlineStr"/>
       <c r="R52">
         <f>COUNTIF(C52:Q52,"✓")</f>
         <v/>
@@ -9966,15 +9330,6 @@
           <t>Privacidad reforzada para datos de salud</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr"/>
-      <c r="D53" t="inlineStr"/>
-      <c r="E53" t="inlineStr"/>
-      <c r="F53" t="inlineStr"/>
-      <c r="G53" t="inlineStr"/>
-      <c r="H53" t="inlineStr"/>
-      <c r="I53" t="inlineStr"/>
-      <c r="J53" t="inlineStr"/>
-      <c r="K53" t="inlineStr"/>
       <c r="L53" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9985,10 +9340,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="N53" t="inlineStr"/>
-      <c r="O53" t="inlineStr"/>
-      <c r="P53" t="inlineStr"/>
-      <c r="Q53" t="inlineStr"/>
       <c r="R53">
         <f>COUNTIF(C53:Q53,"✓")</f>
         <v/>
@@ -10005,20 +9356,6 @@
           <t>Modelo freemium y suscripción</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr"/>
-      <c r="D54" t="inlineStr"/>
-      <c r="E54" t="inlineStr"/>
-      <c r="F54" t="inlineStr"/>
-      <c r="G54" t="inlineStr"/>
-      <c r="H54" t="inlineStr"/>
-      <c r="I54" t="inlineStr"/>
-      <c r="J54" t="inlineStr"/>
-      <c r="K54" t="inlineStr"/>
-      <c r="L54" t="inlineStr"/>
-      <c r="M54" t="inlineStr"/>
-      <c r="N54" t="inlineStr"/>
-      <c r="O54" t="inlineStr"/>
-      <c r="P54" t="inlineStr"/>
       <c r="Q54" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10040,25 +9377,11 @@
           <t>Pagos con criptomoneda</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr"/>
-      <c r="D55" t="inlineStr"/>
-      <c r="E55" t="inlineStr"/>
-      <c r="F55" t="inlineStr"/>
-      <c r="G55" t="inlineStr"/>
-      <c r="H55" t="inlineStr"/>
-      <c r="I55" t="inlineStr"/>
       <c r="J55" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="K55" t="inlineStr"/>
-      <c r="L55" t="inlineStr"/>
-      <c r="M55" t="inlineStr"/>
-      <c r="N55" t="inlineStr"/>
-      <c r="O55" t="inlineStr"/>
-      <c r="P55" t="inlineStr"/>
-      <c r="Q55" t="inlineStr"/>
       <c r="R55">
         <f>COUNTIF(C55:Q55,"✓")</f>
         <v/>
@@ -10075,25 +9398,11 @@
           <t>Reclamos y trámites con seguros</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr"/>
-      <c r="D56" t="inlineStr"/>
-      <c r="E56" t="inlineStr"/>
-      <c r="F56" t="inlineStr"/>
-      <c r="G56" t="inlineStr"/>
-      <c r="H56" t="inlineStr"/>
       <c r="I56" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="J56" t="inlineStr"/>
-      <c r="K56" t="inlineStr"/>
-      <c r="L56" t="inlineStr"/>
-      <c r="M56" t="inlineStr"/>
-      <c r="N56" t="inlineStr"/>
-      <c r="O56" t="inlineStr"/>
-      <c r="P56" t="inlineStr"/>
-      <c r="Q56" t="inlineStr"/>
       <c r="R56">
         <f>COUNTIF(C56:Q56,"✓")</f>
         <v/>
@@ -10110,25 +9419,11 @@
           <t>Teleconsulta con profesionales</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr"/>
-      <c r="D57" t="inlineStr"/>
-      <c r="E57" t="inlineStr"/>
-      <c r="F57" t="inlineStr"/>
-      <c r="G57" t="inlineStr"/>
-      <c r="H57" t="inlineStr"/>
-      <c r="I57" t="inlineStr"/>
       <c r="J57" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="K57" t="inlineStr"/>
-      <c r="L57" t="inlineStr"/>
-      <c r="M57" t="inlineStr"/>
-      <c r="N57" t="inlineStr"/>
-      <c r="O57" t="inlineStr"/>
-      <c r="P57" t="inlineStr"/>
-      <c r="Q57" t="inlineStr"/>
       <c r="R57">
         <f>COUNTIF(C57:Q57,"✓")</f>
         <v/>
@@ -10145,7 +9440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A17"/>
+  <dimension ref="A1:A18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -10270,6 +9565,13 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Vuelta 4 (iter. 1, 2026-10-08 06:08 UTC): Meedika, Infomed, MediPlanner, Clingot verificados (+1 fila). CANDIDATO A COMPETIDOR (no agregado a la lista, a decisión del usuario): HealthChain (Chile), startup de registros médicos con blockchain; CEO Javier Leyton; fuente: entrevista en Diario Bitcoin sin fecha visible. Pendientes: Healfies, Patientory, MediBloc, Medicalchain, etc.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Benchmark: vuelta 4, iteración 2 (Healfies, Patientory, MediBloc, Medicalchain)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MVcXu8vTBu7EKfj3YdEvae
</commit_message>
<xml_diff>
--- a/Outputs/Benchmark_Anamnesis.xlsx
+++ b/Outputs/Benchmark_Anamnesis.xlsx
@@ -673,12 +673,12 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>[REGIONAL · Brasil] Fundada ene-2015 en Florianópolis por Helyson Lewis Velasco. Centraliza registros de salud personales: carpetas, etiquetas, línea de tiempo (medicación, exámenes, citas, dieta), compartir con familia o profesionales. Gratis; web, iOS y Android. Estado actual NO verificado (fuentes de 2015-2016). Referencia funcional cercana a etapas A+B. [Vuelta 2] Lanzada simultáneamente en Brasil, Argentina y EE.UU.; permite compartir con no registrados vía clave por email. Sin novedades posteriores a 2016. [Vuelta 3] Sin evidencia de actividad reciente ni de cierre; Gust/Dealroom la listan en Florianópolis (10 empleados, healfies.com) sin fecha de actualización. Estado sin confirmar.</t>
+          <t>[REGIONAL · Brasil] Fundada ene-2015 en Florianópolis por Helyson Lewis Velasco. Centraliza registros de salud personales: carpetas, etiquetas, línea de tiempo (medicación, exámenes, citas, dieta), compartir con familia o profesionales. Gratis; web, iOS y Android. Estado actual NO verificado (fuentes de 2015-2016). Referencia funcional cercana a etapas A+B. [Vuelta 2] Lanzada simultáneamente en Brasil, Argentina y EE.UU.; permite compartir con no registrados vía clave por email. Sin novedades posteriores a 2016. [Vuelta 3] Sin evidencia de actividad reciente ni de cierre; Gust/Dealroom la listan en Florianópolis (10 empleados, healfies.com) sin fecha de actualización. Estado sin confirmar. [Vuelta 4] Sin Google Play localizado; no confundir con la app Healfy (otro producto). Sin novedades.</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G6" t="n">
@@ -713,12 +713,12 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>[BLOCKCHAIN · EE.UU.] Atlanta, fundada 2015, ~9 empleados. Levantó US$7,2M vía financiamiento cripto. App con registros de hospitales y wearables, coaching de salud con IA y recompensas en cripto; también dashboard empresarial Neith. PitchBook indica actividad y financiamiento hasta abr-2026: sigue operando. Sin presencia conocida en Chile. Referencia directa para la hipótesis blockchain. [Vuelta 2] Sin noticias 2026 encontradas en búsqueda; sitio oficial bloqueado. [Vuelta 3] Búsqueda adicional solo devuelve hitos de 2017 (token sale US$7,2M) y 2019 (Serie A de US$5,3M, cierre no confirmado); sin datos 2025-26 propios.</t>
+          <t>[BLOCKCHAIN · EE.UU.] Atlanta, fundada 2015, ~9 empleados. Levantó US$7,2M vía financiamiento cripto. App con registros de hospitales y wearables, coaching de salud con IA y recompensas en cripto; también dashboard empresarial Neith. PitchBook indica actividad y financiamiento hasta abr-2026: sigue operando. Sin presencia conocida en Chile. Referencia directa para la hipótesis blockchain. [Vuelta 2] Sin noticias 2026 encontradas en búsqueda; sitio oficial bloqueado. [Vuelta 3] Búsqueda adicional solo devuelve hitos de 2017 (token sale US$7,2M) y 2019 (Serie A de US$5,3M, cierre no confirmado); sin datos 2025-26 propios. [Vuelta 4] App pública lanzada en la conferencia JP Morgan Healthcare (2019); red PTOYMatrix (blockchain HIPAA); socios reportados: StartUp Health y Kaiser Permanente (beta). Estado actual en App Store/Google Play sin confirmar.</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G7" t="n">
@@ -753,12 +753,12 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>[BLOCKCHAIN · Corea del Sur] Fundada 2017, Seúl. Blockchain propia Panacea (Cosmos SDK, mainnet 2019) para que el paciente gestione y transfiera sus registros; app Medipass para seguros. Serie A de ₩4.000 millones (Naver); alianzas con hospitales (Seoul National, Severance). Estado 2025-26 NO verificado. Referencia sobre seguros + blockchain. [Vuelta 2] Panacea incluye DID, Append Only Log, IBC y PNFT; sin anuncios 2026 localizados. [Vuelta 3] Medipass: app en Corea con 20 hospitales/aseguradoras integrados (fecha de la lista desconocida) y plan 2022 de superapp con marketplace de datos; operación actual sin confirmar.</t>
+          <t>[BLOCKCHAIN · Corea del Sur] Fundada 2017, Seúl. Blockchain propia Panacea (Cosmos SDK, mainnet 2019) para que el paciente gestione y transfiera sus registros; app Medipass para seguros. Serie A de ₩4.000 millones (Naver); alianzas con hospitales (Seoul National, Severance). Estado 2025-26 NO verificado. Referencia sobre seguros + blockchain. [Vuelta 2] Panacea incluye DID, Append Only Log, IBC y PNFT; sin anuncios 2026 localizados. [Vuelta 3] Medipass: app en Corea con 20 hospitales/aseguradoras integrados (fecha de la lista desconocida) y plan 2022 de superapp con marketplace de datos; operación actual sin confirmar. [Vuelta 4] Sin búsqueda nueva (revisada en vuelta 3); sin cambios.</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G8" t="n">
@@ -793,12 +793,12 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>[BLOCKCHAIN · Reino Unido · INACTIVO] Londres, 2017, Ethereum, con telemedicina. Piloto según registro de la UE (2020). Tracxn/PitchBook lo marcan fuera de operación (ago-2025). Solo caso de aprendizaje: no cuenta como competidor activo. [Vuelta 2] Token MTN deslistado de Bitfinex el 26-mar-2021; sin hallazgos de actividad posterior. [Vuelta 3] Seedtable la marca activa sin fuente; no hallé registro en Companies House. Sigue tratándose como caso de aprendizaje.</t>
+          <t>[BLOCKCHAIN · Reino Unido · INACTIVO] Londres, 2017, Ethereum, con telemedicina. Piloto según registro de la UE (2020). Tracxn/PitchBook lo marcan fuera de operación (ago-2025). Solo caso de aprendizaje: no cuenta como competidor activo. [Vuelta 2] Token MTN deslistado de Bitfinex el 26-mar-2021; sin hallazgos de actividad posterior. [Vuelta 3] Seedtable la marca activa sin fuente; no hallé registro en Companies House. Sigue tratándose como caso de aprendizaje. [Vuelta 4] Pre-venta reportada de US$20M en MedTokens (un solo artículo secundario, sin verificar); modelo de token en revisión y exploración de security token según AMA; integraciones y servicios de 2019 sin confirmar.</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G9" t="n">
@@ -1102,7 +1102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F115"/>
+  <dimension ref="A1:F120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4790,6 +4790,166 @@
       <c r="F115" t="inlineStr">
         <is>
           <t>Búsqueda web (ficha App Store MX); vuelta 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>Patientory</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Seguimiento y bienestar</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Comunidad de pacientes con condiciones similares</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>Los usuarios con condiciones similares pueden preguntar, recibir recomendaciones y compartir experiencias.</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>Búsqueda web (BioSpace, Bitcoin Magazine; app pública 2019)</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Patientory</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Historial y perfil clínico</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Seguimiento de visitas, facturas médicas, seguros, vacunas y medicamentos</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>App gratuita para seguir visitas al médico, facturas médicas, datos personales, seguros, inmunizaciones y medicamentos de farmacia.</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>Búsqueda web (BioSpace); estado actual sin verificar</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>Medicalchain</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Seguros y pagos</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Pago de consultas con tarjeta o MedTokens (piloto The Groves Medical Centre)</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>Piloto en New Malden (Londres): consultas por video pagables con tarjeta o con MedTokens.</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>Búsqueda web (Digital Health 2018, HTN); inactivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Medicalchain</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Incentivos y monetización de datos</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Recompensas por compartir datos con investigación (planificado)</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>Centros de investigación y farmacéuticas recompensarían con MedTokens a quienes compartan sus datos; no confirmado como ejecutado.</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>Búsqueda web (Digital Health, HTN)</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>Medicalchain</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Interoperabilidad y fuentes de datos</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Integración con sistemas de médicos generales del Reino Unido (planificado)</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>Según una AMA sin fecha, integraba dos sistemas de GP que cubren ~80% del mercado UK; no confirmado como ejecutado.</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>Búsqueda web (AMA comunitaria); confianza baja</t>
         </is>
       </c>
     </row>
@@ -9440,7 +9600,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A18"/>
+  <dimension ref="A1:A19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -9572,6 +9732,13 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Vuelta 4 (iter. 2, 2026-10-08 08:08 UTC): Healfies, Patientory, MediBloc, Medicalchain verificados (+5 filas). Pendientes: Apple Health, ChatGPT Health, Claude for Healthcare, Apps de clínicas, Clinia, MiRedSalud, Mediko.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Benchmark: vuelta 4, iteración 3 (Apple Health, ChatGPT Health, Claude for Healthcare, Apps de clínicas)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MVcXu8vTBu7EKfj3YdEvae
</commit_message>
<xml_diff>
--- a/Outputs/Benchmark_Anamnesis.xlsx
+++ b/Outputs/Benchmark_Anamnesis.xlsx
@@ -833,12 +833,12 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>[ADYACENTE · global] Agrega registros clínicos vía FHIR; &gt;500 instituciones conectadas en EE.UU. (2018). Sin evidencia de disponibilidad en Chile. Incluida en el dispositivo. Amenaza si FHIR/IPS-CL se adopta en Chile. [Vuelta 2] Sin disponibilidad de registros clínicos en Chile (solo EE.UU., Reino Unido, Canadá). [Vuelta 3] iOS 27 (WWDC 8-jun-2026; publicado ~14-sep-2026): rediseño del app Health, menopausia, nutrición por cámara. El coach de salud con IA no se anunció. Sin ampliación de Health Records a Chile.</t>
+          <t>[ADYACENTE · global] Agrega registros clínicos vía FHIR; &gt;500 instituciones conectadas en EE.UU. (2018). Sin evidencia de disponibilidad en Chile. Incluida en el dispositivo. Amenaza si FHIR/IPS-CL se adopta en Chile. [Vuelta 2] Sin disponibilidad de registros clínicos en Chile (solo EE.UU., Reino Unido, Canadá). [Vuelta 3] iOS 27 (WWDC 8-jun-2026; publicado ~14-sep-2026): rediseño del app Health, menopausia, nutrición por cámara. El coach de salud con IA no se anunció. Sin ampliación de Health Records a Chile. [Vuelta 4] Sin búsqueda nueva (revisada en vuelta 3); sin cambios.</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G10" t="n">
@@ -873,12 +873,12 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>[ADYACENTE · global] Lanzado 7-ene-2026. Conecta registros médicos; conectores solo en EE.UU. Dentro de suscripción del asistente. Fija la expectativa de consultar y resumir el historial. [Vuelta 2] Confirmado: registros solo EE.UU.; sin anuncios para Latinoamérica. Hay inconsistencia de fechas entre fuentes (7-ene-2026 lanzamiento vs. jul-2026 despliegue de registros). [Vuelta 3] Fechas aclaradas: presentación 7-ene-2026 (acceso limitado); despliegue de Health in ChatGPT con Apple Health y registros en EE.UU. el 23-jul-2026; mejora de salud jun-2026. Sin anuncios para Latinoamérica ni para sep-oct 2026.</t>
+          <t>[ADYACENTE · global] Lanzado 7-ene-2026. Conecta registros médicos; conectores solo en EE.UU. Dentro de suscripción del asistente. Fija la expectativa de consultar y resumir el historial. [Vuelta 2] Confirmado: registros solo EE.UU.; sin anuncios para Latinoamérica. Hay inconsistencia de fechas entre fuentes (7-ene-2026 lanzamiento vs. jul-2026 despliegue de registros). [Vuelta 3] Fechas aclaradas: presentación 7-ene-2026 (acceso limitado); despliegue de Health in ChatGPT con Apple Health y registros en EE.UU. el 23-jul-2026; mejora de salud jun-2026. Sin anuncios para Latinoamérica ni para sep-oct 2026. [Vuelta 4] Septiembre 2026: permisos por defecto para datos conectados (14-sep) y explicaciones por gráfico/métrica (28-sep); ChatGPT for Clinicians (abr-2026) para clínicos verificados de EE.UU. Más del 70% de usuarios de Health permite usar datos conectados sin pedir permiso (según OpenAI). Sigue solo EE.UU.</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G11" t="n">
@@ -913,12 +913,12 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>[ADYACENTE · global] Lanzado 11-ene-2026. Conectores solo en EE.UU., planes Pro/Max. Nota: producto de Anthropic, conflicto de interés al evaluarlo. [Vuelta 2] Sin cambios fuera de EE.UU. (HealthEx y Function para Pro/Max). [Vuelta 3] Sin anuncios posteriores a enero de 2026. Hoja de ruta de HealthEx (agendar, buscar prestadores, recetas) sin confirmar como lanzada.</t>
+          <t>[ADYACENTE · global] Lanzado 11-ene-2026. Conectores solo en EE.UU., planes Pro/Max. Nota: producto de Anthropic, conflicto de interés al evaluarlo. [Vuelta 2] Sin cambios fuera de EE.UU. (HealthEx y Function para Pro/Max). [Vuelta 3] Sin anuncios posteriores a enero de 2026. Hoja de ruta de HealthEx (agendar, buscar prestadores, recetas) sin confirmar como lanzada. [Vuelta 4] Sin anuncios nuevos. Fuentes discrepan en el acceso (Pro/Max según Fortune y la mayoría; Pro/Team según Times of AI); sin evidencia de disponibilidad fuera de EE.UU.</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G12" t="n">
@@ -953,12 +953,12 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>[SUSTITUTO PARCIAL · Chile] Reservar hora, ver historial de esa institución, vincular familiar. Gratis; no consolida datos de otras instituciones. [Vuelta 2] App concreta: Mi Alemana Go (Clínica Alemana, Chile), con historial desde 2018, recetas, órdenes, familiar vinculado y resultados. [Vuelta 3] Búsqueda de otras clínicas (Las Condes, Santa María, UC Christus) sin ficha de app confirmada; solo canales digitales genéricos.</t>
+          <t>[SUSTITUTO PARCIAL · Chile] Reservar hora, ver historial de esa institución, vincular familiar. Gratis; no consolida datos de otras instituciones. [Vuelta 2] App concreta: Mi Alemana Go (Clínica Alemana, Chile), con historial desde 2018, recetas, órdenes, familiar vinculado y resultados. [Vuelta 3] Búsqueda de otras clínicas (Las Condes, Santa María, UC Christus) sin ficha de app confirmada; solo canales digitales genéricos. [Vuelta 4] Mi Alemana Go: 3,1/5 con 137 calificaciones (App Store Chile), pantalla de inicio rediseñada para gestionar salud propia y familiar; sin evidencia de teleconsulta ni pagos en la app.</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G13" t="n">
@@ -1102,7 +1102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F120"/>
+  <dimension ref="A1:F124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4950,6 +4950,134 @@
       <c r="F120" t="inlineStr">
         <is>
           <t>Búsqueda web (AMA comunitaria); confianza baja</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>ChatGPT Health (OpenAI)</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>Inteligencia artificial</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Explicaciones personalizadas al seleccionar gráfico, métrica o registro</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>Desde 28-sep-2026, en la pestaña Health se puede elegir un gráfico, métrica o registro y obtener explicaciones basadas en los datos conectados.</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>Búsqueda web (notas de versión de OpenAI); solo EE.UU.</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>ChatGPT Health (OpenAI)</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>Seguridad, privacidad y blockchain</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Permiso por defecto para usar datos de Health conectados</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>Desde 14-sep-2026, las nuevas conexiones heredan la configuración global de plugins: ChatGPT puede usar datos de Health sin pedir permiso cada vez salvo acciones sensibles (web primero, móvil después).</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>Búsqueda web (notas de versión de OpenAI)</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>ChatGPT Health (OpenAI)</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Inteligencia artificial</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>ChatGPT for Clinicians y Healthcare Public Data</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>Producto para clínicos verificados de EE.UU. (gratis, abr-2026); desde 1-sep-2026 un plugin con nueve apps de fuentes públicas (investigación, ensayos, medicamentos, Medicare, prestadores), de solo lectura y sin acceso a fichas de pacientes.</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>Búsqueda web (Fierce Healthcare, PYMNTS, notas de OpenAI); adyacente a nuestro foco</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>Apps de clínicas (ej. Clínica Alemana de Valdivia)</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Familia y dependientes</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Pantalla única para gestionar salud propia y familiar (Mi Alemana Go)</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>Rediseño de la pantalla de inicio para gestionar la salud propia y la de la familia en una sola vista.</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>Ficha App Store Chile (Mi Alemana Go, 3,1/5 con 137 calificaciones)</t>
         </is>
       </c>
     </row>
@@ -9600,7 +9728,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A19"/>
+  <dimension ref="A1:A20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -9739,6 +9867,13 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Vuelta 4 (iter. 3, 2026-10-08 10:08 UTC): Apple Health, ChatGPT Health, Claude for Healthcare, Apps de clínicas verificados (+4 filas). Pendientes: Clinia, MiRedSalud, Mediko (cierran la vuelta 4 y regeneran func_norm/tabla_frecuencia).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Benchmark: cierre vuelta 4; contador=4; func_norm y tabla_frecuencia regenerados
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MVcXu8vTBu7EKfj3YdEvae
</commit_message>
<xml_diff>
--- a/Outputs/Benchmark_Anamnesis.xlsx
+++ b/Outputs/Benchmark_Anamnesis.xlsx
@@ -518,11 +518,11 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -558,11 +558,11 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -598,11 +598,11 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -638,11 +638,11 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -678,11 +678,11 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
@@ -718,11 +718,11 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -758,11 +758,11 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -798,11 +798,11 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
@@ -838,11 +838,11 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
@@ -878,11 +878,11 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
@@ -918,11 +918,11 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G12" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
@@ -958,11 +958,11 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G13" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
@@ -993,7 +993,7 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>[DIRECTO · Chile · etapa A] App móvil anunciada en sep-2026 para centralizar recetas, diagnósticos y laboratorios en un solo lugar; respaldada por Reservo (tecnológica chilena desde 2015, software para profesionales y centros de salud). AMENAZA ALTA: Reservo ya tiene red de profesionales/centros que podrían alimentar el historial. Fuente: solo snippet de búsqueda (sitio bloqueado en este entorno); precio, funciones de compartir y sitio oficial por verificar. [Vuelta 2] Confirmado por el CEO de Reservo (LinkedIn): app para pacientes en App Store y Google Play; guarda y comparte exámenes, recetas, órdenes y certificados. Fecha exacta de lanzamiento, precio y modelo de datos sin verificar. [Vuelta 3] Sin novedades de oct-2026. Reservo (Chile, México, Argentina) declara certificación Fonasa/CENS y cumplimiento de la nueva ley de datos personales; el Portal de Agendamiento de Reservo complementa a Clinia. Precio y modelo de datos sin verificar.</t>
+          <t>[DIRECTO · Chile · etapa A] App móvil anunciada en sep-2026 para centralizar recetas, diagnósticos y laboratorios en un solo lugar; respaldada por Reservo (tecnológica chilena desde 2015, software para profesionales y centros de salud). AMENAZA ALTA: Reservo ya tiene red de profesionales/centros que podrían alimentar el historial. Fuente: solo snippet de búsqueda (sitio bloqueado en este entorno); precio, funciones de compartir y sitio oficial por verificar. [Vuelta 2] Confirmado por el CEO de Reservo (LinkedIn): app para pacientes en App Store y Google Play; guarda y comparte exámenes, recetas, órdenes y certificados. Fecha exacta de lanzamiento, precio y modelo de datos sin verificar. [Vuelta 3] Sin novedades de oct-2026. Reservo (Chile, México, Argentina) declara certificación Fonasa/CENS y cumplimiento de la nueva ley de datos personales; el Portal de Agendamiento de Reservo complementa a Clinia. Precio y modelo de datos sin verificar. [Vuelta 4] Una búsqueda adicional no encontró fuentes independientes sobre Clinia de Reservo (aparecen otras empresas llamadas Clinia); la evidencia sigue siendo la publicación del CEO en LinkedIn y notas de Reservo. Confianza media.</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1002,7 +1002,7 @@
         </is>
       </c>
       <c r="G14" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
@@ -1033,7 +1033,7 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>[SUSTITUTO PARCIAL · Chile] Nueva app móvil de la red RedSalud anunciada dic-2025: acceso a información clínica y servicios, guardar y administrar historial propio y familiar. Limitación: solo datos de la propia red; no consolida otras instituciones. Precio por verificar (probablemente gratis). [Vuelta 2] La búsqueda no encontró fuentes adicionales ni ficha de la app chilena (solo una app RedSalud de otro país); funciones sin confirmar. [Vuelta 3] Rankings de terceros la ubican como app médica gratuita nº 1 en App Store y Google Play Chile (fecha desconocida); sin descripción de funciones ni confirmación del desarrollador en Google Play.</t>
+          <t>[SUSTITUTO PARCIAL · Chile] Nueva app móvil de la red RedSalud anunciada dic-2025: acceso a información clínica y servicios, guardar y administrar historial propio y familiar. Limitación: solo datos de la propia red; no consolida otras instituciones. Precio por verificar (probablemente gratis). [Vuelta 2] La búsqueda no encontró fuentes adicionales ni ficha de la app chilena (solo una app RedSalud de otro país); funciones sin confirmar. [Vuelta 3] Rankings de terceros la ubican como app médica gratuita nº 1 en App Store y Google Play Chile (fecha desconocida); sin descripción de funciones ni confirmación del desarrollador en Google Play. [Vuelta 4] Sin documentación oficial chilena localizada; las fichas con funciones (agendar, telemedicina, historial de hijos) corresponden a una app RedSalud de otro país. Quejas públicas 2020-21 sobre acceso en línea a resultados. Funciones de MiRedSalud sin confirmar.</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1042,7 +1042,7 @@
         </is>
       </c>
       <c r="G15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
@@ -1073,7 +1073,7 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>[ADYACENTE · Chile] Fundada 2022. Orientación médica inmediata, interpretación de exámenes y órdenes médicas digitales con IA; modelo freemium, suscripción y pago por servicio; menciona centralizar registros y monitoreo. Foco asistencial, no archivo personal; vigilar si añade historial. Grants por ~$40M según Descubre.vc. [Vuelta 2] Sin precios ni planes vigentes localizados; sitio oficial bloqueado. [Vuelta 3] Pauta (oct-2024): su fundador, Tomás Riddell, dice que no reemplaza a médicos y apunta a lo ambulatorio y a la espera de derivación a especialidad en el sistema público. Financiamiento: fuentes discrepan (CLP 25M en dic-2023 según Bouncewatch; ~$40M según Descubre.vc). Precios vigentes sin verificar.</t>
+          <t>[ADYACENTE · Chile] Fundada 2022. Orientación médica inmediata, interpretación de exámenes y órdenes médicas digitales con IA; modelo freemium, suscripción y pago por servicio; menciona centralizar registros y monitoreo. Foco asistencial, no archivo personal; vigilar si añade historial. Grants por ~$40M según Descubre.vc. [Vuelta 2] Sin precios ni planes vigentes localizados; sitio oficial bloqueado. [Vuelta 3] Pauta (oct-2024): su fundador, Tomás Riddell, dice que no reemplaza a médicos y apunta a lo ambulatorio y a la espera de derivación a especialidad en el sistema público. Financiamiento: fuentes discrepan (CLP 25M en dic-2023 según Bouncewatch; ~$40M según Descubre.vc). Precios vigentes sin verificar. [Vuelta 4] Entrevista oct-2024 menciona integración con la pasarela Flow. Sin novedades 2025-26 ni rondas verificadas; la cifra de US$40M de Bouncewatch es dudosa (perfil con 2 empleados).</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1082,7 +1082,7 @@
         </is>
       </c>
       <c r="G16" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
@@ -1102,7 +1102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F124"/>
+  <dimension ref="A1:F125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -5081,6 +5081,38 @@
         </is>
       </c>
     </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>Mediko</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Seguros y pagos</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Integración con la pasarela de pagos Flow</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Pagos dentro de la plataforma mediante la pasarela Flow (según resumen de entrevista de Pauta, oct-2024; esperada para mejorar la experiencia).</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>Búsqueda web (Pauta / Descubre.vc, 2024); estado actual sin verificar</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5092,7 +5124,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E114"/>
+  <dimension ref="A1:E125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -5888,7 +5920,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Clingot</t>
+          <t>Apps de clínicas (ej. Clínica Alemana de Valdivia)</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -5903,19 +5935,19 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Los padres pueden monitorear la salud de hijos pequeños.</t>
+          <t>Rediseño de la pantalla de inicio para gestionar la salud propia y la de la familia en una sola vista.</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Latam</t>
+          <t>Chile</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>MediPlanner</t>
+          <t>Clingot</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -5930,7 +5962,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Historial por perfil para cada miembro de la familia.</t>
+          <t>Los padres pueden monitorear la salud de hijos pequeños.</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -5942,7 +5974,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>MiRedSalud (RedSalud)</t>
+          <t>MediPlanner</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -5957,46 +5989,46 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Guardar y administrar historial propio y familiar.</t>
+          <t>Historial por perfil para cada miembro de la familia.</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Latam</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Clingot</t>
+          <t>MiRedSalud (RedSalud)</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Gestión documental</t>
+          <t>Familia y dependientes</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Almacenamiento de documentos médicos</t>
+          <t>Perfiles familiares / dependientes</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Sube estudios, imágenes, indicaciones médicas y notas personales; accesible en consulta o por terceros en emergencias.</t>
+          <t>Guardar y administrar historial propio y familiar.</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Latam</t>
+          <t>Chile</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Clinia (Reservo)</t>
+          <t>Clingot</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -6011,12 +6043,12 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Reúne recetas, diagnósticos y laboratorios en un solo lugar.</t>
+          <t>Sube estudios, imágenes, indicaciones médicas y notas personales; accesible en consulta o por terceros en emergencias.</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Latam</t>
         </is>
       </c>
     </row>
@@ -6038,7 +6070,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Guarda en un solo lugar exámenes, recetas, órdenes y certificados médicos.</t>
+          <t>Reúne recetas, diagnósticos y laboratorios en un solo lugar.</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -6050,7 +6082,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Healfies</t>
+          <t>Clinia (Reservo)</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -6065,19 +6097,19 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Organiza registros con carpetas y etiquetas.</t>
+          <t>Guarda en un solo lugar exámenes, recetas, órdenes y certificados médicos.</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Latam</t>
+          <t>Chile</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Meedika</t>
+          <t>Healfies</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -6092,19 +6124,19 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Almacena documentos clínicos del usuario en la app.</t>
+          <t>Organiza registros con carpetas y etiquetas.</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Latam</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Patientory</t>
+          <t>Meedika</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -6119,19 +6151,19 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Administra fechas, prescripciones, archivos y citas desde la app.</t>
+          <t>Almacena documentos clínicos del usuario en la app.</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Chile</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Apps de clínicas (ej. Clínica Alemana de Valdivia)</t>
+          <t>Patientory</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -6141,24 +6173,24 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Almacenamiento de recetas</t>
+          <t>Almacenamiento de documentos médicos</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Ver y descargar recetas, órdenes de examen y derivaciones.</t>
+          <t>Administra fechas, prescripciones, archivos y citas desde la app.</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Global</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>MediPlanner</t>
+          <t>Apps de clínicas (ej. Clínica Alemana de Valdivia)</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -6173,12 +6205,12 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Guarda recetas digitales.</t>
+          <t>Ver y descargar recetas, órdenes de examen y derivaciones.</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Latam</t>
+          <t>Chile</t>
         </is>
       </c>
     </row>
@@ -6195,12 +6227,12 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Búsqueda y filtros de documentos</t>
+          <t>Almacenamiento de recetas</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Guarda resultados de laboratorio, imágenes y PDFs; búsqueda y filtros.</t>
+          <t>Guarda recetas digitales.</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -6212,7 +6244,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>MediBloc</t>
+          <t>MediPlanner</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -6222,24 +6254,24 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Emisión de certificados médicos</t>
+          <t>Búsqueda y filtros de documentos</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>La ficha de la app incluye consulta de chequeos de salud y emisión de certificados médicos.</t>
+          <t>Guarda resultados de laboratorio, imágenes y PDFs; búsqueda y filtros.</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Latam</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Mediko</t>
+          <t>MediBloc</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -6249,24 +6281,24 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Importación de órdenes/solicitudes médicas</t>
+          <t>Emisión de certificados médicos</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Descarga/genera órdenes médicas digitales.</t>
+          <t>La ficha de la app incluye consulta de chequeos de salud y emisión de certificados médicos.</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Global</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Meedika</t>
+          <t>Mediko</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -6281,7 +6313,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Importa solicitudes (órdenes) médicas a la app.</t>
+          <t>Descarga/genera órdenes médicas digitales.</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -6293,7 +6325,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Apps de clínicas (ej. Clínica Alemana de Valdivia)</t>
+          <t>Meedika</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -6303,12 +6335,12 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Notificación y envío de resultados</t>
+          <t>Importación de órdenes/solicitudes médicas</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Avisa cuando hay exámenes/documentos disponibles; resultados de laboratorio y anatomía patológica compartibles por email o WhatsApp.</t>
+          <t>Importa solicitudes (órdenes) médicas a la app.</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -6325,17 +6357,17 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Historial y perfil clínico</t>
+          <t>Gestión documental</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Historial institucional (solo datos de la propia red)</t>
+          <t>Notificación y envío de resultados</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Ve historial de esa institución.</t>
+          <t>Avisa cuando hay exámenes/documentos disponibles; resultados de laboratorio y anatomía patológica compartibles por email o WhatsApp.</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -6362,7 +6394,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Historial institucional de consultas, urgencias y hospitalizaciones (solo datos de esa clínica).</t>
+          <t>Ve historial de esa institución.</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -6374,7 +6406,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>MiRedSalud (RedSalud)</t>
+          <t>Apps de clínicas (ej. Clínica Alemana de Valdivia)</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -6389,7 +6421,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Acceso a información clínica de la red.</t>
+          <t>Historial institucional de consultas, urgencias y hospitalizaciones (solo datos de esa clínica).</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -6401,7 +6433,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Apple Health (Health Records)</t>
+          <t>MiRedSalud (RedSalud)</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -6411,24 +6443,24 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Historial médico centralizado</t>
+          <t>Historial institucional (solo datos de la propia red)</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Información clínica unificada.</t>
+          <t>Acceso a información clínica de la red.</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Chile</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Clingot</t>
+          <t>Apple Health (Health Records)</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -6443,19 +6475,19 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>El usuario registra sus antecedentes médicos en la app.</t>
+          <t>Información clínica unificada.</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Latam</t>
+          <t>Global</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Infomed</t>
+          <t>Clingot</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -6470,19 +6502,19 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Centraliza el historial médico personal en el móvil.</t>
+          <t>El usuario registra sus antecedentes médicos en la app.</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Latam</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>MediBloc</t>
+          <t>Infomed</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -6497,19 +6529,19 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Permite compilar datos de vida/salud, gestionarlos y pasarlos a instituciones médicas.</t>
+          <t>Centraliza el historial médico personal en el móvil.</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Chile</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Mediko</t>
+          <t>MediBloc</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -6524,19 +6556,19 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Centralizar registros y monitoreo desde el móvil.</t>
+          <t>Permite compilar datos de vida/salud, gestionarlos y pasarlos a instituciones médicas.</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Global</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Healfies</t>
+          <t>Mediko</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -6546,17 +6578,17 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Línea de tiempo de salud</t>
+          <t>Historial médico centralizado</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Línea de tiempo con medicación, exámenes, citas y dieta.</t>
+          <t>Centralizar registros y monitoreo desde el móvil.</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Latam</t>
+          <t>Chile</t>
         </is>
       </c>
     </row>
@@ -6578,7 +6610,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Registra notas de medicación, exámenes (laboratorio e imagen), actividad física, recetas, dieta y citas.</t>
+          <t>Línea de tiempo con medicación, exámenes, citas y dieta.</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -6590,7 +6622,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>MediPlanner</t>
+          <t>Healfies</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -6600,12 +6632,12 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Registro de alergias y vacunas</t>
+          <t>Línea de tiempo de salud</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Registro de alergias y vacunas.</t>
+          <t>Registra notas de medicación, exámenes (laboratorio e imagen), actividad física, recetas, dieta y citas.</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -6617,27 +6649,27 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>MediBloc</t>
+          <t>MediPlanner</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Incentivos y monetización de datos</t>
+          <t>Historial y perfil clínico</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Recompensas / monetización de datos del usuario</t>
+          <t>Registro de alergias y vacunas</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Plan de convertir Medipass en superapp con gestión de salud diaria y mercado de datos, integrada con la EMR Dr.Palette.</t>
+          <t>Registro de alergias y vacunas.</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Latam</t>
         </is>
       </c>
     </row>
@@ -6649,17 +6681,17 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Incentivos y monetización de datos</t>
+          <t>Historial y perfil clínico</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Recompensas / monetización de datos del usuario</t>
+          <t>Seguimiento de visitas, gastos y seguros</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>El usuario puede agregar y monetizar sus datos; recompensas en cripto.</t>
+          <t>App gratuita para seguir visitas al médico, facturas médicas, datos personales, seguros, inmunizaciones y medicamentos de farmacia.</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -6671,22 +6703,22 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Patientory</t>
+          <t>MediBloc</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Inteligencia artificial</t>
+          <t>Incentivos y monetización de datos</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Coaching de salud con IA</t>
+          <t>Recompensas / monetización de datos del usuario</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Coaching personalizado con IA.</t>
+          <t>Plan de convertir Medipass en superapp con gestión de salud diaria y mercado de datos, integrada con la EMR Dr.Palette.</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -6698,22 +6730,22 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>ChatGPT Health (OpenAI)</t>
+          <t>Medicalchain</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Inteligencia artificial</t>
+          <t>Incentivos y monetización de datos</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Detección de patrones en métricas de salud con IA</t>
+          <t>Recompensas / monetización de datos del usuario</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Interpreta datos de Apple Health y registros en contexto y detecta cambios.</t>
+          <t>Centros de investigación y farmacéuticas recompensarían con MedTokens a quienes compartan sus datos; no confirmado como ejecutado.</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -6725,22 +6757,22 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Claude for Healthcare (Anthropic)</t>
+          <t>Patientory</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Inteligencia artificial</t>
+          <t>Incentivos y monetización de datos</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Detección de patrones en métricas de salud con IA</t>
+          <t>Recompensas / monetización de datos del usuario</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Detecta patrones entre métricas de salud y fitness.</t>
+          <t>El usuario puede agregar y monetizar sus datos; recompensas en cripto.</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -6762,12 +6794,12 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Interpretación de exámenes con IA</t>
+          <t>Asistente de IA para profesionales de salud</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Explica resultados complejos en lenguaje simple.</t>
+          <t>Producto para clínicos verificados de EE.UU. (gratis, abr-2026); desde 1-sep-2026 un plugin con nueve apps de fuentes públicas (investigación, ensayos, medicamentos, Medicare, prestadores), de solo lectura y sin acceso a fichas de pacientes.</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -6779,7 +6811,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Claude for Healthcare (Anthropic)</t>
+          <t>Patientory</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -6789,12 +6821,12 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Interpretación de exámenes con IA</t>
+          <t>Coaching de salud con IA</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Explica exámenes en lenguaje simple.</t>
+          <t>Coaching personalizado con IA.</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -6806,7 +6838,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Mediko</t>
+          <t>ChatGPT Health (OpenAI)</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -6816,24 +6848,24 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Interpretación de exámenes con IA</t>
+          <t>Detección de patrones en métricas de salud con IA</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Interpreta exámenes de laboratorio.</t>
+          <t>Interpreta datos de Apple Health y registros en contexto y detecta cambios.</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Global</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>ChatGPT Health (OpenAI)</t>
+          <t>Claude for Healthcare (Anthropic)</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -6843,12 +6875,12 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Orientación médica con IA</t>
+          <t>Detección de patrones en métricas de salud con IA</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Mejora de jun-2026 (GPT-5.5 Instant): detecta cuándo puede requerirse atención urgente, pide contexto y explica la incertidumbre.</t>
+          <t>Detecta patrones entre métricas de salud y fitness.</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -6860,7 +6892,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Mediko</t>
+          <t>ChatGPT Health (OpenAI)</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -6870,17 +6902,17 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Orientación médica con IA</t>
+          <t>Interpretación de exámenes con IA</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Orientación médica instantánea mediante IA.</t>
+          <t>Explica resultados complejos en lenguaje simple.</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Global</t>
         </is>
       </c>
     </row>
@@ -6897,12 +6929,12 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Preparación de consultas médicas con IA</t>
+          <t>Interpretación de exámenes con IA</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Prepara preguntas para el médico.</t>
+          <t>Desde 28-sep-2026, en la pestaña Health se puede elegir un gráfico, métrica o registro y obtener explicaciones basadas en los datos conectados.</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -6924,12 +6956,12 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Preparación de consultas médicas con IA</t>
+          <t>Interpretación de exámenes con IA</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Prepara preguntas para el médico.</t>
+          <t>Explica exámenes en lenguaje simple.</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -6941,7 +6973,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>ChatGPT Health (OpenAI)</t>
+          <t>Mediko</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -6951,24 +6983,24 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Resumen de historial con IA</t>
+          <t>Interpretación de exámenes con IA</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Resume instrucciones de atención.</t>
+          <t>Interpreta exámenes de laboratorio.</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Chile</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Claude for Healthcare (Anthropic)</t>
+          <t>ChatGPT Health (OpenAI)</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -6978,12 +7010,12 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Resumen de historial con IA</t>
+          <t>Orientación médica con IA</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Resume el historial del usuario.</t>
+          <t>Mejora de jun-2026 (GPT-5.5 Instant): detecta cuándo puede requerirse atención urgente, pide contexto y explica la incertidumbre.</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -6995,27 +7027,27 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Apple Health (Health Records)</t>
+          <t>Mediko</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Interoperabilidad y fuentes de datos</t>
+          <t>Inteligencia artificial</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Agregación de registros de múltiples instituciones</t>
+          <t>Orientación médica con IA</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Vista central de alergias, condiciones, vacunas, laboratorio, medicación, procedimientos y signos vitales.</t>
+          <t>Orientación médica instantánea mediante IA.</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Chile</t>
         </is>
       </c>
     </row>
@@ -7027,17 +7059,17 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Interoperabilidad y fuentes de datos</t>
+          <t>Inteligencia artificial</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Agregación de registros de múltiples instituciones</t>
+          <t>Preparación de consultas médicas con IA</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Conexión de historiales electrónicos y apps como Apple Health, MyFitnessPal, Peloton.</t>
+          <t>Prepara preguntas para el médico.</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -7049,22 +7081,22 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>ChatGPT Health (OpenAI)</t>
+          <t>Claude for Healthcare (Anthropic)</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Interoperabilidad y fuentes de datos</t>
+          <t>Inteligencia artificial</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Agregación de registros de múltiples instituciones</t>
+          <t>Preparación de consultas médicas con IA</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Acceso a historiales electrónicos de proveedores de EE.UU. vía b.well; solo EE.UU., sin plazo anunciado para Latinoamérica.</t>
+          <t>Prepara preguntas para el médico.</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -7081,17 +7113,17 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Interoperabilidad y fuentes de datos</t>
+          <t>Inteligencia artificial</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Agregación de registros de múltiples instituciones</t>
+          <t>Resumen de historial con IA</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Además de b.well y Apple Health, vincula registros de One Medical y Function Health (solo EE.UU., Free/Go/Plus/Pro, web e iOS).</t>
+          <t>Resume instrucciones de atención.</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -7108,17 +7140,17 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Interoperabilidad y fuentes de datos</t>
+          <t>Inteligencia artificial</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Agregación de registros de múltiples instituciones</t>
+          <t>Resumen de historial con IA</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Acceso a resultados y registros de salud (beta, Pro/Max, EE.UU.).</t>
+          <t>Resume el historial del usuario.</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -7130,7 +7162,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Clinia (Reservo)</t>
+          <t>Apple Health (Health Records)</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -7145,19 +7177,19 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Datos desde profesionales/centros que usan Reservo (fichas clínicas, agenda, telemedicina).</t>
+          <t>Vista central de alergias, condiciones, vacunas, laboratorio, medicación, procedimientos y signos vitales.</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Global</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>MediBloc</t>
+          <t>ChatGPT Health (OpenAI)</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -7172,7 +7204,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Tras autenticación simple, trae los últimos 3 años de historial de hospitales integrados (p. ej. Samsung Seoul, SNUH, Severance).</t>
+          <t>Conexión de historiales electrónicos y apps como Apple Health, MyFitnessPal, Peloton.</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -7184,7 +7216,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Meedika</t>
+          <t>ChatGPT Health (OpenAI)</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -7199,19 +7231,19 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Sincroniza resultados desde centros de salud y permite subir fotos o documentos de las solicitudes médicas.</t>
+          <t>Acceso a historiales electrónicos de proveedores de EE.UU. vía b.well; solo EE.UU., sin plazo anunciado para Latinoamérica.</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Global</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Patientory</t>
+          <t>ChatGPT Health (OpenAI)</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -7226,7 +7258,7 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Reúne registros de hospitales, resultados de laboratorio y datos genómicos.</t>
+          <t>Además de b.well y Apple Health, vincula registros de One Medical y Function Health (solo EE.UU., Free/Go/Plus/Pro, web e iOS).</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -7238,7 +7270,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Patientory</t>
+          <t>Claude for Healthcare (Anthropic)</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -7248,12 +7280,12 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Analítica poblacional B2B</t>
+          <t>Agregación de registros de múltiples instituciones</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Analítica poblacional on-chain; integrada con Epic, Cerner, Meditech y Allscripts (B2B).</t>
+          <t>Acceso a resultados y registros de salud (beta, Pro/Max, EE.UU.).</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
@@ -7265,7 +7297,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Clingot</t>
+          <t>Clinia (Reservo)</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -7275,24 +7307,24 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Disponibilidad multiplataforma (web/iOS/Android)</t>
+          <t>Agregación de registros de múltiples instituciones</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Android, iOS y escritorio; médicos acceden a historias digitalizadas, envían estudios e indicaciones y organizan agenda.</t>
+          <t>Datos desde profesionales/centros que usan Reservo (fichas clínicas, agenda, telemedicina).</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Latam</t>
+          <t>Chile</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Clinia (Reservo)</t>
+          <t>MediBloc</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -7302,24 +7334,24 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Disponibilidad multiplataforma (web/iOS/Android)</t>
+          <t>Agregación de registros de múltiples instituciones</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Disponible en App Store y Google Play. Reservo opera en Chile, México y Argentina y está certificada por FONASA y CENS.</t>
+          <t>Tras autenticación simple, trae los últimos 3 años de historial de hospitales integrados (p. ej. Samsung Seoul, SNUH, Severance).</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Global</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Healfies</t>
+          <t>Meedika</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -7329,24 +7361,24 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Disponibilidad multiplataforma (web/iOS/Android)</t>
+          <t>Agregación de registros de múltiples instituciones</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Disponible en web, iOS y Android.</t>
+          <t>Sincroniza resultados desde centros de salud y permite subir fotos o documentos de las solicitudes médicas.</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Latam</t>
+          <t>Chile</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Medicalchain</t>
+          <t>Patientory</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -7356,12 +7388,12 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Historial médico centralizado</t>
+          <t>Agregación de registros de múltiples instituciones</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Versión digital de los registros con acceso por móvil o web.</t>
+          <t>Reúne registros de hospitales, resultados de laboratorio y datos genómicos.</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -7373,7 +7405,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>MediPlanner</t>
+          <t>Patientory</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -7383,24 +7415,24 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Importación y exportación de datos</t>
+          <t>Analítica poblacional B2B</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Importar/exportar datos para compartir de forma segura con familias o cuidadores. Es MediPlanner Pro, de otro desarrollador (App Store MX, $39 MXN).</t>
+          <t>Analítica poblacional on-chain; integrada con Epic, Cerner, Meditech y Allscripts (B2B).</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Latam</t>
+          <t>Global</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Claude for Healthcare (Anthropic)</t>
+          <t>Clingot</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -7410,24 +7442,24 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Integración con wearables y apps de salud</t>
+          <t>Disponibilidad multiplataforma (web/iOS/Android)</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Integración beta en apps iOS/Android.</t>
+          <t>Android, iOS y escritorio; médicos acceden a historias digitalizadas, envían estudios e indicaciones y organizan agenda.</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Latam</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Claude for Healthcare (Anthropic)</t>
+          <t>Clinia (Reservo)</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -7437,24 +7469,24 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Integración con wearables y apps de salud</t>
+          <t>Disponibilidad multiplataforma (web/iOS/Android)</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Integración beta con Health Connect en la app móvil; conectores de registros (HealthEx, Function) solo para Pro/Max en EE.UU.</t>
+          <t>Disponible en App Store y Google Play. Reservo opera en Chile, México y Argentina y está certificada por FONASA y CENS.</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Chile</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Patientory</t>
+          <t>Healfies</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -7464,39 +7496,39 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Integración con wearables y apps de salud</t>
+          <t>Disponibilidad multiplataforma (web/iOS/Android)</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Se integra con wearables y apps móviles populares y muestra vitales en un panel unificado.</t>
+          <t>Disponible en web, iOS y Android.</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Latam</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Apple Health (Health Records)</t>
+          <t>Medicalchain</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Medicación y recordatorios</t>
+          <t>Interoperabilidad y fuentes de datos</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Gestión de lista de medicamentos</t>
+          <t>Historial médico centralizado</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Listas de medicamentos, vitaminas y suplementos con horarios; escaneo de etiqueta del frasco solo en EE.UU.</t>
+          <t>Versión digital de los registros con acceso por móvil o web.</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
@@ -7508,135 +7540,135 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Apple Health (Health Records)</t>
+          <t>MediPlanner</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Medicación y recordatorios</t>
+          <t>Interoperabilidad y fuentes de datos</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Recordatorios de medicación y citas</t>
+          <t>Importación y exportación de datos</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Recordatorios desde el app.</t>
+          <t>Importar/exportar datos para compartir de forma segura con familias o cuidadores. Es MediPlanner Pro, de otro desarrollador (App Store MX, $39 MXN).</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Latam</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Meedika</t>
+          <t>Medicalchain</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Medicación y recordatorios</t>
+          <t>Interoperabilidad y fuentes de datos</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Recordatorios de medicación y citas</t>
+          <t>Integración con EHR de proveedores</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Recordatorios de citas/medicación.</t>
+          <t>Según una AMA sin fecha, integraba dos sistemas de GP que cubren ~80% del mercado UK; no confirmado como ejecutado.</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Global</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>MediPlanner</t>
+          <t>Claude for Healthcare (Anthropic)</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Medicación y recordatorios</t>
+          <t>Interoperabilidad y fuentes de datos</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Registro de tomas y adherencia al tratamiento</t>
+          <t>Integración con wearables y apps de salud</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Registro de cada toma y control de adherencia; gestiona medicamentos propios y de familiares.</t>
+          <t>Integración beta en apps iOS/Android.</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Latam</t>
+          <t>Global</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Infomed</t>
+          <t>Claude for Healthcare (Anthropic)</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Seguimiento y bienestar</t>
+          <t>Interoperabilidad y fuentes de datos</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Contenido educativo sobre salud</t>
+          <t>Integración con wearables y apps de salud</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Busca que el paciente aprenda sobre sus enfermedades y sea más autónomo.</t>
+          <t>Integración beta con Health Connect en la app móvil; conectores de registros (HealthEx, Function) solo para Pro/Max en EE.UU.</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Global</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>MediPlanner</t>
+          <t>Patientory</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Seguimiento y bienestar</t>
+          <t>Interoperabilidad y fuentes de datos</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Gráficas de evolución de indicadores</t>
+          <t>Integración con wearables y apps de salud</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Gráficas de evolución de indicadores de salud.</t>
+          <t>Se integra con wearables y apps móviles populares y muestra vitales en un panel unificado.</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Latam</t>
+          <t>Global</t>
         </is>
       </c>
     </row>
@@ -7648,17 +7680,17 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Seguimiento y bienestar</t>
+          <t>Medicación y recordatorios</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Integración con wearables y apps de salud</t>
+          <t>Gestión de lista de medicamentos</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Datos de pasos, sueño, peso junto a registros.</t>
+          <t>Listas de medicamentos, vitaminas y suplementos con horarios; escaneo de etiqueta del frasco solo en EE.UU.</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
@@ -7670,27 +7702,27 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Patientory</t>
+          <t>MediPlanner</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Seguimiento y bienestar</t>
+          <t>Medicación y recordatorios</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Panel de seguimiento de salud y bienestar</t>
+          <t>Importación automática de tratamientos desde receta digital</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Seguimiento de hábitos saludables y monitoreo de progreso.</t>
+          <t>Según la ficha de la App Store MX, los tratamientos llegan automáticamente desde la receta digital del médico (autodeclarado, sin verificar).</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Latam</t>
         </is>
       </c>
     </row>
@@ -7702,17 +7734,17 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Seguimiento y bienestar</t>
+          <t>Medicación y recordatorios</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Registro de nutrición</t>
+          <t>Recordatorios de medicación y citas</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Escaneo de etiquetas nutricionales con la cámara; según un análisis, no escribe en HealthKit.</t>
+          <t>Recordatorios desde el app.</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
@@ -7724,49 +7756,49 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Apple Health (Health Records)</t>
+          <t>Meedika</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Seguimiento y bienestar</t>
+          <t>Medicación y recordatorios</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Seguimiento de salud femenina</t>
+          <t>Recordatorios de medicación y citas</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Extiende el seguimiento de ciclo con perimenopausia y menopausia.</t>
+          <t>Recordatorios de citas/medicación.</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Chile</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Clingot</t>
+          <t>MediPlanner</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Seguimiento y bienestar</t>
+          <t>Medicación y recordatorios</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Valoración de profesionales</t>
+          <t>Registro de tomas y adherencia al tratamiento</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Calificación de la atención de profesionales con autorización previa, compartible con otros usuarios.</t>
+          <t>Registro de cada toma y control de adherencia; gestiona medicamentos propios y de familiares.</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
@@ -7778,22 +7810,22 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>MediBloc</t>
+          <t>Patientory</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Seguridad, privacidad y blockchain</t>
+          <t>Seguimiento y bienestar</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Blockchain para integridad y trazabilidad de datos</t>
+          <t>Comunidad de pacientes</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Blockchain propia (Cosmos SDK) para que el paciente almacene, use, actualice y transfiera sus registros; los datos no se guardan en la cadena, solo en el usuario, cifrados.</t>
+          <t>Los usuarios con condiciones similares pueden preguntar, recibir recomendaciones y compartir experiencias.</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
@@ -7805,76 +7837,76 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>MediBloc</t>
+          <t>Infomed</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Seguridad, privacidad y blockchain</t>
+          <t>Seguimiento y bienestar</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Blockchain para integridad y trazabilidad de datos</t>
+          <t>Contenido educativo sobre salud</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Almacena huellas de datos médicos en un registro de solo escritura, sin guardar datos clínicos en cadena.</t>
+          <t>Busca que el paciente aprenda sobre sus enfermedades y sea más autónomo.</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Chile</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Medicalchain</t>
+          <t>MediPlanner</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Seguridad, privacidad y blockchain</t>
+          <t>Seguimiento y bienestar</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Blockchain para integridad y trazabilidad de datos</t>
+          <t>Gráficas de evolución de indicadores</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Cada solicitud de acceso queda en un libro distribuido; acceso temporal por contratos inteligentes.</t>
+          <t>Gráficas de evolución de indicadores de salud.</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Latam</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Patientory</t>
+          <t>Apple Health (Health Records)</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Seguridad, privacidad y blockchain</t>
+          <t>Seguimiento y bienestar</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Blockchain para integridad y trazabilidad de datos</t>
+          <t>Integración con wearables y apps de salud</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Registro respaldado en blockchain para seguridad y trazabilidad.</t>
+          <t>Datos de pasos, sueño, peso junto a registros.</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
@@ -7886,22 +7918,22 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Apple Health (Health Records)</t>
+          <t>Patientory</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Seguridad, privacidad y blockchain</t>
+          <t>Seguimiento y bienestar</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Cifrado y control de acceso</t>
+          <t>Panel de seguimiento de salud y bienestar</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Registros cifrados en el dispositivo, protegidos por Face ID/Touch ID/código.</t>
+          <t>Seguimiento de hábitos saludables y monitoreo de progreso.</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
@@ -7913,88 +7945,88 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Infomed</t>
+          <t>Apple Health (Health Records)</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Seguridad, privacidad y blockchain</t>
+          <t>Seguimiento y bienestar</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Cifrado y control de acceso</t>
+          <t>Registro de nutrición</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Almacenamiento seguro del historial con criterios de seguridad estrictos, comparable a apps bancarias.</t>
+          <t>Escaneo de etiquetas nutricionales con la cámara; según un análisis, no escribe en HealthKit.</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Global</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Clinia (Reservo)</t>
+          <t>Apple Health (Health Records)</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Seguridad, privacidad y blockchain</t>
+          <t>Seguimiento y bienestar</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Cumplimiento regulatorio de salud y datos</t>
+          <t>Seguimiento de salud femenina</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Reservo declara plataforma certificada por Fonasa y CENS, cumplimiento de estándares de telemedicina del Minsal y de la nueva ley chilena de datos personales (declaración de la empresa).</t>
+          <t>Extiende el seguimiento de ciclo con perimenopausia y menopausia.</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Global</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>MediBloc</t>
+          <t>Clingot</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Seguridad, privacidad y blockchain</t>
+          <t>Seguimiento y bienestar</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Identidad descentralizada (DID)</t>
+          <t>Valoración de profesionales</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Gestión de identificadores descentralizados en Panacea.</t>
+          <t>Calificación de la atención de profesionales con autorización previa, compartible con otros usuarios.</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Latam</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>ChatGPT Health (OpenAI)</t>
+          <t>MediBloc</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -8004,12 +8036,12 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Privacidad reforzada para datos de salud</t>
+          <t>Blockchain para integridad y trazabilidad de datos</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Chats y memoria de salud separados, no usados para entrenar modelos.</t>
+          <t>Blockchain propia (Cosmos SDK) para que el paciente almacene, use, actualice y transfiera sus registros; los datos no se guardan en la cadena, solo en el usuario, cifrados.</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
@@ -8021,7 +8053,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Claude for Healthcare (Anthropic)</t>
+          <t>MediBloc</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -8031,12 +8063,12 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Privacidad reforzada para datos de salud</t>
+          <t>Blockchain para integridad y trazabilidad de datos</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>El usuario activa y revoca permisos; los datos de salud compartidos se excluyen de la memoria de Claude y del entrenamiento.</t>
+          <t>Almacena huellas de datos médicos en un registro de solo escritura, sin guardar datos clínicos en cadena.</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
@@ -8048,49 +8080,49 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Mediko</t>
+          <t>Medicalchain</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Seguros y pagos</t>
+          <t>Seguridad, privacidad y blockchain</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Modelo freemium y suscripción</t>
+          <t>Blockchain para integridad y trazabilidad de datos</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Planes para personas y empresas.</t>
+          <t>Cada solicitud de acceso queda en un libro distribuido; acceso temporal por contratos inteligentes.</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Global</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Medicalchain</t>
+          <t>Patientory</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Seguros y pagos</t>
+          <t>Seguridad, privacidad y blockchain</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Pagos con criptomoneda</t>
+          <t>Blockchain para integridad y trazabilidad de datos</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Pago de consultas con token.</t>
+          <t>Registro respaldado en blockchain para seguridad y trazabilidad.</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
@@ -8102,22 +8134,22 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>MediBloc</t>
+          <t>Apple Health (Health Records)</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Seguros y pagos</t>
+          <t>Seguridad, privacidad y blockchain</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Reclamos y trámites con seguros</t>
+          <t>Cifrado y control de acceso</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Simplifica el envío a aseguradoras sin gestionar papeles en hospitales.</t>
+          <t>Registros cifrados en el dispositivo, protegidos por Face ID/Touch ID/código.</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
@@ -8129,52 +8161,349 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>MediBloc</t>
+          <t>Infomed</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Seguros y pagos</t>
+          <t>Seguridad, privacidad y blockchain</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Reclamos y trámites con seguros</t>
+          <t>Cifrado y control de acceso</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Reclamo de seguro médico (indemnización) desde la app, con verificación de autenticidad de los registros vía blockchain por la aseguradora.</t>
+          <t>Almacenamiento seguro del historial con criterios de seguridad estrictos, comparable a apps bancarias.</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Chile</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
+          <t>Clinia (Reservo)</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Seguridad, privacidad y blockchain</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Cumplimiento regulatorio de salud y datos</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>Reservo declara plataforma certificada por Fonasa y CENS, cumplimiento de estándares de telemedicina del Minsal y de la nueva ley chilena de datos personales (declaración de la empresa).</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>ChatGPT Health (OpenAI)</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Seguridad, privacidad y blockchain</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Gestión de consentimiento sobre uso de datos</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>Desde 14-sep-2026, las nuevas conexiones heredan la configuración global de plugins: ChatGPT puede usar datos de Health sin pedir permiso cada vez salvo acciones sensibles (web primero, móvil después).</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>MediBloc</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Seguridad, privacidad y blockchain</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Identidad descentralizada (DID)</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>Gestión de identificadores descentralizados en Panacea.</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>ChatGPT Health (OpenAI)</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Seguridad, privacidad y blockchain</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Privacidad reforzada para datos de salud</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>Chats y memoria de salud separados, no usados para entrenar modelos.</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>Claude for Healthcare (Anthropic)</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Seguridad, privacidad y blockchain</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Privacidad reforzada para datos de salud</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>El usuario activa y revoca permisos; los datos de salud compartidos se excluyen de la memoria de Claude y del entrenamiento.</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Mediko</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Seguros y pagos</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Modelo freemium y suscripción</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>Planes para personas y empresas.</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
           <t>Medicalchain</t>
         </is>
       </c>
-      <c r="B114" t="inlineStr">
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Seguros y pagos</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Pagos con criptomoneda</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>Pago de consultas con token.</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>Medicalchain</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>Seguros y pagos</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Pagos con criptomoneda</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>Piloto en New Malden (Londres): consultas por video pagables con tarjeta o con MedTokens.</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>Mediko</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>Seguros y pagos</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Pagos dentro de la app</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>Pagos dentro de la plataforma mediante la pasarela Flow (según resumen de entrevista de Pauta, oct-2024; esperada para mejorar la experiencia).</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>MediBloc</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Seguros y pagos</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Reclamos y trámites con seguros</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>Simplifica el envío a aseguradoras sin gestionar papeles en hospitales.</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>MediBloc</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Seguros y pagos</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Reclamos y trámites con seguros</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>Reclamo de seguro médico (indemnización) desde la app, con verificación de autenticidad de los registros vía blockchain por la aseguradora.</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>Medicalchain</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
         <is>
           <t>Telemedicina y atención remota</t>
         </is>
       </c>
-      <c r="C114" t="inlineStr">
+      <c r="C125" t="inlineStr">
         <is>
           <t>Teleconsulta con profesionales</t>
         </is>
       </c>
-      <c r="D114" t="inlineStr">
+      <c r="D125" t="inlineStr">
         <is>
           <t>Teleconsultas con GP.</t>
         </is>
       </c>
-      <c r="E114" t="inlineStr">
+      <c r="E125" t="inlineStr">
         <is>
           <t>Global</t>
         </is>
@@ -8191,7 +8520,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R57"/>
+  <dimension ref="A1:R64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8317,6 +8646,8 @@
           <t>Búsqueda de profesionales de salud</t>
         </is>
       </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
           <t>✓</t>
@@ -8327,6 +8658,17 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr"/>
       <c r="R2">
         <f>COUNTIF(C2:Q2,"✓")</f>
         <v/>
@@ -8348,11 +8690,24 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr"/>
       <c r="R3">
         <f>COUNTIF(C3:Q3,"✓")</f>
         <v/>
@@ -8369,11 +8724,25 @@
           <t>Integración con calendario del dispositivo</t>
         </is>
       </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr"/>
       <c r="R4">
         <f>COUNTIF(C4:Q4,"✓")</f>
         <v/>
@@ -8390,11 +8759,25 @@
           <t>Localización de centros médicos y farmacias</t>
         </is>
       </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr"/>
       <c r="R5">
         <f>COUNTIF(C5:Q5,"✓")</f>
         <v/>
@@ -8411,6 +8794,17 @@
           <t>Reserva de citas médicas</t>
         </is>
       </c>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr">
         <is>
           <t>✓</t>
@@ -8421,6 +8815,8 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr"/>
       <c r="R6">
         <f>COUNTIF(C6:Q6,"✓")</f>
         <v/>
@@ -8437,11 +8833,25 @@
           <t>Acceso del profesional al historial del paciente</t>
         </is>
       </c>
+      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr"/>
+      <c r="Q7" t="inlineStr"/>
       <c r="R7">
         <f>COUNTIF(C7:Q7,"✓")</f>
         <v/>
@@ -8458,11 +8868,25 @@
           <t>Compartir con personas sin cuenta mediante clave segura</t>
         </is>
       </c>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr"/>
+      <c r="Q8" t="inlineStr"/>
       <c r="R8">
         <f>COUNTIF(C8:Q8,"✓")</f>
         <v/>
@@ -8479,11 +8903,25 @@
           <t>Compartir datos con cuidador o persona de confianza</t>
         </is>
       </c>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr"/>
+      <c r="Q9" t="inlineStr"/>
       <c r="R9">
         <f>COUNTIF(C9:Q9,"✓")</f>
         <v/>
@@ -8505,11 +8943,13 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
           <t>✓</t>
@@ -8535,11 +8975,16 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
       <c r="O10" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="P10" t="inlineStr"/>
+      <c r="Q10" t="inlineStr"/>
       <c r="R10">
         <f>COUNTIF(C10:Q10,"✓")</f>
         <v/>
@@ -8556,11 +9001,25 @@
           <t>Gestión de consentimiento sobre uso de datos</t>
         </is>
       </c>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr"/>
       <c r="R11">
         <f>COUNTIF(C11:Q11,"✓")</f>
         <v/>
@@ -8577,11 +9036,25 @@
           <t>Ingreso de datos por profesional con consentimiento</t>
         </is>
       </c>
+      <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr"/>
+      <c r="Q12" t="inlineStr"/>
       <c r="R12">
         <f>COUNTIF(C12:Q12,"✓")</f>
         <v/>
@@ -8598,11 +9071,25 @@
           <t>Red social con profesionales y familiares</t>
         </is>
       </c>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr"/>
+      <c r="Q13" t="inlineStr"/>
       <c r="R13">
         <f>COUNTIF(C13:Q13,"✓")</f>
         <v/>
@@ -8629,11 +9116,23 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr"/>
+      <c r="O14" t="inlineStr"/>
+      <c r="P14" t="inlineStr"/>
+      <c r="Q14" t="inlineStr"/>
       <c r="R14">
         <f>COUNTIF(C14:Q14,"✓")</f>
         <v/>
@@ -8650,6 +9149,8 @@
           <t>Perfiles familiares / dependientes</t>
         </is>
       </c>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
           <t>✓</t>
@@ -8660,16 +9161,25 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr"/>
       <c r="N15" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="Q15" t="inlineStr"/>
       <c r="R15">
         <f>COUNTIF(C15:Q15,"✓")</f>
         <v/>
@@ -8691,6 +9201,8 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
           <t>✓</t>
@@ -8706,11 +9218,19 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="inlineStr"/>
       <c r="O16" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="P16" t="inlineStr"/>
+      <c r="Q16" t="inlineStr"/>
       <c r="R16">
         <f>COUNTIF(C16:Q16,"✓")</f>
         <v/>
@@ -8727,16 +9247,29 @@
           <t>Almacenamiento de recetas</t>
         </is>
       </c>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr"/>
       <c r="N17" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="O17" t="inlineStr"/>
+      <c r="P17" t="inlineStr"/>
+      <c r="Q17" t="inlineStr"/>
       <c r="R17">
         <f>COUNTIF(C17:Q17,"✓")</f>
         <v/>
@@ -8753,11 +9286,25 @@
           <t>Búsqueda y filtros de documentos</t>
         </is>
       </c>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="inlineStr"/>
+      <c r="O18" t="inlineStr"/>
+      <c r="P18" t="inlineStr"/>
+      <c r="Q18" t="inlineStr"/>
       <c r="R18">
         <f>COUNTIF(C18:Q18,"✓")</f>
         <v/>
@@ -8774,11 +9321,25 @@
           <t>Emisión de certificados médicos</t>
         </is>
       </c>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="inlineStr"/>
+      <c r="O19" t="inlineStr"/>
+      <c r="P19" t="inlineStr"/>
+      <c r="Q19" t="inlineStr"/>
       <c r="R19">
         <f>COUNTIF(C19:Q19,"✓")</f>
         <v/>
@@ -8800,6 +9361,19 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="inlineStr"/>
+      <c r="O20" t="inlineStr"/>
+      <c r="P20" t="inlineStr"/>
       <c r="Q20" t="inlineStr">
         <is>
           <t>✓</t>
@@ -8821,11 +9395,25 @@
           <t>Notificación y envío de resultados</t>
         </is>
       </c>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr"/>
       <c r="N21" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="O21" t="inlineStr"/>
+      <c r="P21" t="inlineStr"/>
+      <c r="Q21" t="inlineStr"/>
       <c r="R21">
         <f>COUNTIF(C21:Q21,"✓")</f>
         <v/>
@@ -8842,16 +9430,29 @@
           <t>Historial institucional (solo datos de la propia red)</t>
         </is>
       </c>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr"/>
       <c r="N22" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="O22" t="inlineStr"/>
       <c r="P22" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="Q22" t="inlineStr"/>
       <c r="R22">
         <f>COUNTIF(C22:Q22,"✓")</f>
         <v/>
@@ -8868,26 +9469,36 @@
           <t>Historial médico centralizado</t>
         </is>
       </c>
+      <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr"/>
+      <c r="N23" t="inlineStr"/>
+      <c r="O23" t="inlineStr"/>
+      <c r="P23" t="inlineStr"/>
       <c r="Q23" t="inlineStr">
         <is>
           <t>✓</t>
@@ -8909,11 +9520,25 @@
           <t>Línea de tiempo de salud</t>
         </is>
       </c>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="inlineStr"/>
+      <c r="O24" t="inlineStr"/>
+      <c r="P24" t="inlineStr"/>
+      <c r="Q24" t="inlineStr"/>
       <c r="R24">
         <f>COUNTIF(C24:Q24,"✓")</f>
         <v/>
@@ -8930,11 +9555,25 @@
           <t>Registro de alergias y vacunas</t>
         </is>
       </c>
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" t="inlineStr"/>
+      <c r="O25" t="inlineStr"/>
+      <c r="P25" t="inlineStr"/>
+      <c r="Q25" t="inlineStr"/>
       <c r="R25">
         <f>COUNTIF(C25:Q25,"✓")</f>
         <v/>
@@ -8943,24 +9582,33 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Incentivos y monetización de datos</t>
+          <t>Historial y perfil clínico</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Recompensas / monetización de datos del usuario</t>
-        </is>
-      </c>
+          <t>Seguimiento de visitas, gastos y seguros</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" t="inlineStr"/>
+      <c r="O26" t="inlineStr"/>
+      <c r="P26" t="inlineStr"/>
+      <c r="Q26" t="inlineStr"/>
       <c r="R26">
         <f>COUNTIF(C26:Q26,"✓")</f>
         <v/>
@@ -8969,19 +9617,41 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Inteligencia artificial</t>
+          <t>Incentivos y monetización de datos</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Coaching de salud con IA</t>
-        </is>
-      </c>
+          <t>Recompensas / monetización de datos del usuario</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr"/>
+      <c r="N27" t="inlineStr"/>
+      <c r="O27" t="inlineStr"/>
+      <c r="P27" t="inlineStr"/>
+      <c r="Q27" t="inlineStr"/>
       <c r="R27">
         <f>COUNTIF(C27:Q27,"✓")</f>
         <v/>
@@ -8995,19 +9665,28 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Detección de patrones en métricas de salud con IA</t>
-        </is>
-      </c>
+          <t>Asistente de IA para profesionales de salud</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="M28" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="M28" t="inlineStr"/>
+      <c r="N28" t="inlineStr"/>
+      <c r="O28" t="inlineStr"/>
+      <c r="P28" t="inlineStr"/>
+      <c r="Q28" t="inlineStr"/>
       <c r="R28">
         <f>COUNTIF(C28:Q28,"✓")</f>
         <v/>
@@ -9021,24 +9700,28 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Interpretación de exámenes con IA</t>
-        </is>
-      </c>
-      <c r="L29" t="inlineStr">
+          <t>Coaching de salud con IA</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr"/>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="M29" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Q29" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr"/>
+      <c r="L29" t="inlineStr"/>
+      <c r="M29" t="inlineStr"/>
+      <c r="N29" t="inlineStr"/>
+      <c r="O29" t="inlineStr"/>
+      <c r="P29" t="inlineStr"/>
+      <c r="Q29" t="inlineStr"/>
       <c r="R29">
         <f>COUNTIF(C29:Q29,"✓")</f>
         <v/>
@@ -9052,19 +9735,32 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Orientación médica con IA</t>
-        </is>
-      </c>
+          <t>Detección de patrones en métricas de salud con IA</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="Q30" t="inlineStr">
+      <c r="M30" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="N30" t="inlineStr"/>
+      <c r="O30" t="inlineStr"/>
+      <c r="P30" t="inlineStr"/>
+      <c r="Q30" t="inlineStr"/>
       <c r="R30">
         <f>COUNTIF(C30:Q30,"✓")</f>
         <v/>
@@ -9078,15 +9774,32 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Preparación de consultas médicas con IA</t>
-        </is>
-      </c>
+          <t>Interpretación de exámenes con IA</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr"/>
+      <c r="O31" t="inlineStr"/>
+      <c r="P31" t="inlineStr"/>
+      <c r="Q31" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -9104,15 +9817,28 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Resumen de historial con IA</t>
-        </is>
-      </c>
+          <t>Orientación médica con IA</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="M32" t="inlineStr">
+      <c r="M32" t="inlineStr"/>
+      <c r="N32" t="inlineStr"/>
+      <c r="O32" t="inlineStr"/>
+      <c r="P32" t="inlineStr"/>
+      <c r="Q32" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -9125,49 +9851,37 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Interoperabilidad y fuentes de datos</t>
+          <t>Inteligencia artificial</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Agregación de registros de múltiples instituciones</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
+          <t>Preparación de consultas médicas con IA</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr"/>
+      <c r="L33" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr">
+      <c r="M33" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="I33" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="K33" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="L33" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="M33" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="O33" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="N33" t="inlineStr"/>
+      <c r="O33" t="inlineStr"/>
+      <c r="P33" t="inlineStr"/>
+      <c r="Q33" t="inlineStr"/>
       <c r="R33">
         <f>COUNTIF(C33:Q33,"✓")</f>
         <v/>
@@ -9176,19 +9890,37 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Interoperabilidad y fuentes de datos</t>
+          <t>Inteligencia artificial</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Analítica poblacional B2B</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr">
+          <t>Resumen de historial con IA</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="inlineStr"/>
+      <c r="K34" t="inlineStr"/>
+      <c r="L34" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr"/>
+      <c r="O34" t="inlineStr"/>
+      <c r="P34" t="inlineStr"/>
+      <c r="Q34" t="inlineStr"/>
       <c r="R34">
         <f>COUNTIF(C34:Q34,"✓")</f>
         <v/>
@@ -9202,24 +9934,52 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Disponibilidad multiplataforma (web/iOS/Android)</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
+          <t>Agregación de registros de múltiples instituciones</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr">
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr"/>
       <c r="O35" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="P35" t="inlineStr"/>
+      <c r="Q35" t="inlineStr"/>
       <c r="R35">
         <f>COUNTIF(C35:Q35,"✓")</f>
         <v/>
@@ -9233,14 +9993,28 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Historial médico centralizado</t>
-        </is>
-      </c>
-      <c r="J36" t="inlineStr">
+          <t>Analítica poblacional B2B</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr"/>
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="inlineStr"/>
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="I36" t="inlineStr"/>
+      <c r="J36" t="inlineStr"/>
+      <c r="K36" t="inlineStr"/>
+      <c r="L36" t="inlineStr"/>
+      <c r="M36" t="inlineStr"/>
+      <c r="N36" t="inlineStr"/>
+      <c r="O36" t="inlineStr"/>
+      <c r="P36" t="inlineStr"/>
+      <c r="Q36" t="inlineStr"/>
       <c r="R36">
         <f>COUNTIF(C36:Q36,"✓")</f>
         <v/>
@@ -9254,14 +10028,36 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Importación y exportación de datos</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
+          <t>Disponibilidad multiplataforma (web/iOS/Android)</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr"/>
+      <c r="D37" t="inlineStr"/>
+      <c r="E37" t="inlineStr"/>
+      <c r="F37" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr"/>
+      <c r="J37" t="inlineStr"/>
+      <c r="K37" t="inlineStr"/>
+      <c r="L37" t="inlineStr"/>
+      <c r="M37" t="inlineStr"/>
+      <c r="N37" t="inlineStr"/>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr"/>
+      <c r="Q37" t="inlineStr"/>
       <c r="R37">
         <f>COUNTIF(C37:Q37,"✓")</f>
         <v/>
@@ -9275,19 +10071,28 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Integración con wearables y apps de salud</t>
-        </is>
-      </c>
-      <c r="H38" t="inlineStr">
+          <t>Historial médico centralizado</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr"/>
+      <c r="D38" t="inlineStr"/>
+      <c r="E38" t="inlineStr"/>
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" t="inlineStr"/>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr"/>
+      <c r="J38" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="M38" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="K38" t="inlineStr"/>
+      <c r="L38" t="inlineStr"/>
+      <c r="M38" t="inlineStr"/>
+      <c r="N38" t="inlineStr"/>
+      <c r="O38" t="inlineStr"/>
+      <c r="P38" t="inlineStr"/>
+      <c r="Q38" t="inlineStr"/>
       <c r="R38">
         <f>COUNTIF(C38:Q38,"✓")</f>
         <v/>
@@ -9296,19 +10101,33 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Medicación y recordatorios</t>
+          <t>Interoperabilidad y fuentes de datos</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Gestión de lista de medicamentos</t>
-        </is>
-      </c>
-      <c r="K39" t="inlineStr">
+          <t>Importación y exportación de datos</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr"/>
+      <c r="D39" t="inlineStr"/>
+      <c r="E39" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="F39" t="inlineStr"/>
+      <c r="G39" t="inlineStr"/>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr"/>
+      <c r="J39" t="inlineStr"/>
+      <c r="K39" t="inlineStr"/>
+      <c r="L39" t="inlineStr"/>
+      <c r="M39" t="inlineStr"/>
+      <c r="N39" t="inlineStr"/>
+      <c r="O39" t="inlineStr"/>
+      <c r="P39" t="inlineStr"/>
+      <c r="Q39" t="inlineStr"/>
       <c r="R39">
         <f>COUNTIF(C39:Q39,"✓")</f>
         <v/>
@@ -9317,24 +10136,33 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Medicación y recordatorios</t>
+          <t>Interoperabilidad y fuentes de datos</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Recordatorios de medicación y citas</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
+          <t>Integración con EHR de proveedores</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr"/>
+      <c r="D40" t="inlineStr"/>
+      <c r="E40" t="inlineStr"/>
+      <c r="F40" t="inlineStr"/>
+      <c r="G40" t="inlineStr"/>
+      <c r="H40" t="inlineStr"/>
+      <c r="I40" t="inlineStr"/>
+      <c r="J40" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="K40" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="K40" t="inlineStr"/>
+      <c r="L40" t="inlineStr"/>
+      <c r="M40" t="inlineStr"/>
+      <c r="N40" t="inlineStr"/>
+      <c r="O40" t="inlineStr"/>
+      <c r="P40" t="inlineStr"/>
+      <c r="Q40" t="inlineStr"/>
       <c r="R40">
         <f>COUNTIF(C40:Q40,"✓")</f>
         <v/>
@@ -9343,19 +10171,37 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Medicación y recordatorios</t>
+          <t>Interoperabilidad y fuentes de datos</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Registro de tomas y adherencia al tratamiento</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
+          <t>Integración con wearables y apps de salud</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr"/>
+      <c r="D41" t="inlineStr"/>
+      <c r="E41" t="inlineStr"/>
+      <c r="F41" t="inlineStr"/>
+      <c r="G41" t="inlineStr"/>
+      <c r="H41" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="I41" t="inlineStr"/>
+      <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr"/>
+      <c r="L41" t="inlineStr"/>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr"/>
+      <c r="O41" t="inlineStr"/>
+      <c r="P41" t="inlineStr"/>
+      <c r="Q41" t="inlineStr"/>
       <c r="R41">
         <f>COUNTIF(C41:Q41,"✓")</f>
         <v/>
@@ -9364,19 +10210,33 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Seguimiento y bienestar</t>
+          <t>Medicación y recordatorios</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Contenido educativo sobre salud</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
+          <t>Gestión de lista de medicamentos</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr"/>
+      <c r="D42" t="inlineStr"/>
+      <c r="E42" t="inlineStr"/>
+      <c r="F42" t="inlineStr"/>
+      <c r="G42" t="inlineStr"/>
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" t="inlineStr"/>
+      <c r="J42" t="inlineStr"/>
+      <c r="K42" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="L42" t="inlineStr"/>
+      <c r="M42" t="inlineStr"/>
+      <c r="N42" t="inlineStr"/>
+      <c r="O42" t="inlineStr"/>
+      <c r="P42" t="inlineStr"/>
+      <c r="Q42" t="inlineStr"/>
       <c r="R42">
         <f>COUNTIF(C42:Q42,"✓")</f>
         <v/>
@@ -9385,19 +10245,33 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Seguimiento y bienestar</t>
+          <t>Medicación y recordatorios</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Gráficas de evolución de indicadores</t>
-        </is>
-      </c>
+          <t>Importación automática de tratamientos desde receta digital</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr"/>
+      <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="F43" t="inlineStr"/>
+      <c r="G43" t="inlineStr"/>
+      <c r="H43" t="inlineStr"/>
+      <c r="I43" t="inlineStr"/>
+      <c r="J43" t="inlineStr"/>
+      <c r="K43" t="inlineStr"/>
+      <c r="L43" t="inlineStr"/>
+      <c r="M43" t="inlineStr"/>
+      <c r="N43" t="inlineStr"/>
+      <c r="O43" t="inlineStr"/>
+      <c r="P43" t="inlineStr"/>
+      <c r="Q43" t="inlineStr"/>
       <c r="R43">
         <f>COUNTIF(C43:Q43,"✓")</f>
         <v/>
@@ -9406,19 +10280,37 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Seguimiento y bienestar</t>
+          <t>Medicación y recordatorios</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Integración con wearables y apps de salud</t>
-        </is>
-      </c>
+          <t>Recordatorios de medicación y citas</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr"/>
+      <c r="E44" t="inlineStr"/>
+      <c r="F44" t="inlineStr"/>
+      <c r="G44" t="inlineStr"/>
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr"/>
+      <c r="J44" t="inlineStr"/>
       <c r="K44" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="L44" t="inlineStr"/>
+      <c r="M44" t="inlineStr"/>
+      <c r="N44" t="inlineStr"/>
+      <c r="O44" t="inlineStr"/>
+      <c r="P44" t="inlineStr"/>
+      <c r="Q44" t="inlineStr"/>
       <c r="R44">
         <f>COUNTIF(C44:Q44,"✓")</f>
         <v/>
@@ -9427,19 +10319,33 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Seguimiento y bienestar</t>
+          <t>Medicación y recordatorios</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Panel de seguimiento de salud y bienestar</t>
-        </is>
-      </c>
-      <c r="H45" t="inlineStr">
+          <t>Registro de tomas y adherencia al tratamiento</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr"/>
+      <c r="D45" t="inlineStr"/>
+      <c r="E45" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="F45" t="inlineStr"/>
+      <c r="G45" t="inlineStr"/>
+      <c r="H45" t="inlineStr"/>
+      <c r="I45" t="inlineStr"/>
+      <c r="J45" t="inlineStr"/>
+      <c r="K45" t="inlineStr"/>
+      <c r="L45" t="inlineStr"/>
+      <c r="M45" t="inlineStr"/>
+      <c r="N45" t="inlineStr"/>
+      <c r="O45" t="inlineStr"/>
+      <c r="P45" t="inlineStr"/>
+      <c r="Q45" t="inlineStr"/>
       <c r="R45">
         <f>COUNTIF(C45:Q45,"✓")</f>
         <v/>
@@ -9453,14 +10359,28 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Registro de nutrición</t>
-        </is>
-      </c>
-      <c r="K46" t="inlineStr">
+          <t>Comunidad de pacientes</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr"/>
+      <c r="D46" t="inlineStr"/>
+      <c r="E46" t="inlineStr"/>
+      <c r="F46" t="inlineStr"/>
+      <c r="G46" t="inlineStr"/>
+      <c r="H46" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="I46" t="inlineStr"/>
+      <c r="J46" t="inlineStr"/>
+      <c r="K46" t="inlineStr"/>
+      <c r="L46" t="inlineStr"/>
+      <c r="M46" t="inlineStr"/>
+      <c r="N46" t="inlineStr"/>
+      <c r="O46" t="inlineStr"/>
+      <c r="P46" t="inlineStr"/>
+      <c r="Q46" t="inlineStr"/>
       <c r="R46">
         <f>COUNTIF(C46:Q46,"✓")</f>
         <v/>
@@ -9474,14 +10394,28 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Seguimiento de salud femenina</t>
-        </is>
-      </c>
-      <c r="K47" t="inlineStr">
+          <t>Contenido educativo sobre salud</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr"/>
+      <c r="D47" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="E47" t="inlineStr"/>
+      <c r="F47" t="inlineStr"/>
+      <c r="G47" t="inlineStr"/>
+      <c r="H47" t="inlineStr"/>
+      <c r="I47" t="inlineStr"/>
+      <c r="J47" t="inlineStr"/>
+      <c r="K47" t="inlineStr"/>
+      <c r="L47" t="inlineStr"/>
+      <c r="M47" t="inlineStr"/>
+      <c r="N47" t="inlineStr"/>
+      <c r="O47" t="inlineStr"/>
+      <c r="P47" t="inlineStr"/>
+      <c r="Q47" t="inlineStr"/>
       <c r="R47">
         <f>COUNTIF(C47:Q47,"✓")</f>
         <v/>
@@ -9495,14 +10429,28 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Valoración de profesionales</t>
-        </is>
-      </c>
-      <c r="F48" t="inlineStr">
+          <t>Gráficas de evolución de indicadores</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr"/>
+      <c r="D48" t="inlineStr"/>
+      <c r="E48" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="F48" t="inlineStr"/>
+      <c r="G48" t="inlineStr"/>
+      <c r="H48" t="inlineStr"/>
+      <c r="I48" t="inlineStr"/>
+      <c r="J48" t="inlineStr"/>
+      <c r="K48" t="inlineStr"/>
+      <c r="L48" t="inlineStr"/>
+      <c r="M48" t="inlineStr"/>
+      <c r="N48" t="inlineStr"/>
+      <c r="O48" t="inlineStr"/>
+      <c r="P48" t="inlineStr"/>
+      <c r="Q48" t="inlineStr"/>
       <c r="R48">
         <f>COUNTIF(C48:Q48,"✓")</f>
         <v/>
@@ -9511,29 +10459,33 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Seguridad, privacidad y blockchain</t>
+          <t>Seguimiento y bienestar</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Blockchain para integridad y trazabilidad de datos</t>
-        </is>
-      </c>
-      <c r="H49" t="inlineStr">
+          <t>Integración con wearables y apps de salud</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="inlineStr"/>
+      <c r="E49" t="inlineStr"/>
+      <c r="F49" t="inlineStr"/>
+      <c r="G49" t="inlineStr"/>
+      <c r="H49" t="inlineStr"/>
+      <c r="I49" t="inlineStr"/>
+      <c r="J49" t="inlineStr"/>
+      <c r="K49" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="I49" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="J49" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="L49" t="inlineStr"/>
+      <c r="M49" t="inlineStr"/>
+      <c r="N49" t="inlineStr"/>
+      <c r="O49" t="inlineStr"/>
+      <c r="P49" t="inlineStr"/>
+      <c r="Q49" t="inlineStr"/>
       <c r="R49">
         <f>COUNTIF(C49:Q49,"✓")</f>
         <v/>
@@ -9542,24 +10494,33 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Seguridad, privacidad y blockchain</t>
+          <t>Seguimiento y bienestar</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Cifrado y control de acceso</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
+          <t>Panel de seguimiento de salud y bienestar</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr"/>
+      <c r="D50" t="inlineStr"/>
+      <c r="E50" t="inlineStr"/>
+      <c r="F50" t="inlineStr"/>
+      <c r="G50" t="inlineStr"/>
+      <c r="H50" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="K50" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="I50" t="inlineStr"/>
+      <c r="J50" t="inlineStr"/>
+      <c r="K50" t="inlineStr"/>
+      <c r="L50" t="inlineStr"/>
+      <c r="M50" t="inlineStr"/>
+      <c r="N50" t="inlineStr"/>
+      <c r="O50" t="inlineStr"/>
+      <c r="P50" t="inlineStr"/>
+      <c r="Q50" t="inlineStr"/>
       <c r="R50">
         <f>COUNTIF(C50:Q50,"✓")</f>
         <v/>
@@ -9568,19 +10529,33 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Seguridad, privacidad y blockchain</t>
+          <t>Seguimiento y bienestar</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Cumplimiento regulatorio de salud y datos</t>
-        </is>
-      </c>
-      <c r="O51" t="inlineStr">
+          <t>Registro de nutrición</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr"/>
+      <c r="D51" t="inlineStr"/>
+      <c r="E51" t="inlineStr"/>
+      <c r="F51" t="inlineStr"/>
+      <c r="G51" t="inlineStr"/>
+      <c r="H51" t="inlineStr"/>
+      <c r="I51" t="inlineStr"/>
+      <c r="J51" t="inlineStr"/>
+      <c r="K51" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="L51" t="inlineStr"/>
+      <c r="M51" t="inlineStr"/>
+      <c r="N51" t="inlineStr"/>
+      <c r="O51" t="inlineStr"/>
+      <c r="P51" t="inlineStr"/>
+      <c r="Q51" t="inlineStr"/>
       <c r="R51">
         <f>COUNTIF(C51:Q51,"✓")</f>
         <v/>
@@ -9589,19 +10564,33 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Seguridad, privacidad y blockchain</t>
+          <t>Seguimiento y bienestar</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Identidad descentralizada (DID)</t>
-        </is>
-      </c>
-      <c r="I52" t="inlineStr">
+          <t>Seguimiento de salud femenina</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr"/>
+      <c r="D52" t="inlineStr"/>
+      <c r="E52" t="inlineStr"/>
+      <c r="F52" t="inlineStr"/>
+      <c r="G52" t="inlineStr"/>
+      <c r="H52" t="inlineStr"/>
+      <c r="I52" t="inlineStr"/>
+      <c r="J52" t="inlineStr"/>
+      <c r="K52" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="L52" t="inlineStr"/>
+      <c r="M52" t="inlineStr"/>
+      <c r="N52" t="inlineStr"/>
+      <c r="O52" t="inlineStr"/>
+      <c r="P52" t="inlineStr"/>
+      <c r="Q52" t="inlineStr"/>
       <c r="R52">
         <f>COUNTIF(C52:Q52,"✓")</f>
         <v/>
@@ -9610,24 +10599,33 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Seguridad, privacidad y blockchain</t>
+          <t>Seguimiento y bienestar</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Privacidad reforzada para datos de salud</t>
-        </is>
-      </c>
-      <c r="L53" t="inlineStr">
+          <t>Valoración de profesionales</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr"/>
+      <c r="D53" t="inlineStr"/>
+      <c r="E53" t="inlineStr"/>
+      <c r="F53" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="M53" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="G53" t="inlineStr"/>
+      <c r="H53" t="inlineStr"/>
+      <c r="I53" t="inlineStr"/>
+      <c r="J53" t="inlineStr"/>
+      <c r="K53" t="inlineStr"/>
+      <c r="L53" t="inlineStr"/>
+      <c r="M53" t="inlineStr"/>
+      <c r="N53" t="inlineStr"/>
+      <c r="O53" t="inlineStr"/>
+      <c r="P53" t="inlineStr"/>
+      <c r="Q53" t="inlineStr"/>
       <c r="R53">
         <f>COUNTIF(C53:Q53,"✓")</f>
         <v/>
@@ -9636,19 +10634,41 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Seguros y pagos</t>
+          <t>Seguridad, privacidad y blockchain</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Modelo freemium y suscripción</t>
-        </is>
-      </c>
-      <c r="Q54" t="inlineStr">
+          <t>Blockchain para integridad y trazabilidad de datos</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr"/>
+      <c r="D54" t="inlineStr"/>
+      <c r="E54" t="inlineStr"/>
+      <c r="F54" t="inlineStr"/>
+      <c r="G54" t="inlineStr"/>
+      <c r="H54" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr"/>
+      <c r="L54" t="inlineStr"/>
+      <c r="M54" t="inlineStr"/>
+      <c r="N54" t="inlineStr"/>
+      <c r="O54" t="inlineStr"/>
+      <c r="P54" t="inlineStr"/>
+      <c r="Q54" t="inlineStr"/>
       <c r="R54">
         <f>COUNTIF(C54:Q54,"✓")</f>
         <v/>
@@ -9657,19 +10677,37 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Seguros y pagos</t>
+          <t>Seguridad, privacidad y blockchain</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Pagos con criptomoneda</t>
-        </is>
-      </c>
-      <c r="J55" t="inlineStr">
+          <t>Cifrado y control de acceso</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr"/>
+      <c r="D55" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="E55" t="inlineStr"/>
+      <c r="F55" t="inlineStr"/>
+      <c r="G55" t="inlineStr"/>
+      <c r="H55" t="inlineStr"/>
+      <c r="I55" t="inlineStr"/>
+      <c r="J55" t="inlineStr"/>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr"/>
+      <c r="M55" t="inlineStr"/>
+      <c r="N55" t="inlineStr"/>
+      <c r="O55" t="inlineStr"/>
+      <c r="P55" t="inlineStr"/>
+      <c r="Q55" t="inlineStr"/>
       <c r="R55">
         <f>COUNTIF(C55:Q55,"✓")</f>
         <v/>
@@ -9678,19 +10716,33 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Seguros y pagos</t>
+          <t>Seguridad, privacidad y blockchain</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Reclamos y trámites con seguros</t>
-        </is>
-      </c>
-      <c r="I56" t="inlineStr">
+          <t>Cumplimiento regulatorio de salud y datos</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr"/>
+      <c r="D56" t="inlineStr"/>
+      <c r="E56" t="inlineStr"/>
+      <c r="F56" t="inlineStr"/>
+      <c r="G56" t="inlineStr"/>
+      <c r="H56" t="inlineStr"/>
+      <c r="I56" t="inlineStr"/>
+      <c r="J56" t="inlineStr"/>
+      <c r="K56" t="inlineStr"/>
+      <c r="L56" t="inlineStr"/>
+      <c r="M56" t="inlineStr"/>
+      <c r="N56" t="inlineStr"/>
+      <c r="O56" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="P56" t="inlineStr"/>
+      <c r="Q56" t="inlineStr"/>
       <c r="R56">
         <f>COUNTIF(C56:Q56,"✓")</f>
         <v/>
@@ -9699,21 +10751,284 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Telemedicina y atención remota</t>
+          <t>Seguridad, privacidad y blockchain</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Teleconsulta con profesionales</t>
-        </is>
-      </c>
-      <c r="J57" t="inlineStr">
+          <t>Gestión de consentimiento sobre uso de datos</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr"/>
+      <c r="D57" t="inlineStr"/>
+      <c r="E57" t="inlineStr"/>
+      <c r="F57" t="inlineStr"/>
+      <c r="G57" t="inlineStr"/>
+      <c r="H57" t="inlineStr"/>
+      <c r="I57" t="inlineStr"/>
+      <c r="J57" t="inlineStr"/>
+      <c r="K57" t="inlineStr"/>
+      <c r="L57" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="M57" t="inlineStr"/>
+      <c r="N57" t="inlineStr"/>
+      <c r="O57" t="inlineStr"/>
+      <c r="P57" t="inlineStr"/>
+      <c r="Q57" t="inlineStr"/>
       <c r="R57">
         <f>COUNTIF(C57:Q57,"✓")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Seguridad, privacidad y blockchain</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Identidad descentralizada (DID)</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr"/>
+      <c r="D58" t="inlineStr"/>
+      <c r="E58" t="inlineStr"/>
+      <c r="F58" t="inlineStr"/>
+      <c r="G58" t="inlineStr"/>
+      <c r="H58" t="inlineStr"/>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr"/>
+      <c r="K58" t="inlineStr"/>
+      <c r="L58" t="inlineStr"/>
+      <c r="M58" t="inlineStr"/>
+      <c r="N58" t="inlineStr"/>
+      <c r="O58" t="inlineStr"/>
+      <c r="P58" t="inlineStr"/>
+      <c r="Q58" t="inlineStr"/>
+      <c r="R58">
+        <f>COUNTIF(C58:Q58,"✓")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Seguridad, privacidad y blockchain</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Privacidad reforzada para datos de salud</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr"/>
+      <c r="D59" t="inlineStr"/>
+      <c r="E59" t="inlineStr"/>
+      <c r="F59" t="inlineStr"/>
+      <c r="G59" t="inlineStr"/>
+      <c r="H59" t="inlineStr"/>
+      <c r="I59" t="inlineStr"/>
+      <c r="J59" t="inlineStr"/>
+      <c r="K59" t="inlineStr"/>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="N59" t="inlineStr"/>
+      <c r="O59" t="inlineStr"/>
+      <c r="P59" t="inlineStr"/>
+      <c r="Q59" t="inlineStr"/>
+      <c r="R59">
+        <f>COUNTIF(C59:Q59,"✓")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Seguros y pagos</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Modelo freemium y suscripción</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr"/>
+      <c r="D60" t="inlineStr"/>
+      <c r="E60" t="inlineStr"/>
+      <c r="F60" t="inlineStr"/>
+      <c r="G60" t="inlineStr"/>
+      <c r="H60" t="inlineStr"/>
+      <c r="I60" t="inlineStr"/>
+      <c r="J60" t="inlineStr"/>
+      <c r="K60" t="inlineStr"/>
+      <c r="L60" t="inlineStr"/>
+      <c r="M60" t="inlineStr"/>
+      <c r="N60" t="inlineStr"/>
+      <c r="O60" t="inlineStr"/>
+      <c r="P60" t="inlineStr"/>
+      <c r="Q60" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="R60">
+        <f>COUNTIF(C60:Q60,"✓")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Seguros y pagos</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Pagos con criptomoneda</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr"/>
+      <c r="D61" t="inlineStr"/>
+      <c r="E61" t="inlineStr"/>
+      <c r="F61" t="inlineStr"/>
+      <c r="G61" t="inlineStr"/>
+      <c r="H61" t="inlineStr"/>
+      <c r="I61" t="inlineStr"/>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr"/>
+      <c r="L61" t="inlineStr"/>
+      <c r="M61" t="inlineStr"/>
+      <c r="N61" t="inlineStr"/>
+      <c r="O61" t="inlineStr"/>
+      <c r="P61" t="inlineStr"/>
+      <c r="Q61" t="inlineStr"/>
+      <c r="R61">
+        <f>COUNTIF(C61:Q61,"✓")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Seguros y pagos</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Pagos dentro de la app</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr"/>
+      <c r="D62" t="inlineStr"/>
+      <c r="E62" t="inlineStr"/>
+      <c r="F62" t="inlineStr"/>
+      <c r="G62" t="inlineStr"/>
+      <c r="H62" t="inlineStr"/>
+      <c r="I62" t="inlineStr"/>
+      <c r="J62" t="inlineStr"/>
+      <c r="K62" t="inlineStr"/>
+      <c r="L62" t="inlineStr"/>
+      <c r="M62" t="inlineStr"/>
+      <c r="N62" t="inlineStr"/>
+      <c r="O62" t="inlineStr"/>
+      <c r="P62" t="inlineStr"/>
+      <c r="Q62" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="R62">
+        <f>COUNTIF(C62:Q62,"✓")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Seguros y pagos</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Reclamos y trámites con seguros</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr"/>
+      <c r="D63" t="inlineStr"/>
+      <c r="E63" t="inlineStr"/>
+      <c r="F63" t="inlineStr"/>
+      <c r="G63" t="inlineStr"/>
+      <c r="H63" t="inlineStr"/>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr"/>
+      <c r="K63" t="inlineStr"/>
+      <c r="L63" t="inlineStr"/>
+      <c r="M63" t="inlineStr"/>
+      <c r="N63" t="inlineStr"/>
+      <c r="O63" t="inlineStr"/>
+      <c r="P63" t="inlineStr"/>
+      <c r="Q63" t="inlineStr"/>
+      <c r="R63">
+        <f>COUNTIF(C63:Q63,"✓")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Telemedicina y atención remota</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Teleconsulta con profesionales</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr"/>
+      <c r="D64" t="inlineStr"/>
+      <c r="E64" t="inlineStr"/>
+      <c r="F64" t="inlineStr"/>
+      <c r="G64" t="inlineStr"/>
+      <c r="H64" t="inlineStr"/>
+      <c r="I64" t="inlineStr"/>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr"/>
+      <c r="L64" t="inlineStr"/>
+      <c r="M64" t="inlineStr"/>
+      <c r="N64" t="inlineStr"/>
+      <c r="O64" t="inlineStr"/>
+      <c r="P64" t="inlineStr"/>
+      <c r="Q64" t="inlineStr"/>
+      <c r="R64">
+        <f>COUNTIF(C64:Q64,"✓")</f>
         <v/>
       </c>
     </row>
@@ -9728,7 +11043,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A20"/>
+  <dimension ref="A1:A21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -9874,6 +11189,13 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>VUELTA 4 COMPLETA (2026-10-08 12:08 UTC): Clinia, MiRedSalud y Mediko verificados (+1 fila). Contador de loops = 4 para todos, Revisado reiniciado a "No". func_norm (124 filas) y tabla_frecuencia (63 funcionalidades) regenerados. Vuelta 5 parte con Meedika, Infomed, MediPlanner, Clingot. Candidato a competidor sin agregar: HealthChain (Chile).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Benchmark: vuelta 5, iteración 1 (Meedika, Infomed, MediPlanner, Clingot)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MVcXu8vTBu7EKfj3YdEvae
</commit_message>
<xml_diff>
--- a/Outputs/Benchmark_Anamnesis.xlsx
+++ b/Outputs/Benchmark_Anamnesis.xlsx
@@ -513,12 +513,12 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>[DIRECTO · Chile · etapas A+B] Lanzada 25-sep-2024 en App Store (Android previsto la misma semana). &gt;1.500 usuarios en los primeros días; meta 32.000 (cofundador Francisco González). Funciones: gestión de documentos, importar solicitudes, SOS con alergias/medicación, calendario de citas, recordatorios, compartir con profesionales elegidos. Sin blockchain. Precio y estado actual NO verificados; única fuente es una nota de prensa. Sitio oficial por confirmar. [Iter. 2] Hay cobertura adicional en Portal Innova (portalinnova.cl); sitio bloqueado en este entorno, estado actual sigue sin verificar. [Vuelta 3] Sin novedades 2026 ni confirmación de la app Android en Google Play; usuarios actuales desconocidos. Nota de prensa no indica año de lanzamiento explícito. [Vuelta 4] Sin fuentes nuevas; portalinnova.cl no aparece en búsquedas. Sigue dependiendo de una sola nota de prensa.</t>
+          <t>[DIRECTO · Chile · etapas A+B] Lanzada 25-sep-2024 en App Store (Android previsto la misma semana). &gt;1.500 usuarios en los primeros días; meta 32.000 (cofundador Francisco González). Funciones: gestión de documentos, importar solicitudes, SOS con alergias/medicación, calendario de citas, recordatorios, compartir con profesionales elegidos. Sin blockchain. Precio y estado actual NO verificados; única fuente es una nota de prensa. Sitio oficial por confirmar. [Iter. 2] Hay cobertura adicional en Portal Innova (portalinnova.cl); sitio bloqueado en este entorno, estado actual sigue sin verificar. [Vuelta 3] Sin novedades 2026 ni confirmación de la app Android en Google Play; usuarios actuales desconocidos. Nota de prensa no indica año de lanzamiento explícito. [Vuelta 4] Sin fuentes nuevas; portalinnova.cl no aparece en búsquedas. Sigue dependiendo de una sola nota de prensa. [Vuelta 5] Sin fuentes nuevas (ni entrevistas ni financiamiento); sigue dependiendo de una sola nota de prensa sin año explícito.</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G2" t="n">
@@ -526,7 +526,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
     </row>
@@ -553,12 +553,12 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>[DIRECTO · Chile · etapa A] Fundada 2019 por Diego Ibarra, Andrés Fantuzzi y Gabriel Zamora. Lanzada mar-2021 en App Store y Play Store con 1.200 usuarios; planeaba nueva versión jul-2021 y ronda de US$500 mil. Objetivo: llevar el historial en el celular, acceso en emergencias, médico puede ingresar datos con consentimiento. Estado actual NO verificado (posible app inactiva). URL es la nota de prensa; sitio oficial por confirmar. [Vuelta 3] Sin evidencia posterior a 2021; relanzamiento previsto jul-2021 no confirmado. Probable app inactiva. [Vuelta 4] Sin cambios; sigue sin evidencia posterior a 2021.</t>
+          <t>[DIRECTO · Chile · etapa A] Fundada 2019 por Diego Ibarra, Andrés Fantuzzi y Gabriel Zamora. Lanzada mar-2021 en App Store y Play Store con 1.200 usuarios; planeaba nueva versión jul-2021 y ronda de US$500 mil. Objetivo: llevar el historial en el celular, acceso en emergencias, médico puede ingresar datos con consentimiento. Estado actual NO verificado (posible app inactiva). URL es la nota de prensa; sitio oficial por confirmar. [Vuelta 3] Sin evidencia posterior a 2021; relanzamiento previsto jul-2021 no confirmado. Probable app inactiva. [Vuelta 4] Sin cambios; sigue sin evidencia posterior a 2021. [Vuelta 5] Cofundador Andrés Fantuzzi es cardiólogo de la Clínica Santa María. Sin ronda de inversión ni relanzamiento confirmados; no confundir con Infomed de Cuba (portal del Minsap).</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G3" t="n">
@@ -566,7 +566,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
     </row>
@@ -593,12 +593,12 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>[REGIONAL · México] Historial por perfil familiar, alergias, vacunas, recetas digitales, gráficas de evolución, agendamiento, compartir con profesionales. Gratis en App Store MX. Sin evidencia de uso en Chile. Cubre parte de la etapa C (familia). [Vuelta 3] Existen dos apps distintas: MediPlanner (gratis, Rym Solutions, MX, 3,7/5 con 3 calificaciones) y MediPlanner Pro (otro desarrollador, $39 MXN). Sin presencia verificada en Chile. [Vuelta 4] No pude confirmar el desarrollador de la versión gratuita (Rym Solutions no se repite en esta búsqueda). MediPlanner Pro (fichas BR/OM) guardaría datos solo en el dispositivo, sin nube; no confundir con MedPlanner/AskHEMI (otra empresa).</t>
+          <t>[REGIONAL · México] Historial por perfil familiar, alergias, vacunas, recetas digitales, gráficas de evolución, agendamiento, compartir con profesionales. Gratis en App Store MX. Sin evidencia de uso en Chile. Cubre parte de la etapa C (familia). [Vuelta 3] Existen dos apps distintas: MediPlanner (gratis, Rym Solutions, MX, 3,7/5 con 3 calificaciones) y MediPlanner Pro (otro desarrollador, $39 MXN). Sin presencia verificada en Chile. [Vuelta 4] No pude confirmar el desarrollador de la versión gratuita (Rym Solutions no se repite en esta búsqueda). MediPlanner Pro (fichas BR/OM) guardaría datos solo en el dispositivo, sin nube; no confundir con MedPlanner/AskHEMI (otra empresa). [Vuelta 5] Sin búsqueda nueva (revisada en vuelta 4); sin cambios.</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G4" t="n">
@@ -606,7 +606,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
     </row>
@@ -633,12 +633,12 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>[REGIONAL · Argentina · débil] App para cargar antecedentes médicos propios. Única referencia: nota de opinión en grupoanimal.mx sin fecha verificada. Estado y sitio por confirmar. [Vuelta 3] Referencias de 2017 (apps4citizens, La Nación); sitio y precio no verificados; puede estar inactiva. [Vuelta 4] Sin fuentes nuevas.</t>
+          <t>[REGIONAL · Argentina · débil] App para cargar antecedentes médicos propios. Única referencia: nota de opinión en grupoanimal.mx sin fecha verificada. Estado y sitio por confirmar. [Vuelta 3] Referencias de 2017 (apps4citizens, La Nación); sitio y precio no verificados; puede estar inactiva. [Vuelta 4] Sin fuentes nuevas. [Vuelta 5] Registro empresarial (indicadores.ar, datos a jul-2026) muestra CLINGOT S.A. activa en CABA, constituida el 4-abr-2016; no confirma que la app siga operando. Programa federal argentino de historias clínicas digitales como contexto regulatorio.</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G5" t="n">
@@ -646,7 +646,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
     </row>
@@ -8646,8 +8646,6 @@
           <t>Búsqueda de profesionales de salud</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
           <t>✓</t>
@@ -8658,17 +8656,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
       <c r="R2">
         <f>COUNTIF(C2:Q2,"✓")</f>
         <v/>
@@ -8690,24 +8677,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
       <c r="R3">
         <f>COUNTIF(C3:Q3,"✓")</f>
         <v/>
@@ -8724,25 +8698,11 @@
           <t>Integración con calendario del dispositivo</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
       <c r="R4">
         <f>COUNTIF(C4:Q4,"✓")</f>
         <v/>
@@ -8759,25 +8719,11 @@
           <t>Localización de centros médicos y farmacias</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr"/>
       <c r="R5">
         <f>COUNTIF(C5:Q5,"✓")</f>
         <v/>
@@ -8794,17 +8740,6 @@
           <t>Reserva de citas médicas</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr">
         <is>
           <t>✓</t>
@@ -8815,8 +8750,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="inlineStr"/>
       <c r="R6">
         <f>COUNTIF(C6:Q6,"✓")</f>
         <v/>
@@ -8833,25 +8766,11 @@
           <t>Acceso del profesional al historial del paciente</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr"/>
-      <c r="Q7" t="inlineStr"/>
       <c r="R7">
         <f>COUNTIF(C7:Q7,"✓")</f>
         <v/>
@@ -8868,25 +8787,11 @@
           <t>Compartir con personas sin cuenta mediante clave segura</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
-      <c r="P8" t="inlineStr"/>
-      <c r="Q8" t="inlineStr"/>
       <c r="R8">
         <f>COUNTIF(C8:Q8,"✓")</f>
         <v/>
@@ -8903,25 +8808,11 @@
           <t>Compartir datos con cuidador o persona de confianza</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
-      <c r="P9" t="inlineStr"/>
-      <c r="Q9" t="inlineStr"/>
       <c r="R9">
         <f>COUNTIF(C9:Q9,"✓")</f>
         <v/>
@@ -8943,13 +8834,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
           <t>✓</t>
@@ -8975,16 +8864,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
       <c r="O10" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="P10" t="inlineStr"/>
-      <c r="Q10" t="inlineStr"/>
       <c r="R10">
         <f>COUNTIF(C10:Q10,"✓")</f>
         <v/>
@@ -9001,25 +8885,11 @@
           <t>Gestión de consentimiento sobre uso de datos</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr"/>
-      <c r="P11" t="inlineStr"/>
-      <c r="Q11" t="inlineStr"/>
       <c r="R11">
         <f>COUNTIF(C11:Q11,"✓")</f>
         <v/>
@@ -9036,25 +8906,11 @@
           <t>Ingreso de datos por profesional con consentimiento</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
-      <c r="O12" t="inlineStr"/>
-      <c r="P12" t="inlineStr"/>
-      <c r="Q12" t="inlineStr"/>
       <c r="R12">
         <f>COUNTIF(C12:Q12,"✓")</f>
         <v/>
@@ -9071,25 +8927,11 @@
           <t>Red social con profesionales y familiares</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr"/>
-      <c r="O13" t="inlineStr"/>
-      <c r="P13" t="inlineStr"/>
-      <c r="Q13" t="inlineStr"/>
       <c r="R13">
         <f>COUNTIF(C13:Q13,"✓")</f>
         <v/>
@@ -9116,23 +8958,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
-      <c r="M14" t="inlineStr"/>
-      <c r="N14" t="inlineStr"/>
-      <c r="O14" t="inlineStr"/>
-      <c r="P14" t="inlineStr"/>
-      <c r="Q14" t="inlineStr"/>
       <c r="R14">
         <f>COUNTIF(C14:Q14,"✓")</f>
         <v/>
@@ -9149,8 +8979,6 @@
           <t>Perfiles familiares / dependientes</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9161,25 +8989,16 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr"/>
       <c r="N15" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="Q15" t="inlineStr"/>
       <c r="R15">
         <f>COUNTIF(C15:Q15,"✓")</f>
         <v/>
@@ -9201,8 +9020,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9218,19 +9035,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
-      <c r="M16" t="inlineStr"/>
-      <c r="N16" t="inlineStr"/>
       <c r="O16" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="P16" t="inlineStr"/>
-      <c r="Q16" t="inlineStr"/>
       <c r="R16">
         <f>COUNTIF(C16:Q16,"✓")</f>
         <v/>
@@ -9247,29 +9056,16 @@
           <t>Almacenamiento de recetas</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr"/>
       <c r="N17" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="O17" t="inlineStr"/>
-      <c r="P17" t="inlineStr"/>
-      <c r="Q17" t="inlineStr"/>
       <c r="R17">
         <f>COUNTIF(C17:Q17,"✓")</f>
         <v/>
@@ -9286,25 +9082,11 @@
           <t>Búsqueda y filtros de documentos</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr"/>
-      <c r="M18" t="inlineStr"/>
-      <c r="N18" t="inlineStr"/>
-      <c r="O18" t="inlineStr"/>
-      <c r="P18" t="inlineStr"/>
-      <c r="Q18" t="inlineStr"/>
       <c r="R18">
         <f>COUNTIF(C18:Q18,"✓")</f>
         <v/>
@@ -9321,25 +9103,11 @@
           <t>Emisión de certificados médicos</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr"/>
-      <c r="M19" t="inlineStr"/>
-      <c r="N19" t="inlineStr"/>
-      <c r="O19" t="inlineStr"/>
-      <c r="P19" t="inlineStr"/>
-      <c r="Q19" t="inlineStr"/>
       <c r="R19">
         <f>COUNTIF(C19:Q19,"✓")</f>
         <v/>
@@ -9361,19 +9129,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr"/>
-      <c r="M20" t="inlineStr"/>
-      <c r="N20" t="inlineStr"/>
-      <c r="O20" t="inlineStr"/>
-      <c r="P20" t="inlineStr"/>
       <c r="Q20" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9395,25 +9150,11 @@
           <t>Notificación y envío de resultados</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr"/>
-      <c r="M21" t="inlineStr"/>
       <c r="N21" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="O21" t="inlineStr"/>
-      <c r="P21" t="inlineStr"/>
-      <c r="Q21" t="inlineStr"/>
       <c r="R21">
         <f>COUNTIF(C21:Q21,"✓")</f>
         <v/>
@@ -9430,29 +9171,16 @@
           <t>Historial institucional (solo datos de la propia red)</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
-      <c r="L22" t="inlineStr"/>
-      <c r="M22" t="inlineStr"/>
       <c r="N22" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="O22" t="inlineStr"/>
       <c r="P22" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="Q22" t="inlineStr"/>
       <c r="R22">
         <f>COUNTIF(C22:Q22,"✓")</f>
         <v/>
@@ -9469,36 +9197,26 @@
           <t>Historial médico centralizado</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="L23" t="inlineStr"/>
-      <c r="M23" t="inlineStr"/>
-      <c r="N23" t="inlineStr"/>
-      <c r="O23" t="inlineStr"/>
-      <c r="P23" t="inlineStr"/>
       <c r="Q23" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9520,25 +9238,11 @@
           <t>Línea de tiempo de salud</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
-      <c r="L24" t="inlineStr"/>
-      <c r="M24" t="inlineStr"/>
-      <c r="N24" t="inlineStr"/>
-      <c r="O24" t="inlineStr"/>
-      <c r="P24" t="inlineStr"/>
-      <c r="Q24" t="inlineStr"/>
       <c r="R24">
         <f>COUNTIF(C24:Q24,"✓")</f>
         <v/>
@@ -9555,25 +9259,11 @@
           <t>Registro de alergias y vacunas</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr"/>
-      <c r="L25" t="inlineStr"/>
-      <c r="M25" t="inlineStr"/>
-      <c r="N25" t="inlineStr"/>
-      <c r="O25" t="inlineStr"/>
-      <c r="P25" t="inlineStr"/>
-      <c r="Q25" t="inlineStr"/>
       <c r="R25">
         <f>COUNTIF(C25:Q25,"✓")</f>
         <v/>
@@ -9590,25 +9280,11 @@
           <t>Seguimiento de visitas, gastos y seguros</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr"/>
-      <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr"/>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
-      <c r="L26" t="inlineStr"/>
-      <c r="M26" t="inlineStr"/>
-      <c r="N26" t="inlineStr"/>
-      <c r="O26" t="inlineStr"/>
-      <c r="P26" t="inlineStr"/>
-      <c r="Q26" t="inlineStr"/>
       <c r="R26">
         <f>COUNTIF(C26:Q26,"✓")</f>
         <v/>
@@ -9625,11 +9301,6 @@
           <t>Recompensas / monetización de datos del usuario</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr"/>
-      <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9645,13 +9316,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="K27" t="inlineStr"/>
-      <c r="L27" t="inlineStr"/>
-      <c r="M27" t="inlineStr"/>
-      <c r="N27" t="inlineStr"/>
-      <c r="O27" t="inlineStr"/>
-      <c r="P27" t="inlineStr"/>
-      <c r="Q27" t="inlineStr"/>
       <c r="R27">
         <f>COUNTIF(C27:Q27,"✓")</f>
         <v/>
@@ -9668,25 +9332,11 @@
           <t>Asistente de IA para profesionales de salud</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="M28" t="inlineStr"/>
-      <c r="N28" t="inlineStr"/>
-      <c r="O28" t="inlineStr"/>
-      <c r="P28" t="inlineStr"/>
-      <c r="Q28" t="inlineStr"/>
       <c r="R28">
         <f>COUNTIF(C28:Q28,"✓")</f>
         <v/>
@@ -9703,25 +9353,11 @@
           <t>Coaching de salud con IA</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr"/>
-      <c r="D29" t="inlineStr"/>
-      <c r="E29" t="inlineStr"/>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr"/>
-      <c r="L29" t="inlineStr"/>
-      <c r="M29" t="inlineStr"/>
-      <c r="N29" t="inlineStr"/>
-      <c r="O29" t="inlineStr"/>
-      <c r="P29" t="inlineStr"/>
-      <c r="Q29" t="inlineStr"/>
       <c r="R29">
         <f>COUNTIF(C29:Q29,"✓")</f>
         <v/>
@@ -9738,15 +9374,6 @@
           <t>Detección de patrones en métricas de salud con IA</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr"/>
-      <c r="E30" t="inlineStr"/>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr"/>
-      <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9757,10 +9384,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="N30" t="inlineStr"/>
-      <c r="O30" t="inlineStr"/>
-      <c r="P30" t="inlineStr"/>
-      <c r="Q30" t="inlineStr"/>
       <c r="R30">
         <f>COUNTIF(C30:Q30,"✓")</f>
         <v/>
@@ -9777,15 +9400,6 @@
           <t>Interpretación de exámenes con IA</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr"/>
-      <c r="D31" t="inlineStr"/>
-      <c r="E31" t="inlineStr"/>
-      <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr"/>
-      <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9796,9 +9410,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="N31" t="inlineStr"/>
-      <c r="O31" t="inlineStr"/>
-      <c r="P31" t="inlineStr"/>
       <c r="Q31" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9820,24 +9431,11 @@
           <t>Orientación médica con IA</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr"/>
-      <c r="D32" t="inlineStr"/>
-      <c r="E32" t="inlineStr"/>
-      <c r="F32" t="inlineStr"/>
-      <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr"/>
-      <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr"/>
-      <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="M32" t="inlineStr"/>
-      <c r="N32" t="inlineStr"/>
-      <c r="O32" t="inlineStr"/>
-      <c r="P32" t="inlineStr"/>
       <c r="Q32" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9859,15 +9457,6 @@
           <t>Preparación de consultas médicas con IA</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr"/>
-      <c r="D33" t="inlineStr"/>
-      <c r="E33" t="inlineStr"/>
-      <c r="F33" t="inlineStr"/>
-      <c r="G33" t="inlineStr"/>
-      <c r="H33" t="inlineStr"/>
-      <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr"/>
-      <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9878,10 +9467,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="N33" t="inlineStr"/>
-      <c r="O33" t="inlineStr"/>
-      <c r="P33" t="inlineStr"/>
-      <c r="Q33" t="inlineStr"/>
       <c r="R33">
         <f>COUNTIF(C33:Q33,"✓")</f>
         <v/>
@@ -9898,15 +9483,6 @@
           <t>Resumen de historial con IA</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr"/>
-      <c r="D34" t="inlineStr"/>
-      <c r="E34" t="inlineStr"/>
-      <c r="F34" t="inlineStr"/>
-      <c r="G34" t="inlineStr"/>
-      <c r="H34" t="inlineStr"/>
-      <c r="I34" t="inlineStr"/>
-      <c r="J34" t="inlineStr"/>
-      <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9917,10 +9493,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="N34" t="inlineStr"/>
-      <c r="O34" t="inlineStr"/>
-      <c r="P34" t="inlineStr"/>
-      <c r="Q34" t="inlineStr"/>
       <c r="R34">
         <f>COUNTIF(C34:Q34,"✓")</f>
         <v/>
@@ -9942,10 +9514,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr"/>
-      <c r="E35" t="inlineStr"/>
-      <c r="F35" t="inlineStr"/>
-      <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9956,7 +9524,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="J35" t="inlineStr"/>
       <c r="K35" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9972,14 +9539,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="N35" t="inlineStr"/>
       <c r="O35" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="P35" t="inlineStr"/>
-      <c r="Q35" t="inlineStr"/>
       <c r="R35">
         <f>COUNTIF(C35:Q35,"✓")</f>
         <v/>
@@ -9996,25 +9560,11 @@
           <t>Analítica poblacional B2B</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr"/>
-      <c r="D36" t="inlineStr"/>
-      <c r="E36" t="inlineStr"/>
-      <c r="F36" t="inlineStr"/>
-      <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="I36" t="inlineStr"/>
-      <c r="J36" t="inlineStr"/>
-      <c r="K36" t="inlineStr"/>
-      <c r="L36" t="inlineStr"/>
-      <c r="M36" t="inlineStr"/>
-      <c r="N36" t="inlineStr"/>
-      <c r="O36" t="inlineStr"/>
-      <c r="P36" t="inlineStr"/>
-      <c r="Q36" t="inlineStr"/>
       <c r="R36">
         <f>COUNTIF(C36:Q36,"✓")</f>
         <v/>
@@ -10031,9 +9581,6 @@
           <t>Disponibilidad multiplataforma (web/iOS/Android)</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr"/>
-      <c r="D37" t="inlineStr"/>
-      <c r="E37" t="inlineStr"/>
       <c r="F37" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10044,20 +9591,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr"/>
-      <c r="J37" t="inlineStr"/>
-      <c r="K37" t="inlineStr"/>
-      <c r="L37" t="inlineStr"/>
-      <c r="M37" t="inlineStr"/>
-      <c r="N37" t="inlineStr"/>
       <c r="O37" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="P37" t="inlineStr"/>
-      <c r="Q37" t="inlineStr"/>
       <c r="R37">
         <f>COUNTIF(C37:Q37,"✓")</f>
         <v/>
@@ -10074,25 +9612,11 @@
           <t>Historial médico centralizado</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr"/>
-      <c r="D38" t="inlineStr"/>
-      <c r="E38" t="inlineStr"/>
-      <c r="F38" t="inlineStr"/>
-      <c r="G38" t="inlineStr"/>
-      <c r="H38" t="inlineStr"/>
-      <c r="I38" t="inlineStr"/>
       <c r="J38" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="K38" t="inlineStr"/>
-      <c r="L38" t="inlineStr"/>
-      <c r="M38" t="inlineStr"/>
-      <c r="N38" t="inlineStr"/>
-      <c r="O38" t="inlineStr"/>
-      <c r="P38" t="inlineStr"/>
-      <c r="Q38" t="inlineStr"/>
       <c r="R38">
         <f>COUNTIF(C38:Q38,"✓")</f>
         <v/>
@@ -10109,25 +9633,11 @@
           <t>Importación y exportación de datos</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr"/>
-      <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr"/>
-      <c r="G39" t="inlineStr"/>
-      <c r="H39" t="inlineStr"/>
-      <c r="I39" t="inlineStr"/>
-      <c r="J39" t="inlineStr"/>
-      <c r="K39" t="inlineStr"/>
-      <c r="L39" t="inlineStr"/>
-      <c r="M39" t="inlineStr"/>
-      <c r="N39" t="inlineStr"/>
-      <c r="O39" t="inlineStr"/>
-      <c r="P39" t="inlineStr"/>
-      <c r="Q39" t="inlineStr"/>
       <c r="R39">
         <f>COUNTIF(C39:Q39,"✓")</f>
         <v/>
@@ -10144,25 +9654,11 @@
           <t>Integración con EHR de proveedores</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr"/>
-      <c r="D40" t="inlineStr"/>
-      <c r="E40" t="inlineStr"/>
-      <c r="F40" t="inlineStr"/>
-      <c r="G40" t="inlineStr"/>
-      <c r="H40" t="inlineStr"/>
-      <c r="I40" t="inlineStr"/>
       <c r="J40" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="K40" t="inlineStr"/>
-      <c r="L40" t="inlineStr"/>
-      <c r="M40" t="inlineStr"/>
-      <c r="N40" t="inlineStr"/>
-      <c r="O40" t="inlineStr"/>
-      <c r="P40" t="inlineStr"/>
-      <c r="Q40" t="inlineStr"/>
       <c r="R40">
         <f>COUNTIF(C40:Q40,"✓")</f>
         <v/>
@@ -10179,29 +9675,16 @@
           <t>Integración con wearables y apps de salud</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr"/>
-      <c r="D41" t="inlineStr"/>
-      <c r="E41" t="inlineStr"/>
-      <c r="F41" t="inlineStr"/>
-      <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="I41" t="inlineStr"/>
-      <c r="J41" t="inlineStr"/>
-      <c r="K41" t="inlineStr"/>
-      <c r="L41" t="inlineStr"/>
       <c r="M41" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="N41" t="inlineStr"/>
-      <c r="O41" t="inlineStr"/>
-      <c r="P41" t="inlineStr"/>
-      <c r="Q41" t="inlineStr"/>
       <c r="R41">
         <f>COUNTIF(C41:Q41,"✓")</f>
         <v/>
@@ -10218,25 +9701,11 @@
           <t>Gestión de lista de medicamentos</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr"/>
-      <c r="D42" t="inlineStr"/>
-      <c r="E42" t="inlineStr"/>
-      <c r="F42" t="inlineStr"/>
-      <c r="G42" t="inlineStr"/>
-      <c r="H42" t="inlineStr"/>
-      <c r="I42" t="inlineStr"/>
-      <c r="J42" t="inlineStr"/>
       <c r="K42" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="L42" t="inlineStr"/>
-      <c r="M42" t="inlineStr"/>
-      <c r="N42" t="inlineStr"/>
-      <c r="O42" t="inlineStr"/>
-      <c r="P42" t="inlineStr"/>
-      <c r="Q42" t="inlineStr"/>
       <c r="R42">
         <f>COUNTIF(C42:Q42,"✓")</f>
         <v/>
@@ -10253,25 +9722,11 @@
           <t>Importación automática de tratamientos desde receta digital</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr"/>
-      <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr"/>
-      <c r="G43" t="inlineStr"/>
-      <c r="H43" t="inlineStr"/>
-      <c r="I43" t="inlineStr"/>
-      <c r="J43" t="inlineStr"/>
-      <c r="K43" t="inlineStr"/>
-      <c r="L43" t="inlineStr"/>
-      <c r="M43" t="inlineStr"/>
-      <c r="N43" t="inlineStr"/>
-      <c r="O43" t="inlineStr"/>
-      <c r="P43" t="inlineStr"/>
-      <c r="Q43" t="inlineStr"/>
       <c r="R43">
         <f>COUNTIF(C43:Q43,"✓")</f>
         <v/>
@@ -10293,24 +9748,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr"/>
-      <c r="E44" t="inlineStr"/>
-      <c r="F44" t="inlineStr"/>
-      <c r="G44" t="inlineStr"/>
-      <c r="H44" t="inlineStr"/>
-      <c r="I44" t="inlineStr"/>
-      <c r="J44" t="inlineStr"/>
       <c r="K44" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="L44" t="inlineStr"/>
-      <c r="M44" t="inlineStr"/>
-      <c r="N44" t="inlineStr"/>
-      <c r="O44" t="inlineStr"/>
-      <c r="P44" t="inlineStr"/>
-      <c r="Q44" t="inlineStr"/>
       <c r="R44">
         <f>COUNTIF(C44:Q44,"✓")</f>
         <v/>
@@ -10327,25 +9769,11 @@
           <t>Registro de tomas y adherencia al tratamiento</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr"/>
-      <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr"/>
-      <c r="G45" t="inlineStr"/>
-      <c r="H45" t="inlineStr"/>
-      <c r="I45" t="inlineStr"/>
-      <c r="J45" t="inlineStr"/>
-      <c r="K45" t="inlineStr"/>
-      <c r="L45" t="inlineStr"/>
-      <c r="M45" t="inlineStr"/>
-      <c r="N45" t="inlineStr"/>
-      <c r="O45" t="inlineStr"/>
-      <c r="P45" t="inlineStr"/>
-      <c r="Q45" t="inlineStr"/>
       <c r="R45">
         <f>COUNTIF(C45:Q45,"✓")</f>
         <v/>
@@ -10362,25 +9790,11 @@
           <t>Comunidad de pacientes</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr"/>
-      <c r="D46" t="inlineStr"/>
-      <c r="E46" t="inlineStr"/>
-      <c r="F46" t="inlineStr"/>
-      <c r="G46" t="inlineStr"/>
       <c r="H46" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="I46" t="inlineStr"/>
-      <c r="J46" t="inlineStr"/>
-      <c r="K46" t="inlineStr"/>
-      <c r="L46" t="inlineStr"/>
-      <c r="M46" t="inlineStr"/>
-      <c r="N46" t="inlineStr"/>
-      <c r="O46" t="inlineStr"/>
-      <c r="P46" t="inlineStr"/>
-      <c r="Q46" t="inlineStr"/>
       <c r="R46">
         <f>COUNTIF(C46:Q46,"✓")</f>
         <v/>
@@ -10397,25 +9811,11 @@
           <t>Contenido educativo sobre salud</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr"/>
       <c r="D47" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr"/>
-      <c r="F47" t="inlineStr"/>
-      <c r="G47" t="inlineStr"/>
-      <c r="H47" t="inlineStr"/>
-      <c r="I47" t="inlineStr"/>
-      <c r="J47" t="inlineStr"/>
-      <c r="K47" t="inlineStr"/>
-      <c r="L47" t="inlineStr"/>
-      <c r="M47" t="inlineStr"/>
-      <c r="N47" t="inlineStr"/>
-      <c r="O47" t="inlineStr"/>
-      <c r="P47" t="inlineStr"/>
-      <c r="Q47" t="inlineStr"/>
       <c r="R47">
         <f>COUNTIF(C47:Q47,"✓")</f>
         <v/>
@@ -10432,25 +9832,11 @@
           <t>Gráficas de evolución de indicadores</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr"/>
-      <c r="D48" t="inlineStr"/>
       <c r="E48" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr"/>
-      <c r="G48" t="inlineStr"/>
-      <c r="H48" t="inlineStr"/>
-      <c r="I48" t="inlineStr"/>
-      <c r="J48" t="inlineStr"/>
-      <c r="K48" t="inlineStr"/>
-      <c r="L48" t="inlineStr"/>
-      <c r="M48" t="inlineStr"/>
-      <c r="N48" t="inlineStr"/>
-      <c r="O48" t="inlineStr"/>
-      <c r="P48" t="inlineStr"/>
-      <c r="Q48" t="inlineStr"/>
       <c r="R48">
         <f>COUNTIF(C48:Q48,"✓")</f>
         <v/>
@@ -10467,25 +9853,11 @@
           <t>Integración con wearables y apps de salud</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr"/>
-      <c r="D49" t="inlineStr"/>
-      <c r="E49" t="inlineStr"/>
-      <c r="F49" t="inlineStr"/>
-      <c r="G49" t="inlineStr"/>
-      <c r="H49" t="inlineStr"/>
-      <c r="I49" t="inlineStr"/>
-      <c r="J49" t="inlineStr"/>
       <c r="K49" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="L49" t="inlineStr"/>
-      <c r="M49" t="inlineStr"/>
-      <c r="N49" t="inlineStr"/>
-      <c r="O49" t="inlineStr"/>
-      <c r="P49" t="inlineStr"/>
-      <c r="Q49" t="inlineStr"/>
       <c r="R49">
         <f>COUNTIF(C49:Q49,"✓")</f>
         <v/>
@@ -10502,25 +9874,11 @@
           <t>Panel de seguimiento de salud y bienestar</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr"/>
-      <c r="D50" t="inlineStr"/>
-      <c r="E50" t="inlineStr"/>
-      <c r="F50" t="inlineStr"/>
-      <c r="G50" t="inlineStr"/>
       <c r="H50" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="I50" t="inlineStr"/>
-      <c r="J50" t="inlineStr"/>
-      <c r="K50" t="inlineStr"/>
-      <c r="L50" t="inlineStr"/>
-      <c r="M50" t="inlineStr"/>
-      <c r="N50" t="inlineStr"/>
-      <c r="O50" t="inlineStr"/>
-      <c r="P50" t="inlineStr"/>
-      <c r="Q50" t="inlineStr"/>
       <c r="R50">
         <f>COUNTIF(C50:Q50,"✓")</f>
         <v/>
@@ -10537,25 +9895,11 @@
           <t>Registro de nutrición</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr"/>
-      <c r="D51" t="inlineStr"/>
-      <c r="E51" t="inlineStr"/>
-      <c r="F51" t="inlineStr"/>
-      <c r="G51" t="inlineStr"/>
-      <c r="H51" t="inlineStr"/>
-      <c r="I51" t="inlineStr"/>
-      <c r="J51" t="inlineStr"/>
       <c r="K51" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="L51" t="inlineStr"/>
-      <c r="M51" t="inlineStr"/>
-      <c r="N51" t="inlineStr"/>
-      <c r="O51" t="inlineStr"/>
-      <c r="P51" t="inlineStr"/>
-      <c r="Q51" t="inlineStr"/>
       <c r="R51">
         <f>COUNTIF(C51:Q51,"✓")</f>
         <v/>
@@ -10572,25 +9916,11 @@
           <t>Seguimiento de salud femenina</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr"/>
-      <c r="D52" t="inlineStr"/>
-      <c r="E52" t="inlineStr"/>
-      <c r="F52" t="inlineStr"/>
-      <c r="G52" t="inlineStr"/>
-      <c r="H52" t="inlineStr"/>
-      <c r="I52" t="inlineStr"/>
-      <c r="J52" t="inlineStr"/>
       <c r="K52" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="L52" t="inlineStr"/>
-      <c r="M52" t="inlineStr"/>
-      <c r="N52" t="inlineStr"/>
-      <c r="O52" t="inlineStr"/>
-      <c r="P52" t="inlineStr"/>
-      <c r="Q52" t="inlineStr"/>
       <c r="R52">
         <f>COUNTIF(C52:Q52,"✓")</f>
         <v/>
@@ -10607,25 +9937,11 @@
           <t>Valoración de profesionales</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr"/>
-      <c r="D53" t="inlineStr"/>
-      <c r="E53" t="inlineStr"/>
       <c r="F53" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="G53" t="inlineStr"/>
-      <c r="H53" t="inlineStr"/>
-      <c r="I53" t="inlineStr"/>
-      <c r="J53" t="inlineStr"/>
-      <c r="K53" t="inlineStr"/>
-      <c r="L53" t="inlineStr"/>
-      <c r="M53" t="inlineStr"/>
-      <c r="N53" t="inlineStr"/>
-      <c r="O53" t="inlineStr"/>
-      <c r="P53" t="inlineStr"/>
-      <c r="Q53" t="inlineStr"/>
       <c r="R53">
         <f>COUNTIF(C53:Q53,"✓")</f>
         <v/>
@@ -10642,11 +9958,6 @@
           <t>Blockchain para integridad y trazabilidad de datos</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr"/>
-      <c r="D54" t="inlineStr"/>
-      <c r="E54" t="inlineStr"/>
-      <c r="F54" t="inlineStr"/>
-      <c r="G54" t="inlineStr"/>
       <c r="H54" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10662,13 +9973,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="K54" t="inlineStr"/>
-      <c r="L54" t="inlineStr"/>
-      <c r="M54" t="inlineStr"/>
-      <c r="N54" t="inlineStr"/>
-      <c r="O54" t="inlineStr"/>
-      <c r="P54" t="inlineStr"/>
-      <c r="Q54" t="inlineStr"/>
       <c r="R54">
         <f>COUNTIF(C54:Q54,"✓")</f>
         <v/>
@@ -10685,29 +9989,16 @@
           <t>Cifrado y control de acceso</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr"/>
       <c r="D55" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr"/>
-      <c r="F55" t="inlineStr"/>
-      <c r="G55" t="inlineStr"/>
-      <c r="H55" t="inlineStr"/>
-      <c r="I55" t="inlineStr"/>
-      <c r="J55" t="inlineStr"/>
       <c r="K55" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="L55" t="inlineStr"/>
-      <c r="M55" t="inlineStr"/>
-      <c r="N55" t="inlineStr"/>
-      <c r="O55" t="inlineStr"/>
-      <c r="P55" t="inlineStr"/>
-      <c r="Q55" t="inlineStr"/>
       <c r="R55">
         <f>COUNTIF(C55:Q55,"✓")</f>
         <v/>
@@ -10724,25 +10015,11 @@
           <t>Cumplimiento regulatorio de salud y datos</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr"/>
-      <c r="D56" t="inlineStr"/>
-      <c r="E56" t="inlineStr"/>
-      <c r="F56" t="inlineStr"/>
-      <c r="G56" t="inlineStr"/>
-      <c r="H56" t="inlineStr"/>
-      <c r="I56" t="inlineStr"/>
-      <c r="J56" t="inlineStr"/>
-      <c r="K56" t="inlineStr"/>
-      <c r="L56" t="inlineStr"/>
-      <c r="M56" t="inlineStr"/>
-      <c r="N56" t="inlineStr"/>
       <c r="O56" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="P56" t="inlineStr"/>
-      <c r="Q56" t="inlineStr"/>
       <c r="R56">
         <f>COUNTIF(C56:Q56,"✓")</f>
         <v/>
@@ -10759,25 +10036,11 @@
           <t>Gestión de consentimiento sobre uso de datos</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr"/>
-      <c r="D57" t="inlineStr"/>
-      <c r="E57" t="inlineStr"/>
-      <c r="F57" t="inlineStr"/>
-      <c r="G57" t="inlineStr"/>
-      <c r="H57" t="inlineStr"/>
-      <c r="I57" t="inlineStr"/>
-      <c r="J57" t="inlineStr"/>
-      <c r="K57" t="inlineStr"/>
       <c r="L57" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="M57" t="inlineStr"/>
-      <c r="N57" t="inlineStr"/>
-      <c r="O57" t="inlineStr"/>
-      <c r="P57" t="inlineStr"/>
-      <c r="Q57" t="inlineStr"/>
       <c r="R57">
         <f>COUNTIF(C57:Q57,"✓")</f>
         <v/>
@@ -10794,25 +10057,11 @@
           <t>Identidad descentralizada (DID)</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr"/>
-      <c r="D58" t="inlineStr"/>
-      <c r="E58" t="inlineStr"/>
-      <c r="F58" t="inlineStr"/>
-      <c r="G58" t="inlineStr"/>
-      <c r="H58" t="inlineStr"/>
       <c r="I58" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="J58" t="inlineStr"/>
-      <c r="K58" t="inlineStr"/>
-      <c r="L58" t="inlineStr"/>
-      <c r="M58" t="inlineStr"/>
-      <c r="N58" t="inlineStr"/>
-      <c r="O58" t="inlineStr"/>
-      <c r="P58" t="inlineStr"/>
-      <c r="Q58" t="inlineStr"/>
       <c r="R58">
         <f>COUNTIF(C58:Q58,"✓")</f>
         <v/>
@@ -10829,15 +10078,6 @@
           <t>Privacidad reforzada para datos de salud</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr"/>
-      <c r="D59" t="inlineStr"/>
-      <c r="E59" t="inlineStr"/>
-      <c r="F59" t="inlineStr"/>
-      <c r="G59" t="inlineStr"/>
-      <c r="H59" t="inlineStr"/>
-      <c r="I59" t="inlineStr"/>
-      <c r="J59" t="inlineStr"/>
-      <c r="K59" t="inlineStr"/>
       <c r="L59" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10848,10 +10088,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="N59" t="inlineStr"/>
-      <c r="O59" t="inlineStr"/>
-      <c r="P59" t="inlineStr"/>
-      <c r="Q59" t="inlineStr"/>
       <c r="R59">
         <f>COUNTIF(C59:Q59,"✓")</f>
         <v/>
@@ -10868,20 +10104,6 @@
           <t>Modelo freemium y suscripción</t>
         </is>
       </c>
-      <c r="C60" t="inlineStr"/>
-      <c r="D60" t="inlineStr"/>
-      <c r="E60" t="inlineStr"/>
-      <c r="F60" t="inlineStr"/>
-      <c r="G60" t="inlineStr"/>
-      <c r="H60" t="inlineStr"/>
-      <c r="I60" t="inlineStr"/>
-      <c r="J60" t="inlineStr"/>
-      <c r="K60" t="inlineStr"/>
-      <c r="L60" t="inlineStr"/>
-      <c r="M60" t="inlineStr"/>
-      <c r="N60" t="inlineStr"/>
-      <c r="O60" t="inlineStr"/>
-      <c r="P60" t="inlineStr"/>
       <c r="Q60" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10903,25 +10125,11 @@
           <t>Pagos con criptomoneda</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr"/>
-      <c r="D61" t="inlineStr"/>
-      <c r="E61" t="inlineStr"/>
-      <c r="F61" t="inlineStr"/>
-      <c r="G61" t="inlineStr"/>
-      <c r="H61" t="inlineStr"/>
-      <c r="I61" t="inlineStr"/>
       <c r="J61" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="K61" t="inlineStr"/>
-      <c r="L61" t="inlineStr"/>
-      <c r="M61" t="inlineStr"/>
-      <c r="N61" t="inlineStr"/>
-      <c r="O61" t="inlineStr"/>
-      <c r="P61" t="inlineStr"/>
-      <c r="Q61" t="inlineStr"/>
       <c r="R61">
         <f>COUNTIF(C61:Q61,"✓")</f>
         <v/>
@@ -10938,20 +10146,6 @@
           <t>Pagos dentro de la app</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr"/>
-      <c r="D62" t="inlineStr"/>
-      <c r="E62" t="inlineStr"/>
-      <c r="F62" t="inlineStr"/>
-      <c r="G62" t="inlineStr"/>
-      <c r="H62" t="inlineStr"/>
-      <c r="I62" t="inlineStr"/>
-      <c r="J62" t="inlineStr"/>
-      <c r="K62" t="inlineStr"/>
-      <c r="L62" t="inlineStr"/>
-      <c r="M62" t="inlineStr"/>
-      <c r="N62" t="inlineStr"/>
-      <c r="O62" t="inlineStr"/>
-      <c r="P62" t="inlineStr"/>
       <c r="Q62" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10973,25 +10167,11 @@
           <t>Reclamos y trámites con seguros</t>
         </is>
       </c>
-      <c r="C63" t="inlineStr"/>
-      <c r="D63" t="inlineStr"/>
-      <c r="E63" t="inlineStr"/>
-      <c r="F63" t="inlineStr"/>
-      <c r="G63" t="inlineStr"/>
-      <c r="H63" t="inlineStr"/>
       <c r="I63" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="J63" t="inlineStr"/>
-      <c r="K63" t="inlineStr"/>
-      <c r="L63" t="inlineStr"/>
-      <c r="M63" t="inlineStr"/>
-      <c r="N63" t="inlineStr"/>
-      <c r="O63" t="inlineStr"/>
-      <c r="P63" t="inlineStr"/>
-      <c r="Q63" t="inlineStr"/>
       <c r="R63">
         <f>COUNTIF(C63:Q63,"✓")</f>
         <v/>
@@ -11008,25 +10188,11 @@
           <t>Teleconsulta con profesionales</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr"/>
-      <c r="D64" t="inlineStr"/>
-      <c r="E64" t="inlineStr"/>
-      <c r="F64" t="inlineStr"/>
-      <c r="G64" t="inlineStr"/>
-      <c r="H64" t="inlineStr"/>
-      <c r="I64" t="inlineStr"/>
       <c r="J64" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="K64" t="inlineStr"/>
-      <c r="L64" t="inlineStr"/>
-      <c r="M64" t="inlineStr"/>
-      <c r="N64" t="inlineStr"/>
-      <c r="O64" t="inlineStr"/>
-      <c r="P64" t="inlineStr"/>
-      <c r="Q64" t="inlineStr"/>
       <c r="R64">
         <f>COUNTIF(C64:Q64,"✓")</f>
         <v/>
@@ -11043,7 +10209,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A21"/>
+  <dimension ref="A1:A22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -11196,6 +10362,13 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Vuelta 5 (iter. 1, 2026-10-09 12:16 UTC): Meedika, Infomed, MediPlanner, Clingot verificados (+0 filas). Nota: la rutina pasó a ejecución diaria (12:15 UTC) por cambio del usuario del 2026-10-08. Pendientes: Healfies, Patientory, MediBloc, Medicalchain, Apple Health, ChatGPT Health, Claude for Healthcare, Apps de clínicas, Clinia, MiRedSalud, Mediko.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Benchmark: vuelta 5, iteración 2 (Healfies, Patientory, MediBloc, Medicalchain)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MVcXu8vTBu7EKfj3YdEvae
</commit_message>
<xml_diff>
--- a/Outputs/Benchmark_Anamnesis.xlsx
+++ b/Outputs/Benchmark_Anamnesis.xlsx
@@ -673,12 +673,12 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>[REGIONAL · Brasil] Fundada ene-2015 en Florianópolis por Helyson Lewis Velasco. Centraliza registros de salud personales: carpetas, etiquetas, línea de tiempo (medicación, exámenes, citas, dieta), compartir con familia o profesionales. Gratis; web, iOS y Android. Estado actual NO verificado (fuentes de 2015-2016). Referencia funcional cercana a etapas A+B. [Vuelta 2] Lanzada simultáneamente en Brasil, Argentina y EE.UU.; permite compartir con no registrados vía clave por email. Sin novedades posteriores a 2016. [Vuelta 3] Sin evidencia de actividad reciente ni de cierre; Gust/Dealroom la listan en Florianópolis (10 empleados, healfies.com) sin fecha de actualización. Estado sin confirmar. [Vuelta 4] Sin Google Play localizado; no confundir con la app Healfy (otro producto). Sin novedades.</t>
+          <t>[REGIONAL · Brasil] Fundada ene-2015 en Florianópolis por Helyson Lewis Velasco. Centraliza registros de salud personales: carpetas, etiquetas, línea de tiempo (medicación, exámenes, citas, dieta), compartir con familia o profesionales. Gratis; web, iOS y Android. Estado actual NO verificado (fuentes de 2015-2016). Referencia funcional cercana a etapas A+B. [Vuelta 2] Lanzada simultáneamente en Brasil, Argentina y EE.UU.; permite compartir con no registrados vía clave por email. Sin novedades posteriores a 2016. [Vuelta 3] Sin evidencia de actividad reciente ni de cierre; Gust/Dealroom la listan en Florianópolis (10 empleados, healfies.com) sin fecha de actualización. Estado sin confirmar. [Vuelta 4] Sin Google Play localizado; no confundir con la app Healfy (otro producto). Sin novedades. [Vuelta 5] Sin búsqueda nueva (revisada en vuelta 4); sin cambios.</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G6" t="n">
@@ -686,7 +686,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-10</t>
         </is>
       </c>
     </row>
@@ -713,12 +713,12 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>[BLOCKCHAIN · EE.UU.] Atlanta, fundada 2015, ~9 empleados. Levantó US$7,2M vía financiamiento cripto. App con registros de hospitales y wearables, coaching de salud con IA y recompensas en cripto; también dashboard empresarial Neith. PitchBook indica actividad y financiamiento hasta abr-2026: sigue operando. Sin presencia conocida en Chile. Referencia directa para la hipótesis blockchain. [Vuelta 2] Sin noticias 2026 encontradas en búsqueda; sitio oficial bloqueado. [Vuelta 3] Búsqueda adicional solo devuelve hitos de 2017 (token sale US$7,2M) y 2019 (Serie A de US$5,3M, cierre no confirmado); sin datos 2025-26 propios. [Vuelta 4] App pública lanzada en la conferencia JP Morgan Healthcare (2019); red PTOYMatrix (blockchain HIPAA); socios reportados: StartUp Health y Kaiser Permanente (beta). Estado actual en App Store/Google Play sin confirmar.</t>
+          <t>[BLOCKCHAIN · EE.UU.] Atlanta, fundada 2015, ~9 empleados. Levantó US$7,2M vía financiamiento cripto. App con registros de hospitales y wearables, coaching de salud con IA y recompensas en cripto; también dashboard empresarial Neith. PitchBook indica actividad y financiamiento hasta abr-2026: sigue operando. Sin presencia conocida en Chile. Referencia directa para la hipótesis blockchain. [Vuelta 2] Sin noticias 2026 encontradas en búsqueda; sitio oficial bloqueado. [Vuelta 3] Búsqueda adicional solo devuelve hitos de 2017 (token sale US$7,2M) y 2019 (Serie A de US$5,3M, cierre no confirmado); sin datos 2025-26 propios. [Vuelta 4] App pública lanzada en la conferencia JP Morgan Healthcare (2019); red PTOYMatrix (blockchain HIPAA); socios reportados: StartUp Health y Kaiser Permanente (beta). Estado actual en App Store/Google Play sin confirmar. [Vuelta 5] Sin noticias 2026 del equipo. Token PTOY con capitalización de ~US$53K a fines de ago-2026 según Phantom (KuCoin discrepa en la circulación): señal de baja actividad, no prueba de cierre. Esto relativiza la actividad hasta abr-2026 mencionada en la ficha original.</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G7" t="n">
@@ -726,7 +726,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-10</t>
         </is>
       </c>
     </row>
@@ -753,12 +753,12 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>[BLOCKCHAIN · Corea del Sur] Fundada 2017, Seúl. Blockchain propia Panacea (Cosmos SDK, mainnet 2019) para que el paciente gestione y transfiera sus registros; app Medipass para seguros. Serie A de ₩4.000 millones (Naver); alianzas con hospitales (Seoul National, Severance). Estado 2025-26 NO verificado. Referencia sobre seguros + blockchain. [Vuelta 2] Panacea incluye DID, Append Only Log, IBC y PNFT; sin anuncios 2026 localizados. [Vuelta 3] Medipass: app en Corea con 20 hospitales/aseguradoras integrados (fecha de la lista desconocida) y plan 2022 de superapp con marketplace de datos; operación actual sin confirmar. [Vuelta 4] Sin búsqueda nueva (revisada en vuelta 3); sin cambios.</t>
+          <t>[BLOCKCHAIN · Corea del Sur] Fundada 2017, Seúl. Blockchain propia Panacea (Cosmos SDK, mainnet 2019) para que el paciente gestione y transfiera sus registros; app Medipass para seguros. Serie A de ₩4.000 millones (Naver); alianzas con hospitales (Seoul National, Severance). Estado 2025-26 NO verificado. Referencia sobre seguros + blockchain. [Vuelta 2] Panacea incluye DID, Append Only Log, IBC y PNFT; sin anuncios 2026 localizados. [Vuelta 3] Medipass: app en Corea con 20 hospitales/aseguradoras integrados (fecha de la lista desconocida) y plan 2022 de superapp con marketplace de datos; operación actual sin confirmar. [Vuelta 4] Sin búsqueda nueva (revisada en vuelta 3); sin cambios. [Vuelta 5] Medipass: ~400.000 usuarios acumulados (CEO, jun-2022); integración con aseguradoras Shinhan Life, Samsung Fire y Hyundai Marine (2020); renovación completa en mar-2023 (dashboard de salud, gestión familiar, certificados). Sin noticias 2026 encontradas.</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G8" t="n">
@@ -766,7 +766,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-10</t>
         </is>
       </c>
     </row>
@@ -793,12 +793,12 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>[BLOCKCHAIN · Reino Unido · INACTIVO] Londres, 2017, Ethereum, con telemedicina. Piloto según registro de la UE (2020). Tracxn/PitchBook lo marcan fuera de operación (ago-2025). Solo caso de aprendizaje: no cuenta como competidor activo. [Vuelta 2] Token MTN deslistado de Bitfinex el 26-mar-2021; sin hallazgos de actividad posterior. [Vuelta 3] Seedtable la marca activa sin fuente; no hallé registro en Companies House. Sigue tratándose como caso de aprendizaje. [Vuelta 4] Pre-venta reportada de US$20M en MedTokens (un solo artículo secundario, sin verificar); modelo de token en revisión y exploración de security token según AMA; integraciones y servicios de 2019 sin confirmar.</t>
+          <t>[BLOCKCHAIN · Reino Unido · INACTIVO] Londres, 2017, Ethereum, con telemedicina. Piloto según registro de la UE (2020). Tracxn/PitchBook lo marcan fuera de operación (ago-2025). Solo caso de aprendizaje: no cuenta como competidor activo. [Vuelta 2] Token MTN deslistado de Bitfinex el 26-mar-2021; sin hallazgos de actividad posterior. [Vuelta 3] Seedtable la marca activa sin fuente; no hallé registro en Companies House. Sigue tratándose como caso de aprendizaje. [Vuelta 4] Pre-venta reportada de US$20M en MedTokens (un solo artículo secundario, sin verificar); modelo de token en revisión y exploración de security token según AMA; integraciones y servicios de 2019 sin confirmar. [Vuelta 5] Un agregador indica sitio medicalchain.com fuera de línea desde 15-feb-2025, último commit en GitHub hace ~3 años y proyecto en «fase de mantenimiento»; preventa de MedTokens reportada entre US$20M y US$24M (fuentes discrepan). Confirma tratarlo como inactivo.</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G9" t="n">
@@ -806,7 +806,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-10</t>
         </is>
       </c>
     </row>
@@ -1102,7 +1102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F125"/>
+  <dimension ref="A1:F127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -5110,6 +5110,70 @@
       <c r="F125" t="inlineStr">
         <is>
           <t>Búsqueda web (Pauta / Descubre.vc, 2024); estado actual sin verificar</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>MediBloc</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Familia y dependientes</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Gestión familiar (Medipass renovado, 2023)</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>El relanzamiento de Medipass (mar-2023) incorporó gestión de la salud de familiares.</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>Búsqueda web (Medigate News, mar-2023)</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>MediBloc</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Seguimiento y bienestar</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Dashboard de gestión de información de salud</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>El relanzamiento de Medipass (mar-2023) agregó un panel para gestionar la información de salud del usuario.</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>Búsqueda web (Medigate News, mar-2023)</t>
         </is>
       </c>
     </row>
@@ -10209,7 +10273,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A22"/>
+  <dimension ref="A1:A23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -10369,6 +10433,13 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Vuelta 5 (iter. 2, 2026-10-10 12:15 UTC): Healfies, Patientory, MediBloc, Medicalchain verificados (+2 filas, de MediBloc). Pendientes: Apple Health, ChatGPT Health, Claude for Healthcare, Apps de clínicas, Clinia, MiRedSalud, Mediko.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Benchmark: vuelta 5, iteración 3 (Apple Health, ChatGPT Health, Claude for Healthcare, Apps de clínicas)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MVcXu8vTBu7EKfj3YdEvae
</commit_message>
<xml_diff>
--- a/Outputs/Benchmark_Anamnesis.xlsx
+++ b/Outputs/Benchmark_Anamnesis.xlsx
@@ -833,12 +833,12 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>[ADYACENTE · global] Agrega registros clínicos vía FHIR; &gt;500 instituciones conectadas en EE.UU. (2018). Sin evidencia de disponibilidad en Chile. Incluida en el dispositivo. Amenaza si FHIR/IPS-CL se adopta en Chile. [Vuelta 2] Sin disponibilidad de registros clínicos en Chile (solo EE.UU., Reino Unido, Canadá). [Vuelta 3] iOS 27 (WWDC 8-jun-2026; publicado ~14-sep-2026): rediseño del app Health, menopausia, nutrición por cámara. El coach de salud con IA no se anunció. Sin ampliación de Health Records a Chile. [Vuelta 4] Sin búsqueda nueva (revisada en vuelta 3); sin cambios.</t>
+          <t>[ADYACENTE · global] Agrega registros clínicos vía FHIR; &gt;500 instituciones conectadas en EE.UU. (2018). Sin evidencia de disponibilidad en Chile. Incluida en el dispositivo. Amenaza si FHIR/IPS-CL se adopta en Chile. [Vuelta 2] Sin disponibilidad de registros clínicos en Chile (solo EE.UU., Reino Unido, Canadá). [Vuelta 3] iOS 27 (WWDC 8-jun-2026; publicado ~14-sep-2026): rediseño del app Health, menopausia, nutrición por cámara. El coach de salud con IA no se anunció. Sin ampliación de Health Records a Chile. [Vuelta 4] Sin búsqueda nueva (revisada en vuelta 3); sin cambios. [Vuelta 5] Sin ampliación de Health Records a Australia, Europa ni Latinoamérica (solo EE.UU., UK, Canadá). Funciones de dispositivo (apnea del sueño, prueba auditiva) sí se amplían a países latinoamericanos, pero no son registros clínicos.</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G10" t="n">
@@ -846,7 +846,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-11</t>
         </is>
       </c>
     </row>
@@ -873,12 +873,12 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>[ADYACENTE · global] Lanzado 7-ene-2026. Conecta registros médicos; conectores solo en EE.UU. Dentro de suscripción del asistente. Fija la expectativa de consultar y resumir el historial. [Vuelta 2] Confirmado: registros solo EE.UU.; sin anuncios para Latinoamérica. Hay inconsistencia de fechas entre fuentes (7-ene-2026 lanzamiento vs. jul-2026 despliegue de registros). [Vuelta 3] Fechas aclaradas: presentación 7-ene-2026 (acceso limitado); despliegue de Health in ChatGPT con Apple Health y registros en EE.UU. el 23-jul-2026; mejora de salud jun-2026. Sin anuncios para Latinoamérica ni para sep-oct 2026. [Vuelta 4] Septiembre 2026: permisos por defecto para datos conectados (14-sep) y explicaciones por gráfico/métrica (28-sep); ChatGPT for Clinicians (abr-2026) para clínicos verificados de EE.UU. Más del 70% de usuarios de Health permite usar datos conectados sin pedir permiso (según OpenAI). Sigue solo EE.UU.</t>
+          <t>[ADYACENTE · global] Lanzado 7-ene-2026. Conecta registros médicos; conectores solo en EE.UU. Dentro de suscripción del asistente. Fija la expectativa de consultar y resumir el historial. [Vuelta 2] Confirmado: registros solo EE.UU.; sin anuncios para Latinoamérica. Hay inconsistencia de fechas entre fuentes (7-ene-2026 lanzamiento vs. jul-2026 despliegue de registros). [Vuelta 3] Fechas aclaradas: presentación 7-ene-2026 (acceso limitado); despliegue de Health in ChatGPT con Apple Health y registros en EE.UU. el 23-jul-2026; mejora de salud jun-2026. Sin anuncios para Latinoamérica ni para sep-oct 2026. [Vuelta 4] Septiembre 2026: permisos por defecto para datos conectados (14-sep) y explicaciones por gráfico/métrica (28-sep); ChatGPT for Clinicians (abr-2026) para clínicos verificados de EE.UU. Más del 70% de usuarios de Health permite usar datos conectados sin pedir permiso (según OpenAI). Sigue solo EE.UU. [Vuelta 5] Nota de jul-2026: Health no está disponible en México, Android, modo de voz ni Codex; web e iOS en EE.UU., adultos con sesión iniciada. Sin anuncio para Chile ni Latinoamérica.</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G11" t="n">
@@ -886,7 +886,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-11</t>
         </is>
       </c>
     </row>
@@ -913,12 +913,12 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>[ADYACENTE · global] Lanzado 11-ene-2026. Conectores solo en EE.UU., planes Pro/Max. Nota: producto de Anthropic, conflicto de interés al evaluarlo. [Vuelta 2] Sin cambios fuera de EE.UU. (HealthEx y Function para Pro/Max). [Vuelta 3] Sin anuncios posteriores a enero de 2026. Hoja de ruta de HealthEx (agendar, buscar prestadores, recetas) sin confirmar como lanzada. [Vuelta 4] Sin anuncios nuevos. Fuentes discrepan en el acceso (Pro/Max según Fortune y la mayoría; Pro/Team según Times of AI); sin evidencia de disponibilidad fuera de EE.UU.</t>
+          <t>[ADYACENTE · global] Lanzado 11-ene-2026. Conectores solo en EE.UU., planes Pro/Max. Nota: producto de Anthropic, conflicto de interés al evaluarlo. [Vuelta 2] Sin cambios fuera de EE.UU. (HealthEx y Function para Pro/Max). [Vuelta 3] Sin anuncios posteriores a enero de 2026. Hoja de ruta de HealthEx (agendar, buscar prestadores, recetas) sin confirmar como lanzada. [Vuelta 4] Sin anuncios nuevos. Fuentes discrepan en el acceso (Pro/Max según Fortune y la mayoría; Pro/Team según Times of AI); sin evidencia de disponibilidad fuera de EE.UU. [Vuelta 5] Sin noticias de oct-2026; HealthEx agrega datos de &gt;50.000 sistemas de EE.UU. y Claude pide solo las categorías relevantes vía MCP.</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G12" t="n">
@@ -926,7 +926,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-11</t>
         </is>
       </c>
     </row>
@@ -953,12 +953,12 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>[SUSTITUTO PARCIAL · Chile] Reservar hora, ver historial de esa institución, vincular familiar. Gratis; no consolida datos de otras instituciones. [Vuelta 2] App concreta: Mi Alemana Go (Clínica Alemana, Chile), con historial desde 2018, recetas, órdenes, familiar vinculado y resultados. [Vuelta 3] Búsqueda de otras clínicas (Las Condes, Santa María, UC Christus) sin ficha de app confirmada; solo canales digitales genéricos. [Vuelta 4] Mi Alemana Go: 3,1/5 con 137 calificaciones (App Store Chile), pantalla de inicio rediseñada para gestionar salud propia y familiar; sin evidencia de teleconsulta ni pagos en la app.</t>
+          <t>[SUSTITUTO PARCIAL · Chile] Reservar hora, ver historial de esa institución, vincular familiar. Gratis; no consolida datos de otras instituciones. [Vuelta 2] App concreta: Mi Alemana Go (Clínica Alemana, Chile), con historial desde 2018, recetas, órdenes, familiar vinculado y resultados. [Vuelta 3] Búsqueda de otras clínicas (Las Condes, Santa María, UC Christus) sin ficha de app confirmada; solo canales digitales genéricos. [Vuelta 4] Mi Alemana Go: 3,1/5 con 137 calificaciones (App Store Chile), pantalla de inicio rediseñada para gestionar salud propia y familiar; sin evidencia de teleconsulta ni pagos en la app. [Vuelta 5] Sin búsqueda nueva (revisada en vuelta 4); sin cambios.</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G13" t="n">
@@ -966,7 +966,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-11</t>
         </is>
       </c>
     </row>
@@ -1102,7 +1102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F127"/>
+  <dimension ref="A1:F128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -5174,6 +5174,38 @@
       <c r="F127" t="inlineStr">
         <is>
           <t>Búsqueda web (Medigate News, mar-2023)</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>Claude for Healthcare (Anthropic)</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Seguridad, privacidad y blockchain</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Acceso por categorías de datos vía MCP (HealthEx)</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>Claude solicita solo las categorías relevantes (p. ej. medicamentos o laboratorio) y no fichas completas; HealthEx agrega datos de más de 50.000 sistemas de salud de EE.UU.</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>Búsqueda web (Unite.ai, Fortune, TechStrong); solo EE.UU., Pro/Max</t>
         </is>
       </c>
     </row>
@@ -10273,7 +10305,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A23"/>
+  <dimension ref="A1:A24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -10440,6 +10472,13 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Vuelta 5 (iter. 3, 2026-10-11 12:16 UTC): Apple Health, ChatGPT Health, Claude for Healthcare, Apps de clínicas verificados (+1 fila). Pendientes: Clinia, MiRedSalud, Mediko (cierran la vuelta 5 y regeneran func_norm/tabla_frecuencia).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Benchmark: cierre vuelta 5; contador=5; func_norm y tabla_frecuencia regenerados
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MVcXu8vTBu7EKfj3YdEvae
</commit_message>
<xml_diff>
--- a/Outputs/Benchmark_Anamnesis.xlsx
+++ b/Outputs/Benchmark_Anamnesis.xlsx
@@ -518,15 +518,15 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -558,15 +558,15 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -598,15 +598,15 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -638,15 +638,15 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G5" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -678,15 +678,15 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -718,15 +718,15 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -758,15 +758,15 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G8" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -798,15 +798,15 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G9" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -838,15 +838,15 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -878,15 +878,15 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G11" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -918,15 +918,15 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G12" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -958,15 +958,15 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G13" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -993,7 +993,7 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>[DIRECTO · Chile · etapa A] App móvil anunciada en sep-2026 para centralizar recetas, diagnósticos y laboratorios en un solo lugar; respaldada por Reservo (tecnológica chilena desde 2015, software para profesionales y centros de salud). AMENAZA ALTA: Reservo ya tiene red de profesionales/centros que podrían alimentar el historial. Fuente: solo snippet de búsqueda (sitio bloqueado en este entorno); precio, funciones de compartir y sitio oficial por verificar. [Vuelta 2] Confirmado por el CEO de Reservo (LinkedIn): app para pacientes en App Store y Google Play; guarda y comparte exámenes, recetas, órdenes y certificados. Fecha exacta de lanzamiento, precio y modelo de datos sin verificar. [Vuelta 3] Sin novedades de oct-2026. Reservo (Chile, México, Argentina) declara certificación Fonasa/CENS y cumplimiento de la nueva ley de datos personales; el Portal de Agendamiento de Reservo complementa a Clinia. Precio y modelo de datos sin verificar. [Vuelta 4] Una búsqueda adicional no encontró fuentes independientes sobre Clinia de Reservo (aparecen otras empresas llamadas Clinia); la evidencia sigue siendo la publicación del CEO en LinkedIn y notas de Reservo. Confianza media.</t>
+          <t>[DIRECTO · Chile · etapa A] App móvil anunciada en sep-2026 para centralizar recetas, diagnósticos y laboratorios en un solo lugar; respaldada por Reservo (tecnológica chilena desde 2015, software para profesionales y centros de salud). AMENAZA ALTA: Reservo ya tiene red de profesionales/centros que podrían alimentar el historial. Fuente: solo snippet de búsqueda (sitio bloqueado en este entorno); precio, funciones de compartir y sitio oficial por verificar. [Vuelta 2] Confirmado por el CEO de Reservo (LinkedIn): app para pacientes en App Store y Google Play; guarda y comparte exámenes, recetas, órdenes y certificados. Fecha exacta de lanzamiento, precio y modelo de datos sin verificar. [Vuelta 3] Sin novedades de oct-2026. Reservo (Chile, México, Argentina) declara certificación Fonasa/CENS y cumplimiento de la nueva ley de datos personales; el Portal de Agendamiento de Reservo complementa a Clinia. Precio y modelo de datos sin verificar. [Vuelta 4] Una búsqueda adicional no encontró fuentes independientes sobre Clinia de Reservo (aparecen otras empresas llamadas Clinia); la evidencia sigue siendo la publicación del CEO en LinkedIn y notas de Reservo. Confianza media. [Vuelta 5] Sin fecha verificable del lanzamiento (publicación de LinkedIn del CEO sin fecha visible); existe otra empresa homónima en Brasil (Porto Alegre, IA para clínicas) que no es este producto. Sin funciones nuevas.</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1002,11 +1002,11 @@
         </is>
       </c>
       <c r="G14" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -1033,7 +1033,7 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>[SUSTITUTO PARCIAL · Chile] Nueva app móvil de la red RedSalud anunciada dic-2025: acceso a información clínica y servicios, guardar y administrar historial propio y familiar. Limitación: solo datos de la propia red; no consolida otras instituciones. Precio por verificar (probablemente gratis). [Vuelta 2] La búsqueda no encontró fuentes adicionales ni ficha de la app chilena (solo una app RedSalud de otro país); funciones sin confirmar. [Vuelta 3] Rankings de terceros la ubican como app médica gratuita nº 1 en App Store y Google Play Chile (fecha desconocida); sin descripción de funciones ni confirmación del desarrollador en Google Play. [Vuelta 4] Sin documentación oficial chilena localizada; las fichas con funciones (agendar, telemedicina, historial de hijos) corresponden a una app RedSalud de otro país. Quejas públicas 2020-21 sobre acceso en línea a resultados. Funciones de MiRedSalud sin confirmar.</t>
+          <t>[SUSTITUTO PARCIAL · Chile] Nueva app móvil de la red RedSalud anunciada dic-2025: acceso a información clínica y servicios, guardar y administrar historial propio y familiar. Limitación: solo datos de la propia red; no consolida otras instituciones. Precio por verificar (probablemente gratis). [Vuelta 2] La búsqueda no encontró fuentes adicionales ni ficha de la app chilena (solo una app RedSalud de otro país); funciones sin confirmar. [Vuelta 3] Rankings de terceros la ubican como app médica gratuita nº 1 en App Store y Google Play Chile (fecha desconocida); sin descripción de funciones ni confirmación del desarrollador en Google Play. [Vuelta 4] Sin documentación oficial chilena localizada; las fichas con funciones (agendar, telemedicina, historial de hijos) corresponden a una app RedSalud de otro país. Quejas públicas 2020-21 sobre acceso en línea a resultados. Funciones de MiRedSalud sin confirmar. [Vuelta 5] Una búsqueda adicional no halló cobertura del lanzamiento de dic-2025 ni de la app chilena; solo apps de otras empresas Red Salud (Paraguay, Perú). Sigue sin confirmarse más allá de la nota de RedSalud.</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1042,11 +1042,11 @@
         </is>
       </c>
       <c r="G15" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -1073,7 +1073,7 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>[ADYACENTE · Chile] Fundada 2022. Orientación médica inmediata, interpretación de exámenes y órdenes médicas digitales con IA; modelo freemium, suscripción y pago por servicio; menciona centralizar registros y monitoreo. Foco asistencial, no archivo personal; vigilar si añade historial. Grants por ~$40M según Descubre.vc. [Vuelta 2] Sin precios ni planes vigentes localizados; sitio oficial bloqueado. [Vuelta 3] Pauta (oct-2024): su fundador, Tomás Riddell, dice que no reemplaza a médicos y apunta a lo ambulatorio y a la espera de derivación a especialidad en el sistema público. Financiamiento: fuentes discrepan (CLP 25M en dic-2023 según Bouncewatch; ~$40M según Descubre.vc). Precios vigentes sin verificar. [Vuelta 4] Entrevista oct-2024 menciona integración con la pasarela Flow. Sin novedades 2025-26 ni rondas verificadas; la cifra de US$40M de Bouncewatch es dudosa (perfil con 2 empleados).</t>
+          <t>[ADYACENTE · Chile] Fundada 2022. Orientación médica inmediata, interpretación de exámenes y órdenes médicas digitales con IA; modelo freemium, suscripción y pago por servicio; menciona centralizar registros y monitoreo. Foco asistencial, no archivo personal; vigilar si añade historial. Grants por ~$40M según Descubre.vc. [Vuelta 2] Sin precios ni planes vigentes localizados; sitio oficial bloqueado. [Vuelta 3] Pauta (oct-2024): su fundador, Tomás Riddell, dice que no reemplaza a médicos y apunta a lo ambulatorio y a la espera de derivación a especialidad en el sistema público. Financiamiento: fuentes discrepan (CLP 25M en dic-2023 según Bouncewatch; ~$40M según Descubre.vc). Precios vigentes sin verificar. [Vuelta 4] Entrevista oct-2024 menciona integración con la pasarela Flow. Sin novedades 2025-26 ni rondas verificadas; la cifra de US$40M de Bouncewatch es dudosa (perfil con 2 empleados). [Vuelta 5] CORRECCIÓN de financiamiento: Bouncewatch registra dos subvenciones (CLP 15M en ago-2022 y CLP 25M en dic-2023 = CLP 40M en total), no US$40M; 2 empleados; etapa Seed según Descubre.vc. No hay inversionistas de capital listados.</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1082,11 +1082,11 @@
         </is>
       </c>
       <c r="G16" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -5220,7 +5220,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E125"/>
+  <dimension ref="A1:E128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -6070,7 +6070,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>MediPlanner</t>
+          <t>MediBloc</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -6085,19 +6085,19 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Historial por perfil para cada miembro de la familia.</t>
+          <t>El relanzamiento de Medipass (mar-2023) incorporó gestión de la salud de familiares.</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Latam</t>
+          <t>Global</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>MiRedSalud (RedSalud)</t>
+          <t>MediPlanner</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -6112,46 +6112,46 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Guardar y administrar historial propio y familiar.</t>
+          <t>Historial por perfil para cada miembro de la familia.</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Latam</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Clingot</t>
+          <t>MiRedSalud (RedSalud)</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Gestión documental</t>
+          <t>Familia y dependientes</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Almacenamiento de documentos médicos</t>
+          <t>Perfiles familiares / dependientes</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Sube estudios, imágenes, indicaciones médicas y notas personales; accesible en consulta o por terceros en emergencias.</t>
+          <t>Guardar y administrar historial propio y familiar.</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Latam</t>
+          <t>Chile</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Clinia (Reservo)</t>
+          <t>Clingot</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -6166,12 +6166,12 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Reúne recetas, diagnósticos y laboratorios en un solo lugar.</t>
+          <t>Sube estudios, imágenes, indicaciones médicas y notas personales; accesible en consulta o por terceros en emergencias.</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Latam</t>
         </is>
       </c>
     </row>
@@ -6193,7 +6193,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Guarda en un solo lugar exámenes, recetas, órdenes y certificados médicos.</t>
+          <t>Reúne recetas, diagnósticos y laboratorios en un solo lugar.</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -6205,7 +6205,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Healfies</t>
+          <t>Clinia (Reservo)</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -6220,19 +6220,19 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Organiza registros con carpetas y etiquetas.</t>
+          <t>Guarda en un solo lugar exámenes, recetas, órdenes y certificados médicos.</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Latam</t>
+          <t>Chile</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Meedika</t>
+          <t>Healfies</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -6247,19 +6247,19 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Almacena documentos clínicos del usuario en la app.</t>
+          <t>Organiza registros con carpetas y etiquetas.</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Latam</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Patientory</t>
+          <t>Meedika</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -6274,19 +6274,19 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Administra fechas, prescripciones, archivos y citas desde la app.</t>
+          <t>Almacena documentos clínicos del usuario en la app.</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Chile</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Apps de clínicas (ej. Clínica Alemana de Valdivia)</t>
+          <t>Patientory</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -6296,24 +6296,24 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Almacenamiento de recetas</t>
+          <t>Almacenamiento de documentos médicos</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Ver y descargar recetas, órdenes de examen y derivaciones.</t>
+          <t>Administra fechas, prescripciones, archivos y citas desde la app.</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Global</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>MediPlanner</t>
+          <t>Apps de clínicas (ej. Clínica Alemana de Valdivia)</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -6328,12 +6328,12 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Guarda recetas digitales.</t>
+          <t>Ver y descargar recetas, órdenes de examen y derivaciones.</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Latam</t>
+          <t>Chile</t>
         </is>
       </c>
     </row>
@@ -6350,12 +6350,12 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Búsqueda y filtros de documentos</t>
+          <t>Almacenamiento de recetas</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Guarda resultados de laboratorio, imágenes y PDFs; búsqueda y filtros.</t>
+          <t>Guarda recetas digitales.</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -6367,7 +6367,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>MediBloc</t>
+          <t>MediPlanner</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -6377,24 +6377,24 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Emisión de certificados médicos</t>
+          <t>Búsqueda y filtros de documentos</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>La ficha de la app incluye consulta de chequeos de salud y emisión de certificados médicos.</t>
+          <t>Guarda resultados de laboratorio, imágenes y PDFs; búsqueda y filtros.</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Latam</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Mediko</t>
+          <t>MediBloc</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -6404,24 +6404,24 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Importación de órdenes/solicitudes médicas</t>
+          <t>Emisión de certificados médicos</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Descarga/genera órdenes médicas digitales.</t>
+          <t>La ficha de la app incluye consulta de chequeos de salud y emisión de certificados médicos.</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Global</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Meedika</t>
+          <t>Mediko</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -6436,7 +6436,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Importa solicitudes (órdenes) médicas a la app.</t>
+          <t>Descarga/genera órdenes médicas digitales.</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -6448,7 +6448,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Apps de clínicas (ej. Clínica Alemana de Valdivia)</t>
+          <t>Meedika</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -6458,12 +6458,12 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Notificación y envío de resultados</t>
+          <t>Importación de órdenes/solicitudes médicas</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Avisa cuando hay exámenes/documentos disponibles; resultados de laboratorio y anatomía patológica compartibles por email o WhatsApp.</t>
+          <t>Importa solicitudes (órdenes) médicas a la app.</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -6480,17 +6480,17 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Historial y perfil clínico</t>
+          <t>Gestión documental</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Historial institucional (solo datos de la propia red)</t>
+          <t>Notificación y envío de resultados</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Ve historial de esa institución.</t>
+          <t>Avisa cuando hay exámenes/documentos disponibles; resultados de laboratorio y anatomía patológica compartibles por email o WhatsApp.</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -6517,7 +6517,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Historial institucional de consultas, urgencias y hospitalizaciones (solo datos de esa clínica).</t>
+          <t>Ve historial de esa institución.</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -6529,7 +6529,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>MiRedSalud (RedSalud)</t>
+          <t>Apps de clínicas (ej. Clínica Alemana de Valdivia)</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -6544,7 +6544,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Acceso a información clínica de la red.</t>
+          <t>Historial institucional de consultas, urgencias y hospitalizaciones (solo datos de esa clínica).</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -6556,7 +6556,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Apple Health (Health Records)</t>
+          <t>MiRedSalud (RedSalud)</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -6566,24 +6566,24 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Historial médico centralizado</t>
+          <t>Historial institucional (solo datos de la propia red)</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Información clínica unificada.</t>
+          <t>Acceso a información clínica de la red.</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Chile</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Clingot</t>
+          <t>Apple Health (Health Records)</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -6598,19 +6598,19 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>El usuario registra sus antecedentes médicos en la app.</t>
+          <t>Información clínica unificada.</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Latam</t>
+          <t>Global</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Infomed</t>
+          <t>Clingot</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -6625,19 +6625,19 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Centraliza el historial médico personal en el móvil.</t>
+          <t>El usuario registra sus antecedentes médicos en la app.</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Latam</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>MediBloc</t>
+          <t>Infomed</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -6652,19 +6652,19 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Permite compilar datos de vida/salud, gestionarlos y pasarlos a instituciones médicas.</t>
+          <t>Centraliza el historial médico personal en el móvil.</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Chile</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Mediko</t>
+          <t>MediBloc</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -6679,19 +6679,19 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Centralizar registros y monitoreo desde el móvil.</t>
+          <t>Permite compilar datos de vida/salud, gestionarlos y pasarlos a instituciones médicas.</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Global</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Healfies</t>
+          <t>Mediko</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -6701,17 +6701,17 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Línea de tiempo de salud</t>
+          <t>Historial médico centralizado</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Línea de tiempo con medicación, exámenes, citas y dieta.</t>
+          <t>Centralizar registros y monitoreo desde el móvil.</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Latam</t>
+          <t>Chile</t>
         </is>
       </c>
     </row>
@@ -6733,7 +6733,7 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Registra notas de medicación, exámenes (laboratorio e imagen), actividad física, recetas, dieta y citas.</t>
+          <t>Línea de tiempo con medicación, exámenes, citas y dieta.</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -6745,7 +6745,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>MediPlanner</t>
+          <t>Healfies</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -6755,12 +6755,12 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Registro de alergias y vacunas</t>
+          <t>Línea de tiempo de salud</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Registro de alergias y vacunas.</t>
+          <t>Registra notas de medicación, exámenes (laboratorio e imagen), actividad física, recetas, dieta y citas.</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -6772,7 +6772,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Patientory</t>
+          <t>MediPlanner</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -6782,39 +6782,39 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Seguimiento de visitas, gastos y seguros</t>
+          <t>Registro de alergias y vacunas</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>App gratuita para seguir visitas al médico, facturas médicas, datos personales, seguros, inmunizaciones y medicamentos de farmacia.</t>
+          <t>Registro de alergias y vacunas.</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Latam</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>MediBloc</t>
+          <t>Patientory</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Incentivos y monetización de datos</t>
+          <t>Historial y perfil clínico</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Recompensas / monetización de datos del usuario</t>
+          <t>Seguimiento de visitas, gastos y seguros</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Plan de convertir Medipass en superapp con gestión de salud diaria y mercado de datos, integrada con la EMR Dr.Palette.</t>
+          <t>App gratuita para seguir visitas al médico, facturas médicas, datos personales, seguros, inmunizaciones y medicamentos de farmacia.</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -6826,7 +6826,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Medicalchain</t>
+          <t>MediBloc</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -6841,7 +6841,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Centros de investigación y farmacéuticas recompensarían con MedTokens a quienes compartan sus datos; no confirmado como ejecutado.</t>
+          <t>Plan de convertir Medipass en superapp con gestión de salud diaria y mercado de datos, integrada con la EMR Dr.Palette.</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -6853,7 +6853,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Patientory</t>
+          <t>Medicalchain</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -6868,7 +6868,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>El usuario puede agregar y monetizar sus datos; recompensas en cripto.</t>
+          <t>Centros de investigación y farmacéuticas recompensarían con MedTokens a quienes compartan sus datos; no confirmado como ejecutado.</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -6880,22 +6880,22 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>ChatGPT Health (OpenAI)</t>
+          <t>Patientory</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Inteligencia artificial</t>
+          <t>Incentivos y monetización de datos</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Asistente de IA para profesionales de salud</t>
+          <t>Recompensas / monetización de datos del usuario</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Producto para clínicos verificados de EE.UU. (gratis, abr-2026); desde 1-sep-2026 un plugin con nueve apps de fuentes públicas (investigación, ensayos, medicamentos, Medicare, prestadores), de solo lectura y sin acceso a fichas de pacientes.</t>
+          <t>El usuario puede agregar y monetizar sus datos; recompensas en cripto.</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -6907,7 +6907,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Patientory</t>
+          <t>ChatGPT Health (OpenAI)</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -6917,12 +6917,12 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Coaching de salud con IA</t>
+          <t>Asistente de IA para profesionales de salud</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Coaching personalizado con IA.</t>
+          <t>Producto para clínicos verificados de EE.UU. (gratis, abr-2026); desde 1-sep-2026 un plugin con nueve apps de fuentes públicas (investigación, ensayos, medicamentos, Medicare, prestadores), de solo lectura y sin acceso a fichas de pacientes.</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -6934,7 +6934,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>ChatGPT Health (OpenAI)</t>
+          <t>Patientory</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -6944,12 +6944,12 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Detección de patrones en métricas de salud con IA</t>
+          <t>Coaching de salud con IA</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Interpreta datos de Apple Health y registros en contexto y detecta cambios.</t>
+          <t>Coaching personalizado con IA.</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -6961,7 +6961,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Claude for Healthcare (Anthropic)</t>
+          <t>ChatGPT Health (OpenAI)</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -6976,7 +6976,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Detecta patrones entre métricas de salud y fitness.</t>
+          <t>Interpreta datos de Apple Health y registros en contexto y detecta cambios.</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -6988,7 +6988,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>ChatGPT Health (OpenAI)</t>
+          <t>Claude for Healthcare (Anthropic)</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -6998,12 +6998,12 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Interpretación de exámenes con IA</t>
+          <t>Detección de patrones en métricas de salud con IA</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Explica resultados complejos en lenguaje simple.</t>
+          <t>Detecta patrones entre métricas de salud y fitness.</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -7030,7 +7030,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Desde 28-sep-2026, en la pestaña Health se puede elegir un gráfico, métrica o registro y obtener explicaciones basadas en los datos conectados.</t>
+          <t>Explica resultados complejos en lenguaje simple.</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -7042,7 +7042,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Claude for Healthcare (Anthropic)</t>
+          <t>ChatGPT Health (OpenAI)</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -7057,7 +7057,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Explica exámenes en lenguaje simple.</t>
+          <t>Desde 28-sep-2026, en la pestaña Health se puede elegir un gráfico, métrica o registro y obtener explicaciones basadas en los datos conectados.</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -7069,7 +7069,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Mediko</t>
+          <t>Claude for Healthcare (Anthropic)</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -7084,19 +7084,19 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Interpreta exámenes de laboratorio.</t>
+          <t>Explica exámenes en lenguaje simple.</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Global</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>ChatGPT Health (OpenAI)</t>
+          <t>Mediko</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -7106,24 +7106,24 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Orientación médica con IA</t>
+          <t>Interpretación de exámenes con IA</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Mejora de jun-2026 (GPT-5.5 Instant): detecta cuándo puede requerirse atención urgente, pide contexto y explica la incertidumbre.</t>
+          <t>Interpreta exámenes de laboratorio.</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Chile</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Mediko</t>
+          <t>ChatGPT Health (OpenAI)</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -7138,19 +7138,19 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Orientación médica instantánea mediante IA.</t>
+          <t>Mejora de jun-2026 (GPT-5.5 Instant): detecta cuándo puede requerirse atención urgente, pide contexto y explica la incertidumbre.</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Global</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>ChatGPT Health (OpenAI)</t>
+          <t>Mediko</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -7160,24 +7160,24 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Preparación de consultas médicas con IA</t>
+          <t>Orientación médica con IA</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Prepara preguntas para el médico.</t>
+          <t>Orientación médica instantánea mediante IA.</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Chile</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Claude for Healthcare (Anthropic)</t>
+          <t>ChatGPT Health (OpenAI)</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -7204,7 +7204,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>ChatGPT Health (OpenAI)</t>
+          <t>Claude for Healthcare (Anthropic)</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -7214,12 +7214,12 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Resumen de historial con IA</t>
+          <t>Preparación de consultas médicas con IA</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Resume instrucciones de atención.</t>
+          <t>Prepara preguntas para el médico.</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -7231,7 +7231,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Claude for Healthcare (Anthropic)</t>
+          <t>ChatGPT Health (OpenAI)</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -7246,7 +7246,7 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Resume el historial del usuario.</t>
+          <t>Resume instrucciones de atención.</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -7258,22 +7258,22 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Apple Health (Health Records)</t>
+          <t>Claude for Healthcare (Anthropic)</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Interoperabilidad y fuentes de datos</t>
+          <t>Inteligencia artificial</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Agregación de registros de múltiples instituciones</t>
+          <t>Resumen de historial con IA</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Vista central de alergias, condiciones, vacunas, laboratorio, medicación, procedimientos y signos vitales.</t>
+          <t>Resume el historial del usuario.</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -7285,7 +7285,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>ChatGPT Health (OpenAI)</t>
+          <t>Apple Health (Health Records)</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -7300,7 +7300,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Conexión de historiales electrónicos y apps como Apple Health, MyFitnessPal, Peloton.</t>
+          <t>Vista central de alergias, condiciones, vacunas, laboratorio, medicación, procedimientos y signos vitales.</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -7327,7 +7327,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Acceso a historiales electrónicos de proveedores de EE.UU. vía b.well; solo EE.UU., sin plazo anunciado para Latinoamérica.</t>
+          <t>Conexión de historiales electrónicos y apps como Apple Health, MyFitnessPal, Peloton.</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -7354,7 +7354,7 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Además de b.well y Apple Health, vincula registros de One Medical y Function Health (solo EE.UU., Free/Go/Plus/Pro, web e iOS).</t>
+          <t>Acceso a historiales electrónicos de proveedores de EE.UU. vía b.well; solo EE.UU., sin plazo anunciado para Latinoamérica.</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -7366,7 +7366,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Claude for Healthcare (Anthropic)</t>
+          <t>ChatGPT Health (OpenAI)</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -7381,7 +7381,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Acceso a resultados y registros de salud (beta, Pro/Max, EE.UU.).</t>
+          <t>Además de b.well y Apple Health, vincula registros de One Medical y Function Health (solo EE.UU., Free/Go/Plus/Pro, web e iOS).</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
@@ -7393,7 +7393,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Clinia (Reservo)</t>
+          <t>Claude for Healthcare (Anthropic)</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -7408,19 +7408,19 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Datos desde profesionales/centros que usan Reservo (fichas clínicas, agenda, telemedicina).</t>
+          <t>Acceso a resultados y registros de salud (beta, Pro/Max, EE.UU.).</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Global</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>MediBloc</t>
+          <t>Clinia (Reservo)</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -7435,19 +7435,19 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Tras autenticación simple, trae los últimos 3 años de historial de hospitales integrados (p. ej. Samsung Seoul, SNUH, Severance).</t>
+          <t>Datos desde profesionales/centros que usan Reservo (fichas clínicas, agenda, telemedicina).</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Chile</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Meedika</t>
+          <t>MediBloc</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -7462,19 +7462,19 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Sincroniza resultados desde centros de salud y permite subir fotos o documentos de las solicitudes médicas.</t>
+          <t>Tras autenticación simple, trae los últimos 3 años de historial de hospitales integrados (p. ej. Samsung Seoul, SNUH, Severance).</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Global</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Patientory</t>
+          <t>Meedika</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -7489,12 +7489,12 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Reúne registros de hospitales, resultados de laboratorio y datos genómicos.</t>
+          <t>Sincroniza resultados desde centros de salud y permite subir fotos o documentos de las solicitudes médicas.</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Chile</t>
         </is>
       </c>
     </row>
@@ -7511,12 +7511,12 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Analítica poblacional B2B</t>
+          <t>Agregación de registros de múltiples instituciones</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Analítica poblacional on-chain; integrada con Epic, Cerner, Meditech y Allscripts (B2B).</t>
+          <t>Reúne registros de hospitales, resultados de laboratorio y datos genómicos.</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -7528,7 +7528,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Clingot</t>
+          <t>Patientory</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -7538,24 +7538,24 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Disponibilidad multiplataforma (web/iOS/Android)</t>
+          <t>Analítica poblacional B2B</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Android, iOS y escritorio; médicos acceden a historias digitalizadas, envían estudios e indicaciones y organizan agenda.</t>
+          <t>Analítica poblacional on-chain; integrada con Epic, Cerner, Meditech y Allscripts (B2B).</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Latam</t>
+          <t>Global</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Clinia (Reservo)</t>
+          <t>Clingot</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -7570,19 +7570,19 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Disponible en App Store y Google Play. Reservo opera en Chile, México y Argentina y está certificada por FONASA y CENS.</t>
+          <t>Android, iOS y escritorio; médicos acceden a historias digitalizadas, envían estudios e indicaciones y organizan agenda.</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Latam</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Healfies</t>
+          <t>Clinia (Reservo)</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -7597,19 +7597,19 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Disponible en web, iOS y Android.</t>
+          <t>Disponible en App Store y Google Play. Reservo opera en Chile, México y Argentina y está certificada por FONASA y CENS.</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Latam</t>
+          <t>Chile</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Medicalchain</t>
+          <t>Healfies</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -7619,24 +7619,24 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Historial médico centralizado</t>
+          <t>Disponibilidad multiplataforma (web/iOS/Android)</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Versión digital de los registros con acceso por móvil o web.</t>
+          <t>Disponible en web, iOS y Android.</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Latam</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>MediPlanner</t>
+          <t>Medicalchain</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -7646,24 +7646,24 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Importación y exportación de datos</t>
+          <t>Historial médico centralizado</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Importar/exportar datos para compartir de forma segura con familias o cuidadores. Es MediPlanner Pro, de otro desarrollador (App Store MX, $39 MXN).</t>
+          <t>Versión digital de los registros con acceso por móvil o web.</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Latam</t>
+          <t>Global</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Medicalchain</t>
+          <t>MediPlanner</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -7673,24 +7673,24 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Integración con EHR de proveedores</t>
+          <t>Importación y exportación de datos</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Según una AMA sin fecha, integraba dos sistemas de GP que cubren ~80% del mercado UK; no confirmado como ejecutado.</t>
+          <t>Importar/exportar datos para compartir de forma segura con familias o cuidadores. Es MediPlanner Pro, de otro desarrollador (App Store MX, $39 MXN).</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Latam</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Claude for Healthcare (Anthropic)</t>
+          <t>Medicalchain</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -7700,12 +7700,12 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Integración con wearables y apps de salud</t>
+          <t>Integración con EHR de proveedores</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Integración beta en apps iOS/Android.</t>
+          <t>Según una AMA sin fecha, integraba dos sistemas de GP que cubren ~80% del mercado UK; no confirmado como ejecutado.</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
@@ -7732,7 +7732,7 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Integración beta con Health Connect en la app móvil; conectores de registros (HealthEx, Function) solo para Pro/Max en EE.UU.</t>
+          <t>Integración beta en apps iOS/Android.</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
@@ -7744,7 +7744,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Patientory</t>
+          <t>Claude for Healthcare (Anthropic)</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -7759,7 +7759,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Se integra con wearables y apps móviles populares y muestra vitales en un panel unificado.</t>
+          <t>Integración beta con Health Connect en la app móvil; conectores de registros (HealthEx, Function) solo para Pro/Max en EE.UU.</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
@@ -7771,22 +7771,22 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Apple Health (Health Records)</t>
+          <t>Patientory</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Medicación y recordatorios</t>
+          <t>Interoperabilidad y fuentes de datos</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Gestión de lista de medicamentos</t>
+          <t>Integración con wearables y apps de salud</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Listas de medicamentos, vitaminas y suplementos con horarios; escaneo de etiqueta del frasco solo en EE.UU.</t>
+          <t>Se integra con wearables y apps móviles populares y muestra vitales en un panel unificado.</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
@@ -7798,7 +7798,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>MediPlanner</t>
+          <t>Apple Health (Health Records)</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -7808,24 +7808,24 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Importación automática de tratamientos desde receta digital</t>
+          <t>Gestión de lista de medicamentos</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Según la ficha de la App Store MX, los tratamientos llegan automáticamente desde la receta digital del médico (autodeclarado, sin verificar).</t>
+          <t>Listas de medicamentos, vitaminas y suplementos con horarios; escaneo de etiqueta del frasco solo en EE.UU.</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Latam</t>
+          <t>Global</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Apple Health (Health Records)</t>
+          <t>MediPlanner</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -7835,24 +7835,24 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Recordatorios de medicación y citas</t>
+          <t>Importación automática de tratamientos desde receta digital</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Recordatorios desde el app.</t>
+          <t>Según la ficha de la App Store MX, los tratamientos llegan automáticamente desde la receta digital del médico (autodeclarado, sin verificar).</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Latam</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Meedika</t>
+          <t>Apple Health (Health Records)</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -7867,19 +7867,19 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Recordatorios de citas/medicación.</t>
+          <t>Recordatorios desde el app.</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Global</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>MediPlanner</t>
+          <t>Meedika</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -7889,51 +7889,51 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Registro de tomas y adherencia al tratamiento</t>
+          <t>Recordatorios de medicación y citas</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Registro de cada toma y control de adherencia; gestiona medicamentos propios y de familiares.</t>
+          <t>Recordatorios de citas/medicación.</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Latam</t>
+          <t>Chile</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Patientory</t>
+          <t>MediPlanner</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Seguimiento y bienestar</t>
+          <t>Medicación y recordatorios</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Comunidad de pacientes</t>
+          <t>Registro de tomas y adherencia al tratamiento</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Los usuarios con condiciones similares pueden preguntar, recibir recomendaciones y compartir experiencias.</t>
+          <t>Registro de cada toma y control de adherencia; gestiona medicamentos propios y de familiares.</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Latam</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Infomed</t>
+          <t>Patientory</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -7943,24 +7943,24 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Contenido educativo sobre salud</t>
+          <t>Comunidad de pacientes</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Busca que el paciente aprenda sobre sus enfermedades y sea más autónomo.</t>
+          <t>Los usuarios con condiciones similares pueden preguntar, recibir recomendaciones y compartir experiencias.</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Global</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>MediPlanner</t>
+          <t>Infomed</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -7970,24 +7970,24 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Gráficas de evolución de indicadores</t>
+          <t>Contenido educativo sobre salud</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Gráficas de evolución de indicadores de salud.</t>
+          <t>Busca que el paciente aprenda sobre sus enfermedades y sea más autónomo.</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Latam</t>
+          <t>Chile</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Apple Health (Health Records)</t>
+          <t>MediPlanner</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -7997,24 +7997,24 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Integración con wearables y apps de salud</t>
+          <t>Gráficas de evolución de indicadores</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Datos de pasos, sueño, peso junto a registros.</t>
+          <t>Gráficas de evolución de indicadores de salud.</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Latam</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Patientory</t>
+          <t>Apple Health (Health Records)</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -8024,12 +8024,12 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Panel de seguimiento de salud y bienestar</t>
+          <t>Integración con wearables y apps de salud</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Seguimiento de hábitos saludables y monitoreo de progreso.</t>
+          <t>Datos de pasos, sueño, peso junto a registros.</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
@@ -8041,7 +8041,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Apple Health (Health Records)</t>
+          <t>MediBloc</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -8051,12 +8051,12 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Registro de nutrición</t>
+          <t>Panel de seguimiento de salud y bienestar</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Escaneo de etiquetas nutricionales con la cámara; según un análisis, no escribe en HealthKit.</t>
+          <t>El relanzamiento de Medipass (mar-2023) agregó un panel para gestionar la información de salud del usuario.</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
@@ -8068,7 +8068,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Apple Health (Health Records)</t>
+          <t>Patientory</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -8078,12 +8078,12 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Seguimiento de salud femenina</t>
+          <t>Panel de seguimiento de salud y bienestar</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Extiende el seguimiento de ciclo con perimenopausia y menopausia.</t>
+          <t>Seguimiento de hábitos saludables y monitoreo de progreso.</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
@@ -8095,7 +8095,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Clingot</t>
+          <t>Apple Health (Health Records)</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -8105,39 +8105,39 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Valoración de profesionales</t>
+          <t>Registro de nutrición</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Calificación de la atención de profesionales con autorización previa, compartible con otros usuarios.</t>
+          <t>Escaneo de etiquetas nutricionales con la cámara; según un análisis, no escribe en HealthKit.</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>Latam</t>
+          <t>Global</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>MediBloc</t>
+          <t>Apple Health (Health Records)</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Seguridad, privacidad y blockchain</t>
+          <t>Seguimiento y bienestar</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Blockchain para integridad y trazabilidad de datos</t>
+          <t>Seguimiento de salud femenina</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Blockchain propia (Cosmos SDK) para que el paciente almacene, use, actualice y transfiera sus registros; los datos no se guardan en la cadena, solo en el usuario, cifrados.</t>
+          <t>Extiende el seguimiento de ciclo con perimenopausia y menopausia.</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
@@ -8149,34 +8149,34 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>MediBloc</t>
+          <t>Clingot</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Seguridad, privacidad y blockchain</t>
+          <t>Seguimiento y bienestar</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Blockchain para integridad y trazabilidad de datos</t>
+          <t>Valoración de profesionales</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Almacena huellas de datos médicos en un registro de solo escritura, sin guardar datos clínicos en cadena.</t>
+          <t>Calificación de la atención de profesionales con autorización previa, compartible con otros usuarios.</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Latam</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Medicalchain</t>
+          <t>Claude for Healthcare (Anthropic)</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -8186,12 +8186,12 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Blockchain para integridad y trazabilidad de datos</t>
+          <t>Acceso mínimo por categorías de datos</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Cada solicitud de acceso queda en un libro distribuido; acceso temporal por contratos inteligentes.</t>
+          <t>Claude solicita solo las categorías relevantes (p. ej. medicamentos o laboratorio) y no fichas completas; HealthEx agrega datos de más de 50.000 sistemas de salud de EE.UU.</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
@@ -8203,7 +8203,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Patientory</t>
+          <t>MediBloc</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -8218,7 +8218,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Registro respaldado en blockchain para seguridad y trazabilidad.</t>
+          <t>Blockchain propia (Cosmos SDK) para que el paciente almacene, use, actualice y transfiera sus registros; los datos no se guardan en la cadena, solo en el usuario, cifrados.</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
@@ -8230,7 +8230,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Apple Health (Health Records)</t>
+          <t>MediBloc</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -8240,12 +8240,12 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Cifrado y control de acceso</t>
+          <t>Blockchain para integridad y trazabilidad de datos</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Registros cifrados en el dispositivo, protegidos por Face ID/Touch ID/código.</t>
+          <t>Almacena huellas de datos médicos en un registro de solo escritura, sin guardar datos clínicos en cadena.</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
@@ -8257,7 +8257,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Infomed</t>
+          <t>Medicalchain</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -8267,24 +8267,24 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Cifrado y control de acceso</t>
+          <t>Blockchain para integridad y trazabilidad de datos</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Almacenamiento seguro del historial con criterios de seguridad estrictos, comparable a apps bancarias.</t>
+          <t>Cada solicitud de acceso queda en un libro distribuido; acceso temporal por contratos inteligentes.</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Global</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Clinia (Reservo)</t>
+          <t>Patientory</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -8294,24 +8294,24 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Cumplimiento regulatorio de salud y datos</t>
+          <t>Blockchain para integridad y trazabilidad de datos</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Reservo declara plataforma certificada por Fonasa y CENS, cumplimiento de estándares de telemedicina del Minsal y de la nueva ley chilena de datos personales (declaración de la empresa).</t>
+          <t>Registro respaldado en blockchain para seguridad y trazabilidad.</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Global</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>ChatGPT Health (OpenAI)</t>
+          <t>Apple Health (Health Records)</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -8321,12 +8321,12 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Gestión de consentimiento sobre uso de datos</t>
+          <t>Cifrado y control de acceso</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Desde 14-sep-2026, las nuevas conexiones heredan la configuración global de plugins: ChatGPT puede usar datos de Health sin pedir permiso cada vez salvo acciones sensibles (web primero, móvil después).</t>
+          <t>Registros cifrados en el dispositivo, protegidos por Face ID/Touch ID/código.</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
@@ -8338,7 +8338,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>MediBloc</t>
+          <t>Infomed</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -8348,24 +8348,24 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Identidad descentralizada (DID)</t>
+          <t>Cifrado y control de acceso</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Gestión de identificadores descentralizados en Panacea.</t>
+          <t>Almacenamiento seguro del historial con criterios de seguridad estrictos, comparable a apps bancarias.</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Chile</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>ChatGPT Health (OpenAI)</t>
+          <t>Clinia (Reservo)</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -8375,24 +8375,24 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Privacidad reforzada para datos de salud</t>
+          <t>Cumplimiento regulatorio de salud y datos</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Chats y memoria de salud separados, no usados para entrenar modelos.</t>
+          <t>Reservo declara plataforma certificada por Fonasa y CENS, cumplimiento de estándares de telemedicina del Minsal y de la nueva ley chilena de datos personales (declaración de la empresa).</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Chile</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Claude for Healthcare (Anthropic)</t>
+          <t>ChatGPT Health (OpenAI)</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -8402,12 +8402,12 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Privacidad reforzada para datos de salud</t>
+          <t>Gestión de consentimiento sobre uso de datos</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>El usuario activa y revoca permisos; los datos de salud compartidos se excluyen de la memoria de Claude y del entrenamiento.</t>
+          <t>Desde 14-sep-2026, las nuevas conexiones heredan la configuración global de plugins: ChatGPT puede usar datos de Health sin pedir permiso cada vez salvo acciones sensibles (web primero, móvil después).</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
@@ -8419,49 +8419,49 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Mediko</t>
+          <t>MediBloc</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Seguros y pagos</t>
+          <t>Seguridad, privacidad y blockchain</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Modelo freemium y suscripción</t>
+          <t>Identidad descentralizada (DID)</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Planes para personas y empresas.</t>
+          <t>Gestión de identificadores descentralizados en Panacea.</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Global</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>Medicalchain</t>
+          <t>ChatGPT Health (OpenAI)</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Seguros y pagos</t>
+          <t>Seguridad, privacidad y blockchain</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Pagos con criptomoneda</t>
+          <t>Privacidad reforzada para datos de salud</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>Pago de consultas con token.</t>
+          <t>Chats y memoria de salud separados, no usados para entrenar modelos.</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
@@ -8473,22 +8473,22 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Medicalchain</t>
+          <t>Claude for Healthcare (Anthropic)</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Seguros y pagos</t>
+          <t>Seguridad, privacidad y blockchain</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Pagos con criptomoneda</t>
+          <t>Privacidad reforzada para datos de salud</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>Piloto en New Malden (Londres): consultas por video pagables con tarjeta o con MedTokens.</t>
+          <t>El usuario activa y revoca permisos; los datos de salud compartidos se excluyen de la memoria de Claude y del entrenamiento.</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
@@ -8510,12 +8510,12 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Pagos dentro de la app</t>
+          <t>Modelo freemium y suscripción</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Pagos dentro de la plataforma mediante la pasarela Flow (según resumen de entrevista de Pauta, oct-2024; esperada para mejorar la experiencia).</t>
+          <t>Planes para personas y empresas.</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
@@ -8527,7 +8527,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>MediBloc</t>
+          <t>Medicalchain</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -8537,12 +8537,12 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Reclamos y trámites con seguros</t>
+          <t>Pagos con criptomoneda</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>Simplifica el envío a aseguradoras sin gestionar papeles en hospitales.</t>
+          <t>Pago de consultas con token.</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
@@ -8554,7 +8554,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>MediBloc</t>
+          <t>Medicalchain</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -8564,12 +8564,12 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Reclamos y trámites con seguros</t>
+          <t>Pagos con criptomoneda</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Reclamo de seguro médico (indemnización) desde la app, con verificación de autenticidad de los registros vía blockchain por la aseguradora.</t>
+          <t>Piloto en New Malden (Londres): consultas por video pagables con tarjeta o con MedTokens.</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
@@ -8581,25 +8581,106 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
+          <t>Mediko</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Seguros y pagos</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Pagos dentro de la app</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Pagos dentro de la plataforma mediante la pasarela Flow (según resumen de entrevista de Pauta, oct-2024; esperada para mejorar la experiencia).</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>MediBloc</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Seguros y pagos</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Reclamos y trámites con seguros</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Simplifica el envío a aseguradoras sin gestionar papeles en hospitales.</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>MediBloc</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Seguros y pagos</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Reclamos y trámites con seguros</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>Reclamo de seguro médico (indemnización) desde la app, con verificación de autenticidad de los registros vía blockchain por la aseguradora.</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
           <t>Medicalchain</t>
         </is>
       </c>
-      <c r="B125" t="inlineStr">
+      <c r="B128" t="inlineStr">
         <is>
           <t>Telemedicina y atención remota</t>
         </is>
       </c>
-      <c r="C125" t="inlineStr">
+      <c r="C128" t="inlineStr">
         <is>
           <t>Teleconsulta con profesionales</t>
         </is>
       </c>
-      <c r="D125" t="inlineStr">
+      <c r="D128" t="inlineStr">
         <is>
           <t>Teleconsultas con GP.</t>
         </is>
       </c>
-      <c r="E125" t="inlineStr">
+      <c r="E128" t="inlineStr">
         <is>
           <t>Global</t>
         </is>
@@ -8616,7 +8697,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R64"/>
+  <dimension ref="A1:R65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8742,6 +8823,8 @@
           <t>Búsqueda de profesionales de salud</t>
         </is>
       </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
           <t>✓</t>
@@ -8752,6 +8835,17 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr"/>
       <c r="R2">
         <f>COUNTIF(C2:Q2,"✓")</f>
         <v/>
@@ -8773,11 +8867,24 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr"/>
       <c r="R3">
         <f>COUNTIF(C3:Q3,"✓")</f>
         <v/>
@@ -8794,11 +8901,25 @@
           <t>Integración con calendario del dispositivo</t>
         </is>
       </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr"/>
       <c r="R4">
         <f>COUNTIF(C4:Q4,"✓")</f>
         <v/>
@@ -8815,11 +8936,25 @@
           <t>Localización de centros médicos y farmacias</t>
         </is>
       </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr"/>
       <c r="R5">
         <f>COUNTIF(C5:Q5,"✓")</f>
         <v/>
@@ -8836,6 +8971,17 @@
           <t>Reserva de citas médicas</t>
         </is>
       </c>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr">
         <is>
           <t>✓</t>
@@ -8846,6 +8992,8 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr"/>
       <c r="R6">
         <f>COUNTIF(C6:Q6,"✓")</f>
         <v/>
@@ -8862,11 +9010,25 @@
           <t>Acceso del profesional al historial del paciente</t>
         </is>
       </c>
+      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr"/>
+      <c r="Q7" t="inlineStr"/>
       <c r="R7">
         <f>COUNTIF(C7:Q7,"✓")</f>
         <v/>
@@ -8883,11 +9045,25 @@
           <t>Compartir con personas sin cuenta mediante clave segura</t>
         </is>
       </c>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr"/>
+      <c r="Q8" t="inlineStr"/>
       <c r="R8">
         <f>COUNTIF(C8:Q8,"✓")</f>
         <v/>
@@ -8904,11 +9080,25 @@
           <t>Compartir datos con cuidador o persona de confianza</t>
         </is>
       </c>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr"/>
+      <c r="Q9" t="inlineStr"/>
       <c r="R9">
         <f>COUNTIF(C9:Q9,"✓")</f>
         <v/>
@@ -8930,11 +9120,13 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
           <t>✓</t>
@@ -8960,11 +9152,16 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
       <c r="O10" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="P10" t="inlineStr"/>
+      <c r="Q10" t="inlineStr"/>
       <c r="R10">
         <f>COUNTIF(C10:Q10,"✓")</f>
         <v/>
@@ -8981,11 +9178,25 @@
           <t>Gestión de consentimiento sobre uso de datos</t>
         </is>
       </c>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr"/>
       <c r="R11">
         <f>COUNTIF(C11:Q11,"✓")</f>
         <v/>
@@ -9002,11 +9213,25 @@
           <t>Ingreso de datos por profesional con consentimiento</t>
         </is>
       </c>
+      <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr"/>
+      <c r="Q12" t="inlineStr"/>
       <c r="R12">
         <f>COUNTIF(C12:Q12,"✓")</f>
         <v/>
@@ -9023,11 +9248,25 @@
           <t>Red social con profesionales y familiares</t>
         </is>
       </c>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr"/>
+      <c r="Q13" t="inlineStr"/>
       <c r="R13">
         <f>COUNTIF(C13:Q13,"✓")</f>
         <v/>
@@ -9054,11 +9293,23 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr"/>
+      <c r="O14" t="inlineStr"/>
+      <c r="P14" t="inlineStr"/>
+      <c r="Q14" t="inlineStr"/>
       <c r="R14">
         <f>COUNTIF(C14:Q14,"✓")</f>
         <v/>
@@ -9075,6 +9326,8 @@
           <t>Perfiles familiares / dependientes</t>
         </is>
       </c>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9085,16 +9338,29 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr"/>
       <c r="N15" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="Q15" t="inlineStr"/>
       <c r="R15">
         <f>COUNTIF(C15:Q15,"✓")</f>
         <v/>
@@ -9116,6 +9382,8 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9131,11 +9399,19 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="inlineStr"/>
       <c r="O16" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="P16" t="inlineStr"/>
+      <c r="Q16" t="inlineStr"/>
       <c r="R16">
         <f>COUNTIF(C16:Q16,"✓")</f>
         <v/>
@@ -9152,16 +9428,29 @@
           <t>Almacenamiento de recetas</t>
         </is>
       </c>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr"/>
       <c r="N17" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="O17" t="inlineStr"/>
+      <c r="P17" t="inlineStr"/>
+      <c r="Q17" t="inlineStr"/>
       <c r="R17">
         <f>COUNTIF(C17:Q17,"✓")</f>
         <v/>
@@ -9178,11 +9467,25 @@
           <t>Búsqueda y filtros de documentos</t>
         </is>
       </c>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="inlineStr"/>
+      <c r="O18" t="inlineStr"/>
+      <c r="P18" t="inlineStr"/>
+      <c r="Q18" t="inlineStr"/>
       <c r="R18">
         <f>COUNTIF(C18:Q18,"✓")</f>
         <v/>
@@ -9199,11 +9502,25 @@
           <t>Emisión de certificados médicos</t>
         </is>
       </c>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="inlineStr"/>
+      <c r="O19" t="inlineStr"/>
+      <c r="P19" t="inlineStr"/>
+      <c r="Q19" t="inlineStr"/>
       <c r="R19">
         <f>COUNTIF(C19:Q19,"✓")</f>
         <v/>
@@ -9225,6 +9542,19 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="inlineStr"/>
+      <c r="O20" t="inlineStr"/>
+      <c r="P20" t="inlineStr"/>
       <c r="Q20" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9246,11 +9576,25 @@
           <t>Notificación y envío de resultados</t>
         </is>
       </c>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr"/>
       <c r="N21" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="O21" t="inlineStr"/>
+      <c r="P21" t="inlineStr"/>
+      <c r="Q21" t="inlineStr"/>
       <c r="R21">
         <f>COUNTIF(C21:Q21,"✓")</f>
         <v/>
@@ -9267,16 +9611,29 @@
           <t>Historial institucional (solo datos de la propia red)</t>
         </is>
       </c>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr"/>
       <c r="N22" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="O22" t="inlineStr"/>
       <c r="P22" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="Q22" t="inlineStr"/>
       <c r="R22">
         <f>COUNTIF(C22:Q22,"✓")</f>
         <v/>
@@ -9293,26 +9650,36 @@
           <t>Historial médico centralizado</t>
         </is>
       </c>
+      <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr"/>
+      <c r="N23" t="inlineStr"/>
+      <c r="O23" t="inlineStr"/>
+      <c r="P23" t="inlineStr"/>
       <c r="Q23" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9334,11 +9701,25 @@
           <t>Línea de tiempo de salud</t>
         </is>
       </c>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="inlineStr"/>
+      <c r="O24" t="inlineStr"/>
+      <c r="P24" t="inlineStr"/>
+      <c r="Q24" t="inlineStr"/>
       <c r="R24">
         <f>COUNTIF(C24:Q24,"✓")</f>
         <v/>
@@ -9355,11 +9736,25 @@
           <t>Registro de alergias y vacunas</t>
         </is>
       </c>
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" t="inlineStr"/>
+      <c r="O25" t="inlineStr"/>
+      <c r="P25" t="inlineStr"/>
+      <c r="Q25" t="inlineStr"/>
       <c r="R25">
         <f>COUNTIF(C25:Q25,"✓")</f>
         <v/>
@@ -9376,11 +9771,25 @@
           <t>Seguimiento de visitas, gastos y seguros</t>
         </is>
       </c>
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" t="inlineStr"/>
+      <c r="O26" t="inlineStr"/>
+      <c r="P26" t="inlineStr"/>
+      <c r="Q26" t="inlineStr"/>
       <c r="R26">
         <f>COUNTIF(C26:Q26,"✓")</f>
         <v/>
@@ -9397,6 +9806,11 @@
           <t>Recompensas / monetización de datos del usuario</t>
         </is>
       </c>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9412,6 +9826,13 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr"/>
+      <c r="N27" t="inlineStr"/>
+      <c r="O27" t="inlineStr"/>
+      <c r="P27" t="inlineStr"/>
+      <c r="Q27" t="inlineStr"/>
       <c r="R27">
         <f>COUNTIF(C27:Q27,"✓")</f>
         <v/>
@@ -9428,11 +9849,25 @@
           <t>Asistente de IA para profesionales de salud</t>
         </is>
       </c>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="M28" t="inlineStr"/>
+      <c r="N28" t="inlineStr"/>
+      <c r="O28" t="inlineStr"/>
+      <c r="P28" t="inlineStr"/>
+      <c r="Q28" t="inlineStr"/>
       <c r="R28">
         <f>COUNTIF(C28:Q28,"✓")</f>
         <v/>
@@ -9449,11 +9884,25 @@
           <t>Coaching de salud con IA</t>
         </is>
       </c>
+      <c r="C29" t="inlineStr"/>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr"/>
+      <c r="L29" t="inlineStr"/>
+      <c r="M29" t="inlineStr"/>
+      <c r="N29" t="inlineStr"/>
+      <c r="O29" t="inlineStr"/>
+      <c r="P29" t="inlineStr"/>
+      <c r="Q29" t="inlineStr"/>
       <c r="R29">
         <f>COUNTIF(C29:Q29,"✓")</f>
         <v/>
@@ -9470,6 +9919,15 @@
           <t>Detección de patrones en métricas de salud con IA</t>
         </is>
       </c>
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9480,6 +9938,10 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="N30" t="inlineStr"/>
+      <c r="O30" t="inlineStr"/>
+      <c r="P30" t="inlineStr"/>
+      <c r="Q30" t="inlineStr"/>
       <c r="R30">
         <f>COUNTIF(C30:Q30,"✓")</f>
         <v/>
@@ -9496,6 +9958,15 @@
           <t>Interpretación de exámenes con IA</t>
         </is>
       </c>
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9506,6 +9977,9 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="N31" t="inlineStr"/>
+      <c r="O31" t="inlineStr"/>
+      <c r="P31" t="inlineStr"/>
       <c r="Q31" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9527,11 +10001,24 @@
           <t>Orientación médica con IA</t>
         </is>
       </c>
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="M32" t="inlineStr"/>
+      <c r="N32" t="inlineStr"/>
+      <c r="O32" t="inlineStr"/>
+      <c r="P32" t="inlineStr"/>
       <c r="Q32" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9553,6 +10040,15 @@
           <t>Preparación de consultas médicas con IA</t>
         </is>
       </c>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9563,6 +10059,10 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="N33" t="inlineStr"/>
+      <c r="O33" t="inlineStr"/>
+      <c r="P33" t="inlineStr"/>
+      <c r="Q33" t="inlineStr"/>
       <c r="R33">
         <f>COUNTIF(C33:Q33,"✓")</f>
         <v/>
@@ -9579,6 +10079,15 @@
           <t>Resumen de historial con IA</t>
         </is>
       </c>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="inlineStr"/>
+      <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9589,6 +10098,10 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="N34" t="inlineStr"/>
+      <c r="O34" t="inlineStr"/>
+      <c r="P34" t="inlineStr"/>
+      <c r="Q34" t="inlineStr"/>
       <c r="R34">
         <f>COUNTIF(C34:Q34,"✓")</f>
         <v/>
@@ -9610,6 +10123,10 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9620,6 +10137,7 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="J35" t="inlineStr"/>
       <c r="K35" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9635,11 +10153,14 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="N35" t="inlineStr"/>
       <c r="O35" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="P35" t="inlineStr"/>
+      <c r="Q35" t="inlineStr"/>
       <c r="R35">
         <f>COUNTIF(C35:Q35,"✓")</f>
         <v/>
@@ -9656,11 +10177,25 @@
           <t>Analítica poblacional B2B</t>
         </is>
       </c>
+      <c r="C36" t="inlineStr"/>
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="inlineStr"/>
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="I36" t="inlineStr"/>
+      <c r="J36" t="inlineStr"/>
+      <c r="K36" t="inlineStr"/>
+      <c r="L36" t="inlineStr"/>
+      <c r="M36" t="inlineStr"/>
+      <c r="N36" t="inlineStr"/>
+      <c r="O36" t="inlineStr"/>
+      <c r="P36" t="inlineStr"/>
+      <c r="Q36" t="inlineStr"/>
       <c r="R36">
         <f>COUNTIF(C36:Q36,"✓")</f>
         <v/>
@@ -9677,6 +10212,9 @@
           <t>Disponibilidad multiplataforma (web/iOS/Android)</t>
         </is>
       </c>
+      <c r="C37" t="inlineStr"/>
+      <c r="D37" t="inlineStr"/>
+      <c r="E37" t="inlineStr"/>
       <c r="F37" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9687,11 +10225,20 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr"/>
+      <c r="J37" t="inlineStr"/>
+      <c r="K37" t="inlineStr"/>
+      <c r="L37" t="inlineStr"/>
+      <c r="M37" t="inlineStr"/>
+      <c r="N37" t="inlineStr"/>
       <c r="O37" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="P37" t="inlineStr"/>
+      <c r="Q37" t="inlineStr"/>
       <c r="R37">
         <f>COUNTIF(C37:Q37,"✓")</f>
         <v/>
@@ -9708,11 +10255,25 @@
           <t>Historial médico centralizado</t>
         </is>
       </c>
+      <c r="C38" t="inlineStr"/>
+      <c r="D38" t="inlineStr"/>
+      <c r="E38" t="inlineStr"/>
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" t="inlineStr"/>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr"/>
       <c r="J38" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="K38" t="inlineStr"/>
+      <c r="L38" t="inlineStr"/>
+      <c r="M38" t="inlineStr"/>
+      <c r="N38" t="inlineStr"/>
+      <c r="O38" t="inlineStr"/>
+      <c r="P38" t="inlineStr"/>
+      <c r="Q38" t="inlineStr"/>
       <c r="R38">
         <f>COUNTIF(C38:Q38,"✓")</f>
         <v/>
@@ -9729,11 +10290,25 @@
           <t>Importación y exportación de datos</t>
         </is>
       </c>
+      <c r="C39" t="inlineStr"/>
+      <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="F39" t="inlineStr"/>
+      <c r="G39" t="inlineStr"/>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr"/>
+      <c r="J39" t="inlineStr"/>
+      <c r="K39" t="inlineStr"/>
+      <c r="L39" t="inlineStr"/>
+      <c r="M39" t="inlineStr"/>
+      <c r="N39" t="inlineStr"/>
+      <c r="O39" t="inlineStr"/>
+      <c r="P39" t="inlineStr"/>
+      <c r="Q39" t="inlineStr"/>
       <c r="R39">
         <f>COUNTIF(C39:Q39,"✓")</f>
         <v/>
@@ -9750,11 +10325,25 @@
           <t>Integración con EHR de proveedores</t>
         </is>
       </c>
+      <c r="C40" t="inlineStr"/>
+      <c r="D40" t="inlineStr"/>
+      <c r="E40" t="inlineStr"/>
+      <c r="F40" t="inlineStr"/>
+      <c r="G40" t="inlineStr"/>
+      <c r="H40" t="inlineStr"/>
+      <c r="I40" t="inlineStr"/>
       <c r="J40" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="K40" t="inlineStr"/>
+      <c r="L40" t="inlineStr"/>
+      <c r="M40" t="inlineStr"/>
+      <c r="N40" t="inlineStr"/>
+      <c r="O40" t="inlineStr"/>
+      <c r="P40" t="inlineStr"/>
+      <c r="Q40" t="inlineStr"/>
       <c r="R40">
         <f>COUNTIF(C40:Q40,"✓")</f>
         <v/>
@@ -9771,16 +10360,29 @@
           <t>Integración con wearables y apps de salud</t>
         </is>
       </c>
+      <c r="C41" t="inlineStr"/>
+      <c r="D41" t="inlineStr"/>
+      <c r="E41" t="inlineStr"/>
+      <c r="F41" t="inlineStr"/>
+      <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="I41" t="inlineStr"/>
+      <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr"/>
+      <c r="L41" t="inlineStr"/>
       <c r="M41" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="N41" t="inlineStr"/>
+      <c r="O41" t="inlineStr"/>
+      <c r="P41" t="inlineStr"/>
+      <c r="Q41" t="inlineStr"/>
       <c r="R41">
         <f>COUNTIF(C41:Q41,"✓")</f>
         <v/>
@@ -9797,11 +10399,25 @@
           <t>Gestión de lista de medicamentos</t>
         </is>
       </c>
+      <c r="C42" t="inlineStr"/>
+      <c r="D42" t="inlineStr"/>
+      <c r="E42" t="inlineStr"/>
+      <c r="F42" t="inlineStr"/>
+      <c r="G42" t="inlineStr"/>
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" t="inlineStr"/>
+      <c r="J42" t="inlineStr"/>
       <c r="K42" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="L42" t="inlineStr"/>
+      <c r="M42" t="inlineStr"/>
+      <c r="N42" t="inlineStr"/>
+      <c r="O42" t="inlineStr"/>
+      <c r="P42" t="inlineStr"/>
+      <c r="Q42" t="inlineStr"/>
       <c r="R42">
         <f>COUNTIF(C42:Q42,"✓")</f>
         <v/>
@@ -9818,11 +10434,25 @@
           <t>Importación automática de tratamientos desde receta digital</t>
         </is>
       </c>
+      <c r="C43" t="inlineStr"/>
+      <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="F43" t="inlineStr"/>
+      <c r="G43" t="inlineStr"/>
+      <c r="H43" t="inlineStr"/>
+      <c r="I43" t="inlineStr"/>
+      <c r="J43" t="inlineStr"/>
+      <c r="K43" t="inlineStr"/>
+      <c r="L43" t="inlineStr"/>
+      <c r="M43" t="inlineStr"/>
+      <c r="N43" t="inlineStr"/>
+      <c r="O43" t="inlineStr"/>
+      <c r="P43" t="inlineStr"/>
+      <c r="Q43" t="inlineStr"/>
       <c r="R43">
         <f>COUNTIF(C43:Q43,"✓")</f>
         <v/>
@@ -9844,11 +10474,24 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="D44" t="inlineStr"/>
+      <c r="E44" t="inlineStr"/>
+      <c r="F44" t="inlineStr"/>
+      <c r="G44" t="inlineStr"/>
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr"/>
+      <c r="J44" t="inlineStr"/>
       <c r="K44" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="L44" t="inlineStr"/>
+      <c r="M44" t="inlineStr"/>
+      <c r="N44" t="inlineStr"/>
+      <c r="O44" t="inlineStr"/>
+      <c r="P44" t="inlineStr"/>
+      <c r="Q44" t="inlineStr"/>
       <c r="R44">
         <f>COUNTIF(C44:Q44,"✓")</f>
         <v/>
@@ -9865,11 +10508,25 @@
           <t>Registro de tomas y adherencia al tratamiento</t>
         </is>
       </c>
+      <c r="C45" t="inlineStr"/>
+      <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="F45" t="inlineStr"/>
+      <c r="G45" t="inlineStr"/>
+      <c r="H45" t="inlineStr"/>
+      <c r="I45" t="inlineStr"/>
+      <c r="J45" t="inlineStr"/>
+      <c r="K45" t="inlineStr"/>
+      <c r="L45" t="inlineStr"/>
+      <c r="M45" t="inlineStr"/>
+      <c r="N45" t="inlineStr"/>
+      <c r="O45" t="inlineStr"/>
+      <c r="P45" t="inlineStr"/>
+      <c r="Q45" t="inlineStr"/>
       <c r="R45">
         <f>COUNTIF(C45:Q45,"✓")</f>
         <v/>
@@ -9886,11 +10543,25 @@
           <t>Comunidad de pacientes</t>
         </is>
       </c>
+      <c r="C46" t="inlineStr"/>
+      <c r="D46" t="inlineStr"/>
+      <c r="E46" t="inlineStr"/>
+      <c r="F46" t="inlineStr"/>
+      <c r="G46" t="inlineStr"/>
       <c r="H46" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="I46" t="inlineStr"/>
+      <c r="J46" t="inlineStr"/>
+      <c r="K46" t="inlineStr"/>
+      <c r="L46" t="inlineStr"/>
+      <c r="M46" t="inlineStr"/>
+      <c r="N46" t="inlineStr"/>
+      <c r="O46" t="inlineStr"/>
+      <c r="P46" t="inlineStr"/>
+      <c r="Q46" t="inlineStr"/>
       <c r="R46">
         <f>COUNTIF(C46:Q46,"✓")</f>
         <v/>
@@ -9907,11 +10578,25 @@
           <t>Contenido educativo sobre salud</t>
         </is>
       </c>
+      <c r="C47" t="inlineStr"/>
       <c r="D47" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="E47" t="inlineStr"/>
+      <c r="F47" t="inlineStr"/>
+      <c r="G47" t="inlineStr"/>
+      <c r="H47" t="inlineStr"/>
+      <c r="I47" t="inlineStr"/>
+      <c r="J47" t="inlineStr"/>
+      <c r="K47" t="inlineStr"/>
+      <c r="L47" t="inlineStr"/>
+      <c r="M47" t="inlineStr"/>
+      <c r="N47" t="inlineStr"/>
+      <c r="O47" t="inlineStr"/>
+      <c r="P47" t="inlineStr"/>
+      <c r="Q47" t="inlineStr"/>
       <c r="R47">
         <f>COUNTIF(C47:Q47,"✓")</f>
         <v/>
@@ -9928,11 +10613,25 @@
           <t>Gráficas de evolución de indicadores</t>
         </is>
       </c>
+      <c r="C48" t="inlineStr"/>
+      <c r="D48" t="inlineStr"/>
       <c r="E48" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="F48" t="inlineStr"/>
+      <c r="G48" t="inlineStr"/>
+      <c r="H48" t="inlineStr"/>
+      <c r="I48" t="inlineStr"/>
+      <c r="J48" t="inlineStr"/>
+      <c r="K48" t="inlineStr"/>
+      <c r="L48" t="inlineStr"/>
+      <c r="M48" t="inlineStr"/>
+      <c r="N48" t="inlineStr"/>
+      <c r="O48" t="inlineStr"/>
+      <c r="P48" t="inlineStr"/>
+      <c r="Q48" t="inlineStr"/>
       <c r="R48">
         <f>COUNTIF(C48:Q48,"✓")</f>
         <v/>
@@ -9949,11 +10648,25 @@
           <t>Integración con wearables y apps de salud</t>
         </is>
       </c>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="inlineStr"/>
+      <c r="E49" t="inlineStr"/>
+      <c r="F49" t="inlineStr"/>
+      <c r="G49" t="inlineStr"/>
+      <c r="H49" t="inlineStr"/>
+      <c r="I49" t="inlineStr"/>
+      <c r="J49" t="inlineStr"/>
       <c r="K49" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="L49" t="inlineStr"/>
+      <c r="M49" t="inlineStr"/>
+      <c r="N49" t="inlineStr"/>
+      <c r="O49" t="inlineStr"/>
+      <c r="P49" t="inlineStr"/>
+      <c r="Q49" t="inlineStr"/>
       <c r="R49">
         <f>COUNTIF(C49:Q49,"✓")</f>
         <v/>
@@ -9970,11 +10683,29 @@
           <t>Panel de seguimiento de salud y bienestar</t>
         </is>
       </c>
+      <c r="C50" t="inlineStr"/>
+      <c r="D50" t="inlineStr"/>
+      <c r="E50" t="inlineStr"/>
+      <c r="F50" t="inlineStr"/>
+      <c r="G50" t="inlineStr"/>
       <c r="H50" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr"/>
+      <c r="K50" t="inlineStr"/>
+      <c r="L50" t="inlineStr"/>
+      <c r="M50" t="inlineStr"/>
+      <c r="N50" t="inlineStr"/>
+      <c r="O50" t="inlineStr"/>
+      <c r="P50" t="inlineStr"/>
+      <c r="Q50" t="inlineStr"/>
       <c r="R50">
         <f>COUNTIF(C50:Q50,"✓")</f>
         <v/>
@@ -9991,11 +10722,25 @@
           <t>Registro de nutrición</t>
         </is>
       </c>
+      <c r="C51" t="inlineStr"/>
+      <c r="D51" t="inlineStr"/>
+      <c r="E51" t="inlineStr"/>
+      <c r="F51" t="inlineStr"/>
+      <c r="G51" t="inlineStr"/>
+      <c r="H51" t="inlineStr"/>
+      <c r="I51" t="inlineStr"/>
+      <c r="J51" t="inlineStr"/>
       <c r="K51" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="L51" t="inlineStr"/>
+      <c r="M51" t="inlineStr"/>
+      <c r="N51" t="inlineStr"/>
+      <c r="O51" t="inlineStr"/>
+      <c r="P51" t="inlineStr"/>
+      <c r="Q51" t="inlineStr"/>
       <c r="R51">
         <f>COUNTIF(C51:Q51,"✓")</f>
         <v/>
@@ -10012,11 +10757,25 @@
           <t>Seguimiento de salud femenina</t>
         </is>
       </c>
+      <c r="C52" t="inlineStr"/>
+      <c r="D52" t="inlineStr"/>
+      <c r="E52" t="inlineStr"/>
+      <c r="F52" t="inlineStr"/>
+      <c r="G52" t="inlineStr"/>
+      <c r="H52" t="inlineStr"/>
+      <c r="I52" t="inlineStr"/>
+      <c r="J52" t="inlineStr"/>
       <c r="K52" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="L52" t="inlineStr"/>
+      <c r="M52" t="inlineStr"/>
+      <c r="N52" t="inlineStr"/>
+      <c r="O52" t="inlineStr"/>
+      <c r="P52" t="inlineStr"/>
+      <c r="Q52" t="inlineStr"/>
       <c r="R52">
         <f>COUNTIF(C52:Q52,"✓")</f>
         <v/>
@@ -10033,11 +10792,25 @@
           <t>Valoración de profesionales</t>
         </is>
       </c>
+      <c r="C53" t="inlineStr"/>
+      <c r="D53" t="inlineStr"/>
+      <c r="E53" t="inlineStr"/>
       <c r="F53" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="G53" t="inlineStr"/>
+      <c r="H53" t="inlineStr"/>
+      <c r="I53" t="inlineStr"/>
+      <c r="J53" t="inlineStr"/>
+      <c r="K53" t="inlineStr"/>
+      <c r="L53" t="inlineStr"/>
+      <c r="M53" t="inlineStr"/>
+      <c r="N53" t="inlineStr"/>
+      <c r="O53" t="inlineStr"/>
+      <c r="P53" t="inlineStr"/>
+      <c r="Q53" t="inlineStr"/>
       <c r="R53">
         <f>COUNTIF(C53:Q53,"✓")</f>
         <v/>
@@ -10051,24 +10824,28 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Blockchain para integridad y trazabilidad de datos</t>
-        </is>
-      </c>
-      <c r="H54" t="inlineStr">
+          <t>Acceso mínimo por categorías de datos</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr"/>
+      <c r="D54" t="inlineStr"/>
+      <c r="E54" t="inlineStr"/>
+      <c r="F54" t="inlineStr"/>
+      <c r="G54" t="inlineStr"/>
+      <c r="H54" t="inlineStr"/>
+      <c r="I54" t="inlineStr"/>
+      <c r="J54" t="inlineStr"/>
+      <c r="K54" t="inlineStr"/>
+      <c r="L54" t="inlineStr"/>
+      <c r="M54" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="I54" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="J54" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="N54" t="inlineStr"/>
+      <c r="O54" t="inlineStr"/>
+      <c r="P54" t="inlineStr"/>
+      <c r="Q54" t="inlineStr"/>
       <c r="R54">
         <f>COUNTIF(C54:Q54,"✓")</f>
         <v/>
@@ -10082,19 +10859,36 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Cifrado y control de acceso</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
+          <t>Blockchain para integridad y trazabilidad de datos</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr"/>
+      <c r="D55" t="inlineStr"/>
+      <c r="E55" t="inlineStr"/>
+      <c r="F55" t="inlineStr"/>
+      <c r="G55" t="inlineStr"/>
+      <c r="H55" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="K55" t="inlineStr">
+      <c r="I55" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr"/>
+      <c r="L55" t="inlineStr"/>
+      <c r="M55" t="inlineStr"/>
+      <c r="N55" t="inlineStr"/>
+      <c r="O55" t="inlineStr"/>
+      <c r="P55" t="inlineStr"/>
+      <c r="Q55" t="inlineStr"/>
       <c r="R55">
         <f>COUNTIF(C55:Q55,"✓")</f>
         <v/>
@@ -10108,14 +10902,32 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Cumplimiento regulatorio de salud y datos</t>
-        </is>
-      </c>
-      <c r="O56" t="inlineStr">
+          <t>Cifrado y control de acceso</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr"/>
+      <c r="D56" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="E56" t="inlineStr"/>
+      <c r="F56" t="inlineStr"/>
+      <c r="G56" t="inlineStr"/>
+      <c r="H56" t="inlineStr"/>
+      <c r="I56" t="inlineStr"/>
+      <c r="J56" t="inlineStr"/>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr"/>
+      <c r="M56" t="inlineStr"/>
+      <c r="N56" t="inlineStr"/>
+      <c r="O56" t="inlineStr"/>
+      <c r="P56" t="inlineStr"/>
+      <c r="Q56" t="inlineStr"/>
       <c r="R56">
         <f>COUNTIF(C56:Q56,"✓")</f>
         <v/>
@@ -10129,14 +10941,28 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Gestión de consentimiento sobre uso de datos</t>
-        </is>
-      </c>
-      <c r="L57" t="inlineStr">
+          <t>Cumplimiento regulatorio de salud y datos</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr"/>
+      <c r="D57" t="inlineStr"/>
+      <c r="E57" t="inlineStr"/>
+      <c r="F57" t="inlineStr"/>
+      <c r="G57" t="inlineStr"/>
+      <c r="H57" t="inlineStr"/>
+      <c r="I57" t="inlineStr"/>
+      <c r="J57" t="inlineStr"/>
+      <c r="K57" t="inlineStr"/>
+      <c r="L57" t="inlineStr"/>
+      <c r="M57" t="inlineStr"/>
+      <c r="N57" t="inlineStr"/>
+      <c r="O57" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="P57" t="inlineStr"/>
+      <c r="Q57" t="inlineStr"/>
       <c r="R57">
         <f>COUNTIF(C57:Q57,"✓")</f>
         <v/>
@@ -10150,14 +10976,28 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Identidad descentralizada (DID)</t>
-        </is>
-      </c>
-      <c r="I58" t="inlineStr">
+          <t>Gestión de consentimiento sobre uso de datos</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr"/>
+      <c r="D58" t="inlineStr"/>
+      <c r="E58" t="inlineStr"/>
+      <c r="F58" t="inlineStr"/>
+      <c r="G58" t="inlineStr"/>
+      <c r="H58" t="inlineStr"/>
+      <c r="I58" t="inlineStr"/>
+      <c r="J58" t="inlineStr"/>
+      <c r="K58" t="inlineStr"/>
+      <c r="L58" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="M58" t="inlineStr"/>
+      <c r="N58" t="inlineStr"/>
+      <c r="O58" t="inlineStr"/>
+      <c r="P58" t="inlineStr"/>
+      <c r="Q58" t="inlineStr"/>
       <c r="R58">
         <f>COUNTIF(C58:Q58,"✓")</f>
         <v/>
@@ -10171,19 +11011,28 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Privacidad reforzada para datos de salud</t>
-        </is>
-      </c>
-      <c r="L59" t="inlineStr">
+          <t>Identidad descentralizada (DID)</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr"/>
+      <c r="D59" t="inlineStr"/>
+      <c r="E59" t="inlineStr"/>
+      <c r="F59" t="inlineStr"/>
+      <c r="G59" t="inlineStr"/>
+      <c r="H59" t="inlineStr"/>
+      <c r="I59" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="M59" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="J59" t="inlineStr"/>
+      <c r="K59" t="inlineStr"/>
+      <c r="L59" t="inlineStr"/>
+      <c r="M59" t="inlineStr"/>
+      <c r="N59" t="inlineStr"/>
+      <c r="O59" t="inlineStr"/>
+      <c r="P59" t="inlineStr"/>
+      <c r="Q59" t="inlineStr"/>
       <c r="R59">
         <f>COUNTIF(C59:Q59,"✓")</f>
         <v/>
@@ -10192,19 +11041,37 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Seguros y pagos</t>
+          <t>Seguridad, privacidad y blockchain</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Modelo freemium y suscripción</t>
-        </is>
-      </c>
-      <c r="Q60" t="inlineStr">
+          <t>Privacidad reforzada para datos de salud</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr"/>
+      <c r="D60" t="inlineStr"/>
+      <c r="E60" t="inlineStr"/>
+      <c r="F60" t="inlineStr"/>
+      <c r="G60" t="inlineStr"/>
+      <c r="H60" t="inlineStr"/>
+      <c r="I60" t="inlineStr"/>
+      <c r="J60" t="inlineStr"/>
+      <c r="K60" t="inlineStr"/>
+      <c r="L60" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="N60" t="inlineStr"/>
+      <c r="O60" t="inlineStr"/>
+      <c r="P60" t="inlineStr"/>
+      <c r="Q60" t="inlineStr"/>
       <c r="R60">
         <f>COUNTIF(C60:Q60,"✓")</f>
         <v/>
@@ -10218,10 +11085,24 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Pagos con criptomoneda</t>
-        </is>
-      </c>
-      <c r="J61" t="inlineStr">
+          <t>Modelo freemium y suscripción</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr"/>
+      <c r="D61" t="inlineStr"/>
+      <c r="E61" t="inlineStr"/>
+      <c r="F61" t="inlineStr"/>
+      <c r="G61" t="inlineStr"/>
+      <c r="H61" t="inlineStr"/>
+      <c r="I61" t="inlineStr"/>
+      <c r="J61" t="inlineStr"/>
+      <c r="K61" t="inlineStr"/>
+      <c r="L61" t="inlineStr"/>
+      <c r="M61" t="inlineStr"/>
+      <c r="N61" t="inlineStr"/>
+      <c r="O61" t="inlineStr"/>
+      <c r="P61" t="inlineStr"/>
+      <c r="Q61" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -10239,14 +11120,28 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Pagos dentro de la app</t>
-        </is>
-      </c>
-      <c r="Q62" t="inlineStr">
+          <t>Pagos con criptomoneda</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr"/>
+      <c r="D62" t="inlineStr"/>
+      <c r="E62" t="inlineStr"/>
+      <c r="F62" t="inlineStr"/>
+      <c r="G62" t="inlineStr"/>
+      <c r="H62" t="inlineStr"/>
+      <c r="I62" t="inlineStr"/>
+      <c r="J62" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="K62" t="inlineStr"/>
+      <c r="L62" t="inlineStr"/>
+      <c r="M62" t="inlineStr"/>
+      <c r="N62" t="inlineStr"/>
+      <c r="O62" t="inlineStr"/>
+      <c r="P62" t="inlineStr"/>
+      <c r="Q62" t="inlineStr"/>
       <c r="R62">
         <f>COUNTIF(C62:Q62,"✓")</f>
         <v/>
@@ -10260,10 +11155,24 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Reclamos y trámites con seguros</t>
-        </is>
-      </c>
-      <c r="I63" t="inlineStr">
+          <t>Pagos dentro de la app</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr"/>
+      <c r="D63" t="inlineStr"/>
+      <c r="E63" t="inlineStr"/>
+      <c r="F63" t="inlineStr"/>
+      <c r="G63" t="inlineStr"/>
+      <c r="H63" t="inlineStr"/>
+      <c r="I63" t="inlineStr"/>
+      <c r="J63" t="inlineStr"/>
+      <c r="K63" t="inlineStr"/>
+      <c r="L63" t="inlineStr"/>
+      <c r="M63" t="inlineStr"/>
+      <c r="N63" t="inlineStr"/>
+      <c r="O63" t="inlineStr"/>
+      <c r="P63" t="inlineStr"/>
+      <c r="Q63" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -10276,21 +11185,70 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Telemedicina y atención remota</t>
+          <t>Seguros y pagos</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Teleconsulta con profesionales</t>
-        </is>
-      </c>
-      <c r="J64" t="inlineStr">
+          <t>Reclamos y trámites con seguros</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr"/>
+      <c r="D64" t="inlineStr"/>
+      <c r="E64" t="inlineStr"/>
+      <c r="F64" t="inlineStr"/>
+      <c r="G64" t="inlineStr"/>
+      <c r="H64" t="inlineStr"/>
+      <c r="I64" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="J64" t="inlineStr"/>
+      <c r="K64" t="inlineStr"/>
+      <c r="L64" t="inlineStr"/>
+      <c r="M64" t="inlineStr"/>
+      <c r="N64" t="inlineStr"/>
+      <c r="O64" t="inlineStr"/>
+      <c r="P64" t="inlineStr"/>
+      <c r="Q64" t="inlineStr"/>
       <c r="R64">
         <f>COUNTIF(C64:Q64,"✓")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Telemedicina y atención remota</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Teleconsulta con profesionales</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr"/>
+      <c r="D65" t="inlineStr"/>
+      <c r="E65" t="inlineStr"/>
+      <c r="F65" t="inlineStr"/>
+      <c r="G65" t="inlineStr"/>
+      <c r="H65" t="inlineStr"/>
+      <c r="I65" t="inlineStr"/>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr"/>
+      <c r="L65" t="inlineStr"/>
+      <c r="M65" t="inlineStr"/>
+      <c r="N65" t="inlineStr"/>
+      <c r="O65" t="inlineStr"/>
+      <c r="P65" t="inlineStr"/>
+      <c r="Q65" t="inlineStr"/>
+      <c r="R65">
+        <f>COUNTIF(C65:Q65,"✓")</f>
         <v/>
       </c>
     </row>
@@ -10305,7 +11263,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A24"/>
+  <dimension ref="A1:A25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -10479,6 +11437,13 @@
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>VUELTA 5 COMPLETA (2026-10-12 12:16 UTC): Clinia, MiRedSalud y Mediko verificados (+0 filas en esta iteración). Contador de loops = 5 para todos, Revisado reiniciado a "No". func_norm (127 filas) y tabla_frecuencia (64 funcionalidades) regenerados. Corregido financiamiento de Mediko (CLP 40M, no US$40M). Vuelta 6 parte con Meedika, Infomed, MediPlanner, Clingot. Candidato a competidor sin agregar: HealthChain (Chile).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Benchmark: vuelta 6, iteración 1 (Meedika, Infomed, MediPlanner, Clingot)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MVcXu8vTBu7EKfj3YdEvae
</commit_message>
<xml_diff>
--- a/Outputs/Benchmark_Anamnesis.xlsx
+++ b/Outputs/Benchmark_Anamnesis.xlsx
@@ -513,12 +513,12 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>[DIRECTO · Chile · etapas A+B] Lanzada 25-sep-2024 en App Store (Android previsto la misma semana). &gt;1.500 usuarios en los primeros días; meta 32.000 (cofundador Francisco González). Funciones: gestión de documentos, importar solicitudes, SOS con alergias/medicación, calendario de citas, recordatorios, compartir con profesionales elegidos. Sin blockchain. Precio y estado actual NO verificados; única fuente es una nota de prensa. Sitio oficial por confirmar. [Iter. 2] Hay cobertura adicional en Portal Innova (portalinnova.cl); sitio bloqueado en este entorno, estado actual sigue sin verificar. [Vuelta 3] Sin novedades 2026 ni confirmación de la app Android en Google Play; usuarios actuales desconocidos. Nota de prensa no indica año de lanzamiento explícito. [Vuelta 4] Sin fuentes nuevas; portalinnova.cl no aparece en búsquedas. Sigue dependiendo de una sola nota de prensa. [Vuelta 5] Sin fuentes nuevas (ni entrevistas ni financiamiento); sigue dependiendo de una sola nota de prensa sin año explícito.</t>
+          <t>[DIRECTO · Chile · etapas A+B] Lanzada 25-sep-2024 en App Store (Android previsto la misma semana). &gt;1.500 usuarios en los primeros días; meta 32.000 (cofundador Francisco González). Funciones: gestión de documentos, importar solicitudes, SOS con alergias/medicación, calendario de citas, recordatorios, compartir con profesionales elegidos. Sin blockchain. Precio y estado actual NO verificados; única fuente es una nota de prensa. Sitio oficial por confirmar. [Iter. 2] Hay cobertura adicional en Portal Innova (portalinnova.cl); sitio bloqueado en este entorno, estado actual sigue sin verificar. [Vuelta 3] Sin novedades 2026 ni confirmación de la app Android en Google Play; usuarios actuales desconocidos. Nota de prensa no indica año de lanzamiento explícito. [Vuelta 4] Sin fuentes nuevas; portalinnova.cl no aparece en búsquedas. Sigue dependiendo de una sola nota de prensa. [Vuelta 5] Sin fuentes nuevas (ni entrevistas ni financiamiento); sigue dependiendo de una sola nota de prensa sin año explícito. [Vuelta 6] Sin ficha de Google Play ni fuentes nuevas; disponibilidad en Android sin confirmar.</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G2" t="n">
@@ -526,7 +526,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
     </row>
@@ -553,12 +553,12 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>[DIRECTO · Chile · etapa A] Fundada 2019 por Diego Ibarra, Andrés Fantuzzi y Gabriel Zamora. Lanzada mar-2021 en App Store y Play Store con 1.200 usuarios; planeaba nueva versión jul-2021 y ronda de US$500 mil. Objetivo: llevar el historial en el celular, acceso en emergencias, médico puede ingresar datos con consentimiento. Estado actual NO verificado (posible app inactiva). URL es la nota de prensa; sitio oficial por confirmar. [Vuelta 3] Sin evidencia posterior a 2021; relanzamiento previsto jul-2021 no confirmado. Probable app inactiva. [Vuelta 4] Sin cambios; sigue sin evidencia posterior a 2021. [Vuelta 5] Cofundador Andrés Fantuzzi es cardiólogo de la Clínica Santa María. Sin ronda de inversión ni relanzamiento confirmados; no confundir con Infomed de Cuba (portal del Minsap).</t>
+          <t>[DIRECTO · Chile · etapa A] Fundada 2019 por Diego Ibarra, Andrés Fantuzzi y Gabriel Zamora. Lanzada mar-2021 en App Store y Play Store con 1.200 usuarios; planeaba nueva versión jul-2021 y ronda de US$500 mil. Objetivo: llevar el historial en el celular, acceso en emergencias, médico puede ingresar datos con consentimiento. Estado actual NO verificado (posible app inactiva). URL es la nota de prensa; sitio oficial por confirmar. [Vuelta 3] Sin evidencia posterior a 2021; relanzamiento previsto jul-2021 no confirmado. Probable app inactiva. [Vuelta 4] Sin cambios; sigue sin evidencia posterior a 2021. [Vuelta 5] Cofundador Andrés Fantuzzi es cardiólogo de la Clínica Santa María. Sin ronda de inversión ni relanzamiento confirmados; no confundir con Infomed de Cuba (portal del Minsap). [Vuelta 6] Sin búsqueda nueva (fuentes agotadas en vueltas 3-5); sin cambios.</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G3" t="n">
@@ -566,7 +566,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
     </row>
@@ -593,12 +593,12 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>[REGIONAL · México] Historial por perfil familiar, alergias, vacunas, recetas digitales, gráficas de evolución, agendamiento, compartir con profesionales. Gratis en App Store MX. Sin evidencia de uso en Chile. Cubre parte de la etapa C (familia). [Vuelta 3] Existen dos apps distintas: MediPlanner (gratis, Rym Solutions, MX, 3,7/5 con 3 calificaciones) y MediPlanner Pro (otro desarrollador, $39 MXN). Sin presencia verificada en Chile. [Vuelta 4] No pude confirmar el desarrollador de la versión gratuita (Rym Solutions no se repite en esta búsqueda). MediPlanner Pro (fichas BR/OM) guardaría datos solo en el dispositivo, sin nube; no confundir con MedPlanner/AskHEMI (otra empresa). [Vuelta 5] Sin búsqueda nueva (revisada en vuelta 4); sin cambios.</t>
+          <t>[REGIONAL · México] Historial por perfil familiar, alergias, vacunas, recetas digitales, gráficas de evolución, agendamiento, compartir con profesionales. Gratis en App Store MX. Sin evidencia de uso en Chile. Cubre parte de la etapa C (familia). [Vuelta 3] Existen dos apps distintas: MediPlanner (gratis, Rym Solutions, MX, 3,7/5 con 3 calificaciones) y MediPlanner Pro (otro desarrollador, $39 MXN). Sin presencia verificada en Chile. [Vuelta 4] No pude confirmar el desarrollador de la versión gratuita (Rym Solutions no se repite en esta búsqueda). MediPlanner Pro (fichas BR/OM) guardaría datos solo en el dispositivo, sin nube; no confundir con MedPlanner/AskHEMI (otra empresa). [Vuelta 5] Sin búsqueda nueva (revisada en vuelta 4); sin cambios. [Vuelta 6] Se reconfirma en la ficha de App Store MX que el desarrollador de la versión gratuita es Rym Solutions S. de R.L. de C.V. (3,7/5, 3 calificaciones); MediPlanner Pro no menciona a esa empresa, por lo que no se puede asegurar que sea el mismo desarrollador.</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G4" t="n">
@@ -606,7 +606,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
     </row>
@@ -633,12 +633,12 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>[REGIONAL · Argentina · débil] App para cargar antecedentes médicos propios. Única referencia: nota de opinión en grupoanimal.mx sin fecha verificada. Estado y sitio por confirmar. [Vuelta 3] Referencias de 2017 (apps4citizens, La Nación); sitio y precio no verificados; puede estar inactiva. [Vuelta 4] Sin fuentes nuevas. [Vuelta 5] Registro empresarial (indicadores.ar, datos a jul-2026) muestra CLINGOT S.A. activa en CABA, constituida el 4-abr-2016; no confirma que la app siga operando. Programa federal argentino de historias clínicas digitales como contexto regulatorio.</t>
+          <t>[REGIONAL · Argentina · débil] App para cargar antecedentes médicos propios. Única referencia: nota de opinión en grupoanimal.mx sin fecha verificada. Estado y sitio por confirmar. [Vuelta 3] Referencias de 2017 (apps4citizens, La Nación); sitio y precio no verificados; puede estar inactiva. [Vuelta 4] Sin fuentes nuevas. [Vuelta 5] Registro empresarial (indicadores.ar, datos a jul-2026) muestra CLINGOT S.A. activa en CABA, constituida el 4-abr-2016; no confirma que la app siga operando. Programa federal argentino de historias clínicas digitales como contexto regulatorio. [Vuelta 6] Sin búsqueda nueva (fuentes agotadas); sin cambios.</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G5" t="n">
@@ -646,7 +646,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
     </row>
@@ -8823,8 +8823,6 @@
           <t>Búsqueda de profesionales de salud</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
           <t>✓</t>
@@ -8835,17 +8833,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
       <c r="R2">
         <f>COUNTIF(C2:Q2,"✓")</f>
         <v/>
@@ -8867,24 +8854,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
       <c r="R3">
         <f>COUNTIF(C3:Q3,"✓")</f>
         <v/>
@@ -8901,25 +8875,11 @@
           <t>Integración con calendario del dispositivo</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
       <c r="R4">
         <f>COUNTIF(C4:Q4,"✓")</f>
         <v/>
@@ -8936,25 +8896,11 @@
           <t>Localización de centros médicos y farmacias</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr"/>
       <c r="R5">
         <f>COUNTIF(C5:Q5,"✓")</f>
         <v/>
@@ -8971,17 +8917,6 @@
           <t>Reserva de citas médicas</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr">
         <is>
           <t>✓</t>
@@ -8992,8 +8927,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="inlineStr"/>
       <c r="R6">
         <f>COUNTIF(C6:Q6,"✓")</f>
         <v/>
@@ -9010,25 +8943,11 @@
           <t>Acceso del profesional al historial del paciente</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr"/>
-      <c r="Q7" t="inlineStr"/>
       <c r="R7">
         <f>COUNTIF(C7:Q7,"✓")</f>
         <v/>
@@ -9045,25 +8964,11 @@
           <t>Compartir con personas sin cuenta mediante clave segura</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
-      <c r="P8" t="inlineStr"/>
-      <c r="Q8" t="inlineStr"/>
       <c r="R8">
         <f>COUNTIF(C8:Q8,"✓")</f>
         <v/>
@@ -9080,25 +8985,11 @@
           <t>Compartir datos con cuidador o persona de confianza</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
-      <c r="P9" t="inlineStr"/>
-      <c r="Q9" t="inlineStr"/>
       <c r="R9">
         <f>COUNTIF(C9:Q9,"✓")</f>
         <v/>
@@ -9120,13 +9011,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9152,16 +9041,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
       <c r="O10" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="P10" t="inlineStr"/>
-      <c r="Q10" t="inlineStr"/>
       <c r="R10">
         <f>COUNTIF(C10:Q10,"✓")</f>
         <v/>
@@ -9178,25 +9062,11 @@
           <t>Gestión de consentimiento sobre uso de datos</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr"/>
-      <c r="P11" t="inlineStr"/>
-      <c r="Q11" t="inlineStr"/>
       <c r="R11">
         <f>COUNTIF(C11:Q11,"✓")</f>
         <v/>
@@ -9213,25 +9083,11 @@
           <t>Ingreso de datos por profesional con consentimiento</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
-      <c r="O12" t="inlineStr"/>
-      <c r="P12" t="inlineStr"/>
-      <c r="Q12" t="inlineStr"/>
       <c r="R12">
         <f>COUNTIF(C12:Q12,"✓")</f>
         <v/>
@@ -9248,25 +9104,11 @@
           <t>Red social con profesionales y familiares</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr"/>
-      <c r="O13" t="inlineStr"/>
-      <c r="P13" t="inlineStr"/>
-      <c r="Q13" t="inlineStr"/>
       <c r="R13">
         <f>COUNTIF(C13:Q13,"✓")</f>
         <v/>
@@ -9293,23 +9135,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
-      <c r="M14" t="inlineStr"/>
-      <c r="N14" t="inlineStr"/>
-      <c r="O14" t="inlineStr"/>
-      <c r="P14" t="inlineStr"/>
-      <c r="Q14" t="inlineStr"/>
       <c r="R14">
         <f>COUNTIF(C14:Q14,"✓")</f>
         <v/>
@@ -9326,8 +9156,6 @@
           <t>Perfiles familiares / dependientes</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9338,29 +9166,21 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr"/>
       <c r="N15" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="Q15" t="inlineStr"/>
       <c r="R15">
         <f>COUNTIF(C15:Q15,"✓")</f>
         <v/>
@@ -9382,8 +9202,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9399,19 +9217,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
-      <c r="M16" t="inlineStr"/>
-      <c r="N16" t="inlineStr"/>
       <c r="O16" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="P16" t="inlineStr"/>
-      <c r="Q16" t="inlineStr"/>
       <c r="R16">
         <f>COUNTIF(C16:Q16,"✓")</f>
         <v/>
@@ -9428,29 +9238,16 @@
           <t>Almacenamiento de recetas</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr"/>
       <c r="N17" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="O17" t="inlineStr"/>
-      <c r="P17" t="inlineStr"/>
-      <c r="Q17" t="inlineStr"/>
       <c r="R17">
         <f>COUNTIF(C17:Q17,"✓")</f>
         <v/>
@@ -9467,25 +9264,11 @@
           <t>Búsqueda y filtros de documentos</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr"/>
-      <c r="M18" t="inlineStr"/>
-      <c r="N18" t="inlineStr"/>
-      <c r="O18" t="inlineStr"/>
-      <c r="P18" t="inlineStr"/>
-      <c r="Q18" t="inlineStr"/>
       <c r="R18">
         <f>COUNTIF(C18:Q18,"✓")</f>
         <v/>
@@ -9502,25 +9285,11 @@
           <t>Emisión de certificados médicos</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr"/>
-      <c r="M19" t="inlineStr"/>
-      <c r="N19" t="inlineStr"/>
-      <c r="O19" t="inlineStr"/>
-      <c r="P19" t="inlineStr"/>
-      <c r="Q19" t="inlineStr"/>
       <c r="R19">
         <f>COUNTIF(C19:Q19,"✓")</f>
         <v/>
@@ -9542,19 +9311,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr"/>
-      <c r="M20" t="inlineStr"/>
-      <c r="N20" t="inlineStr"/>
-      <c r="O20" t="inlineStr"/>
-      <c r="P20" t="inlineStr"/>
       <c r="Q20" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9576,25 +9332,11 @@
           <t>Notificación y envío de resultados</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr"/>
-      <c r="M21" t="inlineStr"/>
       <c r="N21" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="O21" t="inlineStr"/>
-      <c r="P21" t="inlineStr"/>
-      <c r="Q21" t="inlineStr"/>
       <c r="R21">
         <f>COUNTIF(C21:Q21,"✓")</f>
         <v/>
@@ -9611,29 +9353,16 @@
           <t>Historial institucional (solo datos de la propia red)</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
-      <c r="L22" t="inlineStr"/>
-      <c r="M22" t="inlineStr"/>
       <c r="N22" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="O22" t="inlineStr"/>
       <c r="P22" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="Q22" t="inlineStr"/>
       <c r="R22">
         <f>COUNTIF(C22:Q22,"✓")</f>
         <v/>
@@ -9650,36 +9379,26 @@
           <t>Historial médico centralizado</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="L23" t="inlineStr"/>
-      <c r="M23" t="inlineStr"/>
-      <c r="N23" t="inlineStr"/>
-      <c r="O23" t="inlineStr"/>
-      <c r="P23" t="inlineStr"/>
       <c r="Q23" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9701,25 +9420,11 @@
           <t>Línea de tiempo de salud</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
-      <c r="L24" t="inlineStr"/>
-      <c r="M24" t="inlineStr"/>
-      <c r="N24" t="inlineStr"/>
-      <c r="O24" t="inlineStr"/>
-      <c r="P24" t="inlineStr"/>
-      <c r="Q24" t="inlineStr"/>
       <c r="R24">
         <f>COUNTIF(C24:Q24,"✓")</f>
         <v/>
@@ -9736,25 +9441,11 @@
           <t>Registro de alergias y vacunas</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr"/>
-      <c r="L25" t="inlineStr"/>
-      <c r="M25" t="inlineStr"/>
-      <c r="N25" t="inlineStr"/>
-      <c r="O25" t="inlineStr"/>
-      <c r="P25" t="inlineStr"/>
-      <c r="Q25" t="inlineStr"/>
       <c r="R25">
         <f>COUNTIF(C25:Q25,"✓")</f>
         <v/>
@@ -9771,25 +9462,11 @@
           <t>Seguimiento de visitas, gastos y seguros</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr"/>
-      <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr"/>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
-      <c r="L26" t="inlineStr"/>
-      <c r="M26" t="inlineStr"/>
-      <c r="N26" t="inlineStr"/>
-      <c r="O26" t="inlineStr"/>
-      <c r="P26" t="inlineStr"/>
-      <c r="Q26" t="inlineStr"/>
       <c r="R26">
         <f>COUNTIF(C26:Q26,"✓")</f>
         <v/>
@@ -9806,11 +9483,6 @@
           <t>Recompensas / monetización de datos del usuario</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr"/>
-      <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9826,13 +9498,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="K27" t="inlineStr"/>
-      <c r="L27" t="inlineStr"/>
-      <c r="M27" t="inlineStr"/>
-      <c r="N27" t="inlineStr"/>
-      <c r="O27" t="inlineStr"/>
-      <c r="P27" t="inlineStr"/>
-      <c r="Q27" t="inlineStr"/>
       <c r="R27">
         <f>COUNTIF(C27:Q27,"✓")</f>
         <v/>
@@ -9849,25 +9514,11 @@
           <t>Asistente de IA para profesionales de salud</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="M28" t="inlineStr"/>
-      <c r="N28" t="inlineStr"/>
-      <c r="O28" t="inlineStr"/>
-      <c r="P28" t="inlineStr"/>
-      <c r="Q28" t="inlineStr"/>
       <c r="R28">
         <f>COUNTIF(C28:Q28,"✓")</f>
         <v/>
@@ -9884,25 +9535,11 @@
           <t>Coaching de salud con IA</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr"/>
-      <c r="D29" t="inlineStr"/>
-      <c r="E29" t="inlineStr"/>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr"/>
-      <c r="L29" t="inlineStr"/>
-      <c r="M29" t="inlineStr"/>
-      <c r="N29" t="inlineStr"/>
-      <c r="O29" t="inlineStr"/>
-      <c r="P29" t="inlineStr"/>
-      <c r="Q29" t="inlineStr"/>
       <c r="R29">
         <f>COUNTIF(C29:Q29,"✓")</f>
         <v/>
@@ -9919,15 +9556,6 @@
           <t>Detección de patrones en métricas de salud con IA</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr"/>
-      <c r="E30" t="inlineStr"/>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr"/>
-      <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9938,10 +9566,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="N30" t="inlineStr"/>
-      <c r="O30" t="inlineStr"/>
-      <c r="P30" t="inlineStr"/>
-      <c r="Q30" t="inlineStr"/>
       <c r="R30">
         <f>COUNTIF(C30:Q30,"✓")</f>
         <v/>
@@ -9958,15 +9582,6 @@
           <t>Interpretación de exámenes con IA</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr"/>
-      <c r="D31" t="inlineStr"/>
-      <c r="E31" t="inlineStr"/>
-      <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr"/>
-      <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9977,9 +9592,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="N31" t="inlineStr"/>
-      <c r="O31" t="inlineStr"/>
-      <c r="P31" t="inlineStr"/>
       <c r="Q31" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10001,24 +9613,11 @@
           <t>Orientación médica con IA</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr"/>
-      <c r="D32" t="inlineStr"/>
-      <c r="E32" t="inlineStr"/>
-      <c r="F32" t="inlineStr"/>
-      <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr"/>
-      <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr"/>
-      <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="M32" t="inlineStr"/>
-      <c r="N32" t="inlineStr"/>
-      <c r="O32" t="inlineStr"/>
-      <c r="P32" t="inlineStr"/>
       <c r="Q32" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10040,15 +9639,6 @@
           <t>Preparación de consultas médicas con IA</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr"/>
-      <c r="D33" t="inlineStr"/>
-      <c r="E33" t="inlineStr"/>
-      <c r="F33" t="inlineStr"/>
-      <c r="G33" t="inlineStr"/>
-      <c r="H33" t="inlineStr"/>
-      <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr"/>
-      <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10059,10 +9649,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="N33" t="inlineStr"/>
-      <c r="O33" t="inlineStr"/>
-      <c r="P33" t="inlineStr"/>
-      <c r="Q33" t="inlineStr"/>
       <c r="R33">
         <f>COUNTIF(C33:Q33,"✓")</f>
         <v/>
@@ -10079,15 +9665,6 @@
           <t>Resumen de historial con IA</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr"/>
-      <c r="D34" t="inlineStr"/>
-      <c r="E34" t="inlineStr"/>
-      <c r="F34" t="inlineStr"/>
-      <c r="G34" t="inlineStr"/>
-      <c r="H34" t="inlineStr"/>
-      <c r="I34" t="inlineStr"/>
-      <c r="J34" t="inlineStr"/>
-      <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10098,10 +9675,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="N34" t="inlineStr"/>
-      <c r="O34" t="inlineStr"/>
-      <c r="P34" t="inlineStr"/>
-      <c r="Q34" t="inlineStr"/>
       <c r="R34">
         <f>COUNTIF(C34:Q34,"✓")</f>
         <v/>
@@ -10123,10 +9696,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr"/>
-      <c r="E35" t="inlineStr"/>
-      <c r="F35" t="inlineStr"/>
-      <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10137,7 +9706,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="J35" t="inlineStr"/>
       <c r="K35" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10153,14 +9721,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="N35" t="inlineStr"/>
       <c r="O35" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="P35" t="inlineStr"/>
-      <c r="Q35" t="inlineStr"/>
       <c r="R35">
         <f>COUNTIF(C35:Q35,"✓")</f>
         <v/>
@@ -10177,25 +9742,11 @@
           <t>Analítica poblacional B2B</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr"/>
-      <c r="D36" t="inlineStr"/>
-      <c r="E36" t="inlineStr"/>
-      <c r="F36" t="inlineStr"/>
-      <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="I36" t="inlineStr"/>
-      <c r="J36" t="inlineStr"/>
-      <c r="K36" t="inlineStr"/>
-      <c r="L36" t="inlineStr"/>
-      <c r="M36" t="inlineStr"/>
-      <c r="N36" t="inlineStr"/>
-      <c r="O36" t="inlineStr"/>
-      <c r="P36" t="inlineStr"/>
-      <c r="Q36" t="inlineStr"/>
       <c r="R36">
         <f>COUNTIF(C36:Q36,"✓")</f>
         <v/>
@@ -10212,9 +9763,6 @@
           <t>Disponibilidad multiplataforma (web/iOS/Android)</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr"/>
-      <c r="D37" t="inlineStr"/>
-      <c r="E37" t="inlineStr"/>
       <c r="F37" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10225,20 +9773,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr"/>
-      <c r="J37" t="inlineStr"/>
-      <c r="K37" t="inlineStr"/>
-      <c r="L37" t="inlineStr"/>
-      <c r="M37" t="inlineStr"/>
-      <c r="N37" t="inlineStr"/>
       <c r="O37" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="P37" t="inlineStr"/>
-      <c r="Q37" t="inlineStr"/>
       <c r="R37">
         <f>COUNTIF(C37:Q37,"✓")</f>
         <v/>
@@ -10255,25 +9794,11 @@
           <t>Historial médico centralizado</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr"/>
-      <c r="D38" t="inlineStr"/>
-      <c r="E38" t="inlineStr"/>
-      <c r="F38" t="inlineStr"/>
-      <c r="G38" t="inlineStr"/>
-      <c r="H38" t="inlineStr"/>
-      <c r="I38" t="inlineStr"/>
       <c r="J38" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="K38" t="inlineStr"/>
-      <c r="L38" t="inlineStr"/>
-      <c r="M38" t="inlineStr"/>
-      <c r="N38" t="inlineStr"/>
-      <c r="O38" t="inlineStr"/>
-      <c r="P38" t="inlineStr"/>
-      <c r="Q38" t="inlineStr"/>
       <c r="R38">
         <f>COUNTIF(C38:Q38,"✓")</f>
         <v/>
@@ -10290,25 +9815,11 @@
           <t>Importación y exportación de datos</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr"/>
-      <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr"/>
-      <c r="G39" t="inlineStr"/>
-      <c r="H39" t="inlineStr"/>
-      <c r="I39" t="inlineStr"/>
-      <c r="J39" t="inlineStr"/>
-      <c r="K39" t="inlineStr"/>
-      <c r="L39" t="inlineStr"/>
-      <c r="M39" t="inlineStr"/>
-      <c r="N39" t="inlineStr"/>
-      <c r="O39" t="inlineStr"/>
-      <c r="P39" t="inlineStr"/>
-      <c r="Q39" t="inlineStr"/>
       <c r="R39">
         <f>COUNTIF(C39:Q39,"✓")</f>
         <v/>
@@ -10325,25 +9836,11 @@
           <t>Integración con EHR de proveedores</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr"/>
-      <c r="D40" t="inlineStr"/>
-      <c r="E40" t="inlineStr"/>
-      <c r="F40" t="inlineStr"/>
-      <c r="G40" t="inlineStr"/>
-      <c r="H40" t="inlineStr"/>
-      <c r="I40" t="inlineStr"/>
       <c r="J40" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="K40" t="inlineStr"/>
-      <c r="L40" t="inlineStr"/>
-      <c r="M40" t="inlineStr"/>
-      <c r="N40" t="inlineStr"/>
-      <c r="O40" t="inlineStr"/>
-      <c r="P40" t="inlineStr"/>
-      <c r="Q40" t="inlineStr"/>
       <c r="R40">
         <f>COUNTIF(C40:Q40,"✓")</f>
         <v/>
@@ -10360,29 +9857,16 @@
           <t>Integración con wearables y apps de salud</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr"/>
-      <c r="D41" t="inlineStr"/>
-      <c r="E41" t="inlineStr"/>
-      <c r="F41" t="inlineStr"/>
-      <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="I41" t="inlineStr"/>
-      <c r="J41" t="inlineStr"/>
-      <c r="K41" t="inlineStr"/>
-      <c r="L41" t="inlineStr"/>
       <c r="M41" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="N41" t="inlineStr"/>
-      <c r="O41" t="inlineStr"/>
-      <c r="P41" t="inlineStr"/>
-      <c r="Q41" t="inlineStr"/>
       <c r="R41">
         <f>COUNTIF(C41:Q41,"✓")</f>
         <v/>
@@ -10399,25 +9883,11 @@
           <t>Gestión de lista de medicamentos</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr"/>
-      <c r="D42" t="inlineStr"/>
-      <c r="E42" t="inlineStr"/>
-      <c r="F42" t="inlineStr"/>
-      <c r="G42" t="inlineStr"/>
-      <c r="H42" t="inlineStr"/>
-      <c r="I42" t="inlineStr"/>
-      <c r="J42" t="inlineStr"/>
       <c r="K42" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="L42" t="inlineStr"/>
-      <c r="M42" t="inlineStr"/>
-      <c r="N42" t="inlineStr"/>
-      <c r="O42" t="inlineStr"/>
-      <c r="P42" t="inlineStr"/>
-      <c r="Q42" t="inlineStr"/>
       <c r="R42">
         <f>COUNTIF(C42:Q42,"✓")</f>
         <v/>
@@ -10434,25 +9904,11 @@
           <t>Importación automática de tratamientos desde receta digital</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr"/>
-      <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr"/>
-      <c r="G43" t="inlineStr"/>
-      <c r="H43" t="inlineStr"/>
-      <c r="I43" t="inlineStr"/>
-      <c r="J43" t="inlineStr"/>
-      <c r="K43" t="inlineStr"/>
-      <c r="L43" t="inlineStr"/>
-      <c r="M43" t="inlineStr"/>
-      <c r="N43" t="inlineStr"/>
-      <c r="O43" t="inlineStr"/>
-      <c r="P43" t="inlineStr"/>
-      <c r="Q43" t="inlineStr"/>
       <c r="R43">
         <f>COUNTIF(C43:Q43,"✓")</f>
         <v/>
@@ -10474,24 +9930,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr"/>
-      <c r="E44" t="inlineStr"/>
-      <c r="F44" t="inlineStr"/>
-      <c r="G44" t="inlineStr"/>
-      <c r="H44" t="inlineStr"/>
-      <c r="I44" t="inlineStr"/>
-      <c r="J44" t="inlineStr"/>
       <c r="K44" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="L44" t="inlineStr"/>
-      <c r="M44" t="inlineStr"/>
-      <c r="N44" t="inlineStr"/>
-      <c r="O44" t="inlineStr"/>
-      <c r="P44" t="inlineStr"/>
-      <c r="Q44" t="inlineStr"/>
       <c r="R44">
         <f>COUNTIF(C44:Q44,"✓")</f>
         <v/>
@@ -10508,25 +9951,11 @@
           <t>Registro de tomas y adherencia al tratamiento</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr"/>
-      <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr"/>
-      <c r="G45" t="inlineStr"/>
-      <c r="H45" t="inlineStr"/>
-      <c r="I45" t="inlineStr"/>
-      <c r="J45" t="inlineStr"/>
-      <c r="K45" t="inlineStr"/>
-      <c r="L45" t="inlineStr"/>
-      <c r="M45" t="inlineStr"/>
-      <c r="N45" t="inlineStr"/>
-      <c r="O45" t="inlineStr"/>
-      <c r="P45" t="inlineStr"/>
-      <c r="Q45" t="inlineStr"/>
       <c r="R45">
         <f>COUNTIF(C45:Q45,"✓")</f>
         <v/>
@@ -10543,25 +9972,11 @@
           <t>Comunidad de pacientes</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr"/>
-      <c r="D46" t="inlineStr"/>
-      <c r="E46" t="inlineStr"/>
-      <c r="F46" t="inlineStr"/>
-      <c r="G46" t="inlineStr"/>
       <c r="H46" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="I46" t="inlineStr"/>
-      <c r="J46" t="inlineStr"/>
-      <c r="K46" t="inlineStr"/>
-      <c r="L46" t="inlineStr"/>
-      <c r="M46" t="inlineStr"/>
-      <c r="N46" t="inlineStr"/>
-      <c r="O46" t="inlineStr"/>
-      <c r="P46" t="inlineStr"/>
-      <c r="Q46" t="inlineStr"/>
       <c r="R46">
         <f>COUNTIF(C46:Q46,"✓")</f>
         <v/>
@@ -10578,25 +9993,11 @@
           <t>Contenido educativo sobre salud</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr"/>
       <c r="D47" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr"/>
-      <c r="F47" t="inlineStr"/>
-      <c r="G47" t="inlineStr"/>
-      <c r="H47" t="inlineStr"/>
-      <c r="I47" t="inlineStr"/>
-      <c r="J47" t="inlineStr"/>
-      <c r="K47" t="inlineStr"/>
-      <c r="L47" t="inlineStr"/>
-      <c r="M47" t="inlineStr"/>
-      <c r="N47" t="inlineStr"/>
-      <c r="O47" t="inlineStr"/>
-      <c r="P47" t="inlineStr"/>
-      <c r="Q47" t="inlineStr"/>
       <c r="R47">
         <f>COUNTIF(C47:Q47,"✓")</f>
         <v/>
@@ -10613,25 +10014,11 @@
           <t>Gráficas de evolución de indicadores</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr"/>
-      <c r="D48" t="inlineStr"/>
       <c r="E48" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr"/>
-      <c r="G48" t="inlineStr"/>
-      <c r="H48" t="inlineStr"/>
-      <c r="I48" t="inlineStr"/>
-      <c r="J48" t="inlineStr"/>
-      <c r="K48" t="inlineStr"/>
-      <c r="L48" t="inlineStr"/>
-      <c r="M48" t="inlineStr"/>
-      <c r="N48" t="inlineStr"/>
-      <c r="O48" t="inlineStr"/>
-      <c r="P48" t="inlineStr"/>
-      <c r="Q48" t="inlineStr"/>
       <c r="R48">
         <f>COUNTIF(C48:Q48,"✓")</f>
         <v/>
@@ -10648,25 +10035,11 @@
           <t>Integración con wearables y apps de salud</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr"/>
-      <c r="D49" t="inlineStr"/>
-      <c r="E49" t="inlineStr"/>
-      <c r="F49" t="inlineStr"/>
-      <c r="G49" t="inlineStr"/>
-      <c r="H49" t="inlineStr"/>
-      <c r="I49" t="inlineStr"/>
-      <c r="J49" t="inlineStr"/>
       <c r="K49" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="L49" t="inlineStr"/>
-      <c r="M49" t="inlineStr"/>
-      <c r="N49" t="inlineStr"/>
-      <c r="O49" t="inlineStr"/>
-      <c r="P49" t="inlineStr"/>
-      <c r="Q49" t="inlineStr"/>
       <c r="R49">
         <f>COUNTIF(C49:Q49,"✓")</f>
         <v/>
@@ -10683,11 +10056,6 @@
           <t>Panel de seguimiento de salud y bienestar</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr"/>
-      <c r="D50" t="inlineStr"/>
-      <c r="E50" t="inlineStr"/>
-      <c r="F50" t="inlineStr"/>
-      <c r="G50" t="inlineStr"/>
       <c r="H50" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10698,14 +10066,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="J50" t="inlineStr"/>
-      <c r="K50" t="inlineStr"/>
-      <c r="L50" t="inlineStr"/>
-      <c r="M50" t="inlineStr"/>
-      <c r="N50" t="inlineStr"/>
-      <c r="O50" t="inlineStr"/>
-      <c r="P50" t="inlineStr"/>
-      <c r="Q50" t="inlineStr"/>
       <c r="R50">
         <f>COUNTIF(C50:Q50,"✓")</f>
         <v/>
@@ -10722,25 +10082,11 @@
           <t>Registro de nutrición</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr"/>
-      <c r="D51" t="inlineStr"/>
-      <c r="E51" t="inlineStr"/>
-      <c r="F51" t="inlineStr"/>
-      <c r="G51" t="inlineStr"/>
-      <c r="H51" t="inlineStr"/>
-      <c r="I51" t="inlineStr"/>
-      <c r="J51" t="inlineStr"/>
       <c r="K51" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="L51" t="inlineStr"/>
-      <c r="M51" t="inlineStr"/>
-      <c r="N51" t="inlineStr"/>
-      <c r="O51" t="inlineStr"/>
-      <c r="P51" t="inlineStr"/>
-      <c r="Q51" t="inlineStr"/>
       <c r="R51">
         <f>COUNTIF(C51:Q51,"✓")</f>
         <v/>
@@ -10757,25 +10103,11 @@
           <t>Seguimiento de salud femenina</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr"/>
-      <c r="D52" t="inlineStr"/>
-      <c r="E52" t="inlineStr"/>
-      <c r="F52" t="inlineStr"/>
-      <c r="G52" t="inlineStr"/>
-      <c r="H52" t="inlineStr"/>
-      <c r="I52" t="inlineStr"/>
-      <c r="J52" t="inlineStr"/>
       <c r="K52" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="L52" t="inlineStr"/>
-      <c r="M52" t="inlineStr"/>
-      <c r="N52" t="inlineStr"/>
-      <c r="O52" t="inlineStr"/>
-      <c r="P52" t="inlineStr"/>
-      <c r="Q52" t="inlineStr"/>
       <c r="R52">
         <f>COUNTIF(C52:Q52,"✓")</f>
         <v/>
@@ -10792,25 +10124,11 @@
           <t>Valoración de profesionales</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr"/>
-      <c r="D53" t="inlineStr"/>
-      <c r="E53" t="inlineStr"/>
       <c r="F53" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="G53" t="inlineStr"/>
-      <c r="H53" t="inlineStr"/>
-      <c r="I53" t="inlineStr"/>
-      <c r="J53" t="inlineStr"/>
-      <c r="K53" t="inlineStr"/>
-      <c r="L53" t="inlineStr"/>
-      <c r="M53" t="inlineStr"/>
-      <c r="N53" t="inlineStr"/>
-      <c r="O53" t="inlineStr"/>
-      <c r="P53" t="inlineStr"/>
-      <c r="Q53" t="inlineStr"/>
       <c r="R53">
         <f>COUNTIF(C53:Q53,"✓")</f>
         <v/>
@@ -10827,25 +10145,11 @@
           <t>Acceso mínimo por categorías de datos</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr"/>
-      <c r="D54" t="inlineStr"/>
-      <c r="E54" t="inlineStr"/>
-      <c r="F54" t="inlineStr"/>
-      <c r="G54" t="inlineStr"/>
-      <c r="H54" t="inlineStr"/>
-      <c r="I54" t="inlineStr"/>
-      <c r="J54" t="inlineStr"/>
-      <c r="K54" t="inlineStr"/>
-      <c r="L54" t="inlineStr"/>
       <c r="M54" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="N54" t="inlineStr"/>
-      <c r="O54" t="inlineStr"/>
-      <c r="P54" t="inlineStr"/>
-      <c r="Q54" t="inlineStr"/>
       <c r="R54">
         <f>COUNTIF(C54:Q54,"✓")</f>
         <v/>
@@ -10862,11 +10166,6 @@
           <t>Blockchain para integridad y trazabilidad de datos</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr"/>
-      <c r="D55" t="inlineStr"/>
-      <c r="E55" t="inlineStr"/>
-      <c r="F55" t="inlineStr"/>
-      <c r="G55" t="inlineStr"/>
       <c r="H55" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10882,13 +10181,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="K55" t="inlineStr"/>
-      <c r="L55" t="inlineStr"/>
-      <c r="M55" t="inlineStr"/>
-      <c r="N55" t="inlineStr"/>
-      <c r="O55" t="inlineStr"/>
-      <c r="P55" t="inlineStr"/>
-      <c r="Q55" t="inlineStr"/>
       <c r="R55">
         <f>COUNTIF(C55:Q55,"✓")</f>
         <v/>
@@ -10905,29 +10197,16 @@
           <t>Cifrado y control de acceso</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr"/>
       <c r="D56" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="E56" t="inlineStr"/>
-      <c r="F56" t="inlineStr"/>
-      <c r="G56" t="inlineStr"/>
-      <c r="H56" t="inlineStr"/>
-      <c r="I56" t="inlineStr"/>
-      <c r="J56" t="inlineStr"/>
       <c r="K56" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="L56" t="inlineStr"/>
-      <c r="M56" t="inlineStr"/>
-      <c r="N56" t="inlineStr"/>
-      <c r="O56" t="inlineStr"/>
-      <c r="P56" t="inlineStr"/>
-      <c r="Q56" t="inlineStr"/>
       <c r="R56">
         <f>COUNTIF(C56:Q56,"✓")</f>
         <v/>
@@ -10944,25 +10223,11 @@
           <t>Cumplimiento regulatorio de salud y datos</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr"/>
-      <c r="D57" t="inlineStr"/>
-      <c r="E57" t="inlineStr"/>
-      <c r="F57" t="inlineStr"/>
-      <c r="G57" t="inlineStr"/>
-      <c r="H57" t="inlineStr"/>
-      <c r="I57" t="inlineStr"/>
-      <c r="J57" t="inlineStr"/>
-      <c r="K57" t="inlineStr"/>
-      <c r="L57" t="inlineStr"/>
-      <c r="M57" t="inlineStr"/>
-      <c r="N57" t="inlineStr"/>
       <c r="O57" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="P57" t="inlineStr"/>
-      <c r="Q57" t="inlineStr"/>
       <c r="R57">
         <f>COUNTIF(C57:Q57,"✓")</f>
         <v/>
@@ -10979,25 +10244,11 @@
           <t>Gestión de consentimiento sobre uso de datos</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr"/>
-      <c r="D58" t="inlineStr"/>
-      <c r="E58" t="inlineStr"/>
-      <c r="F58" t="inlineStr"/>
-      <c r="G58" t="inlineStr"/>
-      <c r="H58" t="inlineStr"/>
-      <c r="I58" t="inlineStr"/>
-      <c r="J58" t="inlineStr"/>
-      <c r="K58" t="inlineStr"/>
       <c r="L58" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="M58" t="inlineStr"/>
-      <c r="N58" t="inlineStr"/>
-      <c r="O58" t="inlineStr"/>
-      <c r="P58" t="inlineStr"/>
-      <c r="Q58" t="inlineStr"/>
       <c r="R58">
         <f>COUNTIF(C58:Q58,"✓")</f>
         <v/>
@@ -11014,25 +10265,11 @@
           <t>Identidad descentralizada (DID)</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr"/>
-      <c r="D59" t="inlineStr"/>
-      <c r="E59" t="inlineStr"/>
-      <c r="F59" t="inlineStr"/>
-      <c r="G59" t="inlineStr"/>
-      <c r="H59" t="inlineStr"/>
       <c r="I59" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="J59" t="inlineStr"/>
-      <c r="K59" t="inlineStr"/>
-      <c r="L59" t="inlineStr"/>
-      <c r="M59" t="inlineStr"/>
-      <c r="N59" t="inlineStr"/>
-      <c r="O59" t="inlineStr"/>
-      <c r="P59" t="inlineStr"/>
-      <c r="Q59" t="inlineStr"/>
       <c r="R59">
         <f>COUNTIF(C59:Q59,"✓")</f>
         <v/>
@@ -11049,15 +10286,6 @@
           <t>Privacidad reforzada para datos de salud</t>
         </is>
       </c>
-      <c r="C60" t="inlineStr"/>
-      <c r="D60" t="inlineStr"/>
-      <c r="E60" t="inlineStr"/>
-      <c r="F60" t="inlineStr"/>
-      <c r="G60" t="inlineStr"/>
-      <c r="H60" t="inlineStr"/>
-      <c r="I60" t="inlineStr"/>
-      <c r="J60" t="inlineStr"/>
-      <c r="K60" t="inlineStr"/>
       <c r="L60" t="inlineStr">
         <is>
           <t>✓</t>
@@ -11068,10 +10296,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="N60" t="inlineStr"/>
-      <c r="O60" t="inlineStr"/>
-      <c r="P60" t="inlineStr"/>
-      <c r="Q60" t="inlineStr"/>
       <c r="R60">
         <f>COUNTIF(C60:Q60,"✓")</f>
         <v/>
@@ -11088,20 +10312,6 @@
           <t>Modelo freemium y suscripción</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr"/>
-      <c r="D61" t="inlineStr"/>
-      <c r="E61" t="inlineStr"/>
-      <c r="F61" t="inlineStr"/>
-      <c r="G61" t="inlineStr"/>
-      <c r="H61" t="inlineStr"/>
-      <c r="I61" t="inlineStr"/>
-      <c r="J61" t="inlineStr"/>
-      <c r="K61" t="inlineStr"/>
-      <c r="L61" t="inlineStr"/>
-      <c r="M61" t="inlineStr"/>
-      <c r="N61" t="inlineStr"/>
-      <c r="O61" t="inlineStr"/>
-      <c r="P61" t="inlineStr"/>
       <c r="Q61" t="inlineStr">
         <is>
           <t>✓</t>
@@ -11123,25 +10333,11 @@
           <t>Pagos con criptomoneda</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr"/>
-      <c r="D62" t="inlineStr"/>
-      <c r="E62" t="inlineStr"/>
-      <c r="F62" t="inlineStr"/>
-      <c r="G62" t="inlineStr"/>
-      <c r="H62" t="inlineStr"/>
-      <c r="I62" t="inlineStr"/>
       <c r="J62" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="K62" t="inlineStr"/>
-      <c r="L62" t="inlineStr"/>
-      <c r="M62" t="inlineStr"/>
-      <c r="N62" t="inlineStr"/>
-      <c r="O62" t="inlineStr"/>
-      <c r="P62" t="inlineStr"/>
-      <c r="Q62" t="inlineStr"/>
       <c r="R62">
         <f>COUNTIF(C62:Q62,"✓")</f>
         <v/>
@@ -11158,20 +10354,6 @@
           <t>Pagos dentro de la app</t>
         </is>
       </c>
-      <c r="C63" t="inlineStr"/>
-      <c r="D63" t="inlineStr"/>
-      <c r="E63" t="inlineStr"/>
-      <c r="F63" t="inlineStr"/>
-      <c r="G63" t="inlineStr"/>
-      <c r="H63" t="inlineStr"/>
-      <c r="I63" t="inlineStr"/>
-      <c r="J63" t="inlineStr"/>
-      <c r="K63" t="inlineStr"/>
-      <c r="L63" t="inlineStr"/>
-      <c r="M63" t="inlineStr"/>
-      <c r="N63" t="inlineStr"/>
-      <c r="O63" t="inlineStr"/>
-      <c r="P63" t="inlineStr"/>
       <c r="Q63" t="inlineStr">
         <is>
           <t>✓</t>
@@ -11193,25 +10375,11 @@
           <t>Reclamos y trámites con seguros</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr"/>
-      <c r="D64" t="inlineStr"/>
-      <c r="E64" t="inlineStr"/>
-      <c r="F64" t="inlineStr"/>
-      <c r="G64" t="inlineStr"/>
-      <c r="H64" t="inlineStr"/>
       <c r="I64" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="J64" t="inlineStr"/>
-      <c r="K64" t="inlineStr"/>
-      <c r="L64" t="inlineStr"/>
-      <c r="M64" t="inlineStr"/>
-      <c r="N64" t="inlineStr"/>
-      <c r="O64" t="inlineStr"/>
-      <c r="P64" t="inlineStr"/>
-      <c r="Q64" t="inlineStr"/>
       <c r="R64">
         <f>COUNTIF(C64:Q64,"✓")</f>
         <v/>
@@ -11228,25 +10396,11 @@
           <t>Teleconsulta con profesionales</t>
         </is>
       </c>
-      <c r="C65" t="inlineStr"/>
-      <c r="D65" t="inlineStr"/>
-      <c r="E65" t="inlineStr"/>
-      <c r="F65" t="inlineStr"/>
-      <c r="G65" t="inlineStr"/>
-      <c r="H65" t="inlineStr"/>
-      <c r="I65" t="inlineStr"/>
       <c r="J65" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="K65" t="inlineStr"/>
-      <c r="L65" t="inlineStr"/>
-      <c r="M65" t="inlineStr"/>
-      <c r="N65" t="inlineStr"/>
-      <c r="O65" t="inlineStr"/>
-      <c r="P65" t="inlineStr"/>
-      <c r="Q65" t="inlineStr"/>
       <c r="R65">
         <f>COUNTIF(C65:Q65,"✓")</f>
         <v/>
@@ -11263,7 +10417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A25"/>
+  <dimension ref="A1:A26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -11444,6 +10598,13 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Vuelta 6 (iter. 1, 2026-10-13 12:16 UTC): Meedika, Infomed, MediPlanner, Clingot verificados (+0 filas; fuentes casi agotadas). Pendientes: Healfies, Patientory, MediBloc, Medicalchain, Apple Health, ChatGPT Health, Claude for Healthcare, Apps de clínicas, Clinia, MiRedSalud, Mediko.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Benchmark: vuelta 6, iteración 2 (Healfies, Patientory, MediBloc, Medicalchain)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MVcXu8vTBu7EKfj3YdEvae
</commit_message>
<xml_diff>
--- a/Outputs/Benchmark_Anamnesis.xlsx
+++ b/Outputs/Benchmark_Anamnesis.xlsx
@@ -673,12 +673,12 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>[REGIONAL · Brasil] Fundada ene-2015 en Florianópolis por Helyson Lewis Velasco. Centraliza registros de salud personales: carpetas, etiquetas, línea de tiempo (medicación, exámenes, citas, dieta), compartir con familia o profesionales. Gratis; web, iOS y Android. Estado actual NO verificado (fuentes de 2015-2016). Referencia funcional cercana a etapas A+B. [Vuelta 2] Lanzada simultáneamente en Brasil, Argentina y EE.UU.; permite compartir con no registrados vía clave por email. Sin novedades posteriores a 2016. [Vuelta 3] Sin evidencia de actividad reciente ni de cierre; Gust/Dealroom la listan en Florianópolis (10 empleados, healfies.com) sin fecha de actualización. Estado sin confirmar. [Vuelta 4] Sin Google Play localizado; no confundir con la app Healfy (otro producto). Sin novedades. [Vuelta 5] Sin búsqueda nueva (revisada en vuelta 4); sin cambios.</t>
+          <t>[REGIONAL · Brasil] Fundada ene-2015 en Florianópolis por Helyson Lewis Velasco. Centraliza registros de salud personales: carpetas, etiquetas, línea de tiempo (medicación, exámenes, citas, dieta), compartir con familia o profesionales. Gratis; web, iOS y Android. Estado actual NO verificado (fuentes de 2015-2016). Referencia funcional cercana a etapas A+B. [Vuelta 2] Lanzada simultáneamente en Brasil, Argentina y EE.UU.; permite compartir con no registrados vía clave por email. Sin novedades posteriores a 2016. [Vuelta 3] Sin evidencia de actividad reciente ni de cierre; Gust/Dealroom la listan en Florianópolis (10 empleados, healfies.com) sin fecha de actualización. Estado sin confirmar. [Vuelta 4] Sin Google Play localizado; no confundir con la app Healfy (otro producto). Sin novedades. [Vuelta 5] Sin búsqueda nueva (revisada en vuelta 4); sin cambios. [Vuelta 6] Sin búsqueda nueva (fuentes agotadas); sin cambios.</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G6" t="n">
@@ -686,7 +686,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -713,12 +713,12 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>[BLOCKCHAIN · EE.UU.] Atlanta, fundada 2015, ~9 empleados. Levantó US$7,2M vía financiamiento cripto. App con registros de hospitales y wearables, coaching de salud con IA y recompensas en cripto; también dashboard empresarial Neith. PitchBook indica actividad y financiamiento hasta abr-2026: sigue operando. Sin presencia conocida en Chile. Referencia directa para la hipótesis blockchain. [Vuelta 2] Sin noticias 2026 encontradas en búsqueda; sitio oficial bloqueado. [Vuelta 3] Búsqueda adicional solo devuelve hitos de 2017 (token sale US$7,2M) y 2019 (Serie A de US$5,3M, cierre no confirmado); sin datos 2025-26 propios. [Vuelta 4] App pública lanzada en la conferencia JP Morgan Healthcare (2019); red PTOYMatrix (blockchain HIPAA); socios reportados: StartUp Health y Kaiser Permanente (beta). Estado actual en App Store/Google Play sin confirmar. [Vuelta 5] Sin noticias 2026 del equipo. Token PTOY con capitalización de ~US$53K a fines de ago-2026 según Phantom (KuCoin discrepa en la circulación): señal de baja actividad, no prueba de cierre. Esto relativiza la actividad hasta abr-2026 mencionada en la ficha original.</t>
+          <t>[BLOCKCHAIN · EE.UU.] Atlanta, fundada 2015, ~9 empleados. Levantó US$7,2M vía financiamiento cripto. App con registros de hospitales y wearables, coaching de salud con IA y recompensas en cripto; también dashboard empresarial Neith. PitchBook indica actividad y financiamiento hasta abr-2026: sigue operando. Sin presencia conocida en Chile. Referencia directa para la hipótesis blockchain. [Vuelta 2] Sin noticias 2026 encontradas en búsqueda; sitio oficial bloqueado. [Vuelta 3] Búsqueda adicional solo devuelve hitos de 2017 (token sale US$7,2M) y 2019 (Serie A de US$5,3M, cierre no confirmado); sin datos 2025-26 propios. [Vuelta 4] App pública lanzada en la conferencia JP Morgan Healthcare (2019); red PTOYMatrix (blockchain HIPAA); socios reportados: StartUp Health y Kaiser Permanente (beta). Estado actual en App Store/Google Play sin confirmar. [Vuelta 5] Sin noticias 2026 del equipo. Token PTOY con capitalización de ~US$53K a fines de ago-2026 según Phantom (KuCoin discrepa en la circulación): señal de baja actividad, no prueba de cierre. Esto relativiza la actividad hasta abr-2026 mencionada en la ficha original. [Vuelta 6] Sin noticias posteriores a 2020 localizadas (hitos: token sale 2017, consorcio Hyperledger, alianza con Georgia State, Series A de US$5,3M vía R/GA Ventures, Neith con Prosper Healthtech en Birmingham). Estado actual desconocido.</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G7" t="n">
@@ -726,7 +726,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -753,12 +753,12 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>[BLOCKCHAIN · Corea del Sur] Fundada 2017, Seúl. Blockchain propia Panacea (Cosmos SDK, mainnet 2019) para que el paciente gestione y transfiera sus registros; app Medipass para seguros. Serie A de ₩4.000 millones (Naver); alianzas con hospitales (Seoul National, Severance). Estado 2025-26 NO verificado. Referencia sobre seguros + blockchain. [Vuelta 2] Panacea incluye DID, Append Only Log, IBC y PNFT; sin anuncios 2026 localizados. [Vuelta 3] Medipass: app en Corea con 20 hospitales/aseguradoras integrados (fecha de la lista desconocida) y plan 2022 de superapp con marketplace de datos; operación actual sin confirmar. [Vuelta 4] Sin búsqueda nueva (revisada en vuelta 3); sin cambios. [Vuelta 5] Medipass: ~400.000 usuarios acumulados (CEO, jun-2022); integración con aseguradoras Shinhan Life, Samsung Fire y Hyundai Marine (2020); renovación completa en mar-2023 (dashboard de salud, gestión familiar, certificados). Sin noticias 2026 encontradas.</t>
+          <t>[BLOCKCHAIN · Corea del Sur] Fundada 2017, Seúl. Blockchain propia Panacea (Cosmos SDK, mainnet 2019) para que el paciente gestione y transfiera sus registros; app Medipass para seguros. Serie A de ₩4.000 millones (Naver); alianzas con hospitales (Seoul National, Severance). Estado 2025-26 NO verificado. Referencia sobre seguros + blockchain. [Vuelta 2] Panacea incluye DID, Append Only Log, IBC y PNFT; sin anuncios 2026 localizados. [Vuelta 3] Medipass: app en Corea con 20 hospitales/aseguradoras integrados (fecha de la lista desconocida) y plan 2022 de superapp con marketplace de datos; operación actual sin confirmar. [Vuelta 4] Sin búsqueda nueva (revisada en vuelta 3); sin cambios. [Vuelta 5] Medipass: ~400.000 usuarios acumulados (CEO, jun-2022); integración con aseguradoras Shinhan Life, Samsung Fire y Hyundai Marine (2020); renovación completa en mar-2023 (dashboard de salud, gestión familiar, certificados). Sin noticias 2026 encontradas. [Vuelta 6] Medipass 2023: comunicación bidireccional hospital-paciente y chat MediTalk; en 2019 fue seleccionada para el programa gubernamental de MyData médico con Samsung Fire y SNUH. Sin estrategia 2026 localizada. Meta declarada: usar Medipass como «identificación» de salud.</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G8" t="n">
@@ -766,7 +766,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -793,12 +793,12 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>[BLOCKCHAIN · Reino Unido · INACTIVO] Londres, 2017, Ethereum, con telemedicina. Piloto según registro de la UE (2020). Tracxn/PitchBook lo marcan fuera de operación (ago-2025). Solo caso de aprendizaje: no cuenta como competidor activo. [Vuelta 2] Token MTN deslistado de Bitfinex el 26-mar-2021; sin hallazgos de actividad posterior. [Vuelta 3] Seedtable la marca activa sin fuente; no hallé registro en Companies House. Sigue tratándose como caso de aprendizaje. [Vuelta 4] Pre-venta reportada de US$20M en MedTokens (un solo artículo secundario, sin verificar); modelo de token en revisión y exploración de security token según AMA; integraciones y servicios de 2019 sin confirmar. [Vuelta 5] Un agregador indica sitio medicalchain.com fuera de línea desde 15-feb-2025, último commit en GitHub hace ~3 años y proyecto en «fase de mantenimiento»; preventa de MedTokens reportada entre US$20M y US$24M (fuentes discrepan). Confirma tratarlo como inactivo.</t>
+          <t>[BLOCKCHAIN · Reino Unido · INACTIVO] Londres, 2017, Ethereum, con telemedicina. Piloto según registro de la UE (2020). Tracxn/PitchBook lo marcan fuera de operación (ago-2025). Solo caso de aprendizaje: no cuenta como competidor activo. [Vuelta 2] Token MTN deslistado de Bitfinex el 26-mar-2021; sin hallazgos de actividad posterior. [Vuelta 3] Seedtable la marca activa sin fuente; no hallé registro en Companies House. Sigue tratándose como caso de aprendizaje. [Vuelta 4] Pre-venta reportada de US$20M en MedTokens (un solo artículo secundario, sin verificar); modelo de token en revisión y exploración de security token según AMA; integraciones y servicios de 2019 sin confirmar. [Vuelta 5] Un agregador indica sitio medicalchain.com fuera de línea desde 15-feb-2025, último commit en GitHub hace ~3 años y proyecto en «fase de mantenimiento»; preventa de MedTokens reportada entre US$20M y US$24M (fuentes discrepan). Confirma tratarlo como inactivo. [Vuelta 6] Sin búsqueda nueva (revisada en vuelta 5; sitio fuera de línea desde feb-2025 según un agregador); sin cambios.</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G9" t="n">
@@ -806,7 +806,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -1102,7 +1102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F128"/>
+  <dimension ref="A1:F130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -5206,6 +5206,70 @@
       <c r="F128" t="inlineStr">
         <is>
           <t>Búsqueda web (Unite.ai, Fortune, TechStrong); solo EE.UU., Pro/Max</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>MediBloc</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>Telemedicina y atención remota</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>Chat con hospitales (MediTalk)</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>Chat para consultas a hospitales, orientación simple de síntomas e información de tratamientos; comunicación bidireccional hospital-paciente (nov-2023).</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>Búsqueda web (Medigate News, nov-2023)</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>MediBloc</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Citas y agenda</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Reserva de citas en hospitales</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>Reserva de citas en hospitales integrados, dentro de Medipass.</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>Búsqueda web (ficha App Store Corea, notas de prensa)</t>
         </is>
       </c>
     </row>
@@ -10417,7 +10481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A26"/>
+  <dimension ref="A1:A27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -10605,6 +10669,13 @@
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Vuelta 6 (iter. 2, 2026-10-14 12:15 UTC): Healfies, Patientory, MediBloc, Medicalchain verificados (+2 filas, de MediBloc). Pendientes: Apple Health, ChatGPT Health, Claude for Healthcare, Apps de clínicas, Clinia, MiRedSalud, Mediko.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Benchmark: vuelta 6, iteración 3 (Apple Health, ChatGPT Health, Claude for Healthcare, Apps de clínicas)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MVcXu8vTBu7EKfj3YdEvae
</commit_message>
<xml_diff>
--- a/Outputs/Benchmark_Anamnesis.xlsx
+++ b/Outputs/Benchmark_Anamnesis.xlsx
@@ -833,12 +833,12 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>[ADYACENTE · global] Agrega registros clínicos vía FHIR; &gt;500 instituciones conectadas en EE.UU. (2018). Sin evidencia de disponibilidad en Chile. Incluida en el dispositivo. Amenaza si FHIR/IPS-CL se adopta en Chile. [Vuelta 2] Sin disponibilidad de registros clínicos en Chile (solo EE.UU., Reino Unido, Canadá). [Vuelta 3] iOS 27 (WWDC 8-jun-2026; publicado ~14-sep-2026): rediseño del app Health, menopausia, nutrición por cámara. El coach de salud con IA no se anunció. Sin ampliación de Health Records a Chile. [Vuelta 4] Sin búsqueda nueva (revisada en vuelta 3); sin cambios. [Vuelta 5] Sin ampliación de Health Records a Australia, Europa ni Latinoamérica (solo EE.UU., UK, Canadá). Funciones de dispositivo (apnea del sueño, prueba auditiva) sí se amplían a países latinoamericanos, pero no son registros clínicos.</t>
+          <t>[ADYACENTE · global] Agrega registros clínicos vía FHIR; &gt;500 instituciones conectadas en EE.UU. (2018). Sin evidencia de disponibilidad en Chile. Incluida en el dispositivo. Amenaza si FHIR/IPS-CL se adopta en Chile. [Vuelta 2] Sin disponibilidad de registros clínicos en Chile (solo EE.UU., Reino Unido, Canadá). [Vuelta 3] iOS 27 (WWDC 8-jun-2026; publicado ~14-sep-2026): rediseño del app Health, menopausia, nutrición por cámara. El coach de salud con IA no se anunció. Sin ampliación de Health Records a Chile. [Vuelta 4] Sin búsqueda nueva (revisada en vuelta 3); sin cambios. [Vuelta 5] Sin ampliación de Health Records a Australia, Europa ni Latinoamérica (solo EE.UU., UK, Canadá). Funciones de dispositivo (apnea del sueño, prueba auditiva) sí se amplían a países latinoamericanos, pero no son registros clínicos. [Vuelta 6] Sin novedades de iOS 27.x localizadas. Health Records API permite compartir registros con apps de terceros con control por app; opción de enviar datos de uso a Apple.</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G10" t="n">
@@ -846,7 +846,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -873,12 +873,12 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>[ADYACENTE · global] Lanzado 7-ene-2026. Conecta registros médicos; conectores solo en EE.UU. Dentro de suscripción del asistente. Fija la expectativa de consultar y resumir el historial. [Vuelta 2] Confirmado: registros solo EE.UU.; sin anuncios para Latinoamérica. Hay inconsistencia de fechas entre fuentes (7-ene-2026 lanzamiento vs. jul-2026 despliegue de registros). [Vuelta 3] Fechas aclaradas: presentación 7-ene-2026 (acceso limitado); despliegue de Health in ChatGPT con Apple Health y registros en EE.UU. el 23-jul-2026; mejora de salud jun-2026. Sin anuncios para Latinoamérica ni para sep-oct 2026. [Vuelta 4] Septiembre 2026: permisos por defecto para datos conectados (14-sep) y explicaciones por gráfico/métrica (28-sep); ChatGPT for Clinicians (abr-2026) para clínicos verificados de EE.UU. Más del 70% de usuarios de Health permite usar datos conectados sin pedir permiso (según OpenAI). Sigue solo EE.UU. [Vuelta 5] Nota de jul-2026: Health no está disponible en México, Android, modo de voz ni Codex; web e iOS en EE.UU., adultos con sesión iniciada. Sin anuncio para Chile ni Latinoamérica.</t>
+          <t>[ADYACENTE · global] Lanzado 7-ene-2026. Conecta registros médicos; conectores solo en EE.UU. Dentro de suscripción del asistente. Fija la expectativa de consultar y resumir el historial. [Vuelta 2] Confirmado: registros solo EE.UU.; sin anuncios para Latinoamérica. Hay inconsistencia de fechas entre fuentes (7-ene-2026 lanzamiento vs. jul-2026 despliegue de registros). [Vuelta 3] Fechas aclaradas: presentación 7-ene-2026 (acceso limitado); despliegue de Health in ChatGPT con Apple Health y registros en EE.UU. el 23-jul-2026; mejora de salud jun-2026. Sin anuncios para Latinoamérica ni para sep-oct 2026. [Vuelta 4] Septiembre 2026: permisos por defecto para datos conectados (14-sep) y explicaciones por gráfico/métrica (28-sep); ChatGPT for Clinicians (abr-2026) para clínicos verificados de EE.UU. Más del 70% de usuarios de Health permite usar datos conectados sin pedir permiso (según OpenAI). Sigue solo EE.UU. [Vuelta 5] Nota de jul-2026: Health no está disponible en México, Android, modo de voz ni Codex; web e iOS en EE.UU., adultos con sesión iniciada. Sin anuncio para Chile ni Latinoamérica. [Vuelta 6] Última entrada de Health en las notas de OpenAI sigue siendo la del 23-jul-2026 (más cambios de sep); sin entradas de octubre localizadas. Health tab: laboratorios, medicamentos, actividad y sueño en una vista; solo EE.UU., web e iOS.</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G11" t="n">
@@ -886,7 +886,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -913,12 +913,12 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>[ADYACENTE · global] Lanzado 11-ene-2026. Conectores solo en EE.UU., planes Pro/Max. Nota: producto de Anthropic, conflicto de interés al evaluarlo. [Vuelta 2] Sin cambios fuera de EE.UU. (HealthEx y Function para Pro/Max). [Vuelta 3] Sin anuncios posteriores a enero de 2026. Hoja de ruta de HealthEx (agendar, buscar prestadores, recetas) sin confirmar como lanzada. [Vuelta 4] Sin anuncios nuevos. Fuentes discrepan en el acceso (Pro/Max según Fortune y la mayoría; Pro/Team según Times of AI); sin evidencia de disponibilidad fuera de EE.UU. [Vuelta 5] Sin noticias de oct-2026; HealthEx agrega datos de &gt;50.000 sistemas de EE.UU. y Claude pide solo las categorías relevantes vía MCP.</t>
+          <t>[ADYACENTE · global] Lanzado 11-ene-2026. Conectores solo en EE.UU., planes Pro/Max. Nota: producto de Anthropic, conflicto de interés al evaluarlo. [Vuelta 2] Sin cambios fuera de EE.UU. (HealthEx y Function para Pro/Max). [Vuelta 3] Sin anuncios posteriores a enero de 2026. Hoja de ruta de HealthEx (agendar, buscar prestadores, recetas) sin confirmar como lanzada. [Vuelta 4] Sin anuncios nuevos. Fuentes discrepan en el acceso (Pro/Max según Fortune y la mayoría; Pro/Team según Times of AI); sin evidencia de disponibilidad fuera de EE.UU. [Vuelta 5] Sin noticias de oct-2026; HealthEx agrega datos de &gt;50.000 sistemas de EE.UU. y Claude pide solo las categorías relevantes vía MCP. [Vuelta 6] Sin noticias posteriores a enero de 2026 localizadas.</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G12" t="n">
@@ -926,7 +926,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -953,12 +953,12 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>[SUSTITUTO PARCIAL · Chile] Reservar hora, ver historial de esa institución, vincular familiar. Gratis; no consolida datos de otras instituciones. [Vuelta 2] App concreta: Mi Alemana Go (Clínica Alemana, Chile), con historial desde 2018, recetas, órdenes, familiar vinculado y resultados. [Vuelta 3] Búsqueda de otras clínicas (Las Condes, Santa María, UC Christus) sin ficha de app confirmada; solo canales digitales genéricos. [Vuelta 4] Mi Alemana Go: 3,1/5 con 137 calificaciones (App Store Chile), pantalla de inicio rediseñada para gestionar salud propia y familiar; sin evidencia de teleconsulta ni pagos en la app. [Vuelta 5] Sin búsqueda nueva (revisada en vuelta 4); sin cambios.</t>
+          <t>[SUSTITUTO PARCIAL · Chile] Reservar hora, ver historial de esa institución, vincular familiar. Gratis; no consolida datos de otras instituciones. [Vuelta 2] App concreta: Mi Alemana Go (Clínica Alemana, Chile), con historial desde 2018, recetas, órdenes, familiar vinculado y resultados. [Vuelta 3] Búsqueda de otras clínicas (Las Condes, Santa María, UC Christus) sin ficha de app confirmada; solo canales digitales genéricos. [Vuelta 4] Mi Alemana Go: 3,1/5 con 137 calificaciones (App Store Chile), pantalla de inicio rediseñada para gestionar salud propia y familiar; sin evidencia de teleconsulta ni pagos en la app. [Vuelta 5] Sin búsqueda nueva (revisada en vuelta 4); sin cambios. [Vuelta 6] Sin búsqueda nueva; sin cambios.</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G13" t="n">
@@ -966,7 +966,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -1102,7 +1102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F130"/>
+  <dimension ref="A1:F131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -5270,6 +5270,38 @@
       <c r="F130" t="inlineStr">
         <is>
           <t>Búsqueda web (ficha App Store Corea, notas de prensa)</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>Apple Health (Health Records)</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Interoperabilidad y fuentes de datos</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>API de Health Records para apps de terceros</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>El usuario decide qué registros recibe cada app y si los nuevos se comparten automáticamente (por defecto pide permiso cada vez); ej. importar recetas a Medisafe.</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>Búsqueda web (Apple, TechCrunch, Pharmaphorum); registros solo EE.UU./UK/Canadá</t>
         </is>
       </c>
     </row>
@@ -10481,7 +10513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A27"/>
+  <dimension ref="A1:A28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -10676,6 +10708,13 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Vuelta 6 (iter. 3, 2026-10-15 12:15 UTC): Apple Health, ChatGPT Health, Claude for Healthcare, Apps de clínicas verificados (+1 fila). Pendientes: Clinia, MiRedSalud, Mediko (cierran la vuelta 6 y regeneran func_norm/tabla_frecuencia).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Benchmark: vuelta 7, iteración 1 (Meedika, Infomed, MediPlanner, Clingot)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MVcXu8vTBu7EKfj3YdEvae
</commit_message>
<xml_diff>
--- a/Outputs/Benchmark_Anamnesis.xlsx
+++ b/Outputs/Benchmark_Anamnesis.xlsx
@@ -513,12 +513,12 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>[DIRECTO · Chile · etapas A+B] Lanzada 25-sep-2024 en App Store (Android previsto la misma semana). &gt;1.500 usuarios en los primeros días; meta 32.000 (cofundador Francisco González). Funciones: gestión de documentos, importar solicitudes, SOS con alergias/medicación, calendario de citas, recordatorios, compartir con profesionales elegidos. Sin blockchain. Precio y estado actual NO verificados; única fuente es una nota de prensa. Sitio oficial por confirmar. [Iter. 2] Hay cobertura adicional en Portal Innova (portalinnova.cl); sitio bloqueado en este entorno, estado actual sigue sin verificar. [Vuelta 3] Sin novedades 2026 ni confirmación de la app Android en Google Play; usuarios actuales desconocidos. Nota de prensa no indica año de lanzamiento explícito. [Vuelta 4] Sin fuentes nuevas; portalinnova.cl no aparece en búsquedas. Sigue dependiendo de una sola nota de prensa. [Vuelta 5] Sin fuentes nuevas (ni entrevistas ni financiamiento); sigue dependiendo de una sola nota de prensa sin año explícito. [Vuelta 6] Sin ficha de Google Play ni fuentes nuevas; disponibilidad en Android sin confirmar.</t>
+          <t>[DIRECTO · Chile · etapas A+B] Lanzada 25-sep-2024 en App Store (Android previsto la misma semana). &gt;1.500 usuarios en los primeros días; meta 32.000 (cofundador Francisco González). Funciones: gestión de documentos, importar solicitudes, SOS con alergias/medicación, calendario de citas, recordatorios, compartir con profesionales elegidos. Sin blockchain. Precio y estado actual NO verificados; única fuente es una nota de prensa. Sitio oficial por confirmar. [Iter. 2] Hay cobertura adicional en Portal Innova (portalinnova.cl); sitio bloqueado en este entorno, estado actual sigue sin verificar. [Vuelta 3] Sin novedades 2026 ni confirmación de la app Android en Google Play; usuarios actuales desconocidos. Nota de prensa no indica año de lanzamiento explícito. [Vuelta 4] Sin fuentes nuevas; portalinnova.cl no aparece en búsquedas. Sigue dependiendo de una sola nota de prensa. [Vuelta 5] Sin fuentes nuevas (ni entrevistas ni financiamiento); sigue dependiendo de una sola nota de prensa sin año explícito. [Vuelta 6] Sin ficha de Google Play ni fuentes nuevas; disponibilidad en Android sin confirmar. [Vuelta 7] Sin fuentes nuevas; no hay ficha oficial localizada. No confundir con apps de nombre parecido (Medika App, MEDDI, AI Medik).</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G2" t="n">
@@ -526,7 +526,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -553,12 +553,12 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>[DIRECTO · Chile · etapa A] Fundada 2019 por Diego Ibarra, Andrés Fantuzzi y Gabriel Zamora. Lanzada mar-2021 en App Store y Play Store con 1.200 usuarios; planeaba nueva versión jul-2021 y ronda de US$500 mil. Objetivo: llevar el historial en el celular, acceso en emergencias, médico puede ingresar datos con consentimiento. Estado actual NO verificado (posible app inactiva). URL es la nota de prensa; sitio oficial por confirmar. [Vuelta 3] Sin evidencia posterior a 2021; relanzamiento previsto jul-2021 no confirmado. Probable app inactiva. [Vuelta 4] Sin cambios; sigue sin evidencia posterior a 2021. [Vuelta 5] Cofundador Andrés Fantuzzi es cardiólogo de la Clínica Santa María. Sin ronda de inversión ni relanzamiento confirmados; no confundir con Infomed de Cuba (portal del Minsap). [Vuelta 6] Sin búsqueda nueva (fuentes agotadas en vueltas 3-5); sin cambios.</t>
+          <t>[DIRECTO · Chile · etapa A] Fundada 2019 por Diego Ibarra, Andrés Fantuzzi y Gabriel Zamora. Lanzada mar-2021 en App Store y Play Store con 1.200 usuarios; planeaba nueva versión jul-2021 y ronda de US$500 mil. Objetivo: llevar el historial en el celular, acceso en emergencias, médico puede ingresar datos con consentimiento. Estado actual NO verificado (posible app inactiva). URL es la nota de prensa; sitio oficial por confirmar. [Vuelta 3] Sin evidencia posterior a 2021; relanzamiento previsto jul-2021 no confirmado. Probable app inactiva. [Vuelta 4] Sin cambios; sigue sin evidencia posterior a 2021. [Vuelta 5] Cofundador Andrés Fantuzzi es cardiólogo de la Clínica Santa María. Sin ronda de inversión ni relanzamiento confirmados; no confundir con Infomed de Cuba (portal del Minsap). [Vuelta 6] Sin búsqueda nueva (fuentes agotadas en vueltas 3-5); sin cambios. [Vuelta 7] Sin búsqueda nueva (saturado); sin cambios.</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G3" t="n">
@@ -566,7 +566,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -593,12 +593,12 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>[REGIONAL · México] Historial por perfil familiar, alergias, vacunas, recetas digitales, gráficas de evolución, agendamiento, compartir con profesionales. Gratis en App Store MX. Sin evidencia de uso en Chile. Cubre parte de la etapa C (familia). [Vuelta 3] Existen dos apps distintas: MediPlanner (gratis, Rym Solutions, MX, 3,7/5 con 3 calificaciones) y MediPlanner Pro (otro desarrollador, $39 MXN). Sin presencia verificada en Chile. [Vuelta 4] No pude confirmar el desarrollador de la versión gratuita (Rym Solutions no se repite en esta búsqueda). MediPlanner Pro (fichas BR/OM) guardaría datos solo en el dispositivo, sin nube; no confundir con MedPlanner/AskHEMI (otra empresa). [Vuelta 5] Sin búsqueda nueva (revisada en vuelta 4); sin cambios. [Vuelta 6] Se reconfirma en la ficha de App Store MX que el desarrollador de la versión gratuita es Rym Solutions S. de R.L. de C.V. (3,7/5, 3 calificaciones); MediPlanner Pro no menciona a esa empresa, por lo que no se puede asegurar que sea el mismo desarrollador.</t>
+          <t>[REGIONAL · México] Historial por perfil familiar, alergias, vacunas, recetas digitales, gráficas de evolución, agendamiento, compartir con profesionales. Gratis en App Store MX. Sin evidencia de uso en Chile. Cubre parte de la etapa C (familia). [Vuelta 3] Existen dos apps distintas: MediPlanner (gratis, Rym Solutions, MX, 3,7/5 con 3 calificaciones) y MediPlanner Pro (otro desarrollador, $39 MXN). Sin presencia verificada en Chile. [Vuelta 4] No pude confirmar el desarrollador de la versión gratuita (Rym Solutions no se repite en esta búsqueda). MediPlanner Pro (fichas BR/OM) guardaría datos solo en el dispositivo, sin nube; no confundir con MedPlanner/AskHEMI (otra empresa). [Vuelta 5] Sin búsqueda nueva (revisada en vuelta 4); sin cambios. [Vuelta 6] Se reconfirma en la ficha de App Store MX que el desarrollador de la versión gratuita es Rym Solutions S. de R.L. de C.V. (3,7/5, 3 calificaciones); MediPlanner Pro no menciona a esa empresa, por lo que no se puede asegurar que sea el mismo desarrollador. [Vuelta 7] Sin búsqueda nueva (saturado); sin cambios.</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G4" t="n">
@@ -606,7 +606,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -633,12 +633,12 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>[REGIONAL · Argentina · débil] App para cargar antecedentes médicos propios. Única referencia: nota de opinión en grupoanimal.mx sin fecha verificada. Estado y sitio por confirmar. [Vuelta 3] Referencias de 2017 (apps4citizens, La Nación); sitio y precio no verificados; puede estar inactiva. [Vuelta 4] Sin fuentes nuevas. [Vuelta 5] Registro empresarial (indicadores.ar, datos a jul-2026) muestra CLINGOT S.A. activa en CABA, constituida el 4-abr-2016; no confirma que la app siga operando. Programa federal argentino de historias clínicas digitales como contexto regulatorio. [Vuelta 6] Sin búsqueda nueva (fuentes agotadas); sin cambios.</t>
+          <t>[REGIONAL · Argentina · débil] App para cargar antecedentes médicos propios. Única referencia: nota de opinión en grupoanimal.mx sin fecha verificada. Estado y sitio por confirmar. [Vuelta 3] Referencias de 2017 (apps4citizens, La Nación); sitio y precio no verificados; puede estar inactiva. [Vuelta 4] Sin fuentes nuevas. [Vuelta 5] Registro empresarial (indicadores.ar, datos a jul-2026) muestra CLINGOT S.A. activa en CABA, constituida el 4-abr-2016; no confirma que la app siga operando. Programa federal argentino de historias clínicas digitales como contexto regulatorio. [Vuelta 6] Sin búsqueda nueva (fuentes agotadas); sin cambios. [Vuelta 7] Solo fuentes de 2017; sin evidencia nueva de operación más allá del registro societario.</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G5" t="n">
@@ -646,7 +646,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -9000,8 +9000,6 @@
           <t>Búsqueda de profesionales de salud</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9012,17 +9010,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
       <c r="R2">
         <f>COUNTIF(C2:Q2,"✓")</f>
         <v/>
@@ -9044,24 +9031,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
       <c r="R3">
         <f>COUNTIF(C3:Q3,"✓")</f>
         <v/>
@@ -9078,25 +9052,11 @@
           <t>Integración con calendario del dispositivo</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
       <c r="R4">
         <f>COUNTIF(C4:Q4,"✓")</f>
         <v/>
@@ -9113,25 +9073,11 @@
           <t>Localización de centros médicos y farmacias</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr"/>
       <c r="R5">
         <f>COUNTIF(C5:Q5,"✓")</f>
         <v/>
@@ -9148,21 +9094,11 @@
           <t>Reserva de citas médicas</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9173,8 +9109,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="inlineStr"/>
       <c r="R6">
         <f>COUNTIF(C6:Q6,"✓")</f>
         <v/>
@@ -9191,25 +9125,11 @@
           <t>Acceso del profesional al historial del paciente</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr"/>
-      <c r="Q7" t="inlineStr"/>
       <c r="R7">
         <f>COUNTIF(C7:Q7,"✓")</f>
         <v/>
@@ -9226,25 +9146,11 @@
           <t>Compartir con personas sin cuenta mediante clave segura</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
-      <c r="P8" t="inlineStr"/>
-      <c r="Q8" t="inlineStr"/>
       <c r="R8">
         <f>COUNTIF(C8:Q8,"✓")</f>
         <v/>
@@ -9261,25 +9167,11 @@
           <t>Compartir datos con cuidador o persona de confianza</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
-      <c r="P9" t="inlineStr"/>
-      <c r="Q9" t="inlineStr"/>
       <c r="R9">
         <f>COUNTIF(C9:Q9,"✓")</f>
         <v/>
@@ -9301,13 +9193,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9333,16 +9223,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
       <c r="O10" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="P10" t="inlineStr"/>
-      <c r="Q10" t="inlineStr"/>
       <c r="R10">
         <f>COUNTIF(C10:Q10,"✓")</f>
         <v/>
@@ -9359,25 +9244,11 @@
           <t>Gestión de consentimiento sobre uso de datos</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr"/>
-      <c r="P11" t="inlineStr"/>
-      <c r="Q11" t="inlineStr"/>
       <c r="R11">
         <f>COUNTIF(C11:Q11,"✓")</f>
         <v/>
@@ -9394,25 +9265,11 @@
           <t>Ingreso de datos por profesional con consentimiento</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
-      <c r="O12" t="inlineStr"/>
-      <c r="P12" t="inlineStr"/>
-      <c r="Q12" t="inlineStr"/>
       <c r="R12">
         <f>COUNTIF(C12:Q12,"✓")</f>
         <v/>
@@ -9429,25 +9286,11 @@
           <t>Red social con profesionales y familiares</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr"/>
-      <c r="O13" t="inlineStr"/>
-      <c r="P13" t="inlineStr"/>
-      <c r="Q13" t="inlineStr"/>
       <c r="R13">
         <f>COUNTIF(C13:Q13,"✓")</f>
         <v/>
@@ -9474,23 +9317,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
-      <c r="M14" t="inlineStr"/>
-      <c r="N14" t="inlineStr"/>
-      <c r="O14" t="inlineStr"/>
-      <c r="P14" t="inlineStr"/>
-      <c r="Q14" t="inlineStr"/>
       <c r="R14">
         <f>COUNTIF(C14:Q14,"✓")</f>
         <v/>
@@ -9507,8 +9338,6 @@
           <t>Perfiles familiares / dependientes</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9519,29 +9348,21 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr"/>
       <c r="N15" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="Q15" t="inlineStr"/>
       <c r="R15">
         <f>COUNTIF(C15:Q15,"✓")</f>
         <v/>
@@ -9563,8 +9384,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9580,19 +9399,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
-      <c r="M16" t="inlineStr"/>
-      <c r="N16" t="inlineStr"/>
       <c r="O16" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="P16" t="inlineStr"/>
-      <c r="Q16" t="inlineStr"/>
       <c r="R16">
         <f>COUNTIF(C16:Q16,"✓")</f>
         <v/>
@@ -9609,29 +9420,16 @@
           <t>Almacenamiento de recetas</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr"/>
       <c r="N17" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="O17" t="inlineStr"/>
-      <c r="P17" t="inlineStr"/>
-      <c r="Q17" t="inlineStr"/>
       <c r="R17">
         <f>COUNTIF(C17:Q17,"✓")</f>
         <v/>
@@ -9648,25 +9446,11 @@
           <t>Búsqueda y filtros de documentos</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr"/>
-      <c r="M18" t="inlineStr"/>
-      <c r="N18" t="inlineStr"/>
-      <c r="O18" t="inlineStr"/>
-      <c r="P18" t="inlineStr"/>
-      <c r="Q18" t="inlineStr"/>
       <c r="R18">
         <f>COUNTIF(C18:Q18,"✓")</f>
         <v/>
@@ -9683,25 +9467,11 @@
           <t>Emisión de certificados médicos</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr"/>
-      <c r="M19" t="inlineStr"/>
-      <c r="N19" t="inlineStr"/>
-      <c r="O19" t="inlineStr"/>
-      <c r="P19" t="inlineStr"/>
-      <c r="Q19" t="inlineStr"/>
       <c r="R19">
         <f>COUNTIF(C19:Q19,"✓")</f>
         <v/>
@@ -9723,19 +9493,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr"/>
-      <c r="M20" t="inlineStr"/>
-      <c r="N20" t="inlineStr"/>
-      <c r="O20" t="inlineStr"/>
-      <c r="P20" t="inlineStr"/>
       <c r="Q20" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9757,25 +9514,11 @@
           <t>Notificación y envío de resultados</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr"/>
-      <c r="M21" t="inlineStr"/>
       <c r="N21" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="O21" t="inlineStr"/>
-      <c r="P21" t="inlineStr"/>
-      <c r="Q21" t="inlineStr"/>
       <c r="R21">
         <f>COUNTIF(C21:Q21,"✓")</f>
         <v/>
@@ -9792,29 +9535,16 @@
           <t>Historial institucional (solo datos de la propia red)</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
-      <c r="L22" t="inlineStr"/>
-      <c r="M22" t="inlineStr"/>
       <c r="N22" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="O22" t="inlineStr"/>
       <c r="P22" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="Q22" t="inlineStr"/>
       <c r="R22">
         <f>COUNTIF(C22:Q22,"✓")</f>
         <v/>
@@ -9831,36 +9561,26 @@
           <t>Historial médico centralizado</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="L23" t="inlineStr"/>
-      <c r="M23" t="inlineStr"/>
-      <c r="N23" t="inlineStr"/>
-      <c r="O23" t="inlineStr"/>
-      <c r="P23" t="inlineStr"/>
       <c r="Q23" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9882,25 +9602,11 @@
           <t>Línea de tiempo de salud</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
-      <c r="L24" t="inlineStr"/>
-      <c r="M24" t="inlineStr"/>
-      <c r="N24" t="inlineStr"/>
-      <c r="O24" t="inlineStr"/>
-      <c r="P24" t="inlineStr"/>
-      <c r="Q24" t="inlineStr"/>
       <c r="R24">
         <f>COUNTIF(C24:Q24,"✓")</f>
         <v/>
@@ -9917,25 +9623,11 @@
           <t>Registro de alergias y vacunas</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr"/>
-      <c r="L25" t="inlineStr"/>
-      <c r="M25" t="inlineStr"/>
-      <c r="N25" t="inlineStr"/>
-      <c r="O25" t="inlineStr"/>
-      <c r="P25" t="inlineStr"/>
-      <c r="Q25" t="inlineStr"/>
       <c r="R25">
         <f>COUNTIF(C25:Q25,"✓")</f>
         <v/>
@@ -9952,25 +9644,11 @@
           <t>Seguimiento de visitas, gastos y seguros</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr"/>
-      <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr"/>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
-      <c r="L26" t="inlineStr"/>
-      <c r="M26" t="inlineStr"/>
-      <c r="N26" t="inlineStr"/>
-      <c r="O26" t="inlineStr"/>
-      <c r="P26" t="inlineStr"/>
-      <c r="Q26" t="inlineStr"/>
       <c r="R26">
         <f>COUNTIF(C26:Q26,"✓")</f>
         <v/>
@@ -9987,11 +9665,6 @@
           <t>Recompensas / monetización de datos del usuario</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr"/>
-      <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10007,13 +9680,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="K27" t="inlineStr"/>
-      <c r="L27" t="inlineStr"/>
-      <c r="M27" t="inlineStr"/>
-      <c r="N27" t="inlineStr"/>
-      <c r="O27" t="inlineStr"/>
-      <c r="P27" t="inlineStr"/>
-      <c r="Q27" t="inlineStr"/>
       <c r="R27">
         <f>COUNTIF(C27:Q27,"✓")</f>
         <v/>
@@ -10030,25 +9696,11 @@
           <t>Asistente de IA para profesionales de salud</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="M28" t="inlineStr"/>
-      <c r="N28" t="inlineStr"/>
-      <c r="O28" t="inlineStr"/>
-      <c r="P28" t="inlineStr"/>
-      <c r="Q28" t="inlineStr"/>
       <c r="R28">
         <f>COUNTIF(C28:Q28,"✓")</f>
         <v/>
@@ -10065,25 +9717,11 @@
           <t>Coaching de salud con IA</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr"/>
-      <c r="D29" t="inlineStr"/>
-      <c r="E29" t="inlineStr"/>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr"/>
-      <c r="L29" t="inlineStr"/>
-      <c r="M29" t="inlineStr"/>
-      <c r="N29" t="inlineStr"/>
-      <c r="O29" t="inlineStr"/>
-      <c r="P29" t="inlineStr"/>
-      <c r="Q29" t="inlineStr"/>
       <c r="R29">
         <f>COUNTIF(C29:Q29,"✓")</f>
         <v/>
@@ -10100,15 +9738,6 @@
           <t>Detección de patrones en métricas de salud con IA</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr"/>
-      <c r="E30" t="inlineStr"/>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr"/>
-      <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10119,10 +9748,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="N30" t="inlineStr"/>
-      <c r="O30" t="inlineStr"/>
-      <c r="P30" t="inlineStr"/>
-      <c r="Q30" t="inlineStr"/>
       <c r="R30">
         <f>COUNTIF(C30:Q30,"✓")</f>
         <v/>
@@ -10139,15 +9764,6 @@
           <t>Interpretación de exámenes con IA</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr"/>
-      <c r="D31" t="inlineStr"/>
-      <c r="E31" t="inlineStr"/>
-      <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr"/>
-      <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10158,9 +9774,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="N31" t="inlineStr"/>
-      <c r="O31" t="inlineStr"/>
-      <c r="P31" t="inlineStr"/>
       <c r="Q31" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10182,24 +9795,11 @@
           <t>Orientación médica con IA</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr"/>
-      <c r="D32" t="inlineStr"/>
-      <c r="E32" t="inlineStr"/>
-      <c r="F32" t="inlineStr"/>
-      <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr"/>
-      <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr"/>
-      <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="M32" t="inlineStr"/>
-      <c r="N32" t="inlineStr"/>
-      <c r="O32" t="inlineStr"/>
-      <c r="P32" t="inlineStr"/>
       <c r="Q32" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10221,15 +9821,6 @@
           <t>Preparación de consultas médicas con IA</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr"/>
-      <c r="D33" t="inlineStr"/>
-      <c r="E33" t="inlineStr"/>
-      <c r="F33" t="inlineStr"/>
-      <c r="G33" t="inlineStr"/>
-      <c r="H33" t="inlineStr"/>
-      <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr"/>
-      <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10240,10 +9831,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="N33" t="inlineStr"/>
-      <c r="O33" t="inlineStr"/>
-      <c r="P33" t="inlineStr"/>
-      <c r="Q33" t="inlineStr"/>
       <c r="R33">
         <f>COUNTIF(C33:Q33,"✓")</f>
         <v/>
@@ -10260,15 +9847,6 @@
           <t>Resumen de historial con IA</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr"/>
-      <c r="D34" t="inlineStr"/>
-      <c r="E34" t="inlineStr"/>
-      <c r="F34" t="inlineStr"/>
-      <c r="G34" t="inlineStr"/>
-      <c r="H34" t="inlineStr"/>
-      <c r="I34" t="inlineStr"/>
-      <c r="J34" t="inlineStr"/>
-      <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10279,10 +9857,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="N34" t="inlineStr"/>
-      <c r="O34" t="inlineStr"/>
-      <c r="P34" t="inlineStr"/>
-      <c r="Q34" t="inlineStr"/>
       <c r="R34">
         <f>COUNTIF(C34:Q34,"✓")</f>
         <v/>
@@ -10299,25 +9873,11 @@
           <t>API para apps de terceros</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr"/>
-      <c r="D35" t="inlineStr"/>
-      <c r="E35" t="inlineStr"/>
-      <c r="F35" t="inlineStr"/>
-      <c r="G35" t="inlineStr"/>
-      <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr"/>
       <c r="K35" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="L35" t="inlineStr"/>
-      <c r="M35" t="inlineStr"/>
-      <c r="N35" t="inlineStr"/>
-      <c r="O35" t="inlineStr"/>
-      <c r="P35" t="inlineStr"/>
-      <c r="Q35" t="inlineStr"/>
       <c r="R35">
         <f>COUNTIF(C35:Q35,"✓")</f>
         <v/>
@@ -10339,10 +9899,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr"/>
-      <c r="E36" t="inlineStr"/>
-      <c r="F36" t="inlineStr"/>
-      <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10353,7 +9909,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="J36" t="inlineStr"/>
       <c r="K36" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10369,14 +9924,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="N36" t="inlineStr"/>
       <c r="O36" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="P36" t="inlineStr"/>
-      <c r="Q36" t="inlineStr"/>
       <c r="R36">
         <f>COUNTIF(C36:Q36,"✓")</f>
         <v/>
@@ -10393,25 +9945,11 @@
           <t>Analítica poblacional B2B</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr"/>
-      <c r="D37" t="inlineStr"/>
-      <c r="E37" t="inlineStr"/>
-      <c r="F37" t="inlineStr"/>
-      <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="I37" t="inlineStr"/>
-      <c r="J37" t="inlineStr"/>
-      <c r="K37" t="inlineStr"/>
-      <c r="L37" t="inlineStr"/>
-      <c r="M37" t="inlineStr"/>
-      <c r="N37" t="inlineStr"/>
-      <c r="O37" t="inlineStr"/>
-      <c r="P37" t="inlineStr"/>
-      <c r="Q37" t="inlineStr"/>
       <c r="R37">
         <f>COUNTIF(C37:Q37,"✓")</f>
         <v/>
@@ -10428,9 +9966,6 @@
           <t>Disponibilidad multiplataforma (web/iOS/Android)</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr"/>
-      <c r="D38" t="inlineStr"/>
-      <c r="E38" t="inlineStr"/>
       <c r="F38" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10441,20 +9976,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr"/>
-      <c r="I38" t="inlineStr"/>
-      <c r="J38" t="inlineStr"/>
-      <c r="K38" t="inlineStr"/>
-      <c r="L38" t="inlineStr"/>
-      <c r="M38" t="inlineStr"/>
-      <c r="N38" t="inlineStr"/>
       <c r="O38" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="P38" t="inlineStr"/>
-      <c r="Q38" t="inlineStr"/>
       <c r="R38">
         <f>COUNTIF(C38:Q38,"✓")</f>
         <v/>
@@ -10471,25 +9997,11 @@
           <t>Historial médico centralizado</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr"/>
-      <c r="D39" t="inlineStr"/>
-      <c r="E39" t="inlineStr"/>
-      <c r="F39" t="inlineStr"/>
-      <c r="G39" t="inlineStr"/>
-      <c r="H39" t="inlineStr"/>
-      <c r="I39" t="inlineStr"/>
       <c r="J39" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="K39" t="inlineStr"/>
-      <c r="L39" t="inlineStr"/>
-      <c r="M39" t="inlineStr"/>
-      <c r="N39" t="inlineStr"/>
-      <c r="O39" t="inlineStr"/>
-      <c r="P39" t="inlineStr"/>
-      <c r="Q39" t="inlineStr"/>
       <c r="R39">
         <f>COUNTIF(C39:Q39,"✓")</f>
         <v/>
@@ -10506,25 +10018,11 @@
           <t>Importación y exportación de datos</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr"/>
-      <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr"/>
-      <c r="G40" t="inlineStr"/>
-      <c r="H40" t="inlineStr"/>
-      <c r="I40" t="inlineStr"/>
-      <c r="J40" t="inlineStr"/>
-      <c r="K40" t="inlineStr"/>
-      <c r="L40" t="inlineStr"/>
-      <c r="M40" t="inlineStr"/>
-      <c r="N40" t="inlineStr"/>
-      <c r="O40" t="inlineStr"/>
-      <c r="P40" t="inlineStr"/>
-      <c r="Q40" t="inlineStr"/>
       <c r="R40">
         <f>COUNTIF(C40:Q40,"✓")</f>
         <v/>
@@ -10541,25 +10039,11 @@
           <t>Integración con EHR de proveedores</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr"/>
-      <c r="D41" t="inlineStr"/>
-      <c r="E41" t="inlineStr"/>
-      <c r="F41" t="inlineStr"/>
-      <c r="G41" t="inlineStr"/>
-      <c r="H41" t="inlineStr"/>
-      <c r="I41" t="inlineStr"/>
       <c r="J41" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="K41" t="inlineStr"/>
-      <c r="L41" t="inlineStr"/>
-      <c r="M41" t="inlineStr"/>
-      <c r="N41" t="inlineStr"/>
-      <c r="O41" t="inlineStr"/>
-      <c r="P41" t="inlineStr"/>
-      <c r="Q41" t="inlineStr"/>
       <c r="R41">
         <f>COUNTIF(C41:Q41,"✓")</f>
         <v/>
@@ -10576,29 +10060,16 @@
           <t>Integración con wearables y apps de salud</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr"/>
-      <c r="D42" t="inlineStr"/>
-      <c r="E42" t="inlineStr"/>
-      <c r="F42" t="inlineStr"/>
-      <c r="G42" t="inlineStr"/>
       <c r="H42" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="I42" t="inlineStr"/>
-      <c r="J42" t="inlineStr"/>
-      <c r="K42" t="inlineStr"/>
-      <c r="L42" t="inlineStr"/>
       <c r="M42" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="N42" t="inlineStr"/>
-      <c r="O42" t="inlineStr"/>
-      <c r="P42" t="inlineStr"/>
-      <c r="Q42" t="inlineStr"/>
       <c r="R42">
         <f>COUNTIF(C42:Q42,"✓")</f>
         <v/>
@@ -10615,25 +10086,11 @@
           <t>Gestión de lista de medicamentos</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr"/>
-      <c r="D43" t="inlineStr"/>
-      <c r="E43" t="inlineStr"/>
-      <c r="F43" t="inlineStr"/>
-      <c r="G43" t="inlineStr"/>
-      <c r="H43" t="inlineStr"/>
-      <c r="I43" t="inlineStr"/>
-      <c r="J43" t="inlineStr"/>
       <c r="K43" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="L43" t="inlineStr"/>
-      <c r="M43" t="inlineStr"/>
-      <c r="N43" t="inlineStr"/>
-      <c r="O43" t="inlineStr"/>
-      <c r="P43" t="inlineStr"/>
-      <c r="Q43" t="inlineStr"/>
       <c r="R43">
         <f>COUNTIF(C43:Q43,"✓")</f>
         <v/>
@@ -10650,25 +10107,11 @@
           <t>Importación automática de tratamientos desde receta digital</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr"/>
-      <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr"/>
-      <c r="G44" t="inlineStr"/>
-      <c r="H44" t="inlineStr"/>
-      <c r="I44" t="inlineStr"/>
-      <c r="J44" t="inlineStr"/>
-      <c r="K44" t="inlineStr"/>
-      <c r="L44" t="inlineStr"/>
-      <c r="M44" t="inlineStr"/>
-      <c r="N44" t="inlineStr"/>
-      <c r="O44" t="inlineStr"/>
-      <c r="P44" t="inlineStr"/>
-      <c r="Q44" t="inlineStr"/>
       <c r="R44">
         <f>COUNTIF(C44:Q44,"✓")</f>
         <v/>
@@ -10690,24 +10133,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr"/>
-      <c r="E45" t="inlineStr"/>
-      <c r="F45" t="inlineStr"/>
-      <c r="G45" t="inlineStr"/>
-      <c r="H45" t="inlineStr"/>
-      <c r="I45" t="inlineStr"/>
-      <c r="J45" t="inlineStr"/>
       <c r="K45" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="L45" t="inlineStr"/>
-      <c r="M45" t="inlineStr"/>
-      <c r="N45" t="inlineStr"/>
-      <c r="O45" t="inlineStr"/>
-      <c r="P45" t="inlineStr"/>
-      <c r="Q45" t="inlineStr"/>
       <c r="R45">
         <f>COUNTIF(C45:Q45,"✓")</f>
         <v/>
@@ -10724,25 +10154,11 @@
           <t>Registro de tomas y adherencia al tratamiento</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr"/>
-      <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr"/>
-      <c r="G46" t="inlineStr"/>
-      <c r="H46" t="inlineStr"/>
-      <c r="I46" t="inlineStr"/>
-      <c r="J46" t="inlineStr"/>
-      <c r="K46" t="inlineStr"/>
-      <c r="L46" t="inlineStr"/>
-      <c r="M46" t="inlineStr"/>
-      <c r="N46" t="inlineStr"/>
-      <c r="O46" t="inlineStr"/>
-      <c r="P46" t="inlineStr"/>
-      <c r="Q46" t="inlineStr"/>
       <c r="R46">
         <f>COUNTIF(C46:Q46,"✓")</f>
         <v/>
@@ -10759,25 +10175,11 @@
           <t>Comunidad de pacientes</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr"/>
-      <c r="D47" t="inlineStr"/>
-      <c r="E47" t="inlineStr"/>
-      <c r="F47" t="inlineStr"/>
-      <c r="G47" t="inlineStr"/>
       <c r="H47" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="I47" t="inlineStr"/>
-      <c r="J47" t="inlineStr"/>
-      <c r="K47" t="inlineStr"/>
-      <c r="L47" t="inlineStr"/>
-      <c r="M47" t="inlineStr"/>
-      <c r="N47" t="inlineStr"/>
-      <c r="O47" t="inlineStr"/>
-      <c r="P47" t="inlineStr"/>
-      <c r="Q47" t="inlineStr"/>
       <c r="R47">
         <f>COUNTIF(C47:Q47,"✓")</f>
         <v/>
@@ -10794,25 +10196,11 @@
           <t>Contenido educativo sobre salud</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr"/>
       <c r="D48" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr"/>
-      <c r="F48" t="inlineStr"/>
-      <c r="G48" t="inlineStr"/>
-      <c r="H48" t="inlineStr"/>
-      <c r="I48" t="inlineStr"/>
-      <c r="J48" t="inlineStr"/>
-      <c r="K48" t="inlineStr"/>
-      <c r="L48" t="inlineStr"/>
-      <c r="M48" t="inlineStr"/>
-      <c r="N48" t="inlineStr"/>
-      <c r="O48" t="inlineStr"/>
-      <c r="P48" t="inlineStr"/>
-      <c r="Q48" t="inlineStr"/>
       <c r="R48">
         <f>COUNTIF(C48:Q48,"✓")</f>
         <v/>
@@ -10829,25 +10217,11 @@
           <t>Gráficas de evolución de indicadores</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr"/>
-      <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F49" t="inlineStr"/>
-      <c r="G49" t="inlineStr"/>
-      <c r="H49" t="inlineStr"/>
-      <c r="I49" t="inlineStr"/>
-      <c r="J49" t="inlineStr"/>
-      <c r="K49" t="inlineStr"/>
-      <c r="L49" t="inlineStr"/>
-      <c r="M49" t="inlineStr"/>
-      <c r="N49" t="inlineStr"/>
-      <c r="O49" t="inlineStr"/>
-      <c r="P49" t="inlineStr"/>
-      <c r="Q49" t="inlineStr"/>
       <c r="R49">
         <f>COUNTIF(C49:Q49,"✓")</f>
         <v/>
@@ -10864,25 +10238,11 @@
           <t>Integración con wearables y apps de salud</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr"/>
-      <c r="D50" t="inlineStr"/>
-      <c r="E50" t="inlineStr"/>
-      <c r="F50" t="inlineStr"/>
-      <c r="G50" t="inlineStr"/>
-      <c r="H50" t="inlineStr"/>
-      <c r="I50" t="inlineStr"/>
-      <c r="J50" t="inlineStr"/>
       <c r="K50" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="L50" t="inlineStr"/>
-      <c r="M50" t="inlineStr"/>
-      <c r="N50" t="inlineStr"/>
-      <c r="O50" t="inlineStr"/>
-      <c r="P50" t="inlineStr"/>
-      <c r="Q50" t="inlineStr"/>
       <c r="R50">
         <f>COUNTIF(C50:Q50,"✓")</f>
         <v/>
@@ -10899,11 +10259,6 @@
           <t>Panel de seguimiento de salud y bienestar</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr"/>
-      <c r="D51" t="inlineStr"/>
-      <c r="E51" t="inlineStr"/>
-      <c r="F51" t="inlineStr"/>
-      <c r="G51" t="inlineStr"/>
       <c r="H51" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10914,14 +10269,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="J51" t="inlineStr"/>
-      <c r="K51" t="inlineStr"/>
-      <c r="L51" t="inlineStr"/>
-      <c r="M51" t="inlineStr"/>
-      <c r="N51" t="inlineStr"/>
-      <c r="O51" t="inlineStr"/>
-      <c r="P51" t="inlineStr"/>
-      <c r="Q51" t="inlineStr"/>
       <c r="R51">
         <f>COUNTIF(C51:Q51,"✓")</f>
         <v/>
@@ -10938,25 +10285,11 @@
           <t>Registro de nutrición</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr"/>
-      <c r="D52" t="inlineStr"/>
-      <c r="E52" t="inlineStr"/>
-      <c r="F52" t="inlineStr"/>
-      <c r="G52" t="inlineStr"/>
-      <c r="H52" t="inlineStr"/>
-      <c r="I52" t="inlineStr"/>
-      <c r="J52" t="inlineStr"/>
       <c r="K52" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="L52" t="inlineStr"/>
-      <c r="M52" t="inlineStr"/>
-      <c r="N52" t="inlineStr"/>
-      <c r="O52" t="inlineStr"/>
-      <c r="P52" t="inlineStr"/>
-      <c r="Q52" t="inlineStr"/>
       <c r="R52">
         <f>COUNTIF(C52:Q52,"✓")</f>
         <v/>
@@ -10973,25 +10306,11 @@
           <t>Seguimiento de salud femenina</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr"/>
-      <c r="D53" t="inlineStr"/>
-      <c r="E53" t="inlineStr"/>
-      <c r="F53" t="inlineStr"/>
-      <c r="G53" t="inlineStr"/>
-      <c r="H53" t="inlineStr"/>
-      <c r="I53" t="inlineStr"/>
-      <c r="J53" t="inlineStr"/>
       <c r="K53" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="L53" t="inlineStr"/>
-      <c r="M53" t="inlineStr"/>
-      <c r="N53" t="inlineStr"/>
-      <c r="O53" t="inlineStr"/>
-      <c r="P53" t="inlineStr"/>
-      <c r="Q53" t="inlineStr"/>
       <c r="R53">
         <f>COUNTIF(C53:Q53,"✓")</f>
         <v/>
@@ -11008,25 +10327,11 @@
           <t>Valoración de profesionales</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr"/>
-      <c r="D54" t="inlineStr"/>
-      <c r="E54" t="inlineStr"/>
       <c r="F54" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="G54" t="inlineStr"/>
-      <c r="H54" t="inlineStr"/>
-      <c r="I54" t="inlineStr"/>
-      <c r="J54" t="inlineStr"/>
-      <c r="K54" t="inlineStr"/>
-      <c r="L54" t="inlineStr"/>
-      <c r="M54" t="inlineStr"/>
-      <c r="N54" t="inlineStr"/>
-      <c r="O54" t="inlineStr"/>
-      <c r="P54" t="inlineStr"/>
-      <c r="Q54" t="inlineStr"/>
       <c r="R54">
         <f>COUNTIF(C54:Q54,"✓")</f>
         <v/>
@@ -11043,25 +10348,11 @@
           <t>Acceso mínimo por categorías de datos</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr"/>
-      <c r="D55" t="inlineStr"/>
-      <c r="E55" t="inlineStr"/>
-      <c r="F55" t="inlineStr"/>
-      <c r="G55" t="inlineStr"/>
-      <c r="H55" t="inlineStr"/>
-      <c r="I55" t="inlineStr"/>
-      <c r="J55" t="inlineStr"/>
-      <c r="K55" t="inlineStr"/>
-      <c r="L55" t="inlineStr"/>
       <c r="M55" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="N55" t="inlineStr"/>
-      <c r="O55" t="inlineStr"/>
-      <c r="P55" t="inlineStr"/>
-      <c r="Q55" t="inlineStr"/>
       <c r="R55">
         <f>COUNTIF(C55:Q55,"✓")</f>
         <v/>
@@ -11078,11 +10369,6 @@
           <t>Blockchain para integridad y trazabilidad de datos</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr"/>
-      <c r="D56" t="inlineStr"/>
-      <c r="E56" t="inlineStr"/>
-      <c r="F56" t="inlineStr"/>
-      <c r="G56" t="inlineStr"/>
       <c r="H56" t="inlineStr">
         <is>
           <t>✓</t>
@@ -11098,13 +10384,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="K56" t="inlineStr"/>
-      <c r="L56" t="inlineStr"/>
-      <c r="M56" t="inlineStr"/>
-      <c r="N56" t="inlineStr"/>
-      <c r="O56" t="inlineStr"/>
-      <c r="P56" t="inlineStr"/>
-      <c r="Q56" t="inlineStr"/>
       <c r="R56">
         <f>COUNTIF(C56:Q56,"✓")</f>
         <v/>
@@ -11121,29 +10400,16 @@
           <t>Cifrado y control de acceso</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr"/>
       <c r="D57" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="E57" t="inlineStr"/>
-      <c r="F57" t="inlineStr"/>
-      <c r="G57" t="inlineStr"/>
-      <c r="H57" t="inlineStr"/>
-      <c r="I57" t="inlineStr"/>
-      <c r="J57" t="inlineStr"/>
       <c r="K57" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="L57" t="inlineStr"/>
-      <c r="M57" t="inlineStr"/>
-      <c r="N57" t="inlineStr"/>
-      <c r="O57" t="inlineStr"/>
-      <c r="P57" t="inlineStr"/>
-      <c r="Q57" t="inlineStr"/>
       <c r="R57">
         <f>COUNTIF(C57:Q57,"✓")</f>
         <v/>
@@ -11160,25 +10426,11 @@
           <t>Cumplimiento regulatorio de salud y datos</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr"/>
-      <c r="D58" t="inlineStr"/>
-      <c r="E58" t="inlineStr"/>
-      <c r="F58" t="inlineStr"/>
-      <c r="G58" t="inlineStr"/>
-      <c r="H58" t="inlineStr"/>
-      <c r="I58" t="inlineStr"/>
-      <c r="J58" t="inlineStr"/>
-      <c r="K58" t="inlineStr"/>
-      <c r="L58" t="inlineStr"/>
-      <c r="M58" t="inlineStr"/>
-      <c r="N58" t="inlineStr"/>
       <c r="O58" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="P58" t="inlineStr"/>
-      <c r="Q58" t="inlineStr"/>
       <c r="R58">
         <f>COUNTIF(C58:Q58,"✓")</f>
         <v/>
@@ -11195,25 +10447,11 @@
           <t>Gestión de consentimiento sobre uso de datos</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr"/>
-      <c r="D59" t="inlineStr"/>
-      <c r="E59" t="inlineStr"/>
-      <c r="F59" t="inlineStr"/>
-      <c r="G59" t="inlineStr"/>
-      <c r="H59" t="inlineStr"/>
-      <c r="I59" t="inlineStr"/>
-      <c r="J59" t="inlineStr"/>
-      <c r="K59" t="inlineStr"/>
       <c r="L59" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="M59" t="inlineStr"/>
-      <c r="N59" t="inlineStr"/>
-      <c r="O59" t="inlineStr"/>
-      <c r="P59" t="inlineStr"/>
-      <c r="Q59" t="inlineStr"/>
       <c r="R59">
         <f>COUNTIF(C59:Q59,"✓")</f>
         <v/>
@@ -11230,25 +10468,11 @@
           <t>Identidad descentralizada (DID)</t>
         </is>
       </c>
-      <c r="C60" t="inlineStr"/>
-      <c r="D60" t="inlineStr"/>
-      <c r="E60" t="inlineStr"/>
-      <c r="F60" t="inlineStr"/>
-      <c r="G60" t="inlineStr"/>
-      <c r="H60" t="inlineStr"/>
       <c r="I60" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="J60" t="inlineStr"/>
-      <c r="K60" t="inlineStr"/>
-      <c r="L60" t="inlineStr"/>
-      <c r="M60" t="inlineStr"/>
-      <c r="N60" t="inlineStr"/>
-      <c r="O60" t="inlineStr"/>
-      <c r="P60" t="inlineStr"/>
-      <c r="Q60" t="inlineStr"/>
       <c r="R60">
         <f>COUNTIF(C60:Q60,"✓")</f>
         <v/>
@@ -11265,15 +10489,6 @@
           <t>Privacidad reforzada para datos de salud</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr"/>
-      <c r="D61" t="inlineStr"/>
-      <c r="E61" t="inlineStr"/>
-      <c r="F61" t="inlineStr"/>
-      <c r="G61" t="inlineStr"/>
-      <c r="H61" t="inlineStr"/>
-      <c r="I61" t="inlineStr"/>
-      <c r="J61" t="inlineStr"/>
-      <c r="K61" t="inlineStr"/>
       <c r="L61" t="inlineStr">
         <is>
           <t>✓</t>
@@ -11284,10 +10499,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="N61" t="inlineStr"/>
-      <c r="O61" t="inlineStr"/>
-      <c r="P61" t="inlineStr"/>
-      <c r="Q61" t="inlineStr"/>
       <c r="R61">
         <f>COUNTIF(C61:Q61,"✓")</f>
         <v/>
@@ -11304,20 +10515,6 @@
           <t>Modelo freemium y suscripción</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr"/>
-      <c r="D62" t="inlineStr"/>
-      <c r="E62" t="inlineStr"/>
-      <c r="F62" t="inlineStr"/>
-      <c r="G62" t="inlineStr"/>
-      <c r="H62" t="inlineStr"/>
-      <c r="I62" t="inlineStr"/>
-      <c r="J62" t="inlineStr"/>
-      <c r="K62" t="inlineStr"/>
-      <c r="L62" t="inlineStr"/>
-      <c r="M62" t="inlineStr"/>
-      <c r="N62" t="inlineStr"/>
-      <c r="O62" t="inlineStr"/>
-      <c r="P62" t="inlineStr"/>
       <c r="Q62" t="inlineStr">
         <is>
           <t>✓</t>
@@ -11339,25 +10536,11 @@
           <t>Pagos con criptomoneda</t>
         </is>
       </c>
-      <c r="C63" t="inlineStr"/>
-      <c r="D63" t="inlineStr"/>
-      <c r="E63" t="inlineStr"/>
-      <c r="F63" t="inlineStr"/>
-      <c r="G63" t="inlineStr"/>
-      <c r="H63" t="inlineStr"/>
-      <c r="I63" t="inlineStr"/>
       <c r="J63" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="K63" t="inlineStr"/>
-      <c r="L63" t="inlineStr"/>
-      <c r="M63" t="inlineStr"/>
-      <c r="N63" t="inlineStr"/>
-      <c r="O63" t="inlineStr"/>
-      <c r="P63" t="inlineStr"/>
-      <c r="Q63" t="inlineStr"/>
       <c r="R63">
         <f>COUNTIF(C63:Q63,"✓")</f>
         <v/>
@@ -11374,20 +10557,6 @@
           <t>Pagos dentro de la app</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr"/>
-      <c r="D64" t="inlineStr"/>
-      <c r="E64" t="inlineStr"/>
-      <c r="F64" t="inlineStr"/>
-      <c r="G64" t="inlineStr"/>
-      <c r="H64" t="inlineStr"/>
-      <c r="I64" t="inlineStr"/>
-      <c r="J64" t="inlineStr"/>
-      <c r="K64" t="inlineStr"/>
-      <c r="L64" t="inlineStr"/>
-      <c r="M64" t="inlineStr"/>
-      <c r="N64" t="inlineStr"/>
-      <c r="O64" t="inlineStr"/>
-      <c r="P64" t="inlineStr"/>
       <c r="Q64" t="inlineStr">
         <is>
           <t>✓</t>
@@ -11409,25 +10578,11 @@
           <t>Reclamos y trámites con seguros</t>
         </is>
       </c>
-      <c r="C65" t="inlineStr"/>
-      <c r="D65" t="inlineStr"/>
-      <c r="E65" t="inlineStr"/>
-      <c r="F65" t="inlineStr"/>
-      <c r="G65" t="inlineStr"/>
-      <c r="H65" t="inlineStr"/>
       <c r="I65" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="J65" t="inlineStr"/>
-      <c r="K65" t="inlineStr"/>
-      <c r="L65" t="inlineStr"/>
-      <c r="M65" t="inlineStr"/>
-      <c r="N65" t="inlineStr"/>
-      <c r="O65" t="inlineStr"/>
-      <c r="P65" t="inlineStr"/>
-      <c r="Q65" t="inlineStr"/>
       <c r="R65">
         <f>COUNTIF(C65:Q65,"✓")</f>
         <v/>
@@ -11444,25 +10599,11 @@
           <t>Mensajería paciente-institución</t>
         </is>
       </c>
-      <c r="C66" t="inlineStr"/>
-      <c r="D66" t="inlineStr"/>
-      <c r="E66" t="inlineStr"/>
-      <c r="F66" t="inlineStr"/>
-      <c r="G66" t="inlineStr"/>
-      <c r="H66" t="inlineStr"/>
       <c r="I66" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="J66" t="inlineStr"/>
-      <c r="K66" t="inlineStr"/>
-      <c r="L66" t="inlineStr"/>
-      <c r="M66" t="inlineStr"/>
-      <c r="N66" t="inlineStr"/>
-      <c r="O66" t="inlineStr"/>
-      <c r="P66" t="inlineStr"/>
-      <c r="Q66" t="inlineStr"/>
       <c r="R66">
         <f>COUNTIF(C66:Q66,"✓")</f>
         <v/>
@@ -11479,25 +10620,11 @@
           <t>Teleconsulta con profesionales</t>
         </is>
       </c>
-      <c r="C67" t="inlineStr"/>
-      <c r="D67" t="inlineStr"/>
-      <c r="E67" t="inlineStr"/>
-      <c r="F67" t="inlineStr"/>
-      <c r="G67" t="inlineStr"/>
-      <c r="H67" t="inlineStr"/>
-      <c r="I67" t="inlineStr"/>
       <c r="J67" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="K67" t="inlineStr"/>
-      <c r="L67" t="inlineStr"/>
-      <c r="M67" t="inlineStr"/>
-      <c r="N67" t="inlineStr"/>
-      <c r="O67" t="inlineStr"/>
-      <c r="P67" t="inlineStr"/>
-      <c r="Q67" t="inlineStr"/>
       <c r="R67">
         <f>COUNTIF(C67:Q67,"✓")</f>
         <v/>
@@ -11514,7 +10641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A29"/>
+  <dimension ref="A1:A30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -11723,6 +10850,13 @@
         </is>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Vuelta 7 (iter. 1, 2026-10-17 12:15 UTC): Meedika, Infomed, MediPlanner, Clingot verificados (+0 filas; saturado). Pendientes: Healfies, Patientory, MediBloc, Medicalchain, Apple Health, ChatGPT Health, Claude for Healthcare, Apps de clínicas, Clinia, MiRedSalud, Mediko.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Benchmark: vuelta 7, iteración 2 (Healfies, Patientory, MediBloc, Medicalchain)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MVcXu8vTBu7EKfj3YdEvae
</commit_message>
<xml_diff>
--- a/Outputs/Benchmark_Anamnesis.xlsx
+++ b/Outputs/Benchmark_Anamnesis.xlsx
@@ -673,12 +673,12 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>[REGIONAL · Brasil] Fundada ene-2015 en Florianópolis por Helyson Lewis Velasco. Centraliza registros de salud personales: carpetas, etiquetas, línea de tiempo (medicación, exámenes, citas, dieta), compartir con familia o profesionales. Gratis; web, iOS y Android. Estado actual NO verificado (fuentes de 2015-2016). Referencia funcional cercana a etapas A+B. [Vuelta 2] Lanzada simultáneamente en Brasil, Argentina y EE.UU.; permite compartir con no registrados vía clave por email. Sin novedades posteriores a 2016. [Vuelta 3] Sin evidencia de actividad reciente ni de cierre; Gust/Dealroom la listan en Florianópolis (10 empleados, healfies.com) sin fecha de actualización. Estado sin confirmar. [Vuelta 4] Sin Google Play localizado; no confundir con la app Healfy (otro producto). Sin novedades. [Vuelta 5] Sin búsqueda nueva (revisada en vuelta 4); sin cambios. [Vuelta 6] Sin búsqueda nueva (fuentes agotadas); sin cambios.</t>
+          <t>[REGIONAL · Brasil] Fundada ene-2015 en Florianópolis por Helyson Lewis Velasco. Centraliza registros de salud personales: carpetas, etiquetas, línea de tiempo (medicación, exámenes, citas, dieta), compartir con familia o profesionales. Gratis; web, iOS y Android. Estado actual NO verificado (fuentes de 2015-2016). Referencia funcional cercana a etapas A+B. [Vuelta 2] Lanzada simultáneamente en Brasil, Argentina y EE.UU.; permite compartir con no registrados vía clave por email. Sin novedades posteriores a 2016. [Vuelta 3] Sin evidencia de actividad reciente ni de cierre; Gust/Dealroom la listan en Florianópolis (10 empleados, healfies.com) sin fecha de actualización. Estado sin confirmar. [Vuelta 4] Sin Google Play localizado; no confundir con la app Healfy (otro producto). Sin novedades. [Vuelta 5] Sin búsqueda nueva (revisada en vuelta 4); sin cambios. [Vuelta 6] Sin búsqueda nueva (fuentes agotadas); sin cambios. [Vuelta 7] Solo fuentes de 2015-2016; alianza con ClinCard (feb-2016). Sin evidencia de actividad reciente.</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G6" t="n">
@@ -686,7 +686,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -713,12 +713,12 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>[BLOCKCHAIN · EE.UU.] Atlanta, fundada 2015, ~9 empleados. Levantó US$7,2M vía financiamiento cripto. App con registros de hospitales y wearables, coaching de salud con IA y recompensas en cripto; también dashboard empresarial Neith. PitchBook indica actividad y financiamiento hasta abr-2026: sigue operando. Sin presencia conocida en Chile. Referencia directa para la hipótesis blockchain. [Vuelta 2] Sin noticias 2026 encontradas en búsqueda; sitio oficial bloqueado. [Vuelta 3] Búsqueda adicional solo devuelve hitos de 2017 (token sale US$7,2M) y 2019 (Serie A de US$5,3M, cierre no confirmado); sin datos 2025-26 propios. [Vuelta 4] App pública lanzada en la conferencia JP Morgan Healthcare (2019); red PTOYMatrix (blockchain HIPAA); socios reportados: StartUp Health y Kaiser Permanente (beta). Estado actual en App Store/Google Play sin confirmar. [Vuelta 5] Sin noticias 2026 del equipo. Token PTOY con capitalización de ~US$53K a fines de ago-2026 según Phantom (KuCoin discrepa en la circulación): señal de baja actividad, no prueba de cierre. Esto relativiza la actividad hasta abr-2026 mencionada en la ficha original. [Vuelta 6] Sin noticias posteriores a 2020 localizadas (hitos: token sale 2017, consorcio Hyperledger, alianza con Georgia State, Series A de US$5,3M vía R/GA Ventures, Neith con Prosper Healthtech en Birmingham). Estado actual desconocido.</t>
+          <t>[BLOCKCHAIN · EE.UU.] Atlanta, fundada 2015, ~9 empleados. Levantó US$7,2M vía financiamiento cripto. App con registros de hospitales y wearables, coaching de salud con IA y recompensas en cripto; también dashboard empresarial Neith. PitchBook indica actividad y financiamiento hasta abr-2026: sigue operando. Sin presencia conocida en Chile. Referencia directa para la hipótesis blockchain. [Vuelta 2] Sin noticias 2026 encontradas en búsqueda; sitio oficial bloqueado. [Vuelta 3] Búsqueda adicional solo devuelve hitos de 2017 (token sale US$7,2M) y 2019 (Serie A de US$5,3M, cierre no confirmado); sin datos 2025-26 propios. [Vuelta 4] App pública lanzada en la conferencia JP Morgan Healthcare (2019); red PTOYMatrix (blockchain HIPAA); socios reportados: StartUp Health y Kaiser Permanente (beta). Estado actual en App Store/Google Play sin confirmar. [Vuelta 5] Sin noticias 2026 del equipo. Token PTOY con capitalización de ~US$53K a fines de ago-2026 según Phantom (KuCoin discrepa en la circulación): señal de baja actividad, no prueba de cierre. Esto relativiza la actividad hasta abr-2026 mencionada en la ficha original. [Vuelta 6] Sin noticias posteriores a 2020 localizadas (hitos: token sale 2017, consorcio Hyperledger, alianza con Georgia State, Series A de US$5,3M vía R/GA Ventures, Neith con Prosper Healthtech en Birmingham). Estado actual desconocido. [Vuelta 7] Sin búsqueda nueva (saturado); sin cambios.</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G7" t="n">
@@ -726,7 +726,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -753,12 +753,12 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>[BLOCKCHAIN · Corea del Sur] Fundada 2017, Seúl. Blockchain propia Panacea (Cosmos SDK, mainnet 2019) para que el paciente gestione y transfiera sus registros; app Medipass para seguros. Serie A de ₩4.000 millones (Naver); alianzas con hospitales (Seoul National, Severance). Estado 2025-26 NO verificado. Referencia sobre seguros + blockchain. [Vuelta 2] Panacea incluye DID, Append Only Log, IBC y PNFT; sin anuncios 2026 localizados. [Vuelta 3] Medipass: app en Corea con 20 hospitales/aseguradoras integrados (fecha de la lista desconocida) y plan 2022 de superapp con marketplace de datos; operación actual sin confirmar. [Vuelta 4] Sin búsqueda nueva (revisada en vuelta 3); sin cambios. [Vuelta 5] Medipass: ~400.000 usuarios acumulados (CEO, jun-2022); integración con aseguradoras Shinhan Life, Samsung Fire y Hyundai Marine (2020); renovación completa en mar-2023 (dashboard de salud, gestión familiar, certificados). Sin noticias 2026 encontradas. [Vuelta 6] Medipass 2023: comunicación bidireccional hospital-paciente y chat MediTalk; en 2019 fue seleccionada para el programa gubernamental de MyData médico con Samsung Fire y SNUH. Sin estrategia 2026 localizada. Meta declarada: usar Medipass como «identificación» de salud.</t>
+          <t>[BLOCKCHAIN · Corea del Sur] Fundada 2017, Seúl. Blockchain propia Panacea (Cosmos SDK, mainnet 2019) para que el paciente gestione y transfiera sus registros; app Medipass para seguros. Serie A de ₩4.000 millones (Naver); alianzas con hospitales (Seoul National, Severance). Estado 2025-26 NO verificado. Referencia sobre seguros + blockchain. [Vuelta 2] Panacea incluye DID, Append Only Log, IBC y PNFT; sin anuncios 2026 localizados. [Vuelta 3] Medipass: app en Corea con 20 hospitales/aseguradoras integrados (fecha de la lista desconocida) y plan 2022 de superapp con marketplace de datos; operación actual sin confirmar. [Vuelta 4] Sin búsqueda nueva (revisada en vuelta 3); sin cambios. [Vuelta 5] Medipass: ~400.000 usuarios acumulados (CEO, jun-2022); integración con aseguradoras Shinhan Life, Samsung Fire y Hyundai Marine (2020); renovación completa en mar-2023 (dashboard de salud, gestión familiar, certificados). Sin noticias 2026 encontradas. [Vuelta 6] Medipass 2023: comunicación bidireccional hospital-paciente y chat MediTalk; en 2019 fue seleccionada para el programa gubernamental de MyData médico con Samsung Fire y SNUH. Sin estrategia 2026 localizada. Meta declarada: usar Medipass como «identificación» de salud. [Vuelta 7] Una fuente sin fecha atribuye a Medipass más de 600.000 pacientes en 14 hospitales; MoU 2019 con Severance (plataforma de facturación de seguros y detección de falsificación de datos) y piloto con Massachusetts General Hospital. Sin datos 2025-26.</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G8" t="n">
@@ -766,7 +766,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -793,12 +793,12 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>[BLOCKCHAIN · Reino Unido · INACTIVO] Londres, 2017, Ethereum, con telemedicina. Piloto según registro de la UE (2020). Tracxn/PitchBook lo marcan fuera de operación (ago-2025). Solo caso de aprendizaje: no cuenta como competidor activo. [Vuelta 2] Token MTN deslistado de Bitfinex el 26-mar-2021; sin hallazgos de actividad posterior. [Vuelta 3] Seedtable la marca activa sin fuente; no hallé registro en Companies House. Sigue tratándose como caso de aprendizaje. [Vuelta 4] Pre-venta reportada de US$20M en MedTokens (un solo artículo secundario, sin verificar); modelo de token en revisión y exploración de security token según AMA; integraciones y servicios de 2019 sin confirmar. [Vuelta 5] Un agregador indica sitio medicalchain.com fuera de línea desde 15-feb-2025, último commit en GitHub hace ~3 años y proyecto en «fase de mantenimiento»; preventa de MedTokens reportada entre US$20M y US$24M (fuentes discrepan). Confirma tratarlo como inactivo. [Vuelta 6] Sin búsqueda nueva (revisada en vuelta 5; sitio fuera de línea desde feb-2025 según un agregador); sin cambios.</t>
+          <t>[BLOCKCHAIN · Reino Unido · INACTIVO] Londres, 2017, Ethereum, con telemedicina. Piloto según registro de la UE (2020). Tracxn/PitchBook lo marcan fuera de operación (ago-2025). Solo caso de aprendizaje: no cuenta como competidor activo. [Vuelta 2] Token MTN deslistado de Bitfinex el 26-mar-2021; sin hallazgos de actividad posterior. [Vuelta 3] Seedtable la marca activa sin fuente; no hallé registro en Companies House. Sigue tratándose como caso de aprendizaje. [Vuelta 4] Pre-venta reportada de US$20M en MedTokens (un solo artículo secundario, sin verificar); modelo de token en revisión y exploración de security token según AMA; integraciones y servicios de 2019 sin confirmar. [Vuelta 5] Un agregador indica sitio medicalchain.com fuera de línea desde 15-feb-2025, último commit en GitHub hace ~3 años y proyecto en «fase de mantenimiento»; preventa de MedTokens reportada entre US$20M y US$24M (fuentes discrepan). Confirma tratarlo como inactivo. [Vuelta 6] Sin búsqueda nueva (revisada en vuelta 5; sitio fuera de línea desde feb-2025 según un agregador); sin cambios. [Vuelta 7] Sin búsqueda nueva (saturado); sin cambios.</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G9" t="n">
@@ -806,7 +806,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -1102,7 +1102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F131"/>
+  <dimension ref="A1:F132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -5302,6 +5302,38 @@
       <c r="F131" t="inlineStr">
         <is>
           <t>Búsqueda web (Apple, TechCrunch, Pharmaphorum); registros solo EE.UU./UK/Canadá</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>Healfies</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Gestión documental</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Entrega de documentos por terceros (ClinCard)</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>Desde feb-2016, la administradora de tarjetas ClinCard entregaba contratos y documentos a sus clientes dentro de la plataforma.</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>Latam</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>Búsqueda web (Baguete, 2016); estado actual no verificado</t>
         </is>
       </c>
     </row>
@@ -10641,7 +10673,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A30"/>
+  <dimension ref="A1:A31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -10857,6 +10889,13 @@
         </is>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Vuelta 7 (iter. 2, 2026-10-18 12:15 UTC): Healfies, Patientory, MediBloc, Medicalchain verificados (+1 fila, de Healfies). Pendientes: Apple Health, ChatGPT Health, Claude for Healthcare, Apps de clínicas, Clinia, MiRedSalud, Mediko.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Benchmark: vuelta 7, iteración 3 (Apple Health, ChatGPT Health, Claude for Healthcare, Apps de clínicas)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MVcXu8vTBu7EKfj3YdEvae
</commit_message>
<xml_diff>
--- a/Outputs/Benchmark_Anamnesis.xlsx
+++ b/Outputs/Benchmark_Anamnesis.xlsx
@@ -833,12 +833,12 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>[ADYACENTE · global] Agrega registros clínicos vía FHIR; &gt;500 instituciones conectadas en EE.UU. (2018). Sin evidencia de disponibilidad en Chile. Incluida en el dispositivo. Amenaza si FHIR/IPS-CL se adopta en Chile. [Vuelta 2] Sin disponibilidad de registros clínicos en Chile (solo EE.UU., Reino Unido, Canadá). [Vuelta 3] iOS 27 (WWDC 8-jun-2026; publicado ~14-sep-2026): rediseño del app Health, menopausia, nutrición por cámara. El coach de salud con IA no se anunció. Sin ampliación de Health Records a Chile. [Vuelta 4] Sin búsqueda nueva (revisada en vuelta 3); sin cambios. [Vuelta 5] Sin ampliación de Health Records a Australia, Europa ni Latinoamérica (solo EE.UU., UK, Canadá). Funciones de dispositivo (apnea del sueño, prueba auditiva) sí se amplían a países latinoamericanos, pero no son registros clínicos. [Vuelta 6] Sin novedades de iOS 27.x localizadas. Health Records API permite compartir registros con apps de terceros con control por app; opción de enviar datos de uso a Apple.</t>
+          <t>[ADYACENTE · global] Agrega registros clínicos vía FHIR; &gt;500 instituciones conectadas en EE.UU. (2018). Sin evidencia de disponibilidad en Chile. Incluida en el dispositivo. Amenaza si FHIR/IPS-CL se adopta en Chile. [Vuelta 2] Sin disponibilidad de registros clínicos en Chile (solo EE.UU., Reino Unido, Canadá). [Vuelta 3] iOS 27 (WWDC 8-jun-2026; publicado ~14-sep-2026): rediseño del app Health, menopausia, nutrición por cámara. El coach de salud con IA no se anunció. Sin ampliación de Health Records a Chile. [Vuelta 4] Sin búsqueda nueva (revisada en vuelta 3); sin cambios. [Vuelta 5] Sin ampliación de Health Records a Australia, Europa ni Latinoamérica (solo EE.UU., UK, Canadá). Funciones de dispositivo (apnea del sueño, prueba auditiva) sí se amplían a países latinoamericanos, pero no son registros clínicos. [Vuelta 6] Sin novedades de iOS 27.x localizadas. Health Records API permite compartir registros con apps de terceros con control por app; opción de enviar datos de uso a Apple. [Vuelta 7] Coach de salud con IA / Health+ de pago: solo rumores (Gurman), atrasado al menos a iOS 27; no confirmado ni anunciado.</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G10" t="n">
@@ -846,7 +846,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -873,12 +873,12 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>[ADYACENTE · global] Lanzado 7-ene-2026. Conecta registros médicos; conectores solo en EE.UU. Dentro de suscripción del asistente. Fija la expectativa de consultar y resumir el historial. [Vuelta 2] Confirmado: registros solo EE.UU.; sin anuncios para Latinoamérica. Hay inconsistencia de fechas entre fuentes (7-ene-2026 lanzamiento vs. jul-2026 despliegue de registros). [Vuelta 3] Fechas aclaradas: presentación 7-ene-2026 (acceso limitado); despliegue de Health in ChatGPT con Apple Health y registros en EE.UU. el 23-jul-2026; mejora de salud jun-2026. Sin anuncios para Latinoamérica ni para sep-oct 2026. [Vuelta 4] Septiembre 2026: permisos por defecto para datos conectados (14-sep) y explicaciones por gráfico/métrica (28-sep); ChatGPT for Clinicians (abr-2026) para clínicos verificados de EE.UU. Más del 70% de usuarios de Health permite usar datos conectados sin pedir permiso (según OpenAI). Sigue solo EE.UU. [Vuelta 5] Nota de jul-2026: Health no está disponible en México, Android, modo de voz ni Codex; web e iOS en EE.UU., adultos con sesión iniciada. Sin anuncio para Chile ni Latinoamérica. [Vuelta 6] Última entrada de Health en las notas de OpenAI sigue siendo la del 23-jul-2026 (más cambios de sep); sin entradas de octubre localizadas. Health tab: laboratorios, medicamentos, actividad y sueño en una vista; solo EE.UU., web e iOS.</t>
+          <t>[ADYACENTE · global] Lanzado 7-ene-2026. Conecta registros médicos; conectores solo en EE.UU. Dentro de suscripción del asistente. Fija la expectativa de consultar y resumir el historial. [Vuelta 2] Confirmado: registros solo EE.UU.; sin anuncios para Latinoamérica. Hay inconsistencia de fechas entre fuentes (7-ene-2026 lanzamiento vs. jul-2026 despliegue de registros). [Vuelta 3] Fechas aclaradas: presentación 7-ene-2026 (acceso limitado); despliegue de Health in ChatGPT con Apple Health y registros en EE.UU. el 23-jul-2026; mejora de salud jun-2026. Sin anuncios para Latinoamérica ni para sep-oct 2026. [Vuelta 4] Septiembre 2026: permisos por defecto para datos conectados (14-sep) y explicaciones por gráfico/métrica (28-sep); ChatGPT for Clinicians (abr-2026) para clínicos verificados de EE.UU. Más del 70% de usuarios de Health permite usar datos conectados sin pedir permiso (según OpenAI). Sigue solo EE.UU. [Vuelta 5] Nota de jul-2026: Health no está disponible en México, Android, modo de voz ni Codex; web e iOS en EE.UU., adultos con sesión iniciada. Sin anuncio para Chile ni Latinoamérica. [Vuelta 6] Última entrada de Health en las notas de OpenAI sigue siendo la del 23-jul-2026 (más cambios de sep); sin entradas de octubre localizadas. Health tab: laboratorios, medicamentos, actividad y sueño en una vista; solo EE.UU., web e iOS. [Vuelta 7] OpenAI afirma que más de 300 millones de personas usan ChatGPT cada semana para consultas de salud (dato de la empresa). No es una solución con cumplimiento HIPAA declarado. Sin novedades de oct-2026.</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G11" t="n">
@@ -886,7 +886,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -913,12 +913,12 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>[ADYACENTE · global] Lanzado 11-ene-2026. Conectores solo en EE.UU., planes Pro/Max. Nota: producto de Anthropic, conflicto de interés al evaluarlo. [Vuelta 2] Sin cambios fuera de EE.UU. (HealthEx y Function para Pro/Max). [Vuelta 3] Sin anuncios posteriores a enero de 2026. Hoja de ruta de HealthEx (agendar, buscar prestadores, recetas) sin confirmar como lanzada. [Vuelta 4] Sin anuncios nuevos. Fuentes discrepan en el acceso (Pro/Max según Fortune y la mayoría; Pro/Team según Times of AI); sin evidencia de disponibilidad fuera de EE.UU. [Vuelta 5] Sin noticias de oct-2026; HealthEx agrega datos de &gt;50.000 sistemas de EE.UU. y Claude pide solo las categorías relevantes vía MCP. [Vuelta 6] Sin noticias posteriores a enero de 2026 localizadas.</t>
+          <t>[ADYACENTE · global] Lanzado 11-ene-2026. Conectores solo en EE.UU., planes Pro/Max. Nota: producto de Anthropic, conflicto de interés al evaluarlo. [Vuelta 2] Sin cambios fuera de EE.UU. (HealthEx y Function para Pro/Max). [Vuelta 3] Sin anuncios posteriores a enero de 2026. Hoja de ruta de HealthEx (agendar, buscar prestadores, recetas) sin confirmar como lanzada. [Vuelta 4] Sin anuncios nuevos. Fuentes discrepan en el acceso (Pro/Max según Fortune y la mayoría; Pro/Team según Times of AI); sin evidencia de disponibilidad fuera de EE.UU. [Vuelta 5] Sin noticias de oct-2026; HealthEx agrega datos de &gt;50.000 sistemas de EE.UU. y Claude pide solo las categorías relevantes vía MCP. [Vuelta 6] Sin noticias posteriores a enero de 2026 localizadas. [Vuelta 7] Sin novedades posteriores a enero de 2026.</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G12" t="n">
@@ -926,7 +926,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -953,12 +953,12 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>[SUSTITUTO PARCIAL · Chile] Reservar hora, ver historial de esa institución, vincular familiar. Gratis; no consolida datos de otras instituciones. [Vuelta 2] App concreta: Mi Alemana Go (Clínica Alemana, Chile), con historial desde 2018, recetas, órdenes, familiar vinculado y resultados. [Vuelta 3] Búsqueda de otras clínicas (Las Condes, Santa María, UC Christus) sin ficha de app confirmada; solo canales digitales genéricos. [Vuelta 4] Mi Alemana Go: 3,1/5 con 137 calificaciones (App Store Chile), pantalla de inicio rediseñada para gestionar salud propia y familiar; sin evidencia de teleconsulta ni pagos en la app. [Vuelta 5] Sin búsqueda nueva (revisada en vuelta 4); sin cambios. [Vuelta 6] Sin búsqueda nueva; sin cambios.</t>
+          <t>[SUSTITUTO PARCIAL · Chile] Reservar hora, ver historial de esa institución, vincular familiar. Gratis; no consolida datos de otras instituciones. [Vuelta 2] App concreta: Mi Alemana Go (Clínica Alemana, Chile), con historial desde 2018, recetas, órdenes, familiar vinculado y resultados. [Vuelta 3] Búsqueda de otras clínicas (Las Condes, Santa María, UC Christus) sin ficha de app confirmada; solo canales digitales genéricos. [Vuelta 4] Mi Alemana Go: 3,1/5 con 137 calificaciones (App Store Chile), pantalla de inicio rediseñada para gestionar salud propia y familiar; sin evidencia de teleconsulta ni pagos en la app. [Vuelta 5] Sin búsqueda nueva (revisada en vuelta 4); sin cambios. [Vuelta 6] Sin búsqueda nueva; sin cambios. [Vuelta 7] Sin búsqueda nueva; sin cambios.</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G13" t="n">
@@ -966,7 +966,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -10673,7 +10673,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A31"/>
+  <dimension ref="A1:A32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -10896,6 +10896,13 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Vuelta 7 (iter. 3, 2026-10-19 12:23 UTC): Apple Health, ChatGPT Health, Claude for Healthcare, Apps de clínicas verificados (+0 filas). Pendientes: Clinia, MiRedSalud, Mediko (cierran la vuelta 7 y regeneran func_norm/tabla_frecuencia).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Benchmark: cierre vuelta 7; contador=7; func_norm y tabla_frecuencia regenerados
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MVcXu8vTBu7EKfj3YdEvae
</commit_message>
<xml_diff>
--- a/Outputs/Benchmark_Anamnesis.xlsx
+++ b/Outputs/Benchmark_Anamnesis.xlsx
@@ -518,15 +518,15 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
@@ -558,15 +558,15 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
@@ -598,15 +598,15 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
@@ -638,15 +638,15 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G5" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
@@ -678,15 +678,15 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
@@ -718,15 +718,15 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
@@ -758,15 +758,15 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G8" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
@@ -798,15 +798,15 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G9" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
@@ -838,15 +838,15 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
@@ -878,15 +878,15 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G11" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
@@ -918,15 +918,15 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G12" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
@@ -958,15 +958,15 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G13" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
@@ -993,7 +993,7 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>[DIRECTO · Chile · etapa A] App móvil anunciada en sep-2026 para centralizar recetas, diagnósticos y laboratorios en un solo lugar; respaldada por Reservo (tecnológica chilena desde 2015, software para profesionales y centros de salud). AMENAZA ALTA: Reservo ya tiene red de profesionales/centros que podrían alimentar el historial. Fuente: solo snippet de búsqueda (sitio bloqueado en este entorno); precio, funciones de compartir y sitio oficial por verificar. [Vuelta 2] Confirmado por el CEO de Reservo (LinkedIn): app para pacientes en App Store y Google Play; guarda y comparte exámenes, recetas, órdenes y certificados. Fecha exacta de lanzamiento, precio y modelo de datos sin verificar. [Vuelta 3] Sin novedades de oct-2026. Reservo (Chile, México, Argentina) declara certificación Fonasa/CENS y cumplimiento de la nueva ley de datos personales; el Portal de Agendamiento de Reservo complementa a Clinia. Precio y modelo de datos sin verificar. [Vuelta 4] Una búsqueda adicional no encontró fuentes independientes sobre Clinia de Reservo (aparecen otras empresas llamadas Clinia); la evidencia sigue siendo la publicación del CEO en LinkedIn y notas de Reservo. Confianza media. [Vuelta 5] Sin fecha verificable del lanzamiento (publicación de LinkedIn del CEO sin fecha visible); existe otra empresa homónima en Brasil (Porto Alegre, IA para clínicas) que no es este producto. Sin funciones nuevas. [Vuelta 6] Sin novedades de oct-2026. Reservo declara &gt;36.500 profesionales y centros y ~14 millones de reservas al año (Chile, México, Argentina), sello CENS y certificación Fonasa (autodeclarado); la publicación del CEO pide ideas de nuevas funciones. Sigue sin fecha de lanzamiento verificable.</t>
+          <t>[DIRECTO · Chile · etapa A] App móvil anunciada en sep-2026 para centralizar recetas, diagnósticos y laboratorios en un solo lugar; respaldada por Reservo (tecnológica chilena desde 2015, software para profesionales y centros de salud). AMENAZA ALTA: Reservo ya tiene red de profesionales/centros que podrían alimentar el historial. Fuente: solo snippet de búsqueda (sitio bloqueado en este entorno); precio, funciones de compartir y sitio oficial por verificar. [Vuelta 2] Confirmado por el CEO de Reservo (LinkedIn): app para pacientes en App Store y Google Play; guarda y comparte exámenes, recetas, órdenes y certificados. Fecha exacta de lanzamiento, precio y modelo de datos sin verificar. [Vuelta 3] Sin novedades de oct-2026. Reservo (Chile, México, Argentina) declara certificación Fonasa/CENS y cumplimiento de la nueva ley de datos personales; el Portal de Agendamiento de Reservo complementa a Clinia. Precio y modelo de datos sin verificar. [Vuelta 4] Una búsqueda adicional no encontró fuentes independientes sobre Clinia de Reservo (aparecen otras empresas llamadas Clinia); la evidencia sigue siendo la publicación del CEO en LinkedIn y notas de Reservo. Confianza media. [Vuelta 5] Sin fecha verificable del lanzamiento (publicación de LinkedIn del CEO sin fecha visible); existe otra empresa homónima en Brasil (Porto Alegre, IA para clínicas) que no es este producto. Sin funciones nuevas. [Vuelta 6] Sin novedades de oct-2026. Reservo declara &gt;36.500 profesionales y centros y ~14 millones de reservas al año (Chile, México, Argentina), sello CENS y certificación Fonasa (autodeclarado); la publicación del CEO pide ideas de nuevas funciones. Sigue sin fecha de lanzamiento verificable. [Vuelta 7] Sin novedades; sin datos verificables de descargas ni calificación. Reservo: fundada en 2015 según una fuente (otra indica 2017). No confundir con Clinia de Brasil.</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1002,11 +1002,11 @@
         </is>
       </c>
       <c r="G14" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
@@ -1033,7 +1033,7 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>[SUSTITUTO PARCIAL · Chile] Nueva app móvil de la red RedSalud anunciada dic-2025: acceso a información clínica y servicios, guardar y administrar historial propio y familiar. Limitación: solo datos de la propia red; no consolida otras instituciones. Precio por verificar (probablemente gratis). [Vuelta 2] La búsqueda no encontró fuentes adicionales ni ficha de la app chilena (solo una app RedSalud de otro país); funciones sin confirmar. [Vuelta 3] Rankings de terceros la ubican como app médica gratuita nº 1 en App Store y Google Play Chile (fecha desconocida); sin descripción de funciones ni confirmación del desarrollador en Google Play. [Vuelta 4] Sin documentación oficial chilena localizada; las fichas con funciones (agendar, telemedicina, historial de hijos) corresponden a una app RedSalud de otro país. Quejas públicas 2020-21 sobre acceso en línea a resultados. Funciones de MiRedSalud sin confirmar. [Vuelta 5] Una búsqueda adicional no halló cobertura del lanzamiento de dic-2025 ni de la app chilena; solo apps de otras empresas Red Salud (Paraguay, Perú). Sigue sin confirmarse más allá de la nota de RedSalud. [Vuelta 6] Sin cobertura adicional; los resultados corresponden a la plataforma Red Salud de Paraguay (Interasistencia, ~350 especialistas, call center por WhatsApp), que no es la red chilena. Funciones de MiRedSalud sin confirmar.</t>
+          <t>[SUSTITUTO PARCIAL · Chile] Nueva app móvil de la red RedSalud anunciada dic-2025: acceso a información clínica y servicios, guardar y administrar historial propio y familiar. Limitación: solo datos de la propia red; no consolida otras instituciones. Precio por verificar (probablemente gratis). [Vuelta 2] La búsqueda no encontró fuentes adicionales ni ficha de la app chilena (solo una app RedSalud de otro país); funciones sin confirmar. [Vuelta 3] Rankings de terceros la ubican como app médica gratuita nº 1 en App Store y Google Play Chile (fecha desconocida); sin descripción de funciones ni confirmación del desarrollador en Google Play. [Vuelta 4] Sin documentación oficial chilena localizada; las fichas con funciones (agendar, telemedicina, historial de hijos) corresponden a una app RedSalud de otro país. Quejas públicas 2020-21 sobre acceso en línea a resultados. Funciones de MiRedSalud sin confirmar. [Vuelta 5] Una búsqueda adicional no halló cobertura del lanzamiento de dic-2025 ni de la app chilena; solo apps de otras empresas Red Salud (Paraguay, Perú). Sigue sin confirmarse más allá de la nota de RedSalud. [Vuelta 6] Sin cobertura adicional; los resultados corresponden a la plataforma Red Salud de Paraguay (Interasistencia, ~350 especialistas, call center por WhatsApp), que no es la red chilena. Funciones de MiRedSalud sin confirmar. [Vuelta 7] Sin búsqueda nueva (saturado); sin cambios.</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1042,11 +1042,11 @@
         </is>
       </c>
       <c r="G15" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
@@ -1073,7 +1073,7 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>[ADYACENTE · Chile] Fundada 2022. Orientación médica inmediata, interpretación de exámenes y órdenes médicas digitales con IA; modelo freemium, suscripción y pago por servicio; menciona centralizar registros y monitoreo. Foco asistencial, no archivo personal; vigilar si añade historial. Grants por ~$40M según Descubre.vc. [Vuelta 2] Sin precios ni planes vigentes localizados; sitio oficial bloqueado. [Vuelta 3] Pauta (oct-2024): su fundador, Tomás Riddell, dice que no reemplaza a médicos y apunta a lo ambulatorio y a la espera de derivación a especialidad en el sistema público. Financiamiento: fuentes discrepan (CLP 25M en dic-2023 según Bouncewatch; ~$40M según Descubre.vc). Precios vigentes sin verificar. [Vuelta 4] Entrevista oct-2024 menciona integración con la pasarela Flow. Sin novedades 2025-26 ni rondas verificadas; la cifra de US$40M de Bouncewatch es dudosa (perfil con 2 empleados). [Vuelta 5] CORRECCIÓN de financiamiento: Bouncewatch registra dos subvenciones (CLP 15M en ago-2022 y CLP 25M en dic-2023 = CLP 40M en total), no US$40M; 2 empleados; etapa Seed según Descubre.vc. No hay inversionistas de capital listados. [Vuelta 6] Sin noticias 2026 propias. Contexto: evento «IA y Salud en Chile 2026» (12-may) sobre regulación, datos personales e interoperabilidad de fichas clínicas; Doctoralia lanzó Noa Evidence (jul-2026, asistente de IA para profesionales); programa PRISMA IA 2.0 (dic-2025).</t>
+          <t>[ADYACENTE · Chile] Fundada 2022. Orientación médica inmediata, interpretación de exámenes y órdenes médicas digitales con IA; modelo freemium, suscripción y pago por servicio; menciona centralizar registros y monitoreo. Foco asistencial, no archivo personal; vigilar si añade historial. Grants por ~$40M según Descubre.vc. [Vuelta 2] Sin precios ni planes vigentes localizados; sitio oficial bloqueado. [Vuelta 3] Pauta (oct-2024): su fundador, Tomás Riddell, dice que no reemplaza a médicos y apunta a lo ambulatorio y a la espera de derivación a especialidad en el sistema público. Financiamiento: fuentes discrepan (CLP 25M en dic-2023 según Bouncewatch; ~$40M según Descubre.vc). Precios vigentes sin verificar. [Vuelta 4] Entrevista oct-2024 menciona integración con la pasarela Flow. Sin novedades 2025-26 ni rondas verificadas; la cifra de US$40M de Bouncewatch es dudosa (perfil con 2 empleados). [Vuelta 5] CORRECCIÓN de financiamiento: Bouncewatch registra dos subvenciones (CLP 15M en ago-2022 y CLP 25M en dic-2023 = CLP 40M en total), no US$40M; 2 empleados; etapa Seed según Descubre.vc. No hay inversionistas de capital listados. [Vuelta 6] Sin noticias 2026 propias. Contexto: evento «IA y Salud en Chile 2026» (12-may) sobre regulación, datos personales e interoperabilidad de fichas clínicas; Doctoralia lanzó Noa Evidence (jul-2026, asistente de IA para profesionales); programa PRISMA IA 2.0 (dic-2025). [Vuelta 7] Sigue sin precios publicados de planes; un directorio la describe como gratuita y sin cuenta en su nivel básico (sin verificar).</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1082,11 +1082,11 @@
         </is>
       </c>
       <c r="G16" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
@@ -5348,7 +5348,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E131"/>
+  <dimension ref="A1:E132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -6657,27 +6657,27 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Apps de clínicas (ej. Clínica Alemana de Valdivia)</t>
+          <t>Healfies</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Historial y perfil clínico</t>
+          <t>Gestión documental</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Historial institucional (solo datos de la propia red)</t>
+          <t>Recepción de documentos desde terceros</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Ve historial de esa institución.</t>
+          <t>Desde feb-2016, la administradora de tarjetas ClinCard entregaba contratos y documentos a sus clientes dentro de la plataforma.</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Latam</t>
         </is>
       </c>
     </row>
@@ -6699,7 +6699,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Historial institucional de consultas, urgencias y hospitalizaciones (solo datos de esa clínica).</t>
+          <t>Ve historial de esa institución.</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -6711,7 +6711,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>MiRedSalud (RedSalud)</t>
+          <t>Apps de clínicas (ej. Clínica Alemana de Valdivia)</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -6726,7 +6726,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Acceso a información clínica de la red.</t>
+          <t>Historial institucional de consultas, urgencias y hospitalizaciones (solo datos de esa clínica).</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -6738,7 +6738,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Apple Health (Health Records)</t>
+          <t>MiRedSalud (RedSalud)</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -6748,24 +6748,24 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Historial médico centralizado</t>
+          <t>Historial institucional (solo datos de la propia red)</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Información clínica unificada.</t>
+          <t>Acceso a información clínica de la red.</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Chile</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Clingot</t>
+          <t>Apple Health (Health Records)</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -6780,19 +6780,19 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>El usuario registra sus antecedentes médicos en la app.</t>
+          <t>Información clínica unificada.</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Latam</t>
+          <t>Global</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Infomed</t>
+          <t>Clingot</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -6807,19 +6807,19 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Centraliza el historial médico personal en el móvil.</t>
+          <t>El usuario registra sus antecedentes médicos en la app.</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Latam</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>MediBloc</t>
+          <t>Infomed</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -6834,19 +6834,19 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Permite compilar datos de vida/salud, gestionarlos y pasarlos a instituciones médicas.</t>
+          <t>Centraliza el historial médico personal en el móvil.</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Chile</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Mediko</t>
+          <t>MediBloc</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -6861,19 +6861,19 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Centralizar registros y monitoreo desde el móvil.</t>
+          <t>Permite compilar datos de vida/salud, gestionarlos y pasarlos a instituciones médicas.</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Global</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Healfies</t>
+          <t>Mediko</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -6883,17 +6883,17 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Línea de tiempo de salud</t>
+          <t>Historial médico centralizado</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Línea de tiempo con medicación, exámenes, citas y dieta.</t>
+          <t>Centralizar registros y monitoreo desde el móvil.</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Latam</t>
+          <t>Chile</t>
         </is>
       </c>
     </row>
@@ -6915,7 +6915,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Registra notas de medicación, exámenes (laboratorio e imagen), actividad física, recetas, dieta y citas.</t>
+          <t>Línea de tiempo con medicación, exámenes, citas y dieta.</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -6927,7 +6927,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>MediPlanner</t>
+          <t>Healfies</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -6937,12 +6937,12 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Registro de alergias y vacunas</t>
+          <t>Línea de tiempo de salud</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Registro de alergias y vacunas.</t>
+          <t>Registra notas de medicación, exámenes (laboratorio e imagen), actividad física, recetas, dieta y citas.</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -6954,7 +6954,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Patientory</t>
+          <t>MediPlanner</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -6964,39 +6964,39 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Seguimiento de visitas, gastos y seguros</t>
+          <t>Registro de alergias y vacunas</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>App gratuita para seguir visitas al médico, facturas médicas, datos personales, seguros, inmunizaciones y medicamentos de farmacia.</t>
+          <t>Registro de alergias y vacunas.</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Latam</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>MediBloc</t>
+          <t>Patientory</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Incentivos y monetización de datos</t>
+          <t>Historial y perfil clínico</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Recompensas / monetización de datos del usuario</t>
+          <t>Seguimiento de visitas, gastos y seguros</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Plan de convertir Medipass en superapp con gestión de salud diaria y mercado de datos, integrada con la EMR Dr.Palette.</t>
+          <t>App gratuita para seguir visitas al médico, facturas médicas, datos personales, seguros, inmunizaciones y medicamentos de farmacia.</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -7008,7 +7008,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Medicalchain</t>
+          <t>MediBloc</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -7023,7 +7023,7 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Centros de investigación y farmacéuticas recompensarían con MedTokens a quienes compartan sus datos; no confirmado como ejecutado.</t>
+          <t>Plan de convertir Medipass en superapp con gestión de salud diaria y mercado de datos, integrada con la EMR Dr.Palette.</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -7035,7 +7035,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Patientory</t>
+          <t>Medicalchain</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -7050,7 +7050,7 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>El usuario puede agregar y monetizar sus datos; recompensas en cripto.</t>
+          <t>Centros de investigación y farmacéuticas recompensarían con MedTokens a quienes compartan sus datos; no confirmado como ejecutado.</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -7062,22 +7062,22 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>ChatGPT Health (OpenAI)</t>
+          <t>Patientory</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Inteligencia artificial</t>
+          <t>Incentivos y monetización de datos</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Asistente de IA para profesionales de salud</t>
+          <t>Recompensas / monetización de datos del usuario</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Producto para clínicos verificados de EE.UU. (gratis, abr-2026); desde 1-sep-2026 un plugin con nueve apps de fuentes públicas (investigación, ensayos, medicamentos, Medicare, prestadores), de solo lectura y sin acceso a fichas de pacientes.</t>
+          <t>El usuario puede agregar y monetizar sus datos; recompensas en cripto.</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -7089,7 +7089,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Patientory</t>
+          <t>ChatGPT Health (OpenAI)</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -7099,12 +7099,12 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Coaching de salud con IA</t>
+          <t>Asistente de IA para profesionales de salud</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Coaching personalizado con IA.</t>
+          <t>Producto para clínicos verificados de EE.UU. (gratis, abr-2026); desde 1-sep-2026 un plugin con nueve apps de fuentes públicas (investigación, ensayos, medicamentos, Medicare, prestadores), de solo lectura y sin acceso a fichas de pacientes.</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -7116,7 +7116,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>ChatGPT Health (OpenAI)</t>
+          <t>Patientory</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -7126,12 +7126,12 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Detección de patrones en métricas de salud con IA</t>
+          <t>Coaching de salud con IA</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Interpreta datos de Apple Health y registros en contexto y detecta cambios.</t>
+          <t>Coaching personalizado con IA.</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -7143,7 +7143,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Claude for Healthcare (Anthropic)</t>
+          <t>ChatGPT Health (OpenAI)</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -7158,7 +7158,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Detecta patrones entre métricas de salud y fitness.</t>
+          <t>Interpreta datos de Apple Health y registros en contexto y detecta cambios.</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -7170,7 +7170,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>ChatGPT Health (OpenAI)</t>
+          <t>Claude for Healthcare (Anthropic)</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -7180,12 +7180,12 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Interpretación de exámenes con IA</t>
+          <t>Detección de patrones en métricas de salud con IA</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Explica resultados complejos en lenguaje simple.</t>
+          <t>Detecta patrones entre métricas de salud y fitness.</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -7212,7 +7212,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Desde 28-sep-2026, en la pestaña Health se puede elegir un gráfico, métrica o registro y obtener explicaciones basadas en los datos conectados.</t>
+          <t>Explica resultados complejos en lenguaje simple.</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -7224,7 +7224,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Claude for Healthcare (Anthropic)</t>
+          <t>ChatGPT Health (OpenAI)</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -7239,7 +7239,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Explica exámenes en lenguaje simple.</t>
+          <t>Desde 28-sep-2026, en la pestaña Health se puede elegir un gráfico, métrica o registro y obtener explicaciones basadas en los datos conectados.</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -7251,7 +7251,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Mediko</t>
+          <t>Claude for Healthcare (Anthropic)</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -7266,19 +7266,19 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Interpreta exámenes de laboratorio.</t>
+          <t>Explica exámenes en lenguaje simple.</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Global</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>ChatGPT Health (OpenAI)</t>
+          <t>Mediko</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -7288,24 +7288,24 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Orientación médica con IA</t>
+          <t>Interpretación de exámenes con IA</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Mejora de jun-2026 (GPT-5.5 Instant): detecta cuándo puede requerirse atención urgente, pide contexto y explica la incertidumbre.</t>
+          <t>Interpreta exámenes de laboratorio.</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Chile</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Mediko</t>
+          <t>ChatGPT Health (OpenAI)</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -7320,19 +7320,19 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Orientación médica instantánea mediante IA.</t>
+          <t>Mejora de jun-2026 (GPT-5.5 Instant): detecta cuándo puede requerirse atención urgente, pide contexto y explica la incertidumbre.</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Global</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>ChatGPT Health (OpenAI)</t>
+          <t>Mediko</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -7342,24 +7342,24 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Preparación de consultas médicas con IA</t>
+          <t>Orientación médica con IA</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Prepara preguntas para el médico.</t>
+          <t>Orientación médica instantánea mediante IA.</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Chile</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Claude for Healthcare (Anthropic)</t>
+          <t>ChatGPT Health (OpenAI)</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -7386,7 +7386,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>ChatGPT Health (OpenAI)</t>
+          <t>Claude for Healthcare (Anthropic)</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -7396,12 +7396,12 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Resumen de historial con IA</t>
+          <t>Preparación de consultas médicas con IA</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Resume instrucciones de atención.</t>
+          <t>Prepara preguntas para el médico.</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -7413,7 +7413,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Claude for Healthcare (Anthropic)</t>
+          <t>ChatGPT Health (OpenAI)</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -7428,7 +7428,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Resume el historial del usuario.</t>
+          <t>Resume instrucciones de atención.</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -7440,22 +7440,22 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Apple Health (Health Records)</t>
+          <t>Claude for Healthcare (Anthropic)</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Interoperabilidad y fuentes de datos</t>
+          <t>Inteligencia artificial</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>API para apps de terceros</t>
+          <t>Resumen de historial con IA</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>El usuario decide qué registros recibe cada app y si los nuevos se comparten automáticamente (por defecto pide permiso cada vez); ej. importar recetas a Medisafe.</t>
+          <t>Resume el historial del usuario.</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -7477,12 +7477,12 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Agregación de registros de múltiples instituciones</t>
+          <t>API para apps de terceros</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Vista central de alergias, condiciones, vacunas, laboratorio, medicación, procedimientos y signos vitales.</t>
+          <t>El usuario decide qué registros recibe cada app y si los nuevos se comparten automáticamente (por defecto pide permiso cada vez); ej. importar recetas a Medisafe.</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -7494,7 +7494,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>ChatGPT Health (OpenAI)</t>
+          <t>Apple Health (Health Records)</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -7509,7 +7509,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Conexión de historiales electrónicos y apps como Apple Health, MyFitnessPal, Peloton.</t>
+          <t>Vista central de alergias, condiciones, vacunas, laboratorio, medicación, procedimientos y signos vitales.</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
@@ -7536,7 +7536,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Acceso a historiales electrónicos de proveedores de EE.UU. vía b.well; solo EE.UU., sin plazo anunciado para Latinoamérica.</t>
+          <t>Conexión de historiales electrónicos y apps como Apple Health, MyFitnessPal, Peloton.</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -7563,7 +7563,7 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Además de b.well y Apple Health, vincula registros de One Medical y Function Health (solo EE.UU., Free/Go/Plus/Pro, web e iOS).</t>
+          <t>Acceso a historiales electrónicos de proveedores de EE.UU. vía b.well; solo EE.UU., sin plazo anunciado para Latinoamérica.</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
@@ -7575,7 +7575,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Claude for Healthcare (Anthropic)</t>
+          <t>ChatGPT Health (OpenAI)</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -7590,7 +7590,7 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Acceso a resultados y registros de salud (beta, Pro/Max, EE.UU.).</t>
+          <t>Además de b.well y Apple Health, vincula registros de One Medical y Function Health (solo EE.UU., Free/Go/Plus/Pro, web e iOS).</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -7602,7 +7602,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Clinia (Reservo)</t>
+          <t>Claude for Healthcare (Anthropic)</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -7617,19 +7617,19 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Datos desde profesionales/centros que usan Reservo (fichas clínicas, agenda, telemedicina).</t>
+          <t>Acceso a resultados y registros de salud (beta, Pro/Max, EE.UU.).</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Global</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>MediBloc</t>
+          <t>Clinia (Reservo)</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -7644,19 +7644,19 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Tras autenticación simple, trae los últimos 3 años de historial de hospitales integrados (p. ej. Samsung Seoul, SNUH, Severance).</t>
+          <t>Datos desde profesionales/centros que usan Reservo (fichas clínicas, agenda, telemedicina).</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Chile</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Meedika</t>
+          <t>MediBloc</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -7671,19 +7671,19 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Sincroniza resultados desde centros de salud y permite subir fotos o documentos de las solicitudes médicas.</t>
+          <t>Tras autenticación simple, trae los últimos 3 años de historial de hospitales integrados (p. ej. Samsung Seoul, SNUH, Severance).</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Global</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Patientory</t>
+          <t>Meedika</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -7698,12 +7698,12 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Reúne registros de hospitales, resultados de laboratorio y datos genómicos.</t>
+          <t>Sincroniza resultados desde centros de salud y permite subir fotos o documentos de las solicitudes médicas.</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Chile</t>
         </is>
       </c>
     </row>
@@ -7720,12 +7720,12 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Analítica poblacional B2B</t>
+          <t>Agregación de registros de múltiples instituciones</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Analítica poblacional on-chain; integrada con Epic, Cerner, Meditech y Allscripts (B2B).</t>
+          <t>Reúne registros de hospitales, resultados de laboratorio y datos genómicos.</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
@@ -7737,7 +7737,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Clingot</t>
+          <t>Patientory</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -7747,24 +7747,24 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Disponibilidad multiplataforma (web/iOS/Android)</t>
+          <t>Analítica poblacional B2B</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Android, iOS y escritorio; médicos acceden a historias digitalizadas, envían estudios e indicaciones y organizan agenda.</t>
+          <t>Analítica poblacional on-chain; integrada con Epic, Cerner, Meditech y Allscripts (B2B).</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Latam</t>
+          <t>Global</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Clinia (Reservo)</t>
+          <t>Clingot</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -7779,19 +7779,19 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Disponible en App Store y Google Play. Reservo opera en Chile, México y Argentina y está certificada por FONASA y CENS.</t>
+          <t>Android, iOS y escritorio; médicos acceden a historias digitalizadas, envían estudios e indicaciones y organizan agenda.</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Latam</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Healfies</t>
+          <t>Clinia (Reservo)</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -7806,19 +7806,19 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Disponible en web, iOS y Android.</t>
+          <t>Disponible en App Store y Google Play. Reservo opera en Chile, México y Argentina y está certificada por FONASA y CENS.</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Latam</t>
+          <t>Chile</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Medicalchain</t>
+          <t>Healfies</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -7828,24 +7828,24 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Historial médico centralizado</t>
+          <t>Disponibilidad multiplataforma (web/iOS/Android)</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Versión digital de los registros con acceso por móvil o web.</t>
+          <t>Disponible en web, iOS y Android.</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Latam</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>MediPlanner</t>
+          <t>Medicalchain</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -7855,24 +7855,24 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Importación y exportación de datos</t>
+          <t>Historial médico centralizado</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Importar/exportar datos para compartir de forma segura con familias o cuidadores. Es MediPlanner Pro, de otro desarrollador (App Store MX, $39 MXN).</t>
+          <t>Versión digital de los registros con acceso por móvil o web.</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Latam</t>
+          <t>Global</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Medicalchain</t>
+          <t>MediPlanner</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -7882,24 +7882,24 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Integración con EHR de proveedores</t>
+          <t>Importación y exportación de datos</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Según una AMA sin fecha, integraba dos sistemas de GP que cubren ~80% del mercado UK; no confirmado como ejecutado.</t>
+          <t>Importar/exportar datos para compartir de forma segura con familias o cuidadores. Es MediPlanner Pro, de otro desarrollador (App Store MX, $39 MXN).</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Latam</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Claude for Healthcare (Anthropic)</t>
+          <t>Medicalchain</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -7909,12 +7909,12 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Integración con wearables y apps de salud</t>
+          <t>Integración con EHR de proveedores</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Integración beta en apps iOS/Android.</t>
+          <t>Según una AMA sin fecha, integraba dos sistemas de GP que cubren ~80% del mercado UK; no confirmado como ejecutado.</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
@@ -7941,7 +7941,7 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Integración beta con Health Connect en la app móvil; conectores de registros (HealthEx, Function) solo para Pro/Max en EE.UU.</t>
+          <t>Integración beta en apps iOS/Android.</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
@@ -7953,7 +7953,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Patientory</t>
+          <t>Claude for Healthcare (Anthropic)</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -7968,7 +7968,7 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Se integra con wearables y apps móviles populares y muestra vitales en un panel unificado.</t>
+          <t>Integración beta con Health Connect en la app móvil; conectores de registros (HealthEx, Function) solo para Pro/Max en EE.UU.</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
@@ -7980,22 +7980,22 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Apple Health (Health Records)</t>
+          <t>Patientory</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Medicación y recordatorios</t>
+          <t>Interoperabilidad y fuentes de datos</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Gestión de lista de medicamentos</t>
+          <t>Integración con wearables y apps de salud</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Listas de medicamentos, vitaminas y suplementos con horarios; escaneo de etiqueta del frasco solo en EE.UU.</t>
+          <t>Se integra con wearables y apps móviles populares y muestra vitales en un panel unificado.</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
@@ -8007,7 +8007,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>MediPlanner</t>
+          <t>Apple Health (Health Records)</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -8017,24 +8017,24 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Importación automática de tratamientos desde receta digital</t>
+          <t>Gestión de lista de medicamentos</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Según la ficha de la App Store MX, los tratamientos llegan automáticamente desde la receta digital del médico (autodeclarado, sin verificar).</t>
+          <t>Listas de medicamentos, vitaminas y suplementos con horarios; escaneo de etiqueta del frasco solo en EE.UU.</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Latam</t>
+          <t>Global</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Apple Health (Health Records)</t>
+          <t>MediPlanner</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -8044,24 +8044,24 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Recordatorios de medicación y citas</t>
+          <t>Importación automática de tratamientos desde receta digital</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Recordatorios desde el app.</t>
+          <t>Según la ficha de la App Store MX, los tratamientos llegan automáticamente desde la receta digital del médico (autodeclarado, sin verificar).</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Latam</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Meedika</t>
+          <t>Apple Health (Health Records)</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -8076,19 +8076,19 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Recordatorios de citas/medicación.</t>
+          <t>Recordatorios desde el app.</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Global</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>MediPlanner</t>
+          <t>Meedika</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -8098,51 +8098,51 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Registro de tomas y adherencia al tratamiento</t>
+          <t>Recordatorios de medicación y citas</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Registro de cada toma y control de adherencia; gestiona medicamentos propios y de familiares.</t>
+          <t>Recordatorios de citas/medicación.</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Latam</t>
+          <t>Chile</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Patientory</t>
+          <t>MediPlanner</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Seguimiento y bienestar</t>
+          <t>Medicación y recordatorios</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Comunidad de pacientes</t>
+          <t>Registro de tomas y adherencia al tratamiento</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Los usuarios con condiciones similares pueden preguntar, recibir recomendaciones y compartir experiencias.</t>
+          <t>Registro de cada toma y control de adherencia; gestiona medicamentos propios y de familiares.</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Latam</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Infomed</t>
+          <t>Patientory</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -8152,24 +8152,24 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Contenido educativo sobre salud</t>
+          <t>Comunidad de pacientes</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Busca que el paciente aprenda sobre sus enfermedades y sea más autónomo.</t>
+          <t>Los usuarios con condiciones similares pueden preguntar, recibir recomendaciones y compartir experiencias.</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Global</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>MediPlanner</t>
+          <t>Infomed</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -8179,24 +8179,24 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Gráficas de evolución de indicadores</t>
+          <t>Contenido educativo sobre salud</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Gráficas de evolución de indicadores de salud.</t>
+          <t>Busca que el paciente aprenda sobre sus enfermedades y sea más autónomo.</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Latam</t>
+          <t>Chile</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Apple Health (Health Records)</t>
+          <t>MediPlanner</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -8206,24 +8206,24 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Integración con wearables y apps de salud</t>
+          <t>Gráficas de evolución de indicadores</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Datos de pasos, sueño, peso junto a registros.</t>
+          <t>Gráficas de evolución de indicadores de salud.</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Latam</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>MediBloc</t>
+          <t>Apple Health (Health Records)</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -8233,12 +8233,12 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Panel de seguimiento de salud y bienestar</t>
+          <t>Integración con wearables y apps de salud</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>El relanzamiento de Medipass (mar-2023) agregó un panel para gestionar la información de salud del usuario.</t>
+          <t>Datos de pasos, sueño, peso junto a registros.</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
@@ -8250,7 +8250,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Patientory</t>
+          <t>MediBloc</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -8265,7 +8265,7 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Seguimiento de hábitos saludables y monitoreo de progreso.</t>
+          <t>El relanzamiento de Medipass (mar-2023) agregó un panel para gestionar la información de salud del usuario.</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
@@ -8277,7 +8277,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Apple Health (Health Records)</t>
+          <t>Patientory</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -8287,12 +8287,12 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Registro de nutrición</t>
+          <t>Panel de seguimiento de salud y bienestar</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Escaneo de etiquetas nutricionales con la cámara; según un análisis, no escribe en HealthKit.</t>
+          <t>Seguimiento de hábitos saludables y monitoreo de progreso.</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
@@ -8314,12 +8314,12 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Seguimiento de salud femenina</t>
+          <t>Registro de nutrición</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Extiende el seguimiento de ciclo con perimenopausia y menopausia.</t>
+          <t>Escaneo de etiquetas nutricionales con la cámara; según un análisis, no escribe en HealthKit.</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
@@ -8331,7 +8331,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Clingot</t>
+          <t>Apple Health (Health Records)</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -8341,51 +8341,51 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Valoración de profesionales</t>
+          <t>Seguimiento de salud femenina</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Calificación de la atención de profesionales con autorización previa, compartible con otros usuarios.</t>
+          <t>Extiende el seguimiento de ciclo con perimenopausia y menopausia.</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>Latam</t>
+          <t>Global</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Claude for Healthcare (Anthropic)</t>
+          <t>Clingot</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Seguridad, privacidad y blockchain</t>
+          <t>Seguimiento y bienestar</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Acceso mínimo por categorías de datos</t>
+          <t>Valoración de profesionales</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Claude solicita solo las categorías relevantes (p. ej. medicamentos o laboratorio) y no fichas completas; HealthEx agrega datos de más de 50.000 sistemas de salud de EE.UU.</t>
+          <t>Calificación de la atención de profesionales con autorización previa, compartible con otros usuarios.</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Latam</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>MediBloc</t>
+          <t>Claude for Healthcare (Anthropic)</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -8395,12 +8395,12 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Blockchain para integridad y trazabilidad de datos</t>
+          <t>Acceso mínimo por categorías de datos</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Blockchain propia (Cosmos SDK) para que el paciente almacene, use, actualice y transfiera sus registros; los datos no se guardan en la cadena, solo en el usuario, cifrados.</t>
+          <t>Claude solicita solo las categorías relevantes (p. ej. medicamentos o laboratorio) y no fichas completas; HealthEx agrega datos de más de 50.000 sistemas de salud de EE.UU.</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
@@ -8427,7 +8427,7 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Almacena huellas de datos médicos en un registro de solo escritura, sin guardar datos clínicos en cadena.</t>
+          <t>Blockchain propia (Cosmos SDK) para que el paciente almacene, use, actualice y transfiera sus registros; los datos no se guardan en la cadena, solo en el usuario, cifrados.</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
@@ -8439,7 +8439,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Medicalchain</t>
+          <t>MediBloc</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -8454,7 +8454,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Cada solicitud de acceso queda en un libro distribuido; acceso temporal por contratos inteligentes.</t>
+          <t>Almacena huellas de datos médicos en un registro de solo escritura, sin guardar datos clínicos en cadena.</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
@@ -8466,7 +8466,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Patientory</t>
+          <t>Medicalchain</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -8481,7 +8481,7 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Registro respaldado en blockchain para seguridad y trazabilidad.</t>
+          <t>Cada solicitud de acceso queda en un libro distribuido; acceso temporal por contratos inteligentes.</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
@@ -8493,7 +8493,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Apple Health (Health Records)</t>
+          <t>Patientory</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -8503,12 +8503,12 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Cifrado y control de acceso</t>
+          <t>Blockchain para integridad y trazabilidad de datos</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Registros cifrados en el dispositivo, protegidos por Face ID/Touch ID/código.</t>
+          <t>Registro respaldado en blockchain para seguridad y trazabilidad.</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
@@ -8520,7 +8520,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Infomed</t>
+          <t>Apple Health (Health Records)</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -8535,19 +8535,19 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Almacenamiento seguro del historial con criterios de seguridad estrictos, comparable a apps bancarias.</t>
+          <t>Registros cifrados en el dispositivo, protegidos por Face ID/Touch ID/código.</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Global</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Clinia (Reservo)</t>
+          <t>Infomed</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -8557,12 +8557,12 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Cumplimiento regulatorio de salud y datos</t>
+          <t>Cifrado y control de acceso</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Reservo declara plataforma certificada por Fonasa y CENS, cumplimiento de estándares de telemedicina del Minsal y de la nueva ley chilena de datos personales (declaración de la empresa).</t>
+          <t>Almacenamiento seguro del historial con criterios de seguridad estrictos, comparable a apps bancarias.</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
@@ -8574,7 +8574,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>ChatGPT Health (OpenAI)</t>
+          <t>Clinia (Reservo)</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -8584,24 +8584,24 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Gestión de consentimiento sobre uso de datos</t>
+          <t>Cumplimiento regulatorio de salud y datos</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>Desde 14-sep-2026, las nuevas conexiones heredan la configuración global de plugins: ChatGPT puede usar datos de Health sin pedir permiso cada vez salvo acciones sensibles (web primero, móvil después).</t>
+          <t>Reservo declara plataforma certificada por Fonasa y CENS, cumplimiento de estándares de telemedicina del Minsal y de la nueva ley chilena de datos personales (declaración de la empresa).</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Chile</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>MediBloc</t>
+          <t>ChatGPT Health (OpenAI)</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -8611,12 +8611,12 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Identidad descentralizada (DID)</t>
+          <t>Gestión de consentimiento sobre uso de datos</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>Gestión de identificadores descentralizados en Panacea.</t>
+          <t>Desde 14-sep-2026, las nuevas conexiones heredan la configuración global de plugins: ChatGPT puede usar datos de Health sin pedir permiso cada vez salvo acciones sensibles (web primero, móvil después).</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
@@ -8628,7 +8628,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>ChatGPT Health (OpenAI)</t>
+          <t>MediBloc</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -8638,12 +8638,12 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Privacidad reforzada para datos de salud</t>
+          <t>Identidad descentralizada (DID)</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Chats y memoria de salud separados, no usados para entrenar modelos.</t>
+          <t>Gestión de identificadores descentralizados en Panacea.</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
@@ -8655,7 +8655,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Claude for Healthcare (Anthropic)</t>
+          <t>ChatGPT Health (OpenAI)</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -8670,7 +8670,7 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>El usuario activa y revoca permisos; los datos de salud compartidos se excluyen de la memoria de Claude y del entrenamiento.</t>
+          <t>Chats y memoria de salud separados, no usados para entrenar modelos.</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
@@ -8682,34 +8682,34 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>Mediko</t>
+          <t>Claude for Healthcare (Anthropic)</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>Seguros y pagos</t>
+          <t>Seguridad, privacidad y blockchain</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Modelo freemium y suscripción</t>
+          <t>Privacidad reforzada para datos de salud</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Planes para personas y empresas.</t>
+          <t>El usuario activa y revoca permisos; los datos de salud compartidos se excluyen de la memoria de Claude y del entrenamiento.</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Global</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>Medicalchain</t>
+          <t>Mediko</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -8719,17 +8719,17 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Pagos con criptomoneda</t>
+          <t>Modelo freemium y suscripción</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Pago de consultas con token.</t>
+          <t>Planes para personas y empresas.</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Chile</t>
         </is>
       </c>
     </row>
@@ -8751,7 +8751,7 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>Piloto en New Malden (Londres): consultas por video pagables con tarjeta o con MedTokens.</t>
+          <t>Pago de consultas con token.</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
@@ -8763,7 +8763,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>Mediko</t>
+          <t>Medicalchain</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -8773,24 +8773,24 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Pagos dentro de la app</t>
+          <t>Pagos con criptomoneda</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Pagos dentro de la plataforma mediante la pasarela Flow (según resumen de entrevista de Pauta, oct-2024; esperada para mejorar la experiencia).</t>
+          <t>Piloto en New Malden (Londres): consultas por video pagables con tarjeta o con MedTokens.</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Global</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>MediBloc</t>
+          <t>Mediko</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -8800,17 +8800,17 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Reclamos y trámites con seguros</t>
+          <t>Pagos dentro de la app</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>Simplifica el envío a aseguradoras sin gestionar papeles en hospitales.</t>
+          <t>Pagos dentro de la plataforma mediante la pasarela Flow (según resumen de entrevista de Pauta, oct-2024; esperada para mejorar la experiencia).</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Chile</t>
         </is>
       </c>
     </row>
@@ -8832,7 +8832,7 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Reclamo de seguro médico (indemnización) desde la app, con verificación de autenticidad de los registros vía blockchain por la aseguradora.</t>
+          <t>Simplifica el envío a aseguradoras sin gestionar papeles en hospitales.</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
@@ -8849,17 +8849,17 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>Telemedicina y atención remota</t>
+          <t>Seguros y pagos</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>Mensajería paciente-institución</t>
+          <t>Reclamos y trámites con seguros</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>Chat para consultas a hospitales, orientación simple de síntomas e información de tratamientos; comunicación bidireccional hospital-paciente (nov-2023).</t>
+          <t>Reclamo de seguro médico (indemnización) desde la app, con verificación de autenticidad de los registros vía blockchain por la aseguradora.</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
@@ -8871,25 +8871,52 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
+          <t>MediBloc</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Telemedicina y atención remota</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Mensajería paciente-institución</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>Chat para consultas a hospitales, orientación simple de síntomas e información de tratamientos; comunicación bidireccional hospital-paciente (nov-2023).</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
           <t>Medicalchain</t>
         </is>
       </c>
-      <c r="B131" t="inlineStr">
+      <c r="B132" t="inlineStr">
         <is>
           <t>Telemedicina y atención remota</t>
         </is>
       </c>
-      <c r="C131" t="inlineStr">
+      <c r="C132" t="inlineStr">
         <is>
           <t>Teleconsulta con profesionales</t>
         </is>
       </c>
-      <c r="D131" t="inlineStr">
+      <c r="D132" t="inlineStr">
         <is>
           <t>Teleconsultas con GP.</t>
         </is>
       </c>
-      <c r="E131" t="inlineStr">
+      <c r="E132" t="inlineStr">
         <is>
           <t>Global</t>
         </is>
@@ -8906,7 +8933,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R67"/>
+  <dimension ref="A1:R68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9032,6 +9059,8 @@
           <t>Búsqueda de profesionales de salud</t>
         </is>
       </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9042,6 +9071,17 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr"/>
       <c r="R2">
         <f>COUNTIF(C2:Q2,"✓")</f>
         <v/>
@@ -9063,11 +9103,24 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr"/>
       <c r="R3">
         <f>COUNTIF(C3:Q3,"✓")</f>
         <v/>
@@ -9084,11 +9137,25 @@
           <t>Integración con calendario del dispositivo</t>
         </is>
       </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr"/>
       <c r="R4">
         <f>COUNTIF(C4:Q4,"✓")</f>
         <v/>
@@ -9105,11 +9172,25 @@
           <t>Localización de centros médicos y farmacias</t>
         </is>
       </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr"/>
       <c r="R5">
         <f>COUNTIF(C5:Q5,"✓")</f>
         <v/>
@@ -9126,11 +9207,21 @@
           <t>Reserva de citas médicas</t>
         </is>
       </c>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9141,6 +9232,8 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr"/>
       <c r="R6">
         <f>COUNTIF(C6:Q6,"✓")</f>
         <v/>
@@ -9157,11 +9250,25 @@
           <t>Acceso del profesional al historial del paciente</t>
         </is>
       </c>
+      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr"/>
+      <c r="Q7" t="inlineStr"/>
       <c r="R7">
         <f>COUNTIF(C7:Q7,"✓")</f>
         <v/>
@@ -9178,11 +9285,25 @@
           <t>Compartir con personas sin cuenta mediante clave segura</t>
         </is>
       </c>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr"/>
+      <c r="Q8" t="inlineStr"/>
       <c r="R8">
         <f>COUNTIF(C8:Q8,"✓")</f>
         <v/>
@@ -9199,11 +9320,25 @@
           <t>Compartir datos con cuidador o persona de confianza</t>
         </is>
       </c>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr"/>
+      <c r="Q9" t="inlineStr"/>
       <c r="R9">
         <f>COUNTIF(C9:Q9,"✓")</f>
         <v/>
@@ -9225,11 +9360,13 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9255,11 +9392,16 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
       <c r="O10" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="P10" t="inlineStr"/>
+      <c r="Q10" t="inlineStr"/>
       <c r="R10">
         <f>COUNTIF(C10:Q10,"✓")</f>
         <v/>
@@ -9276,11 +9418,25 @@
           <t>Gestión de consentimiento sobre uso de datos</t>
         </is>
       </c>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr"/>
       <c r="R11">
         <f>COUNTIF(C11:Q11,"✓")</f>
         <v/>
@@ -9297,11 +9453,25 @@
           <t>Ingreso de datos por profesional con consentimiento</t>
         </is>
       </c>
+      <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr"/>
+      <c r="Q12" t="inlineStr"/>
       <c r="R12">
         <f>COUNTIF(C12:Q12,"✓")</f>
         <v/>
@@ -9318,11 +9488,25 @@
           <t>Red social con profesionales y familiares</t>
         </is>
       </c>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr"/>
+      <c r="Q13" t="inlineStr"/>
       <c r="R13">
         <f>COUNTIF(C13:Q13,"✓")</f>
         <v/>
@@ -9349,11 +9533,23 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr"/>
+      <c r="O14" t="inlineStr"/>
+      <c r="P14" t="inlineStr"/>
+      <c r="Q14" t="inlineStr"/>
       <c r="R14">
         <f>COUNTIF(C14:Q14,"✓")</f>
         <v/>
@@ -9370,6 +9566,8 @@
           <t>Perfiles familiares / dependientes</t>
         </is>
       </c>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9380,21 +9578,29 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr"/>
       <c r="N15" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="Q15" t="inlineStr"/>
       <c r="R15">
         <f>COUNTIF(C15:Q15,"✓")</f>
         <v/>
@@ -9416,6 +9622,8 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9431,11 +9639,19 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="inlineStr"/>
       <c r="O16" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="P16" t="inlineStr"/>
+      <c r="Q16" t="inlineStr"/>
       <c r="R16">
         <f>COUNTIF(C16:Q16,"✓")</f>
         <v/>
@@ -9452,16 +9668,29 @@
           <t>Almacenamiento de recetas</t>
         </is>
       </c>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr"/>
       <c r="N17" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="O17" t="inlineStr"/>
+      <c r="P17" t="inlineStr"/>
+      <c r="Q17" t="inlineStr"/>
       <c r="R17">
         <f>COUNTIF(C17:Q17,"✓")</f>
         <v/>
@@ -9478,11 +9707,25 @@
           <t>Búsqueda y filtros de documentos</t>
         </is>
       </c>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="inlineStr"/>
+      <c r="O18" t="inlineStr"/>
+      <c r="P18" t="inlineStr"/>
+      <c r="Q18" t="inlineStr"/>
       <c r="R18">
         <f>COUNTIF(C18:Q18,"✓")</f>
         <v/>
@@ -9499,11 +9742,25 @@
           <t>Emisión de certificados médicos</t>
         </is>
       </c>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="inlineStr"/>
+      <c r="O19" t="inlineStr"/>
+      <c r="P19" t="inlineStr"/>
+      <c r="Q19" t="inlineStr"/>
       <c r="R19">
         <f>COUNTIF(C19:Q19,"✓")</f>
         <v/>
@@ -9525,6 +9782,19 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="inlineStr"/>
+      <c r="O20" t="inlineStr"/>
+      <c r="P20" t="inlineStr"/>
       <c r="Q20" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9546,11 +9816,25 @@
           <t>Notificación y envío de resultados</t>
         </is>
       </c>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr"/>
       <c r="N21" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="O21" t="inlineStr"/>
+      <c r="P21" t="inlineStr"/>
+      <c r="Q21" t="inlineStr"/>
       <c r="R21">
         <f>COUNTIF(C21:Q21,"✓")</f>
         <v/>
@@ -9559,24 +9843,33 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Historial y perfil clínico</t>
+          <t>Gestión documental</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Historial institucional (solo datos de la propia red)</t>
-        </is>
-      </c>
-      <c r="N22" t="inlineStr">
+          <t>Recepción de documentos desde terceros</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="P22" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr"/>
+      <c r="N22" t="inlineStr"/>
+      <c r="O22" t="inlineStr"/>
+      <c r="P22" t="inlineStr"/>
+      <c r="Q22" t="inlineStr"/>
       <c r="R22">
         <f>COUNTIF(C22:Q22,"✓")</f>
         <v/>
@@ -9590,34 +9883,32 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Historial médico centralizado</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
+          <t>Historial institucional (solo datos de la propia red)</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr"/>
+      <c r="N23" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
+      <c r="O23" t="inlineStr"/>
+      <c r="P23" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="Q23" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="Q23" t="inlineStr"/>
       <c r="R23">
         <f>COUNTIF(C23:Q23,"✓")</f>
         <v/>
@@ -9631,10 +9922,40 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Línea de tiempo de salud</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
+          <t>Historial médico centralizado</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="inlineStr"/>
+      <c r="O24" t="inlineStr"/>
+      <c r="P24" t="inlineStr"/>
+      <c r="Q24" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -9652,14 +9973,28 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Registro de alergias y vacunas</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
+          <t>Línea de tiempo de salud</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" t="inlineStr"/>
+      <c r="O25" t="inlineStr"/>
+      <c r="P25" t="inlineStr"/>
+      <c r="Q25" t="inlineStr"/>
       <c r="R25">
         <f>COUNTIF(C25:Q25,"✓")</f>
         <v/>
@@ -9673,14 +10008,28 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Seguimiento de visitas, gastos y seguros</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
+          <t>Registro de alergias y vacunas</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" t="inlineStr"/>
+      <c r="O26" t="inlineStr"/>
+      <c r="P26" t="inlineStr"/>
+      <c r="Q26" t="inlineStr"/>
       <c r="R26">
         <f>COUNTIF(C26:Q26,"✓")</f>
         <v/>
@@ -9689,29 +10038,33 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Incentivos y monetización de datos</t>
+          <t>Historial y perfil clínico</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Recompensas / monetización de datos del usuario</t>
-        </is>
-      </c>
+          <t>Seguimiento de visitas, gastos y seguros</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr"/>
+      <c r="N27" t="inlineStr"/>
+      <c r="O27" t="inlineStr"/>
+      <c r="P27" t="inlineStr"/>
+      <c r="Q27" t="inlineStr"/>
       <c r="R27">
         <f>COUNTIF(C27:Q27,"✓")</f>
         <v/>
@@ -9720,19 +10073,41 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Inteligencia artificial</t>
+          <t>Incentivos y monetización de datos</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Asistente de IA para profesionales de salud</t>
-        </is>
-      </c>
-      <c r="L28" t="inlineStr">
+          <t>Recompensas / monetización de datos del usuario</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr"/>
+      <c r="N28" t="inlineStr"/>
+      <c r="O28" t="inlineStr"/>
+      <c r="P28" t="inlineStr"/>
+      <c r="Q28" t="inlineStr"/>
       <c r="R28">
         <f>COUNTIF(C28:Q28,"✓")</f>
         <v/>
@@ -9746,14 +10121,28 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Coaching de salud con IA</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
+          <t>Asistente de IA para profesionales de salud</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr"/>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr"/>
+      <c r="L29" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="M29" t="inlineStr"/>
+      <c r="N29" t="inlineStr"/>
+      <c r="O29" t="inlineStr"/>
+      <c r="P29" t="inlineStr"/>
+      <c r="Q29" t="inlineStr"/>
       <c r="R29">
         <f>COUNTIF(C29:Q29,"✓")</f>
         <v/>
@@ -9767,19 +10156,28 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Detección de patrones en métricas de salud con IA</t>
-        </is>
-      </c>
-      <c r="L30" t="inlineStr">
+          <t>Coaching de salud con IA</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="M30" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
+      <c r="L30" t="inlineStr"/>
+      <c r="M30" t="inlineStr"/>
+      <c r="N30" t="inlineStr"/>
+      <c r="O30" t="inlineStr"/>
+      <c r="P30" t="inlineStr"/>
+      <c r="Q30" t="inlineStr"/>
       <c r="R30">
         <f>COUNTIF(C30:Q30,"✓")</f>
         <v/>
@@ -9793,9 +10191,18 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Interpretación de exámenes con IA</t>
-        </is>
-      </c>
+          <t>Detección de patrones en métricas de salud con IA</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9806,11 +10213,10 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Q31" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="N31" t="inlineStr"/>
+      <c r="O31" t="inlineStr"/>
+      <c r="P31" t="inlineStr"/>
+      <c r="Q31" t="inlineStr"/>
       <c r="R31">
         <f>COUNTIF(C31:Q31,"✓")</f>
         <v/>
@@ -9824,14 +10230,31 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Orientación médica con IA</t>
-        </is>
-      </c>
+          <t>Interpretación de exámenes con IA</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr"/>
+      <c r="O32" t="inlineStr"/>
+      <c r="P32" t="inlineStr"/>
       <c r="Q32" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9850,15 +10273,28 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Preparación de consultas médicas con IA</t>
-        </is>
-      </c>
+          <t>Orientación médica con IA</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="M33" t="inlineStr">
+      <c r="M33" t="inlineStr"/>
+      <c r="N33" t="inlineStr"/>
+      <c r="O33" t="inlineStr"/>
+      <c r="P33" t="inlineStr"/>
+      <c r="Q33" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -9876,9 +10312,18 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Resumen de historial con IA</t>
-        </is>
-      </c>
+          <t>Preparación de consultas médicas con IA</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="inlineStr"/>
+      <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9889,6 +10334,10 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="N34" t="inlineStr"/>
+      <c r="O34" t="inlineStr"/>
+      <c r="P34" t="inlineStr"/>
+      <c r="Q34" t="inlineStr"/>
       <c r="R34">
         <f>COUNTIF(C34:Q34,"✓")</f>
         <v/>
@@ -9897,19 +10346,37 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Interoperabilidad y fuentes de datos</t>
+          <t>Inteligencia artificial</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>API para apps de terceros</t>
-        </is>
-      </c>
-      <c r="K35" t="inlineStr">
+          <t>Resumen de historial con IA</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr"/>
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr"/>
+      <c r="L35" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr"/>
+      <c r="O35" t="inlineStr"/>
+      <c r="P35" t="inlineStr"/>
+      <c r="Q35" t="inlineStr"/>
       <c r="R35">
         <f>COUNTIF(C35:Q35,"✓")</f>
         <v/>
@@ -9923,44 +10390,28 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Agregación de registros de múltiples instituciones</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
+          <t>API para apps de terceros</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr"/>
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="inlineStr"/>
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="inlineStr"/>
+      <c r="J36" t="inlineStr"/>
+      <c r="K36" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="I36" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="K36" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="L36" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="M36" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="O36" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="L36" t="inlineStr"/>
+      <c r="M36" t="inlineStr"/>
+      <c r="N36" t="inlineStr"/>
+      <c r="O36" t="inlineStr"/>
+      <c r="P36" t="inlineStr"/>
+      <c r="Q36" t="inlineStr"/>
       <c r="R36">
         <f>COUNTIF(C36:Q36,"✓")</f>
         <v/>
@@ -9974,14 +10425,52 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Analítica poblacional B2B</t>
-        </is>
-      </c>
+          <t>Agregación de registros de múltiples instituciones</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr"/>
+      <c r="E37" t="inlineStr"/>
+      <c r="F37" t="inlineStr"/>
+      <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr"/>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr"/>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr"/>
+      <c r="Q37" t="inlineStr"/>
       <c r="R37">
         <f>COUNTIF(C37:Q37,"✓")</f>
         <v/>
@@ -9995,24 +10484,28 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Disponibilidad multiplataforma (web/iOS/Android)</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr">
+          <t>Analítica poblacional B2B</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr"/>
+      <c r="D38" t="inlineStr"/>
+      <c r="E38" t="inlineStr"/>
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" t="inlineStr"/>
+      <c r="H38" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="O38" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="I38" t="inlineStr"/>
+      <c r="J38" t="inlineStr"/>
+      <c r="K38" t="inlineStr"/>
+      <c r="L38" t="inlineStr"/>
+      <c r="M38" t="inlineStr"/>
+      <c r="N38" t="inlineStr"/>
+      <c r="O38" t="inlineStr"/>
+      <c r="P38" t="inlineStr"/>
+      <c r="Q38" t="inlineStr"/>
       <c r="R38">
         <f>COUNTIF(C38:Q38,"✓")</f>
         <v/>
@@ -10026,14 +10519,36 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Historial médico centralizado</t>
-        </is>
-      </c>
-      <c r="J39" t="inlineStr">
+          <t>Disponibilidad multiplataforma (web/iOS/Android)</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr"/>
+      <c r="D39" t="inlineStr"/>
+      <c r="E39" t="inlineStr"/>
+      <c r="F39" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr"/>
+      <c r="J39" t="inlineStr"/>
+      <c r="K39" t="inlineStr"/>
+      <c r="L39" t="inlineStr"/>
+      <c r="M39" t="inlineStr"/>
+      <c r="N39" t="inlineStr"/>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr"/>
+      <c r="Q39" t="inlineStr"/>
       <c r="R39">
         <f>COUNTIF(C39:Q39,"✓")</f>
         <v/>
@@ -10047,14 +10562,28 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Importación y exportación de datos</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
+          <t>Historial médico centralizado</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr"/>
+      <c r="D40" t="inlineStr"/>
+      <c r="E40" t="inlineStr"/>
+      <c r="F40" t="inlineStr"/>
+      <c r="G40" t="inlineStr"/>
+      <c r="H40" t="inlineStr"/>
+      <c r="I40" t="inlineStr"/>
+      <c r="J40" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="K40" t="inlineStr"/>
+      <c r="L40" t="inlineStr"/>
+      <c r="M40" t="inlineStr"/>
+      <c r="N40" t="inlineStr"/>
+      <c r="O40" t="inlineStr"/>
+      <c r="P40" t="inlineStr"/>
+      <c r="Q40" t="inlineStr"/>
       <c r="R40">
         <f>COUNTIF(C40:Q40,"✓")</f>
         <v/>
@@ -10068,14 +10597,28 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Integración con EHR de proveedores</t>
-        </is>
-      </c>
-      <c r="J41" t="inlineStr">
+          <t>Importación y exportación de datos</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr"/>
+      <c r="D41" t="inlineStr"/>
+      <c r="E41" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="F41" t="inlineStr"/>
+      <c r="G41" t="inlineStr"/>
+      <c r="H41" t="inlineStr"/>
+      <c r="I41" t="inlineStr"/>
+      <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr"/>
+      <c r="L41" t="inlineStr"/>
+      <c r="M41" t="inlineStr"/>
+      <c r="N41" t="inlineStr"/>
+      <c r="O41" t="inlineStr"/>
+      <c r="P41" t="inlineStr"/>
+      <c r="Q41" t="inlineStr"/>
       <c r="R41">
         <f>COUNTIF(C41:Q41,"✓")</f>
         <v/>
@@ -10089,19 +10632,28 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Integración con wearables y apps de salud</t>
-        </is>
-      </c>
-      <c r="H42" t="inlineStr">
+          <t>Integración con EHR de proveedores</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr"/>
+      <c r="D42" t="inlineStr"/>
+      <c r="E42" t="inlineStr"/>
+      <c r="F42" t="inlineStr"/>
+      <c r="G42" t="inlineStr"/>
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" t="inlineStr"/>
+      <c r="J42" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="M42" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="K42" t="inlineStr"/>
+      <c r="L42" t="inlineStr"/>
+      <c r="M42" t="inlineStr"/>
+      <c r="N42" t="inlineStr"/>
+      <c r="O42" t="inlineStr"/>
+      <c r="P42" t="inlineStr"/>
+      <c r="Q42" t="inlineStr"/>
       <c r="R42">
         <f>COUNTIF(C42:Q42,"✓")</f>
         <v/>
@@ -10110,19 +10662,37 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Medicación y recordatorios</t>
+          <t>Interoperabilidad y fuentes de datos</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Gestión de lista de medicamentos</t>
-        </is>
-      </c>
-      <c r="K43" t="inlineStr">
+          <t>Integración con wearables y apps de salud</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr"/>
+      <c r="D43" t="inlineStr"/>
+      <c r="E43" t="inlineStr"/>
+      <c r="F43" t="inlineStr"/>
+      <c r="G43" t="inlineStr"/>
+      <c r="H43" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="I43" t="inlineStr"/>
+      <c r="J43" t="inlineStr"/>
+      <c r="K43" t="inlineStr"/>
+      <c r="L43" t="inlineStr"/>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr"/>
+      <c r="O43" t="inlineStr"/>
+      <c r="P43" t="inlineStr"/>
+      <c r="Q43" t="inlineStr"/>
       <c r="R43">
         <f>COUNTIF(C43:Q43,"✓")</f>
         <v/>
@@ -10136,14 +10706,28 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Importación automática de tratamientos desde receta digital</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
+          <t>Gestión de lista de medicamentos</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr"/>
+      <c r="D44" t="inlineStr"/>
+      <c r="E44" t="inlineStr"/>
+      <c r="F44" t="inlineStr"/>
+      <c r="G44" t="inlineStr"/>
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr"/>
+      <c r="J44" t="inlineStr"/>
+      <c r="K44" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="L44" t="inlineStr"/>
+      <c r="M44" t="inlineStr"/>
+      <c r="N44" t="inlineStr"/>
+      <c r="O44" t="inlineStr"/>
+      <c r="P44" t="inlineStr"/>
+      <c r="Q44" t="inlineStr"/>
       <c r="R44">
         <f>COUNTIF(C44:Q44,"✓")</f>
         <v/>
@@ -10157,19 +10741,28 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Recordatorios de medicación y citas</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
+          <t>Importación automática de tratamientos desde receta digital</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr"/>
+      <c r="D45" t="inlineStr"/>
+      <c r="E45" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="K45" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="F45" t="inlineStr"/>
+      <c r="G45" t="inlineStr"/>
+      <c r="H45" t="inlineStr"/>
+      <c r="I45" t="inlineStr"/>
+      <c r="J45" t="inlineStr"/>
+      <c r="K45" t="inlineStr"/>
+      <c r="L45" t="inlineStr"/>
+      <c r="M45" t="inlineStr"/>
+      <c r="N45" t="inlineStr"/>
+      <c r="O45" t="inlineStr"/>
+      <c r="P45" t="inlineStr"/>
+      <c r="Q45" t="inlineStr"/>
       <c r="R45">
         <f>COUNTIF(C45:Q45,"✓")</f>
         <v/>
@@ -10183,14 +10776,32 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Registro de tomas y adherencia al tratamiento</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
+          <t>Recordatorios de medicación y citas</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="D46" t="inlineStr"/>
+      <c r="E46" t="inlineStr"/>
+      <c r="F46" t="inlineStr"/>
+      <c r="G46" t="inlineStr"/>
+      <c r="H46" t="inlineStr"/>
+      <c r="I46" t="inlineStr"/>
+      <c r="J46" t="inlineStr"/>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr"/>
+      <c r="M46" t="inlineStr"/>
+      <c r="N46" t="inlineStr"/>
+      <c r="O46" t="inlineStr"/>
+      <c r="P46" t="inlineStr"/>
+      <c r="Q46" t="inlineStr"/>
       <c r="R46">
         <f>COUNTIF(C46:Q46,"✓")</f>
         <v/>
@@ -10199,19 +10810,33 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Seguimiento y bienestar</t>
+          <t>Medicación y recordatorios</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Comunidad de pacientes</t>
-        </is>
-      </c>
-      <c r="H47" t="inlineStr">
+          <t>Registro de tomas y adherencia al tratamiento</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr"/>
+      <c r="D47" t="inlineStr"/>
+      <c r="E47" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="F47" t="inlineStr"/>
+      <c r="G47" t="inlineStr"/>
+      <c r="H47" t="inlineStr"/>
+      <c r="I47" t="inlineStr"/>
+      <c r="J47" t="inlineStr"/>
+      <c r="K47" t="inlineStr"/>
+      <c r="L47" t="inlineStr"/>
+      <c r="M47" t="inlineStr"/>
+      <c r="N47" t="inlineStr"/>
+      <c r="O47" t="inlineStr"/>
+      <c r="P47" t="inlineStr"/>
+      <c r="Q47" t="inlineStr"/>
       <c r="R47">
         <f>COUNTIF(C47:Q47,"✓")</f>
         <v/>
@@ -10225,14 +10850,28 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Contenido educativo sobre salud</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
+          <t>Comunidad de pacientes</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr"/>
+      <c r="D48" t="inlineStr"/>
+      <c r="E48" t="inlineStr"/>
+      <c r="F48" t="inlineStr"/>
+      <c r="G48" t="inlineStr"/>
+      <c r="H48" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="I48" t="inlineStr"/>
+      <c r="J48" t="inlineStr"/>
+      <c r="K48" t="inlineStr"/>
+      <c r="L48" t="inlineStr"/>
+      <c r="M48" t="inlineStr"/>
+      <c r="N48" t="inlineStr"/>
+      <c r="O48" t="inlineStr"/>
+      <c r="P48" t="inlineStr"/>
+      <c r="Q48" t="inlineStr"/>
       <c r="R48">
         <f>COUNTIF(C48:Q48,"✓")</f>
         <v/>
@@ -10246,14 +10885,28 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Gráficas de evolución de indicadores</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr">
+          <t>Contenido educativo sobre salud</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="E49" t="inlineStr"/>
+      <c r="F49" t="inlineStr"/>
+      <c r="G49" t="inlineStr"/>
+      <c r="H49" t="inlineStr"/>
+      <c r="I49" t="inlineStr"/>
+      <c r="J49" t="inlineStr"/>
+      <c r="K49" t="inlineStr"/>
+      <c r="L49" t="inlineStr"/>
+      <c r="M49" t="inlineStr"/>
+      <c r="N49" t="inlineStr"/>
+      <c r="O49" t="inlineStr"/>
+      <c r="P49" t="inlineStr"/>
+      <c r="Q49" t="inlineStr"/>
       <c r="R49">
         <f>COUNTIF(C49:Q49,"✓")</f>
         <v/>
@@ -10267,14 +10920,28 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Integración con wearables y apps de salud</t>
-        </is>
-      </c>
-      <c r="K50" t="inlineStr">
+          <t>Gráficas de evolución de indicadores</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr"/>
+      <c r="D50" t="inlineStr"/>
+      <c r="E50" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="F50" t="inlineStr"/>
+      <c r="G50" t="inlineStr"/>
+      <c r="H50" t="inlineStr"/>
+      <c r="I50" t="inlineStr"/>
+      <c r="J50" t="inlineStr"/>
+      <c r="K50" t="inlineStr"/>
+      <c r="L50" t="inlineStr"/>
+      <c r="M50" t="inlineStr"/>
+      <c r="N50" t="inlineStr"/>
+      <c r="O50" t="inlineStr"/>
+      <c r="P50" t="inlineStr"/>
+      <c r="Q50" t="inlineStr"/>
       <c r="R50">
         <f>COUNTIF(C50:Q50,"✓")</f>
         <v/>
@@ -10288,19 +10955,28 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Panel de seguimiento de salud y bienestar</t>
-        </is>
-      </c>
-      <c r="H51" t="inlineStr">
+          <t>Integración con wearables y apps de salud</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr"/>
+      <c r="D51" t="inlineStr"/>
+      <c r="E51" t="inlineStr"/>
+      <c r="F51" t="inlineStr"/>
+      <c r="G51" t="inlineStr"/>
+      <c r="H51" t="inlineStr"/>
+      <c r="I51" t="inlineStr"/>
+      <c r="J51" t="inlineStr"/>
+      <c r="K51" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="I51" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="L51" t="inlineStr"/>
+      <c r="M51" t="inlineStr"/>
+      <c r="N51" t="inlineStr"/>
+      <c r="O51" t="inlineStr"/>
+      <c r="P51" t="inlineStr"/>
+      <c r="Q51" t="inlineStr"/>
       <c r="R51">
         <f>COUNTIF(C51:Q51,"✓")</f>
         <v/>
@@ -10314,14 +10990,32 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Registro de nutrición</t>
-        </is>
-      </c>
-      <c r="K52" t="inlineStr">
+          <t>Panel de seguimiento de salud y bienestar</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr"/>
+      <c r="D52" t="inlineStr"/>
+      <c r="E52" t="inlineStr"/>
+      <c r="F52" t="inlineStr"/>
+      <c r="G52" t="inlineStr"/>
+      <c r="H52" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr"/>
+      <c r="K52" t="inlineStr"/>
+      <c r="L52" t="inlineStr"/>
+      <c r="M52" t="inlineStr"/>
+      <c r="N52" t="inlineStr"/>
+      <c r="O52" t="inlineStr"/>
+      <c r="P52" t="inlineStr"/>
+      <c r="Q52" t="inlineStr"/>
       <c r="R52">
         <f>COUNTIF(C52:Q52,"✓")</f>
         <v/>
@@ -10335,14 +11029,28 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Seguimiento de salud femenina</t>
-        </is>
-      </c>
+          <t>Registro de nutrición</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr"/>
+      <c r="D53" t="inlineStr"/>
+      <c r="E53" t="inlineStr"/>
+      <c r="F53" t="inlineStr"/>
+      <c r="G53" t="inlineStr"/>
+      <c r="H53" t="inlineStr"/>
+      <c r="I53" t="inlineStr"/>
+      <c r="J53" t="inlineStr"/>
       <c r="K53" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="L53" t="inlineStr"/>
+      <c r="M53" t="inlineStr"/>
+      <c r="N53" t="inlineStr"/>
+      <c r="O53" t="inlineStr"/>
+      <c r="P53" t="inlineStr"/>
+      <c r="Q53" t="inlineStr"/>
       <c r="R53">
         <f>COUNTIF(C53:Q53,"✓")</f>
         <v/>
@@ -10356,14 +11064,28 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Valoración de profesionales</t>
-        </is>
-      </c>
-      <c r="F54" t="inlineStr">
+          <t>Seguimiento de salud femenina</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr"/>
+      <c r="D54" t="inlineStr"/>
+      <c r="E54" t="inlineStr"/>
+      <c r="F54" t="inlineStr"/>
+      <c r="G54" t="inlineStr"/>
+      <c r="H54" t="inlineStr"/>
+      <c r="I54" t="inlineStr"/>
+      <c r="J54" t="inlineStr"/>
+      <c r="K54" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="L54" t="inlineStr"/>
+      <c r="M54" t="inlineStr"/>
+      <c r="N54" t="inlineStr"/>
+      <c r="O54" t="inlineStr"/>
+      <c r="P54" t="inlineStr"/>
+      <c r="Q54" t="inlineStr"/>
       <c r="R54">
         <f>COUNTIF(C54:Q54,"✓")</f>
         <v/>
@@ -10372,19 +11094,33 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Seguridad, privacidad y blockchain</t>
+          <t>Seguimiento y bienestar</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Acceso mínimo por categorías de datos</t>
-        </is>
-      </c>
-      <c r="M55" t="inlineStr">
+          <t>Valoración de profesionales</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr"/>
+      <c r="D55" t="inlineStr"/>
+      <c r="E55" t="inlineStr"/>
+      <c r="F55" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="G55" t="inlineStr"/>
+      <c r="H55" t="inlineStr"/>
+      <c r="I55" t="inlineStr"/>
+      <c r="J55" t="inlineStr"/>
+      <c r="K55" t="inlineStr"/>
+      <c r="L55" t="inlineStr"/>
+      <c r="M55" t="inlineStr"/>
+      <c r="N55" t="inlineStr"/>
+      <c r="O55" t="inlineStr"/>
+      <c r="P55" t="inlineStr"/>
+      <c r="Q55" t="inlineStr"/>
       <c r="R55">
         <f>COUNTIF(C55:Q55,"✓")</f>
         <v/>
@@ -10398,24 +11134,28 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Blockchain para integridad y trazabilidad de datos</t>
-        </is>
-      </c>
-      <c r="H56" t="inlineStr">
+          <t>Acceso mínimo por categorías de datos</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr"/>
+      <c r="D56" t="inlineStr"/>
+      <c r="E56" t="inlineStr"/>
+      <c r="F56" t="inlineStr"/>
+      <c r="G56" t="inlineStr"/>
+      <c r="H56" t="inlineStr"/>
+      <c r="I56" t="inlineStr"/>
+      <c r="J56" t="inlineStr"/>
+      <c r="K56" t="inlineStr"/>
+      <c r="L56" t="inlineStr"/>
+      <c r="M56" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="I56" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="J56" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="N56" t="inlineStr"/>
+      <c r="O56" t="inlineStr"/>
+      <c r="P56" t="inlineStr"/>
+      <c r="Q56" t="inlineStr"/>
       <c r="R56">
         <f>COUNTIF(C56:Q56,"✓")</f>
         <v/>
@@ -10429,19 +11169,36 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Cifrado y control de acceso</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr">
+          <t>Blockchain para integridad y trazabilidad de datos</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr"/>
+      <c r="D57" t="inlineStr"/>
+      <c r="E57" t="inlineStr"/>
+      <c r="F57" t="inlineStr"/>
+      <c r="G57" t="inlineStr"/>
+      <c r="H57" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="K57" t="inlineStr">
+      <c r="I57" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr"/>
+      <c r="L57" t="inlineStr"/>
+      <c r="M57" t="inlineStr"/>
+      <c r="N57" t="inlineStr"/>
+      <c r="O57" t="inlineStr"/>
+      <c r="P57" t="inlineStr"/>
+      <c r="Q57" t="inlineStr"/>
       <c r="R57">
         <f>COUNTIF(C57:Q57,"✓")</f>
         <v/>
@@ -10455,14 +11212,32 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Cumplimiento regulatorio de salud y datos</t>
-        </is>
-      </c>
-      <c r="O58" t="inlineStr">
+          <t>Cifrado y control de acceso</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr"/>
+      <c r="D58" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="E58" t="inlineStr"/>
+      <c r="F58" t="inlineStr"/>
+      <c r="G58" t="inlineStr"/>
+      <c r="H58" t="inlineStr"/>
+      <c r="I58" t="inlineStr"/>
+      <c r="J58" t="inlineStr"/>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr"/>
+      <c r="M58" t="inlineStr"/>
+      <c r="N58" t="inlineStr"/>
+      <c r="O58" t="inlineStr"/>
+      <c r="P58" t="inlineStr"/>
+      <c r="Q58" t="inlineStr"/>
       <c r="R58">
         <f>COUNTIF(C58:Q58,"✓")</f>
         <v/>
@@ -10476,14 +11251,28 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Gestión de consentimiento sobre uso de datos</t>
-        </is>
-      </c>
-      <c r="L59" t="inlineStr">
+          <t>Cumplimiento regulatorio de salud y datos</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr"/>
+      <c r="D59" t="inlineStr"/>
+      <c r="E59" t="inlineStr"/>
+      <c r="F59" t="inlineStr"/>
+      <c r="G59" t="inlineStr"/>
+      <c r="H59" t="inlineStr"/>
+      <c r="I59" t="inlineStr"/>
+      <c r="J59" t="inlineStr"/>
+      <c r="K59" t="inlineStr"/>
+      <c r="L59" t="inlineStr"/>
+      <c r="M59" t="inlineStr"/>
+      <c r="N59" t="inlineStr"/>
+      <c r="O59" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="P59" t="inlineStr"/>
+      <c r="Q59" t="inlineStr"/>
       <c r="R59">
         <f>COUNTIF(C59:Q59,"✓")</f>
         <v/>
@@ -10497,14 +11286,28 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Identidad descentralizada (DID)</t>
-        </is>
-      </c>
-      <c r="I60" t="inlineStr">
+          <t>Gestión de consentimiento sobre uso de datos</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr"/>
+      <c r="D60" t="inlineStr"/>
+      <c r="E60" t="inlineStr"/>
+      <c r="F60" t="inlineStr"/>
+      <c r="G60" t="inlineStr"/>
+      <c r="H60" t="inlineStr"/>
+      <c r="I60" t="inlineStr"/>
+      <c r="J60" t="inlineStr"/>
+      <c r="K60" t="inlineStr"/>
+      <c r="L60" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="M60" t="inlineStr"/>
+      <c r="N60" t="inlineStr"/>
+      <c r="O60" t="inlineStr"/>
+      <c r="P60" t="inlineStr"/>
+      <c r="Q60" t="inlineStr"/>
       <c r="R60">
         <f>COUNTIF(C60:Q60,"✓")</f>
         <v/>
@@ -10518,19 +11321,28 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Privacidad reforzada para datos de salud</t>
-        </is>
-      </c>
-      <c r="L61" t="inlineStr">
+          <t>Identidad descentralizada (DID)</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr"/>
+      <c r="D61" t="inlineStr"/>
+      <c r="E61" t="inlineStr"/>
+      <c r="F61" t="inlineStr"/>
+      <c r="G61" t="inlineStr"/>
+      <c r="H61" t="inlineStr"/>
+      <c r="I61" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="M61" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="J61" t="inlineStr"/>
+      <c r="K61" t="inlineStr"/>
+      <c r="L61" t="inlineStr"/>
+      <c r="M61" t="inlineStr"/>
+      <c r="N61" t="inlineStr"/>
+      <c r="O61" t="inlineStr"/>
+      <c r="P61" t="inlineStr"/>
+      <c r="Q61" t="inlineStr"/>
       <c r="R61">
         <f>COUNTIF(C61:Q61,"✓")</f>
         <v/>
@@ -10539,19 +11351,37 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Seguros y pagos</t>
+          <t>Seguridad, privacidad y blockchain</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Modelo freemium y suscripción</t>
-        </is>
-      </c>
-      <c r="Q62" t="inlineStr">
+          <t>Privacidad reforzada para datos de salud</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr"/>
+      <c r="D62" t="inlineStr"/>
+      <c r="E62" t="inlineStr"/>
+      <c r="F62" t="inlineStr"/>
+      <c r="G62" t="inlineStr"/>
+      <c r="H62" t="inlineStr"/>
+      <c r="I62" t="inlineStr"/>
+      <c r="J62" t="inlineStr"/>
+      <c r="K62" t="inlineStr"/>
+      <c r="L62" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="N62" t="inlineStr"/>
+      <c r="O62" t="inlineStr"/>
+      <c r="P62" t="inlineStr"/>
+      <c r="Q62" t="inlineStr"/>
       <c r="R62">
         <f>COUNTIF(C62:Q62,"✓")</f>
         <v/>
@@ -10565,10 +11395,24 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Pagos con criptomoneda</t>
-        </is>
-      </c>
-      <c r="J63" t="inlineStr">
+          <t>Modelo freemium y suscripción</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr"/>
+      <c r="D63" t="inlineStr"/>
+      <c r="E63" t="inlineStr"/>
+      <c r="F63" t="inlineStr"/>
+      <c r="G63" t="inlineStr"/>
+      <c r="H63" t="inlineStr"/>
+      <c r="I63" t="inlineStr"/>
+      <c r="J63" t="inlineStr"/>
+      <c r="K63" t="inlineStr"/>
+      <c r="L63" t="inlineStr"/>
+      <c r="M63" t="inlineStr"/>
+      <c r="N63" t="inlineStr"/>
+      <c r="O63" t="inlineStr"/>
+      <c r="P63" t="inlineStr"/>
+      <c r="Q63" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -10586,14 +11430,28 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Pagos dentro de la app</t>
-        </is>
-      </c>
-      <c r="Q64" t="inlineStr">
+          <t>Pagos con criptomoneda</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr"/>
+      <c r="D64" t="inlineStr"/>
+      <c r="E64" t="inlineStr"/>
+      <c r="F64" t="inlineStr"/>
+      <c r="G64" t="inlineStr"/>
+      <c r="H64" t="inlineStr"/>
+      <c r="I64" t="inlineStr"/>
+      <c r="J64" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="K64" t="inlineStr"/>
+      <c r="L64" t="inlineStr"/>
+      <c r="M64" t="inlineStr"/>
+      <c r="N64" t="inlineStr"/>
+      <c r="O64" t="inlineStr"/>
+      <c r="P64" t="inlineStr"/>
+      <c r="Q64" t="inlineStr"/>
       <c r="R64">
         <f>COUNTIF(C64:Q64,"✓")</f>
         <v/>
@@ -10607,10 +11465,24 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Reclamos y trámites con seguros</t>
-        </is>
-      </c>
-      <c r="I65" t="inlineStr">
+          <t>Pagos dentro de la app</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr"/>
+      <c r="D65" t="inlineStr"/>
+      <c r="E65" t="inlineStr"/>
+      <c r="F65" t="inlineStr"/>
+      <c r="G65" t="inlineStr"/>
+      <c r="H65" t="inlineStr"/>
+      <c r="I65" t="inlineStr"/>
+      <c r="J65" t="inlineStr"/>
+      <c r="K65" t="inlineStr"/>
+      <c r="L65" t="inlineStr"/>
+      <c r="M65" t="inlineStr"/>
+      <c r="N65" t="inlineStr"/>
+      <c r="O65" t="inlineStr"/>
+      <c r="P65" t="inlineStr"/>
+      <c r="Q65" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -10623,19 +11495,33 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Telemedicina y atención remota</t>
+          <t>Seguros y pagos</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Mensajería paciente-institución</t>
-        </is>
-      </c>
+          <t>Reclamos y trámites con seguros</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr"/>
+      <c r="D66" t="inlineStr"/>
+      <c r="E66" t="inlineStr"/>
+      <c r="F66" t="inlineStr"/>
+      <c r="G66" t="inlineStr"/>
+      <c r="H66" t="inlineStr"/>
       <c r="I66" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="J66" t="inlineStr"/>
+      <c r="K66" t="inlineStr"/>
+      <c r="L66" t="inlineStr"/>
+      <c r="M66" t="inlineStr"/>
+      <c r="N66" t="inlineStr"/>
+      <c r="O66" t="inlineStr"/>
+      <c r="P66" t="inlineStr"/>
+      <c r="Q66" t="inlineStr"/>
       <c r="R66">
         <f>COUNTIF(C66:Q66,"✓")</f>
         <v/>
@@ -10649,16 +11535,65 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Teleconsulta con profesionales</t>
-        </is>
-      </c>
-      <c r="J67" t="inlineStr">
+          <t>Mensajería paciente-institución</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr"/>
+      <c r="D67" t="inlineStr"/>
+      <c r="E67" t="inlineStr"/>
+      <c r="F67" t="inlineStr"/>
+      <c r="G67" t="inlineStr"/>
+      <c r="H67" t="inlineStr"/>
+      <c r="I67" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="J67" t="inlineStr"/>
+      <c r="K67" t="inlineStr"/>
+      <c r="L67" t="inlineStr"/>
+      <c r="M67" t="inlineStr"/>
+      <c r="N67" t="inlineStr"/>
+      <c r="O67" t="inlineStr"/>
+      <c r="P67" t="inlineStr"/>
+      <c r="Q67" t="inlineStr"/>
       <c r="R67">
         <f>COUNTIF(C67:Q67,"✓")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Telemedicina y atención remota</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Teleconsulta con profesionales</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr"/>
+      <c r="D68" t="inlineStr"/>
+      <c r="E68" t="inlineStr"/>
+      <c r="F68" t="inlineStr"/>
+      <c r="G68" t="inlineStr"/>
+      <c r="H68" t="inlineStr"/>
+      <c r="I68" t="inlineStr"/>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr"/>
+      <c r="L68" t="inlineStr"/>
+      <c r="M68" t="inlineStr"/>
+      <c r="N68" t="inlineStr"/>
+      <c r="O68" t="inlineStr"/>
+      <c r="P68" t="inlineStr"/>
+      <c r="Q68" t="inlineStr"/>
+      <c r="R68">
+        <f>COUNTIF(C68:Q68,"✓")</f>
         <v/>
       </c>
     </row>
@@ -10673,7 +11608,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A32"/>
+  <dimension ref="A1:A33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -10903,6 +11838,13 @@
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>VUELTA 7 COMPLETA (2026-10-20 12:19 UTC): Clinia, MiRedSalud y Mediko verificados (+0 filas). Contador de loops = 7 para todos, Revisado reiniciado a "No". func_norm (131 filas) y tabla_frecuencia (67 funcionalidades) regenerados. Vuelta 8 parte con Meedika, Infomed, MediPlanner, Clingot. Candidato a competidor sin agregar: HealthChain (Chile).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Benchmark: vuelta 8, iteración 1 (Meedika, Infomed, MediPlanner, Clingot); ficha del candidato HealthChain
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MVcXu8vTBu7EKfj3YdEvae
</commit_message>
<xml_diff>
--- a/Outputs/Benchmark_Anamnesis.xlsx
+++ b/Outputs/Benchmark_Anamnesis.xlsx
@@ -513,12 +513,12 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>[DIRECTO · Chile · etapas A+B] Lanzada 25-sep-2024 en App Store (Android previsto la misma semana). &gt;1.500 usuarios en los primeros días; meta 32.000 (cofundador Francisco González). Funciones: gestión de documentos, importar solicitudes, SOS con alergias/medicación, calendario de citas, recordatorios, compartir con profesionales elegidos. Sin blockchain. Precio y estado actual NO verificados; única fuente es una nota de prensa. Sitio oficial por confirmar. [Iter. 2] Hay cobertura adicional en Portal Innova (portalinnova.cl); sitio bloqueado en este entorno, estado actual sigue sin verificar. [Vuelta 3] Sin novedades 2026 ni confirmación de la app Android en Google Play; usuarios actuales desconocidos. Nota de prensa no indica año de lanzamiento explícito. [Vuelta 4] Sin fuentes nuevas; portalinnova.cl no aparece en búsquedas. Sigue dependiendo de una sola nota de prensa. [Vuelta 5] Sin fuentes nuevas (ni entrevistas ni financiamiento); sigue dependiendo de una sola nota de prensa sin año explícito. [Vuelta 6] Sin ficha de Google Play ni fuentes nuevas; disponibilidad en Android sin confirmar. [Vuelta 7] Sin fuentes nuevas; no hay ficha oficial localizada. No confundir con apps de nombre parecido (Medika App, MEDDI, AI Medik).</t>
+          <t>[DIRECTO · Chile · etapas A+B] Lanzada 25-sep-2024 en App Store (Android previsto la misma semana). &gt;1.500 usuarios en los primeros días; meta 32.000 (cofundador Francisco González). Funciones: gestión de documentos, importar solicitudes, SOS con alergias/medicación, calendario de citas, recordatorios, compartir con profesionales elegidos. Sin blockchain. Precio y estado actual NO verificados; única fuente es una nota de prensa. Sitio oficial por confirmar. [Iter. 2] Hay cobertura adicional en Portal Innova (portalinnova.cl); sitio bloqueado en este entorno, estado actual sigue sin verificar. [Vuelta 3] Sin novedades 2026 ni confirmación de la app Android en Google Play; usuarios actuales desconocidos. Nota de prensa no indica año de lanzamiento explícito. [Vuelta 4] Sin fuentes nuevas; portalinnova.cl no aparece en búsquedas. Sigue dependiendo de una sola nota de prensa. [Vuelta 5] Sin fuentes nuevas (ni entrevistas ni financiamiento); sigue dependiendo de una sola nota de prensa sin año explícito. [Vuelta 6] Sin ficha de Google Play ni fuentes nuevas; disponibilidad en Android sin confirmar. [Vuelta 7] Sin fuentes nuevas; no hay ficha oficial localizada. No confundir con apps de nombre parecido (Medika App, MEDDI, AI Medik). [Vuelta 8] Sin fuentes nuevas.</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G2" t="n">
@@ -526,7 +526,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -553,12 +553,12 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>[DIRECTO · Chile · etapa A] Fundada 2019 por Diego Ibarra, Andrés Fantuzzi y Gabriel Zamora. Lanzada mar-2021 en App Store y Play Store con 1.200 usuarios; planeaba nueva versión jul-2021 y ronda de US$500 mil. Objetivo: llevar el historial en el celular, acceso en emergencias, médico puede ingresar datos con consentimiento. Estado actual NO verificado (posible app inactiva). URL es la nota de prensa; sitio oficial por confirmar. [Vuelta 3] Sin evidencia posterior a 2021; relanzamiento previsto jul-2021 no confirmado. Probable app inactiva. [Vuelta 4] Sin cambios; sigue sin evidencia posterior a 2021. [Vuelta 5] Cofundador Andrés Fantuzzi es cardiólogo de la Clínica Santa María. Sin ronda de inversión ni relanzamiento confirmados; no confundir con Infomed de Cuba (portal del Minsap). [Vuelta 6] Sin búsqueda nueva (fuentes agotadas en vueltas 3-5); sin cambios. [Vuelta 7] Sin búsqueda nueva (saturado); sin cambios.</t>
+          <t>[DIRECTO · Chile · etapa A] Fundada 2019 por Diego Ibarra, Andrés Fantuzzi y Gabriel Zamora. Lanzada mar-2021 en App Store y Play Store con 1.200 usuarios; planeaba nueva versión jul-2021 y ronda de US$500 mil. Objetivo: llevar el historial en el celular, acceso en emergencias, médico puede ingresar datos con consentimiento. Estado actual NO verificado (posible app inactiva). URL es la nota de prensa; sitio oficial por confirmar. [Vuelta 3] Sin evidencia posterior a 2021; relanzamiento previsto jul-2021 no confirmado. Probable app inactiva. [Vuelta 4] Sin cambios; sigue sin evidencia posterior a 2021. [Vuelta 5] Cofundador Andrés Fantuzzi es cardiólogo de la Clínica Santa María. Sin ronda de inversión ni relanzamiento confirmados; no confundir con Infomed de Cuba (portal del Minsap). [Vuelta 6] Sin búsqueda nueva (fuentes agotadas en vueltas 3-5); sin cambios. [Vuelta 7] Sin búsqueda nueva (saturado); sin cambios. [Vuelta 8] Sin fuentes nuevas; relanzamiento de jul-2021 sigue sin confirmarse.</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G3" t="n">
@@ -566,7 +566,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -593,12 +593,12 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>[REGIONAL · México] Historial por perfil familiar, alergias, vacunas, recetas digitales, gráficas de evolución, agendamiento, compartir con profesionales. Gratis en App Store MX. Sin evidencia de uso en Chile. Cubre parte de la etapa C (familia). [Vuelta 3] Existen dos apps distintas: MediPlanner (gratis, Rym Solutions, MX, 3,7/5 con 3 calificaciones) y MediPlanner Pro (otro desarrollador, $39 MXN). Sin presencia verificada en Chile. [Vuelta 4] No pude confirmar el desarrollador de la versión gratuita (Rym Solutions no se repite en esta búsqueda). MediPlanner Pro (fichas BR/OM) guardaría datos solo en el dispositivo, sin nube; no confundir con MedPlanner/AskHEMI (otra empresa). [Vuelta 5] Sin búsqueda nueva (revisada en vuelta 4); sin cambios. [Vuelta 6] Se reconfirma en la ficha de App Store MX que el desarrollador de la versión gratuita es Rym Solutions S. de R.L. de C.V. (3,7/5, 3 calificaciones); MediPlanner Pro no menciona a esa empresa, por lo que no se puede asegurar que sea el mismo desarrollador. [Vuelta 7] Sin búsqueda nueva (saturado); sin cambios.</t>
+          <t>[REGIONAL · México] Historial por perfil familiar, alergias, vacunas, recetas digitales, gráficas de evolución, agendamiento, compartir con profesionales. Gratis en App Store MX. Sin evidencia de uso en Chile. Cubre parte de la etapa C (familia). [Vuelta 3] Existen dos apps distintas: MediPlanner (gratis, Rym Solutions, MX, 3,7/5 con 3 calificaciones) y MediPlanner Pro (otro desarrollador, $39 MXN). Sin presencia verificada en Chile. [Vuelta 4] No pude confirmar el desarrollador de la versión gratuita (Rym Solutions no se repite en esta búsqueda). MediPlanner Pro (fichas BR/OM) guardaría datos solo en el dispositivo, sin nube; no confundir con MedPlanner/AskHEMI (otra empresa). [Vuelta 5] Sin búsqueda nueva (revisada en vuelta 4); sin cambios. [Vuelta 6] Se reconfirma en la ficha de App Store MX que el desarrollador de la versión gratuita es Rym Solutions S. de R.L. de C.V. (3,7/5, 3 calificaciones); MediPlanner Pro no menciona a esa empresa, por lo que no se puede asegurar que sea el mismo desarrollador. [Vuelta 7] Sin búsqueda nueva (saturado); sin cambios. [Vuelta 8] Sin búsqueda nueva (saturado).</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G4" t="n">
@@ -606,7 +606,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -633,12 +633,12 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>[REGIONAL · Argentina · débil] App para cargar antecedentes médicos propios. Única referencia: nota de opinión en grupoanimal.mx sin fecha verificada. Estado y sitio por confirmar. [Vuelta 3] Referencias de 2017 (apps4citizens, La Nación); sitio y precio no verificados; puede estar inactiva. [Vuelta 4] Sin fuentes nuevas. [Vuelta 5] Registro empresarial (indicadores.ar, datos a jul-2026) muestra CLINGOT S.A. activa en CABA, constituida el 4-abr-2016; no confirma que la app siga operando. Programa federal argentino de historias clínicas digitales como contexto regulatorio. [Vuelta 6] Sin búsqueda nueva (fuentes agotadas); sin cambios. [Vuelta 7] Solo fuentes de 2017; sin evidencia nueva de operación más allá del registro societario.</t>
+          <t>[REGIONAL · Argentina · débil] App para cargar antecedentes médicos propios. Única referencia: nota de opinión en grupoanimal.mx sin fecha verificada. Estado y sitio por confirmar. [Vuelta 3] Referencias de 2017 (apps4citizens, La Nación); sitio y precio no verificados; puede estar inactiva. [Vuelta 4] Sin fuentes nuevas. [Vuelta 5] Registro empresarial (indicadores.ar, datos a jul-2026) muestra CLINGOT S.A. activa en CABA, constituida el 4-abr-2016; no confirma que la app siga operando. Programa federal argentino de historias clínicas digitales como contexto regulatorio. [Vuelta 6] Sin búsqueda nueva (fuentes agotadas); sin cambios. [Vuelta 7] Solo fuentes de 2017; sin evidencia nueva de operación más allá del registro societario. [Vuelta 8] Sin fuentes nuevas.</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G5" t="n">
@@ -646,7 +646,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -9059,8 +9059,6 @@
           <t>Búsqueda de profesionales de salud</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9071,17 +9069,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
       <c r="R2">
         <f>COUNTIF(C2:Q2,"✓")</f>
         <v/>
@@ -9103,24 +9090,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
       <c r="R3">
         <f>COUNTIF(C3:Q3,"✓")</f>
         <v/>
@@ -9137,25 +9111,11 @@
           <t>Integración con calendario del dispositivo</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
       <c r="R4">
         <f>COUNTIF(C4:Q4,"✓")</f>
         <v/>
@@ -9172,25 +9132,11 @@
           <t>Localización de centros médicos y farmacias</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr"/>
       <c r="R5">
         <f>COUNTIF(C5:Q5,"✓")</f>
         <v/>
@@ -9207,21 +9153,11 @@
           <t>Reserva de citas médicas</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9232,8 +9168,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="inlineStr"/>
       <c r="R6">
         <f>COUNTIF(C6:Q6,"✓")</f>
         <v/>
@@ -9250,25 +9184,11 @@
           <t>Acceso del profesional al historial del paciente</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr"/>
-      <c r="Q7" t="inlineStr"/>
       <c r="R7">
         <f>COUNTIF(C7:Q7,"✓")</f>
         <v/>
@@ -9285,25 +9205,11 @@
           <t>Compartir con personas sin cuenta mediante clave segura</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
-      <c r="P8" t="inlineStr"/>
-      <c r="Q8" t="inlineStr"/>
       <c r="R8">
         <f>COUNTIF(C8:Q8,"✓")</f>
         <v/>
@@ -9320,25 +9226,11 @@
           <t>Compartir datos con cuidador o persona de confianza</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
-      <c r="P9" t="inlineStr"/>
-      <c r="Q9" t="inlineStr"/>
       <c r="R9">
         <f>COUNTIF(C9:Q9,"✓")</f>
         <v/>
@@ -9360,13 +9252,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9392,16 +9282,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
       <c r="O10" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="P10" t="inlineStr"/>
-      <c r="Q10" t="inlineStr"/>
       <c r="R10">
         <f>COUNTIF(C10:Q10,"✓")</f>
         <v/>
@@ -9418,25 +9303,11 @@
           <t>Gestión de consentimiento sobre uso de datos</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr"/>
-      <c r="P11" t="inlineStr"/>
-      <c r="Q11" t="inlineStr"/>
       <c r="R11">
         <f>COUNTIF(C11:Q11,"✓")</f>
         <v/>
@@ -9453,25 +9324,11 @@
           <t>Ingreso de datos por profesional con consentimiento</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
-      <c r="O12" t="inlineStr"/>
-      <c r="P12" t="inlineStr"/>
-      <c r="Q12" t="inlineStr"/>
       <c r="R12">
         <f>COUNTIF(C12:Q12,"✓")</f>
         <v/>
@@ -9488,25 +9345,11 @@
           <t>Red social con profesionales y familiares</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr"/>
-      <c r="O13" t="inlineStr"/>
-      <c r="P13" t="inlineStr"/>
-      <c r="Q13" t="inlineStr"/>
       <c r="R13">
         <f>COUNTIF(C13:Q13,"✓")</f>
         <v/>
@@ -9533,23 +9376,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
-      <c r="M14" t="inlineStr"/>
-      <c r="N14" t="inlineStr"/>
-      <c r="O14" t="inlineStr"/>
-      <c r="P14" t="inlineStr"/>
-      <c r="Q14" t="inlineStr"/>
       <c r="R14">
         <f>COUNTIF(C14:Q14,"✓")</f>
         <v/>
@@ -9566,8 +9397,6 @@
           <t>Perfiles familiares / dependientes</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9578,29 +9407,21 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr"/>
       <c r="N15" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="Q15" t="inlineStr"/>
       <c r="R15">
         <f>COUNTIF(C15:Q15,"✓")</f>
         <v/>
@@ -9622,8 +9443,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9639,19 +9458,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
-      <c r="M16" t="inlineStr"/>
-      <c r="N16" t="inlineStr"/>
       <c r="O16" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="P16" t="inlineStr"/>
-      <c r="Q16" t="inlineStr"/>
       <c r="R16">
         <f>COUNTIF(C16:Q16,"✓")</f>
         <v/>
@@ -9668,29 +9479,16 @@
           <t>Almacenamiento de recetas</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr"/>
       <c r="N17" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="O17" t="inlineStr"/>
-      <c r="P17" t="inlineStr"/>
-      <c r="Q17" t="inlineStr"/>
       <c r="R17">
         <f>COUNTIF(C17:Q17,"✓")</f>
         <v/>
@@ -9707,25 +9505,11 @@
           <t>Búsqueda y filtros de documentos</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr"/>
-      <c r="M18" t="inlineStr"/>
-      <c r="N18" t="inlineStr"/>
-      <c r="O18" t="inlineStr"/>
-      <c r="P18" t="inlineStr"/>
-      <c r="Q18" t="inlineStr"/>
       <c r="R18">
         <f>COUNTIF(C18:Q18,"✓")</f>
         <v/>
@@ -9742,25 +9526,11 @@
           <t>Emisión de certificados médicos</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr"/>
-      <c r="M19" t="inlineStr"/>
-      <c r="N19" t="inlineStr"/>
-      <c r="O19" t="inlineStr"/>
-      <c r="P19" t="inlineStr"/>
-      <c r="Q19" t="inlineStr"/>
       <c r="R19">
         <f>COUNTIF(C19:Q19,"✓")</f>
         <v/>
@@ -9782,19 +9552,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr"/>
-      <c r="M20" t="inlineStr"/>
-      <c r="N20" t="inlineStr"/>
-      <c r="O20" t="inlineStr"/>
-      <c r="P20" t="inlineStr"/>
       <c r="Q20" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9816,25 +9573,11 @@
           <t>Notificación y envío de resultados</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr"/>
-      <c r="M21" t="inlineStr"/>
       <c r="N21" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="O21" t="inlineStr"/>
-      <c r="P21" t="inlineStr"/>
-      <c r="Q21" t="inlineStr"/>
       <c r="R21">
         <f>COUNTIF(C21:Q21,"✓")</f>
         <v/>
@@ -9851,25 +9594,11 @@
           <t>Recepción de documentos desde terceros</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
-      <c r="L22" t="inlineStr"/>
-      <c r="M22" t="inlineStr"/>
-      <c r="N22" t="inlineStr"/>
-      <c r="O22" t="inlineStr"/>
-      <c r="P22" t="inlineStr"/>
-      <c r="Q22" t="inlineStr"/>
       <c r="R22">
         <f>COUNTIF(C22:Q22,"✓")</f>
         <v/>
@@ -9886,29 +9615,16 @@
           <t>Historial institucional (solo datos de la propia red)</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
-      <c r="L23" t="inlineStr"/>
-      <c r="M23" t="inlineStr"/>
       <c r="N23" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="O23" t="inlineStr"/>
       <c r="P23" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="Q23" t="inlineStr"/>
       <c r="R23">
         <f>COUNTIF(C23:Q23,"✓")</f>
         <v/>
@@ -9925,36 +9641,26 @@
           <t>Historial médico centralizado</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr"/>
       <c r="K24" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="L24" t="inlineStr"/>
-      <c r="M24" t="inlineStr"/>
-      <c r="N24" t="inlineStr"/>
-      <c r="O24" t="inlineStr"/>
-      <c r="P24" t="inlineStr"/>
       <c r="Q24" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9976,25 +9682,11 @@
           <t>Línea de tiempo de salud</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr"/>
-      <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr"/>
-      <c r="L25" t="inlineStr"/>
-      <c r="M25" t="inlineStr"/>
-      <c r="N25" t="inlineStr"/>
-      <c r="O25" t="inlineStr"/>
-      <c r="P25" t="inlineStr"/>
-      <c r="Q25" t="inlineStr"/>
       <c r="R25">
         <f>COUNTIF(C25:Q25,"✓")</f>
         <v/>
@@ -10011,25 +9703,11 @@
           <t>Registro de alergias y vacunas</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr"/>
-      <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
-      <c r="L26" t="inlineStr"/>
-      <c r="M26" t="inlineStr"/>
-      <c r="N26" t="inlineStr"/>
-      <c r="O26" t="inlineStr"/>
-      <c r="P26" t="inlineStr"/>
-      <c r="Q26" t="inlineStr"/>
       <c r="R26">
         <f>COUNTIF(C26:Q26,"✓")</f>
         <v/>
@@ -10046,25 +9724,11 @@
           <t>Seguimiento de visitas, gastos y seguros</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr"/>
-      <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
-      <c r="L27" t="inlineStr"/>
-      <c r="M27" t="inlineStr"/>
-      <c r="N27" t="inlineStr"/>
-      <c r="O27" t="inlineStr"/>
-      <c r="P27" t="inlineStr"/>
-      <c r="Q27" t="inlineStr"/>
       <c r="R27">
         <f>COUNTIF(C27:Q27,"✓")</f>
         <v/>
@@ -10081,11 +9745,6 @@
           <t>Recompensas / monetización de datos del usuario</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10101,13 +9760,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr"/>
-      <c r="M28" t="inlineStr"/>
-      <c r="N28" t="inlineStr"/>
-      <c r="O28" t="inlineStr"/>
-      <c r="P28" t="inlineStr"/>
-      <c r="Q28" t="inlineStr"/>
       <c r="R28">
         <f>COUNTIF(C28:Q28,"✓")</f>
         <v/>
@@ -10124,25 +9776,11 @@
           <t>Asistente de IA para profesionales de salud</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr"/>
-      <c r="D29" t="inlineStr"/>
-      <c r="E29" t="inlineStr"/>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr"/>
-      <c r="H29" t="inlineStr"/>
-      <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="M29" t="inlineStr"/>
-      <c r="N29" t="inlineStr"/>
-      <c r="O29" t="inlineStr"/>
-      <c r="P29" t="inlineStr"/>
-      <c r="Q29" t="inlineStr"/>
       <c r="R29">
         <f>COUNTIF(C29:Q29,"✓")</f>
         <v/>
@@ -10159,25 +9797,11 @@
           <t>Coaching de salud con IA</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr"/>
-      <c r="E30" t="inlineStr"/>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr"/>
-      <c r="L30" t="inlineStr"/>
-      <c r="M30" t="inlineStr"/>
-      <c r="N30" t="inlineStr"/>
-      <c r="O30" t="inlineStr"/>
-      <c r="P30" t="inlineStr"/>
-      <c r="Q30" t="inlineStr"/>
       <c r="R30">
         <f>COUNTIF(C30:Q30,"✓")</f>
         <v/>
@@ -10194,15 +9818,6 @@
           <t>Detección de patrones en métricas de salud con IA</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr"/>
-      <c r="D31" t="inlineStr"/>
-      <c r="E31" t="inlineStr"/>
-      <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr"/>
-      <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10213,10 +9828,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="N31" t="inlineStr"/>
-      <c r="O31" t="inlineStr"/>
-      <c r="P31" t="inlineStr"/>
-      <c r="Q31" t="inlineStr"/>
       <c r="R31">
         <f>COUNTIF(C31:Q31,"✓")</f>
         <v/>
@@ -10233,15 +9844,6 @@
           <t>Interpretación de exámenes con IA</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr"/>
-      <c r="D32" t="inlineStr"/>
-      <c r="E32" t="inlineStr"/>
-      <c r="F32" t="inlineStr"/>
-      <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr"/>
-      <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr"/>
-      <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10252,9 +9854,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="N32" t="inlineStr"/>
-      <c r="O32" t="inlineStr"/>
-      <c r="P32" t="inlineStr"/>
       <c r="Q32" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10276,24 +9875,11 @@
           <t>Orientación médica con IA</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr"/>
-      <c r="D33" t="inlineStr"/>
-      <c r="E33" t="inlineStr"/>
-      <c r="F33" t="inlineStr"/>
-      <c r="G33" t="inlineStr"/>
-      <c r="H33" t="inlineStr"/>
-      <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr"/>
-      <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="M33" t="inlineStr"/>
-      <c r="N33" t="inlineStr"/>
-      <c r="O33" t="inlineStr"/>
-      <c r="P33" t="inlineStr"/>
       <c r="Q33" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10315,15 +9901,6 @@
           <t>Preparación de consultas médicas con IA</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr"/>
-      <c r="D34" t="inlineStr"/>
-      <c r="E34" t="inlineStr"/>
-      <c r="F34" t="inlineStr"/>
-      <c r="G34" t="inlineStr"/>
-      <c r="H34" t="inlineStr"/>
-      <c r="I34" t="inlineStr"/>
-      <c r="J34" t="inlineStr"/>
-      <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10334,10 +9911,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="N34" t="inlineStr"/>
-      <c r="O34" t="inlineStr"/>
-      <c r="P34" t="inlineStr"/>
-      <c r="Q34" t="inlineStr"/>
       <c r="R34">
         <f>COUNTIF(C34:Q34,"✓")</f>
         <v/>
@@ -10354,15 +9927,6 @@
           <t>Resumen de historial con IA</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr"/>
-      <c r="D35" t="inlineStr"/>
-      <c r="E35" t="inlineStr"/>
-      <c r="F35" t="inlineStr"/>
-      <c r="G35" t="inlineStr"/>
-      <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr"/>
-      <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10373,10 +9937,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="N35" t="inlineStr"/>
-      <c r="O35" t="inlineStr"/>
-      <c r="P35" t="inlineStr"/>
-      <c r="Q35" t="inlineStr"/>
       <c r="R35">
         <f>COUNTIF(C35:Q35,"✓")</f>
         <v/>
@@ -10393,25 +9953,11 @@
           <t>API para apps de terceros</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr"/>
-      <c r="D36" t="inlineStr"/>
-      <c r="E36" t="inlineStr"/>
-      <c r="F36" t="inlineStr"/>
-      <c r="G36" t="inlineStr"/>
-      <c r="H36" t="inlineStr"/>
-      <c r="I36" t="inlineStr"/>
-      <c r="J36" t="inlineStr"/>
       <c r="K36" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="L36" t="inlineStr"/>
-      <c r="M36" t="inlineStr"/>
-      <c r="N36" t="inlineStr"/>
-      <c r="O36" t="inlineStr"/>
-      <c r="P36" t="inlineStr"/>
-      <c r="Q36" t="inlineStr"/>
       <c r="R36">
         <f>COUNTIF(C36:Q36,"✓")</f>
         <v/>
@@ -10433,10 +9979,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr"/>
-      <c r="E37" t="inlineStr"/>
-      <c r="F37" t="inlineStr"/>
-      <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10447,7 +9989,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="J37" t="inlineStr"/>
       <c r="K37" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10463,14 +10004,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="N37" t="inlineStr"/>
       <c r="O37" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="P37" t="inlineStr"/>
-      <c r="Q37" t="inlineStr"/>
       <c r="R37">
         <f>COUNTIF(C37:Q37,"✓")</f>
         <v/>
@@ -10487,25 +10025,11 @@
           <t>Analítica poblacional B2B</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr"/>
-      <c r="D38" t="inlineStr"/>
-      <c r="E38" t="inlineStr"/>
-      <c r="F38" t="inlineStr"/>
-      <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="I38" t="inlineStr"/>
-      <c r="J38" t="inlineStr"/>
-      <c r="K38" t="inlineStr"/>
-      <c r="L38" t="inlineStr"/>
-      <c r="M38" t="inlineStr"/>
-      <c r="N38" t="inlineStr"/>
-      <c r="O38" t="inlineStr"/>
-      <c r="P38" t="inlineStr"/>
-      <c r="Q38" t="inlineStr"/>
       <c r="R38">
         <f>COUNTIF(C38:Q38,"✓")</f>
         <v/>
@@ -10522,9 +10046,6 @@
           <t>Disponibilidad multiplataforma (web/iOS/Android)</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr"/>
-      <c r="D39" t="inlineStr"/>
-      <c r="E39" t="inlineStr"/>
       <c r="F39" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10535,20 +10056,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr"/>
-      <c r="I39" t="inlineStr"/>
-      <c r="J39" t="inlineStr"/>
-      <c r="K39" t="inlineStr"/>
-      <c r="L39" t="inlineStr"/>
-      <c r="M39" t="inlineStr"/>
-      <c r="N39" t="inlineStr"/>
       <c r="O39" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="P39" t="inlineStr"/>
-      <c r="Q39" t="inlineStr"/>
       <c r="R39">
         <f>COUNTIF(C39:Q39,"✓")</f>
         <v/>
@@ -10565,25 +10077,11 @@
           <t>Historial médico centralizado</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr"/>
-      <c r="D40" t="inlineStr"/>
-      <c r="E40" t="inlineStr"/>
-      <c r="F40" t="inlineStr"/>
-      <c r="G40" t="inlineStr"/>
-      <c r="H40" t="inlineStr"/>
-      <c r="I40" t="inlineStr"/>
       <c r="J40" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="K40" t="inlineStr"/>
-      <c r="L40" t="inlineStr"/>
-      <c r="M40" t="inlineStr"/>
-      <c r="N40" t="inlineStr"/>
-      <c r="O40" t="inlineStr"/>
-      <c r="P40" t="inlineStr"/>
-      <c r="Q40" t="inlineStr"/>
       <c r="R40">
         <f>COUNTIF(C40:Q40,"✓")</f>
         <v/>
@@ -10600,25 +10098,11 @@
           <t>Importación y exportación de datos</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr"/>
-      <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr"/>
-      <c r="G41" t="inlineStr"/>
-      <c r="H41" t="inlineStr"/>
-      <c r="I41" t="inlineStr"/>
-      <c r="J41" t="inlineStr"/>
-      <c r="K41" t="inlineStr"/>
-      <c r="L41" t="inlineStr"/>
-      <c r="M41" t="inlineStr"/>
-      <c r="N41" t="inlineStr"/>
-      <c r="O41" t="inlineStr"/>
-      <c r="P41" t="inlineStr"/>
-      <c r="Q41" t="inlineStr"/>
       <c r="R41">
         <f>COUNTIF(C41:Q41,"✓")</f>
         <v/>
@@ -10635,25 +10119,11 @@
           <t>Integración con EHR de proveedores</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr"/>
-      <c r="D42" t="inlineStr"/>
-      <c r="E42" t="inlineStr"/>
-      <c r="F42" t="inlineStr"/>
-      <c r="G42" t="inlineStr"/>
-      <c r="H42" t="inlineStr"/>
-      <c r="I42" t="inlineStr"/>
       <c r="J42" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="K42" t="inlineStr"/>
-      <c r="L42" t="inlineStr"/>
-      <c r="M42" t="inlineStr"/>
-      <c r="N42" t="inlineStr"/>
-      <c r="O42" t="inlineStr"/>
-      <c r="P42" t="inlineStr"/>
-      <c r="Q42" t="inlineStr"/>
       <c r="R42">
         <f>COUNTIF(C42:Q42,"✓")</f>
         <v/>
@@ -10670,29 +10140,16 @@
           <t>Integración con wearables y apps de salud</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr"/>
-      <c r="D43" t="inlineStr"/>
-      <c r="E43" t="inlineStr"/>
-      <c r="F43" t="inlineStr"/>
-      <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="I43" t="inlineStr"/>
-      <c r="J43" t="inlineStr"/>
-      <c r="K43" t="inlineStr"/>
-      <c r="L43" t="inlineStr"/>
       <c r="M43" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="N43" t="inlineStr"/>
-      <c r="O43" t="inlineStr"/>
-      <c r="P43" t="inlineStr"/>
-      <c r="Q43" t="inlineStr"/>
       <c r="R43">
         <f>COUNTIF(C43:Q43,"✓")</f>
         <v/>
@@ -10709,25 +10166,11 @@
           <t>Gestión de lista de medicamentos</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr"/>
-      <c r="D44" t="inlineStr"/>
-      <c r="E44" t="inlineStr"/>
-      <c r="F44" t="inlineStr"/>
-      <c r="G44" t="inlineStr"/>
-      <c r="H44" t="inlineStr"/>
-      <c r="I44" t="inlineStr"/>
-      <c r="J44" t="inlineStr"/>
       <c r="K44" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="L44" t="inlineStr"/>
-      <c r="M44" t="inlineStr"/>
-      <c r="N44" t="inlineStr"/>
-      <c r="O44" t="inlineStr"/>
-      <c r="P44" t="inlineStr"/>
-      <c r="Q44" t="inlineStr"/>
       <c r="R44">
         <f>COUNTIF(C44:Q44,"✓")</f>
         <v/>
@@ -10744,25 +10187,11 @@
           <t>Importación automática de tratamientos desde receta digital</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr"/>
-      <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr"/>
-      <c r="G45" t="inlineStr"/>
-      <c r="H45" t="inlineStr"/>
-      <c r="I45" t="inlineStr"/>
-      <c r="J45" t="inlineStr"/>
-      <c r="K45" t="inlineStr"/>
-      <c r="L45" t="inlineStr"/>
-      <c r="M45" t="inlineStr"/>
-      <c r="N45" t="inlineStr"/>
-      <c r="O45" t="inlineStr"/>
-      <c r="P45" t="inlineStr"/>
-      <c r="Q45" t="inlineStr"/>
       <c r="R45">
         <f>COUNTIF(C45:Q45,"✓")</f>
         <v/>
@@ -10784,24 +10213,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr"/>
-      <c r="E46" t="inlineStr"/>
-      <c r="F46" t="inlineStr"/>
-      <c r="G46" t="inlineStr"/>
-      <c r="H46" t="inlineStr"/>
-      <c r="I46" t="inlineStr"/>
-      <c r="J46" t="inlineStr"/>
       <c r="K46" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="L46" t="inlineStr"/>
-      <c r="M46" t="inlineStr"/>
-      <c r="N46" t="inlineStr"/>
-      <c r="O46" t="inlineStr"/>
-      <c r="P46" t="inlineStr"/>
-      <c r="Q46" t="inlineStr"/>
       <c r="R46">
         <f>COUNTIF(C46:Q46,"✓")</f>
         <v/>
@@ -10818,25 +10234,11 @@
           <t>Registro de tomas y adherencia al tratamiento</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr"/>
-      <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F47" t="inlineStr"/>
-      <c r="G47" t="inlineStr"/>
-      <c r="H47" t="inlineStr"/>
-      <c r="I47" t="inlineStr"/>
-      <c r="J47" t="inlineStr"/>
-      <c r="K47" t="inlineStr"/>
-      <c r="L47" t="inlineStr"/>
-      <c r="M47" t="inlineStr"/>
-      <c r="N47" t="inlineStr"/>
-      <c r="O47" t="inlineStr"/>
-      <c r="P47" t="inlineStr"/>
-      <c r="Q47" t="inlineStr"/>
       <c r="R47">
         <f>COUNTIF(C47:Q47,"✓")</f>
         <v/>
@@ -10853,25 +10255,11 @@
           <t>Comunidad de pacientes</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr"/>
-      <c r="D48" t="inlineStr"/>
-      <c r="E48" t="inlineStr"/>
-      <c r="F48" t="inlineStr"/>
-      <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="I48" t="inlineStr"/>
-      <c r="J48" t="inlineStr"/>
-      <c r="K48" t="inlineStr"/>
-      <c r="L48" t="inlineStr"/>
-      <c r="M48" t="inlineStr"/>
-      <c r="N48" t="inlineStr"/>
-      <c r="O48" t="inlineStr"/>
-      <c r="P48" t="inlineStr"/>
-      <c r="Q48" t="inlineStr"/>
       <c r="R48">
         <f>COUNTIF(C48:Q48,"✓")</f>
         <v/>
@@ -10888,25 +10276,11 @@
           <t>Contenido educativo sobre salud</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr"/>
       <c r="D49" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr"/>
-      <c r="F49" t="inlineStr"/>
-      <c r="G49" t="inlineStr"/>
-      <c r="H49" t="inlineStr"/>
-      <c r="I49" t="inlineStr"/>
-      <c r="J49" t="inlineStr"/>
-      <c r="K49" t="inlineStr"/>
-      <c r="L49" t="inlineStr"/>
-      <c r="M49" t="inlineStr"/>
-      <c r="N49" t="inlineStr"/>
-      <c r="O49" t="inlineStr"/>
-      <c r="P49" t="inlineStr"/>
-      <c r="Q49" t="inlineStr"/>
       <c r="R49">
         <f>COUNTIF(C49:Q49,"✓")</f>
         <v/>
@@ -10923,25 +10297,11 @@
           <t>Gráficas de evolución de indicadores</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr"/>
-      <c r="D50" t="inlineStr"/>
       <c r="E50" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F50" t="inlineStr"/>
-      <c r="G50" t="inlineStr"/>
-      <c r="H50" t="inlineStr"/>
-      <c r="I50" t="inlineStr"/>
-      <c r="J50" t="inlineStr"/>
-      <c r="K50" t="inlineStr"/>
-      <c r="L50" t="inlineStr"/>
-      <c r="M50" t="inlineStr"/>
-      <c r="N50" t="inlineStr"/>
-      <c r="O50" t="inlineStr"/>
-      <c r="P50" t="inlineStr"/>
-      <c r="Q50" t="inlineStr"/>
       <c r="R50">
         <f>COUNTIF(C50:Q50,"✓")</f>
         <v/>
@@ -10958,25 +10318,11 @@
           <t>Integración con wearables y apps de salud</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr"/>
-      <c r="D51" t="inlineStr"/>
-      <c r="E51" t="inlineStr"/>
-      <c r="F51" t="inlineStr"/>
-      <c r="G51" t="inlineStr"/>
-      <c r="H51" t="inlineStr"/>
-      <c r="I51" t="inlineStr"/>
-      <c r="J51" t="inlineStr"/>
       <c r="K51" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="L51" t="inlineStr"/>
-      <c r="M51" t="inlineStr"/>
-      <c r="N51" t="inlineStr"/>
-      <c r="O51" t="inlineStr"/>
-      <c r="P51" t="inlineStr"/>
-      <c r="Q51" t="inlineStr"/>
       <c r="R51">
         <f>COUNTIF(C51:Q51,"✓")</f>
         <v/>
@@ -10993,11 +10339,6 @@
           <t>Panel de seguimiento de salud y bienestar</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr"/>
-      <c r="D52" t="inlineStr"/>
-      <c r="E52" t="inlineStr"/>
-      <c r="F52" t="inlineStr"/>
-      <c r="G52" t="inlineStr"/>
       <c r="H52" t="inlineStr">
         <is>
           <t>✓</t>
@@ -11008,14 +10349,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="J52" t="inlineStr"/>
-      <c r="K52" t="inlineStr"/>
-      <c r="L52" t="inlineStr"/>
-      <c r="M52" t="inlineStr"/>
-      <c r="N52" t="inlineStr"/>
-      <c r="O52" t="inlineStr"/>
-      <c r="P52" t="inlineStr"/>
-      <c r="Q52" t="inlineStr"/>
       <c r="R52">
         <f>COUNTIF(C52:Q52,"✓")</f>
         <v/>
@@ -11032,25 +10365,11 @@
           <t>Registro de nutrición</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr"/>
-      <c r="D53" t="inlineStr"/>
-      <c r="E53" t="inlineStr"/>
-      <c r="F53" t="inlineStr"/>
-      <c r="G53" t="inlineStr"/>
-      <c r="H53" t="inlineStr"/>
-      <c r="I53" t="inlineStr"/>
-      <c r="J53" t="inlineStr"/>
       <c r="K53" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="L53" t="inlineStr"/>
-      <c r="M53" t="inlineStr"/>
-      <c r="N53" t="inlineStr"/>
-      <c r="O53" t="inlineStr"/>
-      <c r="P53" t="inlineStr"/>
-      <c r="Q53" t="inlineStr"/>
       <c r="R53">
         <f>COUNTIF(C53:Q53,"✓")</f>
         <v/>
@@ -11067,25 +10386,11 @@
           <t>Seguimiento de salud femenina</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr"/>
-      <c r="D54" t="inlineStr"/>
-      <c r="E54" t="inlineStr"/>
-      <c r="F54" t="inlineStr"/>
-      <c r="G54" t="inlineStr"/>
-      <c r="H54" t="inlineStr"/>
-      <c r="I54" t="inlineStr"/>
-      <c r="J54" t="inlineStr"/>
       <c r="K54" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="L54" t="inlineStr"/>
-      <c r="M54" t="inlineStr"/>
-      <c r="N54" t="inlineStr"/>
-      <c r="O54" t="inlineStr"/>
-      <c r="P54" t="inlineStr"/>
-      <c r="Q54" t="inlineStr"/>
       <c r="R54">
         <f>COUNTIF(C54:Q54,"✓")</f>
         <v/>
@@ -11102,25 +10407,11 @@
           <t>Valoración de profesionales</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr"/>
-      <c r="D55" t="inlineStr"/>
-      <c r="E55" t="inlineStr"/>
       <c r="F55" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="G55" t="inlineStr"/>
-      <c r="H55" t="inlineStr"/>
-      <c r="I55" t="inlineStr"/>
-      <c r="J55" t="inlineStr"/>
-      <c r="K55" t="inlineStr"/>
-      <c r="L55" t="inlineStr"/>
-      <c r="M55" t="inlineStr"/>
-      <c r="N55" t="inlineStr"/>
-      <c r="O55" t="inlineStr"/>
-      <c r="P55" t="inlineStr"/>
-      <c r="Q55" t="inlineStr"/>
       <c r="R55">
         <f>COUNTIF(C55:Q55,"✓")</f>
         <v/>
@@ -11137,25 +10428,11 @@
           <t>Acceso mínimo por categorías de datos</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr"/>
-      <c r="D56" t="inlineStr"/>
-      <c r="E56" t="inlineStr"/>
-      <c r="F56" t="inlineStr"/>
-      <c r="G56" t="inlineStr"/>
-      <c r="H56" t="inlineStr"/>
-      <c r="I56" t="inlineStr"/>
-      <c r="J56" t="inlineStr"/>
-      <c r="K56" t="inlineStr"/>
-      <c r="L56" t="inlineStr"/>
       <c r="M56" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="N56" t="inlineStr"/>
-      <c r="O56" t="inlineStr"/>
-      <c r="P56" t="inlineStr"/>
-      <c r="Q56" t="inlineStr"/>
       <c r="R56">
         <f>COUNTIF(C56:Q56,"✓")</f>
         <v/>
@@ -11172,11 +10449,6 @@
           <t>Blockchain para integridad y trazabilidad de datos</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr"/>
-      <c r="D57" t="inlineStr"/>
-      <c r="E57" t="inlineStr"/>
-      <c r="F57" t="inlineStr"/>
-      <c r="G57" t="inlineStr"/>
       <c r="H57" t="inlineStr">
         <is>
           <t>✓</t>
@@ -11192,13 +10464,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="K57" t="inlineStr"/>
-      <c r="L57" t="inlineStr"/>
-      <c r="M57" t="inlineStr"/>
-      <c r="N57" t="inlineStr"/>
-      <c r="O57" t="inlineStr"/>
-      <c r="P57" t="inlineStr"/>
-      <c r="Q57" t="inlineStr"/>
       <c r="R57">
         <f>COUNTIF(C57:Q57,"✓")</f>
         <v/>
@@ -11215,29 +10480,16 @@
           <t>Cifrado y control de acceso</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr"/>
       <c r="D58" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr"/>
-      <c r="F58" t="inlineStr"/>
-      <c r="G58" t="inlineStr"/>
-      <c r="H58" t="inlineStr"/>
-      <c r="I58" t="inlineStr"/>
-      <c r="J58" t="inlineStr"/>
       <c r="K58" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="L58" t="inlineStr"/>
-      <c r="M58" t="inlineStr"/>
-      <c r="N58" t="inlineStr"/>
-      <c r="O58" t="inlineStr"/>
-      <c r="P58" t="inlineStr"/>
-      <c r="Q58" t="inlineStr"/>
       <c r="R58">
         <f>COUNTIF(C58:Q58,"✓")</f>
         <v/>
@@ -11254,25 +10506,11 @@
           <t>Cumplimiento regulatorio de salud y datos</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr"/>
-      <c r="D59" t="inlineStr"/>
-      <c r="E59" t="inlineStr"/>
-      <c r="F59" t="inlineStr"/>
-      <c r="G59" t="inlineStr"/>
-      <c r="H59" t="inlineStr"/>
-      <c r="I59" t="inlineStr"/>
-      <c r="J59" t="inlineStr"/>
-      <c r="K59" t="inlineStr"/>
-      <c r="L59" t="inlineStr"/>
-      <c r="M59" t="inlineStr"/>
-      <c r="N59" t="inlineStr"/>
       <c r="O59" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="P59" t="inlineStr"/>
-      <c r="Q59" t="inlineStr"/>
       <c r="R59">
         <f>COUNTIF(C59:Q59,"✓")</f>
         <v/>
@@ -11289,25 +10527,11 @@
           <t>Gestión de consentimiento sobre uso de datos</t>
         </is>
       </c>
-      <c r="C60" t="inlineStr"/>
-      <c r="D60" t="inlineStr"/>
-      <c r="E60" t="inlineStr"/>
-      <c r="F60" t="inlineStr"/>
-      <c r="G60" t="inlineStr"/>
-      <c r="H60" t="inlineStr"/>
-      <c r="I60" t="inlineStr"/>
-      <c r="J60" t="inlineStr"/>
-      <c r="K60" t="inlineStr"/>
       <c r="L60" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="M60" t="inlineStr"/>
-      <c r="N60" t="inlineStr"/>
-      <c r="O60" t="inlineStr"/>
-      <c r="P60" t="inlineStr"/>
-      <c r="Q60" t="inlineStr"/>
       <c r="R60">
         <f>COUNTIF(C60:Q60,"✓")</f>
         <v/>
@@ -11324,25 +10548,11 @@
           <t>Identidad descentralizada (DID)</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr"/>
-      <c r="D61" t="inlineStr"/>
-      <c r="E61" t="inlineStr"/>
-      <c r="F61" t="inlineStr"/>
-      <c r="G61" t="inlineStr"/>
-      <c r="H61" t="inlineStr"/>
       <c r="I61" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="J61" t="inlineStr"/>
-      <c r="K61" t="inlineStr"/>
-      <c r="L61" t="inlineStr"/>
-      <c r="M61" t="inlineStr"/>
-      <c r="N61" t="inlineStr"/>
-      <c r="O61" t="inlineStr"/>
-      <c r="P61" t="inlineStr"/>
-      <c r="Q61" t="inlineStr"/>
       <c r="R61">
         <f>COUNTIF(C61:Q61,"✓")</f>
         <v/>
@@ -11359,15 +10569,6 @@
           <t>Privacidad reforzada para datos de salud</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr"/>
-      <c r="D62" t="inlineStr"/>
-      <c r="E62" t="inlineStr"/>
-      <c r="F62" t="inlineStr"/>
-      <c r="G62" t="inlineStr"/>
-      <c r="H62" t="inlineStr"/>
-      <c r="I62" t="inlineStr"/>
-      <c r="J62" t="inlineStr"/>
-      <c r="K62" t="inlineStr"/>
       <c r="L62" t="inlineStr">
         <is>
           <t>✓</t>
@@ -11378,10 +10579,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="N62" t="inlineStr"/>
-      <c r="O62" t="inlineStr"/>
-      <c r="P62" t="inlineStr"/>
-      <c r="Q62" t="inlineStr"/>
       <c r="R62">
         <f>COUNTIF(C62:Q62,"✓")</f>
         <v/>
@@ -11398,20 +10595,6 @@
           <t>Modelo freemium y suscripción</t>
         </is>
       </c>
-      <c r="C63" t="inlineStr"/>
-      <c r="D63" t="inlineStr"/>
-      <c r="E63" t="inlineStr"/>
-      <c r="F63" t="inlineStr"/>
-      <c r="G63" t="inlineStr"/>
-      <c r="H63" t="inlineStr"/>
-      <c r="I63" t="inlineStr"/>
-      <c r="J63" t="inlineStr"/>
-      <c r="K63" t="inlineStr"/>
-      <c r="L63" t="inlineStr"/>
-      <c r="M63" t="inlineStr"/>
-      <c r="N63" t="inlineStr"/>
-      <c r="O63" t="inlineStr"/>
-      <c r="P63" t="inlineStr"/>
       <c r="Q63" t="inlineStr">
         <is>
           <t>✓</t>
@@ -11433,25 +10616,11 @@
           <t>Pagos con criptomoneda</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr"/>
-      <c r="D64" t="inlineStr"/>
-      <c r="E64" t="inlineStr"/>
-      <c r="F64" t="inlineStr"/>
-      <c r="G64" t="inlineStr"/>
-      <c r="H64" t="inlineStr"/>
-      <c r="I64" t="inlineStr"/>
       <c r="J64" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="K64" t="inlineStr"/>
-      <c r="L64" t="inlineStr"/>
-      <c r="M64" t="inlineStr"/>
-      <c r="N64" t="inlineStr"/>
-      <c r="O64" t="inlineStr"/>
-      <c r="P64" t="inlineStr"/>
-      <c r="Q64" t="inlineStr"/>
       <c r="R64">
         <f>COUNTIF(C64:Q64,"✓")</f>
         <v/>
@@ -11468,20 +10637,6 @@
           <t>Pagos dentro de la app</t>
         </is>
       </c>
-      <c r="C65" t="inlineStr"/>
-      <c r="D65" t="inlineStr"/>
-      <c r="E65" t="inlineStr"/>
-      <c r="F65" t="inlineStr"/>
-      <c r="G65" t="inlineStr"/>
-      <c r="H65" t="inlineStr"/>
-      <c r="I65" t="inlineStr"/>
-      <c r="J65" t="inlineStr"/>
-      <c r="K65" t="inlineStr"/>
-      <c r="L65" t="inlineStr"/>
-      <c r="M65" t="inlineStr"/>
-      <c r="N65" t="inlineStr"/>
-      <c r="O65" t="inlineStr"/>
-      <c r="P65" t="inlineStr"/>
       <c r="Q65" t="inlineStr">
         <is>
           <t>✓</t>
@@ -11503,25 +10658,11 @@
           <t>Reclamos y trámites con seguros</t>
         </is>
       </c>
-      <c r="C66" t="inlineStr"/>
-      <c r="D66" t="inlineStr"/>
-      <c r="E66" t="inlineStr"/>
-      <c r="F66" t="inlineStr"/>
-      <c r="G66" t="inlineStr"/>
-      <c r="H66" t="inlineStr"/>
       <c r="I66" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="J66" t="inlineStr"/>
-      <c r="K66" t="inlineStr"/>
-      <c r="L66" t="inlineStr"/>
-      <c r="M66" t="inlineStr"/>
-      <c r="N66" t="inlineStr"/>
-      <c r="O66" t="inlineStr"/>
-      <c r="P66" t="inlineStr"/>
-      <c r="Q66" t="inlineStr"/>
       <c r="R66">
         <f>COUNTIF(C66:Q66,"✓")</f>
         <v/>
@@ -11538,25 +10679,11 @@
           <t>Mensajería paciente-institución</t>
         </is>
       </c>
-      <c r="C67" t="inlineStr"/>
-      <c r="D67" t="inlineStr"/>
-      <c r="E67" t="inlineStr"/>
-      <c r="F67" t="inlineStr"/>
-      <c r="G67" t="inlineStr"/>
-      <c r="H67" t="inlineStr"/>
       <c r="I67" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="J67" t="inlineStr"/>
-      <c r="K67" t="inlineStr"/>
-      <c r="L67" t="inlineStr"/>
-      <c r="M67" t="inlineStr"/>
-      <c r="N67" t="inlineStr"/>
-      <c r="O67" t="inlineStr"/>
-      <c r="P67" t="inlineStr"/>
-      <c r="Q67" t="inlineStr"/>
       <c r="R67">
         <f>COUNTIF(C67:Q67,"✓")</f>
         <v/>
@@ -11573,25 +10700,11 @@
           <t>Teleconsulta con profesionales</t>
         </is>
       </c>
-      <c r="C68" t="inlineStr"/>
-      <c r="D68" t="inlineStr"/>
-      <c r="E68" t="inlineStr"/>
-      <c r="F68" t="inlineStr"/>
-      <c r="G68" t="inlineStr"/>
-      <c r="H68" t="inlineStr"/>
-      <c r="I68" t="inlineStr"/>
       <c r="J68" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="K68" t="inlineStr"/>
-      <c r="L68" t="inlineStr"/>
-      <c r="M68" t="inlineStr"/>
-      <c r="N68" t="inlineStr"/>
-      <c r="O68" t="inlineStr"/>
-      <c r="P68" t="inlineStr"/>
-      <c r="Q68" t="inlineStr"/>
       <c r="R68">
         <f>COUNTIF(C68:Q68,"✓")</f>
         <v/>
@@ -11608,7 +10721,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A33"/>
+  <dimension ref="A1:A35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -11845,6 +10958,20 @@
         </is>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Vuelta 8 (iter. 1, 2026-10-21 12:23 UTC): Meedika, Infomed, MediPlanner, Clingot verificados (+0 filas; saturado). Pendientes: Healfies, Patientory, MediBloc, Medicalchain, Apple Health, ChatGPT Health, Claude for Healthcare, Apps de clínicas, Clinia, MiRedSalud, Mediko.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>CANDIDATO A COMPETIDOR (no agregado a la lista; decide el usuario): HealthChain (Chile, Santiago). Cofundada en 2018 por Javier Leyton, Ivonne Beltrán y Génesis García; Startup Chile; red Hyperledger Fabric con protocolo de interoperabilidad y API para sistemas hospitalarios (BaaS); en may-2020 anunció una red para unificar el historial clínico en Latinoamérica con IBM Blockchain. Fuentes 2018-2020 (Diario Bitcoin, Meganoticias); estado actual desconocido. Funcionalidades inferidas: interoperabilidad entre instituciones, historial unificado, blockchain. Competidor B2B más que app de paciente.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Benchmark: vuelta 8, iteración 2 (Healfies, Patientory, MediBloc, Medicalchain)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MVcXu8vTBu7EKfj3YdEvae
</commit_message>
<xml_diff>
--- a/Outputs/Benchmark_Anamnesis.xlsx
+++ b/Outputs/Benchmark_Anamnesis.xlsx
@@ -673,12 +673,12 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>[REGIONAL · Brasil] Fundada ene-2015 en Florianópolis por Helyson Lewis Velasco. Centraliza registros de salud personales: carpetas, etiquetas, línea de tiempo (medicación, exámenes, citas, dieta), compartir con familia o profesionales. Gratis; web, iOS y Android. Estado actual NO verificado (fuentes de 2015-2016). Referencia funcional cercana a etapas A+B. [Vuelta 2] Lanzada simultáneamente en Brasil, Argentina y EE.UU.; permite compartir con no registrados vía clave por email. Sin novedades posteriores a 2016. [Vuelta 3] Sin evidencia de actividad reciente ni de cierre; Gust/Dealroom la listan en Florianópolis (10 empleados, healfies.com) sin fecha de actualización. Estado sin confirmar. [Vuelta 4] Sin Google Play localizado; no confundir con la app Healfy (otro producto). Sin novedades. [Vuelta 5] Sin búsqueda nueva (revisada en vuelta 4); sin cambios. [Vuelta 6] Sin búsqueda nueva (fuentes agotadas); sin cambios. [Vuelta 7] Solo fuentes de 2015-2016; alianza con ClinCard (feb-2016). Sin evidencia de actividad reciente.</t>
+          <t>[REGIONAL · Brasil] Fundada ene-2015 en Florianópolis por Helyson Lewis Velasco. Centraliza registros de salud personales: carpetas, etiquetas, línea de tiempo (medicación, exámenes, citas, dieta), compartir con familia o profesionales. Gratis; web, iOS y Android. Estado actual NO verificado (fuentes de 2015-2016). Referencia funcional cercana a etapas A+B. [Vuelta 2] Lanzada simultáneamente en Brasil, Argentina y EE.UU.; permite compartir con no registrados vía clave por email. Sin novedades posteriores a 2016. [Vuelta 3] Sin evidencia de actividad reciente ni de cierre; Gust/Dealroom la listan en Florianópolis (10 empleados, healfies.com) sin fecha de actualización. Estado sin confirmar. [Vuelta 4] Sin Google Play localizado; no confundir con la app Healfy (otro producto). Sin novedades. [Vuelta 5] Sin búsqueda nueva (revisada en vuelta 4); sin cambios. [Vuelta 6] Sin búsqueda nueva (fuentes agotadas); sin cambios. [Vuelta 7] Solo fuentes de 2015-2016; alianza con ClinCard (feb-2016). Sin evidencia de actividad reciente. [Vuelta 8] Sin fuentes nuevas.</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G6" t="n">
@@ -686,7 +686,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -713,12 +713,12 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>[BLOCKCHAIN · EE.UU.] Atlanta, fundada 2015, ~9 empleados. Levantó US$7,2M vía financiamiento cripto. App con registros de hospitales y wearables, coaching de salud con IA y recompensas en cripto; también dashboard empresarial Neith. PitchBook indica actividad y financiamiento hasta abr-2026: sigue operando. Sin presencia conocida en Chile. Referencia directa para la hipótesis blockchain. [Vuelta 2] Sin noticias 2026 encontradas en búsqueda; sitio oficial bloqueado. [Vuelta 3] Búsqueda adicional solo devuelve hitos de 2017 (token sale US$7,2M) y 2019 (Serie A de US$5,3M, cierre no confirmado); sin datos 2025-26 propios. [Vuelta 4] App pública lanzada en la conferencia JP Morgan Healthcare (2019); red PTOYMatrix (blockchain HIPAA); socios reportados: StartUp Health y Kaiser Permanente (beta). Estado actual en App Store/Google Play sin confirmar. [Vuelta 5] Sin noticias 2026 del equipo. Token PTOY con capitalización de ~US$53K a fines de ago-2026 según Phantom (KuCoin discrepa en la circulación): señal de baja actividad, no prueba de cierre. Esto relativiza la actividad hasta abr-2026 mencionada en la ficha original. [Vuelta 6] Sin noticias posteriores a 2020 localizadas (hitos: token sale 2017, consorcio Hyperledger, alianza con Georgia State, Series A de US$5,3M vía R/GA Ventures, Neith con Prosper Healthtech en Birmingham). Estado actual desconocido. [Vuelta 7] Sin búsqueda nueva (saturado); sin cambios.</t>
+          <t>[BLOCKCHAIN · EE.UU.] Atlanta, fundada 2015, ~9 empleados. Levantó US$7,2M vía financiamiento cripto. App con registros de hospitales y wearables, coaching de salud con IA y recompensas en cripto; también dashboard empresarial Neith. PitchBook indica actividad y financiamiento hasta abr-2026: sigue operando. Sin presencia conocida en Chile. Referencia directa para la hipótesis blockchain. [Vuelta 2] Sin noticias 2026 encontradas en búsqueda; sitio oficial bloqueado. [Vuelta 3] Búsqueda adicional solo devuelve hitos de 2017 (token sale US$7,2M) y 2019 (Serie A de US$5,3M, cierre no confirmado); sin datos 2025-26 propios. [Vuelta 4] App pública lanzada en la conferencia JP Morgan Healthcare (2019); red PTOYMatrix (blockchain HIPAA); socios reportados: StartUp Health y Kaiser Permanente (beta). Estado actual en App Store/Google Play sin confirmar. [Vuelta 5] Sin noticias 2026 del equipo. Token PTOY con capitalización de ~US$53K a fines de ago-2026 según Phantom (KuCoin discrepa en la circulación): señal de baja actividad, no prueba de cierre. Esto relativiza la actividad hasta abr-2026 mencionada en la ficha original. [Vuelta 6] Sin noticias posteriores a 2020 localizadas (hitos: token sale 2017, consorcio Hyperledger, alianza con Georgia State, Series A de US$5,3M vía R/GA Ventures, Neith con Prosper Healthtech en Birmingham). Estado actual desconocido. [Vuelta 7] Sin búsqueda nueva (saturado); sin cambios. [Vuelta 8] Sin noticias 2025-26; en 2018 la oferta se dirigía a empresas de salud, con la versión individual planificada después.</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G7" t="n">
@@ -726,7 +726,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -753,12 +753,12 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>[BLOCKCHAIN · Corea del Sur] Fundada 2017, Seúl. Blockchain propia Panacea (Cosmos SDK, mainnet 2019) para que el paciente gestione y transfiera sus registros; app Medipass para seguros. Serie A de ₩4.000 millones (Naver); alianzas con hospitales (Seoul National, Severance). Estado 2025-26 NO verificado. Referencia sobre seguros + blockchain. [Vuelta 2] Panacea incluye DID, Append Only Log, IBC y PNFT; sin anuncios 2026 localizados. [Vuelta 3] Medipass: app en Corea con 20 hospitales/aseguradoras integrados (fecha de la lista desconocida) y plan 2022 de superapp con marketplace de datos; operación actual sin confirmar. [Vuelta 4] Sin búsqueda nueva (revisada en vuelta 3); sin cambios. [Vuelta 5] Medipass: ~400.000 usuarios acumulados (CEO, jun-2022); integración con aseguradoras Shinhan Life, Samsung Fire y Hyundai Marine (2020); renovación completa en mar-2023 (dashboard de salud, gestión familiar, certificados). Sin noticias 2026 encontradas. [Vuelta 6] Medipass 2023: comunicación bidireccional hospital-paciente y chat MediTalk; en 2019 fue seleccionada para el programa gubernamental de MyData médico con Samsung Fire y SNUH. Sin estrategia 2026 localizada. Meta declarada: usar Medipass como «identificación» de salud. [Vuelta 7] Una fuente sin fecha atribuye a Medipass más de 600.000 pacientes en 14 hospitales; MoU 2019 con Severance (plataforma de facturación de seguros y detección de falsificación de datos) y piloto con Massachusetts General Hospital. Sin datos 2025-26.</t>
+          <t>[BLOCKCHAIN · Corea del Sur] Fundada 2017, Seúl. Blockchain propia Panacea (Cosmos SDK, mainnet 2019) para que el paciente gestione y transfiera sus registros; app Medipass para seguros. Serie A de ₩4.000 millones (Naver); alianzas con hospitales (Seoul National, Severance). Estado 2025-26 NO verificado. Referencia sobre seguros + blockchain. [Vuelta 2] Panacea incluye DID, Append Only Log, IBC y PNFT; sin anuncios 2026 localizados. [Vuelta 3] Medipass: app en Corea con 20 hospitales/aseguradoras integrados (fecha de la lista desconocida) y plan 2022 de superapp con marketplace de datos; operación actual sin confirmar. [Vuelta 4] Sin búsqueda nueva (revisada en vuelta 3); sin cambios. [Vuelta 5] Medipass: ~400.000 usuarios acumulados (CEO, jun-2022); integración con aseguradoras Shinhan Life, Samsung Fire y Hyundai Marine (2020); renovación completa en mar-2023 (dashboard de salud, gestión familiar, certificados). Sin noticias 2026 encontradas. [Vuelta 6] Medipass 2023: comunicación bidireccional hospital-paciente y chat MediTalk; en 2019 fue seleccionada para el programa gubernamental de MyData médico con Samsung Fire y SNUH. Sin estrategia 2026 localizada. Meta declarada: usar Medipass como «identificación» de salud. [Vuelta 7] Una fuente sin fecha atribuye a Medipass más de 600.000 pacientes en 14 hospitales; MoU 2019 con Severance (plataforma de facturación de seguros y detección de falsificación de datos) y piloto con Massachusetts General Hospital. Sin datos 2025-26. [Vuelta 8] Sin noticias 2025-26.</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G8" t="n">
@@ -766,7 +766,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -793,12 +793,12 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>[BLOCKCHAIN · Reino Unido · INACTIVO] Londres, 2017, Ethereum, con telemedicina. Piloto según registro de la UE (2020). Tracxn/PitchBook lo marcan fuera de operación (ago-2025). Solo caso de aprendizaje: no cuenta como competidor activo. [Vuelta 2] Token MTN deslistado de Bitfinex el 26-mar-2021; sin hallazgos de actividad posterior. [Vuelta 3] Seedtable la marca activa sin fuente; no hallé registro en Companies House. Sigue tratándose como caso de aprendizaje. [Vuelta 4] Pre-venta reportada de US$20M en MedTokens (un solo artículo secundario, sin verificar); modelo de token en revisión y exploración de security token según AMA; integraciones y servicios de 2019 sin confirmar. [Vuelta 5] Un agregador indica sitio medicalchain.com fuera de línea desde 15-feb-2025, último commit en GitHub hace ~3 años y proyecto en «fase de mantenimiento»; preventa de MedTokens reportada entre US$20M y US$24M (fuentes discrepan). Confirma tratarlo como inactivo. [Vuelta 6] Sin búsqueda nueva (revisada en vuelta 5; sitio fuera de línea desde feb-2025 según un agregador); sin cambios. [Vuelta 7] Sin búsqueda nueva (saturado); sin cambios.</t>
+          <t>[BLOCKCHAIN · Reino Unido · INACTIVO] Londres, 2017, Ethereum, con telemedicina. Piloto según registro de la UE (2020). Tracxn/PitchBook lo marcan fuera de operación (ago-2025). Solo caso de aprendizaje: no cuenta como competidor activo. [Vuelta 2] Token MTN deslistado de Bitfinex el 26-mar-2021; sin hallazgos de actividad posterior. [Vuelta 3] Seedtable la marca activa sin fuente; no hallé registro en Companies House. Sigue tratándose como caso de aprendizaje. [Vuelta 4] Pre-venta reportada de US$20M en MedTokens (un solo artículo secundario, sin verificar); modelo de token en revisión y exploración de security token según AMA; integraciones y servicios de 2019 sin confirmar. [Vuelta 5] Un agregador indica sitio medicalchain.com fuera de línea desde 15-feb-2025, último commit en GitHub hace ~3 años y proyecto en «fase de mantenimiento»; preventa de MedTokens reportada entre US$20M y US$24M (fuentes discrepan). Confirma tratarlo como inactivo. [Vuelta 6] Sin búsqueda nueva (revisada en vuelta 5; sitio fuera de línea desde feb-2025 según un agregador); sin cambios. [Vuelta 7] Sin búsqueda nueva (saturado); sin cambios. [Vuelta 8] Sin fuentes nuevas; se mantiene como inactivo.</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G9" t="n">
@@ -806,7 +806,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -10721,7 +10721,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A35"/>
+  <dimension ref="A1:A36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -10972,6 +10972,13 @@
         </is>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Vuelta 8 (iter. 2, 2026-10-22 12:28 UTC): Healfies, Patientory, MediBloc, Medicalchain verificados (+0 filas; saturado). Pendientes: Apple Health, ChatGPT Health, Claude for Healthcare, Apps de clínicas, Clinia, MiRedSalud, Mediko.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Benchmark: vuelta 8, iteración 3 (Apple Health, ChatGPT Health, Claude for Healthcare, Apps de clínicas)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MVcXu8vTBu7EKfj3YdEvae
</commit_message>
<xml_diff>
--- a/Outputs/Benchmark_Anamnesis.xlsx
+++ b/Outputs/Benchmark_Anamnesis.xlsx
@@ -833,12 +833,12 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>[ADYACENTE · global] Agrega registros clínicos vía FHIR; &gt;500 instituciones conectadas en EE.UU. (2018). Sin evidencia de disponibilidad en Chile. Incluida en el dispositivo. Amenaza si FHIR/IPS-CL se adopta en Chile. [Vuelta 2] Sin disponibilidad de registros clínicos en Chile (solo EE.UU., Reino Unido, Canadá). [Vuelta 3] iOS 27 (WWDC 8-jun-2026; publicado ~14-sep-2026): rediseño del app Health, menopausia, nutrición por cámara. El coach de salud con IA no se anunció. Sin ampliación de Health Records a Chile. [Vuelta 4] Sin búsqueda nueva (revisada en vuelta 3); sin cambios. [Vuelta 5] Sin ampliación de Health Records a Australia, Europa ni Latinoamérica (solo EE.UU., UK, Canadá). Funciones de dispositivo (apnea del sueño, prueba auditiva) sí se amplían a países latinoamericanos, pero no son registros clínicos. [Vuelta 6] Sin novedades de iOS 27.x localizadas. Health Records API permite compartir registros con apps de terceros con control por app; opción de enviar datos de uso a Apple. [Vuelta 7] Coach de salud con IA / Health+ de pago: solo rumores (Gurman), atrasado al menos a iOS 27; no confirmado ni anunciado.</t>
+          <t>[ADYACENTE · global] Agrega registros clínicos vía FHIR; &gt;500 instituciones conectadas en EE.UU. (2018). Sin evidencia de disponibilidad en Chile. Incluida en el dispositivo. Amenaza si FHIR/IPS-CL se adopta en Chile. [Vuelta 2] Sin disponibilidad de registros clínicos en Chile (solo EE.UU., Reino Unido, Canadá). [Vuelta 3] iOS 27 (WWDC 8-jun-2026; publicado ~14-sep-2026): rediseño del app Health, menopausia, nutrición por cámara. El coach de salud con IA no se anunció. Sin ampliación de Health Records a Chile. [Vuelta 4] Sin búsqueda nueva (revisada en vuelta 3); sin cambios. [Vuelta 5] Sin ampliación de Health Records a Australia, Europa ni Latinoamérica (solo EE.UU., UK, Canadá). Funciones de dispositivo (apnea del sueño, prueba auditiva) sí se amplían a países latinoamericanos, pero no son registros clínicos. [Vuelta 6] Sin novedades de iOS 27.x localizadas. Health Records API permite compartir registros con apps de terceros con control por app; opción de enviar datos de uso a Apple. [Vuelta 7] Coach de salud con IA / Health+ de pago: solo rumores (Gurman), atrasado al menos a iOS 27; no confirmado ni anunciado. [Vuelta 8] Sin novedades.</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G10" t="n">
@@ -846,7 +846,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-23</t>
         </is>
       </c>
     </row>
@@ -873,12 +873,12 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>[ADYACENTE · global] Lanzado 7-ene-2026. Conecta registros médicos; conectores solo en EE.UU. Dentro de suscripción del asistente. Fija la expectativa de consultar y resumir el historial. [Vuelta 2] Confirmado: registros solo EE.UU.; sin anuncios para Latinoamérica. Hay inconsistencia de fechas entre fuentes (7-ene-2026 lanzamiento vs. jul-2026 despliegue de registros). [Vuelta 3] Fechas aclaradas: presentación 7-ene-2026 (acceso limitado); despliegue de Health in ChatGPT con Apple Health y registros en EE.UU. el 23-jul-2026; mejora de salud jun-2026. Sin anuncios para Latinoamérica ni para sep-oct 2026. [Vuelta 4] Septiembre 2026: permisos por defecto para datos conectados (14-sep) y explicaciones por gráfico/métrica (28-sep); ChatGPT for Clinicians (abr-2026) para clínicos verificados de EE.UU. Más del 70% de usuarios de Health permite usar datos conectados sin pedir permiso (según OpenAI). Sigue solo EE.UU. [Vuelta 5] Nota de jul-2026: Health no está disponible en México, Android, modo de voz ni Codex; web e iOS en EE.UU., adultos con sesión iniciada. Sin anuncio para Chile ni Latinoamérica. [Vuelta 6] Última entrada de Health en las notas de OpenAI sigue siendo la del 23-jul-2026 (más cambios de sep); sin entradas de octubre localizadas. Health tab: laboratorios, medicamentos, actividad y sueño en una vista; solo EE.UU., web e iOS. [Vuelta 7] OpenAI afirma que más de 300 millones de personas usan ChatGPT cada semana para consultas de salud (dato de la empresa). No es una solución con cumplimiento HIPAA declarado. Sin novedades de oct-2026.</t>
+          <t>[ADYACENTE · global] Lanzado 7-ene-2026. Conecta registros médicos; conectores solo en EE.UU. Dentro de suscripción del asistente. Fija la expectativa de consultar y resumir el historial. [Vuelta 2] Confirmado: registros solo EE.UU.; sin anuncios para Latinoamérica. Hay inconsistencia de fechas entre fuentes (7-ene-2026 lanzamiento vs. jul-2026 despliegue de registros). [Vuelta 3] Fechas aclaradas: presentación 7-ene-2026 (acceso limitado); despliegue de Health in ChatGPT con Apple Health y registros en EE.UU. el 23-jul-2026; mejora de salud jun-2026. Sin anuncios para Latinoamérica ni para sep-oct 2026. [Vuelta 4] Septiembre 2026: permisos por defecto para datos conectados (14-sep) y explicaciones por gráfico/métrica (28-sep); ChatGPT for Clinicians (abr-2026) para clínicos verificados de EE.UU. Más del 70% de usuarios de Health permite usar datos conectados sin pedir permiso (según OpenAI). Sigue solo EE.UU. [Vuelta 5] Nota de jul-2026: Health no está disponible en México, Android, modo de voz ni Codex; web e iOS en EE.UU., adultos con sesión iniciada. Sin anuncio para Chile ni Latinoamérica. [Vuelta 6] Última entrada de Health en las notas de OpenAI sigue siendo la del 23-jul-2026 (más cambios de sep); sin entradas de octubre localizadas. Health tab: laboratorios, medicamentos, actividad y sueño en una vista; solo EE.UU., web e iOS. [Vuelta 7] OpenAI afirma que más de 300 millones de personas usan ChatGPT cada semana para consultas de salud (dato de la empresa). No es una solución con cumplimiento HIPAA declarado. Sin novedades de oct-2026. [Vuelta 8] Sin novedades de fines de oct-2026.</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G11" t="n">
@@ -886,7 +886,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-23</t>
         </is>
       </c>
     </row>
@@ -913,12 +913,12 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>[ADYACENTE · global] Lanzado 11-ene-2026. Conectores solo en EE.UU., planes Pro/Max. Nota: producto de Anthropic, conflicto de interés al evaluarlo. [Vuelta 2] Sin cambios fuera de EE.UU. (HealthEx y Function para Pro/Max). [Vuelta 3] Sin anuncios posteriores a enero de 2026. Hoja de ruta de HealthEx (agendar, buscar prestadores, recetas) sin confirmar como lanzada. [Vuelta 4] Sin anuncios nuevos. Fuentes discrepan en el acceso (Pro/Max según Fortune y la mayoría; Pro/Team según Times of AI); sin evidencia de disponibilidad fuera de EE.UU. [Vuelta 5] Sin noticias de oct-2026; HealthEx agrega datos de &gt;50.000 sistemas de EE.UU. y Claude pide solo las categorías relevantes vía MCP. [Vuelta 6] Sin noticias posteriores a enero de 2026 localizadas. [Vuelta 7] Sin novedades posteriores a enero de 2026.</t>
+          <t>[ADYACENTE · global] Lanzado 11-ene-2026. Conectores solo en EE.UU., planes Pro/Max. Nota: producto de Anthropic, conflicto de interés al evaluarlo. [Vuelta 2] Sin cambios fuera de EE.UU. (HealthEx y Function para Pro/Max). [Vuelta 3] Sin anuncios posteriores a enero de 2026. Hoja de ruta de HealthEx (agendar, buscar prestadores, recetas) sin confirmar como lanzada. [Vuelta 4] Sin anuncios nuevos. Fuentes discrepan en el acceso (Pro/Max según Fortune y la mayoría; Pro/Team según Times of AI); sin evidencia de disponibilidad fuera de EE.UU. [Vuelta 5] Sin noticias de oct-2026; HealthEx agrega datos de &gt;50.000 sistemas de EE.UU. y Claude pide solo las categorías relevantes vía MCP. [Vuelta 6] Sin noticias posteriores a enero de 2026 localizadas. [Vuelta 7] Sin novedades posteriores a enero de 2026. [Vuelta 8] Sin novedades posteriores a enero de 2026.</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G12" t="n">
@@ -926,7 +926,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-23</t>
         </is>
       </c>
     </row>
@@ -953,12 +953,12 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>[SUSTITUTO PARCIAL · Chile] Reservar hora, ver historial de esa institución, vincular familiar. Gratis; no consolida datos de otras instituciones. [Vuelta 2] App concreta: Mi Alemana Go (Clínica Alemana, Chile), con historial desde 2018, recetas, órdenes, familiar vinculado y resultados. [Vuelta 3] Búsqueda de otras clínicas (Las Condes, Santa María, UC Christus) sin ficha de app confirmada; solo canales digitales genéricos. [Vuelta 4] Mi Alemana Go: 3,1/5 con 137 calificaciones (App Store Chile), pantalla de inicio rediseñada para gestionar salud propia y familiar; sin evidencia de teleconsulta ni pagos en la app. [Vuelta 5] Sin búsqueda nueva (revisada en vuelta 4); sin cambios. [Vuelta 6] Sin búsqueda nueva; sin cambios. [Vuelta 7] Sin búsqueda nueva; sin cambios.</t>
+          <t>[SUSTITUTO PARCIAL · Chile] Reservar hora, ver historial de esa institución, vincular familiar. Gratis; no consolida datos de otras instituciones. [Vuelta 2] App concreta: Mi Alemana Go (Clínica Alemana, Chile), con historial desde 2018, recetas, órdenes, familiar vinculado y resultados. [Vuelta 3] Búsqueda de otras clínicas (Las Condes, Santa María, UC Christus) sin ficha de app confirmada; solo canales digitales genéricos. [Vuelta 4] Mi Alemana Go: 3,1/5 con 137 calificaciones (App Store Chile), pantalla de inicio rediseñada para gestionar salud propia y familiar; sin evidencia de teleconsulta ni pagos en la app. [Vuelta 5] Sin búsqueda nueva (revisada en vuelta 4); sin cambios. [Vuelta 6] Sin búsqueda nueva; sin cambios. [Vuelta 7] Sin búsqueda nueva; sin cambios. [Vuelta 8] Mi Alemana Go: notificaciones de deuda pendiente, check-in de admisión y encuestas de salud; DF la describe como segundo paso de la estrategia digital de la clínica (registros de exámenes, indicaciones, historial y recetas). Otras apps de red: Mi Dávila (Red Dávila, gestión de citas en todos sus centros, según un directorio); Clínica Las Condes sin app confirmada.</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G13" t="n">
@@ -966,7 +966,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-23</t>
         </is>
       </c>
     </row>
@@ -1102,7 +1102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F132"/>
+  <dimension ref="A1:F134"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -5334,6 +5334,70 @@
       <c r="F132" t="inlineStr">
         <is>
           <t>Búsqueda web (Baguete, 2016); estado actual no verificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>Apps de clínicas (ej. Clínica Alemana de Valdivia)</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>Seguros y pagos</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Aviso de deudas pendientes y pago (Mi Alemana Go)</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>Sección de notificaciones que avisa cuando hay una deuda disponible para pagar (fecha de la actualización desconocida).</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>Ficha App Store Chile (Mi Alemana Go)</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>Apps de clínicas (ej. Clínica Alemana de Valdivia)</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Citas y agenda</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Check-in de admisión y encuestas de salud (Mi Alemana Go)</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>Notificaciones de check-in de admisión y encuestas de salud previas a la atención.</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>Ficha App Store Chile (Mi Alemana Go)</t>
         </is>
       </c>
     </row>
@@ -10721,7 +10785,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A36"/>
+  <dimension ref="A1:A37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -10979,6 +11043,13 @@
         </is>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Vuelta 8 (iter. 3, 2026-10-23 12:17 UTC): Apple Health, ChatGPT Health, Claude for Healthcare, Apps de clínicas verificados (+2 filas, de Apps de clínicas). Pendientes: Clinia, MiRedSalud, Mediko (cierran la vuelta 8 y regeneran func_norm/tabla_frecuencia).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Benchmark: vuelta 9, iteración 1 (Meedika, Infomed, MediPlanner, Clingot); candidatos Medicyn y DKV
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MVcXu8vTBu7EKfj3YdEvae
</commit_message>
<xml_diff>
--- a/Outputs/Benchmark_Anamnesis.xlsx
+++ b/Outputs/Benchmark_Anamnesis.xlsx
@@ -513,12 +513,12 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>[DIRECTO · Chile · etapas A+B] Lanzada 25-sep-2024 en App Store (Android previsto la misma semana). &gt;1.500 usuarios en los primeros días; meta 32.000 (cofundador Francisco González). Funciones: gestión de documentos, importar solicitudes, SOS con alergias/medicación, calendario de citas, recordatorios, compartir con profesionales elegidos. Sin blockchain. Precio y estado actual NO verificados; única fuente es una nota de prensa. Sitio oficial por confirmar. [Iter. 2] Hay cobertura adicional en Portal Innova (portalinnova.cl); sitio bloqueado en este entorno, estado actual sigue sin verificar. [Vuelta 3] Sin novedades 2026 ni confirmación de la app Android en Google Play; usuarios actuales desconocidos. Nota de prensa no indica año de lanzamiento explícito. [Vuelta 4] Sin fuentes nuevas; portalinnova.cl no aparece en búsquedas. Sigue dependiendo de una sola nota de prensa. [Vuelta 5] Sin fuentes nuevas (ni entrevistas ni financiamiento); sigue dependiendo de una sola nota de prensa sin año explícito. [Vuelta 6] Sin ficha de Google Play ni fuentes nuevas; disponibilidad en Android sin confirmar. [Vuelta 7] Sin fuentes nuevas; no hay ficha oficial localizada. No confundir con apps de nombre parecido (Medika App, MEDDI, AI Medik). [Vuelta 8] Sin fuentes nuevas.</t>
+          <t>[DIRECTO · Chile · etapas A+B] Lanzada 25-sep-2024 en App Store (Android previsto la misma semana). &gt;1.500 usuarios en los primeros días; meta 32.000 (cofundador Francisco González). Funciones: gestión de documentos, importar solicitudes, SOS con alergias/medicación, calendario de citas, recordatorios, compartir con profesionales elegidos. Sin blockchain. Precio y estado actual NO verificados; única fuente es una nota de prensa. Sitio oficial por confirmar. [Iter. 2] Hay cobertura adicional en Portal Innova (portalinnova.cl); sitio bloqueado en este entorno, estado actual sigue sin verificar. [Vuelta 3] Sin novedades 2026 ni confirmación de la app Android en Google Play; usuarios actuales desconocidos. Nota de prensa no indica año de lanzamiento explícito. [Vuelta 4] Sin fuentes nuevas; portalinnova.cl no aparece en búsquedas. Sigue dependiendo de una sola nota de prensa. [Vuelta 5] Sin fuentes nuevas (ni entrevistas ni financiamiento); sigue dependiendo de una sola nota de prensa sin año explícito. [Vuelta 6] Sin ficha de Google Play ni fuentes nuevas; disponibilidad en Android sin confirmar. [Vuelta 7] Sin fuentes nuevas; no hay ficha oficial localizada. No confundir con apps de nombre parecido (Medika App, MEDDI, AI Medik). [Vuelta 8] Sin fuentes nuevas. [Vuelta 9] Sin fuentes nuevas.</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G2" t="n">
@@ -526,7 +526,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
@@ -553,12 +553,12 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>[DIRECTO · Chile · etapa A] Fundada 2019 por Diego Ibarra, Andrés Fantuzzi y Gabriel Zamora. Lanzada mar-2021 en App Store y Play Store con 1.200 usuarios; planeaba nueva versión jul-2021 y ronda de US$500 mil. Objetivo: llevar el historial en el celular, acceso en emergencias, médico puede ingresar datos con consentimiento. Estado actual NO verificado (posible app inactiva). URL es la nota de prensa; sitio oficial por confirmar. [Vuelta 3] Sin evidencia posterior a 2021; relanzamiento previsto jul-2021 no confirmado. Probable app inactiva. [Vuelta 4] Sin cambios; sigue sin evidencia posterior a 2021. [Vuelta 5] Cofundador Andrés Fantuzzi es cardiólogo de la Clínica Santa María. Sin ronda de inversión ni relanzamiento confirmados; no confundir con Infomed de Cuba (portal del Minsap). [Vuelta 6] Sin búsqueda nueva (fuentes agotadas en vueltas 3-5); sin cambios. [Vuelta 7] Sin búsqueda nueva (saturado); sin cambios. [Vuelta 8] Sin fuentes nuevas; relanzamiento de jul-2021 sigue sin confirmarse.</t>
+          <t>[DIRECTO · Chile · etapa A] Fundada 2019 por Diego Ibarra, Andrés Fantuzzi y Gabriel Zamora. Lanzada mar-2021 en App Store y Play Store con 1.200 usuarios; planeaba nueva versión jul-2021 y ronda de US$500 mil. Objetivo: llevar el historial en el celular, acceso en emergencias, médico puede ingresar datos con consentimiento. Estado actual NO verificado (posible app inactiva). URL es la nota de prensa; sitio oficial por confirmar. [Vuelta 3] Sin evidencia posterior a 2021; relanzamiento previsto jul-2021 no confirmado. Probable app inactiva. [Vuelta 4] Sin cambios; sigue sin evidencia posterior a 2021. [Vuelta 5] Cofundador Andrés Fantuzzi es cardiólogo de la Clínica Santa María. Sin ronda de inversión ni relanzamiento confirmados; no confundir con Infomed de Cuba (portal del Minsap). [Vuelta 6] Sin búsqueda nueva (fuentes agotadas en vueltas 3-5); sin cambios. [Vuelta 7] Sin búsqueda nueva (saturado); sin cambios. [Vuelta 8] Sin fuentes nuevas; relanzamiento de jul-2021 sigue sin confirmarse. [Vuelta 9] Sin fuentes nuevas.</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G3" t="n">
@@ -566,7 +566,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
@@ -593,12 +593,12 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>[REGIONAL · México] Historial por perfil familiar, alergias, vacunas, recetas digitales, gráficas de evolución, agendamiento, compartir con profesionales. Gratis en App Store MX. Sin evidencia de uso en Chile. Cubre parte de la etapa C (familia). [Vuelta 3] Existen dos apps distintas: MediPlanner (gratis, Rym Solutions, MX, 3,7/5 con 3 calificaciones) y MediPlanner Pro (otro desarrollador, $39 MXN). Sin presencia verificada en Chile. [Vuelta 4] No pude confirmar el desarrollador de la versión gratuita (Rym Solutions no se repite en esta búsqueda). MediPlanner Pro (fichas BR/OM) guardaría datos solo en el dispositivo, sin nube; no confundir con MedPlanner/AskHEMI (otra empresa). [Vuelta 5] Sin búsqueda nueva (revisada en vuelta 4); sin cambios. [Vuelta 6] Se reconfirma en la ficha de App Store MX que el desarrollador de la versión gratuita es Rym Solutions S. de R.L. de C.V. (3,7/5, 3 calificaciones); MediPlanner Pro no menciona a esa empresa, por lo que no se puede asegurar que sea el mismo desarrollador. [Vuelta 7] Sin búsqueda nueva (saturado); sin cambios. [Vuelta 8] Sin búsqueda nueva (saturado).</t>
+          <t>[REGIONAL · México] Historial por perfil familiar, alergias, vacunas, recetas digitales, gráficas de evolución, agendamiento, compartir con profesionales. Gratis en App Store MX. Sin evidencia de uso en Chile. Cubre parte de la etapa C (familia). [Vuelta 3] Existen dos apps distintas: MediPlanner (gratis, Rym Solutions, MX, 3,7/5 con 3 calificaciones) y MediPlanner Pro (otro desarrollador, $39 MXN). Sin presencia verificada en Chile. [Vuelta 4] No pude confirmar el desarrollador de la versión gratuita (Rym Solutions no se repite en esta búsqueda). MediPlanner Pro (fichas BR/OM) guardaría datos solo en el dispositivo, sin nube; no confundir con MedPlanner/AskHEMI (otra empresa). [Vuelta 5] Sin búsqueda nueva (revisada en vuelta 4); sin cambios. [Vuelta 6] Se reconfirma en la ficha de App Store MX que el desarrollador de la versión gratuita es Rym Solutions S. de R.L. de C.V. (3,7/5, 3 calificaciones); MediPlanner Pro no menciona a esa empresa, por lo que no se puede asegurar que sea el mismo desarrollador. [Vuelta 7] Sin búsqueda nueva (saturado); sin cambios. [Vuelta 8] Sin búsqueda nueva (saturado). [Vuelta 9] Sin fuentes nuevas.</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G4" t="n">
@@ -606,7 +606,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
@@ -633,12 +633,12 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>[REGIONAL · Argentina · débil] App para cargar antecedentes médicos propios. Única referencia: nota de opinión en grupoanimal.mx sin fecha verificada. Estado y sitio por confirmar. [Vuelta 3] Referencias de 2017 (apps4citizens, La Nación); sitio y precio no verificados; puede estar inactiva. [Vuelta 4] Sin fuentes nuevas. [Vuelta 5] Registro empresarial (indicadores.ar, datos a jul-2026) muestra CLINGOT S.A. activa en CABA, constituida el 4-abr-2016; no confirma que la app siga operando. Programa federal argentino de historias clínicas digitales como contexto regulatorio. [Vuelta 6] Sin búsqueda nueva (fuentes agotadas); sin cambios. [Vuelta 7] Solo fuentes de 2017; sin evidencia nueva de operación más allá del registro societario. [Vuelta 8] Sin fuentes nuevas.</t>
+          <t>[REGIONAL · Argentina · débil] App para cargar antecedentes médicos propios. Única referencia: nota de opinión en grupoanimal.mx sin fecha verificada. Estado y sitio por confirmar. [Vuelta 3] Referencias de 2017 (apps4citizens, La Nación); sitio y precio no verificados; puede estar inactiva. [Vuelta 4] Sin fuentes nuevas. [Vuelta 5] Registro empresarial (indicadores.ar, datos a jul-2026) muestra CLINGOT S.A. activa en CABA, constituida el 4-abr-2016; no confirma que la app siga operando. Programa federal argentino de historias clínicas digitales como contexto regulatorio. [Vuelta 6] Sin búsqueda nueva (fuentes agotadas); sin cambios. [Vuelta 7] Solo fuentes de 2017; sin evidencia nueva de operación más allá del registro societario. [Vuelta 8] Sin fuentes nuevas. [Vuelta 9] Sin fuentes nuevas.</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G5" t="n">
@@ -646,7 +646,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
@@ -9177,8 +9177,6 @@
           <t>Búsqueda de profesionales de salud</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9189,17 +9187,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
       <c r="R2">
         <f>COUNTIF(C2:Q2,"✓")</f>
         <v/>
@@ -9221,24 +9208,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
       <c r="R3">
         <f>COUNTIF(C3:Q3,"✓")</f>
         <v/>
@@ -9255,25 +9229,11 @@
           <t>Check-in de admisión digital</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
       <c r="R4">
         <f>COUNTIF(C4:Q4,"✓")</f>
         <v/>
@@ -9290,25 +9250,11 @@
           <t>Integración con calendario del dispositivo</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr"/>
       <c r="R5">
         <f>COUNTIF(C5:Q5,"✓")</f>
         <v/>
@@ -9325,25 +9271,11 @@
           <t>Localización de centros médicos y farmacias</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="inlineStr"/>
       <c r="R6">
         <f>COUNTIF(C6:Q6,"✓")</f>
         <v/>
@@ -9360,21 +9292,11 @@
           <t>Reserva de citas médicas</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9385,8 +9307,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="P7" t="inlineStr"/>
-      <c r="Q7" t="inlineStr"/>
       <c r="R7">
         <f>COUNTIF(C7:Q7,"✓")</f>
         <v/>
@@ -9403,25 +9323,11 @@
           <t>Acceso del profesional al historial del paciente</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
-      <c r="P8" t="inlineStr"/>
-      <c r="Q8" t="inlineStr"/>
       <c r="R8">
         <f>COUNTIF(C8:Q8,"✓")</f>
         <v/>
@@ -9438,25 +9344,11 @@
           <t>Compartir con personas sin cuenta mediante clave segura</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
-      <c r="P9" t="inlineStr"/>
-      <c r="Q9" t="inlineStr"/>
       <c r="R9">
         <f>COUNTIF(C9:Q9,"✓")</f>
         <v/>
@@ -9473,25 +9365,11 @@
           <t>Compartir datos con cuidador o persona de confianza</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
-      <c r="O10" t="inlineStr"/>
-      <c r="P10" t="inlineStr"/>
-      <c r="Q10" t="inlineStr"/>
       <c r="R10">
         <f>COUNTIF(C10:Q10,"✓")</f>
         <v/>
@@ -9513,13 +9391,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9545,16 +9421,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="P11" t="inlineStr"/>
-      <c r="Q11" t="inlineStr"/>
       <c r="R11">
         <f>COUNTIF(C11:Q11,"✓")</f>
         <v/>
@@ -9571,25 +9442,11 @@
           <t>Gestión de consentimiento sobre uso de datos</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
-      <c r="O12" t="inlineStr"/>
-      <c r="P12" t="inlineStr"/>
-      <c r="Q12" t="inlineStr"/>
       <c r="R12">
         <f>COUNTIF(C12:Q12,"✓")</f>
         <v/>
@@ -9606,25 +9463,11 @@
           <t>Ingreso de datos por profesional con consentimiento</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr"/>
-      <c r="O13" t="inlineStr"/>
-      <c r="P13" t="inlineStr"/>
-      <c r="Q13" t="inlineStr"/>
       <c r="R13">
         <f>COUNTIF(C13:Q13,"✓")</f>
         <v/>
@@ -9641,25 +9484,11 @@
           <t>Red social con profesionales y familiares</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
-      <c r="M14" t="inlineStr"/>
-      <c r="N14" t="inlineStr"/>
-      <c r="O14" t="inlineStr"/>
-      <c r="P14" t="inlineStr"/>
-      <c r="Q14" t="inlineStr"/>
       <c r="R14">
         <f>COUNTIF(C14:Q14,"✓")</f>
         <v/>
@@ -9686,23 +9515,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr"/>
-      <c r="N15" t="inlineStr"/>
-      <c r="O15" t="inlineStr"/>
-      <c r="P15" t="inlineStr"/>
-      <c r="Q15" t="inlineStr"/>
       <c r="R15">
         <f>COUNTIF(C15:Q15,"✓")</f>
         <v/>
@@ -9719,8 +9536,6 @@
           <t>Perfiles familiares / dependientes</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9731,29 +9546,21 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
-      <c r="M16" t="inlineStr"/>
       <c r="N16" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="Q16" t="inlineStr"/>
       <c r="R16">
         <f>COUNTIF(C16:Q16,"✓")</f>
         <v/>
@@ -9775,8 +9582,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9792,19 +9597,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr"/>
-      <c r="N17" t="inlineStr"/>
       <c r="O17" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="P17" t="inlineStr"/>
-      <c r="Q17" t="inlineStr"/>
       <c r="R17">
         <f>COUNTIF(C17:Q17,"✓")</f>
         <v/>
@@ -9821,29 +9618,16 @@
           <t>Almacenamiento de recetas</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr"/>
-      <c r="M18" t="inlineStr"/>
       <c r="N18" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="O18" t="inlineStr"/>
-      <c r="P18" t="inlineStr"/>
-      <c r="Q18" t="inlineStr"/>
       <c r="R18">
         <f>COUNTIF(C18:Q18,"✓")</f>
         <v/>
@@ -9860,25 +9644,11 @@
           <t>Búsqueda y filtros de documentos</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr"/>
-      <c r="M19" t="inlineStr"/>
-      <c r="N19" t="inlineStr"/>
-      <c r="O19" t="inlineStr"/>
-      <c r="P19" t="inlineStr"/>
-      <c r="Q19" t="inlineStr"/>
       <c r="R19">
         <f>COUNTIF(C19:Q19,"✓")</f>
         <v/>
@@ -9895,25 +9665,11 @@
           <t>Emisión de certificados médicos</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr"/>
-      <c r="M20" t="inlineStr"/>
-      <c r="N20" t="inlineStr"/>
-      <c r="O20" t="inlineStr"/>
-      <c r="P20" t="inlineStr"/>
-      <c r="Q20" t="inlineStr"/>
       <c r="R20">
         <f>COUNTIF(C20:Q20,"✓")</f>
         <v/>
@@ -9935,19 +9691,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr"/>
-      <c r="M21" t="inlineStr"/>
-      <c r="N21" t="inlineStr"/>
-      <c r="O21" t="inlineStr"/>
-      <c r="P21" t="inlineStr"/>
       <c r="Q21" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9969,25 +9712,11 @@
           <t>Notificación y envío de resultados</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
-      <c r="L22" t="inlineStr"/>
-      <c r="M22" t="inlineStr"/>
       <c r="N22" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="O22" t="inlineStr"/>
-      <c r="P22" t="inlineStr"/>
-      <c r="Q22" t="inlineStr"/>
       <c r="R22">
         <f>COUNTIF(C22:Q22,"✓")</f>
         <v/>
@@ -10004,25 +9733,11 @@
           <t>Recepción de documentos desde terceros</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
-      <c r="L23" t="inlineStr"/>
-      <c r="M23" t="inlineStr"/>
-      <c r="N23" t="inlineStr"/>
-      <c r="O23" t="inlineStr"/>
-      <c r="P23" t="inlineStr"/>
-      <c r="Q23" t="inlineStr"/>
       <c r="R23">
         <f>COUNTIF(C23:Q23,"✓")</f>
         <v/>
@@ -10039,29 +9754,16 @@
           <t>Historial institucional (solo datos de la propia red)</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
-      <c r="L24" t="inlineStr"/>
-      <c r="M24" t="inlineStr"/>
       <c r="N24" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="O24" t="inlineStr"/>
       <c r="P24" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="Q24" t="inlineStr"/>
       <c r="R24">
         <f>COUNTIF(C24:Q24,"✓")</f>
         <v/>
@@ -10078,36 +9780,26 @@
           <t>Historial médico centralizado</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="L25" t="inlineStr"/>
-      <c r="M25" t="inlineStr"/>
-      <c r="N25" t="inlineStr"/>
-      <c r="O25" t="inlineStr"/>
-      <c r="P25" t="inlineStr"/>
       <c r="Q25" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10129,25 +9821,11 @@
           <t>Línea de tiempo de salud</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr"/>
-      <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr"/>
-      <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
-      <c r="L26" t="inlineStr"/>
-      <c r="M26" t="inlineStr"/>
-      <c r="N26" t="inlineStr"/>
-      <c r="O26" t="inlineStr"/>
-      <c r="P26" t="inlineStr"/>
-      <c r="Q26" t="inlineStr"/>
       <c r="R26">
         <f>COUNTIF(C26:Q26,"✓")</f>
         <v/>
@@ -10164,25 +9842,11 @@
           <t>Registro de alergias y vacunas</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr"/>
-      <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr"/>
-      <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
-      <c r="L27" t="inlineStr"/>
-      <c r="M27" t="inlineStr"/>
-      <c r="N27" t="inlineStr"/>
-      <c r="O27" t="inlineStr"/>
-      <c r="P27" t="inlineStr"/>
-      <c r="Q27" t="inlineStr"/>
       <c r="R27">
         <f>COUNTIF(C27:Q27,"✓")</f>
         <v/>
@@ -10199,25 +9863,11 @@
           <t>Seguimiento de visitas, gastos y seguros</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr"/>
-      <c r="M28" t="inlineStr"/>
-      <c r="N28" t="inlineStr"/>
-      <c r="O28" t="inlineStr"/>
-      <c r="P28" t="inlineStr"/>
-      <c r="Q28" t="inlineStr"/>
       <c r="R28">
         <f>COUNTIF(C28:Q28,"✓")</f>
         <v/>
@@ -10234,11 +9884,6 @@
           <t>Recompensas / monetización de datos del usuario</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr"/>
-      <c r="D29" t="inlineStr"/>
-      <c r="E29" t="inlineStr"/>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10254,13 +9899,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="K29" t="inlineStr"/>
-      <c r="L29" t="inlineStr"/>
-      <c r="M29" t="inlineStr"/>
-      <c r="N29" t="inlineStr"/>
-      <c r="O29" t="inlineStr"/>
-      <c r="P29" t="inlineStr"/>
-      <c r="Q29" t="inlineStr"/>
       <c r="R29">
         <f>COUNTIF(C29:Q29,"✓")</f>
         <v/>
@@ -10277,25 +9915,11 @@
           <t>Asistente de IA para profesionales de salud</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr"/>
-      <c r="E30" t="inlineStr"/>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr"/>
-      <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="M30" t="inlineStr"/>
-      <c r="N30" t="inlineStr"/>
-      <c r="O30" t="inlineStr"/>
-      <c r="P30" t="inlineStr"/>
-      <c r="Q30" t="inlineStr"/>
       <c r="R30">
         <f>COUNTIF(C30:Q30,"✓")</f>
         <v/>
@@ -10312,25 +9936,11 @@
           <t>Coaching de salud con IA</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr"/>
-      <c r="D31" t="inlineStr"/>
-      <c r="E31" t="inlineStr"/>
-      <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr"/>
-      <c r="L31" t="inlineStr"/>
-      <c r="M31" t="inlineStr"/>
-      <c r="N31" t="inlineStr"/>
-      <c r="O31" t="inlineStr"/>
-      <c r="P31" t="inlineStr"/>
-      <c r="Q31" t="inlineStr"/>
       <c r="R31">
         <f>COUNTIF(C31:Q31,"✓")</f>
         <v/>
@@ -10347,15 +9957,6 @@
           <t>Detección de patrones en métricas de salud con IA</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr"/>
-      <c r="D32" t="inlineStr"/>
-      <c r="E32" t="inlineStr"/>
-      <c r="F32" t="inlineStr"/>
-      <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr"/>
-      <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr"/>
-      <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10366,10 +9967,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="N32" t="inlineStr"/>
-      <c r="O32" t="inlineStr"/>
-      <c r="P32" t="inlineStr"/>
-      <c r="Q32" t="inlineStr"/>
       <c r="R32">
         <f>COUNTIF(C32:Q32,"✓")</f>
         <v/>
@@ -10386,15 +9983,6 @@
           <t>Interpretación de exámenes con IA</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr"/>
-      <c r="D33" t="inlineStr"/>
-      <c r="E33" t="inlineStr"/>
-      <c r="F33" t="inlineStr"/>
-      <c r="G33" t="inlineStr"/>
-      <c r="H33" t="inlineStr"/>
-      <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr"/>
-      <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10405,9 +9993,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="N33" t="inlineStr"/>
-      <c r="O33" t="inlineStr"/>
-      <c r="P33" t="inlineStr"/>
       <c r="Q33" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10429,24 +10014,11 @@
           <t>Orientación médica con IA</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr"/>
-      <c r="D34" t="inlineStr"/>
-      <c r="E34" t="inlineStr"/>
-      <c r="F34" t="inlineStr"/>
-      <c r="G34" t="inlineStr"/>
-      <c r="H34" t="inlineStr"/>
-      <c r="I34" t="inlineStr"/>
-      <c r="J34" t="inlineStr"/>
-      <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="M34" t="inlineStr"/>
-      <c r="N34" t="inlineStr"/>
-      <c r="O34" t="inlineStr"/>
-      <c r="P34" t="inlineStr"/>
       <c r="Q34" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10468,15 +10040,6 @@
           <t>Preparación de consultas médicas con IA</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr"/>
-      <c r="D35" t="inlineStr"/>
-      <c r="E35" t="inlineStr"/>
-      <c r="F35" t="inlineStr"/>
-      <c r="G35" t="inlineStr"/>
-      <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr"/>
-      <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10487,10 +10050,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="N35" t="inlineStr"/>
-      <c r="O35" t="inlineStr"/>
-      <c r="P35" t="inlineStr"/>
-      <c r="Q35" t="inlineStr"/>
       <c r="R35">
         <f>COUNTIF(C35:Q35,"✓")</f>
         <v/>
@@ -10507,15 +10066,6 @@
           <t>Resumen de historial con IA</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr"/>
-      <c r="D36" t="inlineStr"/>
-      <c r="E36" t="inlineStr"/>
-      <c r="F36" t="inlineStr"/>
-      <c r="G36" t="inlineStr"/>
-      <c r="H36" t="inlineStr"/>
-      <c r="I36" t="inlineStr"/>
-      <c r="J36" t="inlineStr"/>
-      <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10526,10 +10076,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="N36" t="inlineStr"/>
-      <c r="O36" t="inlineStr"/>
-      <c r="P36" t="inlineStr"/>
-      <c r="Q36" t="inlineStr"/>
       <c r="R36">
         <f>COUNTIF(C36:Q36,"✓")</f>
         <v/>
@@ -10546,25 +10092,11 @@
           <t>API para apps de terceros</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr"/>
-      <c r="D37" t="inlineStr"/>
-      <c r="E37" t="inlineStr"/>
-      <c r="F37" t="inlineStr"/>
-      <c r="G37" t="inlineStr"/>
-      <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr"/>
-      <c r="J37" t="inlineStr"/>
       <c r="K37" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="L37" t="inlineStr"/>
-      <c r="M37" t="inlineStr"/>
-      <c r="N37" t="inlineStr"/>
-      <c r="O37" t="inlineStr"/>
-      <c r="P37" t="inlineStr"/>
-      <c r="Q37" t="inlineStr"/>
       <c r="R37">
         <f>COUNTIF(C37:Q37,"✓")</f>
         <v/>
@@ -10586,10 +10118,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr"/>
-      <c r="E38" t="inlineStr"/>
-      <c r="F38" t="inlineStr"/>
-      <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10600,7 +10128,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="J38" t="inlineStr"/>
       <c r="K38" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10616,14 +10143,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="N38" t="inlineStr"/>
       <c r="O38" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="P38" t="inlineStr"/>
-      <c r="Q38" t="inlineStr"/>
       <c r="R38">
         <f>COUNTIF(C38:Q38,"✓")</f>
         <v/>
@@ -10640,25 +10164,11 @@
           <t>Analítica poblacional B2B</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr"/>
-      <c r="D39" t="inlineStr"/>
-      <c r="E39" t="inlineStr"/>
-      <c r="F39" t="inlineStr"/>
-      <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr"/>
-      <c r="J39" t="inlineStr"/>
-      <c r="K39" t="inlineStr"/>
-      <c r="L39" t="inlineStr"/>
-      <c r="M39" t="inlineStr"/>
-      <c r="N39" t="inlineStr"/>
-      <c r="O39" t="inlineStr"/>
-      <c r="P39" t="inlineStr"/>
-      <c r="Q39" t="inlineStr"/>
       <c r="R39">
         <f>COUNTIF(C39:Q39,"✓")</f>
         <v/>
@@ -10675,9 +10185,6 @@
           <t>Disponibilidad multiplataforma (web/iOS/Android)</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr"/>
-      <c r="D40" t="inlineStr"/>
-      <c r="E40" t="inlineStr"/>
       <c r="F40" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10688,20 +10195,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr"/>
-      <c r="I40" t="inlineStr"/>
-      <c r="J40" t="inlineStr"/>
-      <c r="K40" t="inlineStr"/>
-      <c r="L40" t="inlineStr"/>
-      <c r="M40" t="inlineStr"/>
-      <c r="N40" t="inlineStr"/>
       <c r="O40" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="P40" t="inlineStr"/>
-      <c r="Q40" t="inlineStr"/>
       <c r="R40">
         <f>COUNTIF(C40:Q40,"✓")</f>
         <v/>
@@ -10718,25 +10216,11 @@
           <t>Historial médico centralizado</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr"/>
-      <c r="D41" t="inlineStr"/>
-      <c r="E41" t="inlineStr"/>
-      <c r="F41" t="inlineStr"/>
-      <c r="G41" t="inlineStr"/>
-      <c r="H41" t="inlineStr"/>
-      <c r="I41" t="inlineStr"/>
       <c r="J41" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="K41" t="inlineStr"/>
-      <c r="L41" t="inlineStr"/>
-      <c r="M41" t="inlineStr"/>
-      <c r="N41" t="inlineStr"/>
-      <c r="O41" t="inlineStr"/>
-      <c r="P41" t="inlineStr"/>
-      <c r="Q41" t="inlineStr"/>
       <c r="R41">
         <f>COUNTIF(C41:Q41,"✓")</f>
         <v/>
@@ -10753,25 +10237,11 @@
           <t>Importación y exportación de datos</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr"/>
-      <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr"/>
-      <c r="G42" t="inlineStr"/>
-      <c r="H42" t="inlineStr"/>
-      <c r="I42" t="inlineStr"/>
-      <c r="J42" t="inlineStr"/>
-      <c r="K42" t="inlineStr"/>
-      <c r="L42" t="inlineStr"/>
-      <c r="M42" t="inlineStr"/>
-      <c r="N42" t="inlineStr"/>
-      <c r="O42" t="inlineStr"/>
-      <c r="P42" t="inlineStr"/>
-      <c r="Q42" t="inlineStr"/>
       <c r="R42">
         <f>COUNTIF(C42:Q42,"✓")</f>
         <v/>
@@ -10788,25 +10258,11 @@
           <t>Integración con EHR de proveedores</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr"/>
-      <c r="D43" t="inlineStr"/>
-      <c r="E43" t="inlineStr"/>
-      <c r="F43" t="inlineStr"/>
-      <c r="G43" t="inlineStr"/>
-      <c r="H43" t="inlineStr"/>
-      <c r="I43" t="inlineStr"/>
       <c r="J43" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="K43" t="inlineStr"/>
-      <c r="L43" t="inlineStr"/>
-      <c r="M43" t="inlineStr"/>
-      <c r="N43" t="inlineStr"/>
-      <c r="O43" t="inlineStr"/>
-      <c r="P43" t="inlineStr"/>
-      <c r="Q43" t="inlineStr"/>
       <c r="R43">
         <f>COUNTIF(C43:Q43,"✓")</f>
         <v/>
@@ -10823,29 +10279,16 @@
           <t>Integración con wearables y apps de salud</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr"/>
-      <c r="D44" t="inlineStr"/>
-      <c r="E44" t="inlineStr"/>
-      <c r="F44" t="inlineStr"/>
-      <c r="G44" t="inlineStr"/>
       <c r="H44" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="I44" t="inlineStr"/>
-      <c r="J44" t="inlineStr"/>
-      <c r="K44" t="inlineStr"/>
-      <c r="L44" t="inlineStr"/>
       <c r="M44" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="N44" t="inlineStr"/>
-      <c r="O44" t="inlineStr"/>
-      <c r="P44" t="inlineStr"/>
-      <c r="Q44" t="inlineStr"/>
       <c r="R44">
         <f>COUNTIF(C44:Q44,"✓")</f>
         <v/>
@@ -10862,25 +10305,11 @@
           <t>Gestión de lista de medicamentos</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr"/>
-      <c r="D45" t="inlineStr"/>
-      <c r="E45" t="inlineStr"/>
-      <c r="F45" t="inlineStr"/>
-      <c r="G45" t="inlineStr"/>
-      <c r="H45" t="inlineStr"/>
-      <c r="I45" t="inlineStr"/>
-      <c r="J45" t="inlineStr"/>
       <c r="K45" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="L45" t="inlineStr"/>
-      <c r="M45" t="inlineStr"/>
-      <c r="N45" t="inlineStr"/>
-      <c r="O45" t="inlineStr"/>
-      <c r="P45" t="inlineStr"/>
-      <c r="Q45" t="inlineStr"/>
       <c r="R45">
         <f>COUNTIF(C45:Q45,"✓")</f>
         <v/>
@@ -10897,25 +10326,11 @@
           <t>Importación automática de tratamientos desde receta digital</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr"/>
-      <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr"/>
-      <c r="G46" t="inlineStr"/>
-      <c r="H46" t="inlineStr"/>
-      <c r="I46" t="inlineStr"/>
-      <c r="J46" t="inlineStr"/>
-      <c r="K46" t="inlineStr"/>
-      <c r="L46" t="inlineStr"/>
-      <c r="M46" t="inlineStr"/>
-      <c r="N46" t="inlineStr"/>
-      <c r="O46" t="inlineStr"/>
-      <c r="P46" t="inlineStr"/>
-      <c r="Q46" t="inlineStr"/>
       <c r="R46">
         <f>COUNTIF(C46:Q46,"✓")</f>
         <v/>
@@ -10937,24 +10352,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr"/>
-      <c r="E47" t="inlineStr"/>
-      <c r="F47" t="inlineStr"/>
-      <c r="G47" t="inlineStr"/>
-      <c r="H47" t="inlineStr"/>
-      <c r="I47" t="inlineStr"/>
-      <c r="J47" t="inlineStr"/>
       <c r="K47" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="L47" t="inlineStr"/>
-      <c r="M47" t="inlineStr"/>
-      <c r="N47" t="inlineStr"/>
-      <c r="O47" t="inlineStr"/>
-      <c r="P47" t="inlineStr"/>
-      <c r="Q47" t="inlineStr"/>
       <c r="R47">
         <f>COUNTIF(C47:Q47,"✓")</f>
         <v/>
@@ -10971,25 +10373,11 @@
           <t>Registro de tomas y adherencia al tratamiento</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr"/>
-      <c r="D48" t="inlineStr"/>
       <c r="E48" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr"/>
-      <c r="G48" t="inlineStr"/>
-      <c r="H48" t="inlineStr"/>
-      <c r="I48" t="inlineStr"/>
-      <c r="J48" t="inlineStr"/>
-      <c r="K48" t="inlineStr"/>
-      <c r="L48" t="inlineStr"/>
-      <c r="M48" t="inlineStr"/>
-      <c r="N48" t="inlineStr"/>
-      <c r="O48" t="inlineStr"/>
-      <c r="P48" t="inlineStr"/>
-      <c r="Q48" t="inlineStr"/>
       <c r="R48">
         <f>COUNTIF(C48:Q48,"✓")</f>
         <v/>
@@ -11006,25 +10394,11 @@
           <t>Comunidad de pacientes</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr"/>
-      <c r="D49" t="inlineStr"/>
-      <c r="E49" t="inlineStr"/>
-      <c r="F49" t="inlineStr"/>
-      <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="I49" t="inlineStr"/>
-      <c r="J49" t="inlineStr"/>
-      <c r="K49" t="inlineStr"/>
-      <c r="L49" t="inlineStr"/>
-      <c r="M49" t="inlineStr"/>
-      <c r="N49" t="inlineStr"/>
-      <c r="O49" t="inlineStr"/>
-      <c r="P49" t="inlineStr"/>
-      <c r="Q49" t="inlineStr"/>
       <c r="R49">
         <f>COUNTIF(C49:Q49,"✓")</f>
         <v/>
@@ -11041,25 +10415,11 @@
           <t>Contenido educativo sobre salud</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr"/>
       <c r="D50" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr"/>
-      <c r="F50" t="inlineStr"/>
-      <c r="G50" t="inlineStr"/>
-      <c r="H50" t="inlineStr"/>
-      <c r="I50" t="inlineStr"/>
-      <c r="J50" t="inlineStr"/>
-      <c r="K50" t="inlineStr"/>
-      <c r="L50" t="inlineStr"/>
-      <c r="M50" t="inlineStr"/>
-      <c r="N50" t="inlineStr"/>
-      <c r="O50" t="inlineStr"/>
-      <c r="P50" t="inlineStr"/>
-      <c r="Q50" t="inlineStr"/>
       <c r="R50">
         <f>COUNTIF(C50:Q50,"✓")</f>
         <v/>
@@ -11076,25 +10436,11 @@
           <t>Gráficas de evolución de indicadores</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr"/>
-      <c r="D51" t="inlineStr"/>
       <c r="E51" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F51" t="inlineStr"/>
-      <c r="G51" t="inlineStr"/>
-      <c r="H51" t="inlineStr"/>
-      <c r="I51" t="inlineStr"/>
-      <c r="J51" t="inlineStr"/>
-      <c r="K51" t="inlineStr"/>
-      <c r="L51" t="inlineStr"/>
-      <c r="M51" t="inlineStr"/>
-      <c r="N51" t="inlineStr"/>
-      <c r="O51" t="inlineStr"/>
-      <c r="P51" t="inlineStr"/>
-      <c r="Q51" t="inlineStr"/>
       <c r="R51">
         <f>COUNTIF(C51:Q51,"✓")</f>
         <v/>
@@ -11111,25 +10457,11 @@
           <t>Integración con wearables y apps de salud</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr"/>
-      <c r="D52" t="inlineStr"/>
-      <c r="E52" t="inlineStr"/>
-      <c r="F52" t="inlineStr"/>
-      <c r="G52" t="inlineStr"/>
-      <c r="H52" t="inlineStr"/>
-      <c r="I52" t="inlineStr"/>
-      <c r="J52" t="inlineStr"/>
       <c r="K52" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="L52" t="inlineStr"/>
-      <c r="M52" t="inlineStr"/>
-      <c r="N52" t="inlineStr"/>
-      <c r="O52" t="inlineStr"/>
-      <c r="P52" t="inlineStr"/>
-      <c r="Q52" t="inlineStr"/>
       <c r="R52">
         <f>COUNTIF(C52:Q52,"✓")</f>
         <v/>
@@ -11146,11 +10478,6 @@
           <t>Panel de seguimiento de salud y bienestar</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr"/>
-      <c r="D53" t="inlineStr"/>
-      <c r="E53" t="inlineStr"/>
-      <c r="F53" t="inlineStr"/>
-      <c r="G53" t="inlineStr"/>
       <c r="H53" t="inlineStr">
         <is>
           <t>✓</t>
@@ -11161,14 +10488,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="J53" t="inlineStr"/>
-      <c r="K53" t="inlineStr"/>
-      <c r="L53" t="inlineStr"/>
-      <c r="M53" t="inlineStr"/>
-      <c r="N53" t="inlineStr"/>
-      <c r="O53" t="inlineStr"/>
-      <c r="P53" t="inlineStr"/>
-      <c r="Q53" t="inlineStr"/>
       <c r="R53">
         <f>COUNTIF(C53:Q53,"✓")</f>
         <v/>
@@ -11185,25 +10504,11 @@
           <t>Registro de nutrición</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr"/>
-      <c r="D54" t="inlineStr"/>
-      <c r="E54" t="inlineStr"/>
-      <c r="F54" t="inlineStr"/>
-      <c r="G54" t="inlineStr"/>
-      <c r="H54" t="inlineStr"/>
-      <c r="I54" t="inlineStr"/>
-      <c r="J54" t="inlineStr"/>
       <c r="K54" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="L54" t="inlineStr"/>
-      <c r="M54" t="inlineStr"/>
-      <c r="N54" t="inlineStr"/>
-      <c r="O54" t="inlineStr"/>
-      <c r="P54" t="inlineStr"/>
-      <c r="Q54" t="inlineStr"/>
       <c r="R54">
         <f>COUNTIF(C54:Q54,"✓")</f>
         <v/>
@@ -11220,25 +10525,11 @@
           <t>Seguimiento de salud femenina</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr"/>
-      <c r="D55" t="inlineStr"/>
-      <c r="E55" t="inlineStr"/>
-      <c r="F55" t="inlineStr"/>
-      <c r="G55" t="inlineStr"/>
-      <c r="H55" t="inlineStr"/>
-      <c r="I55" t="inlineStr"/>
-      <c r="J55" t="inlineStr"/>
       <c r="K55" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="L55" t="inlineStr"/>
-      <c r="M55" t="inlineStr"/>
-      <c r="N55" t="inlineStr"/>
-      <c r="O55" t="inlineStr"/>
-      <c r="P55" t="inlineStr"/>
-      <c r="Q55" t="inlineStr"/>
       <c r="R55">
         <f>COUNTIF(C55:Q55,"✓")</f>
         <v/>
@@ -11255,25 +10546,11 @@
           <t>Valoración de profesionales</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr"/>
-      <c r="D56" t="inlineStr"/>
-      <c r="E56" t="inlineStr"/>
       <c r="F56" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="G56" t="inlineStr"/>
-      <c r="H56" t="inlineStr"/>
-      <c r="I56" t="inlineStr"/>
-      <c r="J56" t="inlineStr"/>
-      <c r="K56" t="inlineStr"/>
-      <c r="L56" t="inlineStr"/>
-      <c r="M56" t="inlineStr"/>
-      <c r="N56" t="inlineStr"/>
-      <c r="O56" t="inlineStr"/>
-      <c r="P56" t="inlineStr"/>
-      <c r="Q56" t="inlineStr"/>
       <c r="R56">
         <f>COUNTIF(C56:Q56,"✓")</f>
         <v/>
@@ -11290,25 +10567,11 @@
           <t>Acceso mínimo por categorías de datos</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr"/>
-      <c r="D57" t="inlineStr"/>
-      <c r="E57" t="inlineStr"/>
-      <c r="F57" t="inlineStr"/>
-      <c r="G57" t="inlineStr"/>
-      <c r="H57" t="inlineStr"/>
-      <c r="I57" t="inlineStr"/>
-      <c r="J57" t="inlineStr"/>
-      <c r="K57" t="inlineStr"/>
-      <c r="L57" t="inlineStr"/>
       <c r="M57" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="N57" t="inlineStr"/>
-      <c r="O57" t="inlineStr"/>
-      <c r="P57" t="inlineStr"/>
-      <c r="Q57" t="inlineStr"/>
       <c r="R57">
         <f>COUNTIF(C57:Q57,"✓")</f>
         <v/>
@@ -11325,11 +10588,6 @@
           <t>Blockchain para integridad y trazabilidad de datos</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr"/>
-      <c r="D58" t="inlineStr"/>
-      <c r="E58" t="inlineStr"/>
-      <c r="F58" t="inlineStr"/>
-      <c r="G58" t="inlineStr"/>
       <c r="H58" t="inlineStr">
         <is>
           <t>✓</t>
@@ -11345,13 +10603,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="K58" t="inlineStr"/>
-      <c r="L58" t="inlineStr"/>
-      <c r="M58" t="inlineStr"/>
-      <c r="N58" t="inlineStr"/>
-      <c r="O58" t="inlineStr"/>
-      <c r="P58" t="inlineStr"/>
-      <c r="Q58" t="inlineStr"/>
       <c r="R58">
         <f>COUNTIF(C58:Q58,"✓")</f>
         <v/>
@@ -11368,29 +10619,16 @@
           <t>Cifrado y control de acceso</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr"/>
       <c r="D59" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr"/>
-      <c r="F59" t="inlineStr"/>
-      <c r="G59" t="inlineStr"/>
-      <c r="H59" t="inlineStr"/>
-      <c r="I59" t="inlineStr"/>
-      <c r="J59" t="inlineStr"/>
       <c r="K59" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="L59" t="inlineStr"/>
-      <c r="M59" t="inlineStr"/>
-      <c r="N59" t="inlineStr"/>
-      <c r="O59" t="inlineStr"/>
-      <c r="P59" t="inlineStr"/>
-      <c r="Q59" t="inlineStr"/>
       <c r="R59">
         <f>COUNTIF(C59:Q59,"✓")</f>
         <v/>
@@ -11407,25 +10645,11 @@
           <t>Cumplimiento regulatorio de salud y datos</t>
         </is>
       </c>
-      <c r="C60" t="inlineStr"/>
-      <c r="D60" t="inlineStr"/>
-      <c r="E60" t="inlineStr"/>
-      <c r="F60" t="inlineStr"/>
-      <c r="G60" t="inlineStr"/>
-      <c r="H60" t="inlineStr"/>
-      <c r="I60" t="inlineStr"/>
-      <c r="J60" t="inlineStr"/>
-      <c r="K60" t="inlineStr"/>
-      <c r="L60" t="inlineStr"/>
-      <c r="M60" t="inlineStr"/>
-      <c r="N60" t="inlineStr"/>
       <c r="O60" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="P60" t="inlineStr"/>
-      <c r="Q60" t="inlineStr"/>
       <c r="R60">
         <f>COUNTIF(C60:Q60,"✓")</f>
         <v/>
@@ -11442,25 +10666,11 @@
           <t>Gestión de consentimiento sobre uso de datos</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr"/>
-      <c r="D61" t="inlineStr"/>
-      <c r="E61" t="inlineStr"/>
-      <c r="F61" t="inlineStr"/>
-      <c r="G61" t="inlineStr"/>
-      <c r="H61" t="inlineStr"/>
-      <c r="I61" t="inlineStr"/>
-      <c r="J61" t="inlineStr"/>
-      <c r="K61" t="inlineStr"/>
       <c r="L61" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="M61" t="inlineStr"/>
-      <c r="N61" t="inlineStr"/>
-      <c r="O61" t="inlineStr"/>
-      <c r="P61" t="inlineStr"/>
-      <c r="Q61" t="inlineStr"/>
       <c r="R61">
         <f>COUNTIF(C61:Q61,"✓")</f>
         <v/>
@@ -11477,25 +10687,11 @@
           <t>Identidad descentralizada (DID)</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr"/>
-      <c r="D62" t="inlineStr"/>
-      <c r="E62" t="inlineStr"/>
-      <c r="F62" t="inlineStr"/>
-      <c r="G62" t="inlineStr"/>
-      <c r="H62" t="inlineStr"/>
       <c r="I62" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="J62" t="inlineStr"/>
-      <c r="K62" t="inlineStr"/>
-      <c r="L62" t="inlineStr"/>
-      <c r="M62" t="inlineStr"/>
-      <c r="N62" t="inlineStr"/>
-      <c r="O62" t="inlineStr"/>
-      <c r="P62" t="inlineStr"/>
-      <c r="Q62" t="inlineStr"/>
       <c r="R62">
         <f>COUNTIF(C62:Q62,"✓")</f>
         <v/>
@@ -11512,15 +10708,6 @@
           <t>Privacidad reforzada para datos de salud</t>
         </is>
       </c>
-      <c r="C63" t="inlineStr"/>
-      <c r="D63" t="inlineStr"/>
-      <c r="E63" t="inlineStr"/>
-      <c r="F63" t="inlineStr"/>
-      <c r="G63" t="inlineStr"/>
-      <c r="H63" t="inlineStr"/>
-      <c r="I63" t="inlineStr"/>
-      <c r="J63" t="inlineStr"/>
-      <c r="K63" t="inlineStr"/>
       <c r="L63" t="inlineStr">
         <is>
           <t>✓</t>
@@ -11531,10 +10718,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="N63" t="inlineStr"/>
-      <c r="O63" t="inlineStr"/>
-      <c r="P63" t="inlineStr"/>
-      <c r="Q63" t="inlineStr"/>
       <c r="R63">
         <f>COUNTIF(C63:Q63,"✓")</f>
         <v/>
@@ -11551,20 +10734,6 @@
           <t>Modelo freemium y suscripción</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr"/>
-      <c r="D64" t="inlineStr"/>
-      <c r="E64" t="inlineStr"/>
-      <c r="F64" t="inlineStr"/>
-      <c r="G64" t="inlineStr"/>
-      <c r="H64" t="inlineStr"/>
-      <c r="I64" t="inlineStr"/>
-      <c r="J64" t="inlineStr"/>
-      <c r="K64" t="inlineStr"/>
-      <c r="L64" t="inlineStr"/>
-      <c r="M64" t="inlineStr"/>
-      <c r="N64" t="inlineStr"/>
-      <c r="O64" t="inlineStr"/>
-      <c r="P64" t="inlineStr"/>
       <c r="Q64" t="inlineStr">
         <is>
           <t>✓</t>
@@ -11586,25 +10755,11 @@
           <t>Pagos con criptomoneda</t>
         </is>
       </c>
-      <c r="C65" t="inlineStr"/>
-      <c r="D65" t="inlineStr"/>
-      <c r="E65" t="inlineStr"/>
-      <c r="F65" t="inlineStr"/>
-      <c r="G65" t="inlineStr"/>
-      <c r="H65" t="inlineStr"/>
-      <c r="I65" t="inlineStr"/>
       <c r="J65" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="K65" t="inlineStr"/>
-      <c r="L65" t="inlineStr"/>
-      <c r="M65" t="inlineStr"/>
-      <c r="N65" t="inlineStr"/>
-      <c r="O65" t="inlineStr"/>
-      <c r="P65" t="inlineStr"/>
-      <c r="Q65" t="inlineStr"/>
       <c r="R65">
         <f>COUNTIF(C65:Q65,"✓")</f>
         <v/>
@@ -11621,24 +10776,11 @@
           <t>Pagos dentro de la app</t>
         </is>
       </c>
-      <c r="C66" t="inlineStr"/>
-      <c r="D66" t="inlineStr"/>
-      <c r="E66" t="inlineStr"/>
-      <c r="F66" t="inlineStr"/>
-      <c r="G66" t="inlineStr"/>
-      <c r="H66" t="inlineStr"/>
-      <c r="I66" t="inlineStr"/>
-      <c r="J66" t="inlineStr"/>
-      <c r="K66" t="inlineStr"/>
-      <c r="L66" t="inlineStr"/>
-      <c r="M66" t="inlineStr"/>
       <c r="N66" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="O66" t="inlineStr"/>
-      <c r="P66" t="inlineStr"/>
       <c r="Q66" t="inlineStr">
         <is>
           <t>✓</t>
@@ -11660,25 +10802,11 @@
           <t>Reclamos y trámites con seguros</t>
         </is>
       </c>
-      <c r="C67" t="inlineStr"/>
-      <c r="D67" t="inlineStr"/>
-      <c r="E67" t="inlineStr"/>
-      <c r="F67" t="inlineStr"/>
-      <c r="G67" t="inlineStr"/>
-      <c r="H67" t="inlineStr"/>
       <c r="I67" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="J67" t="inlineStr"/>
-      <c r="K67" t="inlineStr"/>
-      <c r="L67" t="inlineStr"/>
-      <c r="M67" t="inlineStr"/>
-      <c r="N67" t="inlineStr"/>
-      <c r="O67" t="inlineStr"/>
-      <c r="P67" t="inlineStr"/>
-      <c r="Q67" t="inlineStr"/>
       <c r="R67">
         <f>COUNTIF(C67:Q67,"✓")</f>
         <v/>
@@ -11695,25 +10823,11 @@
           <t>Mensajería paciente-institución</t>
         </is>
       </c>
-      <c r="C68" t="inlineStr"/>
-      <c r="D68" t="inlineStr"/>
-      <c r="E68" t="inlineStr"/>
-      <c r="F68" t="inlineStr"/>
-      <c r="G68" t="inlineStr"/>
-      <c r="H68" t="inlineStr"/>
       <c r="I68" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="J68" t="inlineStr"/>
-      <c r="K68" t="inlineStr"/>
-      <c r="L68" t="inlineStr"/>
-      <c r="M68" t="inlineStr"/>
-      <c r="N68" t="inlineStr"/>
-      <c r="O68" t="inlineStr"/>
-      <c r="P68" t="inlineStr"/>
-      <c r="Q68" t="inlineStr"/>
       <c r="R68">
         <f>COUNTIF(C68:Q68,"✓")</f>
         <v/>
@@ -11730,25 +10844,11 @@
           <t>Teleconsulta con profesionales</t>
         </is>
       </c>
-      <c r="C69" t="inlineStr"/>
-      <c r="D69" t="inlineStr"/>
-      <c r="E69" t="inlineStr"/>
-      <c r="F69" t="inlineStr"/>
-      <c r="G69" t="inlineStr"/>
-      <c r="H69" t="inlineStr"/>
-      <c r="I69" t="inlineStr"/>
       <c r="J69" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="K69" t="inlineStr"/>
-      <c r="L69" t="inlineStr"/>
-      <c r="M69" t="inlineStr"/>
-      <c r="N69" t="inlineStr"/>
-      <c r="O69" t="inlineStr"/>
-      <c r="P69" t="inlineStr"/>
-      <c r="Q69" t="inlineStr"/>
       <c r="R69">
         <f>COUNTIF(C69:Q69,"✓")</f>
         <v/>
@@ -11765,7 +10865,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A38"/>
+  <dimension ref="A1:A40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -12037,6 +11137,20 @@
         </is>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Vuelta 9 (iter. 1, 2026-10-25 12:16 UTC): Meedika, Infomed, MediPlanner, Clingot verificados (+0 filas; saturado). Pendientes: Healfies, Patientory, MediBloc, Medicalchain, Apple Health, ChatGPT Health, Claude for Healthcare, Apps de clínicas, Clinia, MiRedSalud, Mediko.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>CANDIDATO A COMPETIDOR (no agregado; decide el usuario): Medicyn (global). App de historial médico personal que guarda los datos solo en el dispositivo, sin cuentas ni rastreo; cubre condiciones, medicamentos, alergias y análisis; prueba gratuita de 7 días y pago único. Lanzada en Product Hunt el 12-jun-2026 (fuente: Product Hunt). Enfoque de privacidad local, relevante frente a la propuesta blockchain. Otros no agregados: DKV «Quiero cuidarme Más» v2.9 (España; historial médico compartido consultable por profesionales de cualquier centro; fecha sin confirmar).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Benchmark: vuelta 9, iteración 2 (Healfies, Patientory, MediBloc, Medicalchain); ficha de Medicyn
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MVcXu8vTBu7EKfj3YdEvae
</commit_message>
<xml_diff>
--- a/Outputs/Benchmark_Anamnesis.xlsx
+++ b/Outputs/Benchmark_Anamnesis.xlsx
@@ -673,12 +673,12 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>[REGIONAL · Brasil] Fundada ene-2015 en Florianópolis por Helyson Lewis Velasco. Centraliza registros de salud personales: carpetas, etiquetas, línea de tiempo (medicación, exámenes, citas, dieta), compartir con familia o profesionales. Gratis; web, iOS y Android. Estado actual NO verificado (fuentes de 2015-2016). Referencia funcional cercana a etapas A+B. [Vuelta 2] Lanzada simultáneamente en Brasil, Argentina y EE.UU.; permite compartir con no registrados vía clave por email. Sin novedades posteriores a 2016. [Vuelta 3] Sin evidencia de actividad reciente ni de cierre; Gust/Dealroom la listan en Florianópolis (10 empleados, healfies.com) sin fecha de actualización. Estado sin confirmar. [Vuelta 4] Sin Google Play localizado; no confundir con la app Healfy (otro producto). Sin novedades. [Vuelta 5] Sin búsqueda nueva (revisada en vuelta 4); sin cambios. [Vuelta 6] Sin búsqueda nueva (fuentes agotadas); sin cambios. [Vuelta 7] Solo fuentes de 2015-2016; alianza con ClinCard (feb-2016). Sin evidencia de actividad reciente. [Vuelta 8] Sin fuentes nuevas.</t>
+          <t>[REGIONAL · Brasil] Fundada ene-2015 en Florianópolis por Helyson Lewis Velasco. Centraliza registros de salud personales: carpetas, etiquetas, línea de tiempo (medicación, exámenes, citas, dieta), compartir con familia o profesionales. Gratis; web, iOS y Android. Estado actual NO verificado (fuentes de 2015-2016). Referencia funcional cercana a etapas A+B. [Vuelta 2] Lanzada simultáneamente en Brasil, Argentina y EE.UU.; permite compartir con no registrados vía clave por email. Sin novedades posteriores a 2016. [Vuelta 3] Sin evidencia de actividad reciente ni de cierre; Gust/Dealroom la listan en Florianópolis (10 empleados, healfies.com) sin fecha de actualización. Estado sin confirmar. [Vuelta 4] Sin Google Play localizado; no confundir con la app Healfy (otro producto). Sin novedades. [Vuelta 5] Sin búsqueda nueva (revisada en vuelta 4); sin cambios. [Vuelta 6] Sin búsqueda nueva (fuentes agotadas); sin cambios. [Vuelta 7] Solo fuentes de 2015-2016; alianza con ClinCard (feb-2016). Sin evidencia de actividad reciente. [Vuelta 8] Sin fuentes nuevas. [Vuelta 9] Sin búsqueda nueva (saturado).</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G6" t="n">
@@ -686,7 +686,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -713,12 +713,12 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>[BLOCKCHAIN · EE.UU.] Atlanta, fundada 2015, ~9 empleados. Levantó US$7,2M vía financiamiento cripto. App con registros de hospitales y wearables, coaching de salud con IA y recompensas en cripto; también dashboard empresarial Neith. PitchBook indica actividad y financiamiento hasta abr-2026: sigue operando. Sin presencia conocida en Chile. Referencia directa para la hipótesis blockchain. [Vuelta 2] Sin noticias 2026 encontradas en búsqueda; sitio oficial bloqueado. [Vuelta 3] Búsqueda adicional solo devuelve hitos de 2017 (token sale US$7,2M) y 2019 (Serie A de US$5,3M, cierre no confirmado); sin datos 2025-26 propios. [Vuelta 4] App pública lanzada en la conferencia JP Morgan Healthcare (2019); red PTOYMatrix (blockchain HIPAA); socios reportados: StartUp Health y Kaiser Permanente (beta). Estado actual en App Store/Google Play sin confirmar. [Vuelta 5] Sin noticias 2026 del equipo. Token PTOY con capitalización de ~US$53K a fines de ago-2026 según Phantom (KuCoin discrepa en la circulación): señal de baja actividad, no prueba de cierre. Esto relativiza la actividad hasta abr-2026 mencionada en la ficha original. [Vuelta 6] Sin noticias posteriores a 2020 localizadas (hitos: token sale 2017, consorcio Hyperledger, alianza con Georgia State, Series A de US$5,3M vía R/GA Ventures, Neith con Prosper Healthtech en Birmingham). Estado actual desconocido. [Vuelta 7] Sin búsqueda nueva (saturado); sin cambios. [Vuelta 8] Sin noticias 2025-26; en 2018 la oferta se dirigía a empresas de salud, con la versión individual planificada después.</t>
+          <t>[BLOCKCHAIN · EE.UU.] Atlanta, fundada 2015, ~9 empleados. Levantó US$7,2M vía financiamiento cripto. App con registros de hospitales y wearables, coaching de salud con IA y recompensas en cripto; también dashboard empresarial Neith. PitchBook indica actividad y financiamiento hasta abr-2026: sigue operando. Sin presencia conocida en Chile. Referencia directa para la hipótesis blockchain. [Vuelta 2] Sin noticias 2026 encontradas en búsqueda; sitio oficial bloqueado. [Vuelta 3] Búsqueda adicional solo devuelve hitos de 2017 (token sale US$7,2M) y 2019 (Serie A de US$5,3M, cierre no confirmado); sin datos 2025-26 propios. [Vuelta 4] App pública lanzada en la conferencia JP Morgan Healthcare (2019); red PTOYMatrix (blockchain HIPAA); socios reportados: StartUp Health y Kaiser Permanente (beta). Estado actual en App Store/Google Play sin confirmar. [Vuelta 5] Sin noticias 2026 del equipo. Token PTOY con capitalización de ~US$53K a fines de ago-2026 según Phantom (KuCoin discrepa en la circulación): señal de baja actividad, no prueba de cierre. Esto relativiza la actividad hasta abr-2026 mencionada en la ficha original. [Vuelta 6] Sin noticias posteriores a 2020 localizadas (hitos: token sale 2017, consorcio Hyperledger, alianza con Georgia State, Series A de US$5,3M vía R/GA Ventures, Neith con Prosper Healthtech en Birmingham). Estado actual desconocido. [Vuelta 7] Sin búsqueda nueva (saturado); sin cambios. [Vuelta 8] Sin noticias 2025-26; en 2018 la oferta se dirigía a empresas de salud, con la versión individual planificada después. [Vuelta 9] Sin búsqueda nueva (saturado).</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G7" t="n">
@@ -726,7 +726,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -753,12 +753,12 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>[BLOCKCHAIN · Corea del Sur] Fundada 2017, Seúl. Blockchain propia Panacea (Cosmos SDK, mainnet 2019) para que el paciente gestione y transfiera sus registros; app Medipass para seguros. Serie A de ₩4.000 millones (Naver); alianzas con hospitales (Seoul National, Severance). Estado 2025-26 NO verificado. Referencia sobre seguros + blockchain. [Vuelta 2] Panacea incluye DID, Append Only Log, IBC y PNFT; sin anuncios 2026 localizados. [Vuelta 3] Medipass: app en Corea con 20 hospitales/aseguradoras integrados (fecha de la lista desconocida) y plan 2022 de superapp con marketplace de datos; operación actual sin confirmar. [Vuelta 4] Sin búsqueda nueva (revisada en vuelta 3); sin cambios. [Vuelta 5] Medipass: ~400.000 usuarios acumulados (CEO, jun-2022); integración con aseguradoras Shinhan Life, Samsung Fire y Hyundai Marine (2020); renovación completa en mar-2023 (dashboard de salud, gestión familiar, certificados). Sin noticias 2026 encontradas. [Vuelta 6] Medipass 2023: comunicación bidireccional hospital-paciente y chat MediTalk; en 2019 fue seleccionada para el programa gubernamental de MyData médico con Samsung Fire y SNUH. Sin estrategia 2026 localizada. Meta declarada: usar Medipass como «identificación» de salud. [Vuelta 7] Una fuente sin fecha atribuye a Medipass más de 600.000 pacientes en 14 hospitales; MoU 2019 con Severance (plataforma de facturación de seguros y detección de falsificación de datos) y piloto con Massachusetts General Hospital. Sin datos 2025-26. [Vuelta 8] Sin noticias 2025-26.</t>
+          <t>[BLOCKCHAIN · Corea del Sur] Fundada 2017, Seúl. Blockchain propia Panacea (Cosmos SDK, mainnet 2019) para que el paciente gestione y transfiera sus registros; app Medipass para seguros. Serie A de ₩4.000 millones (Naver); alianzas con hospitales (Seoul National, Severance). Estado 2025-26 NO verificado. Referencia sobre seguros + blockchain. [Vuelta 2] Panacea incluye DID, Append Only Log, IBC y PNFT; sin anuncios 2026 localizados. [Vuelta 3] Medipass: app en Corea con 20 hospitales/aseguradoras integrados (fecha de la lista desconocida) y plan 2022 de superapp con marketplace de datos; operación actual sin confirmar. [Vuelta 4] Sin búsqueda nueva (revisada en vuelta 3); sin cambios. [Vuelta 5] Medipass: ~400.000 usuarios acumulados (CEO, jun-2022); integración con aseguradoras Shinhan Life, Samsung Fire y Hyundai Marine (2020); renovación completa en mar-2023 (dashboard de salud, gestión familiar, certificados). Sin noticias 2026 encontradas. [Vuelta 6] Medipass 2023: comunicación bidireccional hospital-paciente y chat MediTalk; en 2019 fue seleccionada para el programa gubernamental de MyData médico con Samsung Fire y SNUH. Sin estrategia 2026 localizada. Meta declarada: usar Medipass como «identificación» de salud. [Vuelta 7] Una fuente sin fecha atribuye a Medipass más de 600.000 pacientes en 14 hospitales; MoU 2019 con Severance (plataforma de facturación de seguros y detección de falsificación de datos) y piloto con Massachusetts General Hospital. Sin datos 2025-26. [Vuelta 8] Sin noticias 2025-26. [Vuelta 9] Sin búsqueda nueva (saturado).</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G8" t="n">
@@ -766,7 +766,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -793,12 +793,12 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>[BLOCKCHAIN · Reino Unido · INACTIVO] Londres, 2017, Ethereum, con telemedicina. Piloto según registro de la UE (2020). Tracxn/PitchBook lo marcan fuera de operación (ago-2025). Solo caso de aprendizaje: no cuenta como competidor activo. [Vuelta 2] Token MTN deslistado de Bitfinex el 26-mar-2021; sin hallazgos de actividad posterior. [Vuelta 3] Seedtable la marca activa sin fuente; no hallé registro en Companies House. Sigue tratándose como caso de aprendizaje. [Vuelta 4] Pre-venta reportada de US$20M en MedTokens (un solo artículo secundario, sin verificar); modelo de token en revisión y exploración de security token según AMA; integraciones y servicios de 2019 sin confirmar. [Vuelta 5] Un agregador indica sitio medicalchain.com fuera de línea desde 15-feb-2025, último commit en GitHub hace ~3 años y proyecto en «fase de mantenimiento»; preventa de MedTokens reportada entre US$20M y US$24M (fuentes discrepan). Confirma tratarlo como inactivo. [Vuelta 6] Sin búsqueda nueva (revisada en vuelta 5; sitio fuera de línea desde feb-2025 según un agregador); sin cambios. [Vuelta 7] Sin búsqueda nueva (saturado); sin cambios. [Vuelta 8] Sin fuentes nuevas; se mantiene como inactivo.</t>
+          <t>[BLOCKCHAIN · Reino Unido · INACTIVO] Londres, 2017, Ethereum, con telemedicina. Piloto según registro de la UE (2020). Tracxn/PitchBook lo marcan fuera de operación (ago-2025). Solo caso de aprendizaje: no cuenta como competidor activo. [Vuelta 2] Token MTN deslistado de Bitfinex el 26-mar-2021; sin hallazgos de actividad posterior. [Vuelta 3] Seedtable la marca activa sin fuente; no hallé registro en Companies House. Sigue tratándose como caso de aprendizaje. [Vuelta 4] Pre-venta reportada de US$20M en MedTokens (un solo artículo secundario, sin verificar); modelo de token en revisión y exploración de security token según AMA; integraciones y servicios de 2019 sin confirmar. [Vuelta 5] Un agregador indica sitio medicalchain.com fuera de línea desde 15-feb-2025, último commit en GitHub hace ~3 años y proyecto en «fase de mantenimiento»; preventa de MedTokens reportada entre US$20M y US$24M (fuentes discrepan). Confirma tratarlo como inactivo. [Vuelta 6] Sin búsqueda nueva (revisada en vuelta 5; sitio fuera de línea desde feb-2025 según un agregador); sin cambios. [Vuelta 7] Sin búsqueda nueva (saturado); sin cambios. [Vuelta 8] Sin fuentes nuevas; se mantiene como inactivo. [Vuelta 9] Sin búsqueda nueva (saturado).</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G9" t="n">
@@ -806,7 +806,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -10865,7 +10865,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A40"/>
+  <dimension ref="A1:A42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -11151,6 +11151,20 @@
         </is>
       </c>
     </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Vuelta 9 (iter. 2, 2026-10-26 12:21 UTC): Healfies, Patientory, MediBloc, Medicalchain verificados (+0 filas; saturado). Pendientes: Apple Health, ChatGPT Health, Claude for Healthcare, Apps de clínicas, Clinia, MiRedSalud, Mediko.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Ampliación ficha candidato Medicyn (iPhone; desarrollador Pranav Shirole): almacenamiento 100% local (SwiftData con protección de archivos), sin cuentas, nube ni rastreo; guarda condiciones, medicamentos, recetas, alergias, informes de laboratorio y cirugías; escaneo de documentos con IA, seguimiento de síntomas, recordatorios y hasta 6 familiares. Precio inconsistente entre fuentes (prueba de 7 días y pago único según Product Hunt; «gratis» según un directorio). Nota: la política de privacidad menciona suscripciones vía App Store, lo que contradice el «sin suscripciones».</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Benchmark: vuelta 9, iteración 3 (Apple Health, ChatGPT Health, Claude for Healthcare, Apps de clínicas)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MVcXu8vTBu7EKfj3YdEvae
</commit_message>
<xml_diff>
--- a/Outputs/Benchmark_Anamnesis.xlsx
+++ b/Outputs/Benchmark_Anamnesis.xlsx
@@ -833,12 +833,12 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>[ADYACENTE · global] Agrega registros clínicos vía FHIR; &gt;500 instituciones conectadas en EE.UU. (2018). Sin evidencia de disponibilidad en Chile. Incluida en el dispositivo. Amenaza si FHIR/IPS-CL se adopta en Chile. [Vuelta 2] Sin disponibilidad de registros clínicos en Chile (solo EE.UU., Reino Unido, Canadá). [Vuelta 3] iOS 27 (WWDC 8-jun-2026; publicado ~14-sep-2026): rediseño del app Health, menopausia, nutrición por cámara. El coach de salud con IA no se anunció. Sin ampliación de Health Records a Chile. [Vuelta 4] Sin búsqueda nueva (revisada en vuelta 3); sin cambios. [Vuelta 5] Sin ampliación de Health Records a Australia, Europa ni Latinoamérica (solo EE.UU., UK, Canadá). Funciones de dispositivo (apnea del sueño, prueba auditiva) sí se amplían a países latinoamericanos, pero no son registros clínicos. [Vuelta 6] Sin novedades de iOS 27.x localizadas. Health Records API permite compartir registros con apps de terceros con control por app; opción de enviar datos de uso a Apple. [Vuelta 7] Coach de salud con IA / Health+ de pago: solo rumores (Gurman), atrasado al menos a iOS 27; no confirmado ni anunciado. [Vuelta 8] Sin novedades.</t>
+          <t>[ADYACENTE · global] Agrega registros clínicos vía FHIR; &gt;500 instituciones conectadas en EE.UU. (2018). Sin evidencia de disponibilidad en Chile. Incluida en el dispositivo. Amenaza si FHIR/IPS-CL se adopta en Chile. [Vuelta 2] Sin disponibilidad de registros clínicos en Chile (solo EE.UU., Reino Unido, Canadá). [Vuelta 3] iOS 27 (WWDC 8-jun-2026; publicado ~14-sep-2026): rediseño del app Health, menopausia, nutrición por cámara. El coach de salud con IA no se anunció. Sin ampliación de Health Records a Chile. [Vuelta 4] Sin búsqueda nueva (revisada en vuelta 3); sin cambios. [Vuelta 5] Sin ampliación de Health Records a Australia, Europa ni Latinoamérica (solo EE.UU., UK, Canadá). Funciones de dispositivo (apnea del sueño, prueba auditiva) sí se amplían a países latinoamericanos, pero no son registros clínicos. [Vuelta 6] Sin novedades de iOS 27.x localizadas. Health Records API permite compartir registros con apps de terceros con control por app; opción de enviar datos de uso a Apple. [Vuelta 7] Coach de salud con IA / Health+ de pago: solo rumores (Gurman), atrasado al menos a iOS 27; no confirmado ni anunciado. [Vuelta 8] Sin novedades. [Vuelta 9] Sin novedades.</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G10" t="n">
@@ -846,7 +846,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-27</t>
         </is>
       </c>
     </row>
@@ -873,12 +873,12 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>[ADYACENTE · global] Lanzado 7-ene-2026. Conecta registros médicos; conectores solo en EE.UU. Dentro de suscripción del asistente. Fija la expectativa de consultar y resumir el historial. [Vuelta 2] Confirmado: registros solo EE.UU.; sin anuncios para Latinoamérica. Hay inconsistencia de fechas entre fuentes (7-ene-2026 lanzamiento vs. jul-2026 despliegue de registros). [Vuelta 3] Fechas aclaradas: presentación 7-ene-2026 (acceso limitado); despliegue de Health in ChatGPT con Apple Health y registros en EE.UU. el 23-jul-2026; mejora de salud jun-2026. Sin anuncios para Latinoamérica ni para sep-oct 2026. [Vuelta 4] Septiembre 2026: permisos por defecto para datos conectados (14-sep) y explicaciones por gráfico/métrica (28-sep); ChatGPT for Clinicians (abr-2026) para clínicos verificados de EE.UU. Más del 70% de usuarios de Health permite usar datos conectados sin pedir permiso (según OpenAI). Sigue solo EE.UU. [Vuelta 5] Nota de jul-2026: Health no está disponible en México, Android, modo de voz ni Codex; web e iOS en EE.UU., adultos con sesión iniciada. Sin anuncio para Chile ni Latinoamérica. [Vuelta 6] Última entrada de Health en las notas de OpenAI sigue siendo la del 23-jul-2026 (más cambios de sep); sin entradas de octubre localizadas. Health tab: laboratorios, medicamentos, actividad y sueño en una vista; solo EE.UU., web e iOS. [Vuelta 7] OpenAI afirma que más de 300 millones de personas usan ChatGPT cada semana para consultas de salud (dato de la empresa). No es una solución con cumplimiento HIPAA declarado. Sin novedades de oct-2026. [Vuelta 8] Sin novedades de fines de oct-2026.</t>
+          <t>[ADYACENTE · global] Lanzado 7-ene-2026. Conecta registros médicos; conectores solo en EE.UU. Dentro de suscripción del asistente. Fija la expectativa de consultar y resumir el historial. [Vuelta 2] Confirmado: registros solo EE.UU.; sin anuncios para Latinoamérica. Hay inconsistencia de fechas entre fuentes (7-ene-2026 lanzamiento vs. jul-2026 despliegue de registros). [Vuelta 3] Fechas aclaradas: presentación 7-ene-2026 (acceso limitado); despliegue de Health in ChatGPT con Apple Health y registros en EE.UU. el 23-jul-2026; mejora de salud jun-2026. Sin anuncios para Latinoamérica ni para sep-oct 2026. [Vuelta 4] Septiembre 2026: permisos por defecto para datos conectados (14-sep) y explicaciones por gráfico/métrica (28-sep); ChatGPT for Clinicians (abr-2026) para clínicos verificados de EE.UU. Más del 70% de usuarios de Health permite usar datos conectados sin pedir permiso (según OpenAI). Sigue solo EE.UU. [Vuelta 5] Nota de jul-2026: Health no está disponible en México, Android, modo de voz ni Codex; web e iOS en EE.UU., adultos con sesión iniciada. Sin anuncio para Chile ni Latinoamérica. [Vuelta 6] Última entrada de Health en las notas de OpenAI sigue siendo la del 23-jul-2026 (más cambios de sep); sin entradas de octubre localizadas. Health tab: laboratorios, medicamentos, actividad y sueño en una vista; solo EE.UU., web e iOS. [Vuelta 7] OpenAI afirma que más de 300 millones de personas usan ChatGPT cada semana para consultas de salud (dato de la empresa). No es una solución con cumplimiento HIPAA declarado. Sin novedades de oct-2026. [Vuelta 8] Sin novedades de fines de oct-2026. [Vuelta 9] Reporte de sep-2026: OpenAI conecta ChatGPT con Epic EHR para clínicos de EE.UU. (sin confirmar con fuente primaria). Sin novedades de oct-2026 para el consumidor.</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G11" t="n">
@@ -886,7 +886,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-27</t>
         </is>
       </c>
     </row>
@@ -913,12 +913,12 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>[ADYACENTE · global] Lanzado 11-ene-2026. Conectores solo en EE.UU., planes Pro/Max. Nota: producto de Anthropic, conflicto de interés al evaluarlo. [Vuelta 2] Sin cambios fuera de EE.UU. (HealthEx y Function para Pro/Max). [Vuelta 3] Sin anuncios posteriores a enero de 2026. Hoja de ruta de HealthEx (agendar, buscar prestadores, recetas) sin confirmar como lanzada. [Vuelta 4] Sin anuncios nuevos. Fuentes discrepan en el acceso (Pro/Max según Fortune y la mayoría; Pro/Team según Times of AI); sin evidencia de disponibilidad fuera de EE.UU. [Vuelta 5] Sin noticias de oct-2026; HealthEx agrega datos de &gt;50.000 sistemas de EE.UU. y Claude pide solo las categorías relevantes vía MCP. [Vuelta 6] Sin noticias posteriores a enero de 2026 localizadas. [Vuelta 7] Sin novedades posteriores a enero de 2026. [Vuelta 8] Sin novedades posteriores a enero de 2026.</t>
+          <t>[ADYACENTE · global] Lanzado 11-ene-2026. Conectores solo en EE.UU., planes Pro/Max. Nota: producto de Anthropic, conflicto de interés al evaluarlo. [Vuelta 2] Sin cambios fuera de EE.UU. (HealthEx y Function para Pro/Max). [Vuelta 3] Sin anuncios posteriores a enero de 2026. Hoja de ruta de HealthEx (agendar, buscar prestadores, recetas) sin confirmar como lanzada. [Vuelta 4] Sin anuncios nuevos. Fuentes discrepan en el acceso (Pro/Max según Fortune y la mayoría; Pro/Team según Times of AI); sin evidencia de disponibilidad fuera de EE.UU. [Vuelta 5] Sin noticias de oct-2026; HealthEx agrega datos de &gt;50.000 sistemas de EE.UU. y Claude pide solo las categorías relevantes vía MCP. [Vuelta 6] Sin noticias posteriores a enero de 2026 localizadas. [Vuelta 7] Sin novedades posteriores a enero de 2026. [Vuelta 8] Sin novedades posteriores a enero de 2026. [Vuelta 9] Sin novedades posteriores a enero de 2026.</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G12" t="n">
@@ -926,7 +926,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-27</t>
         </is>
       </c>
     </row>
@@ -953,12 +953,12 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>[SUSTITUTO PARCIAL · Chile] Reservar hora, ver historial de esa institución, vincular familiar. Gratis; no consolida datos de otras instituciones. [Vuelta 2] App concreta: Mi Alemana Go (Clínica Alemana, Chile), con historial desde 2018, recetas, órdenes, familiar vinculado y resultados. [Vuelta 3] Búsqueda de otras clínicas (Las Condes, Santa María, UC Christus) sin ficha de app confirmada; solo canales digitales genéricos. [Vuelta 4] Mi Alemana Go: 3,1/5 con 137 calificaciones (App Store Chile), pantalla de inicio rediseñada para gestionar salud propia y familiar; sin evidencia de teleconsulta ni pagos en la app. [Vuelta 5] Sin búsqueda nueva (revisada en vuelta 4); sin cambios. [Vuelta 6] Sin búsqueda nueva; sin cambios. [Vuelta 7] Sin búsqueda nueva; sin cambios. [Vuelta 8] Mi Alemana Go: notificaciones de deuda pendiente, check-in de admisión y encuestas de salud; DF la describe como segundo paso de la estrategia digital de la clínica (registros de exámenes, indicaciones, historial y recetas). Otras apps de red: Mi Dávila (Red Dávila, gestión de citas en todos sus centros, según un directorio); Clínica Las Condes sin app confirmada.</t>
+          <t>[SUSTITUTO PARCIAL · Chile] Reservar hora, ver historial de esa institución, vincular familiar. Gratis; no consolida datos de otras instituciones. [Vuelta 2] App concreta: Mi Alemana Go (Clínica Alemana, Chile), con historial desde 2018, recetas, órdenes, familiar vinculado y resultados. [Vuelta 3] Búsqueda de otras clínicas (Las Condes, Santa María, UC Christus) sin ficha de app confirmada; solo canales digitales genéricos. [Vuelta 4] Mi Alemana Go: 3,1/5 con 137 calificaciones (App Store Chile), pantalla de inicio rediseñada para gestionar salud propia y familiar; sin evidencia de teleconsulta ni pagos en la app. [Vuelta 5] Sin búsqueda nueva (revisada en vuelta 4); sin cambios. [Vuelta 6] Sin búsqueda nueva; sin cambios. [Vuelta 7] Sin búsqueda nueva; sin cambios. [Vuelta 8] Mi Alemana Go: notificaciones de deuda pendiente, check-in de admisión y encuestas de salud; DF la describe como segundo paso de la estrategia digital de la clínica (registros de exámenes, indicaciones, historial y recetas). Otras apps de red: Mi Dávila (Red Dávila, gestión de citas en todos sus centros, según un directorio); Clínica Las Condes sin app confirmada. [Vuelta 9] Sin búsqueda nueva; sin cambios.</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G13" t="n">
@@ -966,7 +966,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-27</t>
         </is>
       </c>
     </row>
@@ -1102,7 +1102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F134"/>
+  <dimension ref="A1:F135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -5398,6 +5398,38 @@
       <c r="F134" t="inlineStr">
         <is>
           <t>Ficha App Store Chile (Mi Alemana Go)</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>ChatGPT Health (OpenAI)</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Interoperabilidad y fuentes de datos</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Conexión directa con Epic EHR para clínicos (reporte sep-2026)</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>Un reporte del 1-sep-2026 indica que OpenAI conecta ChatGPT directamente con los registros electrónicos Epic para clínicos de EE.UU.; lado profesional, no del paciente.</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>Búsqueda web (Healthcare Brew, Becker's); sin confirmar con fuente primaria</t>
         </is>
       </c>
     </row>
@@ -10865,7 +10897,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A42"/>
+  <dimension ref="A1:A43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -11165,6 +11197,13 @@
         </is>
       </c>
     </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Vuelta 9 (iter. 3, 2026-10-27 12:41 UTC): Apple Health, ChatGPT Health, Claude for Healthcare, Apps de clínicas verificados (+1 fila). Pendientes: Clinia, MiRedSalud, Mediko (cierran la vuelta 9 y regeneran func_norm/tabla_frecuencia).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Benchmark: cierre vuelta 9; contador=9; func_norm y tabla_frecuencia regenerados
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MVcXu8vTBu7EKfj3YdEvae
</commit_message>
<xml_diff>
--- a/Outputs/Benchmark_Anamnesis.xlsx
+++ b/Outputs/Benchmark_Anamnesis.xlsx
@@ -518,15 +518,15 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -558,15 +558,15 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -598,15 +598,15 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -638,15 +638,15 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G5" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -678,15 +678,15 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -718,15 +718,15 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -758,15 +758,15 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G8" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -798,15 +798,15 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G9" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -838,15 +838,15 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -878,15 +878,15 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G11" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -918,15 +918,15 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G12" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -958,15 +958,15 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G13" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -993,7 +993,7 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>[DIRECTO · Chile · etapa A] App móvil anunciada en sep-2026 para centralizar recetas, diagnósticos y laboratorios en un solo lugar; respaldada por Reservo (tecnológica chilena desde 2015, software para profesionales y centros de salud). AMENAZA ALTA: Reservo ya tiene red de profesionales/centros que podrían alimentar el historial. Fuente: solo snippet de búsqueda (sitio bloqueado en este entorno); precio, funciones de compartir y sitio oficial por verificar. [Vuelta 2] Confirmado por el CEO de Reservo (LinkedIn): app para pacientes en App Store y Google Play; guarda y comparte exámenes, recetas, órdenes y certificados. Fecha exacta de lanzamiento, precio y modelo de datos sin verificar. [Vuelta 3] Sin novedades de oct-2026. Reservo (Chile, México, Argentina) declara certificación Fonasa/CENS y cumplimiento de la nueva ley de datos personales; el Portal de Agendamiento de Reservo complementa a Clinia. Precio y modelo de datos sin verificar. [Vuelta 4] Una búsqueda adicional no encontró fuentes independientes sobre Clinia de Reservo (aparecen otras empresas llamadas Clinia); la evidencia sigue siendo la publicación del CEO en LinkedIn y notas de Reservo. Confianza media. [Vuelta 5] Sin fecha verificable del lanzamiento (publicación de LinkedIn del CEO sin fecha visible); existe otra empresa homónima en Brasil (Porto Alegre, IA para clínicas) que no es este producto. Sin funciones nuevas. [Vuelta 6] Sin novedades de oct-2026. Reservo declara &gt;36.500 profesionales y centros y ~14 millones de reservas al año (Chile, México, Argentina), sello CENS y certificación Fonasa (autodeclarado); la publicación del CEO pide ideas de nuevas funciones. Sigue sin fecha de lanzamiento verificable. [Vuelta 7] Sin novedades; sin datos verificables de descargas ni calificación. Reservo: fundada en 2015 según una fuente (otra indica 2017). No confundir con Clinia de Brasil. [Vuelta 8] Sin búsqueda nueva (saturado); sin cambios.</t>
+          <t>[DIRECTO · Chile · etapa A] App móvil anunciada en sep-2026 para centralizar recetas, diagnósticos y laboratorios en un solo lugar; respaldada por Reservo (tecnológica chilena desde 2015, software para profesionales y centros de salud). AMENAZA ALTA: Reservo ya tiene red de profesionales/centros que podrían alimentar el historial. Fuente: solo snippet de búsqueda (sitio bloqueado en este entorno); precio, funciones de compartir y sitio oficial por verificar. [Vuelta 2] Confirmado por el CEO de Reservo (LinkedIn): app para pacientes en App Store y Google Play; guarda y comparte exámenes, recetas, órdenes y certificados. Fecha exacta de lanzamiento, precio y modelo de datos sin verificar. [Vuelta 3] Sin novedades de oct-2026. Reservo (Chile, México, Argentina) declara certificación Fonasa/CENS y cumplimiento de la nueva ley de datos personales; el Portal de Agendamiento de Reservo complementa a Clinia. Precio y modelo de datos sin verificar. [Vuelta 4] Una búsqueda adicional no encontró fuentes independientes sobre Clinia de Reservo (aparecen otras empresas llamadas Clinia); la evidencia sigue siendo la publicación del CEO en LinkedIn y notas de Reservo. Confianza media. [Vuelta 5] Sin fecha verificable del lanzamiento (publicación de LinkedIn del CEO sin fecha visible); existe otra empresa homónima en Brasil (Porto Alegre, IA para clínicas) que no es este producto. Sin funciones nuevas. [Vuelta 6] Sin novedades de oct-2026. Reservo declara &gt;36.500 profesionales y centros y ~14 millones de reservas al año (Chile, México, Argentina), sello CENS y certificación Fonasa (autodeclarado); la publicación del CEO pide ideas de nuevas funciones. Sigue sin fecha de lanzamiento verificable. [Vuelta 7] Sin novedades; sin datos verificables de descargas ni calificación. Reservo: fundada en 2015 según una fuente (otra indica 2017). No confundir con Clinia de Brasil. [Vuelta 8] Sin búsqueda nueva (saturado); sin cambios. [Vuelta 9] Sin búsqueda nueva (saturado); sin cambios.</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1002,11 +1002,11 @@
         </is>
       </c>
       <c r="G14" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -1033,7 +1033,7 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>[SUSTITUTO PARCIAL · Chile] Nueva app móvil de la red RedSalud anunciada dic-2025: acceso a información clínica y servicios, guardar y administrar historial propio y familiar. Limitación: solo datos de la propia red; no consolida otras instituciones. Precio por verificar (probablemente gratis). [Vuelta 2] La búsqueda no encontró fuentes adicionales ni ficha de la app chilena (solo una app RedSalud de otro país); funciones sin confirmar. [Vuelta 3] Rankings de terceros la ubican como app médica gratuita nº 1 en App Store y Google Play Chile (fecha desconocida); sin descripción de funciones ni confirmación del desarrollador en Google Play. [Vuelta 4] Sin documentación oficial chilena localizada; las fichas con funciones (agendar, telemedicina, historial de hijos) corresponden a una app RedSalud de otro país. Quejas públicas 2020-21 sobre acceso en línea a resultados. Funciones de MiRedSalud sin confirmar. [Vuelta 5] Una búsqueda adicional no halló cobertura del lanzamiento de dic-2025 ni de la app chilena; solo apps de otras empresas Red Salud (Paraguay, Perú). Sigue sin confirmarse más allá de la nota de RedSalud. [Vuelta 6] Sin cobertura adicional; los resultados corresponden a la plataforma Red Salud de Paraguay (Interasistencia, ~350 especialistas, call center por WhatsApp), que no es la red chilena. Funciones de MiRedSalud sin confirmar. [Vuelta 7] Sin búsqueda nueva (saturado); sin cambios. [Vuelta 8] Sin búsqueda nueva (saturado); sin cambios.</t>
+          <t>[SUSTITUTO PARCIAL · Chile] Nueva app móvil de la red RedSalud anunciada dic-2025: acceso a información clínica y servicios, guardar y administrar historial propio y familiar. Limitación: solo datos de la propia red; no consolida otras instituciones. Precio por verificar (probablemente gratis). [Vuelta 2] La búsqueda no encontró fuentes adicionales ni ficha de la app chilena (solo una app RedSalud de otro país); funciones sin confirmar. [Vuelta 3] Rankings de terceros la ubican como app médica gratuita nº 1 en App Store y Google Play Chile (fecha desconocida); sin descripción de funciones ni confirmación del desarrollador en Google Play. [Vuelta 4] Sin documentación oficial chilena localizada; las fichas con funciones (agendar, telemedicina, historial de hijos) corresponden a una app RedSalud de otro país. Quejas públicas 2020-21 sobre acceso en línea a resultados. Funciones de MiRedSalud sin confirmar. [Vuelta 5] Una búsqueda adicional no halló cobertura del lanzamiento de dic-2025 ni de la app chilena; solo apps de otras empresas Red Salud (Paraguay, Perú). Sigue sin confirmarse más allá de la nota de RedSalud. [Vuelta 6] Sin cobertura adicional; los resultados corresponden a la plataforma Red Salud de Paraguay (Interasistencia, ~350 especialistas, call center por WhatsApp), que no es la red chilena. Funciones de MiRedSalud sin confirmar. [Vuelta 7] Sin búsqueda nueva (saturado); sin cambios. [Vuelta 8] Sin búsqueda nueva (saturado); sin cambios. [Vuelta 9] Sin búsqueda nueva (saturado); sin cambios.</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1042,11 +1042,11 @@
         </is>
       </c>
       <c r="G15" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -1073,7 +1073,7 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>[ADYACENTE · Chile] Fundada 2022. Orientación médica inmediata, interpretación de exámenes y órdenes médicas digitales con IA; modelo freemium, suscripción y pago por servicio; menciona centralizar registros y monitoreo. Foco asistencial, no archivo personal; vigilar si añade historial. Grants por ~$40M según Descubre.vc. [Vuelta 2] Sin precios ni planes vigentes localizados; sitio oficial bloqueado. [Vuelta 3] Pauta (oct-2024): su fundador, Tomás Riddell, dice que no reemplaza a médicos y apunta a lo ambulatorio y a la espera de derivación a especialidad en el sistema público. Financiamiento: fuentes discrepan (CLP 25M en dic-2023 según Bouncewatch; ~$40M según Descubre.vc). Precios vigentes sin verificar. [Vuelta 4] Entrevista oct-2024 menciona integración con la pasarela Flow. Sin novedades 2025-26 ni rondas verificadas; la cifra de US$40M de Bouncewatch es dudosa (perfil con 2 empleados). [Vuelta 5] CORRECCIÓN de financiamiento: Bouncewatch registra dos subvenciones (CLP 15M en ago-2022 y CLP 25M en dic-2023 = CLP 40M en total), no US$40M; 2 empleados; etapa Seed según Descubre.vc. No hay inversionistas de capital listados. [Vuelta 6] Sin noticias 2026 propias. Contexto: evento «IA y Salud en Chile 2026» (12-may) sobre regulación, datos personales e interoperabilidad de fichas clínicas; Doctoralia lanzó Noa Evidence (jul-2026, asistente de IA para profesionales); programa PRISMA IA 2.0 (dic-2025). [Vuelta 7] Sigue sin precios publicados de planes; un directorio la describe como gratuita y sin cuenta en su nivel básico (sin verificar). [Vuelta 8] Sin búsqueda nueva (saturado); sin cambios.</t>
+          <t>[ADYACENTE · Chile] Fundada 2022. Orientación médica inmediata, interpretación de exámenes y órdenes médicas digitales con IA; modelo freemium, suscripción y pago por servicio; menciona centralizar registros y monitoreo. Foco asistencial, no archivo personal; vigilar si añade historial. Grants por ~$40M según Descubre.vc. [Vuelta 2] Sin precios ni planes vigentes localizados; sitio oficial bloqueado. [Vuelta 3] Pauta (oct-2024): su fundador, Tomás Riddell, dice que no reemplaza a médicos y apunta a lo ambulatorio y a la espera de derivación a especialidad en el sistema público. Financiamiento: fuentes discrepan (CLP 25M en dic-2023 según Bouncewatch; ~$40M según Descubre.vc). Precios vigentes sin verificar. [Vuelta 4] Entrevista oct-2024 menciona integración con la pasarela Flow. Sin novedades 2025-26 ni rondas verificadas; la cifra de US$40M de Bouncewatch es dudosa (perfil con 2 empleados). [Vuelta 5] CORRECCIÓN de financiamiento: Bouncewatch registra dos subvenciones (CLP 15M en ago-2022 y CLP 25M en dic-2023 = CLP 40M en total), no US$40M; 2 empleados; etapa Seed según Descubre.vc. No hay inversionistas de capital listados. [Vuelta 6] Sin noticias 2026 propias. Contexto: evento «IA y Salud en Chile 2026» (12-may) sobre regulación, datos personales e interoperabilidad de fichas clínicas; Doctoralia lanzó Noa Evidence (jul-2026, asistente de IA para profesionales); programa PRISMA IA 2.0 (dic-2025). [Vuelta 7] Sigue sin precios publicados de planes; un directorio la describe como gratuita y sin cuenta en su nivel básico (sin verificar). [Vuelta 8] Sin búsqueda nueva (saturado); sin cambios. [Vuelta 9] Sin búsqueda nueva (saturado); sin cambios.</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1082,11 +1082,11 @@
         </is>
       </c>
       <c r="G16" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -5444,7 +5444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E134"/>
+  <dimension ref="A1:E135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -8022,7 +8022,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Medicalchain</t>
+          <t>ChatGPT Health (OpenAI)</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -8037,7 +8037,7 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Según una AMA sin fecha, integraba dos sistemas de GP que cubren ~80% del mercado UK; no confirmado como ejecutado.</t>
+          <t>Un reporte del 1-sep-2026 indica que OpenAI conecta ChatGPT directamente con los registros electrónicos Epic para clínicos de EE.UU.; lado profesional, no del paciente.</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
@@ -8049,7 +8049,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Claude for Healthcare (Anthropic)</t>
+          <t>Medicalchain</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -8059,12 +8059,12 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Integración con wearables y apps de salud</t>
+          <t>Integración con EHR de proveedores</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Integración beta en apps iOS/Android.</t>
+          <t>Según una AMA sin fecha, integraba dos sistemas de GP que cubren ~80% del mercado UK; no confirmado como ejecutado.</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
@@ -8091,7 +8091,7 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Integración beta con Health Connect en la app móvil; conectores de registros (HealthEx, Function) solo para Pro/Max en EE.UU.</t>
+          <t>Integración beta en apps iOS/Android.</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
@@ -8103,7 +8103,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Patientory</t>
+          <t>Claude for Healthcare (Anthropic)</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -8118,7 +8118,7 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Se integra con wearables y apps móviles populares y muestra vitales en un panel unificado.</t>
+          <t>Integración beta con Health Connect en la app móvil; conectores de registros (HealthEx, Function) solo para Pro/Max en EE.UU.</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
@@ -8130,22 +8130,22 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Apple Health (Health Records)</t>
+          <t>Patientory</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Medicación y recordatorios</t>
+          <t>Interoperabilidad y fuentes de datos</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Gestión de lista de medicamentos</t>
+          <t>Integración con wearables y apps de salud</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Listas de medicamentos, vitaminas y suplementos con horarios; escaneo de etiqueta del frasco solo en EE.UU.</t>
+          <t>Se integra con wearables y apps móviles populares y muestra vitales en un panel unificado.</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
@@ -8157,7 +8157,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>MediPlanner</t>
+          <t>Apple Health (Health Records)</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -8167,24 +8167,24 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Importación automática de tratamientos desde receta digital</t>
+          <t>Gestión de lista de medicamentos</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Según la ficha de la App Store MX, los tratamientos llegan automáticamente desde la receta digital del médico (autodeclarado, sin verificar).</t>
+          <t>Listas de medicamentos, vitaminas y suplementos con horarios; escaneo de etiqueta del frasco solo en EE.UU.</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Latam</t>
+          <t>Global</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Apple Health (Health Records)</t>
+          <t>MediPlanner</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -8194,24 +8194,24 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Recordatorios de medicación y citas</t>
+          <t>Importación automática de tratamientos desde receta digital</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Recordatorios desde el app.</t>
+          <t>Según la ficha de la App Store MX, los tratamientos llegan automáticamente desde la receta digital del médico (autodeclarado, sin verificar).</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Latam</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Meedika</t>
+          <t>Apple Health (Health Records)</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -8226,19 +8226,19 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Recordatorios de citas/medicación.</t>
+          <t>Recordatorios desde el app.</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Global</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>MediPlanner</t>
+          <t>Meedika</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -8248,51 +8248,51 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Registro de tomas y adherencia al tratamiento</t>
+          <t>Recordatorios de medicación y citas</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Registro de cada toma y control de adherencia; gestiona medicamentos propios y de familiares.</t>
+          <t>Recordatorios de citas/medicación.</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Latam</t>
+          <t>Chile</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Patientory</t>
+          <t>MediPlanner</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Seguimiento y bienestar</t>
+          <t>Medicación y recordatorios</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Comunidad de pacientes</t>
+          <t>Registro de tomas y adherencia al tratamiento</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Los usuarios con condiciones similares pueden preguntar, recibir recomendaciones y compartir experiencias.</t>
+          <t>Registro de cada toma y control de adherencia; gestiona medicamentos propios y de familiares.</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Latam</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Infomed</t>
+          <t>Patientory</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -8302,24 +8302,24 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Contenido educativo sobre salud</t>
+          <t>Comunidad de pacientes</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Busca que el paciente aprenda sobre sus enfermedades y sea más autónomo.</t>
+          <t>Los usuarios con condiciones similares pueden preguntar, recibir recomendaciones y compartir experiencias.</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Global</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>MediPlanner</t>
+          <t>Infomed</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -8329,24 +8329,24 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Gráficas de evolución de indicadores</t>
+          <t>Contenido educativo sobre salud</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Gráficas de evolución de indicadores de salud.</t>
+          <t>Busca que el paciente aprenda sobre sus enfermedades y sea más autónomo.</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>Latam</t>
+          <t>Chile</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Apple Health (Health Records)</t>
+          <t>MediPlanner</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -8356,24 +8356,24 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Integración con wearables y apps de salud</t>
+          <t>Gráficas de evolución de indicadores</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Datos de pasos, sueño, peso junto a registros.</t>
+          <t>Gráficas de evolución de indicadores de salud.</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Latam</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>MediBloc</t>
+          <t>Apple Health (Health Records)</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -8383,12 +8383,12 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Panel de seguimiento de salud y bienestar</t>
+          <t>Integración con wearables y apps de salud</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>El relanzamiento de Medipass (mar-2023) agregó un panel para gestionar la información de salud del usuario.</t>
+          <t>Datos de pasos, sueño, peso junto a registros.</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
@@ -8400,7 +8400,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Patientory</t>
+          <t>MediBloc</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -8415,7 +8415,7 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Seguimiento de hábitos saludables y monitoreo de progreso.</t>
+          <t>El relanzamiento de Medipass (mar-2023) agregó un panel para gestionar la información de salud del usuario.</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
@@ -8427,7 +8427,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Apple Health (Health Records)</t>
+          <t>Patientory</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -8437,12 +8437,12 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Registro de nutrición</t>
+          <t>Panel de seguimiento de salud y bienestar</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Escaneo de etiquetas nutricionales con la cámara; según un análisis, no escribe en HealthKit.</t>
+          <t>Seguimiento de hábitos saludables y monitoreo de progreso.</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
@@ -8464,12 +8464,12 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Seguimiento de salud femenina</t>
+          <t>Registro de nutrición</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Extiende el seguimiento de ciclo con perimenopausia y menopausia.</t>
+          <t>Escaneo de etiquetas nutricionales con la cámara; según un análisis, no escribe en HealthKit.</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
@@ -8481,7 +8481,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Clingot</t>
+          <t>Apple Health (Health Records)</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -8491,51 +8491,51 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Valoración de profesionales</t>
+          <t>Seguimiento de salud femenina</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Calificación de la atención de profesionales con autorización previa, compartible con otros usuarios.</t>
+          <t>Extiende el seguimiento de ciclo con perimenopausia y menopausia.</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>Latam</t>
+          <t>Global</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Claude for Healthcare (Anthropic)</t>
+          <t>Clingot</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Seguridad, privacidad y blockchain</t>
+          <t>Seguimiento y bienestar</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Acceso mínimo por categorías de datos</t>
+          <t>Valoración de profesionales</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Claude solicita solo las categorías relevantes (p. ej. medicamentos o laboratorio) y no fichas completas; HealthEx agrega datos de más de 50.000 sistemas de salud de EE.UU.</t>
+          <t>Calificación de la atención de profesionales con autorización previa, compartible con otros usuarios.</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Latam</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>MediBloc</t>
+          <t>Claude for Healthcare (Anthropic)</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -8545,12 +8545,12 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Blockchain para integridad y trazabilidad de datos</t>
+          <t>Acceso mínimo por categorías de datos</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Blockchain propia (Cosmos SDK) para que el paciente almacene, use, actualice y transfiera sus registros; los datos no se guardan en la cadena, solo en el usuario, cifrados.</t>
+          <t>Claude solicita solo las categorías relevantes (p. ej. medicamentos o laboratorio) y no fichas completas; HealthEx agrega datos de más de 50.000 sistemas de salud de EE.UU.</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
@@ -8577,7 +8577,7 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Almacena huellas de datos médicos en un registro de solo escritura, sin guardar datos clínicos en cadena.</t>
+          <t>Blockchain propia (Cosmos SDK) para que el paciente almacene, use, actualice y transfiera sus registros; los datos no se guardan en la cadena, solo en el usuario, cifrados.</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
@@ -8589,7 +8589,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Medicalchain</t>
+          <t>MediBloc</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -8604,7 +8604,7 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Cada solicitud de acceso queda en un libro distribuido; acceso temporal por contratos inteligentes.</t>
+          <t>Almacena huellas de datos médicos en un registro de solo escritura, sin guardar datos clínicos en cadena.</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
@@ -8616,7 +8616,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Patientory</t>
+          <t>Medicalchain</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -8631,7 +8631,7 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Registro respaldado en blockchain para seguridad y trazabilidad.</t>
+          <t>Cada solicitud de acceso queda en un libro distribuido; acceso temporal por contratos inteligentes.</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
@@ -8643,7 +8643,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Apple Health (Health Records)</t>
+          <t>Patientory</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -8653,12 +8653,12 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Cifrado y control de acceso</t>
+          <t>Blockchain para integridad y trazabilidad de datos</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Registros cifrados en el dispositivo, protegidos por Face ID/Touch ID/código.</t>
+          <t>Registro respaldado en blockchain para seguridad y trazabilidad.</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
@@ -8670,7 +8670,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>Infomed</t>
+          <t>Apple Health (Health Records)</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -8685,19 +8685,19 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>Almacenamiento seguro del historial con criterios de seguridad estrictos, comparable a apps bancarias.</t>
+          <t>Registros cifrados en el dispositivo, protegidos por Face ID/Touch ID/código.</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Global</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Clinia (Reservo)</t>
+          <t>Infomed</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -8707,12 +8707,12 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Cumplimiento regulatorio de salud y datos</t>
+          <t>Cifrado y control de acceso</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>Reservo declara plataforma certificada por Fonasa y CENS, cumplimiento de estándares de telemedicina del Minsal y de la nueva ley chilena de datos personales (declaración de la empresa).</t>
+          <t>Almacenamiento seguro del historial con criterios de seguridad estrictos, comparable a apps bancarias.</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
@@ -8724,7 +8724,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>ChatGPT Health (OpenAI)</t>
+          <t>Clinia (Reservo)</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -8734,24 +8734,24 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Gestión de consentimiento sobre uso de datos</t>
+          <t>Cumplimiento regulatorio de salud y datos</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Desde 14-sep-2026, las nuevas conexiones heredan la configuración global de plugins: ChatGPT puede usar datos de Health sin pedir permiso cada vez salvo acciones sensibles (web primero, móvil después).</t>
+          <t>Reservo declara plataforma certificada por Fonasa y CENS, cumplimiento de estándares de telemedicina del Minsal y de la nueva ley chilena de datos personales (declaración de la empresa).</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Chile</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>MediBloc</t>
+          <t>ChatGPT Health (OpenAI)</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -8761,12 +8761,12 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Identidad descentralizada (DID)</t>
+          <t>Gestión de consentimiento sobre uso de datos</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>Gestión de identificadores descentralizados en Panacea.</t>
+          <t>Desde 14-sep-2026, las nuevas conexiones heredan la configuración global de plugins: ChatGPT puede usar datos de Health sin pedir permiso cada vez salvo acciones sensibles (web primero, móvil después).</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
@@ -8778,7 +8778,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>ChatGPT Health (OpenAI)</t>
+          <t>MediBloc</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -8788,12 +8788,12 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Privacidad reforzada para datos de salud</t>
+          <t>Identidad descentralizada (DID)</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Chats y memoria de salud separados, no usados para entrenar modelos.</t>
+          <t>Gestión de identificadores descentralizados en Panacea.</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
@@ -8805,7 +8805,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>Claude for Healthcare (Anthropic)</t>
+          <t>ChatGPT Health (OpenAI)</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -8820,7 +8820,7 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>El usuario activa y revoca permisos; los datos de salud compartidos se excluyen de la memoria de Claude y del entrenamiento.</t>
+          <t>Chats y memoria de salud separados, no usados para entrenar modelos.</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
@@ -8832,34 +8832,34 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Mediko</t>
+          <t>Claude for Healthcare (Anthropic)</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>Seguros y pagos</t>
+          <t>Seguridad, privacidad y blockchain</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Modelo freemium y suscripción</t>
+          <t>Privacidad reforzada para datos de salud</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>Planes para personas y empresas.</t>
+          <t>El usuario activa y revoca permisos; los datos de salud compartidos se excluyen de la memoria de Claude y del entrenamiento.</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Global</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>Medicalchain</t>
+          <t>Mediko</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -8869,17 +8869,17 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Pagos con criptomoneda</t>
+          <t>Modelo freemium y suscripción</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Pago de consultas con token.</t>
+          <t>Planes para personas y empresas.</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Chile</t>
         </is>
       </c>
     </row>
@@ -8901,7 +8901,7 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>Piloto en New Malden (Londres): consultas por video pagables con tarjeta o con MedTokens.</t>
+          <t>Pago de consultas con token.</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
@@ -8913,7 +8913,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>Apps de clínicas (ej. Clínica Alemana de Valdivia)</t>
+          <t>Medicalchain</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -8923,24 +8923,24 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Pagos dentro de la app</t>
+          <t>Pagos con criptomoneda</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Sección de notificaciones que avisa cuando hay una deuda disponible para pagar (fecha de la actualización desconocida).</t>
+          <t>Piloto en New Malden (Londres): consultas por video pagables con tarjeta o con MedTokens.</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Global</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>Mediko</t>
+          <t>Apps de clínicas (ej. Clínica Alemana de Valdivia)</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -8955,7 +8955,7 @@
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>Pagos dentro de la plataforma mediante la pasarela Flow (según resumen de entrevista de Pauta, oct-2024; esperada para mejorar la experiencia).</t>
+          <t>Sección de notificaciones que avisa cuando hay una deuda disponible para pagar (fecha de la actualización desconocida).</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
@@ -8967,7 +8967,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>MediBloc</t>
+          <t>Mediko</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -8977,17 +8977,17 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>Reclamos y trámites con seguros</t>
+          <t>Pagos dentro de la app</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Simplifica el envío a aseguradoras sin gestionar papeles en hospitales.</t>
+          <t>Pagos dentro de la plataforma mediante la pasarela Flow (según resumen de entrevista de Pauta, oct-2024; esperada para mejorar la experiencia).</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Chile</t>
         </is>
       </c>
     </row>
@@ -9009,7 +9009,7 @@
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>Reclamo de seguro médico (indemnización) desde la app, con verificación de autenticidad de los registros vía blockchain por la aseguradora.</t>
+          <t>Simplifica el envío a aseguradoras sin gestionar papeles en hospitales.</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
@@ -9026,17 +9026,17 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>Telemedicina y atención remota</t>
+          <t>Seguros y pagos</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>Mensajería paciente-institución</t>
+          <t>Reclamos y trámites con seguros</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>Chat para consultas a hospitales, orientación simple de síntomas e información de tratamientos; comunicación bidireccional hospital-paciente (nov-2023).</t>
+          <t>Reclamo de seguro médico (indemnización) desde la app, con verificación de autenticidad de los registros vía blockchain por la aseguradora.</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
@@ -9048,25 +9048,52 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
+          <t>MediBloc</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Telemedicina y atención remota</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Mensajería paciente-institución</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>Chat para consultas a hospitales, orientación simple de síntomas e información de tratamientos; comunicación bidireccional hospital-paciente (nov-2023).</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
           <t>Medicalchain</t>
         </is>
       </c>
-      <c r="B134" t="inlineStr">
+      <c r="B135" t="inlineStr">
         <is>
           <t>Telemedicina y atención remota</t>
         </is>
       </c>
-      <c r="C134" t="inlineStr">
+      <c r="C135" t="inlineStr">
         <is>
           <t>Teleconsulta con profesionales</t>
         </is>
       </c>
-      <c r="D134" t="inlineStr">
+      <c r="D135" t="inlineStr">
         <is>
           <t>Teleconsultas con GP.</t>
         </is>
       </c>
-      <c r="E134" t="inlineStr">
+      <c r="E135" t="inlineStr">
         <is>
           <t>Global</t>
         </is>
@@ -9209,6 +9236,8 @@
           <t>Búsqueda de profesionales de salud</t>
         </is>
       </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9219,6 +9248,17 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr"/>
       <c r="R2">
         <f>COUNTIF(C2:Q2,"✓")</f>
         <v/>
@@ -9240,11 +9280,24 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr"/>
       <c r="R3">
         <f>COUNTIF(C3:Q3,"✓")</f>
         <v/>
@@ -9261,11 +9314,25 @@
           <t>Check-in de admisión digital</t>
         </is>
       </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr"/>
       <c r="R4">
         <f>COUNTIF(C4:Q4,"✓")</f>
         <v/>
@@ -9282,11 +9349,25 @@
           <t>Integración con calendario del dispositivo</t>
         </is>
       </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr"/>
       <c r="R5">
         <f>COUNTIF(C5:Q5,"✓")</f>
         <v/>
@@ -9303,11 +9384,25 @@
           <t>Localización de centros médicos y farmacias</t>
         </is>
       </c>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr"/>
       <c r="R6">
         <f>COUNTIF(C6:Q6,"✓")</f>
         <v/>
@@ -9324,11 +9419,21 @@
           <t>Reserva de citas médicas</t>
         </is>
       </c>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9339,6 +9444,8 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="P7" t="inlineStr"/>
+      <c r="Q7" t="inlineStr"/>
       <c r="R7">
         <f>COUNTIF(C7:Q7,"✓")</f>
         <v/>
@@ -9355,11 +9462,25 @@
           <t>Acceso del profesional al historial del paciente</t>
         </is>
       </c>
+      <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr"/>
+      <c r="Q8" t="inlineStr"/>
       <c r="R8">
         <f>COUNTIF(C8:Q8,"✓")</f>
         <v/>
@@ -9376,11 +9497,25 @@
           <t>Compartir con personas sin cuenta mediante clave segura</t>
         </is>
       </c>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr"/>
+      <c r="Q9" t="inlineStr"/>
       <c r="R9">
         <f>COUNTIF(C9:Q9,"✓")</f>
         <v/>
@@ -9397,11 +9532,25 @@
           <t>Compartir datos con cuidador o persona de confianza</t>
         </is>
       </c>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr"/>
+      <c r="Q10" t="inlineStr"/>
       <c r="R10">
         <f>COUNTIF(C10:Q10,"✓")</f>
         <v/>
@@ -9423,11 +9572,13 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9453,11 +9604,16 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="P11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr"/>
       <c r="R11">
         <f>COUNTIF(C11:Q11,"✓")</f>
         <v/>
@@ -9474,11 +9630,25 @@
           <t>Gestión de consentimiento sobre uso de datos</t>
         </is>
       </c>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr"/>
+      <c r="Q12" t="inlineStr"/>
       <c r="R12">
         <f>COUNTIF(C12:Q12,"✓")</f>
         <v/>
@@ -9495,11 +9665,25 @@
           <t>Ingreso de datos por profesional con consentimiento</t>
         </is>
       </c>
+      <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr"/>
+      <c r="Q13" t="inlineStr"/>
       <c r="R13">
         <f>COUNTIF(C13:Q13,"✓")</f>
         <v/>
@@ -9516,11 +9700,25 @@
           <t>Red social con profesionales y familiares</t>
         </is>
       </c>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr"/>
+      <c r="O14" t="inlineStr"/>
+      <c r="P14" t="inlineStr"/>
+      <c r="Q14" t="inlineStr"/>
       <c r="R14">
         <f>COUNTIF(C14:Q14,"✓")</f>
         <v/>
@@ -9547,11 +9745,23 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr"/>
+      <c r="O15" t="inlineStr"/>
+      <c r="P15" t="inlineStr"/>
+      <c r="Q15" t="inlineStr"/>
       <c r="R15">
         <f>COUNTIF(C15:Q15,"✓")</f>
         <v/>
@@ -9568,6 +9778,8 @@
           <t>Perfiles familiares / dependientes</t>
         </is>
       </c>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9578,21 +9790,29 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr"/>
       <c r="N16" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="Q16" t="inlineStr"/>
       <c r="R16">
         <f>COUNTIF(C16:Q16,"✓")</f>
         <v/>
@@ -9614,6 +9834,8 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9629,11 +9851,19 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="inlineStr"/>
       <c r="O17" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="P17" t="inlineStr"/>
+      <c r="Q17" t="inlineStr"/>
       <c r="R17">
         <f>COUNTIF(C17:Q17,"✓")</f>
         <v/>
@@ -9650,16 +9880,29 @@
           <t>Almacenamiento de recetas</t>
         </is>
       </c>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr"/>
       <c r="N18" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="O18" t="inlineStr"/>
+      <c r="P18" t="inlineStr"/>
+      <c r="Q18" t="inlineStr"/>
       <c r="R18">
         <f>COUNTIF(C18:Q18,"✓")</f>
         <v/>
@@ -9676,11 +9919,25 @@
           <t>Búsqueda y filtros de documentos</t>
         </is>
       </c>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="inlineStr"/>
+      <c r="O19" t="inlineStr"/>
+      <c r="P19" t="inlineStr"/>
+      <c r="Q19" t="inlineStr"/>
       <c r="R19">
         <f>COUNTIF(C19:Q19,"✓")</f>
         <v/>
@@ -9697,11 +9954,25 @@
           <t>Emisión de certificados médicos</t>
         </is>
       </c>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="inlineStr"/>
+      <c r="O20" t="inlineStr"/>
+      <c r="P20" t="inlineStr"/>
+      <c r="Q20" t="inlineStr"/>
       <c r="R20">
         <f>COUNTIF(C20:Q20,"✓")</f>
         <v/>
@@ -9723,6 +9994,19 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="inlineStr"/>
+      <c r="O21" t="inlineStr"/>
+      <c r="P21" t="inlineStr"/>
       <c r="Q21" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9744,11 +10028,25 @@
           <t>Notificación y envío de resultados</t>
         </is>
       </c>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr"/>
       <c r="N22" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="O22" t="inlineStr"/>
+      <c r="P22" t="inlineStr"/>
+      <c r="Q22" t="inlineStr"/>
       <c r="R22">
         <f>COUNTIF(C22:Q22,"✓")</f>
         <v/>
@@ -9765,11 +10063,25 @@
           <t>Recepción de documentos desde terceros</t>
         </is>
       </c>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr"/>
+      <c r="N23" t="inlineStr"/>
+      <c r="O23" t="inlineStr"/>
+      <c r="P23" t="inlineStr"/>
+      <c r="Q23" t="inlineStr"/>
       <c r="R23">
         <f>COUNTIF(C23:Q23,"✓")</f>
         <v/>
@@ -9786,16 +10098,29 @@
           <t>Historial institucional (solo datos de la propia red)</t>
         </is>
       </c>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="inlineStr"/>
       <c r="N24" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="O24" t="inlineStr"/>
       <c r="P24" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="Q24" t="inlineStr"/>
       <c r="R24">
         <f>COUNTIF(C24:Q24,"✓")</f>
         <v/>
@@ -9812,26 +10137,36 @@
           <t>Historial médico centralizado</t>
         </is>
       </c>
+      <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" t="inlineStr"/>
+      <c r="O25" t="inlineStr"/>
+      <c r="P25" t="inlineStr"/>
       <c r="Q25" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9853,11 +10188,25 @@
           <t>Línea de tiempo de salud</t>
         </is>
       </c>
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" t="inlineStr"/>
+      <c r="O26" t="inlineStr"/>
+      <c r="P26" t="inlineStr"/>
+      <c r="Q26" t="inlineStr"/>
       <c r="R26">
         <f>COUNTIF(C26:Q26,"✓")</f>
         <v/>
@@ -9874,11 +10223,25 @@
           <t>Registro de alergias y vacunas</t>
         </is>
       </c>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr"/>
+      <c r="N27" t="inlineStr"/>
+      <c r="O27" t="inlineStr"/>
+      <c r="P27" t="inlineStr"/>
+      <c r="Q27" t="inlineStr"/>
       <c r="R27">
         <f>COUNTIF(C27:Q27,"✓")</f>
         <v/>
@@ -9895,11 +10258,25 @@
           <t>Seguimiento de visitas, gastos y seguros</t>
         </is>
       </c>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr"/>
+      <c r="N28" t="inlineStr"/>
+      <c r="O28" t="inlineStr"/>
+      <c r="P28" t="inlineStr"/>
+      <c r="Q28" t="inlineStr"/>
       <c r="R28">
         <f>COUNTIF(C28:Q28,"✓")</f>
         <v/>
@@ -9916,6 +10293,11 @@
           <t>Recompensas / monetización de datos del usuario</t>
         </is>
       </c>
+      <c r="C29" t="inlineStr"/>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9931,6 +10313,13 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="K29" t="inlineStr"/>
+      <c r="L29" t="inlineStr"/>
+      <c r="M29" t="inlineStr"/>
+      <c r="N29" t="inlineStr"/>
+      <c r="O29" t="inlineStr"/>
+      <c r="P29" t="inlineStr"/>
+      <c r="Q29" t="inlineStr"/>
       <c r="R29">
         <f>COUNTIF(C29:Q29,"✓")</f>
         <v/>
@@ -9947,11 +10336,25 @@
           <t>Asistente de IA para profesionales de salud</t>
         </is>
       </c>
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="M30" t="inlineStr"/>
+      <c r="N30" t="inlineStr"/>
+      <c r="O30" t="inlineStr"/>
+      <c r="P30" t="inlineStr"/>
+      <c r="Q30" t="inlineStr"/>
       <c r="R30">
         <f>COUNTIF(C30:Q30,"✓")</f>
         <v/>
@@ -9968,11 +10371,25 @@
           <t>Coaching de salud con IA</t>
         </is>
       </c>
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr"/>
+      <c r="L31" t="inlineStr"/>
+      <c r="M31" t="inlineStr"/>
+      <c r="N31" t="inlineStr"/>
+      <c r="O31" t="inlineStr"/>
+      <c r="P31" t="inlineStr"/>
+      <c r="Q31" t="inlineStr"/>
       <c r="R31">
         <f>COUNTIF(C31:Q31,"✓")</f>
         <v/>
@@ -9989,6 +10406,15 @@
           <t>Detección de patrones en métricas de salud con IA</t>
         </is>
       </c>
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9999,6 +10425,10 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="N32" t="inlineStr"/>
+      <c r="O32" t="inlineStr"/>
+      <c r="P32" t="inlineStr"/>
+      <c r="Q32" t="inlineStr"/>
       <c r="R32">
         <f>COUNTIF(C32:Q32,"✓")</f>
         <v/>
@@ -10015,6 +10445,15 @@
           <t>Interpretación de exámenes con IA</t>
         </is>
       </c>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10025,6 +10464,9 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="N33" t="inlineStr"/>
+      <c r="O33" t="inlineStr"/>
+      <c r="P33" t="inlineStr"/>
       <c r="Q33" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10046,11 +10488,24 @@
           <t>Orientación médica con IA</t>
         </is>
       </c>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="inlineStr"/>
+      <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="M34" t="inlineStr"/>
+      <c r="N34" t="inlineStr"/>
+      <c r="O34" t="inlineStr"/>
+      <c r="P34" t="inlineStr"/>
       <c r="Q34" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10072,6 +10527,15 @@
           <t>Preparación de consultas médicas con IA</t>
         </is>
       </c>
+      <c r="C35" t="inlineStr"/>
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10082,6 +10546,10 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="N35" t="inlineStr"/>
+      <c r="O35" t="inlineStr"/>
+      <c r="P35" t="inlineStr"/>
+      <c r="Q35" t="inlineStr"/>
       <c r="R35">
         <f>COUNTIF(C35:Q35,"✓")</f>
         <v/>
@@ -10098,6 +10566,15 @@
           <t>Resumen de historial con IA</t>
         </is>
       </c>
+      <c r="C36" t="inlineStr"/>
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="inlineStr"/>
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="inlineStr"/>
+      <c r="J36" t="inlineStr"/>
+      <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10108,6 +10585,10 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="N36" t="inlineStr"/>
+      <c r="O36" t="inlineStr"/>
+      <c r="P36" t="inlineStr"/>
+      <c r="Q36" t="inlineStr"/>
       <c r="R36">
         <f>COUNTIF(C36:Q36,"✓")</f>
         <v/>
@@ -10124,11 +10605,25 @@
           <t>API para apps de terceros</t>
         </is>
       </c>
+      <c r="C37" t="inlineStr"/>
+      <c r="D37" t="inlineStr"/>
+      <c r="E37" t="inlineStr"/>
+      <c r="F37" t="inlineStr"/>
+      <c r="G37" t="inlineStr"/>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr"/>
+      <c r="J37" t="inlineStr"/>
       <c r="K37" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="L37" t="inlineStr"/>
+      <c r="M37" t="inlineStr"/>
+      <c r="N37" t="inlineStr"/>
+      <c r="O37" t="inlineStr"/>
+      <c r="P37" t="inlineStr"/>
+      <c r="Q37" t="inlineStr"/>
       <c r="R37">
         <f>COUNTIF(C37:Q37,"✓")</f>
         <v/>
@@ -10150,6 +10645,10 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="D38" t="inlineStr"/>
+      <c r="E38" t="inlineStr"/>
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10160,6 +10659,7 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="J38" t="inlineStr"/>
       <c r="K38" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10175,11 +10675,14 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="N38" t="inlineStr"/>
       <c r="O38" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="P38" t="inlineStr"/>
+      <c r="Q38" t="inlineStr"/>
       <c r="R38">
         <f>COUNTIF(C38:Q38,"✓")</f>
         <v/>
@@ -10196,11 +10699,25 @@
           <t>Analítica poblacional B2B</t>
         </is>
       </c>
+      <c r="C39" t="inlineStr"/>
+      <c r="D39" t="inlineStr"/>
+      <c r="E39" t="inlineStr"/>
+      <c r="F39" t="inlineStr"/>
+      <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="I39" t="inlineStr"/>
+      <c r="J39" t="inlineStr"/>
+      <c r="K39" t="inlineStr"/>
+      <c r="L39" t="inlineStr"/>
+      <c r="M39" t="inlineStr"/>
+      <c r="N39" t="inlineStr"/>
+      <c r="O39" t="inlineStr"/>
+      <c r="P39" t="inlineStr"/>
+      <c r="Q39" t="inlineStr"/>
       <c r="R39">
         <f>COUNTIF(C39:Q39,"✓")</f>
         <v/>
@@ -10217,6 +10734,9 @@
           <t>Disponibilidad multiplataforma (web/iOS/Android)</t>
         </is>
       </c>
+      <c r="C40" t="inlineStr"/>
+      <c r="D40" t="inlineStr"/>
+      <c r="E40" t="inlineStr"/>
       <c r="F40" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10227,11 +10747,20 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="H40" t="inlineStr"/>
+      <c r="I40" t="inlineStr"/>
+      <c r="J40" t="inlineStr"/>
+      <c r="K40" t="inlineStr"/>
+      <c r="L40" t="inlineStr"/>
+      <c r="M40" t="inlineStr"/>
+      <c r="N40" t="inlineStr"/>
       <c r="O40" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="P40" t="inlineStr"/>
+      <c r="Q40" t="inlineStr"/>
       <c r="R40">
         <f>COUNTIF(C40:Q40,"✓")</f>
         <v/>
@@ -10248,11 +10777,25 @@
           <t>Historial médico centralizado</t>
         </is>
       </c>
+      <c r="C41" t="inlineStr"/>
+      <c r="D41" t="inlineStr"/>
+      <c r="E41" t="inlineStr"/>
+      <c r="F41" t="inlineStr"/>
+      <c r="G41" t="inlineStr"/>
+      <c r="H41" t="inlineStr"/>
+      <c r="I41" t="inlineStr"/>
       <c r="J41" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="K41" t="inlineStr"/>
+      <c r="L41" t="inlineStr"/>
+      <c r="M41" t="inlineStr"/>
+      <c r="N41" t="inlineStr"/>
+      <c r="O41" t="inlineStr"/>
+      <c r="P41" t="inlineStr"/>
+      <c r="Q41" t="inlineStr"/>
       <c r="R41">
         <f>COUNTIF(C41:Q41,"✓")</f>
         <v/>
@@ -10269,11 +10812,25 @@
           <t>Importación y exportación de datos</t>
         </is>
       </c>
+      <c r="C42" t="inlineStr"/>
+      <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="F42" t="inlineStr"/>
+      <c r="G42" t="inlineStr"/>
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" t="inlineStr"/>
+      <c r="J42" t="inlineStr"/>
+      <c r="K42" t="inlineStr"/>
+      <c r="L42" t="inlineStr"/>
+      <c r="M42" t="inlineStr"/>
+      <c r="N42" t="inlineStr"/>
+      <c r="O42" t="inlineStr"/>
+      <c r="P42" t="inlineStr"/>
+      <c r="Q42" t="inlineStr"/>
       <c r="R42">
         <f>COUNTIF(C42:Q42,"✓")</f>
         <v/>
@@ -10290,11 +10847,29 @@
           <t>Integración con EHR de proveedores</t>
         </is>
       </c>
+      <c r="C43" t="inlineStr"/>
+      <c r="D43" t="inlineStr"/>
+      <c r="E43" t="inlineStr"/>
+      <c r="F43" t="inlineStr"/>
+      <c r="G43" t="inlineStr"/>
+      <c r="H43" t="inlineStr"/>
+      <c r="I43" t="inlineStr"/>
       <c r="J43" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="K43" t="inlineStr"/>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr"/>
+      <c r="N43" t="inlineStr"/>
+      <c r="O43" t="inlineStr"/>
+      <c r="P43" t="inlineStr"/>
+      <c r="Q43" t="inlineStr"/>
       <c r="R43">
         <f>COUNTIF(C43:Q43,"✓")</f>
         <v/>
@@ -10311,16 +10886,29 @@
           <t>Integración con wearables y apps de salud</t>
         </is>
       </c>
+      <c r="C44" t="inlineStr"/>
+      <c r="D44" t="inlineStr"/>
+      <c r="E44" t="inlineStr"/>
+      <c r="F44" t="inlineStr"/>
+      <c r="G44" t="inlineStr"/>
       <c r="H44" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="I44" t="inlineStr"/>
+      <c r="J44" t="inlineStr"/>
+      <c r="K44" t="inlineStr"/>
+      <c r="L44" t="inlineStr"/>
       <c r="M44" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="N44" t="inlineStr"/>
+      <c r="O44" t="inlineStr"/>
+      <c r="P44" t="inlineStr"/>
+      <c r="Q44" t="inlineStr"/>
       <c r="R44">
         <f>COUNTIF(C44:Q44,"✓")</f>
         <v/>
@@ -10337,11 +10925,25 @@
           <t>Gestión de lista de medicamentos</t>
         </is>
       </c>
+      <c r="C45" t="inlineStr"/>
+      <c r="D45" t="inlineStr"/>
+      <c r="E45" t="inlineStr"/>
+      <c r="F45" t="inlineStr"/>
+      <c r="G45" t="inlineStr"/>
+      <c r="H45" t="inlineStr"/>
+      <c r="I45" t="inlineStr"/>
+      <c r="J45" t="inlineStr"/>
       <c r="K45" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="L45" t="inlineStr"/>
+      <c r="M45" t="inlineStr"/>
+      <c r="N45" t="inlineStr"/>
+      <c r="O45" t="inlineStr"/>
+      <c r="P45" t="inlineStr"/>
+      <c r="Q45" t="inlineStr"/>
       <c r="R45">
         <f>COUNTIF(C45:Q45,"✓")</f>
         <v/>
@@ -10358,11 +10960,25 @@
           <t>Importación automática de tratamientos desde receta digital</t>
         </is>
       </c>
+      <c r="C46" t="inlineStr"/>
+      <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="F46" t="inlineStr"/>
+      <c r="G46" t="inlineStr"/>
+      <c r="H46" t="inlineStr"/>
+      <c r="I46" t="inlineStr"/>
+      <c r="J46" t="inlineStr"/>
+      <c r="K46" t="inlineStr"/>
+      <c r="L46" t="inlineStr"/>
+      <c r="M46" t="inlineStr"/>
+      <c r="N46" t="inlineStr"/>
+      <c r="O46" t="inlineStr"/>
+      <c r="P46" t="inlineStr"/>
+      <c r="Q46" t="inlineStr"/>
       <c r="R46">
         <f>COUNTIF(C46:Q46,"✓")</f>
         <v/>
@@ -10384,11 +11000,24 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="D47" t="inlineStr"/>
+      <c r="E47" t="inlineStr"/>
+      <c r="F47" t="inlineStr"/>
+      <c r="G47" t="inlineStr"/>
+      <c r="H47" t="inlineStr"/>
+      <c r="I47" t="inlineStr"/>
+      <c r="J47" t="inlineStr"/>
       <c r="K47" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="L47" t="inlineStr"/>
+      <c r="M47" t="inlineStr"/>
+      <c r="N47" t="inlineStr"/>
+      <c r="O47" t="inlineStr"/>
+      <c r="P47" t="inlineStr"/>
+      <c r="Q47" t="inlineStr"/>
       <c r="R47">
         <f>COUNTIF(C47:Q47,"✓")</f>
         <v/>
@@ -10405,11 +11034,25 @@
           <t>Registro de tomas y adherencia al tratamiento</t>
         </is>
       </c>
+      <c r="C48" t="inlineStr"/>
+      <c r="D48" t="inlineStr"/>
       <c r="E48" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="F48" t="inlineStr"/>
+      <c r="G48" t="inlineStr"/>
+      <c r="H48" t="inlineStr"/>
+      <c r="I48" t="inlineStr"/>
+      <c r="J48" t="inlineStr"/>
+      <c r="K48" t="inlineStr"/>
+      <c r="L48" t="inlineStr"/>
+      <c r="M48" t="inlineStr"/>
+      <c r="N48" t="inlineStr"/>
+      <c r="O48" t="inlineStr"/>
+      <c r="P48" t="inlineStr"/>
+      <c r="Q48" t="inlineStr"/>
       <c r="R48">
         <f>COUNTIF(C48:Q48,"✓")</f>
         <v/>
@@ -10426,11 +11069,25 @@
           <t>Comunidad de pacientes</t>
         </is>
       </c>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="inlineStr"/>
+      <c r="E49" t="inlineStr"/>
+      <c r="F49" t="inlineStr"/>
+      <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="I49" t="inlineStr"/>
+      <c r="J49" t="inlineStr"/>
+      <c r="K49" t="inlineStr"/>
+      <c r="L49" t="inlineStr"/>
+      <c r="M49" t="inlineStr"/>
+      <c r="N49" t="inlineStr"/>
+      <c r="O49" t="inlineStr"/>
+      <c r="P49" t="inlineStr"/>
+      <c r="Q49" t="inlineStr"/>
       <c r="R49">
         <f>COUNTIF(C49:Q49,"✓")</f>
         <v/>
@@ -10447,11 +11104,25 @@
           <t>Contenido educativo sobre salud</t>
         </is>
       </c>
+      <c r="C50" t="inlineStr"/>
       <c r="D50" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="E50" t="inlineStr"/>
+      <c r="F50" t="inlineStr"/>
+      <c r="G50" t="inlineStr"/>
+      <c r="H50" t="inlineStr"/>
+      <c r="I50" t="inlineStr"/>
+      <c r="J50" t="inlineStr"/>
+      <c r="K50" t="inlineStr"/>
+      <c r="L50" t="inlineStr"/>
+      <c r="M50" t="inlineStr"/>
+      <c r="N50" t="inlineStr"/>
+      <c r="O50" t="inlineStr"/>
+      <c r="P50" t="inlineStr"/>
+      <c r="Q50" t="inlineStr"/>
       <c r="R50">
         <f>COUNTIF(C50:Q50,"✓")</f>
         <v/>
@@ -10468,11 +11139,25 @@
           <t>Gráficas de evolución de indicadores</t>
         </is>
       </c>
+      <c r="C51" t="inlineStr"/>
+      <c r="D51" t="inlineStr"/>
       <c r="E51" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="F51" t="inlineStr"/>
+      <c r="G51" t="inlineStr"/>
+      <c r="H51" t="inlineStr"/>
+      <c r="I51" t="inlineStr"/>
+      <c r="J51" t="inlineStr"/>
+      <c r="K51" t="inlineStr"/>
+      <c r="L51" t="inlineStr"/>
+      <c r="M51" t="inlineStr"/>
+      <c r="N51" t="inlineStr"/>
+      <c r="O51" t="inlineStr"/>
+      <c r="P51" t="inlineStr"/>
+      <c r="Q51" t="inlineStr"/>
       <c r="R51">
         <f>COUNTIF(C51:Q51,"✓")</f>
         <v/>
@@ -10489,11 +11174,25 @@
           <t>Integración con wearables y apps de salud</t>
         </is>
       </c>
+      <c r="C52" t="inlineStr"/>
+      <c r="D52" t="inlineStr"/>
+      <c r="E52" t="inlineStr"/>
+      <c r="F52" t="inlineStr"/>
+      <c r="G52" t="inlineStr"/>
+      <c r="H52" t="inlineStr"/>
+      <c r="I52" t="inlineStr"/>
+      <c r="J52" t="inlineStr"/>
       <c r="K52" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="L52" t="inlineStr"/>
+      <c r="M52" t="inlineStr"/>
+      <c r="N52" t="inlineStr"/>
+      <c r="O52" t="inlineStr"/>
+      <c r="P52" t="inlineStr"/>
+      <c r="Q52" t="inlineStr"/>
       <c r="R52">
         <f>COUNTIF(C52:Q52,"✓")</f>
         <v/>
@@ -10510,6 +11209,11 @@
           <t>Panel de seguimiento de salud y bienestar</t>
         </is>
       </c>
+      <c r="C53" t="inlineStr"/>
+      <c r="D53" t="inlineStr"/>
+      <c r="E53" t="inlineStr"/>
+      <c r="F53" t="inlineStr"/>
+      <c r="G53" t="inlineStr"/>
       <c r="H53" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10520,6 +11224,14 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="J53" t="inlineStr"/>
+      <c r="K53" t="inlineStr"/>
+      <c r="L53" t="inlineStr"/>
+      <c r="M53" t="inlineStr"/>
+      <c r="N53" t="inlineStr"/>
+      <c r="O53" t="inlineStr"/>
+      <c r="P53" t="inlineStr"/>
+      <c r="Q53" t="inlineStr"/>
       <c r="R53">
         <f>COUNTIF(C53:Q53,"✓")</f>
         <v/>
@@ -10536,11 +11248,25 @@
           <t>Registro de nutrición</t>
         </is>
       </c>
+      <c r="C54" t="inlineStr"/>
+      <c r="D54" t="inlineStr"/>
+      <c r="E54" t="inlineStr"/>
+      <c r="F54" t="inlineStr"/>
+      <c r="G54" t="inlineStr"/>
+      <c r="H54" t="inlineStr"/>
+      <c r="I54" t="inlineStr"/>
+      <c r="J54" t="inlineStr"/>
       <c r="K54" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="L54" t="inlineStr"/>
+      <c r="M54" t="inlineStr"/>
+      <c r="N54" t="inlineStr"/>
+      <c r="O54" t="inlineStr"/>
+      <c r="P54" t="inlineStr"/>
+      <c r="Q54" t="inlineStr"/>
       <c r="R54">
         <f>COUNTIF(C54:Q54,"✓")</f>
         <v/>
@@ -10557,11 +11283,25 @@
           <t>Seguimiento de salud femenina</t>
         </is>
       </c>
+      <c r="C55" t="inlineStr"/>
+      <c r="D55" t="inlineStr"/>
+      <c r="E55" t="inlineStr"/>
+      <c r="F55" t="inlineStr"/>
+      <c r="G55" t="inlineStr"/>
+      <c r="H55" t="inlineStr"/>
+      <c r="I55" t="inlineStr"/>
+      <c r="J55" t="inlineStr"/>
       <c r="K55" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="L55" t="inlineStr"/>
+      <c r="M55" t="inlineStr"/>
+      <c r="N55" t="inlineStr"/>
+      <c r="O55" t="inlineStr"/>
+      <c r="P55" t="inlineStr"/>
+      <c r="Q55" t="inlineStr"/>
       <c r="R55">
         <f>COUNTIF(C55:Q55,"✓")</f>
         <v/>
@@ -10578,11 +11318,25 @@
           <t>Valoración de profesionales</t>
         </is>
       </c>
+      <c r="C56" t="inlineStr"/>
+      <c r="D56" t="inlineStr"/>
+      <c r="E56" t="inlineStr"/>
       <c r="F56" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="G56" t="inlineStr"/>
+      <c r="H56" t="inlineStr"/>
+      <c r="I56" t="inlineStr"/>
+      <c r="J56" t="inlineStr"/>
+      <c r="K56" t="inlineStr"/>
+      <c r="L56" t="inlineStr"/>
+      <c r="M56" t="inlineStr"/>
+      <c r="N56" t="inlineStr"/>
+      <c r="O56" t="inlineStr"/>
+      <c r="P56" t="inlineStr"/>
+      <c r="Q56" t="inlineStr"/>
       <c r="R56">
         <f>COUNTIF(C56:Q56,"✓")</f>
         <v/>
@@ -10599,11 +11353,25 @@
           <t>Acceso mínimo por categorías de datos</t>
         </is>
       </c>
+      <c r="C57" t="inlineStr"/>
+      <c r="D57" t="inlineStr"/>
+      <c r="E57" t="inlineStr"/>
+      <c r="F57" t="inlineStr"/>
+      <c r="G57" t="inlineStr"/>
+      <c r="H57" t="inlineStr"/>
+      <c r="I57" t="inlineStr"/>
+      <c r="J57" t="inlineStr"/>
+      <c r="K57" t="inlineStr"/>
+      <c r="L57" t="inlineStr"/>
       <c r="M57" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="N57" t="inlineStr"/>
+      <c r="O57" t="inlineStr"/>
+      <c r="P57" t="inlineStr"/>
+      <c r="Q57" t="inlineStr"/>
       <c r="R57">
         <f>COUNTIF(C57:Q57,"✓")</f>
         <v/>
@@ -10620,6 +11388,11 @@
           <t>Blockchain para integridad y trazabilidad de datos</t>
         </is>
       </c>
+      <c r="C58" t="inlineStr"/>
+      <c r="D58" t="inlineStr"/>
+      <c r="E58" t="inlineStr"/>
+      <c r="F58" t="inlineStr"/>
+      <c r="G58" t="inlineStr"/>
       <c r="H58" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10635,6 +11408,13 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="K58" t="inlineStr"/>
+      <c r="L58" t="inlineStr"/>
+      <c r="M58" t="inlineStr"/>
+      <c r="N58" t="inlineStr"/>
+      <c r="O58" t="inlineStr"/>
+      <c r="P58" t="inlineStr"/>
+      <c r="Q58" t="inlineStr"/>
       <c r="R58">
         <f>COUNTIF(C58:Q58,"✓")</f>
         <v/>
@@ -10651,16 +11431,29 @@
           <t>Cifrado y control de acceso</t>
         </is>
       </c>
+      <c r="C59" t="inlineStr"/>
       <c r="D59" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="E59" t="inlineStr"/>
+      <c r="F59" t="inlineStr"/>
+      <c r="G59" t="inlineStr"/>
+      <c r="H59" t="inlineStr"/>
+      <c r="I59" t="inlineStr"/>
+      <c r="J59" t="inlineStr"/>
       <c r="K59" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="L59" t="inlineStr"/>
+      <c r="M59" t="inlineStr"/>
+      <c r="N59" t="inlineStr"/>
+      <c r="O59" t="inlineStr"/>
+      <c r="P59" t="inlineStr"/>
+      <c r="Q59" t="inlineStr"/>
       <c r="R59">
         <f>COUNTIF(C59:Q59,"✓")</f>
         <v/>
@@ -10677,11 +11470,25 @@
           <t>Cumplimiento regulatorio de salud y datos</t>
         </is>
       </c>
+      <c r="C60" t="inlineStr"/>
+      <c r="D60" t="inlineStr"/>
+      <c r="E60" t="inlineStr"/>
+      <c r="F60" t="inlineStr"/>
+      <c r="G60" t="inlineStr"/>
+      <c r="H60" t="inlineStr"/>
+      <c r="I60" t="inlineStr"/>
+      <c r="J60" t="inlineStr"/>
+      <c r="K60" t="inlineStr"/>
+      <c r="L60" t="inlineStr"/>
+      <c r="M60" t="inlineStr"/>
+      <c r="N60" t="inlineStr"/>
       <c r="O60" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="P60" t="inlineStr"/>
+      <c r="Q60" t="inlineStr"/>
       <c r="R60">
         <f>COUNTIF(C60:Q60,"✓")</f>
         <v/>
@@ -10698,11 +11505,25 @@
           <t>Gestión de consentimiento sobre uso de datos</t>
         </is>
       </c>
+      <c r="C61" t="inlineStr"/>
+      <c r="D61" t="inlineStr"/>
+      <c r="E61" t="inlineStr"/>
+      <c r="F61" t="inlineStr"/>
+      <c r="G61" t="inlineStr"/>
+      <c r="H61" t="inlineStr"/>
+      <c r="I61" t="inlineStr"/>
+      <c r="J61" t="inlineStr"/>
+      <c r="K61" t="inlineStr"/>
       <c r="L61" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="M61" t="inlineStr"/>
+      <c r="N61" t="inlineStr"/>
+      <c r="O61" t="inlineStr"/>
+      <c r="P61" t="inlineStr"/>
+      <c r="Q61" t="inlineStr"/>
       <c r="R61">
         <f>COUNTIF(C61:Q61,"✓")</f>
         <v/>
@@ -10719,11 +11540,25 @@
           <t>Identidad descentralizada (DID)</t>
         </is>
       </c>
+      <c r="C62" t="inlineStr"/>
+      <c r="D62" t="inlineStr"/>
+      <c r="E62" t="inlineStr"/>
+      <c r="F62" t="inlineStr"/>
+      <c r="G62" t="inlineStr"/>
+      <c r="H62" t="inlineStr"/>
       <c r="I62" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="J62" t="inlineStr"/>
+      <c r="K62" t="inlineStr"/>
+      <c r="L62" t="inlineStr"/>
+      <c r="M62" t="inlineStr"/>
+      <c r="N62" t="inlineStr"/>
+      <c r="O62" t="inlineStr"/>
+      <c r="P62" t="inlineStr"/>
+      <c r="Q62" t="inlineStr"/>
       <c r="R62">
         <f>COUNTIF(C62:Q62,"✓")</f>
         <v/>
@@ -10740,6 +11575,15 @@
           <t>Privacidad reforzada para datos de salud</t>
         </is>
       </c>
+      <c r="C63" t="inlineStr"/>
+      <c r="D63" t="inlineStr"/>
+      <c r="E63" t="inlineStr"/>
+      <c r="F63" t="inlineStr"/>
+      <c r="G63" t="inlineStr"/>
+      <c r="H63" t="inlineStr"/>
+      <c r="I63" t="inlineStr"/>
+      <c r="J63" t="inlineStr"/>
+      <c r="K63" t="inlineStr"/>
       <c r="L63" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10750,6 +11594,10 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="N63" t="inlineStr"/>
+      <c r="O63" t="inlineStr"/>
+      <c r="P63" t="inlineStr"/>
+      <c r="Q63" t="inlineStr"/>
       <c r="R63">
         <f>COUNTIF(C63:Q63,"✓")</f>
         <v/>
@@ -10766,6 +11614,20 @@
           <t>Modelo freemium y suscripción</t>
         </is>
       </c>
+      <c r="C64" t="inlineStr"/>
+      <c r="D64" t="inlineStr"/>
+      <c r="E64" t="inlineStr"/>
+      <c r="F64" t="inlineStr"/>
+      <c r="G64" t="inlineStr"/>
+      <c r="H64" t="inlineStr"/>
+      <c r="I64" t="inlineStr"/>
+      <c r="J64" t="inlineStr"/>
+      <c r="K64" t="inlineStr"/>
+      <c r="L64" t="inlineStr"/>
+      <c r="M64" t="inlineStr"/>
+      <c r="N64" t="inlineStr"/>
+      <c r="O64" t="inlineStr"/>
+      <c r="P64" t="inlineStr"/>
       <c r="Q64" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10787,11 +11649,25 @@
           <t>Pagos con criptomoneda</t>
         </is>
       </c>
+      <c r="C65" t="inlineStr"/>
+      <c r="D65" t="inlineStr"/>
+      <c r="E65" t="inlineStr"/>
+      <c r="F65" t="inlineStr"/>
+      <c r="G65" t="inlineStr"/>
+      <c r="H65" t="inlineStr"/>
+      <c r="I65" t="inlineStr"/>
       <c r="J65" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="K65" t="inlineStr"/>
+      <c r="L65" t="inlineStr"/>
+      <c r="M65" t="inlineStr"/>
+      <c r="N65" t="inlineStr"/>
+      <c r="O65" t="inlineStr"/>
+      <c r="P65" t="inlineStr"/>
+      <c r="Q65" t="inlineStr"/>
       <c r="R65">
         <f>COUNTIF(C65:Q65,"✓")</f>
         <v/>
@@ -10808,11 +11684,24 @@
           <t>Pagos dentro de la app</t>
         </is>
       </c>
+      <c r="C66" t="inlineStr"/>
+      <c r="D66" t="inlineStr"/>
+      <c r="E66" t="inlineStr"/>
+      <c r="F66" t="inlineStr"/>
+      <c r="G66" t="inlineStr"/>
+      <c r="H66" t="inlineStr"/>
+      <c r="I66" t="inlineStr"/>
+      <c r="J66" t="inlineStr"/>
+      <c r="K66" t="inlineStr"/>
+      <c r="L66" t="inlineStr"/>
+      <c r="M66" t="inlineStr"/>
       <c r="N66" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="O66" t="inlineStr"/>
+      <c r="P66" t="inlineStr"/>
       <c r="Q66" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10834,11 +11723,25 @@
           <t>Reclamos y trámites con seguros</t>
         </is>
       </c>
+      <c r="C67" t="inlineStr"/>
+      <c r="D67" t="inlineStr"/>
+      <c r="E67" t="inlineStr"/>
+      <c r="F67" t="inlineStr"/>
+      <c r="G67" t="inlineStr"/>
+      <c r="H67" t="inlineStr"/>
       <c r="I67" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="J67" t="inlineStr"/>
+      <c r="K67" t="inlineStr"/>
+      <c r="L67" t="inlineStr"/>
+      <c r="M67" t="inlineStr"/>
+      <c r="N67" t="inlineStr"/>
+      <c r="O67" t="inlineStr"/>
+      <c r="P67" t="inlineStr"/>
+      <c r="Q67" t="inlineStr"/>
       <c r="R67">
         <f>COUNTIF(C67:Q67,"✓")</f>
         <v/>
@@ -10855,11 +11758,25 @@
           <t>Mensajería paciente-institución</t>
         </is>
       </c>
+      <c r="C68" t="inlineStr"/>
+      <c r="D68" t="inlineStr"/>
+      <c r="E68" t="inlineStr"/>
+      <c r="F68" t="inlineStr"/>
+      <c r="G68" t="inlineStr"/>
+      <c r="H68" t="inlineStr"/>
       <c r="I68" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="J68" t="inlineStr"/>
+      <c r="K68" t="inlineStr"/>
+      <c r="L68" t="inlineStr"/>
+      <c r="M68" t="inlineStr"/>
+      <c r="N68" t="inlineStr"/>
+      <c r="O68" t="inlineStr"/>
+      <c r="P68" t="inlineStr"/>
+      <c r="Q68" t="inlineStr"/>
       <c r="R68">
         <f>COUNTIF(C68:Q68,"✓")</f>
         <v/>
@@ -10876,11 +11793,25 @@
           <t>Teleconsulta con profesionales</t>
         </is>
       </c>
+      <c r="C69" t="inlineStr"/>
+      <c r="D69" t="inlineStr"/>
+      <c r="E69" t="inlineStr"/>
+      <c r="F69" t="inlineStr"/>
+      <c r="G69" t="inlineStr"/>
+      <c r="H69" t="inlineStr"/>
+      <c r="I69" t="inlineStr"/>
       <c r="J69" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
+      <c r="K69" t="inlineStr"/>
+      <c r="L69" t="inlineStr"/>
+      <c r="M69" t="inlineStr"/>
+      <c r="N69" t="inlineStr"/>
+      <c r="O69" t="inlineStr"/>
+      <c r="P69" t="inlineStr"/>
+      <c r="Q69" t="inlineStr"/>
       <c r="R69">
         <f>COUNTIF(C69:Q69,"✓")</f>
         <v/>
@@ -10897,7 +11828,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A43"/>
+  <dimension ref="A1:A44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -11204,6 +12135,13 @@
         </is>
       </c>
     </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>VUELTA 9 COMPLETA (2026-10-28 12:21 UTC): Clinia, MiRedSalud y Mediko revisados sin búsqueda nueva (saturado). Contador de loops = 9 para todos, Revisado reiniciado a "No". func_norm (134 filas) y tabla_frecuencia (68 funcionalidades) regenerados. Vuelta 10 parte con Meedika, Infomed, MediPlanner, Clingot. Candidatos sin agregar: HealthChain (Chile), Medicyn (global), DKV Quiero cuidarme Más (España).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Benchmark: vuelta 10, iteración 1 (Meedika, Infomed, MediPlanner, Clingot)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MVcXu8vTBu7EKfj3YdEvae
</commit_message>
<xml_diff>
--- a/Outputs/Benchmark_Anamnesis.xlsx
+++ b/Outputs/Benchmark_Anamnesis.xlsx
@@ -513,12 +513,12 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>[DIRECTO · Chile · etapas A+B] Lanzada 25-sep-2024 en App Store (Android previsto la misma semana). &gt;1.500 usuarios en los primeros días; meta 32.000 (cofundador Francisco González). Funciones: gestión de documentos, importar solicitudes, SOS con alergias/medicación, calendario de citas, recordatorios, compartir con profesionales elegidos. Sin blockchain. Precio y estado actual NO verificados; única fuente es una nota de prensa. Sitio oficial por confirmar. [Iter. 2] Hay cobertura adicional en Portal Innova (portalinnova.cl); sitio bloqueado en este entorno, estado actual sigue sin verificar. [Vuelta 3] Sin novedades 2026 ni confirmación de la app Android en Google Play; usuarios actuales desconocidos. Nota de prensa no indica año de lanzamiento explícito. [Vuelta 4] Sin fuentes nuevas; portalinnova.cl no aparece en búsquedas. Sigue dependiendo de una sola nota de prensa. [Vuelta 5] Sin fuentes nuevas (ni entrevistas ni financiamiento); sigue dependiendo de una sola nota de prensa sin año explícito. [Vuelta 6] Sin ficha de Google Play ni fuentes nuevas; disponibilidad en Android sin confirmar. [Vuelta 7] Sin fuentes nuevas; no hay ficha oficial localizada. No confundir con apps de nombre parecido (Medika App, MEDDI, AI Medik). [Vuelta 8] Sin fuentes nuevas. [Vuelta 9] Sin fuentes nuevas.</t>
+          <t>[DIRECTO · Chile · etapas A+B] Lanzada 25-sep-2024 en App Store (Android previsto la misma semana). &gt;1.500 usuarios en los primeros días; meta 32.000 (cofundador Francisco González). Funciones: gestión de documentos, importar solicitudes, SOS con alergias/medicación, calendario de citas, recordatorios, compartir con profesionales elegidos. Sin blockchain. Precio y estado actual NO verificados; única fuente es una nota de prensa. Sitio oficial por confirmar. [Iter. 2] Hay cobertura adicional en Portal Innova (portalinnova.cl); sitio bloqueado en este entorno, estado actual sigue sin verificar. [Vuelta 3] Sin novedades 2026 ni confirmación de la app Android en Google Play; usuarios actuales desconocidos. Nota de prensa no indica año de lanzamiento explícito. [Vuelta 4] Sin fuentes nuevas; portalinnova.cl no aparece en búsquedas. Sigue dependiendo de una sola nota de prensa. [Vuelta 5] Sin fuentes nuevas (ni entrevistas ni financiamiento); sigue dependiendo de una sola nota de prensa sin año explícito. [Vuelta 6] Sin ficha de Google Play ni fuentes nuevas; disponibilidad en Android sin confirmar. [Vuelta 7] Sin fuentes nuevas; no hay ficha oficial localizada. No confundir con apps de nombre parecido (Medika App, MEDDI, AI Medik). [Vuelta 8] Sin fuentes nuevas. [Vuelta 9] Sin fuentes nuevas. [Vuelta 10] Sin novedades.</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G2" t="n">
@@ -526,7 +526,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
     </row>
@@ -553,12 +553,12 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>[DIRECTO · Chile · etapa A] Fundada 2019 por Diego Ibarra, Andrés Fantuzzi y Gabriel Zamora. Lanzada mar-2021 en App Store y Play Store con 1.200 usuarios; planeaba nueva versión jul-2021 y ronda de US$500 mil. Objetivo: llevar el historial en el celular, acceso en emergencias, médico puede ingresar datos con consentimiento. Estado actual NO verificado (posible app inactiva). URL es la nota de prensa; sitio oficial por confirmar. [Vuelta 3] Sin evidencia posterior a 2021; relanzamiento previsto jul-2021 no confirmado. Probable app inactiva. [Vuelta 4] Sin cambios; sigue sin evidencia posterior a 2021. [Vuelta 5] Cofundador Andrés Fantuzzi es cardiólogo de la Clínica Santa María. Sin ronda de inversión ni relanzamiento confirmados; no confundir con Infomed de Cuba (portal del Minsap). [Vuelta 6] Sin búsqueda nueva (fuentes agotadas en vueltas 3-5); sin cambios. [Vuelta 7] Sin búsqueda nueva (saturado); sin cambios. [Vuelta 8] Sin fuentes nuevas; relanzamiento de jul-2021 sigue sin confirmarse. [Vuelta 9] Sin fuentes nuevas.</t>
+          <t>[DIRECTO · Chile · etapa A] Fundada 2019 por Diego Ibarra, Andrés Fantuzzi y Gabriel Zamora. Lanzada mar-2021 en App Store y Play Store con 1.200 usuarios; planeaba nueva versión jul-2021 y ronda de US$500 mil. Objetivo: llevar el historial en el celular, acceso en emergencias, médico puede ingresar datos con consentimiento. Estado actual NO verificado (posible app inactiva). URL es la nota de prensa; sitio oficial por confirmar. [Vuelta 3] Sin evidencia posterior a 2021; relanzamiento previsto jul-2021 no confirmado. Probable app inactiva. [Vuelta 4] Sin cambios; sigue sin evidencia posterior a 2021. [Vuelta 5] Cofundador Andrés Fantuzzi es cardiólogo de la Clínica Santa María. Sin ronda de inversión ni relanzamiento confirmados; no confundir con Infomed de Cuba (portal del Minsap). [Vuelta 6] Sin búsqueda nueva (fuentes agotadas en vueltas 3-5); sin cambios. [Vuelta 7] Sin búsqueda nueva (saturado); sin cambios. [Vuelta 8] Sin fuentes nuevas; relanzamiento de jul-2021 sigue sin confirmarse. [Vuelta 9] Sin fuentes nuevas. [Vuelta 10] Sin novedades; relanzamiento de jul-2021 sigue sin confirmarse.</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G3" t="n">
@@ -566,7 +566,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
     </row>
@@ -593,12 +593,12 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>[REGIONAL · México] Historial por perfil familiar, alergias, vacunas, recetas digitales, gráficas de evolución, agendamiento, compartir con profesionales. Gratis en App Store MX. Sin evidencia de uso en Chile. Cubre parte de la etapa C (familia). [Vuelta 3] Existen dos apps distintas: MediPlanner (gratis, Rym Solutions, MX, 3,7/5 con 3 calificaciones) y MediPlanner Pro (otro desarrollador, $39 MXN). Sin presencia verificada en Chile. [Vuelta 4] No pude confirmar el desarrollador de la versión gratuita (Rym Solutions no se repite en esta búsqueda). MediPlanner Pro (fichas BR/OM) guardaría datos solo en el dispositivo, sin nube; no confundir con MedPlanner/AskHEMI (otra empresa). [Vuelta 5] Sin búsqueda nueva (revisada en vuelta 4); sin cambios. [Vuelta 6] Se reconfirma en la ficha de App Store MX que el desarrollador de la versión gratuita es Rym Solutions S. de R.L. de C.V. (3,7/5, 3 calificaciones); MediPlanner Pro no menciona a esa empresa, por lo que no se puede asegurar que sea el mismo desarrollador. [Vuelta 7] Sin búsqueda nueva (saturado); sin cambios. [Vuelta 8] Sin búsqueda nueva (saturado). [Vuelta 9] Sin fuentes nuevas.</t>
+          <t>[REGIONAL · México] Historial por perfil familiar, alergias, vacunas, recetas digitales, gráficas de evolución, agendamiento, compartir con profesionales. Gratis en App Store MX. Sin evidencia de uso en Chile. Cubre parte de la etapa C (familia). [Vuelta 3] Existen dos apps distintas: MediPlanner (gratis, Rym Solutions, MX, 3,7/5 con 3 calificaciones) y MediPlanner Pro (otro desarrollador, $39 MXN). Sin presencia verificada en Chile. [Vuelta 4] No pude confirmar el desarrollador de la versión gratuita (Rym Solutions no se repite en esta búsqueda). MediPlanner Pro (fichas BR/OM) guardaría datos solo en el dispositivo, sin nube; no confundir con MedPlanner/AskHEMI (otra empresa). [Vuelta 5] Sin búsqueda nueva (revisada en vuelta 4); sin cambios. [Vuelta 6] Se reconfirma en la ficha de App Store MX que el desarrollador de la versión gratuita es Rym Solutions S. de R.L. de C.V. (3,7/5, 3 calificaciones); MediPlanner Pro no menciona a esa empresa, por lo que no se puede asegurar que sea el mismo desarrollador. [Vuelta 7] Sin búsqueda nueva (saturado); sin cambios. [Vuelta 8] Sin búsqueda nueva (saturado). [Vuelta 9] Sin fuentes nuevas. [Vuelta 10] Sin búsqueda nueva (saturado).</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G4" t="n">
@@ -606,7 +606,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
     </row>
@@ -633,12 +633,12 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>[REGIONAL · Argentina · débil] App para cargar antecedentes médicos propios. Única referencia: nota de opinión en grupoanimal.mx sin fecha verificada. Estado y sitio por confirmar. [Vuelta 3] Referencias de 2017 (apps4citizens, La Nación); sitio y precio no verificados; puede estar inactiva. [Vuelta 4] Sin fuentes nuevas. [Vuelta 5] Registro empresarial (indicadores.ar, datos a jul-2026) muestra CLINGOT S.A. activa en CABA, constituida el 4-abr-2016; no confirma que la app siga operando. Programa federal argentino de historias clínicas digitales como contexto regulatorio. [Vuelta 6] Sin búsqueda nueva (fuentes agotadas); sin cambios. [Vuelta 7] Solo fuentes de 2017; sin evidencia nueva de operación más allá del registro societario. [Vuelta 8] Sin fuentes nuevas. [Vuelta 9] Sin fuentes nuevas.</t>
+          <t>[REGIONAL · Argentina · débil] App para cargar antecedentes médicos propios. Única referencia: nota de opinión en grupoanimal.mx sin fecha verificada. Estado y sitio por confirmar. [Vuelta 3] Referencias de 2017 (apps4citizens, La Nación); sitio y precio no verificados; puede estar inactiva. [Vuelta 4] Sin fuentes nuevas. [Vuelta 5] Registro empresarial (indicadores.ar, datos a jul-2026) muestra CLINGOT S.A. activa en CABA, constituida el 4-abr-2016; no confirma que la app siga operando. Programa federal argentino de historias clínicas digitales como contexto regulatorio. [Vuelta 6] Sin búsqueda nueva (fuentes agotadas); sin cambios. [Vuelta 7] Solo fuentes de 2017; sin evidencia nueva de operación más allá del registro societario. [Vuelta 8] Sin fuentes nuevas. [Vuelta 9] Sin fuentes nuevas. [Vuelta 10] Sin búsqueda nueva (saturado).</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G5" t="n">
@@ -646,7 +646,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
     </row>
@@ -9236,8 +9236,6 @@
           <t>Búsqueda de profesionales de salud</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9248,17 +9246,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
       <c r="R2">
         <f>COUNTIF(C2:Q2,"✓")</f>
         <v/>
@@ -9280,24 +9267,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
       <c r="R3">
         <f>COUNTIF(C3:Q3,"✓")</f>
         <v/>
@@ -9314,25 +9288,11 @@
           <t>Check-in de admisión digital</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
       <c r="R4">
         <f>COUNTIF(C4:Q4,"✓")</f>
         <v/>
@@ -9349,25 +9309,11 @@
           <t>Integración con calendario del dispositivo</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr"/>
       <c r="R5">
         <f>COUNTIF(C5:Q5,"✓")</f>
         <v/>
@@ -9384,25 +9330,11 @@
           <t>Localización de centros médicos y farmacias</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="inlineStr"/>
       <c r="R6">
         <f>COUNTIF(C6:Q6,"✓")</f>
         <v/>
@@ -9419,21 +9351,11 @@
           <t>Reserva de citas médicas</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9444,8 +9366,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="P7" t="inlineStr"/>
-      <c r="Q7" t="inlineStr"/>
       <c r="R7">
         <f>COUNTIF(C7:Q7,"✓")</f>
         <v/>
@@ -9462,25 +9382,11 @@
           <t>Acceso del profesional al historial del paciente</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
-      <c r="P8" t="inlineStr"/>
-      <c r="Q8" t="inlineStr"/>
       <c r="R8">
         <f>COUNTIF(C8:Q8,"✓")</f>
         <v/>
@@ -9497,25 +9403,11 @@
           <t>Compartir con personas sin cuenta mediante clave segura</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
-      <c r="P9" t="inlineStr"/>
-      <c r="Q9" t="inlineStr"/>
       <c r="R9">
         <f>COUNTIF(C9:Q9,"✓")</f>
         <v/>
@@ -9532,25 +9424,11 @@
           <t>Compartir datos con cuidador o persona de confianza</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
-      <c r="O10" t="inlineStr"/>
-      <c r="P10" t="inlineStr"/>
-      <c r="Q10" t="inlineStr"/>
       <c r="R10">
         <f>COUNTIF(C10:Q10,"✓")</f>
         <v/>
@@ -9572,13 +9450,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9604,16 +9480,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="P11" t="inlineStr"/>
-      <c r="Q11" t="inlineStr"/>
       <c r="R11">
         <f>COUNTIF(C11:Q11,"✓")</f>
         <v/>
@@ -9630,25 +9501,11 @@
           <t>Gestión de consentimiento sobre uso de datos</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
-      <c r="O12" t="inlineStr"/>
-      <c r="P12" t="inlineStr"/>
-      <c r="Q12" t="inlineStr"/>
       <c r="R12">
         <f>COUNTIF(C12:Q12,"✓")</f>
         <v/>
@@ -9665,25 +9522,11 @@
           <t>Ingreso de datos por profesional con consentimiento</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr"/>
-      <c r="O13" t="inlineStr"/>
-      <c r="P13" t="inlineStr"/>
-      <c r="Q13" t="inlineStr"/>
       <c r="R13">
         <f>COUNTIF(C13:Q13,"✓")</f>
         <v/>
@@ -9700,25 +9543,11 @@
           <t>Red social con profesionales y familiares</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
-      <c r="M14" t="inlineStr"/>
-      <c r="N14" t="inlineStr"/>
-      <c r="O14" t="inlineStr"/>
-      <c r="P14" t="inlineStr"/>
-      <c r="Q14" t="inlineStr"/>
       <c r="R14">
         <f>COUNTIF(C14:Q14,"✓")</f>
         <v/>
@@ -9745,23 +9574,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr"/>
-      <c r="N15" t="inlineStr"/>
-      <c r="O15" t="inlineStr"/>
-      <c r="P15" t="inlineStr"/>
-      <c r="Q15" t="inlineStr"/>
       <c r="R15">
         <f>COUNTIF(C15:Q15,"✓")</f>
         <v/>
@@ -9778,8 +9595,6 @@
           <t>Perfiles familiares / dependientes</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9790,29 +9605,21 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
-      <c r="M16" t="inlineStr"/>
       <c r="N16" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="Q16" t="inlineStr"/>
       <c r="R16">
         <f>COUNTIF(C16:Q16,"✓")</f>
         <v/>
@@ -9834,8 +9641,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
           <t>✓</t>
@@ -9851,19 +9656,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr"/>
-      <c r="N17" t="inlineStr"/>
       <c r="O17" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="P17" t="inlineStr"/>
-      <c r="Q17" t="inlineStr"/>
       <c r="R17">
         <f>COUNTIF(C17:Q17,"✓")</f>
         <v/>
@@ -9880,29 +9677,16 @@
           <t>Almacenamiento de recetas</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr"/>
-      <c r="M18" t="inlineStr"/>
       <c r="N18" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="O18" t="inlineStr"/>
-      <c r="P18" t="inlineStr"/>
-      <c r="Q18" t="inlineStr"/>
       <c r="R18">
         <f>COUNTIF(C18:Q18,"✓")</f>
         <v/>
@@ -9919,25 +9703,11 @@
           <t>Búsqueda y filtros de documentos</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr"/>
-      <c r="M19" t="inlineStr"/>
-      <c r="N19" t="inlineStr"/>
-      <c r="O19" t="inlineStr"/>
-      <c r="P19" t="inlineStr"/>
-      <c r="Q19" t="inlineStr"/>
       <c r="R19">
         <f>COUNTIF(C19:Q19,"✓")</f>
         <v/>
@@ -9954,25 +9724,11 @@
           <t>Emisión de certificados médicos</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr"/>
-      <c r="M20" t="inlineStr"/>
-      <c r="N20" t="inlineStr"/>
-      <c r="O20" t="inlineStr"/>
-      <c r="P20" t="inlineStr"/>
-      <c r="Q20" t="inlineStr"/>
       <c r="R20">
         <f>COUNTIF(C20:Q20,"✓")</f>
         <v/>
@@ -9994,19 +9750,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr"/>
-      <c r="M21" t="inlineStr"/>
-      <c r="N21" t="inlineStr"/>
-      <c r="O21" t="inlineStr"/>
-      <c r="P21" t="inlineStr"/>
       <c r="Q21" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10028,25 +9771,11 @@
           <t>Notificación y envío de resultados</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
-      <c r="L22" t="inlineStr"/>
-      <c r="M22" t="inlineStr"/>
       <c r="N22" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="O22" t="inlineStr"/>
-      <c r="P22" t="inlineStr"/>
-      <c r="Q22" t="inlineStr"/>
       <c r="R22">
         <f>COUNTIF(C22:Q22,"✓")</f>
         <v/>
@@ -10063,25 +9792,11 @@
           <t>Recepción de documentos desde terceros</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
-      <c r="L23" t="inlineStr"/>
-      <c r="M23" t="inlineStr"/>
-      <c r="N23" t="inlineStr"/>
-      <c r="O23" t="inlineStr"/>
-      <c r="P23" t="inlineStr"/>
-      <c r="Q23" t="inlineStr"/>
       <c r="R23">
         <f>COUNTIF(C23:Q23,"✓")</f>
         <v/>
@@ -10098,29 +9813,16 @@
           <t>Historial institucional (solo datos de la propia red)</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
-      <c r="L24" t="inlineStr"/>
-      <c r="M24" t="inlineStr"/>
       <c r="N24" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="O24" t="inlineStr"/>
       <c r="P24" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="Q24" t="inlineStr"/>
       <c r="R24">
         <f>COUNTIF(C24:Q24,"✓")</f>
         <v/>
@@ -10137,36 +9839,26 @@
           <t>Historial médico centralizado</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="L25" t="inlineStr"/>
-      <c r="M25" t="inlineStr"/>
-      <c r="N25" t="inlineStr"/>
-      <c r="O25" t="inlineStr"/>
-      <c r="P25" t="inlineStr"/>
       <c r="Q25" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10188,25 +9880,11 @@
           <t>Línea de tiempo de salud</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr"/>
-      <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr"/>
-      <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
-      <c r="L26" t="inlineStr"/>
-      <c r="M26" t="inlineStr"/>
-      <c r="N26" t="inlineStr"/>
-      <c r="O26" t="inlineStr"/>
-      <c r="P26" t="inlineStr"/>
-      <c r="Q26" t="inlineStr"/>
       <c r="R26">
         <f>COUNTIF(C26:Q26,"✓")</f>
         <v/>
@@ -10223,25 +9901,11 @@
           <t>Registro de alergias y vacunas</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr"/>
-      <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr"/>
-      <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
-      <c r="L27" t="inlineStr"/>
-      <c r="M27" t="inlineStr"/>
-      <c r="N27" t="inlineStr"/>
-      <c r="O27" t="inlineStr"/>
-      <c r="P27" t="inlineStr"/>
-      <c r="Q27" t="inlineStr"/>
       <c r="R27">
         <f>COUNTIF(C27:Q27,"✓")</f>
         <v/>
@@ -10258,25 +9922,11 @@
           <t>Seguimiento de visitas, gastos y seguros</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr"/>
-      <c r="M28" t="inlineStr"/>
-      <c r="N28" t="inlineStr"/>
-      <c r="O28" t="inlineStr"/>
-      <c r="P28" t="inlineStr"/>
-      <c r="Q28" t="inlineStr"/>
       <c r="R28">
         <f>COUNTIF(C28:Q28,"✓")</f>
         <v/>
@@ -10293,11 +9943,6 @@
           <t>Recompensas / monetización de datos del usuario</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr"/>
-      <c r="D29" t="inlineStr"/>
-      <c r="E29" t="inlineStr"/>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10313,13 +9958,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="K29" t="inlineStr"/>
-      <c r="L29" t="inlineStr"/>
-      <c r="M29" t="inlineStr"/>
-      <c r="N29" t="inlineStr"/>
-      <c r="O29" t="inlineStr"/>
-      <c r="P29" t="inlineStr"/>
-      <c r="Q29" t="inlineStr"/>
       <c r="R29">
         <f>COUNTIF(C29:Q29,"✓")</f>
         <v/>
@@ -10336,25 +9974,11 @@
           <t>Asistente de IA para profesionales de salud</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr"/>
-      <c r="E30" t="inlineStr"/>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr"/>
-      <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="M30" t="inlineStr"/>
-      <c r="N30" t="inlineStr"/>
-      <c r="O30" t="inlineStr"/>
-      <c r="P30" t="inlineStr"/>
-      <c r="Q30" t="inlineStr"/>
       <c r="R30">
         <f>COUNTIF(C30:Q30,"✓")</f>
         <v/>
@@ -10371,25 +9995,11 @@
           <t>Coaching de salud con IA</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr"/>
-      <c r="D31" t="inlineStr"/>
-      <c r="E31" t="inlineStr"/>
-      <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr"/>
-      <c r="L31" t="inlineStr"/>
-      <c r="M31" t="inlineStr"/>
-      <c r="N31" t="inlineStr"/>
-      <c r="O31" t="inlineStr"/>
-      <c r="P31" t="inlineStr"/>
-      <c r="Q31" t="inlineStr"/>
       <c r="R31">
         <f>COUNTIF(C31:Q31,"✓")</f>
         <v/>
@@ -10406,15 +10016,6 @@
           <t>Detección de patrones en métricas de salud con IA</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr"/>
-      <c r="D32" t="inlineStr"/>
-      <c r="E32" t="inlineStr"/>
-      <c r="F32" t="inlineStr"/>
-      <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr"/>
-      <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr"/>
-      <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10425,10 +10026,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="N32" t="inlineStr"/>
-      <c r="O32" t="inlineStr"/>
-      <c r="P32" t="inlineStr"/>
-      <c r="Q32" t="inlineStr"/>
       <c r="R32">
         <f>COUNTIF(C32:Q32,"✓")</f>
         <v/>
@@ -10445,15 +10042,6 @@
           <t>Interpretación de exámenes con IA</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr"/>
-      <c r="D33" t="inlineStr"/>
-      <c r="E33" t="inlineStr"/>
-      <c r="F33" t="inlineStr"/>
-      <c r="G33" t="inlineStr"/>
-      <c r="H33" t="inlineStr"/>
-      <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr"/>
-      <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10464,9 +10052,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="N33" t="inlineStr"/>
-      <c r="O33" t="inlineStr"/>
-      <c r="P33" t="inlineStr"/>
       <c r="Q33" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10488,24 +10073,11 @@
           <t>Orientación médica con IA</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr"/>
-      <c r="D34" t="inlineStr"/>
-      <c r="E34" t="inlineStr"/>
-      <c r="F34" t="inlineStr"/>
-      <c r="G34" t="inlineStr"/>
-      <c r="H34" t="inlineStr"/>
-      <c r="I34" t="inlineStr"/>
-      <c r="J34" t="inlineStr"/>
-      <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="M34" t="inlineStr"/>
-      <c r="N34" t="inlineStr"/>
-      <c r="O34" t="inlineStr"/>
-      <c r="P34" t="inlineStr"/>
       <c r="Q34" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10527,15 +10099,6 @@
           <t>Preparación de consultas médicas con IA</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr"/>
-      <c r="D35" t="inlineStr"/>
-      <c r="E35" t="inlineStr"/>
-      <c r="F35" t="inlineStr"/>
-      <c r="G35" t="inlineStr"/>
-      <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr"/>
-      <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10546,10 +10109,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="N35" t="inlineStr"/>
-      <c r="O35" t="inlineStr"/>
-      <c r="P35" t="inlineStr"/>
-      <c r="Q35" t="inlineStr"/>
       <c r="R35">
         <f>COUNTIF(C35:Q35,"✓")</f>
         <v/>
@@ -10566,15 +10125,6 @@
           <t>Resumen de historial con IA</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr"/>
-      <c r="D36" t="inlineStr"/>
-      <c r="E36" t="inlineStr"/>
-      <c r="F36" t="inlineStr"/>
-      <c r="G36" t="inlineStr"/>
-      <c r="H36" t="inlineStr"/>
-      <c r="I36" t="inlineStr"/>
-      <c r="J36" t="inlineStr"/>
-      <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10585,10 +10135,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="N36" t="inlineStr"/>
-      <c r="O36" t="inlineStr"/>
-      <c r="P36" t="inlineStr"/>
-      <c r="Q36" t="inlineStr"/>
       <c r="R36">
         <f>COUNTIF(C36:Q36,"✓")</f>
         <v/>
@@ -10605,25 +10151,11 @@
           <t>API para apps de terceros</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr"/>
-      <c r="D37" t="inlineStr"/>
-      <c r="E37" t="inlineStr"/>
-      <c r="F37" t="inlineStr"/>
-      <c r="G37" t="inlineStr"/>
-      <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr"/>
-      <c r="J37" t="inlineStr"/>
       <c r="K37" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="L37" t="inlineStr"/>
-      <c r="M37" t="inlineStr"/>
-      <c r="N37" t="inlineStr"/>
-      <c r="O37" t="inlineStr"/>
-      <c r="P37" t="inlineStr"/>
-      <c r="Q37" t="inlineStr"/>
       <c r="R37">
         <f>COUNTIF(C37:Q37,"✓")</f>
         <v/>
@@ -10645,10 +10177,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr"/>
-      <c r="E38" t="inlineStr"/>
-      <c r="F38" t="inlineStr"/>
-      <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10659,7 +10187,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="J38" t="inlineStr"/>
       <c r="K38" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10675,14 +10202,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="N38" t="inlineStr"/>
       <c r="O38" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="P38" t="inlineStr"/>
-      <c r="Q38" t="inlineStr"/>
       <c r="R38">
         <f>COUNTIF(C38:Q38,"✓")</f>
         <v/>
@@ -10699,25 +10223,11 @@
           <t>Analítica poblacional B2B</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr"/>
-      <c r="D39" t="inlineStr"/>
-      <c r="E39" t="inlineStr"/>
-      <c r="F39" t="inlineStr"/>
-      <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr"/>
-      <c r="J39" t="inlineStr"/>
-      <c r="K39" t="inlineStr"/>
-      <c r="L39" t="inlineStr"/>
-      <c r="M39" t="inlineStr"/>
-      <c r="N39" t="inlineStr"/>
-      <c r="O39" t="inlineStr"/>
-      <c r="P39" t="inlineStr"/>
-      <c r="Q39" t="inlineStr"/>
       <c r="R39">
         <f>COUNTIF(C39:Q39,"✓")</f>
         <v/>
@@ -10734,9 +10244,6 @@
           <t>Disponibilidad multiplataforma (web/iOS/Android)</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr"/>
-      <c r="D40" t="inlineStr"/>
-      <c r="E40" t="inlineStr"/>
       <c r="F40" t="inlineStr">
         <is>
           <t>✓</t>
@@ -10747,20 +10254,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr"/>
-      <c r="I40" t="inlineStr"/>
-      <c r="J40" t="inlineStr"/>
-      <c r="K40" t="inlineStr"/>
-      <c r="L40" t="inlineStr"/>
-      <c r="M40" t="inlineStr"/>
-      <c r="N40" t="inlineStr"/>
       <c r="O40" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="P40" t="inlineStr"/>
-      <c r="Q40" t="inlineStr"/>
       <c r="R40">
         <f>COUNTIF(C40:Q40,"✓")</f>
         <v/>
@@ -10777,25 +10275,11 @@
           <t>Historial médico centralizado</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr"/>
-      <c r="D41" t="inlineStr"/>
-      <c r="E41" t="inlineStr"/>
-      <c r="F41" t="inlineStr"/>
-      <c r="G41" t="inlineStr"/>
-      <c r="H41" t="inlineStr"/>
-      <c r="I41" t="inlineStr"/>
       <c r="J41" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="K41" t="inlineStr"/>
-      <c r="L41" t="inlineStr"/>
-      <c r="M41" t="inlineStr"/>
-      <c r="N41" t="inlineStr"/>
-      <c r="O41" t="inlineStr"/>
-      <c r="P41" t="inlineStr"/>
-      <c r="Q41" t="inlineStr"/>
       <c r="R41">
         <f>COUNTIF(C41:Q41,"✓")</f>
         <v/>
@@ -10812,25 +10296,11 @@
           <t>Importación y exportación de datos</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr"/>
-      <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr"/>
-      <c r="G42" t="inlineStr"/>
-      <c r="H42" t="inlineStr"/>
-      <c r="I42" t="inlineStr"/>
-      <c r="J42" t="inlineStr"/>
-      <c r="K42" t="inlineStr"/>
-      <c r="L42" t="inlineStr"/>
-      <c r="M42" t="inlineStr"/>
-      <c r="N42" t="inlineStr"/>
-      <c r="O42" t="inlineStr"/>
-      <c r="P42" t="inlineStr"/>
-      <c r="Q42" t="inlineStr"/>
       <c r="R42">
         <f>COUNTIF(C42:Q42,"✓")</f>
         <v/>
@@ -10847,29 +10317,16 @@
           <t>Integración con EHR de proveedores</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr"/>
-      <c r="D43" t="inlineStr"/>
-      <c r="E43" t="inlineStr"/>
-      <c r="F43" t="inlineStr"/>
-      <c r="G43" t="inlineStr"/>
-      <c r="H43" t="inlineStr"/>
-      <c r="I43" t="inlineStr"/>
       <c r="J43" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="K43" t="inlineStr"/>
       <c r="L43" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="M43" t="inlineStr"/>
-      <c r="N43" t="inlineStr"/>
-      <c r="O43" t="inlineStr"/>
-      <c r="P43" t="inlineStr"/>
-      <c r="Q43" t="inlineStr"/>
       <c r="R43">
         <f>COUNTIF(C43:Q43,"✓")</f>
         <v/>
@@ -10886,29 +10343,16 @@
           <t>Integración con wearables y apps de salud</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr"/>
-      <c r="D44" t="inlineStr"/>
-      <c r="E44" t="inlineStr"/>
-      <c r="F44" t="inlineStr"/>
-      <c r="G44" t="inlineStr"/>
       <c r="H44" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="I44" t="inlineStr"/>
-      <c r="J44" t="inlineStr"/>
-      <c r="K44" t="inlineStr"/>
-      <c r="L44" t="inlineStr"/>
       <c r="M44" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="N44" t="inlineStr"/>
-      <c r="O44" t="inlineStr"/>
-      <c r="P44" t="inlineStr"/>
-      <c r="Q44" t="inlineStr"/>
       <c r="R44">
         <f>COUNTIF(C44:Q44,"✓")</f>
         <v/>
@@ -10925,25 +10369,11 @@
           <t>Gestión de lista de medicamentos</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr"/>
-      <c r="D45" t="inlineStr"/>
-      <c r="E45" t="inlineStr"/>
-      <c r="F45" t="inlineStr"/>
-      <c r="G45" t="inlineStr"/>
-      <c r="H45" t="inlineStr"/>
-      <c r="I45" t="inlineStr"/>
-      <c r="J45" t="inlineStr"/>
       <c r="K45" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="L45" t="inlineStr"/>
-      <c r="M45" t="inlineStr"/>
-      <c r="N45" t="inlineStr"/>
-      <c r="O45" t="inlineStr"/>
-      <c r="P45" t="inlineStr"/>
-      <c r="Q45" t="inlineStr"/>
       <c r="R45">
         <f>COUNTIF(C45:Q45,"✓")</f>
         <v/>
@@ -10960,25 +10390,11 @@
           <t>Importación automática de tratamientos desde receta digital</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr"/>
-      <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr"/>
-      <c r="G46" t="inlineStr"/>
-      <c r="H46" t="inlineStr"/>
-      <c r="I46" t="inlineStr"/>
-      <c r="J46" t="inlineStr"/>
-      <c r="K46" t="inlineStr"/>
-      <c r="L46" t="inlineStr"/>
-      <c r="M46" t="inlineStr"/>
-      <c r="N46" t="inlineStr"/>
-      <c r="O46" t="inlineStr"/>
-      <c r="P46" t="inlineStr"/>
-      <c r="Q46" t="inlineStr"/>
       <c r="R46">
         <f>COUNTIF(C46:Q46,"✓")</f>
         <v/>
@@ -11000,24 +10416,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr"/>
-      <c r="E47" t="inlineStr"/>
-      <c r="F47" t="inlineStr"/>
-      <c r="G47" t="inlineStr"/>
-      <c r="H47" t="inlineStr"/>
-      <c r="I47" t="inlineStr"/>
-      <c r="J47" t="inlineStr"/>
       <c r="K47" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="L47" t="inlineStr"/>
-      <c r="M47" t="inlineStr"/>
-      <c r="N47" t="inlineStr"/>
-      <c r="O47" t="inlineStr"/>
-      <c r="P47" t="inlineStr"/>
-      <c r="Q47" t="inlineStr"/>
       <c r="R47">
         <f>COUNTIF(C47:Q47,"✓")</f>
         <v/>
@@ -11034,25 +10437,11 @@
           <t>Registro de tomas y adherencia al tratamiento</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr"/>
-      <c r="D48" t="inlineStr"/>
       <c r="E48" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr"/>
-      <c r="G48" t="inlineStr"/>
-      <c r="H48" t="inlineStr"/>
-      <c r="I48" t="inlineStr"/>
-      <c r="J48" t="inlineStr"/>
-      <c r="K48" t="inlineStr"/>
-      <c r="L48" t="inlineStr"/>
-      <c r="M48" t="inlineStr"/>
-      <c r="N48" t="inlineStr"/>
-      <c r="O48" t="inlineStr"/>
-      <c r="P48" t="inlineStr"/>
-      <c r="Q48" t="inlineStr"/>
       <c r="R48">
         <f>COUNTIF(C48:Q48,"✓")</f>
         <v/>
@@ -11069,25 +10458,11 @@
           <t>Comunidad de pacientes</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr"/>
-      <c r="D49" t="inlineStr"/>
-      <c r="E49" t="inlineStr"/>
-      <c r="F49" t="inlineStr"/>
-      <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="I49" t="inlineStr"/>
-      <c r="J49" t="inlineStr"/>
-      <c r="K49" t="inlineStr"/>
-      <c r="L49" t="inlineStr"/>
-      <c r="M49" t="inlineStr"/>
-      <c r="N49" t="inlineStr"/>
-      <c r="O49" t="inlineStr"/>
-      <c r="P49" t="inlineStr"/>
-      <c r="Q49" t="inlineStr"/>
       <c r="R49">
         <f>COUNTIF(C49:Q49,"✓")</f>
         <v/>
@@ -11104,25 +10479,11 @@
           <t>Contenido educativo sobre salud</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr"/>
       <c r="D50" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr"/>
-      <c r="F50" t="inlineStr"/>
-      <c r="G50" t="inlineStr"/>
-      <c r="H50" t="inlineStr"/>
-      <c r="I50" t="inlineStr"/>
-      <c r="J50" t="inlineStr"/>
-      <c r="K50" t="inlineStr"/>
-      <c r="L50" t="inlineStr"/>
-      <c r="M50" t="inlineStr"/>
-      <c r="N50" t="inlineStr"/>
-      <c r="O50" t="inlineStr"/>
-      <c r="P50" t="inlineStr"/>
-      <c r="Q50" t="inlineStr"/>
       <c r="R50">
         <f>COUNTIF(C50:Q50,"✓")</f>
         <v/>
@@ -11139,25 +10500,11 @@
           <t>Gráficas de evolución de indicadores</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr"/>
-      <c r="D51" t="inlineStr"/>
       <c r="E51" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F51" t="inlineStr"/>
-      <c r="G51" t="inlineStr"/>
-      <c r="H51" t="inlineStr"/>
-      <c r="I51" t="inlineStr"/>
-      <c r="J51" t="inlineStr"/>
-      <c r="K51" t="inlineStr"/>
-      <c r="L51" t="inlineStr"/>
-      <c r="M51" t="inlineStr"/>
-      <c r="N51" t="inlineStr"/>
-      <c r="O51" t="inlineStr"/>
-      <c r="P51" t="inlineStr"/>
-      <c r="Q51" t="inlineStr"/>
       <c r="R51">
         <f>COUNTIF(C51:Q51,"✓")</f>
         <v/>
@@ -11174,25 +10521,11 @@
           <t>Integración con wearables y apps de salud</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr"/>
-      <c r="D52" t="inlineStr"/>
-      <c r="E52" t="inlineStr"/>
-      <c r="F52" t="inlineStr"/>
-      <c r="G52" t="inlineStr"/>
-      <c r="H52" t="inlineStr"/>
-      <c r="I52" t="inlineStr"/>
-      <c r="J52" t="inlineStr"/>
       <c r="K52" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="L52" t="inlineStr"/>
-      <c r="M52" t="inlineStr"/>
-      <c r="N52" t="inlineStr"/>
-      <c r="O52" t="inlineStr"/>
-      <c r="P52" t="inlineStr"/>
-      <c r="Q52" t="inlineStr"/>
       <c r="R52">
         <f>COUNTIF(C52:Q52,"✓")</f>
         <v/>
@@ -11209,11 +10542,6 @@
           <t>Panel de seguimiento de salud y bienestar</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr"/>
-      <c r="D53" t="inlineStr"/>
-      <c r="E53" t="inlineStr"/>
-      <c r="F53" t="inlineStr"/>
-      <c r="G53" t="inlineStr"/>
       <c r="H53" t="inlineStr">
         <is>
           <t>✓</t>
@@ -11224,14 +10552,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="J53" t="inlineStr"/>
-      <c r="K53" t="inlineStr"/>
-      <c r="L53" t="inlineStr"/>
-      <c r="M53" t="inlineStr"/>
-      <c r="N53" t="inlineStr"/>
-      <c r="O53" t="inlineStr"/>
-      <c r="P53" t="inlineStr"/>
-      <c r="Q53" t="inlineStr"/>
       <c r="R53">
         <f>COUNTIF(C53:Q53,"✓")</f>
         <v/>
@@ -11248,25 +10568,11 @@
           <t>Registro de nutrición</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr"/>
-      <c r="D54" t="inlineStr"/>
-      <c r="E54" t="inlineStr"/>
-      <c r="F54" t="inlineStr"/>
-      <c r="G54" t="inlineStr"/>
-      <c r="H54" t="inlineStr"/>
-      <c r="I54" t="inlineStr"/>
-      <c r="J54" t="inlineStr"/>
       <c r="K54" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="L54" t="inlineStr"/>
-      <c r="M54" t="inlineStr"/>
-      <c r="N54" t="inlineStr"/>
-      <c r="O54" t="inlineStr"/>
-      <c r="P54" t="inlineStr"/>
-      <c r="Q54" t="inlineStr"/>
       <c r="R54">
         <f>COUNTIF(C54:Q54,"✓")</f>
         <v/>
@@ -11283,25 +10589,11 @@
           <t>Seguimiento de salud femenina</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr"/>
-      <c r="D55" t="inlineStr"/>
-      <c r="E55" t="inlineStr"/>
-      <c r="F55" t="inlineStr"/>
-      <c r="G55" t="inlineStr"/>
-      <c r="H55" t="inlineStr"/>
-      <c r="I55" t="inlineStr"/>
-      <c r="J55" t="inlineStr"/>
       <c r="K55" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="L55" t="inlineStr"/>
-      <c r="M55" t="inlineStr"/>
-      <c r="N55" t="inlineStr"/>
-      <c r="O55" t="inlineStr"/>
-      <c r="P55" t="inlineStr"/>
-      <c r="Q55" t="inlineStr"/>
       <c r="R55">
         <f>COUNTIF(C55:Q55,"✓")</f>
         <v/>
@@ -11318,25 +10610,11 @@
           <t>Valoración de profesionales</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr"/>
-      <c r="D56" t="inlineStr"/>
-      <c r="E56" t="inlineStr"/>
       <c r="F56" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="G56" t="inlineStr"/>
-      <c r="H56" t="inlineStr"/>
-      <c r="I56" t="inlineStr"/>
-      <c r="J56" t="inlineStr"/>
-      <c r="K56" t="inlineStr"/>
-      <c r="L56" t="inlineStr"/>
-      <c r="M56" t="inlineStr"/>
-      <c r="N56" t="inlineStr"/>
-      <c r="O56" t="inlineStr"/>
-      <c r="P56" t="inlineStr"/>
-      <c r="Q56" t="inlineStr"/>
       <c r="R56">
         <f>COUNTIF(C56:Q56,"✓")</f>
         <v/>
@@ -11353,25 +10631,11 @@
           <t>Acceso mínimo por categorías de datos</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr"/>
-      <c r="D57" t="inlineStr"/>
-      <c r="E57" t="inlineStr"/>
-      <c r="F57" t="inlineStr"/>
-      <c r="G57" t="inlineStr"/>
-      <c r="H57" t="inlineStr"/>
-      <c r="I57" t="inlineStr"/>
-      <c r="J57" t="inlineStr"/>
-      <c r="K57" t="inlineStr"/>
-      <c r="L57" t="inlineStr"/>
       <c r="M57" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="N57" t="inlineStr"/>
-      <c r="O57" t="inlineStr"/>
-      <c r="P57" t="inlineStr"/>
-      <c r="Q57" t="inlineStr"/>
       <c r="R57">
         <f>COUNTIF(C57:Q57,"✓")</f>
         <v/>
@@ -11388,11 +10652,6 @@
           <t>Blockchain para integridad y trazabilidad de datos</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr"/>
-      <c r="D58" t="inlineStr"/>
-      <c r="E58" t="inlineStr"/>
-      <c r="F58" t="inlineStr"/>
-      <c r="G58" t="inlineStr"/>
       <c r="H58" t="inlineStr">
         <is>
           <t>✓</t>
@@ -11408,13 +10667,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="K58" t="inlineStr"/>
-      <c r="L58" t="inlineStr"/>
-      <c r="M58" t="inlineStr"/>
-      <c r="N58" t="inlineStr"/>
-      <c r="O58" t="inlineStr"/>
-      <c r="P58" t="inlineStr"/>
-      <c r="Q58" t="inlineStr"/>
       <c r="R58">
         <f>COUNTIF(C58:Q58,"✓")</f>
         <v/>
@@ -11431,29 +10683,16 @@
           <t>Cifrado y control de acceso</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr"/>
       <c r="D59" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr"/>
-      <c r="F59" t="inlineStr"/>
-      <c r="G59" t="inlineStr"/>
-      <c r="H59" t="inlineStr"/>
-      <c r="I59" t="inlineStr"/>
-      <c r="J59" t="inlineStr"/>
       <c r="K59" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="L59" t="inlineStr"/>
-      <c r="M59" t="inlineStr"/>
-      <c r="N59" t="inlineStr"/>
-      <c r="O59" t="inlineStr"/>
-      <c r="P59" t="inlineStr"/>
-      <c r="Q59" t="inlineStr"/>
       <c r="R59">
         <f>COUNTIF(C59:Q59,"✓")</f>
         <v/>
@@ -11470,25 +10709,11 @@
           <t>Cumplimiento regulatorio de salud y datos</t>
         </is>
       </c>
-      <c r="C60" t="inlineStr"/>
-      <c r="D60" t="inlineStr"/>
-      <c r="E60" t="inlineStr"/>
-      <c r="F60" t="inlineStr"/>
-      <c r="G60" t="inlineStr"/>
-      <c r="H60" t="inlineStr"/>
-      <c r="I60" t="inlineStr"/>
-      <c r="J60" t="inlineStr"/>
-      <c r="K60" t="inlineStr"/>
-      <c r="L60" t="inlineStr"/>
-      <c r="M60" t="inlineStr"/>
-      <c r="N60" t="inlineStr"/>
       <c r="O60" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="P60" t="inlineStr"/>
-      <c r="Q60" t="inlineStr"/>
       <c r="R60">
         <f>COUNTIF(C60:Q60,"✓")</f>
         <v/>
@@ -11505,25 +10730,11 @@
           <t>Gestión de consentimiento sobre uso de datos</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr"/>
-      <c r="D61" t="inlineStr"/>
-      <c r="E61" t="inlineStr"/>
-      <c r="F61" t="inlineStr"/>
-      <c r="G61" t="inlineStr"/>
-      <c r="H61" t="inlineStr"/>
-      <c r="I61" t="inlineStr"/>
-      <c r="J61" t="inlineStr"/>
-      <c r="K61" t="inlineStr"/>
       <c r="L61" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="M61" t="inlineStr"/>
-      <c r="N61" t="inlineStr"/>
-      <c r="O61" t="inlineStr"/>
-      <c r="P61" t="inlineStr"/>
-      <c r="Q61" t="inlineStr"/>
       <c r="R61">
         <f>COUNTIF(C61:Q61,"✓")</f>
         <v/>
@@ -11540,25 +10751,11 @@
           <t>Identidad descentralizada (DID)</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr"/>
-      <c r="D62" t="inlineStr"/>
-      <c r="E62" t="inlineStr"/>
-      <c r="F62" t="inlineStr"/>
-      <c r="G62" t="inlineStr"/>
-      <c r="H62" t="inlineStr"/>
       <c r="I62" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="J62" t="inlineStr"/>
-      <c r="K62" t="inlineStr"/>
-      <c r="L62" t="inlineStr"/>
-      <c r="M62" t="inlineStr"/>
-      <c r="N62" t="inlineStr"/>
-      <c r="O62" t="inlineStr"/>
-      <c r="P62" t="inlineStr"/>
-      <c r="Q62" t="inlineStr"/>
       <c r="R62">
         <f>COUNTIF(C62:Q62,"✓")</f>
         <v/>
@@ -11575,15 +10772,6 @@
           <t>Privacidad reforzada para datos de salud</t>
         </is>
       </c>
-      <c r="C63" t="inlineStr"/>
-      <c r="D63" t="inlineStr"/>
-      <c r="E63" t="inlineStr"/>
-      <c r="F63" t="inlineStr"/>
-      <c r="G63" t="inlineStr"/>
-      <c r="H63" t="inlineStr"/>
-      <c r="I63" t="inlineStr"/>
-      <c r="J63" t="inlineStr"/>
-      <c r="K63" t="inlineStr"/>
       <c r="L63" t="inlineStr">
         <is>
           <t>✓</t>
@@ -11594,10 +10782,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="N63" t="inlineStr"/>
-      <c r="O63" t="inlineStr"/>
-      <c r="P63" t="inlineStr"/>
-      <c r="Q63" t="inlineStr"/>
       <c r="R63">
         <f>COUNTIF(C63:Q63,"✓")</f>
         <v/>
@@ -11614,20 +10798,6 @@
           <t>Modelo freemium y suscripción</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr"/>
-      <c r="D64" t="inlineStr"/>
-      <c r="E64" t="inlineStr"/>
-      <c r="F64" t="inlineStr"/>
-      <c r="G64" t="inlineStr"/>
-      <c r="H64" t="inlineStr"/>
-      <c r="I64" t="inlineStr"/>
-      <c r="J64" t="inlineStr"/>
-      <c r="K64" t="inlineStr"/>
-      <c r="L64" t="inlineStr"/>
-      <c r="M64" t="inlineStr"/>
-      <c r="N64" t="inlineStr"/>
-      <c r="O64" t="inlineStr"/>
-      <c r="P64" t="inlineStr"/>
       <c r="Q64" t="inlineStr">
         <is>
           <t>✓</t>
@@ -11649,25 +10819,11 @@
           <t>Pagos con criptomoneda</t>
         </is>
       </c>
-      <c r="C65" t="inlineStr"/>
-      <c r="D65" t="inlineStr"/>
-      <c r="E65" t="inlineStr"/>
-      <c r="F65" t="inlineStr"/>
-      <c r="G65" t="inlineStr"/>
-      <c r="H65" t="inlineStr"/>
-      <c r="I65" t="inlineStr"/>
       <c r="J65" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="K65" t="inlineStr"/>
-      <c r="L65" t="inlineStr"/>
-      <c r="M65" t="inlineStr"/>
-      <c r="N65" t="inlineStr"/>
-      <c r="O65" t="inlineStr"/>
-      <c r="P65" t="inlineStr"/>
-      <c r="Q65" t="inlineStr"/>
       <c r="R65">
         <f>COUNTIF(C65:Q65,"✓")</f>
         <v/>
@@ -11684,24 +10840,11 @@
           <t>Pagos dentro de la app</t>
         </is>
       </c>
-      <c r="C66" t="inlineStr"/>
-      <c r="D66" t="inlineStr"/>
-      <c r="E66" t="inlineStr"/>
-      <c r="F66" t="inlineStr"/>
-      <c r="G66" t="inlineStr"/>
-      <c r="H66" t="inlineStr"/>
-      <c r="I66" t="inlineStr"/>
-      <c r="J66" t="inlineStr"/>
-      <c r="K66" t="inlineStr"/>
-      <c r="L66" t="inlineStr"/>
-      <c r="M66" t="inlineStr"/>
       <c r="N66" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="O66" t="inlineStr"/>
-      <c r="P66" t="inlineStr"/>
       <c r="Q66" t="inlineStr">
         <is>
           <t>✓</t>
@@ -11723,25 +10866,11 @@
           <t>Reclamos y trámites con seguros</t>
         </is>
       </c>
-      <c r="C67" t="inlineStr"/>
-      <c r="D67" t="inlineStr"/>
-      <c r="E67" t="inlineStr"/>
-      <c r="F67" t="inlineStr"/>
-      <c r="G67" t="inlineStr"/>
-      <c r="H67" t="inlineStr"/>
       <c r="I67" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="J67" t="inlineStr"/>
-      <c r="K67" t="inlineStr"/>
-      <c r="L67" t="inlineStr"/>
-      <c r="M67" t="inlineStr"/>
-      <c r="N67" t="inlineStr"/>
-      <c r="O67" t="inlineStr"/>
-      <c r="P67" t="inlineStr"/>
-      <c r="Q67" t="inlineStr"/>
       <c r="R67">
         <f>COUNTIF(C67:Q67,"✓")</f>
         <v/>
@@ -11758,25 +10887,11 @@
           <t>Mensajería paciente-institución</t>
         </is>
       </c>
-      <c r="C68" t="inlineStr"/>
-      <c r="D68" t="inlineStr"/>
-      <c r="E68" t="inlineStr"/>
-      <c r="F68" t="inlineStr"/>
-      <c r="G68" t="inlineStr"/>
-      <c r="H68" t="inlineStr"/>
       <c r="I68" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="J68" t="inlineStr"/>
-      <c r="K68" t="inlineStr"/>
-      <c r="L68" t="inlineStr"/>
-      <c r="M68" t="inlineStr"/>
-      <c r="N68" t="inlineStr"/>
-      <c r="O68" t="inlineStr"/>
-      <c r="P68" t="inlineStr"/>
-      <c r="Q68" t="inlineStr"/>
       <c r="R68">
         <f>COUNTIF(C68:Q68,"✓")</f>
         <v/>
@@ -11793,25 +10908,11 @@
           <t>Teleconsulta con profesionales</t>
         </is>
       </c>
-      <c r="C69" t="inlineStr"/>
-      <c r="D69" t="inlineStr"/>
-      <c r="E69" t="inlineStr"/>
-      <c r="F69" t="inlineStr"/>
-      <c r="G69" t="inlineStr"/>
-      <c r="H69" t="inlineStr"/>
-      <c r="I69" t="inlineStr"/>
       <c r="J69" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="K69" t="inlineStr"/>
-      <c r="L69" t="inlineStr"/>
-      <c r="M69" t="inlineStr"/>
-      <c r="N69" t="inlineStr"/>
-      <c r="O69" t="inlineStr"/>
-      <c r="P69" t="inlineStr"/>
-      <c r="Q69" t="inlineStr"/>
       <c r="R69">
         <f>COUNTIF(C69:Q69,"✓")</f>
         <v/>
@@ -11828,7 +10929,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A44"/>
+  <dimension ref="A1:A45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -12142,6 +11243,13 @@
         </is>
       </c>
     </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Vuelta 10 (iter. 1, 2026-10-29 12:25 UTC): Meedika, Infomed, MediPlanner, Clingot verificados (+0 filas; saturado). Pendientes: Healfies, Patientory, MediBloc, Medicalchain, Apple Health, ChatGPT Health, Claude for Healthcare, Apps de clínicas, Clinia, MiRedSalud, Mediko.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Benchmark: vuelta 10, iteración 2 (Healfies, Patientory, MediBloc, Medicalchain)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MVcXu8vTBu7EKfj3YdEvae
</commit_message>
<xml_diff>
--- a/Outputs/Benchmark_Anamnesis.xlsx
+++ b/Outputs/Benchmark_Anamnesis.xlsx
@@ -673,12 +673,12 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>[REGIONAL · Brasil] Fundada ene-2015 en Florianópolis por Helyson Lewis Velasco. Centraliza registros de salud personales: carpetas, etiquetas, línea de tiempo (medicación, exámenes, citas, dieta), compartir con familia o profesionales. Gratis; web, iOS y Android. Estado actual NO verificado (fuentes de 2015-2016). Referencia funcional cercana a etapas A+B. [Vuelta 2] Lanzada simultáneamente en Brasil, Argentina y EE.UU.; permite compartir con no registrados vía clave por email. Sin novedades posteriores a 2016. [Vuelta 3] Sin evidencia de actividad reciente ni de cierre; Gust/Dealroom la listan en Florianópolis (10 empleados, healfies.com) sin fecha de actualización. Estado sin confirmar. [Vuelta 4] Sin Google Play localizado; no confundir con la app Healfy (otro producto). Sin novedades. [Vuelta 5] Sin búsqueda nueva (revisada en vuelta 4); sin cambios. [Vuelta 6] Sin búsqueda nueva (fuentes agotadas); sin cambios. [Vuelta 7] Solo fuentes de 2015-2016; alianza con ClinCard (feb-2016). Sin evidencia de actividad reciente. [Vuelta 8] Sin fuentes nuevas. [Vuelta 9] Sin búsqueda nueva (saturado).</t>
+          <t>[REGIONAL · Brasil] Fundada ene-2015 en Florianópolis por Helyson Lewis Velasco. Centraliza registros de salud personales: carpetas, etiquetas, línea de tiempo (medicación, exámenes, citas, dieta), compartir con familia o profesionales. Gratis; web, iOS y Android. Estado actual NO verificado (fuentes de 2015-2016). Referencia funcional cercana a etapas A+B. [Vuelta 2] Lanzada simultáneamente en Brasil, Argentina y EE.UU.; permite compartir con no registrados vía clave por email. Sin novedades posteriores a 2016. [Vuelta 3] Sin evidencia de actividad reciente ni de cierre; Gust/Dealroom la listan en Florianópolis (10 empleados, healfies.com) sin fecha de actualización. Estado sin confirmar. [Vuelta 4] Sin Google Play localizado; no confundir con la app Healfy (otro producto). Sin novedades. [Vuelta 5] Sin búsqueda nueva (revisada en vuelta 4); sin cambios. [Vuelta 6] Sin búsqueda nueva (fuentes agotadas); sin cambios. [Vuelta 7] Solo fuentes de 2015-2016; alianza con ClinCard (feb-2016). Sin evidencia de actividad reciente. [Vuelta 8] Sin fuentes nuevas. [Vuelta 9] Sin búsqueda nueva (saturado). [Vuelta 10] Sin búsqueda nueva (saturado).</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G6" t="n">
@@ -686,7 +686,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-30</t>
         </is>
       </c>
     </row>
@@ -713,12 +713,12 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>[BLOCKCHAIN · EE.UU.] Atlanta, fundada 2015, ~9 empleados. Levantó US$7,2M vía financiamiento cripto. App con registros de hospitales y wearables, coaching de salud con IA y recompensas en cripto; también dashboard empresarial Neith. PitchBook indica actividad y financiamiento hasta abr-2026: sigue operando. Sin presencia conocida en Chile. Referencia directa para la hipótesis blockchain. [Vuelta 2] Sin noticias 2026 encontradas en búsqueda; sitio oficial bloqueado. [Vuelta 3] Búsqueda adicional solo devuelve hitos de 2017 (token sale US$7,2M) y 2019 (Serie A de US$5,3M, cierre no confirmado); sin datos 2025-26 propios. [Vuelta 4] App pública lanzada en la conferencia JP Morgan Healthcare (2019); red PTOYMatrix (blockchain HIPAA); socios reportados: StartUp Health y Kaiser Permanente (beta). Estado actual en App Store/Google Play sin confirmar. [Vuelta 5] Sin noticias 2026 del equipo. Token PTOY con capitalización de ~US$53K a fines de ago-2026 según Phantom (KuCoin discrepa en la circulación): señal de baja actividad, no prueba de cierre. Esto relativiza la actividad hasta abr-2026 mencionada en la ficha original. [Vuelta 6] Sin noticias posteriores a 2020 localizadas (hitos: token sale 2017, consorcio Hyperledger, alianza con Georgia State, Series A de US$5,3M vía R/GA Ventures, Neith con Prosper Healthtech en Birmingham). Estado actual desconocido. [Vuelta 7] Sin búsqueda nueva (saturado); sin cambios. [Vuelta 8] Sin noticias 2025-26; en 2018 la oferta se dirigía a empresas de salud, con la versión individual planificada después. [Vuelta 9] Sin búsqueda nueva (saturado).</t>
+          <t>[BLOCKCHAIN · EE.UU.] Atlanta, fundada 2015, ~9 empleados. Levantó US$7,2M vía financiamiento cripto. App con registros de hospitales y wearables, coaching de salud con IA y recompensas en cripto; también dashboard empresarial Neith. PitchBook indica actividad y financiamiento hasta abr-2026: sigue operando. Sin presencia conocida en Chile. Referencia directa para la hipótesis blockchain. [Vuelta 2] Sin noticias 2026 encontradas en búsqueda; sitio oficial bloqueado. [Vuelta 3] Búsqueda adicional solo devuelve hitos de 2017 (token sale US$7,2M) y 2019 (Serie A de US$5,3M, cierre no confirmado); sin datos 2025-26 propios. [Vuelta 4] App pública lanzada en la conferencia JP Morgan Healthcare (2019); red PTOYMatrix (blockchain HIPAA); socios reportados: StartUp Health y Kaiser Permanente (beta). Estado actual en App Store/Google Play sin confirmar. [Vuelta 5] Sin noticias 2026 del equipo. Token PTOY con capitalización de ~US$53K a fines de ago-2026 según Phantom (KuCoin discrepa en la circulación): señal de baja actividad, no prueba de cierre. Esto relativiza la actividad hasta abr-2026 mencionada en la ficha original. [Vuelta 6] Sin noticias posteriores a 2020 localizadas (hitos: token sale 2017, consorcio Hyperledger, alianza con Georgia State, Series A de US$5,3M vía R/GA Ventures, Neith con Prosper Healthtech en Birmingham). Estado actual desconocido. [Vuelta 7] Sin búsqueda nueva (saturado); sin cambios. [Vuelta 8] Sin noticias 2025-26; en 2018 la oferta se dirigía a empresas de salud, con la versión individual planificada después. [Vuelta 9] Sin búsqueda nueva (saturado). [Vuelta 10] Sin búsqueda nueva (saturado).</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G7" t="n">
@@ -726,7 +726,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-30</t>
         </is>
       </c>
     </row>
@@ -753,12 +753,12 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>[BLOCKCHAIN · Corea del Sur] Fundada 2017, Seúl. Blockchain propia Panacea (Cosmos SDK, mainnet 2019) para que el paciente gestione y transfiera sus registros; app Medipass para seguros. Serie A de ₩4.000 millones (Naver); alianzas con hospitales (Seoul National, Severance). Estado 2025-26 NO verificado. Referencia sobre seguros + blockchain. [Vuelta 2] Panacea incluye DID, Append Only Log, IBC y PNFT; sin anuncios 2026 localizados. [Vuelta 3] Medipass: app en Corea con 20 hospitales/aseguradoras integrados (fecha de la lista desconocida) y plan 2022 de superapp con marketplace de datos; operación actual sin confirmar. [Vuelta 4] Sin búsqueda nueva (revisada en vuelta 3); sin cambios. [Vuelta 5] Medipass: ~400.000 usuarios acumulados (CEO, jun-2022); integración con aseguradoras Shinhan Life, Samsung Fire y Hyundai Marine (2020); renovación completa en mar-2023 (dashboard de salud, gestión familiar, certificados). Sin noticias 2026 encontradas. [Vuelta 6] Medipass 2023: comunicación bidireccional hospital-paciente y chat MediTalk; en 2019 fue seleccionada para el programa gubernamental de MyData médico con Samsung Fire y SNUH. Sin estrategia 2026 localizada. Meta declarada: usar Medipass como «identificación» de salud. [Vuelta 7] Una fuente sin fecha atribuye a Medipass más de 600.000 pacientes en 14 hospitales; MoU 2019 con Severance (plataforma de facturación de seguros y detección de falsificación de datos) y piloto con Massachusetts General Hospital. Sin datos 2025-26. [Vuelta 8] Sin noticias 2025-26. [Vuelta 9] Sin búsqueda nueva (saturado).</t>
+          <t>[BLOCKCHAIN · Corea del Sur] Fundada 2017, Seúl. Blockchain propia Panacea (Cosmos SDK, mainnet 2019) para que el paciente gestione y transfiera sus registros; app Medipass para seguros. Serie A de ₩4.000 millones (Naver); alianzas con hospitales (Seoul National, Severance). Estado 2025-26 NO verificado. Referencia sobre seguros + blockchain. [Vuelta 2] Panacea incluye DID, Append Only Log, IBC y PNFT; sin anuncios 2026 localizados. [Vuelta 3] Medipass: app en Corea con 20 hospitales/aseguradoras integrados (fecha de la lista desconocida) y plan 2022 de superapp con marketplace de datos; operación actual sin confirmar. [Vuelta 4] Sin búsqueda nueva (revisada en vuelta 3); sin cambios. [Vuelta 5] Medipass: ~400.000 usuarios acumulados (CEO, jun-2022); integración con aseguradoras Shinhan Life, Samsung Fire y Hyundai Marine (2020); renovación completa en mar-2023 (dashboard de salud, gestión familiar, certificados). Sin noticias 2026 encontradas. [Vuelta 6] Medipass 2023: comunicación bidireccional hospital-paciente y chat MediTalk; en 2019 fue seleccionada para el programa gubernamental de MyData médico con Samsung Fire y SNUH. Sin estrategia 2026 localizada. Meta declarada: usar Medipass como «identificación» de salud. [Vuelta 7] Una fuente sin fecha atribuye a Medipass más de 600.000 pacientes en 14 hospitales; MoU 2019 con Severance (plataforma de facturación de seguros y detección de falsificación de datos) y piloto con Massachusetts General Hospital. Sin datos 2025-26. [Vuelta 8] Sin noticias 2025-26. [Vuelta 9] Sin búsqueda nueva (saturado). [Vuelta 10] Sin búsqueda nueva (saturado).</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G8" t="n">
@@ -766,7 +766,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-30</t>
         </is>
       </c>
     </row>
@@ -793,12 +793,12 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>[BLOCKCHAIN · Reino Unido · INACTIVO] Londres, 2017, Ethereum, con telemedicina. Piloto según registro de la UE (2020). Tracxn/PitchBook lo marcan fuera de operación (ago-2025). Solo caso de aprendizaje: no cuenta como competidor activo. [Vuelta 2] Token MTN deslistado de Bitfinex el 26-mar-2021; sin hallazgos de actividad posterior. [Vuelta 3] Seedtable la marca activa sin fuente; no hallé registro en Companies House. Sigue tratándose como caso de aprendizaje. [Vuelta 4] Pre-venta reportada de US$20M en MedTokens (un solo artículo secundario, sin verificar); modelo de token en revisión y exploración de security token según AMA; integraciones y servicios de 2019 sin confirmar. [Vuelta 5] Un agregador indica sitio medicalchain.com fuera de línea desde 15-feb-2025, último commit en GitHub hace ~3 años y proyecto en «fase de mantenimiento»; preventa de MedTokens reportada entre US$20M y US$24M (fuentes discrepan). Confirma tratarlo como inactivo. [Vuelta 6] Sin búsqueda nueva (revisada en vuelta 5; sitio fuera de línea desde feb-2025 según un agregador); sin cambios. [Vuelta 7] Sin búsqueda nueva (saturado); sin cambios. [Vuelta 8] Sin fuentes nuevas; se mantiene como inactivo. [Vuelta 9] Sin búsqueda nueva (saturado).</t>
+          <t>[BLOCKCHAIN · Reino Unido · INACTIVO] Londres, 2017, Ethereum, con telemedicina. Piloto según registro de la UE (2020). Tracxn/PitchBook lo marcan fuera de operación (ago-2025). Solo caso de aprendizaje: no cuenta como competidor activo. [Vuelta 2] Token MTN deslistado de Bitfinex el 26-mar-2021; sin hallazgos de actividad posterior. [Vuelta 3] Seedtable la marca activa sin fuente; no hallé registro en Companies House. Sigue tratándose como caso de aprendizaje. [Vuelta 4] Pre-venta reportada de US$20M en MedTokens (un solo artículo secundario, sin verificar); modelo de token en revisión y exploración de security token según AMA; integraciones y servicios de 2019 sin confirmar. [Vuelta 5] Un agregador indica sitio medicalchain.com fuera de línea desde 15-feb-2025, último commit en GitHub hace ~3 años y proyecto en «fase de mantenimiento»; preventa de MedTokens reportada entre US$20M y US$24M (fuentes discrepan). Confirma tratarlo como inactivo. [Vuelta 6] Sin búsqueda nueva (revisada en vuelta 5; sitio fuera de línea desde feb-2025 según un agregador); sin cambios. [Vuelta 7] Sin búsqueda nueva (saturado); sin cambios. [Vuelta 8] Sin fuentes nuevas; se mantiene como inactivo. [Vuelta 9] Sin búsqueda nueva (saturado). [Vuelta 10] Sin búsqueda nueva (saturado).</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G9" t="n">
@@ -806,7 +806,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-30</t>
         </is>
       </c>
     </row>
@@ -10929,7 +10929,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A45"/>
+  <dimension ref="A1:A46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -11250,6 +11250,13 @@
         </is>
       </c>
     </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Vuelta 10 (iter. 2, 2026-10-30 12:35 UTC): Healfies, Patientory, MediBloc, Medicalchain verificados sin búsqueda nueva (+0 filas; saturado). Pendientes: Apple Health, ChatGPT Health, Claude for Healthcare, Apps de clínicas, Clinia, MiRedSalud, Mediko.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Benchmark: vuelta 10, iteración 3 (Apple Health, ChatGPT Health, Claude for Healthcare, Apps de clínicas)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MVcXu8vTBu7EKfj3YdEvae
</commit_message>
<xml_diff>
--- a/Outputs/Benchmark_Anamnesis.xlsx
+++ b/Outputs/Benchmark_Anamnesis.xlsx
@@ -833,12 +833,12 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>[ADYACENTE · global] Agrega registros clínicos vía FHIR; &gt;500 instituciones conectadas en EE.UU. (2018). Sin evidencia de disponibilidad en Chile. Incluida en el dispositivo. Amenaza si FHIR/IPS-CL se adopta en Chile. [Vuelta 2] Sin disponibilidad de registros clínicos en Chile (solo EE.UU., Reino Unido, Canadá). [Vuelta 3] iOS 27 (WWDC 8-jun-2026; publicado ~14-sep-2026): rediseño del app Health, menopausia, nutrición por cámara. El coach de salud con IA no se anunció. Sin ampliación de Health Records a Chile. [Vuelta 4] Sin búsqueda nueva (revisada en vuelta 3); sin cambios. [Vuelta 5] Sin ampliación de Health Records a Australia, Europa ni Latinoamérica (solo EE.UU., UK, Canadá). Funciones de dispositivo (apnea del sueño, prueba auditiva) sí se amplían a países latinoamericanos, pero no son registros clínicos. [Vuelta 6] Sin novedades de iOS 27.x localizadas. Health Records API permite compartir registros con apps de terceros con control por app; opción de enviar datos de uso a Apple. [Vuelta 7] Coach de salud con IA / Health+ de pago: solo rumores (Gurman), atrasado al menos a iOS 27; no confirmado ni anunciado. [Vuelta 8] Sin novedades. [Vuelta 9] Sin novedades.</t>
+          <t>[ADYACENTE · global] Agrega registros clínicos vía FHIR; &gt;500 instituciones conectadas en EE.UU. (2018). Sin evidencia de disponibilidad en Chile. Incluida en el dispositivo. Amenaza si FHIR/IPS-CL se adopta en Chile. [Vuelta 2] Sin disponibilidad de registros clínicos en Chile (solo EE.UU., Reino Unido, Canadá). [Vuelta 3] iOS 27 (WWDC 8-jun-2026; publicado ~14-sep-2026): rediseño del app Health, menopausia, nutrición por cámara. El coach de salud con IA no se anunció. Sin ampliación de Health Records a Chile. [Vuelta 4] Sin búsqueda nueva (revisada en vuelta 3); sin cambios. [Vuelta 5] Sin ampliación de Health Records a Australia, Europa ni Latinoamérica (solo EE.UU., UK, Canadá). Funciones de dispositivo (apnea del sueño, prueba auditiva) sí se amplían a países latinoamericanos, pero no son registros clínicos. [Vuelta 6] Sin novedades de iOS 27.x localizadas. Health Records API permite compartir registros con apps de terceros con control por app; opción de enviar datos de uso a Apple. [Vuelta 7] Coach de salud con IA / Health+ de pago: solo rumores (Gurman), atrasado al menos a iOS 27; no confirmado ni anunciado. [Vuelta 8] Sin novedades. [Vuelta 9] Sin novedades. [Vuelta 10] Sin búsqueda nueva (saturado).</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G10" t="n">
@@ -846,7 +846,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-31</t>
         </is>
       </c>
     </row>
@@ -873,12 +873,12 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>[ADYACENTE · global] Lanzado 7-ene-2026. Conecta registros médicos; conectores solo en EE.UU. Dentro de suscripción del asistente. Fija la expectativa de consultar y resumir el historial. [Vuelta 2] Confirmado: registros solo EE.UU.; sin anuncios para Latinoamérica. Hay inconsistencia de fechas entre fuentes (7-ene-2026 lanzamiento vs. jul-2026 despliegue de registros). [Vuelta 3] Fechas aclaradas: presentación 7-ene-2026 (acceso limitado); despliegue de Health in ChatGPT con Apple Health y registros en EE.UU. el 23-jul-2026; mejora de salud jun-2026. Sin anuncios para Latinoamérica ni para sep-oct 2026. [Vuelta 4] Septiembre 2026: permisos por defecto para datos conectados (14-sep) y explicaciones por gráfico/métrica (28-sep); ChatGPT for Clinicians (abr-2026) para clínicos verificados de EE.UU. Más del 70% de usuarios de Health permite usar datos conectados sin pedir permiso (según OpenAI). Sigue solo EE.UU. [Vuelta 5] Nota de jul-2026: Health no está disponible en México, Android, modo de voz ni Codex; web e iOS en EE.UU., adultos con sesión iniciada. Sin anuncio para Chile ni Latinoamérica. [Vuelta 6] Última entrada de Health en las notas de OpenAI sigue siendo la del 23-jul-2026 (más cambios de sep); sin entradas de octubre localizadas. Health tab: laboratorios, medicamentos, actividad y sueño en una vista; solo EE.UU., web e iOS. [Vuelta 7] OpenAI afirma que más de 300 millones de personas usan ChatGPT cada semana para consultas de salud (dato de la empresa). No es una solución con cumplimiento HIPAA declarado. Sin novedades de oct-2026. [Vuelta 8] Sin novedades de fines de oct-2026. [Vuelta 9] Reporte de sep-2026: OpenAI conecta ChatGPT con Epic EHR para clínicos de EE.UU. (sin confirmar con fuente primaria). Sin novedades de oct-2026 para el consumidor.</t>
+          <t>[ADYACENTE · global] Lanzado 7-ene-2026. Conecta registros médicos; conectores solo en EE.UU. Dentro de suscripción del asistente. Fija la expectativa de consultar y resumir el historial. [Vuelta 2] Confirmado: registros solo EE.UU.; sin anuncios para Latinoamérica. Hay inconsistencia de fechas entre fuentes (7-ene-2026 lanzamiento vs. jul-2026 despliegue de registros). [Vuelta 3] Fechas aclaradas: presentación 7-ene-2026 (acceso limitado); despliegue de Health in ChatGPT con Apple Health y registros en EE.UU. el 23-jul-2026; mejora de salud jun-2026. Sin anuncios para Latinoamérica ni para sep-oct 2026. [Vuelta 4] Septiembre 2026: permisos por defecto para datos conectados (14-sep) y explicaciones por gráfico/métrica (28-sep); ChatGPT for Clinicians (abr-2026) para clínicos verificados de EE.UU. Más del 70% de usuarios de Health permite usar datos conectados sin pedir permiso (según OpenAI). Sigue solo EE.UU. [Vuelta 5] Nota de jul-2026: Health no está disponible en México, Android, modo de voz ni Codex; web e iOS en EE.UU., adultos con sesión iniciada. Sin anuncio para Chile ni Latinoamérica. [Vuelta 6] Última entrada de Health en las notas de OpenAI sigue siendo la del 23-jul-2026 (más cambios de sep); sin entradas de octubre localizadas. Health tab: laboratorios, medicamentos, actividad y sueño en una vista; solo EE.UU., web e iOS. [Vuelta 7] OpenAI afirma que más de 300 millones de personas usan ChatGPT cada semana para consultas de salud (dato de la empresa). No es una solución con cumplimiento HIPAA declarado. Sin novedades de oct-2026. [Vuelta 8] Sin novedades de fines de oct-2026. [Vuelta 9] Reporte de sep-2026: OpenAI conecta ChatGPT con Epic EHR para clínicos de EE.UU. (sin confirmar con fuente primaria). Sin novedades de oct-2026 para el consumidor. [Vuelta 10] Capacidades según cobertura de jul-2026: compara nuevos resultados con pruebas anteriores, resume cambios desde la última cita y relaciona sueño, actividad y rutinas. Sin notas de versión de oct/nov-2026 localizadas.</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G11" t="n">
@@ -886,7 +886,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-31</t>
         </is>
       </c>
     </row>
@@ -913,12 +913,12 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>[ADYACENTE · global] Lanzado 11-ene-2026. Conectores solo en EE.UU., planes Pro/Max. Nota: producto de Anthropic, conflicto de interés al evaluarlo. [Vuelta 2] Sin cambios fuera de EE.UU. (HealthEx y Function para Pro/Max). [Vuelta 3] Sin anuncios posteriores a enero de 2026. Hoja de ruta de HealthEx (agendar, buscar prestadores, recetas) sin confirmar como lanzada. [Vuelta 4] Sin anuncios nuevos. Fuentes discrepan en el acceso (Pro/Max según Fortune y la mayoría; Pro/Team según Times of AI); sin evidencia de disponibilidad fuera de EE.UU. [Vuelta 5] Sin noticias de oct-2026; HealthEx agrega datos de &gt;50.000 sistemas de EE.UU. y Claude pide solo las categorías relevantes vía MCP. [Vuelta 6] Sin noticias posteriores a enero de 2026 localizadas. [Vuelta 7] Sin novedades posteriores a enero de 2026. [Vuelta 8] Sin novedades posteriores a enero de 2026. [Vuelta 9] Sin novedades posteriores a enero de 2026.</t>
+          <t>[ADYACENTE · global] Lanzado 11-ene-2026. Conectores solo en EE.UU., planes Pro/Max. Nota: producto de Anthropic, conflicto de interés al evaluarlo. [Vuelta 2] Sin cambios fuera de EE.UU. (HealthEx y Function para Pro/Max). [Vuelta 3] Sin anuncios posteriores a enero de 2026. Hoja de ruta de HealthEx (agendar, buscar prestadores, recetas) sin confirmar como lanzada. [Vuelta 4] Sin anuncios nuevos. Fuentes discrepan en el acceso (Pro/Max según Fortune y la mayoría; Pro/Team según Times of AI); sin evidencia de disponibilidad fuera de EE.UU. [Vuelta 5] Sin noticias de oct-2026; HealthEx agrega datos de &gt;50.000 sistemas de EE.UU. y Claude pide solo las categorías relevantes vía MCP. [Vuelta 6] Sin noticias posteriores a enero de 2026 localizadas. [Vuelta 7] Sin novedades posteriores a enero de 2026. [Vuelta 8] Sin novedades posteriores a enero de 2026. [Vuelta 9] Sin novedades posteriores a enero de 2026. [Vuelta 10] Sin búsqueda nueva (saturado).</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G12" t="n">
@@ -926,7 +926,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-31</t>
         </is>
       </c>
     </row>
@@ -953,12 +953,12 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>[SUSTITUTO PARCIAL · Chile] Reservar hora, ver historial de esa institución, vincular familiar. Gratis; no consolida datos de otras instituciones. [Vuelta 2] App concreta: Mi Alemana Go (Clínica Alemana, Chile), con historial desde 2018, recetas, órdenes, familiar vinculado y resultados. [Vuelta 3] Búsqueda de otras clínicas (Las Condes, Santa María, UC Christus) sin ficha de app confirmada; solo canales digitales genéricos. [Vuelta 4] Mi Alemana Go: 3,1/5 con 137 calificaciones (App Store Chile), pantalla de inicio rediseñada para gestionar salud propia y familiar; sin evidencia de teleconsulta ni pagos en la app. [Vuelta 5] Sin búsqueda nueva (revisada en vuelta 4); sin cambios. [Vuelta 6] Sin búsqueda nueva; sin cambios. [Vuelta 7] Sin búsqueda nueva; sin cambios. [Vuelta 8] Mi Alemana Go: notificaciones de deuda pendiente, check-in de admisión y encuestas de salud; DF la describe como segundo paso de la estrategia digital de la clínica (registros de exámenes, indicaciones, historial y recetas). Otras apps de red: Mi Dávila (Red Dávila, gestión de citas en todos sus centros, según un directorio); Clínica Las Condes sin app confirmada. [Vuelta 9] Sin búsqueda nueva; sin cambios.</t>
+          <t>[SUSTITUTO PARCIAL · Chile] Reservar hora, ver historial de esa institución, vincular familiar. Gratis; no consolida datos de otras instituciones. [Vuelta 2] App concreta: Mi Alemana Go (Clínica Alemana, Chile), con historial desde 2018, recetas, órdenes, familiar vinculado y resultados. [Vuelta 3] Búsqueda de otras clínicas (Las Condes, Santa María, UC Christus) sin ficha de app confirmada; solo canales digitales genéricos. [Vuelta 4] Mi Alemana Go: 3,1/5 con 137 calificaciones (App Store Chile), pantalla de inicio rediseñada para gestionar salud propia y familiar; sin evidencia de teleconsulta ni pagos en la app. [Vuelta 5] Sin búsqueda nueva (revisada en vuelta 4); sin cambios. [Vuelta 6] Sin búsqueda nueva; sin cambios. [Vuelta 7] Sin búsqueda nueva; sin cambios. [Vuelta 8] Mi Alemana Go: notificaciones de deuda pendiente, check-in de admisión y encuestas de salud; DF la describe como segundo paso de la estrategia digital de la clínica (registros de exámenes, indicaciones, historial y recetas). Otras apps de red: Mi Dávila (Red Dávila, gestión de citas en todos sus centros, según un directorio); Clínica Las Condes sin app confirmada. [Vuelta 9] Sin búsqueda nueva; sin cambios. [Vuelta 10] Sin búsqueda nueva (saturado).</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="G13" t="n">
@@ -966,7 +966,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-31</t>
         </is>
       </c>
     </row>
@@ -10929,7 +10929,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A46"/>
+  <dimension ref="A1:A47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -11257,6 +11257,13 @@
         </is>
       </c>
     </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Vuelta 10 (iter. 3, 2026-10-31 12:16 UTC): Apple Health, ChatGPT Health, Claude for Healthcare, Apps de clínicas verificados (+0 filas). Pendientes: Clinia, MiRedSalud, Mediko (cierran la vuelta 10 y regeneran func_norm/tabla_frecuencia).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>